<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-24 12:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7582,7 +7582,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMIA,ECONOMICIDADE OBRAS,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ECONOMIA,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL</t>
@@ -7714,7 +7714,7 @@
     <t>VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
@@ -7729,7 +7729,7 @@
     <t>RECURSOS HÍDRICOS,ORÇAMENTO</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,URBANISMO,SAÚDE,ECONOMIA,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ORÇAMENTO</t>
+    <t>SAÚDE,URBANISMO,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,PSICOLOGIA</t>
   </si>
 </sst>
 </file>
@@ -18892,7 +18892,7 @@
         <v>1524</v>
       </c>
       <c r="I307" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J307" t="s">
         <v>2023</v>
@@ -30532,7 +30532,7 @@
         <v>1606</v>
       </c>
       <c r="I637" t="s">
-        <v>1613</v>
+        <v>1662</v>
       </c>
       <c r="J637" t="s">
         <v>2335</v>
@@ -30541,7 +30541,7 @@
         <v>2376</v>
       </c>
       <c r="L637" t="s">
-        <v>2540</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="638" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-09 14:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5131,6 +5131,9 @@
     <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
   </si>
   <si>
+    <t>GLAUCO CASTILHO DE ALMEIDA</t>
+  </si>
+  <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,PATRÍCIA FINAMORE ARAÚJO,SIMONE MANNHEIMER DE ALVARENGA</t>
   </si>
   <si>
@@ -5191,9 +5194,6 @@
     <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
   </si>
   <si>
-    <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
     <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
   </si>
   <si>
@@ -5251,28 +5251,28 @@
     <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
   </si>
   <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>DAGER SALLES AMARAL,EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO</t>
+  </si>
+  <si>
     <t>MARCELO KOLBLINGER DE GODOY</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>DAGER SALLES AMARAL,EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO</t>
   </si>
   <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING, _SEM USUARIO ATRIBUIDO</t>
@@ -13026,7 +13026,7 @@
         <v>1609</v>
       </c>
       <c r="I134" t="s">
-        <v>1653</v>
+        <v>1705</v>
       </c>
       <c r="J134" t="s">
         <v>1904</v>
@@ -13061,7 +13061,7 @@
         <v>1609</v>
       </c>
       <c r="I135" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="J135" t="s">
         <v>1905</v>
@@ -13096,7 +13096,7 @@
         <v>1609</v>
       </c>
       <c r="I136" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J136" t="s">
         <v>1906</v>
@@ -13131,7 +13131,7 @@
         <v>1609</v>
       </c>
       <c r="I137" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="J137" t="s">
         <v>1907</v>
@@ -13166,7 +13166,7 @@
         <v>1609</v>
       </c>
       <c r="I138" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J138" t="s">
         <v>1908</v>
@@ -13201,7 +13201,7 @@
         <v>1609</v>
       </c>
       <c r="I139" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J139" t="s">
         <v>1909</v>
@@ -13306,7 +13306,7 @@
         <v>1609</v>
       </c>
       <c r="I142" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J142" t="s">
         <v>1912</v>
@@ -13344,7 +13344,7 @@
         <v>1477</v>
       </c>
       <c r="I143" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J143" t="s">
         <v>1913</v>
@@ -13589,7 +13589,7 @@
         <v>1609</v>
       </c>
       <c r="I150" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J150" t="s">
         <v>1920</v>
@@ -13977,7 +13977,7 @@
         <v>1609</v>
       </c>
       <c r="I161" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J161" t="s">
         <v>1931</v>
@@ -14085,7 +14085,7 @@
         <v>1609</v>
       </c>
       <c r="I164" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J164" t="s">
         <v>1934</v>
@@ -14298,7 +14298,7 @@
         <v>1609</v>
       </c>
       <c r="I170" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J170" t="s">
         <v>1940</v>
@@ -14476,7 +14476,7 @@
         <v>1609</v>
       </c>
       <c r="I175" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J175" t="s">
         <v>1945</v>
@@ -14546,7 +14546,7 @@
         <v>1609</v>
       </c>
       <c r="I177" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J177" t="s">
         <v>1947</v>
@@ -14826,7 +14826,7 @@
         <v>1609</v>
       </c>
       <c r="I185" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J185" t="s">
         <v>1955</v>
@@ -14966,7 +14966,7 @@
         <v>1609</v>
       </c>
       <c r="I189" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J189" t="s">
         <v>1959</v>
@@ -15001,7 +15001,7 @@
         <v>1609</v>
       </c>
       <c r="I190" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J190" t="s">
         <v>1959</v>
@@ -15141,7 +15141,7 @@
         <v>1609</v>
       </c>
       <c r="I194" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J194" t="s">
         <v>1961</v>
@@ -15176,7 +15176,7 @@
         <v>1609</v>
       </c>
       <c r="I195" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J195" t="s">
         <v>1962</v>
@@ -15316,7 +15316,7 @@
         <v>1609</v>
       </c>
       <c r="I199" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J199" t="s">
         <v>1966</v>
@@ -15386,7 +15386,7 @@
         <v>1609</v>
       </c>
       <c r="I201" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J201" t="s">
         <v>1968</v>
@@ -15777,7 +15777,7 @@
         <v>1609</v>
       </c>
       <c r="I212" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J212" t="s">
         <v>1978</v>
@@ -15952,7 +15952,7 @@
         <v>1609</v>
       </c>
       <c r="I217" t="s">
-        <v>1725</v>
+        <v>1705</v>
       </c>
       <c r="J217" t="s">
         <v>1786</v>
@@ -17638,7 +17638,7 @@
         <v>1609</v>
       </c>
       <c r="I265" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J265" t="s">
         <v>2028</v>
@@ -17953,7 +17953,7 @@
         <v>1609</v>
       </c>
       <c r="I274" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J274" t="s">
         <v>2037</v>
@@ -19467,7 +19467,7 @@
         <v>1609</v>
       </c>
       <c r="I317" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J317" t="s">
         <v>2076</v>
@@ -20167,7 +20167,7 @@
         <v>1609</v>
       </c>
       <c r="I337" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J337" t="s">
         <v>2096</v>
@@ -20762,7 +20762,7 @@
         <v>1609</v>
       </c>
       <c r="I354" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J354" t="s">
         <v>2113</v>
@@ -20832,7 +20832,7 @@
         <v>1609</v>
       </c>
       <c r="I356" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J356" t="s">
         <v>2115</v>
@@ -21010,7 +21010,7 @@
         <v>1609</v>
       </c>
       <c r="I361" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J361" t="s">
         <v>2120</v>
@@ -21185,7 +21185,7 @@
         <v>1609</v>
       </c>
       <c r="I366" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J366" t="s">
         <v>2125</v>
@@ -21640,7 +21640,7 @@
         <v>1609</v>
       </c>
       <c r="I379" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J379" t="s">
         <v>2138</v>
@@ -21923,7 +21923,7 @@
         <v>1609</v>
       </c>
       <c r="I387" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J387" t="s">
         <v>2145</v>
@@ -22063,7 +22063,7 @@
         <v>1609</v>
       </c>
       <c r="I391" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J391" t="s">
         <v>2148</v>
@@ -22182,7 +22182,7 @@
     </row>
     <row r="395" spans="1:12">
       <c r="A395" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B395" t="s">
         <v>436</v>
@@ -22203,7 +22203,7 @@
         <v>1609</v>
       </c>
       <c r="I395" t="s">
-        <v>1745</v>
+        <v>1653</v>
       </c>
       <c r="J395" t="s">
         <v>2152</v>
@@ -22273,7 +22273,7 @@
         <v>1609</v>
       </c>
       <c r="I397" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="J397" t="s">
         <v>2154</v>
@@ -22343,7 +22343,7 @@
         <v>1609</v>
       </c>
       <c r="I399" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J399" t="s">
         <v>2156</v>
@@ -22769,7 +22769,7 @@
         <v>1609</v>
       </c>
       <c r="I411" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J411" t="s">
         <v>2167</v>
@@ -22804,7 +22804,7 @@
         <v>1609</v>
       </c>
       <c r="I412" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J412" t="s">
         <v>2168</v>
@@ -22979,7 +22979,7 @@
         <v>1609</v>
       </c>
       <c r="I417" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J417" t="s">
         <v>2172</v>
@@ -23084,7 +23084,7 @@
         <v>1609</v>
       </c>
       <c r="I420" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J420" t="s">
         <v>2175</v>
@@ -23224,7 +23224,7 @@
         <v>1609</v>
       </c>
       <c r="I424" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J424" t="s">
         <v>2179</v>
@@ -23259,7 +23259,7 @@
         <v>1609</v>
       </c>
       <c r="I425" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J425" t="s">
         <v>2180</v>
@@ -23294,7 +23294,7 @@
         <v>1609</v>
       </c>
       <c r="I426" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J426" t="s">
         <v>2181</v>
@@ -23507,7 +23507,7 @@
         <v>1629</v>
       </c>
       <c r="I432" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="J432" t="s">
         <v>2187</v>
@@ -23542,7 +23542,7 @@
         <v>1609</v>
       </c>
       <c r="I433" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J433" t="s">
         <v>2188</v>
@@ -23682,7 +23682,7 @@
         <v>1609</v>
       </c>
       <c r="I437" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J437" t="s">
         <v>2192</v>
@@ -23717,7 +23717,7 @@
         <v>1609</v>
       </c>
       <c r="I438" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J438" t="s">
         <v>2193</v>
@@ -23752,7 +23752,7 @@
         <v>1609</v>
       </c>
       <c r="I439" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J439" t="s">
         <v>2194</v>
@@ -23787,7 +23787,7 @@
         <v>1609</v>
       </c>
       <c r="I440" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J440" t="s">
         <v>2195</v>
@@ -23857,7 +23857,7 @@
         <v>1609</v>
       </c>
       <c r="I442" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J442" t="s">
         <v>2197</v>
@@ -24242,7 +24242,7 @@
         <v>1609</v>
       </c>
       <c r="I453" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J453" t="s">
         <v>2207</v>
@@ -24277,7 +24277,7 @@
         <v>1609</v>
       </c>
       <c r="I454" t="s">
-        <v>1745</v>
+        <v>1752</v>
       </c>
       <c r="J454" t="s">
         <v>2208</v>
@@ -24347,7 +24347,7 @@
         <v>1609</v>
       </c>
       <c r="I456" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J456" t="s">
         <v>2210</v>
@@ -24417,7 +24417,7 @@
         <v>1609</v>
       </c>
       <c r="I458" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J458" t="s">
         <v>1959</v>
@@ -24522,7 +24522,7 @@
         <v>1609</v>
       </c>
       <c r="I461" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J461" t="s">
         <v>2214</v>
@@ -24557,7 +24557,7 @@
         <v>1609</v>
       </c>
       <c r="I462" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J462" t="s">
         <v>2215</v>
@@ -25193,7 +25193,7 @@
         <v>1609</v>
       </c>
       <c r="I480" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J480" t="s">
         <v>2233</v>
@@ -25479,7 +25479,7 @@
         <v>1609</v>
       </c>
       <c r="I488" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J488" t="s">
         <v>2241</v>
@@ -25727,7 +25727,7 @@
         <v>1609</v>
       </c>
       <c r="I495" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J495" t="s">
         <v>2248</v>
@@ -25762,7 +25762,7 @@
         <v>1609</v>
       </c>
       <c r="I496" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J496" t="s">
         <v>2249</v>
@@ -25870,7 +25870,7 @@
         <v>1609</v>
       </c>
       <c r="I499" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J499" t="s">
         <v>2252</v>
@@ -25940,7 +25940,7 @@
         <v>1609</v>
       </c>
       <c r="I501" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J501" t="s">
         <v>2254</v>
@@ -26366,7 +26366,7 @@
         <v>1609</v>
       </c>
       <c r="I513" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J513" t="s">
         <v>2266</v>
@@ -26509,7 +26509,7 @@
         <v>1609</v>
       </c>
       <c r="I517" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J517" t="s">
         <v>2270</v>
@@ -26544,7 +26544,7 @@
         <v>1609</v>
       </c>
       <c r="I518" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J518" t="s">
         <v>2271</v>
@@ -26579,7 +26579,7 @@
         <v>1609</v>
       </c>
       <c r="I519" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J519" t="s">
         <v>2272</v>
@@ -26929,7 +26929,7 @@
         <v>1609</v>
       </c>
       <c r="I529" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J529" t="s">
         <v>2282</v>
@@ -27183,7 +27183,7 @@
         <v>1609</v>
       </c>
       <c r="I536" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J536" t="s">
         <v>2289</v>
@@ -27218,7 +27218,7 @@
         <v>1609</v>
       </c>
       <c r="I537" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J537" t="s">
         <v>2290</v>
@@ -27358,7 +27358,7 @@
         <v>1609</v>
       </c>
       <c r="I541" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J541" t="s">
         <v>2293</v>
@@ -27582,7 +27582,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B548" t="s">
         <v>589</v>
@@ -27603,7 +27603,7 @@
         <v>1609</v>
       </c>
       <c r="I548" t="s">
-        <v>1723</v>
+        <v>1653</v>
       </c>
       <c r="J548" t="s">
         <v>2300</v>
@@ -27743,7 +27743,7 @@
         <v>1609</v>
       </c>
       <c r="I552" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J552" t="s">
         <v>2304</v>
@@ -27813,7 +27813,7 @@
         <v>1609</v>
       </c>
       <c r="I554" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J554" t="s">
         <v>2306</v>
@@ -27862,7 +27862,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B556" t="s">
         <v>597</v>
@@ -27883,7 +27883,7 @@
         <v>1609</v>
       </c>
       <c r="I556" t="s">
-        <v>1754</v>
+        <v>1653</v>
       </c>
       <c r="J556" t="s">
         <v>2308</v>
@@ -28274,7 +28274,7 @@
         <v>1609</v>
       </c>
       <c r="I567" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J567" t="s">
         <v>2318</v>
@@ -28309,7 +28309,7 @@
         <v>1609</v>
       </c>
       <c r="I568" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J568" t="s">
         <v>2319</v>
@@ -28344,7 +28344,7 @@
         <v>1609</v>
       </c>
       <c r="I569" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J569" t="s">
         <v>2320</v>
@@ -28878,7 +28878,7 @@
         <v>1609</v>
       </c>
       <c r="I584" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J584" t="s">
         <v>2333</v>
@@ -29129,7 +29129,7 @@
         <v>1609</v>
       </c>
       <c r="I591" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J591" t="s">
         <v>2340</v>
@@ -29310,7 +29310,7 @@
         <v>1609</v>
       </c>
       <c r="I596" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J596" t="s">
         <v>2344</v>
@@ -29380,7 +29380,7 @@
         <v>1609</v>
       </c>
       <c r="I598" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J598" t="s">
         <v>2346</v>
@@ -29628,7 +29628,7 @@
         <v>1609</v>
       </c>
       <c r="I605" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J605" t="s">
         <v>2353</v>
@@ -30124,7 +30124,7 @@
         <v>1609</v>
       </c>
       <c r="I619" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J619" t="s">
         <v>2367</v>
@@ -30159,7 +30159,7 @@
         <v>1609</v>
       </c>
       <c r="I620" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J620" t="s">
         <v>2368</v>
@@ -30404,7 +30404,7 @@
         <v>1609</v>
       </c>
       <c r="I627" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J627" t="s">
         <v>2374</v>
@@ -30439,7 +30439,7 @@
         <v>1609</v>
       </c>
       <c r="I628" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J628" t="s">
         <v>2375</v>
@@ -30579,7 +30579,7 @@
         <v>1609</v>
       </c>
       <c r="I632" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J632" t="s">
         <v>2379</v>
@@ -30827,7 +30827,7 @@
         <v>1609</v>
       </c>
       <c r="I639" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J639" t="s">
         <v>2386</v>
@@ -31259,7 +31259,7 @@
         <v>1609</v>
       </c>
       <c r="I651" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J651" t="s">
         <v>2398</v>
@@ -31332,7 +31332,7 @@
         <v>1648</v>
       </c>
       <c r="I653" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J653" t="s">
         <v>2400</v>
@@ -31405,7 +31405,7 @@
         <v>1609</v>
       </c>
       <c r="I655" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J655" t="s">
         <v>2402</v>
@@ -31551,7 +31551,7 @@
         <v>1609</v>
       </c>
       <c r="I659" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J659" t="s">
         <v>2406</v>
@@ -31586,7 +31586,7 @@
         <v>1609</v>
       </c>
       <c r="I660" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J660" t="s">
         <v>2407</v>
@@ -31621,7 +31621,7 @@
         <v>1609</v>
       </c>
       <c r="I661" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J661" t="s">
         <v>2408</v>
@@ -31729,7 +31729,7 @@
         <v>1609</v>
       </c>
       <c r="I664" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J664" t="s">
         <v>2411</v>
@@ -31834,7 +31834,7 @@
         <v>1609</v>
       </c>
       <c r="I667" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J667" t="s">
         <v>2414</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-16 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -19997,7 +19997,7 @@
     </row>
     <row r="339" spans="1:12">
       <c r="A339" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="B339" t="s">
         <v>382</v>
@@ -20018,7 +20018,7 @@
         <v>1562</v>
       </c>
       <c r="I339" t="s">
-        <v>1668</v>
+        <v>1602</v>
       </c>
       <c r="J339" t="s">
         <v>2053</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-16 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -30686,7 +30686,7 @@
     </row>
     <row r="642" spans="1:12">
       <c r="A642" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B642" t="s">
         <v>683</v>
@@ -30707,7 +30707,7 @@
         <v>1560</v>
       </c>
       <c r="I642" t="s">
-        <v>1600</v>
+        <v>1728</v>
       </c>
       <c r="J642" t="s">
         <v>2342</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-18 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6759" uniqueCount="2640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6759" uniqueCount="2639">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7852,7 +7852,7 @@
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>FARMÁCIA,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,FARMÁCIA</t>
   </si>
   <si>
     <t>RESÍDUOS SÓLIDOS</t>
@@ -7864,7 +7864,7 @@
     <t>ASSISTÊNCIA SOCIAL</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,EDIFICAÇÕES</t>
+    <t>EDIFICAÇÕES,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7930,10 +7930,7 @@
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMIA,ORÇAMENTO,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,SAÚDE,AVALIAÇÃO DE IMÓVEIS,SAÚDE MENTAL,URBANISMO,ASSISTÊNCIA SOCIAL</t>
+    <t>ECONOMIA,PSICOLOGIA,SAÚDE,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,URBANISMO,ORÇAMENTO,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
 </sst>
 </file>
@@ -13197,7 +13194,7 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B140" t="s">
         <v>184</v>
@@ -13218,7 +13215,7 @@
         <v>1605</v>
       </c>
       <c r="I140" t="s">
-        <v>1679</v>
+        <v>1644</v>
       </c>
       <c r="J140" t="s">
         <v>1910</v>
@@ -31498,7 +31495,7 @@
         <v>2562</v>
       </c>
       <c r="L658" t="s">
-        <v>2604</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="659" spans="1:12">
@@ -31848,7 +31845,7 @@
         <v>2564</v>
       </c>
       <c r="L668" t="s">
-        <v>2638</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="669" spans="1:12">
@@ -31880,7 +31877,7 @@
         <v>2564</v>
       </c>
       <c r="L669" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="670" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-19 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -31174,7 +31174,7 @@
         <v>1607</v>
       </c>
       <c r="I649" t="s">
-        <v>1646</v>
+        <v>1775</v>
       </c>
       <c r="J649" t="s">
         <v>2209</v>
@@ -31188,7 +31188,7 @@
     </row>
     <row r="650" spans="1:12">
       <c r="A650" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B650" t="s">
         <v>693</v>
@@ -31209,7 +31209,7 @@
         <v>1607</v>
       </c>
       <c r="I650" t="s">
-        <v>1646</v>
+        <v>1774</v>
       </c>
       <c r="J650" t="s">
         <v>2399</v>
@@ -31223,7 +31223,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B651" t="s">
         <v>694</v>
@@ -31244,7 +31244,7 @@
         <v>1607</v>
       </c>
       <c r="I651" t="s">
-        <v>1646</v>
+        <v>1774</v>
       </c>
       <c r="J651" t="s">
         <v>2400</v>
@@ -31258,7 +31258,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B652" t="s">
         <v>695</v>
@@ -31279,7 +31279,7 @@
         <v>1607</v>
       </c>
       <c r="I652" t="s">
-        <v>1646</v>
+        <v>1774</v>
       </c>
       <c r="J652" t="s">
         <v>2108</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-20 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -31806,7 +31806,7 @@
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B665" t="s">
         <v>709</v>
@@ -31827,7 +31827,7 @@
         <v>1627</v>
       </c>
       <c r="I665" t="s">
-        <v>1666</v>
+        <v>1797</v>
       </c>
       <c r="J665" t="s">
         <v>2434</v>
@@ -31841,7 +31841,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B666" t="s">
         <v>710</v>
@@ -31862,7 +31862,7 @@
         <v>1627</v>
       </c>
       <c r="I666" t="s">
-        <v>1666</v>
+        <v>1797</v>
       </c>
       <c r="J666" t="s">
         <v>2435</v>
@@ -31876,7 +31876,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B667" t="s">
         <v>711</v>
@@ -31900,7 +31900,7 @@
         <v>1661</v>
       </c>
       <c r="I667" t="s">
-        <v>1666</v>
+        <v>1797</v>
       </c>
       <c r="J667" t="s">
         <v>2436</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-23 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -11987,7 +11987,7 @@
     </row>
     <row r="102" spans="1:12">
       <c r="A102" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B102" t="s">
         <v>144</v>
@@ -12008,7 +12008,7 @@
         <v>1635</v>
       </c>
       <c r="I102" t="s">
-        <v>1716</v>
+        <v>1672</v>
       </c>
       <c r="J102" t="s">
         <v>1899</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-23 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5152,6 +5152,9 @@
     <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>GIULIANA DE ANDRADE CERVAI</t>
   </si>
   <si>
@@ -5279,9 +5282,6 @@
   </si>
   <si>
     <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
@@ -11949,7 +11949,7 @@
         <v>1631</v>
       </c>
       <c r="I101" t="s">
-        <v>1668</v>
+        <v>1712</v>
       </c>
       <c r="J101" t="s">
         <v>1894</v>
@@ -11984,7 +11984,7 @@
         <v>1631</v>
       </c>
       <c r="I102" t="s">
-        <v>1668</v>
+        <v>1712</v>
       </c>
       <c r="J102" t="s">
         <v>1895</v>
@@ -12019,7 +12019,7 @@
         <v>1631</v>
       </c>
       <c r="I103" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J103" t="s">
         <v>1896</v>
@@ -12089,7 +12089,7 @@
         <v>1631</v>
       </c>
       <c r="I105" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J105" t="s">
         <v>1898</v>
@@ -12194,7 +12194,7 @@
         <v>1631</v>
       </c>
       <c r="I108" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J108" t="s">
         <v>1901</v>
@@ -12512,7 +12512,7 @@
         <v>1631</v>
       </c>
       <c r="I117" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J117" t="s">
         <v>1910</v>
@@ -12547,7 +12547,7 @@
         <v>1631</v>
       </c>
       <c r="I118" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J118" t="s">
         <v>1911</v>
@@ -12582,7 +12582,7 @@
         <v>1631</v>
       </c>
       <c r="I119" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J119" t="s">
         <v>1912</v>
@@ -12617,7 +12617,7 @@
         <v>1631</v>
       </c>
       <c r="I120" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J120" t="s">
         <v>1913</v>
@@ -12652,7 +12652,7 @@
         <v>1631</v>
       </c>
       <c r="I121" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J121" t="s">
         <v>1914</v>
@@ -12725,7 +12725,7 @@
         <v>1493</v>
       </c>
       <c r="I123" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J123" t="s">
         <v>1916</v>
@@ -12795,7 +12795,7 @@
         <v>1631</v>
       </c>
       <c r="I125" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J125" t="s">
         <v>1918</v>
@@ -12830,7 +12830,7 @@
         <v>1631</v>
       </c>
       <c r="I126" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J126" t="s">
         <v>1919</v>
@@ -12865,7 +12865,7 @@
         <v>1631</v>
       </c>
       <c r="I127" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J127" t="s">
         <v>1920</v>
@@ -12970,7 +12970,7 @@
         <v>1631</v>
       </c>
       <c r="I130" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J130" t="s">
         <v>1923</v>
@@ -13183,7 +13183,7 @@
         <v>1631</v>
       </c>
       <c r="I136" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J136" t="s">
         <v>1929</v>
@@ -13253,7 +13253,7 @@
         <v>1631</v>
       </c>
       <c r="I138" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="J138" t="s">
         <v>1931</v>
@@ -13361,7 +13361,7 @@
         <v>1639</v>
       </c>
       <c r="I141" t="s">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="J141" t="s">
         <v>1934</v>
@@ -13396,7 +13396,7 @@
         <v>1631</v>
       </c>
       <c r="I142" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="J142" t="s">
         <v>1935</v>
@@ -13434,7 +13434,7 @@
         <v>1640</v>
       </c>
       <c r="I143" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J143" t="s">
         <v>1936</v>
@@ -13574,7 +13574,7 @@
         <v>1631</v>
       </c>
       <c r="I147" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J147" t="s">
         <v>1940</v>
@@ -13717,7 +13717,7 @@
         <v>1631</v>
       </c>
       <c r="I151" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J151" t="s">
         <v>1944</v>
@@ -13787,7 +13787,7 @@
         <v>1631</v>
       </c>
       <c r="I153" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J153" t="s">
         <v>1946</v>
@@ -13997,7 +13997,7 @@
         <v>1631</v>
       </c>
       <c r="I159" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="J159" t="s">
         <v>1952</v>
@@ -14137,7 +14137,7 @@
         <v>1631</v>
       </c>
       <c r="I163" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J163" t="s">
         <v>1956</v>
@@ -14172,7 +14172,7 @@
         <v>1631</v>
       </c>
       <c r="I164" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J164" t="s">
         <v>1956</v>
@@ -14312,7 +14312,7 @@
         <v>1631</v>
       </c>
       <c r="I168" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J168" t="s">
         <v>1958</v>
@@ -14347,7 +14347,7 @@
         <v>1631</v>
       </c>
       <c r="I169" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="J169" t="s">
         <v>1959</v>
@@ -14487,7 +14487,7 @@
         <v>1631</v>
       </c>
       <c r="I173" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J173" t="s">
         <v>1963</v>
@@ -14595,7 +14595,7 @@
         <v>1642</v>
       </c>
       <c r="I176" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J176" t="s">
         <v>1966</v>
@@ -14633,7 +14633,7 @@
         <v>1642</v>
       </c>
       <c r="I177" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J177" t="s">
         <v>1966</v>
@@ -14878,7 +14878,7 @@
         <v>1631</v>
       </c>
       <c r="I184" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J184" t="s">
         <v>1973</v>
@@ -15091,7 +15091,7 @@
         <v>1643</v>
       </c>
       <c r="I190" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="J190" t="s">
         <v>1979</v>
@@ -15196,7 +15196,7 @@
         <v>1631</v>
       </c>
       <c r="I193" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J193" t="s">
         <v>1982</v>
@@ -15371,7 +15371,7 @@
         <v>1631</v>
       </c>
       <c r="I198" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="J198" t="s">
         <v>1987</v>
@@ -15756,7 +15756,7 @@
         <v>1631</v>
       </c>
       <c r="I209" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J209" t="s">
         <v>1996</v>
@@ -15826,7 +15826,7 @@
         <v>1631</v>
       </c>
       <c r="I211" t="s">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="J211" t="s">
         <v>1998</v>
@@ -16071,7 +16071,7 @@
         <v>1631</v>
       </c>
       <c r="I218" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J218" t="s">
         <v>2005</v>
@@ -16141,7 +16141,7 @@
         <v>1631</v>
       </c>
       <c r="I220" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J220" t="s">
         <v>2007</v>
@@ -16526,7 +16526,7 @@
         <v>1631</v>
       </c>
       <c r="I231" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J231" t="s">
         <v>2018</v>
@@ -16631,7 +16631,7 @@
         <v>1631</v>
       </c>
       <c r="I234" t="s">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="J234" t="s">
         <v>2021</v>
@@ -16666,7 +16666,7 @@
         <v>1631</v>
       </c>
       <c r="I235" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J235" t="s">
         <v>2022</v>
@@ -16914,7 +16914,7 @@
         <v>1631</v>
       </c>
       <c r="I242" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J242" t="s">
         <v>2029</v>
@@ -16949,7 +16949,7 @@
         <v>1631</v>
       </c>
       <c r="I243" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J243" t="s">
         <v>2030</v>
@@ -17089,7 +17089,7 @@
         <v>1631</v>
       </c>
       <c r="I247" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J247" t="s">
         <v>2033</v>
@@ -17162,7 +17162,7 @@
         <v>1644</v>
       </c>
       <c r="I249" t="s">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="J249" t="s">
         <v>2035</v>
@@ -17197,7 +17197,7 @@
         <v>1631</v>
       </c>
       <c r="I250" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J250" t="s">
         <v>2036</v>
@@ -17267,7 +17267,7 @@
         <v>1631</v>
       </c>
       <c r="I252" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J252" t="s">
         <v>2038</v>
@@ -17407,7 +17407,7 @@
         <v>1631</v>
       </c>
       <c r="I256" t="s">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="J256" t="s">
         <v>2041</v>
@@ -17547,7 +17547,7 @@
         <v>1631</v>
       </c>
       <c r="I260" t="s">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="J260" t="s">
         <v>2045</v>
@@ -17865,7 +17865,7 @@
         <v>1631</v>
       </c>
       <c r="I269" t="s">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="J269" t="s">
         <v>2052</v>
@@ -17970,7 +17970,7 @@
         <v>1631</v>
       </c>
       <c r="I272" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J272" t="s">
         <v>2055</v>
@@ -18040,7 +18040,7 @@
         <v>1631</v>
       </c>
       <c r="I274" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J274" t="s">
         <v>2057</v>
@@ -18145,7 +18145,7 @@
         <v>1631</v>
       </c>
       <c r="I277" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J277" t="s">
         <v>2060</v>
@@ -18215,7 +18215,7 @@
         <v>1631</v>
       </c>
       <c r="I279" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J279" t="s">
         <v>2062</v>
@@ -18355,7 +18355,7 @@
         <v>1631</v>
       </c>
       <c r="I283" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J283" t="s">
         <v>2066</v>
@@ -18460,7 +18460,7 @@
         <v>1631</v>
       </c>
       <c r="I286" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J286" t="s">
         <v>2069</v>
@@ -18495,7 +18495,7 @@
         <v>1631</v>
       </c>
       <c r="I287" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J287" t="s">
         <v>2070</v>
@@ -18565,7 +18565,7 @@
         <v>1631</v>
       </c>
       <c r="I289" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J289" t="s">
         <v>2072</v>
@@ -18635,7 +18635,7 @@
         <v>1631</v>
       </c>
       <c r="I291" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J291" t="s">
         <v>2074</v>
@@ -18740,7 +18740,7 @@
         <v>1631</v>
       </c>
       <c r="I294" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J294" t="s">
         <v>2077</v>
@@ -18915,7 +18915,7 @@
         <v>1631</v>
       </c>
       <c r="I299" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J299" t="s">
         <v>2082</v>
@@ -18985,7 +18985,7 @@
         <v>1631</v>
       </c>
       <c r="I301" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J301" t="s">
         <v>2084</v>
@@ -19020,7 +19020,7 @@
         <v>1631</v>
       </c>
       <c r="I302" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J302" t="s">
         <v>2085</v>
@@ -19055,7 +19055,7 @@
         <v>1631</v>
       </c>
       <c r="I303" t="s">
-        <v>1755</v>
+        <v>1712</v>
       </c>
       <c r="J303" t="s">
         <v>2086</v>
@@ -19230,7 +19230,7 @@
         <v>1631</v>
       </c>
       <c r="I308" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J308" t="s">
         <v>2091</v>
@@ -19335,7 +19335,7 @@
         <v>1631</v>
       </c>
       <c r="I311" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J311" t="s">
         <v>2094</v>
@@ -19405,7 +19405,7 @@
         <v>1631</v>
       </c>
       <c r="I313" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J313" t="s">
         <v>2096</v>
@@ -19548,7 +19548,7 @@
         <v>1631</v>
       </c>
       <c r="I317" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J317" t="s">
         <v>2100</v>
@@ -19583,7 +19583,7 @@
         <v>1631</v>
       </c>
       <c r="I318" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J318" t="s">
         <v>2101</v>
@@ -19618,7 +19618,7 @@
         <v>1631</v>
       </c>
       <c r="I319" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J319" t="s">
         <v>2102</v>
@@ -20108,7 +20108,7 @@
         <v>1631</v>
       </c>
       <c r="I333" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J333" t="s">
         <v>2116</v>
@@ -20143,7 +20143,7 @@
         <v>1631</v>
       </c>
       <c r="I334" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J334" t="s">
         <v>2117</v>
@@ -20668,7 +20668,7 @@
         <v>1631</v>
       </c>
       <c r="I349" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J349" t="s">
         <v>1880</v>
@@ -20811,7 +20811,7 @@
         <v>1631</v>
       </c>
       <c r="I353" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J353" t="s">
         <v>2133</v>
@@ -21094,7 +21094,7 @@
         <v>1631</v>
       </c>
       <c r="I361" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J361" t="s">
         <v>2141</v>
@@ -21164,7 +21164,7 @@
         <v>1635</v>
       </c>
       <c r="I363" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J363" t="s">
         <v>2143</v>
@@ -21199,7 +21199,7 @@
         <v>1631</v>
       </c>
       <c r="I364" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J364" t="s">
         <v>2144</v>
@@ -21234,7 +21234,7 @@
         <v>1631</v>
       </c>
       <c r="I365" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J365" t="s">
         <v>2072</v>
@@ -21269,7 +21269,7 @@
         <v>1631</v>
       </c>
       <c r="I366" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J366" t="s">
         <v>2145</v>
@@ -21479,7 +21479,7 @@
         <v>1631</v>
       </c>
       <c r="I372" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J372" t="s">
         <v>2151</v>
@@ -21549,7 +21549,7 @@
         <v>1631</v>
       </c>
       <c r="I374" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J374" t="s">
         <v>2153</v>
@@ -21692,7 +21692,7 @@
         <v>1631</v>
       </c>
       <c r="I378" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J378" t="s">
         <v>2157</v>
@@ -21727,7 +21727,7 @@
         <v>1631</v>
       </c>
       <c r="I379" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J379" t="s">
         <v>2158</v>
@@ -21832,7 +21832,7 @@
         <v>1631</v>
       </c>
       <c r="I382" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J382" t="s">
         <v>2161</v>
@@ -21902,7 +21902,7 @@
         <v>1631</v>
       </c>
       <c r="I384" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J384" t="s">
         <v>2163</v>
@@ -22007,7 +22007,7 @@
         <v>1631</v>
       </c>
       <c r="I387" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J387" t="s">
         <v>2166</v>
@@ -22252,7 +22252,7 @@
         <v>1631</v>
       </c>
       <c r="I394" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J394" t="s">
         <v>2173</v>
@@ -22392,7 +22392,7 @@
         <v>1631</v>
       </c>
       <c r="I398" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J398" t="s">
         <v>2176</v>
@@ -22462,7 +22462,7 @@
         <v>1631</v>
       </c>
       <c r="I400" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J400" t="s">
         <v>2178</v>
@@ -22497,7 +22497,7 @@
         <v>1631</v>
       </c>
       <c r="I401" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J401" t="s">
         <v>2179</v>
@@ -22532,7 +22532,7 @@
         <v>1631</v>
       </c>
       <c r="I402" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J402" t="s">
         <v>1956</v>
@@ -22637,7 +22637,7 @@
         <v>1631</v>
       </c>
       <c r="I405" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J405" t="s">
         <v>2182</v>
@@ -22672,7 +22672,7 @@
         <v>1631</v>
       </c>
       <c r="I406" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J406" t="s">
         <v>2183</v>
@@ -22742,7 +22742,7 @@
         <v>1631</v>
       </c>
       <c r="I408" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J408" t="s">
         <v>2185</v>
@@ -23025,7 +23025,7 @@
         <v>1631</v>
       </c>
       <c r="I416" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J416" t="s">
         <v>2193</v>
@@ -23238,7 +23238,7 @@
         <v>1631</v>
       </c>
       <c r="I422" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J422" t="s">
         <v>2199</v>
@@ -23419,7 +23419,7 @@
         <v>1631</v>
       </c>
       <c r="I427" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J427" t="s">
         <v>2204</v>
@@ -23454,7 +23454,7 @@
         <v>1631</v>
       </c>
       <c r="I428" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J428" t="s">
         <v>2205</v>
@@ -23559,7 +23559,7 @@
         <v>1631</v>
       </c>
       <c r="I431" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J431" t="s">
         <v>2208</v>
@@ -23664,7 +23664,7 @@
         <v>1631</v>
       </c>
       <c r="I434" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J434" t="s">
         <v>2211</v>
@@ -23699,7 +23699,7 @@
         <v>1631</v>
       </c>
       <c r="I435" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J435" t="s">
         <v>2212</v>
@@ -23734,7 +23734,7 @@
         <v>1631</v>
       </c>
       <c r="I436" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J436" t="s">
         <v>2213</v>
@@ -23839,7 +23839,7 @@
         <v>1631</v>
       </c>
       <c r="I439" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J439" t="s">
         <v>2216</v>
@@ -23909,7 +23909,7 @@
         <v>1631</v>
       </c>
       <c r="I441" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J441" t="s">
         <v>2218</v>
@@ -23944,7 +23944,7 @@
         <v>1631</v>
       </c>
       <c r="I442" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J442" t="s">
         <v>2219</v>
@@ -23979,7 +23979,7 @@
         <v>1631</v>
       </c>
       <c r="I443" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J443" t="s">
         <v>2220</v>
@@ -24014,7 +24014,7 @@
         <v>1631</v>
       </c>
       <c r="I444" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J444" t="s">
         <v>2221</v>
@@ -24154,7 +24154,7 @@
         <v>1631</v>
       </c>
       <c r="I448" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J448" t="s">
         <v>2225</v>
@@ -24227,7 +24227,7 @@
         <v>1648</v>
       </c>
       <c r="I450" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J450" t="s">
         <v>2227</v>
@@ -24297,7 +24297,7 @@
         <v>1631</v>
       </c>
       <c r="I452" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J452" t="s">
         <v>2229</v>
@@ -24332,7 +24332,7 @@
         <v>1631</v>
       </c>
       <c r="I453" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J453" t="s">
         <v>2230</v>
@@ -24437,7 +24437,7 @@
         <v>1631</v>
       </c>
       <c r="I456" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J456" t="s">
         <v>2233</v>
@@ -24542,7 +24542,7 @@
         <v>1631</v>
       </c>
       <c r="I459" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J459" t="s">
         <v>2236</v>
@@ -24612,7 +24612,7 @@
         <v>1631</v>
       </c>
       <c r="I461" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J461" t="s">
         <v>2238</v>
@@ -24647,7 +24647,7 @@
         <v>1631</v>
       </c>
       <c r="I462" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J462" t="s">
         <v>2239</v>
@@ -24863,7 +24863,7 @@
         <v>1631</v>
       </c>
       <c r="I468" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J468" t="s">
         <v>2245</v>
@@ -24898,7 +24898,7 @@
         <v>1631</v>
       </c>
       <c r="I469" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J469" t="s">
         <v>2246</v>
@@ -25003,7 +25003,7 @@
         <v>1631</v>
       </c>
       <c r="I472" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J472" t="s">
         <v>2248</v>
@@ -25038,7 +25038,7 @@
         <v>1631</v>
       </c>
       <c r="I473" t="s">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="J473" t="s">
         <v>2249</v>
@@ -25178,7 +25178,7 @@
         <v>1631</v>
       </c>
       <c r="I477" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J477" t="s">
         <v>2253</v>
@@ -25283,7 +25283,7 @@
         <v>1631</v>
       </c>
       <c r="I480" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J480" t="s">
         <v>2256</v>
@@ -25636,7 +25636,7 @@
         <v>1631</v>
       </c>
       <c r="I490" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J490" t="s">
         <v>2265</v>
@@ -25671,7 +25671,7 @@
         <v>1631</v>
       </c>
       <c r="I491" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J491" t="s">
         <v>2266</v>
@@ -25706,7 +25706,7 @@
         <v>1631</v>
       </c>
       <c r="I492" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J492" t="s">
         <v>2267</v>
@@ -25741,7 +25741,7 @@
         <v>1631</v>
       </c>
       <c r="I493" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J493" t="s">
         <v>2268</v>
@@ -25776,7 +25776,7 @@
         <v>1631</v>
       </c>
       <c r="I494" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J494" t="s">
         <v>2269</v>
@@ -25811,7 +25811,7 @@
         <v>1631</v>
       </c>
       <c r="I495" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J495" t="s">
         <v>2270</v>
@@ -25916,7 +25916,7 @@
         <v>1631</v>
       </c>
       <c r="I498" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J498" t="s">
         <v>1865</v>
@@ -25986,7 +25986,7 @@
         <v>1631</v>
       </c>
       <c r="I500" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J500" t="s">
         <v>2274</v>
@@ -26056,7 +26056,7 @@
         <v>1631</v>
       </c>
       <c r="I502" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J502" t="s">
         <v>2276</v>
@@ -26091,7 +26091,7 @@
         <v>1631</v>
       </c>
       <c r="I503" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J503" t="s">
         <v>2277</v>
@@ -26161,7 +26161,7 @@
         <v>1631</v>
       </c>
       <c r="I505" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J505" t="s">
         <v>2279</v>
@@ -26307,7 +26307,7 @@
         <v>1631</v>
       </c>
       <c r="I509" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J509" t="s">
         <v>2283</v>
@@ -26342,7 +26342,7 @@
         <v>1631</v>
       </c>
       <c r="I510" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J510" t="s">
         <v>2284</v>
@@ -26377,7 +26377,7 @@
         <v>1631</v>
       </c>
       <c r="I511" t="s">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="J511" t="s">
         <v>2285</v>
@@ -26523,7 +26523,7 @@
         <v>1631</v>
       </c>
       <c r="I515" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J515" t="s">
         <v>2288</v>
@@ -26558,7 +26558,7 @@
         <v>1631</v>
       </c>
       <c r="I516" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J516" t="s">
         <v>2289</v>
@@ -26701,7 +26701,7 @@
         <v>1631</v>
       </c>
       <c r="I520" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J520" t="s">
         <v>2293</v>
@@ -26771,7 +26771,7 @@
         <v>1631</v>
       </c>
       <c r="I522" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J522" t="s">
         <v>2295</v>
@@ -26841,7 +26841,7 @@
         <v>1631</v>
       </c>
       <c r="I524" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J524" t="s">
         <v>2297</v>
@@ -26876,7 +26876,7 @@
         <v>1631</v>
       </c>
       <c r="I525" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J525" t="s">
         <v>2298</v>
@@ -26946,7 +26946,7 @@
         <v>1631</v>
       </c>
       <c r="I527" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J527" t="s">
         <v>2300</v>
@@ -27229,7 +27229,7 @@
         <v>1631</v>
       </c>
       <c r="I535" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J535" t="s">
         <v>2308</v>
@@ -27264,7 +27264,7 @@
         <v>1631</v>
       </c>
       <c r="I536" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J536" t="s">
         <v>2309</v>
@@ -27509,7 +27509,7 @@
         <v>1631</v>
       </c>
       <c r="I543" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J543" t="s">
         <v>2315</v>
@@ -27544,7 +27544,7 @@
         <v>1631</v>
       </c>
       <c r="I544" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J544" t="s">
         <v>2316</v>
@@ -27649,7 +27649,7 @@
         <v>1631</v>
       </c>
       <c r="I547" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J547" t="s">
         <v>2319</v>
@@ -27684,7 +27684,7 @@
         <v>1631</v>
       </c>
       <c r="I548" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J548" t="s">
         <v>2320</v>
@@ -28072,7 +28072,7 @@
         <v>1631</v>
       </c>
       <c r="I559" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J559" t="s">
         <v>2331</v>
@@ -28107,7 +28107,7 @@
         <v>1631</v>
       </c>
       <c r="I560" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J560" t="s">
         <v>2332</v>
@@ -28177,7 +28177,7 @@
         <v>1631</v>
       </c>
       <c r="I562" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J562" t="s">
         <v>2334</v>
@@ -28285,7 +28285,7 @@
         <v>1631</v>
       </c>
       <c r="I565" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J565" t="s">
         <v>2337</v>
@@ -28393,7 +28393,7 @@
         <v>1631</v>
       </c>
       <c r="I568" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J568" t="s">
         <v>2340</v>
@@ -28428,7 +28428,7 @@
         <v>1631</v>
       </c>
       <c r="I569" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J569" t="s">
         <v>2341</v>
@@ -28463,7 +28463,7 @@
         <v>1631</v>
       </c>
       <c r="I570" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J570" t="s">
         <v>2342</v>
@@ -28533,7 +28533,7 @@
         <v>1631</v>
       </c>
       <c r="I572" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J572" t="s">
         <v>2344</v>
@@ -28638,7 +28638,7 @@
         <v>1631</v>
       </c>
       <c r="I575" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J575" t="s">
         <v>2347</v>
@@ -28673,7 +28673,7 @@
         <v>1631</v>
       </c>
       <c r="I576" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J576" t="s">
         <v>2348</v>
@@ -28746,7 +28746,7 @@
         <v>1631</v>
       </c>
       <c r="I578" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J578" t="s">
         <v>2350</v>
@@ -28781,7 +28781,7 @@
         <v>1631</v>
       </c>
       <c r="I579" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J579" t="s">
         <v>2351</v>
@@ -28851,7 +28851,7 @@
         <v>1631</v>
       </c>
       <c r="I581" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J581" t="s">
         <v>2353</v>
@@ -28886,7 +28886,7 @@
         <v>1631</v>
       </c>
       <c r="I582" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J582" t="s">
         <v>2354</v>
@@ -28921,7 +28921,7 @@
         <v>1631</v>
       </c>
       <c r="I583" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J583" t="s">
         <v>2355</v>
@@ -28956,7 +28956,7 @@
         <v>1631</v>
       </c>
       <c r="I584" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J584" t="s">
         <v>2356</v>
@@ -28994,7 +28994,7 @@
         <v>1658</v>
       </c>
       <c r="I585" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J585" t="s">
         <v>2357</v>
@@ -29064,7 +29064,7 @@
         <v>1631</v>
       </c>
       <c r="I587" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J587" t="s">
         <v>2359</v>
@@ -29175,7 +29175,7 @@
         <v>1631</v>
       </c>
       <c r="I590" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J590" t="s">
         <v>2362</v>
@@ -29210,7 +29210,7 @@
         <v>1631</v>
       </c>
       <c r="I591" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J591" t="s">
         <v>2363</v>
@@ -29245,7 +29245,7 @@
         <v>1631</v>
       </c>
       <c r="I592" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J592" t="s">
         <v>2364</v>
@@ -29385,7 +29385,7 @@
         <v>1631</v>
       </c>
       <c r="I596" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J596" t="s">
         <v>2368</v>
@@ -29420,7 +29420,7 @@
         <v>1631</v>
       </c>
       <c r="I597" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J597" t="s">
         <v>2369</v>
@@ -29455,7 +29455,7 @@
         <v>1631</v>
       </c>
       <c r="I598" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J598" t="s">
         <v>2370</v>
@@ -29490,7 +29490,7 @@
         <v>1631</v>
       </c>
       <c r="I599" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J599" t="s">
         <v>2371</v>
@@ -29525,7 +29525,7 @@
         <v>1631</v>
       </c>
       <c r="I600" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J600" t="s">
         <v>2372</v>
@@ -29560,7 +29560,7 @@
         <v>1631</v>
       </c>
       <c r="I601" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J601" t="s">
         <v>2373</v>
@@ -29595,7 +29595,7 @@
         <v>1631</v>
       </c>
       <c r="I602" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J602" t="s">
         <v>2374</v>
@@ -29630,7 +29630,7 @@
         <v>1631</v>
       </c>
       <c r="I603" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J603" t="s">
         <v>2375</v>
@@ -29700,7 +29700,7 @@
         <v>1631</v>
       </c>
       <c r="I605" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J605" t="s">
         <v>2377</v>
@@ -29735,7 +29735,7 @@
         <v>1631</v>
       </c>
       <c r="I606" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J606" t="s">
         <v>2378</v>
@@ -29805,7 +29805,7 @@
         <v>1631</v>
       </c>
       <c r="I608" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J608" t="s">
         <v>2380</v>
@@ -29840,7 +29840,7 @@
         <v>1631</v>
       </c>
       <c r="I609" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J609" t="s">
         <v>2381</v>
@@ -29875,7 +29875,7 @@
         <v>1631</v>
       </c>
       <c r="I610" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J610" t="s">
         <v>2382</v>
@@ -29913,7 +29913,7 @@
         <v>1657</v>
       </c>
       <c r="I611" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J611" t="s">
         <v>2383</v>
@@ -30021,7 +30021,7 @@
         <v>1631</v>
       </c>
       <c r="I614" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J614" t="s">
         <v>2386</v>
@@ -30056,7 +30056,7 @@
         <v>1631</v>
       </c>
       <c r="I615" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J615" t="s">
         <v>2387</v>
@@ -30091,7 +30091,7 @@
         <v>1631</v>
       </c>
       <c r="I616" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J616" t="s">
         <v>2388</v>
@@ -30161,7 +30161,7 @@
         <v>1631</v>
       </c>
       <c r="I618" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J618" t="s">
         <v>2390</v>
@@ -30196,7 +30196,7 @@
         <v>1631</v>
       </c>
       <c r="I619" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J619" t="s">
         <v>1890</v>
@@ -30234,7 +30234,7 @@
         <v>1657</v>
       </c>
       <c r="I620" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J620" t="s">
         <v>2391</v>
@@ -30269,7 +30269,7 @@
         <v>1631</v>
       </c>
       <c r="I621" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J621" t="s">
         <v>2392</v>
@@ -30342,7 +30342,7 @@
         <v>1631</v>
       </c>
       <c r="I623" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J623" t="s">
         <v>2394</v>
@@ -30412,7 +30412,7 @@
         <v>1631</v>
       </c>
       <c r="I625" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J625" t="s">
         <v>2396</v>
@@ -30447,7 +30447,7 @@
         <v>1631</v>
       </c>
       <c r="I626" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J626" t="s">
         <v>2397</v>
@@ -30482,7 +30482,7 @@
         <v>1631</v>
       </c>
       <c r="I627" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J627" t="s">
         <v>2398</v>
@@ -30552,7 +30552,7 @@
         <v>1631</v>
       </c>
       <c r="I629" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J629" t="s">
         <v>2399</v>
@@ -30590,7 +30590,7 @@
         <v>1657</v>
       </c>
       <c r="I630" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J630" t="s">
         <v>2400</v>
@@ -30660,7 +30660,7 @@
         <v>1631</v>
       </c>
       <c r="I632" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J632" t="s">
         <v>2402</v>
@@ -30695,7 +30695,7 @@
         <v>1631</v>
       </c>
       <c r="I633" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J633" t="s">
         <v>2403</v>
@@ -30730,7 +30730,7 @@
         <v>1631</v>
       </c>
       <c r="I634" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J634" t="s">
         <v>2404</v>
@@ -30765,7 +30765,7 @@
         <v>1631</v>
       </c>
       <c r="I635" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J635" t="s">
         <v>2405</v>
@@ -30803,7 +30803,7 @@
         <v>1662</v>
       </c>
       <c r="I636" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J636" t="s">
         <v>2406</v>
@@ -30838,7 +30838,7 @@
         <v>1631</v>
       </c>
       <c r="I637" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J637" t="s">
         <v>2407</v>
@@ -30908,7 +30908,7 @@
         <v>1631</v>
       </c>
       <c r="I639" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J639" t="s">
         <v>2125</v>
@@ -31051,7 +31051,7 @@
         <v>1649</v>
       </c>
       <c r="I643" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J643" t="s">
         <v>2412</v>
@@ -31086,7 +31086,7 @@
         <v>1631</v>
       </c>
       <c r="I644" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J644" t="s">
         <v>2413</v>
@@ -31579,7 +31579,7 @@
         <v>1631</v>
       </c>
       <c r="I658" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J658" t="s">
         <v>2426</v>
@@ -31614,7 +31614,7 @@
         <v>1631</v>
       </c>
       <c r="I659" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J659" t="s">
         <v>2427</v>
@@ -31649,7 +31649,7 @@
         <v>1631</v>
       </c>
       <c r="I660" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J660" t="s">
         <v>2428</v>
@@ -31687,7 +31687,7 @@
         <v>1663</v>
       </c>
       <c r="I661" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J661" t="s">
         <v>2429</v>
@@ -31725,7 +31725,7 @@
         <v>1664</v>
       </c>
       <c r="I662" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J662" t="s">
         <v>2430</v>
@@ -31865,7 +31865,7 @@
         <v>1631</v>
       </c>
       <c r="I666" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J666" t="s">
         <v>2433</v>
@@ -31900,7 +31900,7 @@
         <v>1631</v>
       </c>
       <c r="I667" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J667" t="s">
         <v>2434</v>
@@ -31970,7 +31970,7 @@
         <v>1631</v>
       </c>
       <c r="I669" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J669" t="s">
         <v>2436</v>
@@ -32110,7 +32110,7 @@
         <v>1631</v>
       </c>
       <c r="I673" t="s">
-        <v>1755</v>
+        <v>1712</v>
       </c>
       <c r="J673" t="s">
         <v>2440</v>
@@ -32159,7 +32159,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B675" t="s">
         <v>716</v>
@@ -32180,7 +32180,7 @@
         <v>1631</v>
       </c>
       <c r="I675" t="s">
-        <v>1668</v>
+        <v>1795</v>
       </c>
       <c r="J675" t="s">
         <v>2442</v>
@@ -32194,7 +32194,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B676" t="s">
         <v>717</v>
@@ -32215,7 +32215,7 @@
         <v>1631</v>
       </c>
       <c r="I676" t="s">
-        <v>1668</v>
+        <v>1795</v>
       </c>
       <c r="J676" t="s">
         <v>2443</v>
@@ -32387,7 +32387,7 @@
         <v>1631</v>
       </c>
       <c r="I681" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J681" t="s">
         <v>2448</v>
@@ -32419,7 +32419,7 @@
         <v>1631</v>
       </c>
       <c r="I682" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J682" t="s">
         <v>2449</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-24 12:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5125,135 +5125,135 @@
     <t>LUIZ FRANCISCO PERALTA BRAGA</t>
   </si>
   <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA,CARLOS FELIPE DA GRAÇA SILVA,ERIKA CANTANHEDE WUILLAUME,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA</t>
+  </si>
+  <si>
+    <t>GLAUCO CASTILHO DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,PATRÍCIA FINAMORE ARAÚJO,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>MANOELA DE MORAES SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI</t>
+  </si>
+  <si>
+    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>NIVANA DANIELLE SILVA COSTA</t>
+  </si>
+  <si>
+    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>ANA LÍCIA SOUZA E SILVA</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
+    <t>SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>RAQUEL SILVA FERNANDES LYRA</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA</t>
+  </si>
+  <si>
+    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
     <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA,CARLOS FELIPE DA GRAÇA SILVA,ERIKA CANTANHEDE WUILLAUME,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA</t>
-  </si>
-  <si>
-    <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,PATRÍCIA FINAMORE ARAÚJO,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>MANOELA DE MORAES SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI</t>
-  </si>
-  <si>
-    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>NIVANA DANIELLE SILVA COSTA</t>
-  </si>
-  <si>
-    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>ANA LÍCIA SOUZA E SILVA</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>RAQUEL SILVA FERNANDES LYRA</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA</t>
-  </si>
-  <si>
-    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
   </si>
   <si>
@@ -8011,13 +8011,13 @@
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA QUÍMICA,BIOLOGIA</t>
+    <t>RECURSOS HÍDRICOS,BIOLOGIA</t>
   </si>
   <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,SAÚDE,SAÚDE MENTAL,ECONOMIA,URBANISMO,PSICOLOGIA,ASSISTÊNCIA SOCIAL,ORÇAMENTO</t>
+    <t>ECONOMICIDADE CONTÁBIL,SAÚDE,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,MOBILIDADE E TRANSPORTE,URBANISMO,PSICOLOGIA,SAÚDE MENTAL,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -11265,7 +11265,7 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B83" t="s">
         <v>125</v>
@@ -11289,7 +11289,7 @@
         <v>1505</v>
       </c>
       <c r="I83" t="s">
-        <v>1700</v>
+        <v>1662</v>
       </c>
       <c r="J83" t="s">
         <v>1873</v>
@@ -11677,7 +11677,7 @@
         <v>1633</v>
       </c>
       <c r="I94" t="s">
-        <v>1703</v>
+        <v>1662</v>
       </c>
       <c r="J94" t="s">
         <v>1876</v>
@@ -11785,7 +11785,7 @@
         <v>1465</v>
       </c>
       <c r="I97" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
       <c r="J97" t="s">
         <v>1886</v>
@@ -11820,7 +11820,7 @@
         <v>1626</v>
       </c>
       <c r="I98" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J98" t="s">
         <v>1887</v>
@@ -11925,7 +11925,7 @@
         <v>1626</v>
       </c>
       <c r="I101" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="J101" t="s">
         <v>1890</v>
@@ -11995,7 +11995,7 @@
         <v>1626</v>
       </c>
       <c r="I103" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J103" t="s">
         <v>1892</v>
@@ -12100,7 +12100,7 @@
         <v>1626</v>
       </c>
       <c r="I106" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
       <c r="J106" t="s">
         <v>1895</v>
@@ -12348,7 +12348,7 @@
         <v>1626</v>
       </c>
       <c r="I113" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="J113" t="s">
         <v>1902</v>
@@ -12418,7 +12418,7 @@
         <v>1626</v>
       </c>
       <c r="I115" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J115" t="s">
         <v>1904</v>
@@ -12453,7 +12453,7 @@
         <v>1626</v>
       </c>
       <c r="I116" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="J116" t="s">
         <v>1905</v>
@@ -12488,7 +12488,7 @@
         <v>1626</v>
       </c>
       <c r="I117" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="J117" t="s">
         <v>1906</v>
@@ -12523,7 +12523,7 @@
         <v>1626</v>
       </c>
       <c r="I118" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="J118" t="s">
         <v>1907</v>
@@ -12558,7 +12558,7 @@
         <v>1626</v>
       </c>
       <c r="I119" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J119" t="s">
         <v>1908</v>
@@ -12631,7 +12631,7 @@
         <v>1487</v>
       </c>
       <c r="I121" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J121" t="s">
         <v>1910</v>
@@ -12701,7 +12701,7 @@
         <v>1626</v>
       </c>
       <c r="I123" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J123" t="s">
         <v>1912</v>
@@ -12736,7 +12736,7 @@
         <v>1626</v>
       </c>
       <c r="I124" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J124" t="s">
         <v>1913</v>
@@ -12771,7 +12771,7 @@
         <v>1626</v>
       </c>
       <c r="I125" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J125" t="s">
         <v>1914</v>
@@ -12876,7 +12876,7 @@
         <v>1626</v>
       </c>
       <c r="I128" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="J128" t="s">
         <v>1917</v>
@@ -13089,7 +13089,7 @@
         <v>1626</v>
       </c>
       <c r="I134" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="J134" t="s">
         <v>1923</v>
@@ -13159,7 +13159,7 @@
         <v>1626</v>
       </c>
       <c r="I136" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J136" t="s">
         <v>1925</v>
@@ -13194,7 +13194,7 @@
         <v>1626</v>
       </c>
       <c r="I137" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="J137" t="s">
         <v>1926</v>
@@ -13264,7 +13264,7 @@
         <v>1626</v>
       </c>
       <c r="I139" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J139" t="s">
         <v>1928</v>
@@ -13302,7 +13302,7 @@
         <v>1634</v>
       </c>
       <c r="I140" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J140" t="s">
         <v>1929</v>
@@ -13442,7 +13442,7 @@
         <v>1626</v>
       </c>
       <c r="I144" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J144" t="s">
         <v>1933</v>
@@ -13585,7 +13585,7 @@
         <v>1626</v>
       </c>
       <c r="I148" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J148" t="s">
         <v>1937</v>
@@ -13655,7 +13655,7 @@
         <v>1626</v>
       </c>
       <c r="I150" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J150" t="s">
         <v>1939</v>
@@ -13865,7 +13865,7 @@
         <v>1626</v>
       </c>
       <c r="I156" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J156" t="s">
         <v>1945</v>
@@ -14005,7 +14005,7 @@
         <v>1626</v>
       </c>
       <c r="I160" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J160" t="s">
         <v>1949</v>
@@ -14040,7 +14040,7 @@
         <v>1626</v>
       </c>
       <c r="I161" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J161" t="s">
         <v>1949</v>
@@ -14180,7 +14180,7 @@
         <v>1626</v>
       </c>
       <c r="I165" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J165" t="s">
         <v>1951</v>
@@ -14320,7 +14320,7 @@
         <v>1626</v>
       </c>
       <c r="I169" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J169" t="s">
         <v>1955</v>
@@ -14428,7 +14428,7 @@
         <v>1636</v>
       </c>
       <c r="I172" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J172" t="s">
         <v>1958</v>
@@ -14466,7 +14466,7 @@
         <v>1636</v>
       </c>
       <c r="I173" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J173" t="s">
         <v>1958</v>
@@ -14889,7 +14889,7 @@
         <v>1637</v>
       </c>
       <c r="I185" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J185" t="s">
         <v>1970</v>
@@ -14994,7 +14994,7 @@
         <v>1626</v>
       </c>
       <c r="I188" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J188" t="s">
         <v>1973</v>
@@ -15169,7 +15169,7 @@
         <v>1626</v>
       </c>
       <c r="I193" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J193" t="s">
         <v>1978</v>
@@ -15554,7 +15554,7 @@
         <v>1626</v>
       </c>
       <c r="I204" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J204" t="s">
         <v>1987</v>
@@ -15624,7 +15624,7 @@
         <v>1626</v>
       </c>
       <c r="I206" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J206" t="s">
         <v>1989</v>
@@ -15869,7 +15869,7 @@
         <v>1626</v>
       </c>
       <c r="I213" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J213" t="s">
         <v>1996</v>
@@ -15939,7 +15939,7 @@
         <v>1626</v>
       </c>
       <c r="I215" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J215" t="s">
         <v>1998</v>
@@ -16324,7 +16324,7 @@
         <v>1626</v>
       </c>
       <c r="I226" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J226" t="s">
         <v>2009</v>
@@ -16429,7 +16429,7 @@
         <v>1626</v>
       </c>
       <c r="I229" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J229" t="s">
         <v>2012</v>
@@ -16464,7 +16464,7 @@
         <v>1626</v>
       </c>
       <c r="I230" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J230" t="s">
         <v>2013</v>
@@ -16712,7 +16712,7 @@
         <v>1626</v>
       </c>
       <c r="I237" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="J237" t="s">
         <v>2020</v>
@@ -16747,7 +16747,7 @@
         <v>1626</v>
       </c>
       <c r="I238" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J238" t="s">
         <v>2021</v>
@@ -16887,7 +16887,7 @@
         <v>1626</v>
       </c>
       <c r="I242" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J242" t="s">
         <v>2024</v>
@@ -16957,7 +16957,7 @@
         <v>1626</v>
       </c>
       <c r="I244" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J244" t="s">
         <v>2026</v>
@@ -17027,7 +17027,7 @@
         <v>1626</v>
       </c>
       <c r="I246" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J246" t="s">
         <v>2028</v>
@@ -17167,7 +17167,7 @@
         <v>1626</v>
       </c>
       <c r="I250" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
       <c r="J250" t="s">
         <v>2031</v>
@@ -17307,7 +17307,7 @@
         <v>1626</v>
       </c>
       <c r="I254" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="J254" t="s">
         <v>2035</v>
@@ -17625,7 +17625,7 @@
         <v>1626</v>
       </c>
       <c r="I263" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J263" t="s">
         <v>2042</v>
@@ -17730,7 +17730,7 @@
         <v>1626</v>
       </c>
       <c r="I266" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J266" t="s">
         <v>2045</v>
@@ -17800,7 +17800,7 @@
         <v>1626</v>
       </c>
       <c r="I268" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J268" t="s">
         <v>2047</v>
@@ -17905,7 +17905,7 @@
         <v>1626</v>
       </c>
       <c r="I271" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J271" t="s">
         <v>2050</v>
@@ -17975,7 +17975,7 @@
         <v>1626</v>
       </c>
       <c r="I273" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J273" t="s">
         <v>2052</v>
@@ -18115,7 +18115,7 @@
         <v>1626</v>
       </c>
       <c r="I277" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J277" t="s">
         <v>2056</v>
@@ -18220,7 +18220,7 @@
         <v>1626</v>
       </c>
       <c r="I280" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J280" t="s">
         <v>2059</v>
@@ -18255,7 +18255,7 @@
         <v>1626</v>
       </c>
       <c r="I281" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J281" t="s">
         <v>2060</v>
@@ -18325,7 +18325,7 @@
         <v>1626</v>
       </c>
       <c r="I283" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J283" t="s">
         <v>2062</v>
@@ -18395,7 +18395,7 @@
         <v>1626</v>
       </c>
       <c r="I285" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J285" t="s">
         <v>2064</v>
@@ -18500,7 +18500,7 @@
         <v>1626</v>
       </c>
       <c r="I288" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="J288" t="s">
         <v>2067</v>
@@ -18675,7 +18675,7 @@
         <v>1626</v>
       </c>
       <c r="I293" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J293" t="s">
         <v>2072</v>
@@ -18745,7 +18745,7 @@
         <v>1626</v>
       </c>
       <c r="I295" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="J295" t="s">
         <v>2074</v>
@@ -18780,7 +18780,7 @@
         <v>1626</v>
       </c>
       <c r="I296" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="J296" t="s">
         <v>2075</v>
@@ -18815,7 +18815,7 @@
         <v>1626</v>
       </c>
       <c r="I297" t="s">
-        <v>1703</v>
+        <v>1745</v>
       </c>
       <c r="J297" t="s">
         <v>2076</v>
@@ -18990,7 +18990,7 @@
         <v>1626</v>
       </c>
       <c r="I302" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J302" t="s">
         <v>2081</v>
@@ -19095,7 +19095,7 @@
         <v>1626</v>
       </c>
       <c r="I305" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J305" t="s">
         <v>2084</v>
@@ -19165,7 +19165,7 @@
         <v>1626</v>
       </c>
       <c r="I307" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J307" t="s">
         <v>2086</v>
@@ -19308,7 +19308,7 @@
         <v>1626</v>
       </c>
       <c r="I311" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J311" t="s">
         <v>2090</v>
@@ -19343,7 +19343,7 @@
         <v>1626</v>
       </c>
       <c r="I312" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J312" t="s">
         <v>2091</v>
@@ -19378,7 +19378,7 @@
         <v>1626</v>
       </c>
       <c r="I313" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J313" t="s">
         <v>2092</v>
@@ -19868,7 +19868,7 @@
         <v>1626</v>
       </c>
       <c r="I327" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J327" t="s">
         <v>2106</v>
@@ -19903,7 +19903,7 @@
         <v>1626</v>
       </c>
       <c r="I328" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J328" t="s">
         <v>2107</v>
@@ -20393,7 +20393,7 @@
         <v>1626</v>
       </c>
       <c r="I342" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J342" t="s">
         <v>1876</v>
@@ -20536,7 +20536,7 @@
         <v>1626</v>
       </c>
       <c r="I346" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J346" t="s">
         <v>2122</v>
@@ -20819,7 +20819,7 @@
         <v>1626</v>
       </c>
       <c r="I354" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J354" t="s">
         <v>2130</v>
@@ -20889,7 +20889,7 @@
         <v>1630</v>
       </c>
       <c r="I356" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J356" t="s">
         <v>2132</v>
@@ -20924,7 +20924,7 @@
         <v>1626</v>
       </c>
       <c r="I357" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J357" t="s">
         <v>2133</v>
@@ -20959,7 +20959,7 @@
         <v>1626</v>
       </c>
       <c r="I358" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J358" t="s">
         <v>2062</v>
@@ -20994,7 +20994,7 @@
         <v>1626</v>
       </c>
       <c r="I359" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J359" t="s">
         <v>2134</v>
@@ -21204,7 +21204,7 @@
         <v>1626</v>
       </c>
       <c r="I365" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J365" t="s">
         <v>2140</v>
@@ -21274,7 +21274,7 @@
         <v>1626</v>
       </c>
       <c r="I367" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J367" t="s">
         <v>2142</v>
@@ -21417,7 +21417,7 @@
         <v>1626</v>
       </c>
       <c r="I371" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J371" t="s">
         <v>2146</v>
@@ -21452,7 +21452,7 @@
         <v>1626</v>
       </c>
       <c r="I372" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J372" t="s">
         <v>2147</v>
@@ -21557,7 +21557,7 @@
         <v>1626</v>
       </c>
       <c r="I375" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J375" t="s">
         <v>2150</v>
@@ -21627,7 +21627,7 @@
         <v>1626</v>
       </c>
       <c r="I377" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J377" t="s">
         <v>2152</v>
@@ -21732,7 +21732,7 @@
         <v>1626</v>
       </c>
       <c r="I380" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J380" t="s">
         <v>2155</v>
@@ -21977,7 +21977,7 @@
         <v>1626</v>
       </c>
       <c r="I387" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J387" t="s">
         <v>2162</v>
@@ -22117,7 +22117,7 @@
         <v>1626</v>
       </c>
       <c r="I391" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J391" t="s">
         <v>2165</v>
@@ -22152,7 +22152,7 @@
         <v>1626</v>
       </c>
       <c r="I392" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J392" t="s">
         <v>2166</v>
@@ -22187,7 +22187,7 @@
         <v>1626</v>
       </c>
       <c r="I393" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J393" t="s">
         <v>2167</v>
@@ -22222,7 +22222,7 @@
         <v>1626</v>
       </c>
       <c r="I394" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J394" t="s">
         <v>1949</v>
@@ -22327,7 +22327,7 @@
         <v>1626</v>
       </c>
       <c r="I397" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J397" t="s">
         <v>2170</v>
@@ -22362,7 +22362,7 @@
         <v>1626</v>
       </c>
       <c r="I398" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J398" t="s">
         <v>2171</v>
@@ -22432,7 +22432,7 @@
         <v>1626</v>
       </c>
       <c r="I400" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J400" t="s">
         <v>2173</v>
@@ -22715,7 +22715,7 @@
         <v>1626</v>
       </c>
       <c r="I408" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J408" t="s">
         <v>2181</v>
@@ -22928,7 +22928,7 @@
         <v>1626</v>
       </c>
       <c r="I414" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J414" t="s">
         <v>2187</v>
@@ -23109,7 +23109,7 @@
         <v>1626</v>
       </c>
       <c r="I419" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J419" t="s">
         <v>2192</v>
@@ -23144,7 +23144,7 @@
         <v>1626</v>
       </c>
       <c r="I420" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J420" t="s">
         <v>2193</v>
@@ -23249,7 +23249,7 @@
         <v>1626</v>
       </c>
       <c r="I423" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J423" t="s">
         <v>2196</v>
@@ -23354,7 +23354,7 @@
         <v>1626</v>
       </c>
       <c r="I426" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J426" t="s">
         <v>2199</v>
@@ -23389,7 +23389,7 @@
         <v>1626</v>
       </c>
       <c r="I427" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J427" t="s">
         <v>2200</v>
@@ -23424,7 +23424,7 @@
         <v>1626</v>
       </c>
       <c r="I428" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J428" t="s">
         <v>2201</v>
@@ -23529,7 +23529,7 @@
         <v>1626</v>
       </c>
       <c r="I431" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J431" t="s">
         <v>2204</v>
@@ -23599,7 +23599,7 @@
         <v>1626</v>
       </c>
       <c r="I433" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J433" t="s">
         <v>2206</v>
@@ -23634,7 +23634,7 @@
         <v>1626</v>
       </c>
       <c r="I434" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J434" t="s">
         <v>2207</v>
@@ -23669,7 +23669,7 @@
         <v>1626</v>
       </c>
       <c r="I435" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J435" t="s">
         <v>2208</v>
@@ -23704,7 +23704,7 @@
         <v>1626</v>
       </c>
       <c r="I436" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J436" t="s">
         <v>2209</v>
@@ -23844,7 +23844,7 @@
         <v>1626</v>
       </c>
       <c r="I440" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J440" t="s">
         <v>2213</v>
@@ -23917,7 +23917,7 @@
         <v>1641</v>
       </c>
       <c r="I442" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J442" t="s">
         <v>2215</v>
@@ -23987,7 +23987,7 @@
         <v>1626</v>
       </c>
       <c r="I444" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J444" t="s">
         <v>2217</v>
@@ -24022,7 +24022,7 @@
         <v>1626</v>
       </c>
       <c r="I445" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J445" t="s">
         <v>2218</v>
@@ -24127,7 +24127,7 @@
         <v>1626</v>
       </c>
       <c r="I448" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J448" t="s">
         <v>2221</v>
@@ -24232,7 +24232,7 @@
         <v>1626</v>
       </c>
       <c r="I451" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J451" t="s">
         <v>2224</v>
@@ -24302,7 +24302,7 @@
         <v>1626</v>
       </c>
       <c r="I453" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J453" t="s">
         <v>2226</v>
@@ -24337,7 +24337,7 @@
         <v>1626</v>
       </c>
       <c r="I454" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J454" t="s">
         <v>2227</v>
@@ -24553,7 +24553,7 @@
         <v>1626</v>
       </c>
       <c r="I460" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J460" t="s">
         <v>2233</v>
@@ -24588,7 +24588,7 @@
         <v>1626</v>
       </c>
       <c r="I461" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J461" t="s">
         <v>2234</v>
@@ -24693,7 +24693,7 @@
         <v>1626</v>
       </c>
       <c r="I464" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J464" t="s">
         <v>2236</v>
@@ -24868,7 +24868,7 @@
         <v>1626</v>
       </c>
       <c r="I469" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J469" t="s">
         <v>2241</v>
@@ -25326,7 +25326,7 @@
         <v>1626</v>
       </c>
       <c r="I482" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J482" t="s">
         <v>2253</v>
@@ -25361,7 +25361,7 @@
         <v>1626</v>
       </c>
       <c r="I483" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J483" t="s">
         <v>2254</v>
@@ -25396,7 +25396,7 @@
         <v>1626</v>
       </c>
       <c r="I484" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J484" t="s">
         <v>2255</v>
@@ -25431,7 +25431,7 @@
         <v>1626</v>
       </c>
       <c r="I485" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J485" t="s">
         <v>2256</v>
@@ -25466,7 +25466,7 @@
         <v>1626</v>
       </c>
       <c r="I486" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J486" t="s">
         <v>2257</v>
@@ -25501,7 +25501,7 @@
         <v>1626</v>
       </c>
       <c r="I487" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J487" t="s">
         <v>2258</v>
@@ -25606,7 +25606,7 @@
         <v>1626</v>
       </c>
       <c r="I490" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J490" t="s">
         <v>1861</v>
@@ -25676,7 +25676,7 @@
         <v>1626</v>
       </c>
       <c r="I492" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J492" t="s">
         <v>2262</v>
@@ -25746,7 +25746,7 @@
         <v>1626</v>
       </c>
       <c r="I494" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J494" t="s">
         <v>2264</v>
@@ -25781,7 +25781,7 @@
         <v>1626</v>
       </c>
       <c r="I495" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J495" t="s">
         <v>2265</v>
@@ -25851,7 +25851,7 @@
         <v>1626</v>
       </c>
       <c r="I497" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J497" t="s">
         <v>2267</v>
@@ -25997,7 +25997,7 @@
         <v>1626</v>
       </c>
       <c r="I501" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J501" t="s">
         <v>2271</v>
@@ -26032,7 +26032,7 @@
         <v>1626</v>
       </c>
       <c r="I502" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J502" t="s">
         <v>2272</v>
@@ -26067,7 +26067,7 @@
         <v>1626</v>
       </c>
       <c r="I503" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="J503" t="s">
         <v>2273</v>
@@ -26213,7 +26213,7 @@
         <v>1626</v>
       </c>
       <c r="I507" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J507" t="s">
         <v>2276</v>
@@ -26248,7 +26248,7 @@
         <v>1626</v>
       </c>
       <c r="I508" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J508" t="s">
         <v>2277</v>
@@ -26391,7 +26391,7 @@
         <v>1626</v>
       </c>
       <c r="I512" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J512" t="s">
         <v>2281</v>
@@ -26461,7 +26461,7 @@
         <v>1626</v>
       </c>
       <c r="I514" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J514" t="s">
         <v>2283</v>
@@ -26531,7 +26531,7 @@
         <v>1626</v>
       </c>
       <c r="I516" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J516" t="s">
         <v>2285</v>
@@ -26566,7 +26566,7 @@
         <v>1626</v>
       </c>
       <c r="I517" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J517" t="s">
         <v>2286</v>
@@ -26636,7 +26636,7 @@
         <v>1626</v>
       </c>
       <c r="I519" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J519" t="s">
         <v>2288</v>
@@ -26919,7 +26919,7 @@
         <v>1626</v>
       </c>
       <c r="I527" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J527" t="s">
         <v>2296</v>
@@ -26954,7 +26954,7 @@
         <v>1626</v>
       </c>
       <c r="I528" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J528" t="s">
         <v>2297</v>
@@ -27199,7 +27199,7 @@
         <v>1626</v>
       </c>
       <c r="I535" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J535" t="s">
         <v>2303</v>
@@ -27234,7 +27234,7 @@
         <v>1626</v>
       </c>
       <c r="I536" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J536" t="s">
         <v>2304</v>
@@ -27339,7 +27339,7 @@
         <v>1626</v>
       </c>
       <c r="I539" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J539" t="s">
         <v>2307</v>
@@ -27374,7 +27374,7 @@
         <v>1626</v>
       </c>
       <c r="I540" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J540" t="s">
         <v>2308</v>
@@ -27762,7 +27762,7 @@
         <v>1626</v>
       </c>
       <c r="I551" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J551" t="s">
         <v>2319</v>
@@ -27797,7 +27797,7 @@
         <v>1626</v>
       </c>
       <c r="I552" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J552" t="s">
         <v>2320</v>
@@ -27867,7 +27867,7 @@
         <v>1626</v>
       </c>
       <c r="I554" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J554" t="s">
         <v>2322</v>
@@ -27975,7 +27975,7 @@
         <v>1626</v>
       </c>
       <c r="I557" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J557" t="s">
         <v>2325</v>
@@ -28083,7 +28083,7 @@
         <v>1626</v>
       </c>
       <c r="I560" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J560" t="s">
         <v>2328</v>
@@ -28118,7 +28118,7 @@
         <v>1626</v>
       </c>
       <c r="I561" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J561" t="s">
         <v>2329</v>
@@ -28153,7 +28153,7 @@
         <v>1626</v>
       </c>
       <c r="I562" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J562" t="s">
         <v>2330</v>
@@ -28223,7 +28223,7 @@
         <v>1626</v>
       </c>
       <c r="I564" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J564" t="s">
         <v>2332</v>
@@ -28328,7 +28328,7 @@
         <v>1626</v>
       </c>
       <c r="I567" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J567" t="s">
         <v>2335</v>
@@ -28363,7 +28363,7 @@
         <v>1626</v>
       </c>
       <c r="I568" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J568" t="s">
         <v>2336</v>
@@ -28436,7 +28436,7 @@
         <v>1626</v>
       </c>
       <c r="I570" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J570" t="s">
         <v>2338</v>
@@ -28471,7 +28471,7 @@
         <v>1626</v>
       </c>
       <c r="I571" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J571" t="s">
         <v>2339</v>
@@ -28541,7 +28541,7 @@
         <v>1626</v>
       </c>
       <c r="I573" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J573" t="s">
         <v>2341</v>
@@ -28576,7 +28576,7 @@
         <v>1626</v>
       </c>
       <c r="I574" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J574" t="s">
         <v>2342</v>
@@ -28611,7 +28611,7 @@
         <v>1626</v>
       </c>
       <c r="I575" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J575" t="s">
         <v>2343</v>
@@ -28646,7 +28646,7 @@
         <v>1626</v>
       </c>
       <c r="I576" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J576" t="s">
         <v>2344</v>
@@ -28684,7 +28684,7 @@
         <v>1651</v>
       </c>
       <c r="I577" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="J577" t="s">
         <v>2345</v>
@@ -28754,7 +28754,7 @@
         <v>1626</v>
       </c>
       <c r="I579" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J579" t="s">
         <v>2347</v>
@@ -28865,7 +28865,7 @@
         <v>1626</v>
       </c>
       <c r="I582" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J582" t="s">
         <v>2350</v>
@@ -28900,7 +28900,7 @@
         <v>1626</v>
       </c>
       <c r="I583" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J583" t="s">
         <v>2351</v>
@@ -28935,7 +28935,7 @@
         <v>1626</v>
       </c>
       <c r="I584" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J584" t="s">
         <v>2352</v>
@@ -29075,7 +29075,7 @@
         <v>1626</v>
       </c>
       <c r="I588" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J588" t="s">
         <v>2356</v>
@@ -29110,7 +29110,7 @@
         <v>1626</v>
       </c>
       <c r="I589" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J589" t="s">
         <v>2357</v>
@@ -29180,7 +29180,7 @@
         <v>1626</v>
       </c>
       <c r="I591" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J591" t="s">
         <v>2359</v>
@@ -29215,7 +29215,7 @@
         <v>1626</v>
       </c>
       <c r="I592" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J592" t="s">
         <v>2360</v>
@@ -29250,7 +29250,7 @@
         <v>1626</v>
       </c>
       <c r="I593" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J593" t="s">
         <v>2361</v>
@@ -29285,7 +29285,7 @@
         <v>1626</v>
       </c>
       <c r="I594" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J594" t="s">
         <v>2362</v>
@@ -29355,7 +29355,7 @@
         <v>1626</v>
       </c>
       <c r="I596" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J596" t="s">
         <v>2364</v>
@@ -29390,7 +29390,7 @@
         <v>1626</v>
       </c>
       <c r="I597" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J597" t="s">
         <v>2365</v>
@@ -29460,7 +29460,7 @@
         <v>1626</v>
       </c>
       <c r="I599" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J599" t="s">
         <v>2367</v>
@@ -29495,7 +29495,7 @@
         <v>1626</v>
       </c>
       <c r="I600" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J600" t="s">
         <v>2368</v>
@@ -29530,7 +29530,7 @@
         <v>1626</v>
       </c>
       <c r="I601" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J601" t="s">
         <v>2369</v>
@@ -29568,7 +29568,7 @@
         <v>1650</v>
       </c>
       <c r="I602" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J602" t="s">
         <v>2370</v>
@@ -29676,7 +29676,7 @@
         <v>1626</v>
       </c>
       <c r="I605" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J605" t="s">
         <v>2373</v>
@@ -29746,7 +29746,7 @@
         <v>1626</v>
       </c>
       <c r="I607" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J607" t="s">
         <v>2375</v>
@@ -29816,7 +29816,7 @@
         <v>1626</v>
       </c>
       <c r="I609" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J609" t="s">
         <v>2377</v>
@@ -29924,7 +29924,7 @@
         <v>1626</v>
       </c>
       <c r="I612" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J612" t="s">
         <v>2379</v>
@@ -29997,7 +29997,7 @@
         <v>1626</v>
       </c>
       <c r="I614" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J614" t="s">
         <v>2381</v>
@@ -30067,7 +30067,7 @@
         <v>1626</v>
       </c>
       <c r="I616" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J616" t="s">
         <v>2383</v>
@@ -30102,7 +30102,7 @@
         <v>1626</v>
       </c>
       <c r="I617" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J617" t="s">
         <v>2384</v>
@@ -30137,7 +30137,7 @@
         <v>1626</v>
       </c>
       <c r="I618" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J618" t="s">
         <v>2385</v>
@@ -30315,7 +30315,7 @@
         <v>1626</v>
       </c>
       <c r="I623" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J623" t="s">
         <v>2389</v>
@@ -30350,7 +30350,7 @@
         <v>1626</v>
       </c>
       <c r="I624" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J624" t="s">
         <v>2390</v>
@@ -30385,7 +30385,7 @@
         <v>1626</v>
       </c>
       <c r="I625" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J625" t="s">
         <v>2391</v>
@@ -30420,7 +30420,7 @@
         <v>1626</v>
       </c>
       <c r="I626" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J626" t="s">
         <v>2392</v>
@@ -30455,7 +30455,7 @@
         <v>1626</v>
       </c>
       <c r="I627" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J627" t="s">
         <v>2393</v>
@@ -30525,7 +30525,7 @@
         <v>1626</v>
       </c>
       <c r="I629" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J629" t="s">
         <v>2115</v>
@@ -30665,7 +30665,7 @@
         <v>1626</v>
       </c>
       <c r="I633" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J633" t="s">
         <v>2398</v>
@@ -31158,7 +31158,7 @@
         <v>1626</v>
       </c>
       <c r="I647" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J647" t="s">
         <v>2411</v>
@@ -31193,7 +31193,7 @@
         <v>1626</v>
       </c>
       <c r="I648" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J648" t="s">
         <v>2412</v>
@@ -31228,7 +31228,7 @@
         <v>1626</v>
       </c>
       <c r="I649" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J649" t="s">
         <v>2413</v>
@@ -31266,7 +31266,7 @@
         <v>1655</v>
       </c>
       <c r="I650" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J650" t="s">
         <v>2414</v>
@@ -31304,7 +31304,7 @@
         <v>1656</v>
       </c>
       <c r="I651" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J651" t="s">
         <v>2415</v>
@@ -31444,7 +31444,7 @@
         <v>1626</v>
       </c>
       <c r="I655" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J655" t="s">
         <v>2418</v>
@@ -31479,7 +31479,7 @@
         <v>1626</v>
       </c>
       <c r="I656" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J656" t="s">
         <v>2419</v>
@@ -31549,7 +31549,7 @@
         <v>1626</v>
       </c>
       <c r="I658" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J658" t="s">
         <v>2421</v>
@@ -31689,7 +31689,7 @@
         <v>1626</v>
       </c>
       <c r="I662" t="s">
-        <v>1703</v>
+        <v>1745</v>
       </c>
       <c r="J662" t="s">
         <v>2425</v>
@@ -31733,7 +31733,7 @@
         <v>2453</v>
       </c>
       <c r="L663" t="s">
-        <v>2607</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -31759,7 +31759,7 @@
         <v>1626</v>
       </c>
       <c r="I664" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J664" t="s">
         <v>2427</v>
@@ -31981,7 +31981,7 @@
         <v>2463</v>
       </c>
       <c r="L670" t="s">
-        <v>2665</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="671" spans="1:12">
@@ -32057,7 +32057,7 @@
         <v>2475</v>
       </c>
       <c r="L672" t="s">
-        <v>2629</v>
+        <v>2665</v>
       </c>
     </row>
     <row r="673" spans="1:12">
@@ -32118,7 +32118,7 @@
         <v>1626</v>
       </c>
       <c r="I674" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J674" t="s">
         <v>2436</v>
@@ -32255,7 +32255,7 @@
         <v>1626</v>
       </c>
       <c r="I678" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J678" t="s">
         <v>2439</v>
@@ -32287,7 +32287,7 @@
         <v>1626</v>
       </c>
       <c r="I679" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J679" t="s">
         <v>2440</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-25 22:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -97,10 +97,10 @@
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
-  </si>
-  <si>
-    <t>SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
@@ -11058,7 +11058,7 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B74" t="s">
         <v>117</v>
@@ -11079,7 +11079,7 @@
         <v>1649</v>
       </c>
       <c r="I74" t="s">
-        <v>1720</v>
+        <v>1687</v>
       </c>
       <c r="J74" t="s">
         <v>1891</v>
@@ -11373,7 +11373,7 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B83" t="s">
         <v>126</v>
@@ -11904,7 +11904,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B98" t="s">
         <v>141</v>
@@ -13103,7 +13103,7 @@
     </row>
     <row r="132" spans="1:12">
       <c r="A132" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B132" t="s">
         <v>175</v>
@@ -13949,7 +13949,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B156" t="s">
         <v>199</v>
@@ -13984,7 +13984,7 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B157" t="s">
         <v>200</v>
@@ -15848,7 +15848,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B210" t="s">
         <v>253</v>
@@ -17068,7 +17068,7 @@
         <v>1836</v>
       </c>
       <c r="K244" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L244" t="s">
         <v>2629</v>
@@ -18619,7 +18619,7 @@
     </row>
     <row r="289" spans="1:12">
       <c r="A289" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B289" t="s">
         <v>332</v>
@@ -18829,7 +18829,7 @@
     </row>
     <row r="295" spans="1:12">
       <c r="A295" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B295" t="s">
         <v>338</v>
@@ -19039,7 +19039,7 @@
     </row>
     <row r="301" spans="1:12">
       <c r="A301" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B301" t="s">
         <v>344</v>
@@ -19497,7 +19497,7 @@
     </row>
     <row r="314" spans="1:12">
       <c r="A314" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B314" t="s">
         <v>357</v>
@@ -22446,7 +22446,7 @@
     </row>
     <row r="398" spans="1:12">
       <c r="A398" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B398" t="s">
         <v>441</v>
@@ -23508,7 +23508,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B428" t="s">
         <v>471</v>
@@ -25725,7 +25725,7 @@
     </row>
     <row r="491" spans="1:12">
       <c r="A491" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B491" t="s">
         <v>534</v>
@@ -25865,7 +25865,7 @@
     </row>
     <row r="495" spans="1:12">
       <c r="A495" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B495" t="s">
         <v>538</v>
@@ -25970,7 +25970,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B498" t="s">
         <v>541</v>
@@ -29197,7 +29197,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B589" t="s">
         <v>631</v>
@@ -29232,7 +29232,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B590" t="s">
         <v>632</v>
@@ -29407,7 +29407,7 @@
     </row>
     <row r="595" spans="1:12">
       <c r="A595" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B595" t="s">
         <v>637</v>
@@ -29760,7 +29760,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B605" t="s">
         <v>647</v>
@@ -29830,7 +29830,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B607" t="s">
         <v>649</v>
@@ -29976,7 +29976,7 @@
     </row>
     <row r="611" spans="1:12">
       <c r="A611" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B611" t="s">
         <v>653</v>
@@ -30151,7 +30151,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B616" t="s">
         <v>658</v>
@@ -30504,7 +30504,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B626" t="s">
         <v>668</v>
@@ -30539,7 +30539,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B627" t="s">
         <v>669</v>
@@ -30749,7 +30749,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B633" t="s">
         <v>675</v>
@@ -30784,7 +30784,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B634" t="s">
         <v>676</v>
@@ -30819,7 +30819,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B635" t="s">
         <v>677</v>
@@ -30854,7 +30854,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B636" t="s">
         <v>678</v>
@@ -30889,7 +30889,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B637" t="s">
         <v>679</v>
@@ -30924,7 +30924,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B638" t="s">
         <v>680</v>
@@ -31210,7 +31210,7 @@
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B646" t="s">
         <v>688</v>
@@ -31280,7 +31280,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B648" t="s">
         <v>690</v>
@@ -31385,7 +31385,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B651" t="s">
         <v>693</v>
@@ -31525,7 +31525,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B655" t="s">
         <v>697</v>
@@ -31630,7 +31630,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B658" t="s">
         <v>700</v>
@@ -31700,7 +31700,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B660" t="s">
         <v>702</v>
@@ -31735,7 +31735,7 @@
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B661" t="s">
         <v>703</v>
@@ -31770,7 +31770,7 @@
     </row>
     <row r="662" spans="1:12">
       <c r="A662" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B662" t="s">
         <v>704</v>
@@ -31846,7 +31846,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B664" t="s">
         <v>706</v>
@@ -31954,7 +31954,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B667" t="s">
         <v>709</v>
@@ -31989,7 +31989,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B668" t="s">
         <v>710</v>
@@ -32024,7 +32024,7 @@
     </row>
     <row r="669" spans="1:12">
       <c r="A669" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B669" t="s">
         <v>711</v>
@@ -32094,7 +32094,7 @@
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B671" t="s">
         <v>713</v>
@@ -32132,7 +32132,7 @@
     </row>
     <row r="672" spans="1:12">
       <c r="A672" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B672" t="s">
         <v>714</v>
@@ -32167,7 +32167,7 @@
     </row>
     <row r="673" spans="1:12">
       <c r="A673" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B673" t="s">
         <v>715</v>
@@ -32272,7 +32272,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B676" t="s">
         <v>718</v>
@@ -32307,7 +32307,7 @@
     </row>
     <row r="677" spans="1:12">
       <c r="A677" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B677" t="s">
         <v>719</v>
@@ -32342,7 +32342,7 @@
     </row>
     <row r="678" spans="1:12">
       <c r="A678" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B678" t="s">
         <v>720</v>
@@ -32377,7 +32377,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B679" t="s">
         <v>721</v>
@@ -32412,7 +32412,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B680" t="s">
         <v>722</v>
@@ -32450,7 +32450,7 @@
     </row>
     <row r="681" spans="1:12">
       <c r="A681" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B681" t="s">
         <v>723</v>
@@ -32561,7 +32561,7 @@
     </row>
     <row r="684" spans="1:12">
       <c r="A684" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B684" t="s">
         <v>726</v>
@@ -32596,7 +32596,7 @@
     </row>
     <row r="685" spans="1:12">
       <c r="A685" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B685" t="s">
         <v>727</v>
@@ -32707,7 +32707,7 @@
     </row>
     <row r="688" spans="1:12">
       <c r="A688" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B688" t="s">
         <v>730</v>
@@ -32739,7 +32739,7 @@
     </row>
     <row r="689" spans="1:12">
       <c r="A689" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B689" t="s">
         <v>731</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-27 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -10599,7 +10599,7 @@
         <v>1660</v>
       </c>
       <c r="I59" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
       <c r="J59" t="s">
         <v>1886</v>
@@ -12361,7 +12361,7 @@
         <v>1660</v>
       </c>
       <c r="I109" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
       <c r="J109" t="s">
         <v>1936</v>
@@ -24671,7 +24671,7 @@
         <v>1660</v>
       </c>
       <c r="I459" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
       <c r="J459" t="s">
         <v>2269</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-30 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -26141,7 +26141,7 @@
     </row>
     <row r="501" spans="1:12">
       <c r="A501" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B501" t="s">
         <v>545</v>
@@ -26162,7 +26162,7 @@
         <v>1661</v>
       </c>
       <c r="I501" t="s">
-        <v>1781</v>
+        <v>1703</v>
       </c>
       <c r="J501" t="s">
         <v>2310</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-01 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -32256,7 +32256,7 @@
     </row>
     <row r="677" spans="1:12">
       <c r="A677" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B677" t="s">
         <v>721</v>
@@ -32280,7 +32280,7 @@
         <v>1663</v>
       </c>
       <c r="I677" t="s">
-        <v>1670</v>
+        <v>1780</v>
       </c>
       <c r="J677" t="s">
         <v>2447</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-02 12:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -97,6 +97,9 @@
     <t>NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -116,9 +119,6 @@
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE CONTABILIDADE,NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS, NÚCLEO TÉCNICO DE ENGENHARIA</t>
@@ -11672,7 +11672,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B93" t="s">
         <v>138</v>
@@ -11696,7 +11696,7 @@
         <v>1473</v>
       </c>
       <c r="I93" t="s">
-        <v>1680</v>
+        <v>1676</v>
       </c>
       <c r="J93" t="s">
         <v>1895</v>
@@ -11815,7 +11815,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B97" t="s">
         <v>142</v>
@@ -11850,7 +11850,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B98" t="s">
         <v>143</v>
@@ -12346,7 +12346,7 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B112" t="s">
         <v>157</v>
@@ -12629,7 +12629,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B120" t="s">
         <v>165</v>
@@ -13122,7 +13122,7 @@
     </row>
     <row r="134" spans="1:12">
       <c r="A134" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B134" t="s">
         <v>179</v>
@@ -13157,7 +13157,7 @@
     </row>
     <row r="135" spans="1:12">
       <c r="A135" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B135" t="s">
         <v>180</v>
@@ -13192,7 +13192,7 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B136" t="s">
         <v>181</v>
@@ -13227,7 +13227,7 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B137" t="s">
         <v>182</v>
@@ -13402,7 +13402,7 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B142" t="s">
         <v>187</v>
@@ -13437,7 +13437,7 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B143" t="s">
         <v>188</v>
@@ -13583,7 +13583,7 @@
     </row>
     <row r="147" spans="1:12">
       <c r="A147" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B147" t="s">
         <v>192</v>
@@ -13618,7 +13618,7 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B148" t="s">
         <v>193</v>
@@ -13653,7 +13653,7 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B149" t="s">
         <v>194</v>
@@ -13933,7 +13933,7 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B157" t="s">
         <v>202</v>
@@ -14076,7 +14076,7 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B161" t="s">
         <v>206</v>
@@ -14146,7 +14146,7 @@
     </row>
     <row r="163" spans="1:12">
       <c r="A163" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B163" t="s">
         <v>208</v>
@@ -14251,7 +14251,7 @@
     </row>
     <row r="166" spans="1:12">
       <c r="A166" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B166" t="s">
         <v>211</v>
@@ -14286,7 +14286,7 @@
     </row>
     <row r="167" spans="1:12">
       <c r="A167" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B167" t="s">
         <v>212</v>
@@ -14321,7 +14321,7 @@
     </row>
     <row r="168" spans="1:12">
       <c r="A168" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B168" t="s">
         <v>213</v>
@@ -14391,7 +14391,7 @@
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B170" t="s">
         <v>215</v>
@@ -14671,7 +14671,7 @@
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B178" t="s">
         <v>223</v>
@@ -14811,7 +14811,7 @@
     </row>
     <row r="182" spans="1:12">
       <c r="A182" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B182" t="s">
         <v>227</v>
@@ -14881,7 +14881,7 @@
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B184" t="s">
         <v>229</v>
@@ -14916,7 +14916,7 @@
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B185" t="s">
         <v>230</v>
@@ -14951,7 +14951,7 @@
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B186" t="s">
         <v>231</v>
@@ -15231,7 +15231,7 @@
     </row>
     <row r="194" spans="1:12">
       <c r="A194" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B194" t="s">
         <v>239</v>
@@ -15266,7 +15266,7 @@
     </row>
     <row r="195" spans="1:12">
       <c r="A195" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B195" t="s">
         <v>240</v>
@@ -15581,7 +15581,7 @@
     </row>
     <row r="204" spans="1:12">
       <c r="A204" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B204" t="s">
         <v>249</v>
@@ -15794,7 +15794,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B210" t="s">
         <v>255</v>
@@ -15864,7 +15864,7 @@
     </row>
     <row r="212" spans="1:12">
       <c r="A212" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B212" t="s">
         <v>257</v>
@@ -15934,7 +15934,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B214" t="s">
         <v>259</v>
@@ -16004,7 +16004,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B216" t="s">
         <v>261</v>
@@ -16136,7 +16136,7 @@
         <v>1818</v>
       </c>
       <c r="K219" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="L219" t="s">
         <v>2611</v>
@@ -16144,7 +16144,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B220" t="s">
         <v>265</v>
@@ -16389,7 +16389,7 @@
     </row>
     <row r="227" spans="1:12">
       <c r="A227" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B227" t="s">
         <v>272</v>
@@ -16459,7 +16459,7 @@
     </row>
     <row r="229" spans="1:12">
       <c r="A229" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B229" t="s">
         <v>274</v>
@@ -16529,7 +16529,7 @@
     </row>
     <row r="231" spans="1:12">
       <c r="A231" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B231" t="s">
         <v>276</v>
@@ -16742,7 +16742,7 @@
     </row>
     <row r="237" spans="1:12">
       <c r="A237" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B237" t="s">
         <v>282</v>
@@ -16777,7 +16777,7 @@
     </row>
     <row r="238" spans="1:12">
       <c r="A238" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B238" t="s">
         <v>283</v>
@@ -16812,7 +16812,7 @@
     </row>
     <row r="239" spans="1:12">
       <c r="A239" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B239" t="s">
         <v>284</v>
@@ -16882,7 +16882,7 @@
     </row>
     <row r="241" spans="1:12">
       <c r="A241" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B241" t="s">
         <v>286</v>
@@ -16952,7 +16952,7 @@
     </row>
     <row r="243" spans="1:12">
       <c r="A243" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B243" t="s">
         <v>288</v>
@@ -17092,7 +17092,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B247" t="s">
         <v>292</v>
@@ -17127,7 +17127,7 @@
     </row>
     <row r="248" spans="1:12">
       <c r="A248" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B248" t="s">
         <v>293</v>
@@ -17162,7 +17162,7 @@
     </row>
     <row r="249" spans="1:12">
       <c r="A249" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B249" t="s">
         <v>294</v>
@@ -17197,7 +17197,7 @@
     </row>
     <row r="250" spans="1:12">
       <c r="A250" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B250" t="s">
         <v>295</v>
@@ -17232,7 +17232,7 @@
     </row>
     <row r="251" spans="1:12">
       <c r="A251" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B251" t="s">
         <v>296</v>
@@ -17477,7 +17477,7 @@
     </row>
     <row r="258" spans="1:12">
       <c r="A258" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B258" t="s">
         <v>303</v>
@@ -17547,7 +17547,7 @@
     </row>
     <row r="260" spans="1:12">
       <c r="A260" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B260" t="s">
         <v>305</v>
@@ -17617,7 +17617,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B262" t="s">
         <v>307</v>
@@ -17897,7 +17897,7 @@
     </row>
     <row r="270" spans="1:12">
       <c r="A270" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B270" t="s">
         <v>315</v>
@@ -17932,7 +17932,7 @@
     </row>
     <row r="271" spans="1:12">
       <c r="A271" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B271" t="s">
         <v>316</v>
@@ -18002,7 +18002,7 @@
     </row>
     <row r="273" spans="1:12">
       <c r="A273" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B273" t="s">
         <v>318</v>
@@ -18215,7 +18215,7 @@
     </row>
     <row r="279" spans="1:12">
       <c r="A279" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B279" t="s">
         <v>324</v>
@@ -18250,7 +18250,7 @@
     </row>
     <row r="280" spans="1:12">
       <c r="A280" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B280" t="s">
         <v>325</v>
@@ -18320,7 +18320,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B282" t="s">
         <v>327</v>
@@ -18530,7 +18530,7 @@
     </row>
     <row r="288" spans="1:12">
       <c r="A288" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B288" t="s">
         <v>333</v>
@@ -18775,7 +18775,7 @@
     </row>
     <row r="295" spans="1:12">
       <c r="A295" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B295" t="s">
         <v>340</v>
@@ -18915,7 +18915,7 @@
     </row>
     <row r="299" spans="1:12">
       <c r="A299" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B299" t="s">
         <v>344</v>
@@ -19265,7 +19265,7 @@
     </row>
     <row r="309" spans="1:12">
       <c r="A309" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B309" t="s">
         <v>354</v>
@@ -19408,7 +19408,7 @@
     </row>
     <row r="313" spans="1:12">
       <c r="A313" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B313" t="s">
         <v>358</v>
@@ -19443,7 +19443,7 @@
     </row>
     <row r="314" spans="1:12">
       <c r="A314" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B314" t="s">
         <v>359</v>
@@ -19618,7 +19618,7 @@
     </row>
     <row r="319" spans="1:12">
       <c r="A319" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B319" t="s">
         <v>364</v>
@@ -19691,7 +19691,7 @@
     </row>
     <row r="321" spans="1:12">
       <c r="A321" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B321" t="s">
         <v>366</v>
@@ -19726,7 +19726,7 @@
     </row>
     <row r="322" spans="1:12">
       <c r="A322" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B322" t="s">
         <v>367</v>
@@ -19761,7 +19761,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B323" t="s">
         <v>368</v>
@@ -19796,7 +19796,7 @@
     </row>
     <row r="324" spans="1:12">
       <c r="A324" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B324" t="s">
         <v>369</v>
@@ -19831,7 +19831,7 @@
     </row>
     <row r="325" spans="1:12">
       <c r="A325" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B325" t="s">
         <v>370</v>
@@ -19866,7 +19866,7 @@
     </row>
     <row r="326" spans="1:12">
       <c r="A326" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B326" t="s">
         <v>371</v>
@@ -19971,7 +19971,7 @@
     </row>
     <row r="329" spans="1:12">
       <c r="A329" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B329" t="s">
         <v>374</v>
@@ -20111,7 +20111,7 @@
     </row>
     <row r="333" spans="1:12">
       <c r="A333" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B333" t="s">
         <v>378</v>
@@ -20146,7 +20146,7 @@
     </row>
     <row r="334" spans="1:12">
       <c r="A334" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B334" t="s">
         <v>379</v>
@@ -20181,7 +20181,7 @@
     </row>
     <row r="335" spans="1:12">
       <c r="A335" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B335" t="s">
         <v>380</v>
@@ -20216,7 +20216,7 @@
     </row>
     <row r="336" spans="1:12">
       <c r="A336" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B336" t="s">
         <v>381</v>
@@ -20251,7 +20251,7 @@
     </row>
     <row r="337" spans="1:12">
       <c r="A337" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B337" t="s">
         <v>382</v>
@@ -20286,7 +20286,7 @@
     </row>
     <row r="338" spans="1:12">
       <c r="A338" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B338" t="s">
         <v>383</v>
@@ -20356,7 +20356,7 @@
     </row>
     <row r="340" spans="1:12">
       <c r="A340" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B340" t="s">
         <v>385</v>
@@ -20391,7 +20391,7 @@
     </row>
     <row r="341" spans="1:12">
       <c r="A341" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B341" t="s">
         <v>386</v>
@@ -20461,7 +20461,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B343" t="s">
         <v>388</v>
@@ -20566,7 +20566,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B346" t="s">
         <v>391</v>
@@ -20811,7 +20811,7 @@
     </row>
     <row r="353" spans="1:12">
       <c r="A353" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B353" t="s">
         <v>398</v>
@@ -20951,7 +20951,7 @@
     </row>
     <row r="357" spans="1:12">
       <c r="A357" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B357" t="s">
         <v>402</v>
@@ -21091,7 +21091,7 @@
     </row>
     <row r="361" spans="1:12">
       <c r="A361" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B361" t="s">
         <v>406</v>
@@ -21126,7 +21126,7 @@
     </row>
     <row r="362" spans="1:12">
       <c r="A362" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B362" t="s">
         <v>407</v>
@@ -21196,7 +21196,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B364" t="s">
         <v>409</v>
@@ -21231,7 +21231,7 @@
     </row>
     <row r="365" spans="1:12">
       <c r="A365" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B365" t="s">
         <v>410</v>
@@ -21266,7 +21266,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B366" t="s">
         <v>411</v>
@@ -21514,7 +21514,7 @@
     </row>
     <row r="373" spans="1:12">
       <c r="A373" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B373" t="s">
         <v>418</v>
@@ -21727,7 +21727,7 @@
     </row>
     <row r="379" spans="1:12">
       <c r="A379" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B379" t="s">
         <v>424</v>
@@ -21838,7 +21838,7 @@
     </row>
     <row r="382" spans="1:12">
       <c r="A382" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B382" t="s">
         <v>427</v>
@@ -21908,7 +21908,7 @@
     </row>
     <row r="384" spans="1:12">
       <c r="A384" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B384" t="s">
         <v>429</v>
@@ -21943,7 +21943,7 @@
     </row>
     <row r="385" spans="1:12">
       <c r="A385" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B385" t="s">
         <v>430</v>
@@ -22013,7 +22013,7 @@
     </row>
     <row r="387" spans="1:12">
       <c r="A387" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B387" t="s">
         <v>432</v>
@@ -22048,7 +22048,7 @@
     </row>
     <row r="388" spans="1:12">
       <c r="A388" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B388" t="s">
         <v>433</v>
@@ -22153,7 +22153,7 @@
     </row>
     <row r="391" spans="1:12">
       <c r="A391" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B391" t="s">
         <v>436</v>
@@ -22188,7 +22188,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B392" t="s">
         <v>437</v>
@@ -22223,7 +22223,7 @@
     </row>
     <row r="393" spans="1:12">
       <c r="A393" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B393" t="s">
         <v>438</v>
@@ -22293,7 +22293,7 @@
     </row>
     <row r="395" spans="1:12">
       <c r="A395" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B395" t="s">
         <v>440</v>
@@ -22363,7 +22363,7 @@
     </row>
     <row r="397" spans="1:12">
       <c r="A397" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B397" t="s">
         <v>442</v>
@@ -22398,7 +22398,7 @@
     </row>
     <row r="398" spans="1:12">
       <c r="A398" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B398" t="s">
         <v>443</v>
@@ -22433,7 +22433,7 @@
     </row>
     <row r="399" spans="1:12">
       <c r="A399" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B399" t="s">
         <v>444</v>
@@ -22468,7 +22468,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B400" t="s">
         <v>445</v>
@@ -22608,7 +22608,7 @@
     </row>
     <row r="404" spans="1:12">
       <c r="A404" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B404" t="s">
         <v>449</v>
@@ -22678,7 +22678,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B406" t="s">
         <v>451</v>
@@ -22751,7 +22751,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B408" t="s">
         <v>453</v>
@@ -22786,7 +22786,7 @@
     </row>
     <row r="409" spans="1:12">
       <c r="A409" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B409" t="s">
         <v>454</v>
@@ -22891,7 +22891,7 @@
     </row>
     <row r="412" spans="1:12">
       <c r="A412" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B412" t="s">
         <v>457</v>
@@ -22961,7 +22961,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B414" t="s">
         <v>459</v>
@@ -22996,7 +22996,7 @@
     </row>
     <row r="415" spans="1:12">
       <c r="A415" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B415" t="s">
         <v>460</v>
@@ -23031,7 +23031,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B416" t="s">
         <v>461</v>
@@ -23066,7 +23066,7 @@
     </row>
     <row r="417" spans="1:12">
       <c r="A417" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B417" t="s">
         <v>462</v>
@@ -23101,7 +23101,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B418" t="s">
         <v>463</v>
@@ -23206,7 +23206,7 @@
     </row>
     <row r="421" spans="1:12">
       <c r="A421" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B421" t="s">
         <v>466</v>
@@ -23241,7 +23241,7 @@
     </row>
     <row r="422" spans="1:12">
       <c r="A422" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B422" t="s">
         <v>467</v>
@@ -23276,7 +23276,7 @@
     </row>
     <row r="423" spans="1:12">
       <c r="A423" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B423" t="s">
         <v>468</v>
@@ -23381,7 +23381,7 @@
     </row>
     <row r="426" spans="1:12">
       <c r="A426" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B426" t="s">
         <v>471</v>
@@ -23451,7 +23451,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B428" t="s">
         <v>473</v>
@@ -23521,7 +23521,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B430" t="s">
         <v>475</v>
@@ -23766,7 +23766,7 @@
     </row>
     <row r="437" spans="1:12">
       <c r="A437" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B437" t="s">
         <v>482</v>
@@ -23909,7 +23909,7 @@
     </row>
     <row r="441" spans="1:12">
       <c r="A441" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B441" t="s">
         <v>486</v>
@@ -24014,7 +24014,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B444" t="s">
         <v>489</v>
@@ -24049,7 +24049,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B445" t="s">
         <v>490</v>
@@ -24084,7 +24084,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B446" t="s">
         <v>491</v>
@@ -24189,7 +24189,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B449" t="s">
         <v>494</v>
@@ -24259,7 +24259,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B451" t="s">
         <v>496</v>
@@ -24329,7 +24329,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B453" t="s">
         <v>498</v>
@@ -24364,7 +24364,7 @@
     </row>
     <row r="454" spans="1:12">
       <c r="A454" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B454" t="s">
         <v>499</v>
@@ -24399,7 +24399,7 @@
     </row>
     <row r="455" spans="1:12">
       <c r="A455" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B455" t="s">
         <v>500</v>
@@ -24434,7 +24434,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B456" t="s">
         <v>501</v>
@@ -24469,7 +24469,7 @@
     </row>
     <row r="457" spans="1:12">
       <c r="A457" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B457" t="s">
         <v>502</v>
@@ -24542,7 +24542,7 @@
     </row>
     <row r="459" spans="1:12">
       <c r="A459" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B459" t="s">
         <v>504</v>
@@ -24577,7 +24577,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B460" t="s">
         <v>505</v>
@@ -24758,7 +24758,7 @@
     </row>
     <row r="465" spans="1:12">
       <c r="A465" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B465" t="s">
         <v>509</v>
@@ -24793,7 +24793,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B466" t="s">
         <v>510</v>
@@ -24901,7 +24901,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B469" t="s">
         <v>513</v>
@@ -24971,7 +24971,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B471" t="s">
         <v>515</v>
@@ -25041,7 +25041,7 @@
     </row>
     <row r="473" spans="1:12">
       <c r="A473" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B473" t="s">
         <v>517</v>
@@ -25076,7 +25076,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B474" t="s">
         <v>518</v>
@@ -25111,7 +25111,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B475" t="s">
         <v>519</v>
@@ -25289,7 +25289,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B480" t="s">
         <v>524</v>
@@ -25324,7 +25324,7 @@
     </row>
     <row r="481" spans="1:12">
       <c r="A481" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B481" t="s">
         <v>525</v>
@@ -25429,7 +25429,7 @@
     </row>
     <row r="484" spans="1:12">
       <c r="A484" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B484" t="s">
         <v>528</v>
@@ -25464,7 +25464,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B485" t="s">
         <v>529</v>
@@ -25499,7 +25499,7 @@
     </row>
     <row r="486" spans="1:12">
       <c r="A486" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B486" t="s">
         <v>530</v>
@@ -25534,7 +25534,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B487" t="s">
         <v>531</v>
@@ -25569,7 +25569,7 @@
     </row>
     <row r="488" spans="1:12">
       <c r="A488" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B488" t="s">
         <v>532</v>
@@ -25604,7 +25604,7 @@
     </row>
     <row r="489" spans="1:12">
       <c r="A489" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B489" t="s">
         <v>533</v>
@@ -25709,7 +25709,7 @@
     </row>
     <row r="492" spans="1:12">
       <c r="A492" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B492" t="s">
         <v>536</v>
@@ -25744,7 +25744,7 @@
     </row>
     <row r="493" spans="1:12">
       <c r="A493" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B493" t="s">
         <v>537</v>
@@ -25779,7 +25779,7 @@
     </row>
     <row r="494" spans="1:12">
       <c r="A494" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B494" t="s">
         <v>538</v>
@@ -25852,7 +25852,7 @@
     </row>
     <row r="496" spans="1:12">
       <c r="A496" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B496" t="s">
         <v>540</v>
@@ -25922,7 +25922,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B498" t="s">
         <v>542</v>
@@ -26135,7 +26135,7 @@
     </row>
     <row r="504" spans="1:12">
       <c r="A504" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B504" t="s">
         <v>548</v>
@@ -26170,7 +26170,7 @@
     </row>
     <row r="505" spans="1:12">
       <c r="A505" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B505" t="s">
         <v>549</v>
@@ -26205,7 +26205,7 @@
     </row>
     <row r="506" spans="1:12">
       <c r="A506" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B506" t="s">
         <v>550</v>
@@ -26240,7 +26240,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B507" t="s">
         <v>551</v>
@@ -26275,7 +26275,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B508" t="s">
         <v>552</v>
@@ -26348,7 +26348,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B510" t="s">
         <v>554</v>
@@ -26383,7 +26383,7 @@
     </row>
     <row r="511" spans="1:12">
       <c r="A511" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B511" t="s">
         <v>555</v>
@@ -26456,7 +26456,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B513" t="s">
         <v>557</v>
@@ -26491,7 +26491,7 @@
     </row>
     <row r="514" spans="1:12">
       <c r="A514" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B514" t="s">
         <v>558</v>
@@ -26526,7 +26526,7 @@
     </row>
     <row r="515" spans="1:12">
       <c r="A515" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B515" t="s">
         <v>559</v>
@@ -26596,7 +26596,7 @@
     </row>
     <row r="517" spans="1:12">
       <c r="A517" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B517" t="s">
         <v>561</v>
@@ -26631,7 +26631,7 @@
     </row>
     <row r="518" spans="1:12">
       <c r="A518" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B518" t="s">
         <v>562</v>
@@ -26701,7 +26701,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B520" t="s">
         <v>564</v>
@@ -26736,7 +26736,7 @@
     </row>
     <row r="521" spans="1:12">
       <c r="A521" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B521" t="s">
         <v>565</v>
@@ -26809,7 +26809,7 @@
     </row>
     <row r="523" spans="1:12">
       <c r="A523" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B523" t="s">
         <v>567</v>
@@ -26844,7 +26844,7 @@
     </row>
     <row r="524" spans="1:12">
       <c r="A524" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B524" t="s">
         <v>568</v>
@@ -26879,7 +26879,7 @@
     </row>
     <row r="525" spans="1:12">
       <c r="A525" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B525" t="s">
         <v>569</v>
@@ -26914,7 +26914,7 @@
     </row>
     <row r="526" spans="1:12">
       <c r="A526" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B526" t="s">
         <v>570</v>
@@ -26949,7 +26949,7 @@
     </row>
     <row r="527" spans="1:12">
       <c r="A527" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B527" t="s">
         <v>571</v>
@@ -26984,7 +26984,7 @@
     </row>
     <row r="528" spans="1:12">
       <c r="A528" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B528" t="s">
         <v>572</v>
@@ -27019,7 +27019,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B529" t="s">
         <v>573</v>
@@ -27127,7 +27127,7 @@
     </row>
     <row r="532" spans="1:12">
       <c r="A532" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B532" t="s">
         <v>576</v>
@@ -27238,7 +27238,7 @@
     </row>
     <row r="535" spans="1:12">
       <c r="A535" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B535" t="s">
         <v>579</v>
@@ -27273,7 +27273,7 @@
     </row>
     <row r="536" spans="1:12">
       <c r="A536" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B536" t="s">
         <v>580</v>
@@ -27308,7 +27308,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B537" t="s">
         <v>581</v>
@@ -27343,7 +27343,7 @@
     </row>
     <row r="538" spans="1:12">
       <c r="A538" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B538" t="s">
         <v>582</v>
@@ -27378,7 +27378,7 @@
     </row>
     <row r="539" spans="1:12">
       <c r="A539" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B539" t="s">
         <v>583</v>
@@ -27413,7 +27413,7 @@
     </row>
     <row r="540" spans="1:12">
       <c r="A540" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B540" t="s">
         <v>584</v>
@@ -27448,7 +27448,7 @@
     </row>
     <row r="541" spans="1:12">
       <c r="A541" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B541" t="s">
         <v>585</v>
@@ -27483,7 +27483,7 @@
     </row>
     <row r="542" spans="1:12">
       <c r="A542" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B542" t="s">
         <v>586</v>
@@ -27553,7 +27553,7 @@
     </row>
     <row r="544" spans="1:12">
       <c r="A544" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B544" t="s">
         <v>588</v>
@@ -27623,7 +27623,7 @@
     </row>
     <row r="546" spans="1:12">
       <c r="A546" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B546" t="s">
         <v>590</v>
@@ -27658,7 +27658,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B547" t="s">
         <v>591</v>
@@ -27693,7 +27693,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B548" t="s">
         <v>592</v>
@@ -27728,7 +27728,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B549" t="s">
         <v>593</v>
@@ -27763,7 +27763,7 @@
     </row>
     <row r="550" spans="1:12">
       <c r="A550" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B550" t="s">
         <v>594</v>
@@ -27833,7 +27833,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B552" t="s">
         <v>596</v>
@@ -27868,7 +27868,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B553" t="s">
         <v>597</v>
@@ -27903,7 +27903,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B554" t="s">
         <v>598</v>
@@ -27973,7 +27973,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B556" t="s">
         <v>600</v>
@@ -28011,7 +28011,7 @@
     </row>
     <row r="557" spans="1:12">
       <c r="A557" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B557" t="s">
         <v>601</v>
@@ -28081,7 +28081,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B559" t="s">
         <v>603</v>
@@ -28116,7 +28116,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B560" t="s">
         <v>604</v>
@@ -28151,7 +28151,7 @@
     </row>
     <row r="561" spans="1:12">
       <c r="A561" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B561" t="s">
         <v>605</v>
@@ -28186,7 +28186,7 @@
     </row>
     <row r="562" spans="1:12">
       <c r="A562" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B562" t="s">
         <v>606</v>
@@ -28221,7 +28221,7 @@
     </row>
     <row r="563" spans="1:12">
       <c r="A563" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B563" t="s">
         <v>607</v>
@@ -28294,7 +28294,7 @@
     </row>
     <row r="565" spans="1:12">
       <c r="A565" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B565" t="s">
         <v>609</v>
@@ -28364,7 +28364,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B567" t="s">
         <v>611</v>
@@ -28399,7 +28399,7 @@
     </row>
     <row r="568" spans="1:12">
       <c r="A568" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B568" t="s">
         <v>612</v>
@@ -28469,7 +28469,7 @@
     </row>
     <row r="570" spans="1:12">
       <c r="A570" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B570" t="s">
         <v>614</v>
@@ -28504,7 +28504,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B571" t="s">
         <v>615</v>
@@ -28539,7 +28539,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B572" t="s">
         <v>616</v>
@@ -28574,7 +28574,7 @@
     </row>
     <row r="573" spans="1:12">
       <c r="A573" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B573" t="s">
         <v>617</v>
@@ -28609,7 +28609,7 @@
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B574" t="s">
         <v>618</v>
@@ -28644,7 +28644,7 @@
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B575" t="s">
         <v>619</v>
@@ -28679,7 +28679,7 @@
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B576" t="s">
         <v>620</v>
@@ -28714,7 +28714,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B577" t="s">
         <v>621</v>
@@ -28749,7 +28749,7 @@
     </row>
     <row r="578" spans="1:12">
       <c r="A578" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B578" t="s">
         <v>622</v>
@@ -28784,7 +28784,7 @@
     </row>
     <row r="579" spans="1:12">
       <c r="A579" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B579" t="s">
         <v>623</v>
@@ -28819,7 +28819,7 @@
     </row>
     <row r="580" spans="1:12">
       <c r="A580" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B580" t="s">
         <v>624</v>
@@ -28889,7 +28889,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B582" t="s">
         <v>626</v>
@@ -29029,7 +29029,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B586" t="s">
         <v>630</v>
@@ -29064,7 +29064,7 @@
     </row>
     <row r="587" spans="1:12">
       <c r="A587" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B587" t="s">
         <v>631</v>
@@ -29099,7 +29099,7 @@
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B588" t="s">
         <v>632</v>
@@ -29134,7 +29134,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B589" t="s">
         <v>633</v>
@@ -29169,7 +29169,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B590" t="s">
         <v>634</v>
@@ -29204,7 +29204,7 @@
     </row>
     <row r="591" spans="1:12">
       <c r="A591" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B591" t="s">
         <v>635</v>
@@ -29239,7 +29239,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B592" t="s">
         <v>636</v>
@@ -29274,7 +29274,7 @@
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B593" t="s">
         <v>637</v>
@@ -29420,7 +29420,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B597" t="s">
         <v>641</v>
@@ -29455,7 +29455,7 @@
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B598" t="s">
         <v>642</v>
@@ -29490,7 +29490,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B599" t="s">
         <v>643</v>
@@ -29525,7 +29525,7 @@
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B600" t="s">
         <v>644</v>
@@ -29560,7 +29560,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B601" t="s">
         <v>645</v>
@@ -29595,7 +29595,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B602" t="s">
         <v>646</v>
@@ -29630,7 +29630,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B603" t="s">
         <v>647</v>
@@ -29665,7 +29665,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B604" t="s">
         <v>648</v>
@@ -29700,7 +29700,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B605" t="s">
         <v>649</v>
@@ -29735,7 +29735,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B606" t="s">
         <v>650</v>
@@ -29770,7 +29770,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B607" t="s">
         <v>651</v>
@@ -29805,7 +29805,7 @@
     </row>
     <row r="608" spans="1:12">
       <c r="A608" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B608" t="s">
         <v>652</v>
@@ -29840,7 +29840,7 @@
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B609" t="s">
         <v>653</v>
@@ -29875,7 +29875,7 @@
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B610" t="s">
         <v>654</v>
@@ -29910,7 +29910,7 @@
     </row>
     <row r="611" spans="1:12">
       <c r="A611" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B611" t="s">
         <v>655</v>
@@ -30024,7 +30024,7 @@
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B614" t="s">
         <v>658</v>
@@ -30059,7 +30059,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B615" t="s">
         <v>659</v>
@@ -30094,7 +30094,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B616" t="s">
         <v>660</v>
@@ -30129,7 +30129,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B617" t="s">
         <v>661</v>
@@ -30164,7 +30164,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B618" t="s">
         <v>662</v>
@@ -30199,7 +30199,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B619" t="s">
         <v>663</v>
@@ -30272,7 +30272,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B621" t="s">
         <v>665</v>
@@ -30342,7 +30342,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B623" t="s">
         <v>667</v>
@@ -30377,7 +30377,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B624" t="s">
         <v>668</v>
@@ -30412,7 +30412,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B625" t="s">
         <v>669</v>
@@ -30447,7 +30447,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B626" t="s">
         <v>670</v>
@@ -30482,7 +30482,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B627" t="s">
         <v>671</v>
@@ -30631,7 +30631,7 @@
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B631" t="s">
         <v>675</v>
@@ -30739,7 +30739,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B634" t="s">
         <v>678</v>
@@ -30812,7 +30812,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B636" t="s">
         <v>680</v>
@@ -30847,7 +30847,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B637" t="s">
         <v>681</v>
@@ -30882,7 +30882,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B638" t="s">
         <v>682</v>
@@ -30917,7 +30917,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B639" t="s">
         <v>683</v>
@@ -30987,7 +30987,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B641" t="s">
         <v>685</v>
@@ -31060,7 +31060,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B643" t="s">
         <v>687</v>
@@ -31095,7 +31095,7 @@
     </row>
     <row r="644" spans="1:12">
       <c r="A644" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B644" t="s">
         <v>688</v>
@@ -31168,7 +31168,7 @@
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B646" t="s">
         <v>690</v>
@@ -31203,7 +31203,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B647" t="s">
         <v>691</v>
@@ -31238,7 +31238,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B648" t="s">
         <v>692</v>
@@ -31422,7 +31422,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B653" t="s">
         <v>697</v>
@@ -31457,7 +31457,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B654" t="s">
         <v>698</v>
@@ -31495,7 +31495,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B655" t="s">
         <v>699</v>
@@ -31530,7 +31530,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B656" t="s">
         <v>700</v>
@@ -31565,7 +31565,7 @@
     </row>
     <row r="657" spans="1:12">
       <c r="A657" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B657" t="s">
         <v>701</v>
@@ -31603,7 +31603,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B658" t="s">
         <v>702</v>
@@ -31676,7 +31676,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B660" t="s">
         <v>704</v>
@@ -31711,7 +31711,7 @@
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B661" t="s">
         <v>705</v>
@@ -31781,7 +31781,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B663" t="s">
         <v>707</v>
@@ -31816,7 +31816,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B664" t="s">
         <v>708</v>
@@ -31851,7 +31851,7 @@
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B665" t="s">
         <v>709</v>
@@ -31921,7 +31921,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B667" t="s">
         <v>711</v>
@@ -31959,7 +31959,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B668" t="s">
         <v>712</v>
@@ -31994,7 +31994,7 @@
     </row>
     <row r="669" spans="1:12">
       <c r="A669" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B669" t="s">
         <v>713</v>
@@ -32029,7 +32029,7 @@
     </row>
     <row r="670" spans="1:12">
       <c r="A670" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B670" t="s">
         <v>714</v>
@@ -32064,7 +32064,7 @@
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B671" t="s">
         <v>715</v>
@@ -32099,7 +32099,7 @@
     </row>
     <row r="672" spans="1:12">
       <c r="A672" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B672" t="s">
         <v>716</v>
@@ -32134,7 +32134,7 @@
     </row>
     <row r="673" spans="1:12">
       <c r="A673" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B673" t="s">
         <v>717</v>
@@ -32207,7 +32207,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B675" t="s">
         <v>719</v>
@@ -32242,7 +32242,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B676" t="s">
         <v>720</v>
@@ -32280,7 +32280,7 @@
     </row>
     <row r="677" spans="1:12">
       <c r="A677" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B677" t="s">
         <v>721</v>
@@ -32356,7 +32356,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B679" t="s">
         <v>723</v>
@@ -32394,7 +32394,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B680" t="s">
         <v>724</v>
@@ -32432,7 +32432,7 @@
     </row>
     <row r="681" spans="1:12">
       <c r="A681" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B681" t="s">
         <v>725</v>
@@ -32464,7 +32464,7 @@
     </row>
     <row r="682" spans="1:12">
       <c r="A682" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B682" t="s">
         <v>726</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-06 14:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6815" uniqueCount="2674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6815" uniqueCount="2676">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -1930,6 +1930,9 @@
     <t>20.22.0001.0018256.2026-49</t>
   </si>
   <si>
+    <t>20.22.0001.0018245.2026-55</t>
+  </si>
+  <si>
     <t>20.22.0001.0018236.2026-07</t>
   </si>
   <si>
@@ -2089,9 +2092,6 @@
     <t>20.22.0001.0020528.2026-09</t>
   </si>
   <si>
-    <t>20.22.0001.0020434.2026-25</t>
-  </si>
-  <si>
     <t>20.22.0001.0020420.2026-15</t>
   </si>
   <si>
@@ -3949,6 +3949,9 @@
     <t>2026.0304</t>
   </si>
   <si>
+    <t>2026.0303</t>
+  </si>
+  <si>
     <t>2026.0302</t>
   </si>
   <si>
@@ -4108,9 +4111,6 @@
     <t>2026.0349</t>
   </si>
   <si>
-    <t>2026.0347</t>
-  </si>
-  <si>
     <t>2026.0346</t>
   </si>
   <si>
@@ -5251,156 +5251,156 @@
     <t>DANIEL FONTANA OBERLING,IZABEL REGINA BENITE AGUIAR DA SILVA</t>
   </si>
   <si>
+    <t>DAGER SALLES AMARAL,LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>REINALDO DE SOUZA MACHADO</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO</t>
+  </si>
+  <si>
+    <t>DAGER SALLES AMARAL</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI,HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>RAQUEL SILVA FERNANDES LYRA</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,MARINA DE AQUINO PARREIRA XAVIER,PEDRO DE OLIVEIRA PERES,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>PATRÍCIA FINAMORE ARAÚJO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>GLAUCO CASTILHO DE ALMEIDA,MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
+  </si>
+  <si>
+    <t>PAULA DE ARAUJO CRUZ VIGIO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>RENATA PASCOAL FREIRE,ROSEMARY RODRIGUES CRUZ,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
+    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO</t>
+  </si>
+  <si>
+    <t>MARCELO SILVA DE AZEVEDO</t>
+  </si>
+  <si>
+    <t>RENATA PASCOAL FREIRE</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,SIMONE MANNHEIMER DE ALVARENGA,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>PATRICIA FONTES ESTEVES</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>MARCELO KOLBLINGER DE GODOY</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO,ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
     <t>JOELSON SANTANA DE CARVALHO</t>
   </si>
   <si>
-    <t>DAGER SALLES AMARAL,LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO</t>
-  </si>
-  <si>
-    <t>DAGER SALLES AMARAL</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI,HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>RAQUEL SILVA FERNANDES LYRA</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,MARINA DE AQUINO PARREIRA XAVIER,PEDRO DE OLIVEIRA PERES,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>PATRÍCIA FINAMORE ARAÚJO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>GLAUCO CASTILHO DE ALMEIDA,MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
-  </si>
-  <si>
-    <t>PAULA DE ARAUJO CRUZ VIGIO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE,ROSEMARY RODRIGUES CRUZ,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
-    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO</t>
-  </si>
-  <si>
-    <t>MARCELO SILVA DE AZEVEDO</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE</t>
-  </si>
-  <si>
     <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
   </si>
   <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,SIMONE MANNHEIMER DE ALVARENGA,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>PATRICIA FONTES ESTEVES</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>MARCELO KOLBLINGER DE GODOY</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO,ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
     <t>ERIKA CANTANHEDE WUILLAUME,MARCELO TEIXEIRA SANTANA</t>
   </si>
   <si>
@@ -7108,6 +7108,9 @@
     <t>202500650662</t>
   </si>
   <si>
+    <t>202100813199</t>
+  </si>
+  <si>
     <t>202501227870</t>
   </si>
   <si>
@@ -7258,9 +7261,6 @@
     <t>201101145301</t>
   </si>
   <si>
-    <t>202600341107</t>
-  </si>
-  <si>
     <t>202400657916</t>
   </si>
   <si>
@@ -7954,7 +7954,7 @@
     <t>ASSISTÊNCIA SOCIAL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7987,13 +7987,13 @@
     <t>AVALIAÇÃO DE IMÓVEIS,BIOLOGIA,URBANISMO</t>
   </si>
   <si>
-    <t>URBANISMO,BIOLOGIA</t>
+    <t>GEOLOGIA,ENGENHARIA QUÍMICA</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>ORÇAMENTO,RECURSOS HÍDRICOS</t>
@@ -8005,21 +8005,24 @@
     <t>ECONOMIA,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
+    <t>RECURSOS HÍDRICOS,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
+  </si>
+  <si>
+    <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOTECNIA,ENGENHARIA QUÍMICA</t>
+  </si>
+  <si>
     <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
-  </si>
-  <si>
-    <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>GEOTECNIA,BIOLOGIA,ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
@@ -8035,7 +8038,10 @@
     <t>BIOLOGIA,GEOLOGIA</t>
   </si>
   <si>
-    <t>URBANISMO,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,SAÚDE,ORÇAMENTO,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ECONOMIA,ASSISTÊNCIA SOCIAL</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>SAÚDE MENTAL,PSICOLOGIA,ASSISTÊNCIA SOCIAL,ECONOMICIDADE CONTÁBIL,ORÇAMENTO,URBANISMO,AVALIAÇÃO DE IMÓVEIS,SAÚDE,MOBILIDADE E TRANSPORTE,ECONOMIA</t>
   </si>
 </sst>
 </file>
@@ -16108,7 +16114,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B220" t="s">
         <v>267</v>
@@ -16129,7 +16135,7 @@
         <v>1621</v>
       </c>
       <c r="I220" t="s">
-        <v>1724</v>
+        <v>1700</v>
       </c>
       <c r="J220" t="s">
         <v>2007</v>
@@ -17441,7 +17447,7 @@
     </row>
     <row r="258" spans="1:12">
       <c r="A258" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B258" t="s">
         <v>305</v>
@@ -17462,7 +17468,7 @@
         <v>1621</v>
       </c>
       <c r="I258" t="s">
-        <v>1724</v>
+        <v>1700</v>
       </c>
       <c r="J258" t="s">
         <v>2043</v>
@@ -18375,7 +18381,7 @@
         <v>1621</v>
       </c>
       <c r="I284" t="s">
-        <v>1745</v>
+        <v>1665</v>
       </c>
       <c r="J284" t="s">
         <v>2069</v>
@@ -18445,7 +18451,7 @@
         <v>1621</v>
       </c>
       <c r="I286" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="J286" t="s">
         <v>2071</v>
@@ -18865,7 +18871,7 @@
         <v>1621</v>
       </c>
       <c r="I298" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J298" t="s">
         <v>2083</v>
@@ -18935,7 +18941,7 @@
         <v>1621</v>
       </c>
       <c r="I300" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J300" t="s">
         <v>1919</v>
@@ -19180,7 +19186,7 @@
         <v>1621</v>
       </c>
       <c r="I307" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J307" t="s">
         <v>2090</v>
@@ -19215,7 +19221,7 @@
         <v>1621</v>
       </c>
       <c r="I308" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="J308" t="s">
         <v>2091</v>
@@ -20271,7 +20277,7 @@
         <v>1621</v>
       </c>
       <c r="I338" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J338" t="s">
         <v>2119</v>
@@ -20376,7 +20382,7 @@
         <v>1621</v>
       </c>
       <c r="I341" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J341" t="s">
         <v>2122</v>
@@ -20446,7 +20452,7 @@
         <v>1621</v>
       </c>
       <c r="I343" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="J343" t="s">
         <v>2124</v>
@@ -20621,7 +20627,7 @@
         <v>1621</v>
       </c>
       <c r="I348" t="s">
-        <v>1754</v>
+        <v>1753</v>
       </c>
       <c r="J348" t="s">
         <v>2129</v>
@@ -20691,7 +20697,7 @@
         <v>1621</v>
       </c>
       <c r="I350" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="J350" t="s">
         <v>2131</v>
@@ -20726,7 +20732,7 @@
         <v>1621</v>
       </c>
       <c r="I351" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J351" t="s">
         <v>2132</v>
@@ -21429,7 +21435,7 @@
         <v>1621</v>
       </c>
       <c r="I371" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="J371" t="s">
         <v>2150</v>
@@ -21572,7 +21578,7 @@
         <v>1568</v>
       </c>
       <c r="I375" t="s">
-        <v>1757</v>
+        <v>1756</v>
       </c>
       <c r="J375" t="s">
         <v>2154</v>
@@ -21753,7 +21759,7 @@
         <v>1533</v>
       </c>
       <c r="I380" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="J380" t="s">
         <v>2159</v>
@@ -22103,7 +22109,7 @@
         <v>1621</v>
       </c>
       <c r="I390" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J390" t="s">
         <v>2169</v>
@@ -22488,7 +22494,7 @@
         <v>1621</v>
       </c>
       <c r="I401" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J401" t="s">
         <v>2180</v>
@@ -22523,7 +22529,7 @@
         <v>1621</v>
       </c>
       <c r="I402" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J402" t="s">
         <v>2181</v>
@@ -22567,7 +22573,7 @@
         <v>2474</v>
       </c>
       <c r="L403" t="s">
-        <v>2611</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="404" spans="1:12">
@@ -22710,7 +22716,7 @@
         <v>2504</v>
       </c>
       <c r="L407" t="s">
-        <v>2657</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22736,7 +22742,7 @@
         <v>1621</v>
       </c>
       <c r="I408" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J408" t="s">
         <v>2187</v>
@@ -22806,7 +22812,7 @@
         <v>1621</v>
       </c>
       <c r="I410" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J410" t="s">
         <v>2189</v>
@@ -23051,7 +23057,7 @@
         <v>1621</v>
       </c>
       <c r="I417" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J417" t="s">
         <v>2196</v>
@@ -23121,7 +23127,7 @@
         <v>1621</v>
       </c>
       <c r="I419" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J419" t="s">
         <v>2198</v>
@@ -23261,7 +23267,7 @@
         <v>1621</v>
       </c>
       <c r="I423" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J423" t="s">
         <v>2202</v>
@@ -23331,7 +23337,7 @@
         <v>1621</v>
       </c>
       <c r="I425" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J425" t="s">
         <v>2203</v>
@@ -23611,7 +23617,7 @@
         <v>1621</v>
       </c>
       <c r="I433" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="J433" t="s">
         <v>2211</v>
@@ -24422,7 +24428,7 @@
         <v>1637</v>
       </c>
       <c r="I456" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J456" t="s">
         <v>2233</v>
@@ -24492,7 +24498,7 @@
         <v>1621</v>
       </c>
       <c r="I458" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J458" t="s">
         <v>2235</v>
@@ -24600,7 +24606,7 @@
         <v>1605</v>
       </c>
       <c r="I461" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
       <c r="J461" t="s">
         <v>2238</v>
@@ -24638,7 +24644,7 @@
         <v>1605</v>
       </c>
       <c r="I462" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
       <c r="J462" t="s">
         <v>2238</v>
@@ -24673,7 +24679,7 @@
         <v>1621</v>
       </c>
       <c r="I463" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J463" t="s">
         <v>2239</v>
@@ -24781,7 +24787,7 @@
         <v>1621</v>
       </c>
       <c r="I466" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J466" t="s">
         <v>2242</v>
@@ -25096,7 +25102,7 @@
         <v>1621</v>
       </c>
       <c r="I475" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J475" t="s">
         <v>2251</v>
@@ -25134,7 +25140,7 @@
         <v>1639</v>
       </c>
       <c r="I476" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
       <c r="J476" t="s">
         <v>2252</v>
@@ -25274,7 +25280,7 @@
         <v>1621</v>
       </c>
       <c r="I480" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J480" t="s">
         <v>2086</v>
@@ -25519,7 +25525,7 @@
         <v>1621</v>
       </c>
       <c r="I487" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J487" t="s">
         <v>2262</v>
@@ -25554,7 +25560,7 @@
         <v>1621</v>
       </c>
       <c r="I488" t="s">
-        <v>1770</v>
+        <v>1769</v>
       </c>
       <c r="J488" t="s">
         <v>2263</v>
@@ -25659,7 +25665,7 @@
         <v>1621</v>
       </c>
       <c r="I491" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J491" t="s">
         <v>2266</v>
@@ -25907,7 +25913,7 @@
         <v>1621</v>
       </c>
       <c r="I498" t="s">
-        <v>1771</v>
+        <v>1770</v>
       </c>
       <c r="J498" t="s">
         <v>2273</v>
@@ -25956,7 +25962,7 @@
     </row>
     <row r="500" spans="1:12">
       <c r="A500" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B500" t="s">
         <v>546</v>
@@ -25980,7 +25986,7 @@
         <v>1641</v>
       </c>
       <c r="I500" t="s">
-        <v>1772</v>
+        <v>1700</v>
       </c>
       <c r="J500" t="s">
         <v>2275</v>
@@ -26015,7 +26021,7 @@
         <v>1621</v>
       </c>
       <c r="I501" t="s">
-        <v>1773</v>
+        <v>1771</v>
       </c>
       <c r="J501" t="s">
         <v>2276</v>
@@ -26228,7 +26234,7 @@
         <v>1642</v>
       </c>
       <c r="I507" t="s">
-        <v>1774</v>
+        <v>1772</v>
       </c>
       <c r="J507" t="s">
         <v>2282</v>
@@ -26406,7 +26412,7 @@
         <v>1621</v>
       </c>
       <c r="I512" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J512" t="s">
         <v>2287</v>
@@ -26511,7 +26517,7 @@
         <v>1621</v>
       </c>
       <c r="I515" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J515" t="s">
         <v>2290</v>
@@ -26581,7 +26587,7 @@
         <v>1621</v>
       </c>
       <c r="I517" t="s">
-        <v>1775</v>
+        <v>1773</v>
       </c>
       <c r="J517" t="s">
         <v>2292</v>
@@ -26616,7 +26622,7 @@
         <v>1621</v>
       </c>
       <c r="I518" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J518" t="s">
         <v>2293</v>
@@ -26689,7 +26695,7 @@
         <v>1612</v>
       </c>
       <c r="I520" t="s">
-        <v>1776</v>
+        <v>1774</v>
       </c>
       <c r="J520" t="s">
         <v>2295</v>
@@ -26724,7 +26730,7 @@
         <v>1621</v>
       </c>
       <c r="I521" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J521" t="s">
         <v>2296</v>
@@ -27007,7 +27013,7 @@
         <v>1621</v>
       </c>
       <c r="I529" t="s">
-        <v>1777</v>
+        <v>1775</v>
       </c>
       <c r="J529" t="s">
         <v>2304</v>
@@ -27118,7 +27124,7 @@
         <v>1607</v>
       </c>
       <c r="I532" t="s">
-        <v>1778</v>
+        <v>1776</v>
       </c>
       <c r="J532" t="s">
         <v>2307</v>
@@ -27503,7 +27509,7 @@
         <v>1621</v>
       </c>
       <c r="I543" t="s">
-        <v>1779</v>
+        <v>1777</v>
       </c>
       <c r="J543" t="s">
         <v>2318</v>
@@ -27783,7 +27789,7 @@
         <v>1621</v>
       </c>
       <c r="I551" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J551" t="s">
         <v>2326</v>
@@ -27891,7 +27897,7 @@
         <v>1645</v>
       </c>
       <c r="I554" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J554" t="s">
         <v>2329</v>
@@ -27926,7 +27932,7 @@
         <v>1621</v>
       </c>
       <c r="I555" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J555" t="s">
         <v>2330</v>
@@ -27961,7 +27967,7 @@
         <v>1621</v>
       </c>
       <c r="I556" t="s">
-        <v>1781</v>
+        <v>1779</v>
       </c>
       <c r="J556" t="s">
         <v>2331</v>
@@ -27996,7 +28002,7 @@
         <v>1621</v>
       </c>
       <c r="I557" t="s">
-        <v>1782</v>
+        <v>1780</v>
       </c>
       <c r="J557" t="s">
         <v>2332</v>
@@ -28031,7 +28037,7 @@
         <v>1621</v>
       </c>
       <c r="I558" t="s">
-        <v>1783</v>
+        <v>1781</v>
       </c>
       <c r="J558" t="s">
         <v>2333</v>
@@ -28101,7 +28107,7 @@
         <v>1621</v>
       </c>
       <c r="I560" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J560" t="s">
         <v>1874</v>
@@ -28174,7 +28180,7 @@
         <v>1596</v>
       </c>
       <c r="I562" t="s">
-        <v>1774</v>
+        <v>1772</v>
       </c>
       <c r="J562" t="s">
         <v>2336</v>
@@ -28349,7 +28355,7 @@
         <v>1621</v>
       </c>
       <c r="I567" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J567" t="s">
         <v>2181</v>
@@ -28594,7 +28600,7 @@
         <v>1621</v>
       </c>
       <c r="I574" t="s">
-        <v>1754</v>
+        <v>1753</v>
       </c>
       <c r="J574" t="s">
         <v>2347</v>
@@ -28664,7 +28670,7 @@
         <v>1621</v>
       </c>
       <c r="I576" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J576" t="s">
         <v>2088</v>
@@ -28699,7 +28705,7 @@
         <v>1621</v>
       </c>
       <c r="I577" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J577" t="s">
         <v>2349</v>
@@ -28734,7 +28740,7 @@
         <v>1621</v>
       </c>
       <c r="I578" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J578" t="s">
         <v>2350</v>
@@ -28909,7 +28915,7 @@
         <v>1621</v>
       </c>
       <c r="I583" t="s">
-        <v>1784</v>
+        <v>1782</v>
       </c>
       <c r="J583" t="s">
         <v>2355</v>
@@ -28944,7 +28950,7 @@
         <v>1621</v>
       </c>
       <c r="I584" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J584" t="s">
         <v>2356</v>
@@ -28979,7 +28985,7 @@
         <v>1621</v>
       </c>
       <c r="I585" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J585" t="s">
         <v>2357</v>
@@ -29014,7 +29020,7 @@
         <v>1621</v>
       </c>
       <c r="I586" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J586" t="s">
         <v>2358</v>
@@ -29209,7 +29215,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B592" t="s">
         <v>638</v>
@@ -29230,21 +29236,21 @@
         <v>1621</v>
       </c>
       <c r="I592" t="s">
-        <v>1719</v>
+        <v>1768</v>
       </c>
       <c r="J592" t="s">
         <v>2364</v>
       </c>
       <c r="K592" t="s">
-        <v>2453</v>
+        <v>2499</v>
       </c>
       <c r="L592" t="s">
-        <v>2596</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B593" t="s">
         <v>639</v>
@@ -29265,21 +29271,21 @@
         <v>1621</v>
       </c>
       <c r="I593" t="s">
-        <v>1665</v>
+        <v>1719</v>
       </c>
       <c r="J593" t="s">
-        <v>1809</v>
+        <v>2365</v>
       </c>
       <c r="K593" t="s">
-        <v>2586</v>
+        <v>2453</v>
       </c>
       <c r="L593" t="s">
-        <v>2666</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B594" t="s">
         <v>640</v>
@@ -29300,16 +29306,16 @@
         <v>1621</v>
       </c>
       <c r="I594" t="s">
-        <v>1759</v>
+        <v>1665</v>
       </c>
       <c r="J594" t="s">
-        <v>2365</v>
+        <v>1809</v>
       </c>
       <c r="K594" t="s">
-        <v>2486</v>
+        <v>2586</v>
       </c>
       <c r="L594" t="s">
-        <v>2626</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -29335,7 +29341,7 @@
         <v>1621</v>
       </c>
       <c r="I595" t="s">
-        <v>1734</v>
+        <v>1758</v>
       </c>
       <c r="J595" t="s">
         <v>2366</v>
@@ -29376,7 +29382,7 @@
         <v>2367</v>
       </c>
       <c r="K596" t="s">
-        <v>2513</v>
+        <v>2486</v>
       </c>
       <c r="L596" t="s">
         <v>2626</v>
@@ -29384,7 +29390,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B597" t="s">
         <v>643</v>
@@ -29393,10 +29399,10 @@
         <v>1316</v>
       </c>
       <c r="D597" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="E597">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F597" t="s">
         <v>1616</v>
@@ -29405,21 +29411,21 @@
         <v>1621</v>
       </c>
       <c r="I597" t="s">
-        <v>1780</v>
+        <v>1734</v>
       </c>
       <c r="J597" t="s">
         <v>2368</v>
       </c>
       <c r="K597" t="s">
-        <v>2457</v>
+        <v>2513</v>
       </c>
       <c r="L597" t="s">
-        <v>2611</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B598" t="s">
         <v>644</v>
@@ -29440,16 +29446,16 @@
         <v>1621</v>
       </c>
       <c r="I598" t="s">
-        <v>1734</v>
+        <v>1778</v>
       </c>
       <c r="J598" t="s">
         <v>2369</v>
       </c>
       <c r="K598" t="s">
-        <v>2514</v>
+        <v>2457</v>
       </c>
       <c r="L598" t="s">
-        <v>2626</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="599" spans="1:12">
@@ -29475,21 +29481,21 @@
         <v>1621</v>
       </c>
       <c r="I599" t="s">
-        <v>1719</v>
+        <v>1734</v>
       </c>
       <c r="J599" t="s">
         <v>2370</v>
       </c>
       <c r="K599" t="s">
-        <v>2473</v>
+        <v>2514</v>
       </c>
       <c r="L599" t="s">
-        <v>2604</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B600" t="s">
         <v>646</v>
@@ -29510,16 +29516,16 @@
         <v>1621</v>
       </c>
       <c r="I600" t="s">
-        <v>1780</v>
+        <v>1719</v>
       </c>
       <c r="J600" t="s">
         <v>2371</v>
       </c>
       <c r="K600" t="s">
-        <v>2490</v>
+        <v>2473</v>
       </c>
       <c r="L600" t="s">
-        <v>2632</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="601" spans="1:12">
@@ -29545,21 +29551,21 @@
         <v>1621</v>
       </c>
       <c r="I601" t="s">
-        <v>1700</v>
+        <v>1778</v>
       </c>
       <c r="J601" t="s">
         <v>2372</v>
       </c>
       <c r="K601" t="s">
-        <v>2477</v>
+        <v>2490</v>
       </c>
       <c r="L601" t="s">
-        <v>2626</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B602" t="s">
         <v>648</v>
@@ -29580,7 +29586,7 @@
         <v>1621</v>
       </c>
       <c r="I602" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J602" t="s">
         <v>2373</v>
@@ -29589,12 +29595,12 @@
         <v>2477</v>
       </c>
       <c r="L602" t="s">
-        <v>2625</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B603" t="s">
         <v>649</v>
@@ -29615,21 +29621,21 @@
         <v>1621</v>
       </c>
       <c r="I603" t="s">
-        <v>1785</v>
+        <v>1699</v>
       </c>
       <c r="J603" t="s">
         <v>2374</v>
       </c>
       <c r="K603" t="s">
-        <v>2587</v>
+        <v>2477</v>
       </c>
       <c r="L603" t="s">
-        <v>2633</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B604" t="s">
         <v>650</v>
@@ -29638,36 +29644,33 @@
         <v>1323</v>
       </c>
       <c r="D604" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="E604">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F604" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G604" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H604" t="s">
-        <v>1542</v>
+        <v>1621</v>
       </c>
       <c r="I604" t="s">
-        <v>1780</v>
+        <v>1774</v>
       </c>
       <c r="J604" t="s">
-        <v>1874</v>
+        <v>2375</v>
       </c>
       <c r="K604" t="s">
-        <v>2466</v>
+        <v>2587</v>
       </c>
       <c r="L604" t="s">
-        <v>2667</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B605" t="s">
         <v>651</v>
@@ -29682,30 +29685,30 @@
         <v>14</v>
       </c>
       <c r="F605" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G605" t="s">
-        <v>1625</v>
+        <v>1623</v>
       </c>
       <c r="H605" t="s">
-        <v>1648</v>
+        <v>1542</v>
       </c>
       <c r="I605" t="s">
-        <v>1665</v>
+        <v>1778</v>
       </c>
       <c r="J605" t="s">
-        <v>2375</v>
+        <v>1874</v>
       </c>
       <c r="K605" t="s">
-        <v>2545</v>
+        <v>2466</v>
       </c>
       <c r="L605" t="s">
-        <v>2626</v>
+        <v>2667</v>
       </c>
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B606" t="s">
         <v>652</v>
@@ -29720,30 +29723,30 @@
         <v>14</v>
       </c>
       <c r="F606" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G606" t="s">
-        <v>1623</v>
+        <v>1625</v>
       </c>
       <c r="H606" t="s">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="I606" t="s">
-        <v>1772</v>
+        <v>1665</v>
       </c>
       <c r="J606" t="s">
         <v>2376</v>
       </c>
       <c r="K606" t="s">
-        <v>2476</v>
+        <v>2545</v>
       </c>
       <c r="L606" t="s">
-        <v>2663</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B607" t="s">
         <v>653</v>
@@ -29758,22 +29761,25 @@
         <v>14</v>
       </c>
       <c r="F607" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G607" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H607" t="s">
+        <v>1649</v>
       </c>
       <c r="I607" t="s">
-        <v>1726</v>
+        <v>1783</v>
       </c>
       <c r="J607" t="s">
         <v>2377</v>
       </c>
       <c r="K607" t="s">
-        <v>2454</v>
+        <v>2476</v>
       </c>
       <c r="L607" t="s">
-        <v>2604</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29799,21 +29805,21 @@
         <v>1621</v>
       </c>
       <c r="I608" t="s">
-        <v>1722</v>
+        <v>1726</v>
       </c>
       <c r="J608" t="s">
         <v>2378</v>
       </c>
       <c r="K608" t="s">
-        <v>2502</v>
+        <v>2454</v>
       </c>
       <c r="L608" t="s">
-        <v>2597</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B609" t="s">
         <v>655</v>
@@ -29834,21 +29840,21 @@
         <v>1621</v>
       </c>
       <c r="I609" t="s">
-        <v>1665</v>
+        <v>1722</v>
       </c>
       <c r="J609" t="s">
         <v>2379</v>
       </c>
       <c r="K609" t="s">
-        <v>2505</v>
+        <v>2502</v>
       </c>
       <c r="L609" t="s">
-        <v>2668</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B610" t="s">
         <v>656</v>
@@ -29869,21 +29875,21 @@
         <v>1621</v>
       </c>
       <c r="I610" t="s">
-        <v>1780</v>
+        <v>1665</v>
       </c>
       <c r="J610" t="s">
         <v>2380</v>
       </c>
       <c r="K610" t="s">
-        <v>2458</v>
+        <v>2505</v>
       </c>
       <c r="L610" t="s">
-        <v>2632</v>
+        <v>2669</v>
       </c>
     </row>
     <row r="611" spans="1:12">
       <c r="A611" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B611" t="s">
         <v>657</v>
@@ -29892,10 +29898,10 @@
         <v>1330</v>
       </c>
       <c r="D611" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="E611">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F611" t="s">
         <v>1616</v>
@@ -29904,21 +29910,21 @@
         <v>1621</v>
       </c>
       <c r="I611" t="s">
-        <v>1724</v>
+        <v>1778</v>
       </c>
       <c r="J611" t="s">
         <v>2381</v>
       </c>
       <c r="K611" t="s">
-        <v>2530</v>
+        <v>2458</v>
       </c>
       <c r="L611" t="s">
-        <v>2604</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B612" t="s">
         <v>658</v>
@@ -29933,30 +29939,27 @@
         <v>13</v>
       </c>
       <c r="F612" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G612" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H612" t="s">
-        <v>1650</v>
+        <v>1621</v>
       </c>
       <c r="I612" t="s">
-        <v>1786</v>
+        <v>1724</v>
       </c>
       <c r="J612" t="s">
         <v>2382</v>
       </c>
       <c r="K612" t="s">
-        <v>2452</v>
+        <v>2530</v>
       </c>
       <c r="L612" t="s">
-        <v>2644</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B613" t="s">
         <v>659</v>
@@ -29971,27 +29974,30 @@
         <v>13</v>
       </c>
       <c r="F613" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G613" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H613" t="s">
+        <v>1650</v>
       </c>
       <c r="I613" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
       <c r="J613" t="s">
         <v>2383</v>
       </c>
       <c r="K613" t="s">
-        <v>2556</v>
+        <v>2452</v>
       </c>
       <c r="L613" t="s">
-        <v>2633</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B614" t="s">
         <v>660</v>
@@ -30018,15 +30024,15 @@
         <v>2384</v>
       </c>
       <c r="K614" t="s">
-        <v>2477</v>
+        <v>2556</v>
       </c>
       <c r="L614" t="s">
-        <v>2625</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B615" t="s">
         <v>661</v>
@@ -30047,16 +30053,16 @@
         <v>1621</v>
       </c>
       <c r="I615" t="s">
-        <v>1734</v>
+        <v>1665</v>
       </c>
       <c r="J615" t="s">
         <v>2385</v>
       </c>
       <c r="K615" t="s">
-        <v>2470</v>
+        <v>2477</v>
       </c>
       <c r="L615" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="616" spans="1:12">
@@ -30082,7 +30088,7 @@
         <v>1621</v>
       </c>
       <c r="I616" t="s">
-        <v>1726</v>
+        <v>1734</v>
       </c>
       <c r="J616" t="s">
         <v>2386</v>
@@ -30091,12 +30097,12 @@
         <v>2470</v>
       </c>
       <c r="L616" t="s">
-        <v>2604</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B617" t="s">
         <v>663</v>
@@ -30105,10 +30111,10 @@
         <v>1336</v>
       </c>
       <c r="D617" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="E617">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F617" t="s">
         <v>1616</v>
@@ -30117,21 +30123,21 @@
         <v>1621</v>
       </c>
       <c r="I617" t="s">
-        <v>1785</v>
+        <v>1726</v>
       </c>
       <c r="J617" t="s">
         <v>2387</v>
       </c>
       <c r="K617" t="s">
-        <v>2541</v>
+        <v>2470</v>
       </c>
       <c r="L617" t="s">
-        <v>2615</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B618" t="s">
         <v>664</v>
@@ -30152,13 +30158,13 @@
         <v>1621</v>
       </c>
       <c r="I618" t="s">
-        <v>1785</v>
+        <v>1698</v>
       </c>
       <c r="J618" t="s">
         <v>2388</v>
       </c>
       <c r="K618" t="s">
-        <v>2499</v>
+        <v>2541</v>
       </c>
       <c r="L618" t="s">
         <v>2615</v>
@@ -30166,7 +30172,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B619" t="s">
         <v>665</v>
@@ -30187,21 +30193,21 @@
         <v>1621</v>
       </c>
       <c r="I619" t="s">
-        <v>1785</v>
+        <v>1741</v>
       </c>
       <c r="J619" t="s">
         <v>2389</v>
       </c>
       <c r="K619" t="s">
-        <v>2588</v>
+        <v>2499</v>
       </c>
       <c r="L619" t="s">
-        <v>2645</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B620" t="s">
         <v>666</v>
@@ -30216,30 +30222,27 @@
         <v>12</v>
       </c>
       <c r="F620" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G620" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H620" t="s">
-        <v>1651</v>
+        <v>1621</v>
       </c>
       <c r="I620" t="s">
-        <v>1753</v>
+        <v>1665</v>
       </c>
       <c r="J620" t="s">
         <v>2390</v>
       </c>
       <c r="K620" t="s">
-        <v>2564</v>
+        <v>2588</v>
       </c>
       <c r="L620" t="s">
-        <v>2600</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B621" t="s">
         <v>667</v>
@@ -30260,24 +30263,24 @@
         <v>1623</v>
       </c>
       <c r="H621" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="I621" t="s">
-        <v>1787</v>
+        <v>1752</v>
       </c>
       <c r="J621" t="s">
         <v>2391</v>
       </c>
       <c r="K621" t="s">
-        <v>2452</v>
+        <v>2564</v>
       </c>
       <c r="L621" t="s">
-        <v>2663</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B622" t="s">
         <v>668</v>
@@ -30298,24 +30301,24 @@
         <v>1623</v>
       </c>
       <c r="H622" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="I622" t="s">
-        <v>1665</v>
+        <v>1785</v>
       </c>
       <c r="J622" t="s">
         <v>2392</v>
       </c>
       <c r="K622" t="s">
-        <v>2506</v>
+        <v>2452</v>
       </c>
       <c r="L622" t="s">
-        <v>2626</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B623" t="s">
         <v>669</v>
@@ -30330,27 +30333,30 @@
         <v>12</v>
       </c>
       <c r="F623" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G623" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H623" t="s">
+        <v>1653</v>
       </c>
       <c r="I623" t="s">
-        <v>1722</v>
+        <v>1665</v>
       </c>
       <c r="J623" t="s">
         <v>2393</v>
       </c>
       <c r="K623" t="s">
-        <v>2526</v>
+        <v>2506</v>
       </c>
       <c r="L623" t="s">
-        <v>2632</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B624" t="s">
         <v>670</v>
@@ -30371,21 +30377,21 @@
         <v>1621</v>
       </c>
       <c r="I624" t="s">
-        <v>1712</v>
+        <v>1722</v>
       </c>
       <c r="J624" t="s">
         <v>2394</v>
       </c>
       <c r="K624" t="s">
-        <v>2581</v>
+        <v>2526</v>
       </c>
       <c r="L624" t="s">
-        <v>2631</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B625" t="s">
         <v>671</v>
@@ -30400,30 +30406,27 @@
         <v>12</v>
       </c>
       <c r="F625" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G625" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H625" t="s">
-        <v>1639</v>
+        <v>1621</v>
       </c>
       <c r="I625" t="s">
-        <v>1788</v>
+        <v>1712</v>
       </c>
       <c r="J625" t="s">
         <v>2395</v>
       </c>
       <c r="K625" t="s">
-        <v>2474</v>
+        <v>2581</v>
       </c>
       <c r="L625" t="s">
-        <v>2669</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B626" t="s">
         <v>672</v>
@@ -30441,24 +30444,27 @@
         <v>1617</v>
       </c>
       <c r="G626" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H626" t="s">
+        <v>1639</v>
       </c>
       <c r="I626" t="s">
-        <v>1665</v>
+        <v>1786</v>
       </c>
       <c r="J626" t="s">
         <v>2396</v>
       </c>
       <c r="K626" t="s">
-        <v>2449</v>
+        <v>2474</v>
       </c>
       <c r="L626" t="s">
-        <v>2626</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B627" t="s">
         <v>673</v>
@@ -30476,27 +30482,24 @@
         <v>1617</v>
       </c>
       <c r="G627" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H627" t="s">
-        <v>1651</v>
+        <v>1621</v>
       </c>
       <c r="I627" t="s">
-        <v>1714</v>
+        <v>1665</v>
       </c>
       <c r="J627" t="s">
         <v>2397</v>
       </c>
       <c r="K627" t="s">
-        <v>2453</v>
+        <v>2449</v>
       </c>
       <c r="L627" t="s">
-        <v>2604</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="628" spans="1:12">
       <c r="A628" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B628" t="s">
         <v>674</v>
@@ -30511,19 +30514,22 @@
         <v>12</v>
       </c>
       <c r="F628" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G628" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H628" t="s">
+        <v>1651</v>
       </c>
       <c r="I628" t="s">
-        <v>1726</v>
+        <v>1714</v>
       </c>
       <c r="J628" t="s">
         <v>2398</v>
       </c>
       <c r="K628" t="s">
-        <v>2514</v>
+        <v>2453</v>
       </c>
       <c r="L628" t="s">
         <v>2604</v>
@@ -30540,10 +30546,10 @@
         <v>1348</v>
       </c>
       <c r="D629" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="E629">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F629" t="s">
         <v>1616</v>
@@ -30552,13 +30558,13 @@
         <v>1621</v>
       </c>
       <c r="I629" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="J629" t="s">
         <v>2399</v>
       </c>
       <c r="K629" t="s">
-        <v>2589</v>
+        <v>2514</v>
       </c>
       <c r="L629" t="s">
         <v>2604</v>
@@ -30587,13 +30593,13 @@
         <v>1621</v>
       </c>
       <c r="I630" t="s">
-        <v>1719</v>
+        <v>1724</v>
       </c>
       <c r="J630" t="s">
         <v>2400</v>
       </c>
       <c r="K630" t="s">
-        <v>2524</v>
+        <v>2589</v>
       </c>
       <c r="L630" t="s">
         <v>2604</v>
@@ -30636,7 +30642,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B632" t="s">
         <v>678</v>
@@ -30657,21 +30663,21 @@
         <v>1621</v>
       </c>
       <c r="I632" t="s">
-        <v>1665</v>
+        <v>1719</v>
       </c>
       <c r="J632" t="s">
         <v>2402</v>
       </c>
       <c r="K632" t="s">
-        <v>2452</v>
+        <v>2524</v>
       </c>
       <c r="L632" t="s">
-        <v>2617</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B633" t="s">
         <v>679</v>
@@ -30692,21 +30698,21 @@
         <v>1621</v>
       </c>
       <c r="I633" t="s">
-        <v>1734</v>
+        <v>1665</v>
       </c>
       <c r="J633" t="s">
         <v>2403</v>
       </c>
       <c r="K633" t="s">
-        <v>2531</v>
+        <v>2452</v>
       </c>
       <c r="L633" t="s">
-        <v>2626</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B634" t="s">
         <v>680</v>
@@ -30721,30 +30727,27 @@
         <v>11</v>
       </c>
       <c r="F634" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G634" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H634" t="s">
-        <v>1654</v>
+        <v>1621</v>
       </c>
       <c r="I634" t="s">
-        <v>1789</v>
+        <v>1734</v>
       </c>
       <c r="J634" t="s">
         <v>2404</v>
       </c>
       <c r="K634" t="s">
-        <v>2505</v>
+        <v>2531</v>
       </c>
       <c r="L634" t="s">
-        <v>2670</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B635" t="s">
         <v>681</v>
@@ -30759,27 +30762,30 @@
         <v>11</v>
       </c>
       <c r="F635" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G635" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H635" t="s">
+        <v>1654</v>
       </c>
       <c r="I635" t="s">
-        <v>1780</v>
+        <v>1787</v>
       </c>
       <c r="J635" t="s">
         <v>2405</v>
       </c>
       <c r="K635" t="s">
-        <v>2458</v>
+        <v>2505</v>
       </c>
       <c r="L635" t="s">
-        <v>2632</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B636" t="s">
         <v>682</v>
@@ -30800,21 +30806,21 @@
         <v>1621</v>
       </c>
       <c r="I636" t="s">
-        <v>1759</v>
+        <v>1778</v>
       </c>
       <c r="J636" t="s">
         <v>2406</v>
       </c>
       <c r="K636" t="s">
-        <v>2590</v>
+        <v>2458</v>
       </c>
       <c r="L636" t="s">
-        <v>2626</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B637" t="s">
         <v>683</v>
@@ -30829,30 +30835,27 @@
         <v>11</v>
       </c>
       <c r="F637" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G637" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H637" t="s">
-        <v>1655</v>
+        <v>1621</v>
       </c>
       <c r="I637" t="s">
-        <v>1786</v>
+        <v>1758</v>
       </c>
       <c r="J637" t="s">
         <v>2407</v>
       </c>
       <c r="K637" t="s">
-        <v>2474</v>
+        <v>2590</v>
       </c>
       <c r="L637" t="s">
-        <v>2644</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B638" t="s">
         <v>684</v>
@@ -30867,22 +30870,25 @@
         <v>11</v>
       </c>
       <c r="F638" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G638" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H638" t="s">
+        <v>1655</v>
       </c>
       <c r="I638" t="s">
-        <v>1719</v>
+        <v>1784</v>
       </c>
       <c r="J638" t="s">
-        <v>1973</v>
+        <v>2408</v>
       </c>
       <c r="K638" t="s">
-        <v>2480</v>
+        <v>2474</v>
       </c>
       <c r="L638" t="s">
-        <v>2604</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30908,13 +30914,13 @@
         <v>1621</v>
       </c>
       <c r="I639" t="s">
-        <v>1724</v>
+        <v>1719</v>
       </c>
       <c r="J639" t="s">
-        <v>2408</v>
+        <v>1973</v>
       </c>
       <c r="K639" t="s">
-        <v>2575</v>
+        <v>2480</v>
       </c>
       <c r="L639" t="s">
         <v>2604</v>
@@ -30931,10 +30937,10 @@
         <v>1359</v>
       </c>
       <c r="D640" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="E640">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F640" t="s">
         <v>1616</v>
@@ -30943,13 +30949,13 @@
         <v>1621</v>
       </c>
       <c r="I640" t="s">
-        <v>1719</v>
+        <v>1724</v>
       </c>
       <c r="J640" t="s">
         <v>2409</v>
       </c>
       <c r="K640" t="s">
-        <v>2498</v>
+        <v>2575</v>
       </c>
       <c r="L640" t="s">
         <v>2604</v>
@@ -30957,7 +30963,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B641" t="s">
         <v>687</v>
@@ -30972,30 +30978,27 @@
         <v>10</v>
       </c>
       <c r="F641" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G641" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H641" t="s">
-        <v>1649</v>
+        <v>1621</v>
       </c>
       <c r="I641" t="s">
-        <v>1678</v>
+        <v>1719</v>
       </c>
       <c r="J641" t="s">
         <v>2410</v>
       </c>
       <c r="K641" t="s">
-        <v>2476</v>
+        <v>2498</v>
       </c>
       <c r="L641" t="s">
-        <v>2608</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="642" spans="1:12">
       <c r="A642" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B642" t="s">
         <v>688</v>
@@ -31010,27 +31013,30 @@
         <v>10</v>
       </c>
       <c r="F642" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G642" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H642" t="s">
+        <v>1649</v>
       </c>
       <c r="I642" t="s">
-        <v>1665</v>
+        <v>1678</v>
       </c>
       <c r="J642" t="s">
         <v>2411</v>
       </c>
       <c r="K642" t="s">
-        <v>2480</v>
+        <v>2476</v>
       </c>
       <c r="L642" t="s">
-        <v>2626</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B643" t="s">
         <v>689</v>
@@ -31045,25 +31051,22 @@
         <v>10</v>
       </c>
       <c r="F643" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G643" t="s">
-        <v>1623</v>
-      </c>
-      <c r="H643" t="s">
-        <v>1656</v>
+        <v>1621</v>
       </c>
       <c r="I643" t="s">
-        <v>1699</v>
+        <v>1665</v>
       </c>
       <c r="J643" t="s">
         <v>2412</v>
       </c>
       <c r="K643" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="L643" t="s">
-        <v>2625</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="644" spans="1:12">
@@ -31089,24 +31092,24 @@
         <v>1623</v>
       </c>
       <c r="H644" t="s">
-        <v>1657</v>
+        <v>1656</v>
       </c>
       <c r="I644" t="s">
-        <v>1790</v>
+        <v>1699</v>
       </c>
       <c r="J644" t="s">
         <v>2413</v>
       </c>
       <c r="K644" t="s">
-        <v>2531</v>
+        <v>2477</v>
       </c>
       <c r="L644" t="s">
-        <v>2671</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B645" t="s">
         <v>691</v>
@@ -31121,22 +31124,25 @@
         <v>10</v>
       </c>
       <c r="F645" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="G645" t="s">
-        <v>1621</v>
+        <v>1623</v>
+      </c>
+      <c r="H645" t="s">
+        <v>1657</v>
       </c>
       <c r="I645" t="s">
-        <v>1785</v>
+        <v>1788</v>
       </c>
       <c r="J645" t="s">
         <v>2414</v>
       </c>
       <c r="K645" t="s">
-        <v>2588</v>
+        <v>2531</v>
       </c>
       <c r="L645" t="s">
-        <v>2632</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -31273,7 +31279,7 @@
         <v>1658</v>
       </c>
       <c r="I649" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
       <c r="J649" t="s">
         <v>2418</v>
@@ -31346,7 +31352,7 @@
         <v>1659</v>
       </c>
       <c r="I651" t="s">
-        <v>1792</v>
+        <v>1790</v>
       </c>
       <c r="J651" t="s">
         <v>2420</v>
@@ -31355,7 +31361,7 @@
         <v>2504</v>
       </c>
       <c r="L651" t="s">
-        <v>2672</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31451,7 +31457,7 @@
         <v>1621</v>
       </c>
       <c r="I654" t="s">
-        <v>1793</v>
+        <v>1791</v>
       </c>
       <c r="J654" t="s">
         <v>2423</v>
@@ -31486,7 +31492,7 @@
         <v>1621</v>
       </c>
       <c r="I655" t="s">
-        <v>1794</v>
+        <v>1792</v>
       </c>
       <c r="J655" t="s">
         <v>2424</v>
@@ -31591,7 +31597,7 @@
         <v>1621</v>
       </c>
       <c r="I658" t="s">
-        <v>1665</v>
+        <v>1793</v>
       </c>
       <c r="J658" t="s">
         <v>2427</v>
@@ -31629,7 +31635,7 @@
         <v>1660</v>
       </c>
       <c r="I659" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
       <c r="J659" t="s">
         <v>2428</v>
@@ -31664,7 +31670,7 @@
         <v>1621</v>
       </c>
       <c r="I660" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="J660" t="s">
         <v>2429</v>
@@ -31699,7 +31705,7 @@
         <v>1621</v>
       </c>
       <c r="I661" t="s">
-        <v>1785</v>
+        <v>1794</v>
       </c>
       <c r="J661" t="s">
         <v>2430</v>
@@ -31708,7 +31714,7 @@
         <v>2483</v>
       </c>
       <c r="L661" t="s">
-        <v>2632</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="662" spans="1:12">
@@ -31734,7 +31740,7 @@
         <v>1621</v>
       </c>
       <c r="I662" t="s">
-        <v>1785</v>
+        <v>1794</v>
       </c>
       <c r="J662" t="s">
         <v>2431</v>
@@ -32026,7 +32032,7 @@
         <v>1658</v>
       </c>
       <c r="I670" t="s">
-        <v>1776</v>
+        <v>1774</v>
       </c>
       <c r="J670" t="s">
         <v>2439</v>
@@ -32064,7 +32070,7 @@
         <v>1658</v>
       </c>
       <c r="I671" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
       <c r="J671" t="s">
         <v>2440</v>
@@ -32102,7 +32108,7 @@
         <v>1658</v>
       </c>
       <c r="I672" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
       <c r="J672" t="s">
         <v>2441</v>
@@ -32111,7 +32117,7 @@
         <v>2471</v>
       </c>
       <c r="L672" t="s">
-        <v>2632</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="673" spans="1:12">
@@ -32178,7 +32184,7 @@
         <v>2595</v>
       </c>
       <c r="L674" t="s">
-        <v>2634</v>
+        <v>2674</v>
       </c>
     </row>
     <row r="675" spans="1:12">
@@ -32210,7 +32216,7 @@
         <v>2595</v>
       </c>
       <c r="L675" t="s">
-        <v>2673</v>
+        <v>2675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-08 04:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -30370,7 +30370,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B622" t="s">
         <v>669</v>
@@ -30391,7 +30391,7 @@
         <v>1641</v>
       </c>
       <c r="I622" t="s">
-        <v>1780</v>
+        <v>1685</v>
       </c>
       <c r="J622" t="s">
         <v>2417</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-09 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -8011,7 +8011,7 @@
     <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
   </si>
   <si>
-    <t>GEOTECNIA,BIOLOGIA,ENGENHARIA QUÍMICA</t>
+    <t>ENGENHARIA QUÍMICA,BIOLOGIA,GEOTECNIA</t>
   </si>
   <si>
     <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
@@ -8029,16 +8029,16 @@
     <t>BIOLOGIA,GEOLOGIA</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA AMBIENTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
-    <t>ASSISTÊNCIA SOCIAL,URBANISMO,RECURSOS HÍDRICOS,BIOLOGIA,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>SAÚDE,AVALIAÇÃO DE IMÓVEIS,ASSISTÊNCIA SOCIAL,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ECONOMIA,PSICOLOGIA,ORÇAMENTO,URBANISMO,ECONOMICIDADE CONTÁBIL</t>
+    <t>ENGENHARIA FLORESTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
+    <t>ASSISTÊNCIA SOCIAL,RECURSOS HÍDRICOS,GEOLOGIA,BIOLOGIA,URBANISMO</t>
+  </si>
+  <si>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ORÇAMENTO,SAÚDE MENTAL,ECONOMIA,PSICOLOGIA,URBANISMO,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ASSISTÊNCIA SOCIAL</t>
   </si>
 </sst>
 </file>
@@ -31133,7 +31133,7 @@
         <v>2501</v>
       </c>
       <c r="L645" t="s">
-        <v>2671</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -31273,7 +31273,7 @@
         <v>2493</v>
       </c>
       <c r="L649" t="s">
-        <v>2672</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="650" spans="1:12">
@@ -31600,7 +31600,7 @@
         <v>2576</v>
       </c>
       <c r="L658" t="s">
-        <v>2642</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="659" spans="1:12">
@@ -31673,7 +31673,7 @@
         <v>2468</v>
       </c>
       <c r="L660" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="661" spans="1:12">
@@ -32160,7 +32160,7 @@
         <v>2597</v>
       </c>
       <c r="L674" t="s">
-        <v>2636</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="675" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-15 18:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5134,19 +5134,19 @@
     <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
   </si>
   <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>ANA LÍCIA SOUZA E SILVA</t>
+  </si>
+  <si>
     <t>SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>ANA LÍCIA SOUZA E SILVA</t>
   </si>
   <si>
     <t>EDUARDO COUTO SOLEDADE</t>
@@ -12743,7 +12743,7 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B126" t="s">
         <v>170</v>
@@ -12764,7 +12764,7 @@
         <v>1620</v>
       </c>
       <c r="I126" t="s">
-        <v>1706</v>
+        <v>1665</v>
       </c>
       <c r="J126" t="s">
         <v>1901</v>
@@ -12834,7 +12834,7 @@
         <v>1620</v>
       </c>
       <c r="I128" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J128" t="s">
         <v>1903</v>
@@ -12869,7 +12869,7 @@
         <v>1620</v>
       </c>
       <c r="I129" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
       <c r="J129" t="s">
         <v>1904</v>
@@ -12904,7 +12904,7 @@
         <v>1620</v>
       </c>
       <c r="I130" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
       <c r="J130" t="s">
         <v>1904</v>
@@ -12939,7 +12939,7 @@
         <v>1620</v>
       </c>
       <c r="I131" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J131" t="s">
         <v>1790</v>
@@ -13009,7 +13009,7 @@
         <v>1620</v>
       </c>
       <c r="I133" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="J133" t="s">
         <v>1906</v>
@@ -13079,7 +13079,7 @@
         <v>1620</v>
       </c>
       <c r="I135" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J135" t="s">
         <v>1908</v>
@@ -13114,7 +13114,7 @@
         <v>1620</v>
       </c>
       <c r="I136" t="s">
-        <v>1706</v>
+        <v>1710</v>
       </c>
       <c r="J136" t="s">
         <v>1909</v>
@@ -13260,7 +13260,7 @@
         <v>1620</v>
       </c>
       <c r="I140" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J140" t="s">
         <v>1912</v>
@@ -13295,7 +13295,7 @@
         <v>1620</v>
       </c>
       <c r="I141" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J141" t="s">
         <v>1913</v>
@@ -13610,7 +13610,7 @@
         <v>1623</v>
       </c>
       <c r="I150" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J150" t="s">
         <v>1922</v>
@@ -13788,7 +13788,7 @@
         <v>1620</v>
       </c>
       <c r="I155" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J155" t="s">
         <v>1927</v>
@@ -13928,7 +13928,7 @@
         <v>1620</v>
       </c>
       <c r="I159" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J159" t="s">
         <v>1931</v>
@@ -13963,7 +13963,7 @@
         <v>1620</v>
       </c>
       <c r="I160" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J160" t="s">
         <v>1931</v>
@@ -14558,7 +14558,7 @@
         <v>1620</v>
       </c>
       <c r="I177" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J177" t="s">
         <v>1948</v>
@@ -14908,7 +14908,7 @@
         <v>1620</v>
       </c>
       <c r="I187" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J187" t="s">
         <v>1958</v>
@@ -15223,7 +15223,7 @@
         <v>1620</v>
       </c>
       <c r="I196" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J196" t="s">
         <v>1967</v>
@@ -15506,7 +15506,7 @@
         <v>1620</v>
       </c>
       <c r="I204" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J204" t="s">
         <v>1974</v>
@@ -15996,7 +15996,7 @@
         <v>1620</v>
       </c>
       <c r="I218" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J218" t="s">
         <v>1790</v>
@@ -16066,7 +16066,7 @@
         <v>1620</v>
       </c>
       <c r="I220" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J220" t="s">
         <v>1988</v>
@@ -16139,7 +16139,7 @@
         <v>1630</v>
       </c>
       <c r="I222" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J222" t="s">
         <v>1790</v>
@@ -16384,7 +16384,7 @@
         <v>1620</v>
       </c>
       <c r="I229" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J229" t="s">
         <v>1996</v>
@@ -16398,7 +16398,7 @@
     </row>
     <row r="230" spans="1:12">
       <c r="A230" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="B230" t="s">
         <v>274</v>
@@ -16419,7 +16419,7 @@
         <v>1620</v>
       </c>
       <c r="I230" t="s">
-        <v>1721</v>
+        <v>1665</v>
       </c>
       <c r="J230" t="s">
         <v>1997</v>
@@ -16454,7 +16454,7 @@
         <v>1620</v>
       </c>
       <c r="I231" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J231" t="s">
         <v>1998</v>
@@ -16734,7 +16734,7 @@
         <v>1620</v>
       </c>
       <c r="I239" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J239" t="s">
         <v>2006</v>
@@ -16839,7 +16839,7 @@
         <v>1620</v>
       </c>
       <c r="I242" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J242" t="s">
         <v>2009</v>
@@ -18067,7 +18067,7 @@
         <v>1620</v>
       </c>
       <c r="I277" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J277" t="s">
         <v>2044</v>
@@ -18452,7 +18452,7 @@
         <v>1620</v>
       </c>
       <c r="I288" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J288" t="s">
         <v>2055</v>
@@ -19053,7 +19053,7 @@
         <v>1631</v>
       </c>
       <c r="I305" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J305" t="s">
         <v>2070</v>
@@ -19123,7 +19123,7 @@
         <v>1620</v>
       </c>
       <c r="I307" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J307" t="s">
         <v>2072</v>
@@ -19298,7 +19298,7 @@
         <v>1620</v>
       </c>
       <c r="I312" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J312" t="s">
         <v>2076</v>
@@ -19403,7 +19403,7 @@
         <v>1620</v>
       </c>
       <c r="I315" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J315" t="s">
         <v>2079</v>
@@ -19543,7 +19543,7 @@
         <v>1620</v>
       </c>
       <c r="I319" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J319" t="s">
         <v>2083</v>
@@ -19648,7 +19648,7 @@
         <v>1620</v>
       </c>
       <c r="I322" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J322" t="s">
         <v>2086</v>
@@ -19858,7 +19858,7 @@
         <v>1620</v>
       </c>
       <c r="I328" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J328" t="s">
         <v>2092</v>
@@ -20418,7 +20418,7 @@
         <v>1620</v>
       </c>
       <c r="I344" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J344" t="s">
         <v>2107</v>
@@ -20453,7 +20453,7 @@
         <v>1620</v>
       </c>
       <c r="I345" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J345" t="s">
         <v>2108</v>
@@ -21089,7 +21089,7 @@
         <v>1620</v>
       </c>
       <c r="I363" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J363" t="s">
         <v>2126</v>
@@ -22107,7 +22107,7 @@
         <v>1620</v>
       </c>
       <c r="I392" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J392" t="s">
         <v>2155</v>
@@ -22597,7 +22597,7 @@
         <v>1620</v>
       </c>
       <c r="I406" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J406" t="s">
         <v>2168</v>
@@ -22915,7 +22915,7 @@
         <v>1633</v>
       </c>
       <c r="I415" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J415" t="s">
         <v>2177</v>
@@ -23125,7 +23125,7 @@
         <v>1620</v>
       </c>
       <c r="I421" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J421" t="s">
         <v>2182</v>
@@ -23545,7 +23545,7 @@
         <v>1620</v>
       </c>
       <c r="I433" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J433" t="s">
         <v>2194</v>
@@ -24076,7 +24076,7 @@
         <v>1620</v>
       </c>
       <c r="I448" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J448" t="s">
         <v>2209</v>
@@ -24111,7 +24111,7 @@
         <v>1620</v>
       </c>
       <c r="I449" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J449" t="s">
         <v>2210</v>
@@ -24356,7 +24356,7 @@
         <v>1620</v>
       </c>
       <c r="I456" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J456" t="s">
         <v>2217</v>
@@ -24461,7 +24461,7 @@
         <v>1620</v>
       </c>
       <c r="I459" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J459" t="s">
         <v>2220</v>
@@ -24636,7 +24636,7 @@
         <v>1620</v>
       </c>
       <c r="I464" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J464" t="s">
         <v>2225</v>
@@ -24709,7 +24709,7 @@
         <v>1620</v>
       </c>
       <c r="I466" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J466" t="s">
         <v>2227</v>
@@ -24779,7 +24779,7 @@
         <v>1620</v>
       </c>
       <c r="I468" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J468" t="s">
         <v>2229</v>
@@ -25024,7 +25024,7 @@
         <v>1620</v>
       </c>
       <c r="I475" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J475" t="s">
         <v>2236</v>
@@ -25167,7 +25167,7 @@
         <v>1637</v>
       </c>
       <c r="I479" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J479" t="s">
         <v>2240</v>
@@ -26045,7 +26045,7 @@
         <v>1620</v>
       </c>
       <c r="I504" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J504" t="s">
         <v>2265</v>
@@ -27028,7 +27028,7 @@
         <v>1620</v>
       </c>
       <c r="I532" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J532" t="s">
         <v>2292</v>
@@ -27133,7 +27133,7 @@
         <v>1620</v>
       </c>
       <c r="I535" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J535" t="s">
         <v>2295</v>
@@ -27343,7 +27343,7 @@
         <v>1620</v>
       </c>
       <c r="I541" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J541" t="s">
         <v>2300</v>
@@ -27661,7 +27661,7 @@
         <v>1620</v>
       </c>
       <c r="I550" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J550" t="s">
         <v>2309</v>
@@ -27906,7 +27906,7 @@
         <v>1620</v>
       </c>
       <c r="I557" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J557" t="s">
         <v>2315</v>
@@ -28119,7 +28119,7 @@
         <v>1620</v>
       </c>
       <c r="I563" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J563" t="s">
         <v>2321</v>
@@ -28580,7 +28580,7 @@
         <v>1620</v>
       </c>
       <c r="I576" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J576" t="s">
         <v>2334</v>
@@ -28793,7 +28793,7 @@
         <v>1620</v>
       </c>
       <c r="I582" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J582" t="s">
         <v>2340</v>
@@ -28828,7 +28828,7 @@
         <v>1620</v>
       </c>
       <c r="I583" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J583" t="s">
         <v>2341</v>
@@ -29006,7 +29006,7 @@
         <v>1620</v>
       </c>
       <c r="I588" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J588" t="s">
         <v>1947</v>
@@ -29076,7 +29076,7 @@
         <v>1620</v>
       </c>
       <c r="I590" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J590" t="s">
         <v>2347</v>
@@ -29254,7 +29254,7 @@
         <v>1620</v>
       </c>
       <c r="I595" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J595" t="s">
         <v>2352</v>
@@ -29715,7 +29715,7 @@
         <v>1620</v>
       </c>
       <c r="I608" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J608" t="s">
         <v>2365</v>
@@ -30036,7 +30036,7 @@
         <v>1620</v>
       </c>
       <c r="I617" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="J617" t="s">
         <v>2374</v>
@@ -30147,7 +30147,7 @@
         <v>1620</v>
       </c>
       <c r="I620" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J620" t="s">
         <v>2377</v>
@@ -30471,7 +30471,7 @@
         <v>1620</v>
       </c>
       <c r="I629" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J629" t="s">
         <v>2386</v>
@@ -30541,7 +30541,7 @@
         <v>1620</v>
       </c>
       <c r="I631" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J631" t="s">
         <v>2388</v>
@@ -30751,7 +30751,7 @@
         <v>1620</v>
       </c>
       <c r="I637" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J637" t="s">
         <v>2394</v>
@@ -31323,7 +31323,7 @@
         <v>1620</v>
       </c>
       <c r="I653" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J653" t="s">
         <v>2410</v>
@@ -31746,7 +31746,7 @@
         <v>1620</v>
       </c>
       <c r="I665" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J665" t="s">
         <v>2422</v>
@@ -31851,7 +31851,7 @@
         <v>1620</v>
       </c>
       <c r="I668" t="s">
-        <v>1665</v>
+        <v>1776</v>
       </c>
       <c r="J668" t="s">
         <v>2425</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-16 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -13245,7 +13245,7 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B140" t="s">
         <v>184</v>
@@ -13266,7 +13266,7 @@
         <v>1620</v>
       </c>
       <c r="I140" t="s">
-        <v>1705</v>
+        <v>1670</v>
       </c>
       <c r="J140" t="s">
         <v>1913</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-20 04:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5161,9 +5161,6 @@
     <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
   </si>
   <si>
-    <t>LILIAN ALVES DE ARAUJO</t>
-  </si>
-  <si>
     <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
   </si>
   <si>
@@ -5270,6 +5267,9 @@
   </si>
   <si>
     <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>LEONARDO DE SOUZA DA CONCEIÇÃO</t>
   </si>
   <si>
     <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,JULIANA MARTINS BAHIENSE,MARCELO TEIXEIRA SANTANA,MARINA DE AQUINO PARREIRA XAVIER,RENATA DE ARAUJO RIOS,RODRIGO VENTURA MARRA,SIMONE MANNHEIMER DE ALVARENGA</t>
@@ -19379,7 +19379,7 @@
     </row>
     <row r="318" spans="1:12">
       <c r="A318" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B318" t="s">
         <v>362</v>
@@ -19400,7 +19400,7 @@
         <v>1602</v>
       </c>
       <c r="I318" t="s">
-        <v>1715</v>
+        <v>1645</v>
       </c>
       <c r="J318" t="s">
         <v>2061</v>
@@ -19610,7 +19610,7 @@
         <v>1602</v>
       </c>
       <c r="I324" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J324" t="s">
         <v>2067</v>
@@ -19855,7 +19855,7 @@
         <v>1602</v>
       </c>
       <c r="I331" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J331" t="s">
         <v>2074</v>
@@ -20275,7 +20275,7 @@
         <v>1602</v>
       </c>
       <c r="I343" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="J343" t="s">
         <v>2085</v>
@@ -20383,7 +20383,7 @@
         <v>1538</v>
       </c>
       <c r="I346" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="J346" t="s">
         <v>2088</v>
@@ -20841,7 +20841,7 @@
         <v>1602</v>
       </c>
       <c r="I359" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J359" t="s">
         <v>2101</v>
@@ -21016,7 +21016,7 @@
         <v>1602</v>
       </c>
       <c r="I364" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J364" t="s">
         <v>2106</v>
@@ -21509,7 +21509,7 @@
         <v>1602</v>
       </c>
       <c r="I378" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J378" t="s">
         <v>2120</v>
@@ -21684,7 +21684,7 @@
         <v>1602</v>
       </c>
       <c r="I383" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J383" t="s">
         <v>2125</v>
@@ -21754,7 +21754,7 @@
         <v>1602</v>
       </c>
       <c r="I385" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J385" t="s">
         <v>2127</v>
@@ -21894,7 +21894,7 @@
         <v>1602</v>
       </c>
       <c r="I389" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J389" t="s">
         <v>2131</v>
@@ -21964,7 +21964,7 @@
         <v>1602</v>
       </c>
       <c r="I391" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J391" t="s">
         <v>2132</v>
@@ -21999,7 +21999,7 @@
         <v>1602</v>
       </c>
       <c r="I392" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J392" t="s">
         <v>2133</v>
@@ -22139,7 +22139,7 @@
         <v>1602</v>
       </c>
       <c r="I396" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J396" t="s">
         <v>2137</v>
@@ -22209,7 +22209,7 @@
         <v>1602</v>
       </c>
       <c r="I398" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J398" t="s">
         <v>2139</v>
@@ -22279,7 +22279,7 @@
         <v>1602</v>
       </c>
       <c r="I400" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J400" t="s">
         <v>2141</v>
@@ -22527,7 +22527,7 @@
         <v>1602</v>
       </c>
       <c r="I407" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J407" t="s">
         <v>2147</v>
@@ -22702,7 +22702,7 @@
         <v>1602</v>
       </c>
       <c r="I412" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J412" t="s">
         <v>2152</v>
@@ -22912,7 +22912,7 @@
         <v>1602</v>
       </c>
       <c r="I418" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J418" t="s">
         <v>2158</v>
@@ -23020,7 +23020,7 @@
         <v>1617</v>
       </c>
       <c r="I421" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J421" t="s">
         <v>2161</v>
@@ -23090,7 +23090,7 @@
         <v>1602</v>
       </c>
       <c r="I423" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J423" t="s">
         <v>2163</v>
@@ -23195,7 +23195,7 @@
         <v>1602</v>
       </c>
       <c r="I426" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J426" t="s">
         <v>2166</v>
@@ -23303,7 +23303,7 @@
         <v>1602</v>
       </c>
       <c r="I429" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J429" t="s">
         <v>2169</v>
@@ -23688,7 +23688,7 @@
         <v>1602</v>
       </c>
       <c r="I440" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J440" t="s">
         <v>2180</v>
@@ -23933,7 +23933,7 @@
         <v>1602</v>
       </c>
       <c r="I447" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J447" t="s">
         <v>2187</v>
@@ -24076,7 +24076,7 @@
         <v>1619</v>
       </c>
       <c r="I451" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J451" t="s">
         <v>2191</v>
@@ -24321,7 +24321,7 @@
         <v>1602</v>
       </c>
       <c r="I458" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J458" t="s">
         <v>2198</v>
@@ -24531,7 +24531,7 @@
         <v>1602</v>
       </c>
       <c r="I464" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J464" t="s">
         <v>2204</v>
@@ -24674,7 +24674,7 @@
         <v>1602</v>
       </c>
       <c r="I468" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J468" t="s">
         <v>2208</v>
@@ -24779,7 +24779,7 @@
         <v>1602</v>
       </c>
       <c r="I471" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J471" t="s">
         <v>2211</v>
@@ -24849,7 +24849,7 @@
         <v>1602</v>
       </c>
       <c r="I473" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J473" t="s">
         <v>2213</v>
@@ -24884,7 +24884,7 @@
         <v>1602</v>
       </c>
       <c r="I474" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J474" t="s">
         <v>2214</v>
@@ -24954,7 +24954,7 @@
         <v>1602</v>
       </c>
       <c r="I476" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J476" t="s">
         <v>2216</v>
@@ -25199,7 +25199,7 @@
         <v>1602</v>
       </c>
       <c r="I483" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J483" t="s">
         <v>2223</v>
@@ -25272,7 +25272,7 @@
         <v>1577</v>
       </c>
       <c r="I485" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="J485" t="s">
         <v>2225</v>
@@ -25587,7 +25587,7 @@
         <v>1602</v>
       </c>
       <c r="I494" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J494" t="s">
         <v>2234</v>
@@ -25622,7 +25622,7 @@
         <v>1602</v>
       </c>
       <c r="I495" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
       <c r="J495" t="s">
         <v>2235</v>
@@ -25902,7 +25902,7 @@
         <v>1602</v>
       </c>
       <c r="I503" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J503" t="s">
         <v>2243</v>
@@ -26007,7 +26007,7 @@
         <v>1602</v>
       </c>
       <c r="I506" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J506" t="s">
         <v>2246</v>
@@ -26150,7 +26150,7 @@
         <v>1566</v>
       </c>
       <c r="I510" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="J510" t="s">
         <v>2250</v>
@@ -26570,7 +26570,7 @@
         <v>1602</v>
       </c>
       <c r="I522" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J522" t="s">
         <v>2028</v>
@@ -26640,7 +26640,7 @@
         <v>1602</v>
       </c>
       <c r="I524" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J524" t="s">
         <v>2262</v>
@@ -26815,7 +26815,7 @@
         <v>1602</v>
       </c>
       <c r="I529" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J529" t="s">
         <v>2267</v>
@@ -26850,7 +26850,7 @@
         <v>1602</v>
       </c>
       <c r="I530" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J530" t="s">
         <v>2268</v>
@@ -26885,7 +26885,7 @@
         <v>1602</v>
       </c>
       <c r="I531" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J531" t="s">
         <v>2269</v>
@@ -27098,7 +27098,7 @@
         <v>1602</v>
       </c>
       <c r="I537" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J537" t="s">
         <v>2274</v>
@@ -27308,7 +27308,7 @@
         <v>1602</v>
       </c>
       <c r="I543" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J543" t="s">
         <v>2280</v>
@@ -27378,7 +27378,7 @@
         <v>1602</v>
       </c>
       <c r="I545" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J545" t="s">
         <v>2282</v>
@@ -27416,7 +27416,7 @@
         <v>1622</v>
       </c>
       <c r="I546" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J546" t="s">
         <v>2283</v>
@@ -27556,7 +27556,7 @@
         <v>1602</v>
       </c>
       <c r="I550" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J550" t="s">
         <v>2287</v>
@@ -27839,7 +27839,7 @@
         <v>1623</v>
       </c>
       <c r="I558" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="J558" t="s">
         <v>2295</v>
@@ -27909,7 +27909,7 @@
         <v>1602</v>
       </c>
       <c r="I560" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="J560" t="s">
         <v>2297</v>
@@ -27982,7 +27982,7 @@
         <v>1594</v>
       </c>
       <c r="I562" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="J562" t="s">
         <v>2299</v>
@@ -28230,7 +28230,7 @@
         <v>1624</v>
       </c>
       <c r="I569" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J569" t="s">
         <v>2306</v>
@@ -28265,7 +28265,7 @@
         <v>1602</v>
       </c>
       <c r="I570" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J570" t="s">
         <v>2307</v>
@@ -28443,7 +28443,7 @@
         <v>1625</v>
       </c>
       <c r="I575" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J575" t="s">
         <v>2311</v>
@@ -28723,7 +28723,7 @@
         <v>1602</v>
       </c>
       <c r="I583" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J583" t="s">
         <v>2319</v>
@@ -29149,7 +29149,7 @@
         <v>1602</v>
       </c>
       <c r="I595" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J595" t="s">
         <v>2331</v>
@@ -29254,7 +29254,7 @@
         <v>1602</v>
       </c>
       <c r="I598" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="J598" t="s">
         <v>2334</v>
@@ -29292,7 +29292,7 @@
         <v>1628</v>
       </c>
       <c r="I599" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J599" t="s">
         <v>2335</v>
@@ -29330,7 +29330,7 @@
         <v>1629</v>
       </c>
       <c r="I600" t="s">
-        <v>1645</v>
+        <v>1751</v>
       </c>
       <c r="J600" t="s">
         <v>2336</v>
@@ -29435,7 +29435,7 @@
         <v>1602</v>
       </c>
       <c r="I603" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J603" t="s">
         <v>2339</v>
@@ -29473,7 +29473,7 @@
         <v>1587</v>
       </c>
       <c r="I604" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J604" t="s">
         <v>2340</v>
@@ -29508,7 +29508,7 @@
         <v>1602</v>
       </c>
       <c r="I605" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J605" t="s">
         <v>2341</v>
@@ -29756,7 +29756,7 @@
         <v>1602</v>
       </c>
       <c r="I612" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J612" t="s">
         <v>2348</v>
@@ -29966,7 +29966,7 @@
         <v>1602</v>
       </c>
       <c r="I618" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J618" t="s">
         <v>2354</v>
@@ -30176,7 +30176,7 @@
         <v>1602</v>
       </c>
       <c r="I624" t="s">
-        <v>1645</v>
+        <v>1731</v>
       </c>
       <c r="J624" t="s">
         <v>2360</v>
@@ -30214,7 +30214,7 @@
         <v>1631</v>
       </c>
       <c r="I625" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J625" t="s">
         <v>2361</v>
@@ -30249,7 +30249,7 @@
         <v>1602</v>
       </c>
       <c r="I626" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J626" t="s">
         <v>2362</v>
@@ -30398,7 +30398,7 @@
         <v>1592</v>
       </c>
       <c r="I630" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J630" t="s">
         <v>2366</v>
@@ -30678,7 +30678,7 @@
         <v>1602</v>
       </c>
       <c r="I638" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J638" t="s">
         <v>2374</v>
@@ -30961,7 +30961,7 @@
         <v>1602</v>
       </c>
       <c r="I646" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J646" t="s">
         <v>2382</v>
@@ -31101,7 +31101,7 @@
         <v>1602</v>
       </c>
       <c r="I650" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J650" t="s">
         <v>2386</v>
@@ -31174,7 +31174,7 @@
         <v>1634</v>
       </c>
       <c r="I652" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J652" t="s">
         <v>2388</v>
@@ -31209,7 +31209,7 @@
         <v>1602</v>
       </c>
       <c r="I653" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J653" t="s">
         <v>2389</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-20 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -17710,7 +17710,7 @@
     </row>
     <row r="268" spans="1:12">
       <c r="A268" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B268" t="s">
         <v>310</v>
@@ -17731,7 +17731,7 @@
         <v>1618</v>
       </c>
       <c r="I268" t="s">
-        <v>1678</v>
+        <v>1659</v>
       </c>
       <c r="J268" t="s">
         <v>2029</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-21 12:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4984,18 +4984,21 @@
     <t>RODRIGO VALENTE SERRA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>REGINA SILBERSTEIN RACHEVSKY</t>
+  </si>
+  <si>
     <t>_SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO, EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>REGINA SILBERSTEIN RACHEVSKY</t>
-  </si>
-  <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,FERNANDA FERREIRA FONTES</t>
   </si>
   <si>
@@ -5024,9 +5027,6 @@
   </si>
   <si>
     <t>LILIAN ALVES DE ARAUJO,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>RODRIGO VENTURA MARRA</t>
@@ -8945,7 +8945,7 @@
         <v>1618</v>
       </c>
       <c r="I18" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J18" t="s">
         <v>1786</v>
@@ -8980,7 +8980,7 @@
         <v>1618</v>
       </c>
       <c r="I19" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J19" t="s">
         <v>1787</v>
@@ -9015,7 +9015,7 @@
         <v>1618</v>
       </c>
       <c r="I20" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J20" t="s">
         <v>1788</v>
@@ -9050,7 +9050,7 @@
         <v>1618</v>
       </c>
       <c r="I21" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J21" t="s">
         <v>1789</v>
@@ -9085,7 +9085,7 @@
         <v>1618</v>
       </c>
       <c r="I22" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J22" t="s">
         <v>1790</v>
@@ -9120,7 +9120,7 @@
         <v>1618</v>
       </c>
       <c r="I23" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J23" t="s">
         <v>1791</v>
@@ -9155,7 +9155,7 @@
         <v>1618</v>
       </c>
       <c r="I24" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J24" t="s">
         <v>1792</v>
@@ -9225,7 +9225,7 @@
         <v>1618</v>
       </c>
       <c r="I26" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J26" t="s">
         <v>1794</v>
@@ -9260,7 +9260,7 @@
         <v>1618</v>
       </c>
       <c r="I27" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J27" t="s">
         <v>1790</v>
@@ -9295,7 +9295,7 @@
         <v>1618</v>
       </c>
       <c r="I28" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J28" t="s">
         <v>1795</v>
@@ -9330,7 +9330,7 @@
         <v>1618</v>
       </c>
       <c r="I29" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J29" t="s">
         <v>1796</v>
@@ -9365,7 +9365,7 @@
         <v>1618</v>
       </c>
       <c r="I30" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J30" t="s">
         <v>1797</v>
@@ -9400,7 +9400,7 @@
         <v>1618</v>
       </c>
       <c r="I31" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J31" t="s">
         <v>1798</v>
@@ -9435,7 +9435,7 @@
         <v>1618</v>
       </c>
       <c r="I32" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J32" t="s">
         <v>1799</v>
@@ -9470,7 +9470,7 @@
         <v>1618</v>
       </c>
       <c r="I33" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J33" t="s">
         <v>1800</v>
@@ -9505,7 +9505,7 @@
         <v>1618</v>
       </c>
       <c r="I34" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J34" t="s">
         <v>1801</v>
@@ -9540,7 +9540,7 @@
         <v>1618</v>
       </c>
       <c r="I35" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J35" t="s">
         <v>1802</v>
@@ -9575,7 +9575,7 @@
         <v>1618</v>
       </c>
       <c r="I36" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J36" t="s">
         <v>1803</v>
@@ -9610,7 +9610,7 @@
         <v>1618</v>
       </c>
       <c r="I37" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J37" t="s">
         <v>1804</v>
@@ -9645,7 +9645,7 @@
         <v>1618</v>
       </c>
       <c r="I38" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J38" t="s">
         <v>1805</v>
@@ -9680,7 +9680,7 @@
         <v>1618</v>
       </c>
       <c r="I39" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J39" t="s">
         <v>1806</v>
@@ -9750,7 +9750,7 @@
         <v>1618</v>
       </c>
       <c r="I41" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J41" t="s">
         <v>1808</v>
@@ -9925,7 +9925,7 @@
         <v>1618</v>
       </c>
       <c r="I46" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J46" t="s">
         <v>1813</v>
@@ -9960,7 +9960,7 @@
         <v>1618</v>
       </c>
       <c r="I47" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J47" t="s">
         <v>1814</v>
@@ -9995,7 +9995,7 @@
         <v>1618</v>
       </c>
       <c r="I48" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J48" t="s">
         <v>1815</v>
@@ -10030,7 +10030,7 @@
         <v>1618</v>
       </c>
       <c r="I49" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J49" t="s">
         <v>1816</v>
@@ -10065,7 +10065,7 @@
         <v>1618</v>
       </c>
       <c r="I50" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J50" t="s">
         <v>1817</v>
@@ -10100,7 +10100,7 @@
         <v>1618</v>
       </c>
       <c r="I51" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J51" t="s">
         <v>1818</v>
@@ -10205,7 +10205,7 @@
         <v>1618</v>
       </c>
       <c r="I54" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J54" t="s">
         <v>1821</v>
@@ -10240,7 +10240,7 @@
         <v>1618</v>
       </c>
       <c r="I55" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J55" t="s">
         <v>1822</v>
@@ -10278,7 +10278,7 @@
         <v>1624</v>
       </c>
       <c r="I56" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J56" t="s">
         <v>1823</v>
@@ -10313,7 +10313,7 @@
         <v>1618</v>
       </c>
       <c r="I57" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J57" t="s">
         <v>1824</v>
@@ -10348,7 +10348,7 @@
         <v>1618</v>
       </c>
       <c r="I58" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J58" t="s">
         <v>1825</v>
@@ -10383,7 +10383,7 @@
         <v>1618</v>
       </c>
       <c r="I59" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J59" t="s">
         <v>1826</v>
@@ -10666,7 +10666,7 @@
         <v>1618</v>
       </c>
       <c r="I67" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J67" t="s">
         <v>1834</v>
@@ -10701,7 +10701,7 @@
         <v>1618</v>
       </c>
       <c r="I68" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J68" t="s">
         <v>1835</v>
@@ -10771,7 +10771,7 @@
         <v>1618</v>
       </c>
       <c r="I70" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J70" t="s">
         <v>1837</v>
@@ -10806,7 +10806,7 @@
         <v>1618</v>
       </c>
       <c r="I71" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J71" t="s">
         <v>1838</v>
@@ -10841,7 +10841,7 @@
         <v>1618</v>
       </c>
       <c r="I72" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J72" t="s">
         <v>1839</v>
@@ -10911,7 +10911,7 @@
         <v>1618</v>
       </c>
       <c r="I74" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J74" t="s">
         <v>1841</v>
@@ -11054,7 +11054,7 @@
         <v>1618</v>
       </c>
       <c r="I78" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J78" t="s">
         <v>1845</v>
@@ -11089,7 +11089,7 @@
         <v>1618</v>
       </c>
       <c r="I79" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J79" t="s">
         <v>1846</v>
@@ -11124,7 +11124,7 @@
         <v>1618</v>
       </c>
       <c r="I80" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J80" t="s">
         <v>1847</v>
@@ -11159,7 +11159,7 @@
         <v>1618</v>
       </c>
       <c r="I81" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J81" t="s">
         <v>1848</v>
@@ -11264,7 +11264,7 @@
         <v>1618</v>
       </c>
       <c r="I84" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J84" t="s">
         <v>1851</v>
@@ -11334,7 +11334,7 @@
         <v>1618</v>
       </c>
       <c r="I86" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J86" t="s">
         <v>1853</v>
@@ -11369,7 +11369,7 @@
         <v>1618</v>
       </c>
       <c r="I87" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J87" t="s">
         <v>1854</v>
@@ -11547,7 +11547,7 @@
         <v>1618</v>
       </c>
       <c r="I92" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J92" t="s">
         <v>1859</v>
@@ -11617,7 +11617,7 @@
         <v>1618</v>
       </c>
       <c r="I94" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J94" t="s">
         <v>1861</v>
@@ -11687,7 +11687,7 @@
         <v>1618</v>
       </c>
       <c r="I96" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J96" t="s">
         <v>1863</v>
@@ -11792,7 +11792,7 @@
         <v>1618</v>
       </c>
       <c r="I99" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J99" t="s">
         <v>1866</v>
@@ -11830,7 +11830,7 @@
         <v>1524</v>
       </c>
       <c r="I100" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J100" t="s">
         <v>1867</v>
@@ -11865,7 +11865,7 @@
         <v>1618</v>
       </c>
       <c r="I101" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J101" t="s">
         <v>1868</v>
@@ -11900,7 +11900,7 @@
         <v>1618</v>
       </c>
       <c r="I102" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J102" t="s">
         <v>1869</v>
@@ -11970,7 +11970,7 @@
         <v>1618</v>
       </c>
       <c r="I104" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J104" t="s">
         <v>1871</v>
@@ -12075,7 +12075,7 @@
         <v>1618</v>
       </c>
       <c r="I107" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J107" t="s">
         <v>1874</v>
@@ -12145,7 +12145,7 @@
         <v>1618</v>
       </c>
       <c r="I109" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J109" t="s">
         <v>1876</v>
@@ -12218,7 +12218,7 @@
         <v>1618</v>
       </c>
       <c r="I111" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J111" t="s">
         <v>1878</v>
@@ -12358,7 +12358,7 @@
         <v>1618</v>
       </c>
       <c r="I115" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J115" t="s">
         <v>1882</v>
@@ -12393,7 +12393,7 @@
         <v>1618</v>
       </c>
       <c r="I116" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J116" t="s">
         <v>1883</v>
@@ -12428,7 +12428,7 @@
         <v>1618</v>
       </c>
       <c r="I117" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J117" t="s">
         <v>1884</v>
@@ -12463,7 +12463,7 @@
         <v>1618</v>
       </c>
       <c r="I118" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J118" t="s">
         <v>1885</v>
@@ -12498,7 +12498,7 @@
         <v>1618</v>
       </c>
       <c r="I119" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J119" t="s">
         <v>1886</v>
@@ -12848,7 +12848,7 @@
         <v>1618</v>
       </c>
       <c r="I129" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J129" t="s">
         <v>1894</v>
@@ -13029,7 +13029,7 @@
         <v>1618</v>
       </c>
       <c r="I134" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J134" t="s">
         <v>1898</v>
@@ -13099,7 +13099,7 @@
         <v>1618</v>
       </c>
       <c r="I136" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J136" t="s">
         <v>1900</v>
@@ -13204,7 +13204,7 @@
         <v>1618</v>
       </c>
       <c r="I139" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J139" t="s">
         <v>1903</v>
@@ -13239,7 +13239,7 @@
         <v>1618</v>
       </c>
       <c r="I140" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J140" t="s">
         <v>1904</v>
@@ -13347,7 +13347,7 @@
         <v>1618</v>
       </c>
       <c r="I143" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J143" t="s">
         <v>1907</v>
@@ -13382,7 +13382,7 @@
         <v>1618</v>
       </c>
       <c r="I144" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J144" t="s">
         <v>1908</v>
@@ -13417,7 +13417,7 @@
         <v>1618</v>
       </c>
       <c r="I145" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J145" t="s">
         <v>1909</v>
@@ -13487,7 +13487,7 @@
         <v>1618</v>
       </c>
       <c r="I147" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J147" t="s">
         <v>1911</v>
@@ -13522,7 +13522,7 @@
         <v>1618</v>
       </c>
       <c r="I148" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J148" t="s">
         <v>1912</v>
@@ -13662,7 +13662,7 @@
         <v>1618</v>
       </c>
       <c r="I152" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J152" t="s">
         <v>1915</v>
@@ -13732,7 +13732,7 @@
         <v>1618</v>
       </c>
       <c r="I154" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J154" t="s">
         <v>1917</v>
@@ -13767,7 +13767,7 @@
         <v>1618</v>
       </c>
       <c r="I155" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J155" t="s">
         <v>1918</v>
@@ -13802,7 +13802,7 @@
         <v>1618</v>
       </c>
       <c r="I156" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J156" t="s">
         <v>1919</v>
@@ -13837,7 +13837,7 @@
         <v>1618</v>
       </c>
       <c r="I157" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J157" t="s">
         <v>1920</v>
@@ -13872,7 +13872,7 @@
         <v>1618</v>
       </c>
       <c r="I158" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J158" t="s">
         <v>1921</v>
@@ -13907,7 +13907,7 @@
         <v>1618</v>
       </c>
       <c r="I159" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J159" t="s">
         <v>1922</v>
@@ -14047,7 +14047,7 @@
         <v>1618</v>
       </c>
       <c r="I163" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J163" t="s">
         <v>1926</v>
@@ -14082,7 +14082,7 @@
         <v>1618</v>
       </c>
       <c r="I164" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J164" t="s">
         <v>1927</v>
@@ -14152,7 +14152,7 @@
         <v>1618</v>
       </c>
       <c r="I166" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J166" t="s">
         <v>1929</v>
@@ -14257,7 +14257,7 @@
         <v>1618</v>
       </c>
       <c r="I169" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J169" t="s">
         <v>1932</v>
@@ -14292,7 +14292,7 @@
         <v>1618</v>
       </c>
       <c r="I170" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J170" t="s">
         <v>1933</v>
@@ -14362,7 +14362,7 @@
         <v>1618</v>
       </c>
       <c r="I172" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J172" t="s">
         <v>1935</v>
@@ -14467,7 +14467,7 @@
         <v>1618</v>
       </c>
       <c r="I175" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J175" t="s">
         <v>1938</v>
@@ -14572,7 +14572,7 @@
         <v>1618</v>
       </c>
       <c r="I178" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J178" t="s">
         <v>1941</v>
@@ -14607,7 +14607,7 @@
         <v>1618</v>
       </c>
       <c r="I179" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J179" t="s">
         <v>1942</v>
@@ -14712,7 +14712,7 @@
         <v>1618</v>
       </c>
       <c r="I182" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J182" t="s">
         <v>1945</v>
@@ -14747,7 +14747,7 @@
         <v>1618</v>
       </c>
       <c r="I183" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J183" t="s">
         <v>1946</v>
@@ -14817,7 +14817,7 @@
         <v>1618</v>
       </c>
       <c r="I185" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J185" t="s">
         <v>1948</v>
@@ -14922,7 +14922,7 @@
         <v>1618</v>
       </c>
       <c r="I188" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J188" t="s">
         <v>1951</v>
@@ -14960,7 +14960,7 @@
         <v>1531</v>
       </c>
       <c r="I189" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J189" t="s">
         <v>1952</v>
@@ -14995,7 +14995,7 @@
         <v>1618</v>
       </c>
       <c r="I190" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J190" t="s">
         <v>1953</v>
@@ -15100,7 +15100,7 @@
         <v>1618</v>
       </c>
       <c r="I193" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J193" t="s">
         <v>1782</v>
@@ -15240,7 +15240,7 @@
         <v>1618</v>
       </c>
       <c r="I197" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J197" t="s">
         <v>1959</v>
@@ -15310,7 +15310,7 @@
         <v>1618</v>
       </c>
       <c r="I199" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J199" t="s">
         <v>1961</v>
@@ -15380,7 +15380,7 @@
         <v>1618</v>
       </c>
       <c r="I201" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J201" t="s">
         <v>1782</v>
@@ -15415,7 +15415,7 @@
         <v>1618</v>
       </c>
       <c r="I202" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J202" t="s">
         <v>1963</v>
@@ -15450,7 +15450,7 @@
         <v>1618</v>
       </c>
       <c r="I203" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J203" t="s">
         <v>1964</v>
@@ -15485,7 +15485,7 @@
         <v>1618</v>
       </c>
       <c r="I204" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J204" t="s">
         <v>1965</v>
@@ -15590,7 +15590,7 @@
         <v>1618</v>
       </c>
       <c r="I207" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J207" t="s">
         <v>1968</v>
@@ -15660,7 +15660,7 @@
         <v>1618</v>
       </c>
       <c r="I209" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J209" t="s">
         <v>1969</v>
@@ -15730,7 +15730,7 @@
         <v>1618</v>
       </c>
       <c r="I211" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J211" t="s">
         <v>1971</v>
@@ -15803,7 +15803,7 @@
         <v>1618</v>
       </c>
       <c r="I213" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J213" t="s">
         <v>1972</v>
@@ -15838,7 +15838,7 @@
         <v>1618</v>
       </c>
       <c r="I214" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J214" t="s">
         <v>1973</v>
@@ -15908,7 +15908,7 @@
         <v>1618</v>
       </c>
       <c r="I216" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J216" t="s">
         <v>1975</v>
@@ -15943,7 +15943,7 @@
         <v>1618</v>
       </c>
       <c r="I217" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J217" t="s">
         <v>1976</v>
@@ -16118,7 +16118,7 @@
         <v>1618</v>
       </c>
       <c r="I222" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J222" t="s">
         <v>1981</v>
@@ -16188,7 +16188,7 @@
         <v>1618</v>
       </c>
       <c r="I224" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J224" t="s">
         <v>1983</v>
@@ -16258,7 +16258,7 @@
         <v>1618</v>
       </c>
       <c r="I226" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J226" t="s">
         <v>1985</v>
@@ -16328,7 +16328,7 @@
         <v>1618</v>
       </c>
       <c r="I228" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J228" t="s">
         <v>1987</v>
@@ -16398,7 +16398,7 @@
         <v>1618</v>
       </c>
       <c r="I230" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J230" t="s">
         <v>1989</v>
@@ -16538,7 +16538,7 @@
         <v>1618</v>
       </c>
       <c r="I234" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J234" t="s">
         <v>1993</v>
@@ -16608,7 +16608,7 @@
         <v>1618</v>
       </c>
       <c r="I236" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J236" t="s">
         <v>1995</v>
@@ -16678,7 +16678,7 @@
         <v>1618</v>
       </c>
       <c r="I238" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J238" t="s">
         <v>1997</v>
@@ -16748,7 +16748,7 @@
         <v>1618</v>
       </c>
       <c r="I240" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J240" t="s">
         <v>1999</v>
@@ -16783,7 +16783,7 @@
         <v>1618</v>
       </c>
       <c r="I241" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J241" t="s">
         <v>2000</v>
@@ -16853,7 +16853,7 @@
         <v>1618</v>
       </c>
       <c r="I243" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J243" t="s">
         <v>2002</v>
@@ -16923,7 +16923,7 @@
         <v>1618</v>
       </c>
       <c r="I245" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J245" t="s">
         <v>2004</v>
@@ -16958,7 +16958,7 @@
         <v>1618</v>
       </c>
       <c r="I246" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J246" t="s">
         <v>2005</v>
@@ -17028,7 +17028,7 @@
         <v>1618</v>
       </c>
       <c r="I248" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J248" t="s">
         <v>2007</v>
@@ -17133,7 +17133,7 @@
         <v>1618</v>
       </c>
       <c r="I251" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J251" t="s">
         <v>2010</v>
@@ -17203,7 +17203,7 @@
         <v>1618</v>
       </c>
       <c r="I253" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J253" t="s">
         <v>2012</v>
@@ -17238,7 +17238,7 @@
         <v>1618</v>
       </c>
       <c r="I254" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J254" t="s">
         <v>2013</v>
@@ -17346,7 +17346,7 @@
         <v>1618</v>
       </c>
       <c r="I257" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J257" t="s">
         <v>2016</v>
@@ -17521,7 +17521,7 @@
         <v>1618</v>
       </c>
       <c r="I262" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J262" t="s">
         <v>2021</v>
@@ -17556,7 +17556,7 @@
         <v>1618</v>
       </c>
       <c r="I263" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J263" t="s">
         <v>2022</v>
@@ -17591,7 +17591,7 @@
         <v>1618</v>
       </c>
       <c r="I264" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J264" t="s">
         <v>2023</v>
@@ -17731,7 +17731,7 @@
         <v>1618</v>
       </c>
       <c r="I268" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J268" t="s">
         <v>2027</v>
@@ -17801,7 +17801,7 @@
         <v>1618</v>
       </c>
       <c r="I270" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J270" t="s">
         <v>2029</v>
@@ -17836,7 +17836,7 @@
         <v>1618</v>
       </c>
       <c r="I271" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J271" t="s">
         <v>2030</v>
@@ -17871,7 +17871,7 @@
         <v>1618</v>
       </c>
       <c r="I272" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J272" t="s">
         <v>2031</v>
@@ -17906,7 +17906,7 @@
         <v>1618</v>
       </c>
       <c r="I273" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J273" t="s">
         <v>2032</v>
@@ -17976,7 +17976,7 @@
         <v>1618</v>
       </c>
       <c r="I275" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J275" t="s">
         <v>2034</v>
@@ -18011,7 +18011,7 @@
         <v>1618</v>
       </c>
       <c r="I276" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J276" t="s">
         <v>2035</v>
@@ -18151,7 +18151,7 @@
         <v>1618</v>
       </c>
       <c r="I280" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J280" t="s">
         <v>2038</v>
@@ -18186,7 +18186,7 @@
         <v>1618</v>
       </c>
       <c r="I281" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J281" t="s">
         <v>1782</v>
@@ -18221,7 +18221,7 @@
         <v>1618</v>
       </c>
       <c r="I282" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J282" t="s">
         <v>2039</v>
@@ -18256,7 +18256,7 @@
         <v>1618</v>
       </c>
       <c r="I283" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J283" t="s">
         <v>2040</v>
@@ -18291,7 +18291,7 @@
         <v>1618</v>
       </c>
       <c r="I284" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J284" t="s">
         <v>2041</v>
@@ -18326,7 +18326,7 @@
         <v>1618</v>
       </c>
       <c r="I285" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J285" t="s">
         <v>2042</v>
@@ -18431,7 +18431,7 @@
         <v>1618</v>
       </c>
       <c r="I288" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J288" t="s">
         <v>2044</v>
@@ -18469,7 +18469,7 @@
         <v>1542</v>
       </c>
       <c r="I289" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J289" t="s">
         <v>2045</v>
@@ -18504,7 +18504,7 @@
         <v>1618</v>
       </c>
       <c r="I290" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J290" t="s">
         <v>2046</v>
@@ -18609,7 +18609,7 @@
         <v>1618</v>
       </c>
       <c r="I293" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J293" t="s">
         <v>2049</v>
@@ -18644,7 +18644,7 @@
         <v>1618</v>
       </c>
       <c r="I294" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J294" t="s">
         <v>2050</v>
@@ -18679,7 +18679,7 @@
         <v>1618</v>
       </c>
       <c r="I295" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J295" t="s">
         <v>2051</v>
@@ -18752,7 +18752,7 @@
         <v>1618</v>
       </c>
       <c r="I297" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J297" t="s">
         <v>2053</v>
@@ -19032,7 +19032,7 @@
         <v>1618</v>
       </c>
       <c r="I305" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J305" t="s">
         <v>2060</v>
@@ -19102,7 +19102,7 @@
         <v>1618</v>
       </c>
       <c r="I307" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J307" t="s">
         <v>2062</v>
@@ -19137,7 +19137,7 @@
         <v>1618</v>
       </c>
       <c r="I308" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J308" t="s">
         <v>2063</v>
@@ -19172,7 +19172,7 @@
         <v>1618</v>
       </c>
       <c r="I309" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J309" t="s">
         <v>2064</v>
@@ -19242,7 +19242,7 @@
         <v>1618</v>
       </c>
       <c r="I311" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J311" t="s">
         <v>2066</v>
@@ -19347,7 +19347,7 @@
         <v>1618</v>
       </c>
       <c r="I314" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J314" t="s">
         <v>2069</v>
@@ -19522,7 +19522,7 @@
         <v>1618</v>
       </c>
       <c r="I319" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J319" t="s">
         <v>2074</v>
@@ -19557,7 +19557,7 @@
         <v>1618</v>
       </c>
       <c r="I320" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J320" t="s">
         <v>2075</v>
@@ -19592,7 +19592,7 @@
         <v>1618</v>
       </c>
       <c r="I321" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J321" t="s">
         <v>2076</v>
@@ -19627,7 +19627,7 @@
         <v>1618</v>
       </c>
       <c r="I322" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J322" t="s">
         <v>2077</v>
@@ -19662,7 +19662,7 @@
         <v>1618</v>
       </c>
       <c r="I323" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J323" t="s">
         <v>2078</v>
@@ -19767,7 +19767,7 @@
         <v>1618</v>
       </c>
       <c r="I326" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J326" t="s">
         <v>2081</v>
@@ -19837,7 +19837,7 @@
         <v>1618</v>
       </c>
       <c r="I328" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J328" t="s">
         <v>2083</v>
@@ -19872,7 +19872,7 @@
         <v>1618</v>
       </c>
       <c r="I329" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J329" t="s">
         <v>2084</v>
@@ -19907,7 +19907,7 @@
         <v>1618</v>
       </c>
       <c r="I330" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J330" t="s">
         <v>2085</v>
@@ -20082,7 +20082,7 @@
         <v>1618</v>
       </c>
       <c r="I335" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J335" t="s">
         <v>2089</v>
@@ -20117,7 +20117,7 @@
         <v>1618</v>
       </c>
       <c r="I336" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J336" t="s">
         <v>2090</v>
@@ -20152,7 +20152,7 @@
         <v>1618</v>
       </c>
       <c r="I337" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J337" t="s">
         <v>2091</v>
@@ -20222,7 +20222,7 @@
         <v>1618</v>
       </c>
       <c r="I339" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J339" t="s">
         <v>2093</v>
@@ -20257,7 +20257,7 @@
         <v>1618</v>
       </c>
       <c r="I340" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J340" t="s">
         <v>2094</v>
@@ -20292,7 +20292,7 @@
         <v>1618</v>
       </c>
       <c r="I341" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J341" t="s">
         <v>2095</v>
@@ -20327,7 +20327,7 @@
         <v>1618</v>
       </c>
       <c r="I342" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J342" t="s">
         <v>2096</v>
@@ -20505,7 +20505,7 @@
         <v>1618</v>
       </c>
       <c r="I347" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J347" t="s">
         <v>2101</v>
@@ -20540,7 +20540,7 @@
         <v>1618</v>
       </c>
       <c r="I348" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J348" t="s">
         <v>2102</v>
@@ -20645,7 +20645,7 @@
         <v>1618</v>
       </c>
       <c r="I351" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J351" t="s">
         <v>2105</v>
@@ -20750,7 +20750,7 @@
         <v>1618</v>
       </c>
       <c r="I354" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J354" t="s">
         <v>2108</v>
@@ -20820,7 +20820,7 @@
         <v>1618</v>
       </c>
       <c r="I356" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J356" t="s">
         <v>2110</v>
@@ -20855,7 +20855,7 @@
         <v>1618</v>
       </c>
       <c r="I357" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J357" t="s">
         <v>2111</v>
@@ -20925,7 +20925,7 @@
         <v>1618</v>
       </c>
       <c r="I359" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J359" t="s">
         <v>2113</v>
@@ -20960,7 +20960,7 @@
         <v>1618</v>
       </c>
       <c r="I360" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J360" t="s">
         <v>2114</v>
@@ -20995,7 +20995,7 @@
         <v>1618</v>
       </c>
       <c r="I361" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J361" t="s">
         <v>2115</v>
@@ -21030,7 +21030,7 @@
         <v>1618</v>
       </c>
       <c r="I362" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J362" t="s">
         <v>2116</v>
@@ -21065,7 +21065,7 @@
         <v>1618</v>
       </c>
       <c r="I363" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J363" t="s">
         <v>2117</v>
@@ -21205,7 +21205,7 @@
         <v>1618</v>
       </c>
       <c r="I367" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J367" t="s">
         <v>2121</v>
@@ -21275,7 +21275,7 @@
         <v>1618</v>
       </c>
       <c r="I369" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J369" t="s">
         <v>2123</v>
@@ -21310,7 +21310,7 @@
         <v>1618</v>
       </c>
       <c r="I370" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J370" t="s">
         <v>2124</v>
@@ -21383,7 +21383,7 @@
         <v>1618</v>
       </c>
       <c r="I372" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J372" t="s">
         <v>2126</v>
@@ -21418,7 +21418,7 @@
         <v>1618</v>
       </c>
       <c r="I373" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J373" t="s">
         <v>2127</v>
@@ -21453,7 +21453,7 @@
         <v>1618</v>
       </c>
       <c r="I374" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J374" t="s">
         <v>2128</v>
@@ -21488,7 +21488,7 @@
         <v>1618</v>
       </c>
       <c r="I375" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J375" t="s">
         <v>2129</v>
@@ -21628,7 +21628,7 @@
         <v>1618</v>
       </c>
       <c r="I379" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J379" t="s">
         <v>2133</v>
@@ -21663,7 +21663,7 @@
         <v>1618</v>
       </c>
       <c r="I380" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J380" t="s">
         <v>2134</v>
@@ -21733,7 +21733,7 @@
         <v>1618</v>
       </c>
       <c r="I382" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J382" t="s">
         <v>2136</v>
@@ -21838,7 +21838,7 @@
         <v>1618</v>
       </c>
       <c r="I385" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J385" t="s">
         <v>2139</v>
@@ -21943,7 +21943,7 @@
         <v>1618</v>
       </c>
       <c r="I388" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J388" t="s">
         <v>1790</v>
@@ -22083,7 +22083,7 @@
         <v>1618</v>
       </c>
       <c r="I392" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J392" t="s">
         <v>2145</v>
@@ -22188,7 +22188,7 @@
         <v>1618</v>
       </c>
       <c r="I395" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J395" t="s">
         <v>2148</v>
@@ -22328,7 +22328,7 @@
         <v>1618</v>
       </c>
       <c r="I399" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J399" t="s">
         <v>2152</v>
@@ -22401,7 +22401,7 @@
         <v>1618</v>
       </c>
       <c r="I401" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J401" t="s">
         <v>2078</v>
@@ -22436,7 +22436,7 @@
         <v>1618</v>
       </c>
       <c r="I402" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J402" t="s">
         <v>2154</v>
@@ -22471,7 +22471,7 @@
         <v>1618</v>
       </c>
       <c r="I403" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J403" t="s">
         <v>2155</v>
@@ -22611,7 +22611,7 @@
         <v>1618</v>
       </c>
       <c r="I407" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J407" t="s">
         <v>2159</v>
@@ -22646,7 +22646,7 @@
         <v>1618</v>
       </c>
       <c r="I408" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J408" t="s">
         <v>2160</v>
@@ -22681,7 +22681,7 @@
         <v>1618</v>
       </c>
       <c r="I409" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J409" t="s">
         <v>2161</v>
@@ -22786,7 +22786,7 @@
         <v>1618</v>
       </c>
       <c r="I412" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J412" t="s">
         <v>2164</v>
@@ -22821,7 +22821,7 @@
         <v>1618</v>
       </c>
       <c r="I413" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J413" t="s">
         <v>2165</v>
@@ -23174,7 +23174,7 @@
         <v>1618</v>
       </c>
       <c r="I423" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J423" t="s">
         <v>2175</v>
@@ -23282,7 +23282,7 @@
         <v>1634</v>
       </c>
       <c r="I426" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J426" t="s">
         <v>2178</v>
@@ -23387,7 +23387,7 @@
         <v>1618</v>
       </c>
       <c r="I429" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J429" t="s">
         <v>2181</v>
@@ -23457,7 +23457,7 @@
         <v>1618</v>
       </c>
       <c r="I431" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J431" t="s">
         <v>2183</v>
@@ -23597,7 +23597,7 @@
         <v>1618</v>
       </c>
       <c r="I435" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J435" t="s">
         <v>2187</v>
@@ -23632,7 +23632,7 @@
         <v>1618</v>
       </c>
       <c r="I436" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J436" t="s">
         <v>2188</v>
@@ -23667,7 +23667,7 @@
         <v>1618</v>
       </c>
       <c r="I437" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J437" t="s">
         <v>2189</v>
@@ -23737,7 +23737,7 @@
         <v>1618</v>
       </c>
       <c r="I439" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J439" t="s">
         <v>2191</v>
@@ -23912,7 +23912,7 @@
         <v>1618</v>
       </c>
       <c r="I444" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J444" t="s">
         <v>2196</v>
@@ -23982,7 +23982,7 @@
         <v>1618</v>
       </c>
       <c r="I446" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J446" t="s">
         <v>2198</v>
@@ -24160,7 +24160,7 @@
         <v>1618</v>
       </c>
       <c r="I451" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J451" t="s">
         <v>2203</v>
@@ -24230,7 +24230,7 @@
         <v>1618</v>
       </c>
       <c r="I453" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J453" t="s">
         <v>2205</v>
@@ -24618,7 +24618,7 @@
         <v>1618</v>
       </c>
       <c r="I464" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J464" t="s">
         <v>2216</v>
@@ -24723,7 +24723,7 @@
         <v>1618</v>
       </c>
       <c r="I467" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J467" t="s">
         <v>2219</v>
@@ -24758,7 +24758,7 @@
         <v>1618</v>
       </c>
       <c r="I468" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J468" t="s">
         <v>2220</v>
@@ -25073,7 +25073,7 @@
         <v>1618</v>
       </c>
       <c r="I477" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J477" t="s">
         <v>2229</v>
@@ -25248,7 +25248,7 @@
         <v>1618</v>
       </c>
       <c r="I482" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J482" t="s">
         <v>2234</v>
@@ -25356,7 +25356,7 @@
         <v>1618</v>
       </c>
       <c r="I485" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J485" t="s">
         <v>2237</v>
@@ -25531,7 +25531,7 @@
         <v>1618</v>
       </c>
       <c r="I490" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J490" t="s">
         <v>2242</v>
@@ -25566,7 +25566,7 @@
         <v>1618</v>
       </c>
       <c r="I491" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J491" t="s">
         <v>2243</v>
@@ -25811,7 +25811,7 @@
         <v>1618</v>
       </c>
       <c r="I498" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J498" t="s">
         <v>2250</v>
@@ -25846,7 +25846,7 @@
         <v>1618</v>
       </c>
       <c r="I499" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J499" t="s">
         <v>2251</v>
@@ -25881,7 +25881,7 @@
         <v>1618</v>
       </c>
       <c r="I500" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J500" t="s">
         <v>2252</v>
@@ -25986,7 +25986,7 @@
         <v>1618</v>
       </c>
       <c r="I503" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J503" t="s">
         <v>2255</v>
@@ -26056,7 +26056,7 @@
         <v>1618</v>
       </c>
       <c r="I505" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J505" t="s">
         <v>2257</v>
@@ -26091,7 +26091,7 @@
         <v>1618</v>
       </c>
       <c r="I506" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J506" t="s">
         <v>2258</v>
@@ -26199,7 +26199,7 @@
         <v>1618</v>
       </c>
       <c r="I509" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J509" t="s">
         <v>2261</v>
@@ -26269,7 +26269,7 @@
         <v>1618</v>
       </c>
       <c r="I511" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J511" t="s">
         <v>2263</v>
@@ -26374,7 +26374,7 @@
         <v>1618</v>
       </c>
       <c r="I514" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J514" t="s">
         <v>2265</v>
@@ -26619,7 +26619,7 @@
         <v>1618</v>
       </c>
       <c r="I521" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J521" t="s">
         <v>2271</v>
@@ -26689,7 +26689,7 @@
         <v>1618</v>
       </c>
       <c r="I523" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J523" t="s">
         <v>2273</v>
@@ -26759,7 +26759,7 @@
         <v>1618</v>
       </c>
       <c r="I525" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J525" t="s">
         <v>2275</v>
@@ -26794,7 +26794,7 @@
         <v>1618</v>
       </c>
       <c r="I526" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J526" t="s">
         <v>2276</v>
@@ -27007,7 +27007,7 @@
         <v>1618</v>
       </c>
       <c r="I532" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J532" t="s">
         <v>2282</v>
@@ -27077,7 +27077,7 @@
         <v>1618</v>
       </c>
       <c r="I534" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J534" t="s">
         <v>1782</v>
@@ -27357,7 +27357,7 @@
         <v>1618</v>
       </c>
       <c r="I542" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J542" t="s">
         <v>2291</v>
@@ -27497,7 +27497,7 @@
         <v>1618</v>
       </c>
       <c r="I546" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J546" t="s">
         <v>2295</v>
@@ -27602,7 +27602,7 @@
         <v>1618</v>
       </c>
       <c r="I549" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J549" t="s">
         <v>2298</v>
@@ -27637,7 +27637,7 @@
         <v>1618</v>
       </c>
       <c r="I550" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J550" t="s">
         <v>2299</v>
@@ -27742,7 +27742,7 @@
         <v>1618</v>
       </c>
       <c r="I553" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J553" t="s">
         <v>2302</v>
@@ -27777,7 +27777,7 @@
         <v>1618</v>
       </c>
       <c r="I554" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J554" t="s">
         <v>2303</v>
@@ -28133,7 +28133,7 @@
         <v>1618</v>
       </c>
       <c r="I564" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J564" t="s">
         <v>2313</v>
@@ -28381,7 +28381,7 @@
         <v>1618</v>
       </c>
       <c r="I571" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J571" t="s">
         <v>2319</v>
@@ -28454,7 +28454,7 @@
         <v>1618</v>
       </c>
       <c r="I573" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J573" t="s">
         <v>2321</v>
@@ -28559,7 +28559,7 @@
         <v>1618</v>
       </c>
       <c r="I576" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J576" t="s">
         <v>2324</v>
@@ -28594,7 +28594,7 @@
         <v>1618</v>
       </c>
       <c r="I577" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J577" t="s">
         <v>2325</v>
@@ -28629,7 +28629,7 @@
         <v>1618</v>
       </c>
       <c r="I578" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J578" t="s">
         <v>2326</v>
@@ -28772,7 +28772,7 @@
         <v>1618</v>
       </c>
       <c r="I582" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J582" t="s">
         <v>2330</v>
@@ -28807,7 +28807,7 @@
         <v>1618</v>
       </c>
       <c r="I583" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J583" t="s">
         <v>2331</v>
@@ -29020,7 +29020,7 @@
         <v>1618</v>
       </c>
       <c r="I589" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J589" t="s">
         <v>2337</v>
@@ -29160,7 +29160,7 @@
         <v>1618</v>
       </c>
       <c r="I593" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J593" t="s">
         <v>2341</v>
@@ -29484,7 +29484,7 @@
         <v>1618</v>
       </c>
       <c r="I602" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J602" t="s">
         <v>2350</v>
@@ -29977,7 +29977,7 @@
         <v>1618</v>
       </c>
       <c r="I616" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J616" t="s">
         <v>2364</v>
@@ -30263,7 +30263,7 @@
         <v>1618</v>
       </c>
       <c r="I624" t="s">
-        <v>1656</v>
+        <v>1660</v>
       </c>
       <c r="J624" t="s">
         <v>2372</v>
@@ -30899,7 +30899,7 @@
         <v>1618</v>
       </c>
       <c r="I642" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J642" t="s">
         <v>2390</v>
@@ -31255,7 +31255,7 @@
         <v>1618</v>
       </c>
       <c r="I652" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J652" t="s">
         <v>2400</v>
@@ -31465,7 +31465,7 @@
         <v>1618</v>
       </c>
       <c r="I658" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J658" t="s">
         <v>2405</v>
@@ -31535,7 +31535,7 @@
         <v>1618</v>
       </c>
       <c r="I660" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J660" t="s">
         <v>2407</v>
@@ -31570,7 +31570,7 @@
         <v>1618</v>
       </c>
       <c r="I661" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J661" t="s">
         <v>2408</v>
@@ -31605,7 +31605,7 @@
         <v>1618</v>
       </c>
       <c r="I662" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J662" t="s">
         <v>2409</v>
@@ -31815,7 +31815,7 @@
         <v>1618</v>
       </c>
       <c r="I668" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J668" t="s">
         <v>2415</v>
@@ -31850,7 +31850,7 @@
         <v>1618</v>
       </c>
       <c r="I669" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J669" t="s">
         <v>2416</v>
@@ -31920,7 +31920,7 @@
         <v>1618</v>
       </c>
       <c r="I671" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J671" t="s">
         <v>2418</v>
@@ -31955,7 +31955,7 @@
         <v>1618</v>
       </c>
       <c r="I672" t="s">
-        <v>1670</v>
+        <v>1656</v>
       </c>
       <c r="J672" t="s">
         <v>2419</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-01 16:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -32388,7 +32388,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B680" t="s">
         <v>712</v>
@@ -32409,7 +32409,7 @@
         <v>1645</v>
       </c>
       <c r="I680" t="s">
-        <v>1779</v>
+        <v>1689</v>
       </c>
       <c r="J680" t="s">
         <v>2457</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-11 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -82,15 +82,15 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA</t>
   </si>
   <si>
@@ -5098,7 +5098,7 @@
     <t>RODRIGO VALENTE SERRA, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
-    <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
+    <t>CLAUDIA DA SILVA LUNARDI, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
     <t>LILIAN ALVES DE ARAUJO,SERGIO PEDRO LOPES,VANESSA FERNANDES LEÃO</t>
@@ -5293,6 +5293,9 @@
     <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
     <t>GIULIANA DE ANDRADE CERVAI, PABLO GINIO VIMERCATI SIMAS</t>
   </si>
   <si>
@@ -5345,9 +5348,6 @@
   </si>
   <si>
     <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
   </si>
   <si>
     <t>ITAMAR COSTA KALIL, VÍTOR MENDONÇA CELANE PINHEIRO</t>
@@ -10290,7 +10290,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B53" t="s">
         <v>92</v>
@@ -10325,7 +10325,7 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B54" t="s">
         <v>93</v>
@@ -10713,7 +10713,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B65" t="s">
         <v>104</v>
@@ -10783,7 +10783,7 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B67" t="s">
         <v>106</v>
@@ -10818,7 +10818,7 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B68" t="s">
         <v>107</v>
@@ -10853,7 +10853,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B69" t="s">
         <v>108</v>
@@ -11098,7 +11098,7 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B76" t="s">
         <v>115</v>
@@ -11206,7 +11206,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B79" t="s">
         <v>118</v>
@@ -11276,7 +11276,7 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B81" t="s">
         <v>120</v>
@@ -11384,7 +11384,7 @@
     </row>
     <row r="84" spans="1:12">
       <c r="A84" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B84" t="s">
         <v>123</v>
@@ -11842,7 +11842,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B97" t="s">
         <v>136</v>
@@ -11982,7 +11982,7 @@
     </row>
     <row r="101" spans="1:12">
       <c r="A101" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B101" t="s">
         <v>140</v>
@@ -12227,7 +12227,7 @@
     </row>
     <row r="108" spans="1:12">
       <c r="A108" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B108" t="s">
         <v>147</v>
@@ -12373,7 +12373,7 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B112" t="s">
         <v>151</v>
@@ -12583,7 +12583,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B118" t="s">
         <v>157</v>
@@ -12723,7 +12723,7 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B122" t="s">
         <v>161</v>
@@ -12793,7 +12793,7 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B124" t="s">
         <v>163</v>
@@ -13003,7 +13003,7 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B130" t="s">
         <v>169</v>
@@ -13388,7 +13388,7 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B141" t="s">
         <v>180</v>
@@ -13703,7 +13703,7 @@
     </row>
     <row r="150" spans="1:12">
       <c r="A150" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B150" t="s">
         <v>189</v>
@@ -13773,7 +13773,7 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B152" t="s">
         <v>191</v>
@@ -13913,7 +13913,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B156" t="s">
         <v>195</v>
@@ -14686,7 +14686,7 @@
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B178" t="s">
         <v>217</v>
@@ -15459,7 +15459,7 @@
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B200" t="s">
         <v>239</v>
@@ -15634,7 +15634,7 @@
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B205" t="s">
         <v>244</v>
@@ -15739,7 +15739,7 @@
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B208" t="s">
         <v>247</v>
@@ -16159,7 +16159,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B220" t="s">
         <v>258</v>
@@ -16264,7 +16264,7 @@
     </row>
     <row r="223" spans="1:12">
       <c r="A223" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B223" t="s">
         <v>261</v>
@@ -16369,7 +16369,7 @@
     </row>
     <row r="226" spans="1:12">
       <c r="A226" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B226" t="s">
         <v>264</v>
@@ -16404,7 +16404,7 @@
     </row>
     <row r="227" spans="1:12">
       <c r="A227" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B227" t="s">
         <v>265</v>
@@ -16439,7 +16439,7 @@
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B228" t="s">
         <v>266</v>
@@ -16509,7 +16509,7 @@
     </row>
     <row r="230" spans="1:12">
       <c r="A230" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B230" t="s">
         <v>268</v>
@@ -16789,7 +16789,7 @@
     </row>
     <row r="238" spans="1:12">
       <c r="A238" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B238" t="s">
         <v>276</v>
@@ -16964,7 +16964,7 @@
     </row>
     <row r="243" spans="1:12">
       <c r="A243" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B243" t="s">
         <v>281</v>
@@ -17107,7 +17107,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B247" t="s">
         <v>285</v>
@@ -17128,7 +17128,7 @@
         <v>1642</v>
       </c>
       <c r="I247" t="s">
-        <v>1733</v>
+        <v>1759</v>
       </c>
       <c r="J247" t="s">
         <v>2033</v>
@@ -17212,7 +17212,7 @@
     </row>
     <row r="250" spans="1:12">
       <c r="A250" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B250" t="s">
         <v>288</v>
@@ -17411,7 +17411,7 @@
         <v>1644</v>
       </c>
       <c r="I255" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="J255" t="s">
         <v>2041</v>
@@ -17530,7 +17530,7 @@
     </row>
     <row r="259" spans="1:12">
       <c r="A259" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B259" t="s">
         <v>297</v>
@@ -17656,7 +17656,7 @@
         <v>1642</v>
       </c>
       <c r="I262" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J262" t="s">
         <v>2048</v>
@@ -17691,7 +17691,7 @@
         <v>1642</v>
       </c>
       <c r="I263" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J263" t="s">
         <v>2049</v>
@@ -17705,7 +17705,7 @@
     </row>
     <row r="264" spans="1:12">
       <c r="A264" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B264" t="s">
         <v>302</v>
@@ -17726,7 +17726,7 @@
         <v>1642</v>
       </c>
       <c r="I264" t="s">
-        <v>1724</v>
+        <v>1759</v>
       </c>
       <c r="J264" t="s">
         <v>2050</v>
@@ -17761,7 +17761,7 @@
         <v>1642</v>
       </c>
       <c r="I265" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J265" t="s">
         <v>2051</v>
@@ -17915,7 +17915,7 @@
     </row>
     <row r="270" spans="1:12">
       <c r="A270" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B270" t="s">
         <v>308</v>
@@ -17936,7 +17936,7 @@
         <v>1642</v>
       </c>
       <c r="I270" t="s">
-        <v>1733</v>
+        <v>1759</v>
       </c>
       <c r="J270" t="s">
         <v>2056</v>
@@ -17971,7 +17971,7 @@
         <v>1642</v>
       </c>
       <c r="I271" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J271" t="s">
         <v>2057</v>
@@ -18160,7 +18160,7 @@
     </row>
     <row r="277" spans="1:12">
       <c r="A277" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B277" t="s">
         <v>315</v>
@@ -18216,7 +18216,7 @@
         <v>1642</v>
       </c>
       <c r="I278" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J278" t="s">
         <v>2064</v>
@@ -18251,7 +18251,7 @@
         <v>1642</v>
       </c>
       <c r="I279" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="J279" t="s">
         <v>2065</v>
@@ -18321,7 +18321,7 @@
         <v>1642</v>
       </c>
       <c r="I281" t="s">
-        <v>1764</v>
+        <v>1765</v>
       </c>
       <c r="J281" t="s">
         <v>2067</v>
@@ -18335,7 +18335,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B282" t="s">
         <v>320</v>
@@ -18461,7 +18461,7 @@
         <v>1642</v>
       </c>
       <c r="I285" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J285" t="s">
         <v>2071</v>
@@ -18496,7 +18496,7 @@
         <v>1642</v>
       </c>
       <c r="I286" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J286" t="s">
         <v>1898</v>
@@ -18881,7 +18881,7 @@
         <v>1642</v>
       </c>
       <c r="I297" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J297" t="s">
         <v>2082</v>
@@ -18989,7 +18989,7 @@
         <v>1563</v>
       </c>
       <c r="I300" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J300" t="s">
         <v>2085</v>
@@ -19038,7 +19038,7 @@
     </row>
     <row r="302" spans="1:12">
       <c r="A302" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B302" t="s">
         <v>340</v>
@@ -19283,7 +19283,7 @@
     </row>
     <row r="309" spans="1:12">
       <c r="A309" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B309" t="s">
         <v>347</v>
@@ -19374,7 +19374,7 @@
         <v>1642</v>
       </c>
       <c r="I311" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J311" t="s">
         <v>2096</v>
@@ -19479,7 +19479,7 @@
         <v>1642</v>
       </c>
       <c r="I314" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="J314" t="s">
         <v>2099</v>
@@ -19493,7 +19493,7 @@
     </row>
     <row r="315" spans="1:12">
       <c r="A315" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B315" t="s">
         <v>353</v>
@@ -19668,7 +19668,7 @@
     </row>
     <row r="320" spans="1:12">
       <c r="A320" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B320" t="s">
         <v>358</v>
@@ -19773,7 +19773,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B323" t="s">
         <v>361</v>
@@ -19867,7 +19867,7 @@
         <v>1642</v>
       </c>
       <c r="I325" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J325" t="s">
         <v>2110</v>
@@ -19916,7 +19916,7 @@
     </row>
     <row r="327" spans="1:12">
       <c r="A327" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B327" t="s">
         <v>365</v>
@@ -20112,7 +20112,7 @@
         <v>1642</v>
       </c>
       <c r="I332" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
       <c r="J332" t="s">
         <v>2117</v>
@@ -20217,7 +20217,7 @@
         <v>1642</v>
       </c>
       <c r="I335" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="J335" t="s">
         <v>2120</v>
@@ -20392,7 +20392,7 @@
         <v>1642</v>
       </c>
       <c r="I340" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J340" t="s">
         <v>2124</v>
@@ -20546,7 +20546,7 @@
     </row>
     <row r="345" spans="1:12">
       <c r="A345" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B345" t="s">
         <v>383</v>
@@ -20581,7 +20581,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B346" t="s">
         <v>384</v>
@@ -20654,7 +20654,7 @@
     </row>
     <row r="348" spans="1:12">
       <c r="A348" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B348" t="s">
         <v>386</v>
@@ -20689,7 +20689,7 @@
     </row>
     <row r="349" spans="1:12">
       <c r="A349" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B349" t="s">
         <v>387</v>
@@ -20815,7 +20815,7 @@
         <v>1642</v>
       </c>
       <c r="I352" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J352" t="s">
         <v>2135</v>
@@ -20934,7 +20934,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B356" t="s">
         <v>394</v>
@@ -21238,7 +21238,7 @@
         <v>1654</v>
       </c>
       <c r="I364" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
       <c r="J364" t="s">
         <v>2147</v>
@@ -21322,7 +21322,7 @@
     </row>
     <row r="367" spans="1:12">
       <c r="A367" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B367" t="s">
         <v>405</v>
@@ -21486,7 +21486,7 @@
         <v>1642</v>
       </c>
       <c r="I371" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="J371" t="s">
         <v>2154</v>
@@ -21535,7 +21535,7 @@
     </row>
     <row r="373" spans="1:12">
       <c r="A373" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B373" t="s">
         <v>411</v>
@@ -21605,7 +21605,7 @@
     </row>
     <row r="375" spans="1:12">
       <c r="A375" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B375" t="s">
         <v>413</v>
@@ -21766,7 +21766,7 @@
         <v>1642</v>
       </c>
       <c r="I379" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
       <c r="J379" t="s">
         <v>2162</v>
@@ -21871,7 +21871,7 @@
         <v>1642</v>
       </c>
       <c r="I382" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="J382" t="s">
         <v>2165</v>
@@ -22116,7 +22116,7 @@
         <v>1642</v>
       </c>
       <c r="I389" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J389" t="s">
         <v>2172</v>
@@ -22480,7 +22480,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B400" t="s">
         <v>438</v>
@@ -22501,7 +22501,7 @@
         <v>1642</v>
       </c>
       <c r="I400" t="s">
-        <v>1740</v>
+        <v>1759</v>
       </c>
       <c r="J400" t="s">
         <v>2183</v>
@@ -22693,7 +22693,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B406" t="s">
         <v>444</v>
@@ -22784,7 +22784,7 @@
         <v>1642</v>
       </c>
       <c r="I408" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J408" t="s">
         <v>2191</v>
@@ -22833,7 +22833,7 @@
     </row>
     <row r="410" spans="1:12">
       <c r="A410" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B410" t="s">
         <v>448</v>
@@ -22994,7 +22994,7 @@
         <v>1642</v>
       </c>
       <c r="I414" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J414" t="s">
         <v>2197</v>
@@ -23064,7 +23064,7 @@
         <v>1642</v>
       </c>
       <c r="I416" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J416" t="s">
         <v>2199</v>
@@ -23358,7 +23358,7 @@
     </row>
     <row r="425" spans="1:12">
       <c r="A425" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B425" t="s">
         <v>463</v>
@@ -23641,7 +23641,7 @@
     </row>
     <row r="433" spans="1:12">
       <c r="A433" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B433" t="s">
         <v>471</v>
@@ -23676,7 +23676,7 @@
     </row>
     <row r="434" spans="1:12">
       <c r="A434" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B434" t="s">
         <v>472</v>
@@ -23711,7 +23711,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B435" t="s">
         <v>473</v>
@@ -23886,7 +23886,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B440" t="s">
         <v>478</v>
@@ -23921,7 +23921,7 @@
     </row>
     <row r="441" spans="1:12">
       <c r="A441" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B441" t="s">
         <v>479</v>
@@ -24012,7 +24012,7 @@
         <v>1642</v>
       </c>
       <c r="I443" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J443" t="s">
         <v>2226</v>
@@ -24061,7 +24061,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B445" t="s">
         <v>483</v>
@@ -24117,7 +24117,7 @@
         <v>1642</v>
       </c>
       <c r="I446" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J446" t="s">
         <v>2229</v>
@@ -24680,7 +24680,7 @@
         <v>1642</v>
       </c>
       <c r="I462" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J462" t="s">
         <v>2026</v>
@@ -24764,7 +24764,7 @@
     </row>
     <row r="465" spans="1:12">
       <c r="A465" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B465" t="s">
         <v>503</v>
@@ -24834,7 +24834,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B467" t="s">
         <v>505</v>
@@ -24869,7 +24869,7 @@
     </row>
     <row r="468" spans="1:12">
       <c r="A468" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B468" t="s">
         <v>506</v>
@@ -25082,7 +25082,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B474" t="s">
         <v>512</v>
@@ -25208,7 +25208,7 @@
         <v>1642</v>
       </c>
       <c r="I477" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J477" t="s">
         <v>2257</v>
@@ -25782,7 +25782,7 @@
     </row>
     <row r="494" spans="1:12">
       <c r="A494" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B494" t="s">
         <v>532</v>
@@ -25887,7 +25887,7 @@
     </row>
     <row r="497" spans="1:12">
       <c r="A497" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B497" t="s">
         <v>535</v>
@@ -26631,7 +26631,7 @@
     </row>
     <row r="518" spans="1:12">
       <c r="A518" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B518" t="s">
         <v>556</v>
@@ -26841,7 +26841,7 @@
     </row>
     <row r="524" spans="1:12">
       <c r="A524" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B524" t="s">
         <v>562</v>
@@ -27212,7 +27212,7 @@
         <v>1642</v>
       </c>
       <c r="I534" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J534" t="s">
         <v>2314</v>
@@ -27226,7 +27226,7 @@
     </row>
     <row r="535" spans="1:12">
       <c r="A535" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B535" t="s">
         <v>573</v>
@@ -27422,7 +27422,7 @@
         <v>1642</v>
       </c>
       <c r="I540" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J540" t="s">
         <v>2320</v>
@@ -27492,7 +27492,7 @@
         <v>1642</v>
       </c>
       <c r="I542" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J542" t="s">
         <v>2322</v>
@@ -27632,7 +27632,7 @@
         <v>1642</v>
       </c>
       <c r="I546" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J546" t="s">
         <v>2326</v>
@@ -27786,7 +27786,7 @@
     </row>
     <row r="551" spans="1:12">
       <c r="A551" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B551" t="s">
         <v>589</v>
@@ -27856,7 +27856,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B553" t="s">
         <v>591</v>
@@ -27877,7 +27877,7 @@
         <v>1642</v>
       </c>
       <c r="I553" t="s">
-        <v>1733</v>
+        <v>1759</v>
       </c>
       <c r="J553" t="s">
         <v>2333</v>
@@ -27947,7 +27947,7 @@
         <v>1642</v>
       </c>
       <c r="I555" t="s">
-        <v>1786</v>
+        <v>1678</v>
       </c>
       <c r="J555" t="s">
         <v>2335</v>
@@ -28017,7 +28017,7 @@
         <v>1642</v>
       </c>
       <c r="I557" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J557" t="s">
         <v>2337</v>
@@ -28031,7 +28031,7 @@
     </row>
     <row r="558" spans="1:12">
       <c r="A558" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B558" t="s">
         <v>596</v>
@@ -28314,7 +28314,7 @@
     </row>
     <row r="566" spans="1:12">
       <c r="A566" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B566" t="s">
         <v>604</v>
@@ -28349,7 +28349,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B567" t="s">
         <v>605</v>
@@ -28489,7 +28489,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B571" t="s">
         <v>609</v>
@@ -28510,7 +28510,7 @@
         <v>1642</v>
       </c>
       <c r="I571" t="s">
-        <v>1724</v>
+        <v>1759</v>
       </c>
       <c r="J571" t="s">
         <v>2351</v>
@@ -28524,7 +28524,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B572" t="s">
         <v>610</v>
@@ -28664,7 +28664,7 @@
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B576" t="s">
         <v>614</v>
@@ -28874,7 +28874,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B582" t="s">
         <v>620</v>
@@ -28909,7 +28909,7 @@
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B583" t="s">
         <v>621</v>
@@ -28979,7 +28979,7 @@
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B585" t="s">
         <v>623</v>
@@ -29014,7 +29014,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B586" t="s">
         <v>624</v>
@@ -29049,7 +29049,7 @@
     </row>
     <row r="587" spans="1:12">
       <c r="A587" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B587" t="s">
         <v>625</v>
@@ -29084,7 +29084,7 @@
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B588" t="s">
         <v>626</v>
@@ -29402,7 +29402,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B597" t="s">
         <v>635</v>
@@ -29472,7 +29472,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B599" t="s">
         <v>637</v>
@@ -29542,7 +29542,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -29563,7 +29563,7 @@
         <v>1642</v>
       </c>
       <c r="I601" t="s">
-        <v>1733</v>
+        <v>1759</v>
       </c>
       <c r="J601" t="s">
         <v>2380</v>
@@ -29682,7 +29682,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B605" t="s">
         <v>643</v>
@@ -29703,7 +29703,7 @@
         <v>1642</v>
       </c>
       <c r="I605" t="s">
-        <v>1724</v>
+        <v>1759</v>
       </c>
       <c r="J605" t="s">
         <v>2384</v>
@@ -29738,7 +29738,7 @@
         <v>1642</v>
       </c>
       <c r="I606" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J606" t="s">
         <v>2385</v>
@@ -29936,7 +29936,7 @@
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B612" t="s">
         <v>650</v>
@@ -30482,7 +30482,7 @@
         <v>1642</v>
       </c>
       <c r="I627" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J627" t="s">
         <v>2406</v>
@@ -30517,7 +30517,7 @@
         <v>1642</v>
       </c>
       <c r="I628" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J628" t="s">
         <v>2407</v>
@@ -30590,7 +30590,7 @@
         <v>1642</v>
       </c>
       <c r="I630" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J630" t="s">
         <v>2409</v>
@@ -30660,7 +30660,7 @@
         <v>1642</v>
       </c>
       <c r="I632" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J632" t="s">
         <v>2411</v>
@@ -30835,7 +30835,7 @@
         <v>1642</v>
       </c>
       <c r="I637" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J637" t="s">
         <v>2416</v>
@@ -30905,7 +30905,7 @@
         <v>1642</v>
       </c>
       <c r="I639" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J639" t="s">
         <v>2418</v>
@@ -30940,7 +30940,7 @@
         <v>1642</v>
       </c>
       <c r="I640" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J640" t="s">
         <v>2419</v>
@@ -31013,7 +31013,7 @@
         <v>1642</v>
       </c>
       <c r="I642" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J642" t="s">
         <v>2421</v>
@@ -31167,7 +31167,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B647" t="s">
         <v>685</v>
@@ -31342,7 +31342,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B652" t="s">
         <v>690</v>
@@ -31363,7 +31363,7 @@
         <v>1642</v>
       </c>
       <c r="I652" t="s">
-        <v>1740</v>
+        <v>1759</v>
       </c>
       <c r="J652" t="s">
         <v>2431</v>
@@ -31608,7 +31608,7 @@
         <v>1642</v>
       </c>
       <c r="I659" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J659" t="s">
         <v>2438</v>
@@ -31643,7 +31643,7 @@
         <v>1642</v>
       </c>
       <c r="I660" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J660" t="s">
         <v>2439</v>
@@ -31716,7 +31716,7 @@
         <v>1642</v>
       </c>
       <c r="I662" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J662" t="s">
         <v>2441</v>
@@ -31894,7 +31894,7 @@
         <v>1668</v>
       </c>
       <c r="I667" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J667" t="s">
         <v>2446</v>
@@ -32282,7 +32282,7 @@
         <v>1642</v>
       </c>
       <c r="I678" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J678" t="s">
         <v>2457</v>
@@ -32317,7 +32317,7 @@
         <v>1642</v>
       </c>
       <c r="I679" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J679" t="s">
         <v>2458</v>
@@ -32460,7 +32460,7 @@
         <v>1658</v>
       </c>
       <c r="I683" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J683" t="s">
         <v>2462</v>
@@ -32492,7 +32492,7 @@
         <v>1642</v>
       </c>
       <c r="I684" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J684" t="s">
         <v>2463</v>
@@ -32524,7 +32524,7 @@
         <v>1642</v>
       </c>
       <c r="I685" t="s">
-        <v>1777</v>
+        <v>1759</v>
       </c>
       <c r="J685" t="s">
         <v>2464</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-13 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5164,7 +5164,7 @@
     <t>RENATA PASCOAL FREIRE</t>
   </si>
   <si>
-    <t>RENATA PASCOAL FREIRE, _SEM USUARIO ATRIBUIDO</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, RENATA PASCOAL FREIRE</t>
   </si>
   <si>
     <t>PEDRO MARCELO ROCHA GOMES</t>
@@ -11994,7 +11994,7 @@
         <v>1659</v>
       </c>
       <c r="I98" t="s">
-        <v>1697</v>
+        <v>1693</v>
       </c>
       <c r="J98" t="s">
         <v>1919</v>
@@ -14712,7 +14712,7 @@
     </row>
     <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B176" t="s">
         <v>216</v>
@@ -14733,7 +14733,7 @@
         <v>1659</v>
       </c>
       <c r="I176" t="s">
-        <v>1762</v>
+        <v>1697</v>
       </c>
       <c r="J176" t="s">
         <v>1991</v>
@@ -25969,7 +25969,7 @@
         <v>1659</v>
       </c>
       <c r="I496" t="s">
-        <v>1697</v>
+        <v>1693</v>
       </c>
       <c r="J496" t="s">
         <v>2301</v>
@@ -29945,7 +29945,7 @@
         <v>1659</v>
       </c>
       <c r="I609" t="s">
-        <v>1697</v>
+        <v>1693</v>
       </c>
       <c r="J609" t="s">
         <v>2413</v>
@@ -32360,7 +32360,7 @@
     </row>
     <row r="678" spans="1:12">
       <c r="A678" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B678" t="s">
         <v>717</v>
@@ -32381,7 +32381,7 @@
         <v>1659</v>
       </c>
       <c r="I678" t="s">
-        <v>1697</v>
+        <v>1771</v>
       </c>
       <c r="J678" t="s">
         <v>2482</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-14 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5293,73 +5293,73 @@
     <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SUZAN NIGRI</t>
   </si>
   <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>REINALDO DE SOUZA MACHADO</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI, PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI, PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
+  </si>
+  <si>
+    <t>NIVANA DANIELLE SILVA COSTA</t>
+  </si>
+  <si>
     <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI, PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI, PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
-  </si>
-  <si>
-    <t>NIVANA DANIELLE SILVA COSTA</t>
   </si>
   <si>
     <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
@@ -14219,7 +14219,7 @@
     </row>
     <row r="162" spans="1:12">
       <c r="A162" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B162" t="s">
         <v>200</v>
@@ -14240,7 +14240,7 @@
         <v>1660</v>
       </c>
       <c r="I162" t="s">
-        <v>1759</v>
+        <v>1693</v>
       </c>
       <c r="J162" t="s">
         <v>1974</v>
@@ -14415,7 +14415,7 @@
         <v>1660</v>
       </c>
       <c r="I167" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J167" t="s">
         <v>1978</v>
@@ -14485,7 +14485,7 @@
         <v>1660</v>
       </c>
       <c r="I169" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J169" t="s">
         <v>1980</v>
@@ -14520,7 +14520,7 @@
         <v>1660</v>
       </c>
       <c r="I170" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J170" t="s">
         <v>1830</v>
@@ -14768,7 +14768,7 @@
         <v>1660</v>
       </c>
       <c r="I177" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="J177" t="s">
         <v>1986</v>
@@ -14838,7 +14838,7 @@
         <v>1660</v>
       </c>
       <c r="I179" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J179" t="s">
         <v>1988</v>
@@ -14908,7 +14908,7 @@
         <v>1660</v>
       </c>
       <c r="I181" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
       <c r="J181" t="s">
         <v>1990</v>
@@ -15153,7 +15153,7 @@
         <v>1660</v>
       </c>
       <c r="I188" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J188" t="s">
         <v>1997</v>
@@ -15188,7 +15188,7 @@
         <v>1660</v>
       </c>
       <c r="I189" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J189" t="s">
         <v>1998</v>
@@ -15573,7 +15573,7 @@
         <v>1660</v>
       </c>
       <c r="I200" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J200" t="s">
         <v>2009</v>
@@ -15608,7 +15608,7 @@
         <v>1660</v>
       </c>
       <c r="I201" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
       <c r="J201" t="s">
         <v>2010</v>
@@ -15783,7 +15783,7 @@
         <v>1660</v>
       </c>
       <c r="I206" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J206" t="s">
         <v>2015</v>
@@ -15853,7 +15853,7 @@
         <v>1660</v>
       </c>
       <c r="I208" t="s">
-        <v>1770</v>
+        <v>1769</v>
       </c>
       <c r="J208" t="s">
         <v>2017</v>
@@ -15923,7 +15923,7 @@
         <v>1660</v>
       </c>
       <c r="I210" t="s">
-        <v>1771</v>
+        <v>1770</v>
       </c>
       <c r="J210" t="s">
         <v>2019</v>
@@ -15958,7 +15958,7 @@
         <v>1660</v>
       </c>
       <c r="I211" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J211" t="s">
         <v>2020</v>
@@ -15993,7 +15993,7 @@
         <v>1660</v>
       </c>
       <c r="I212" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
       <c r="J212" t="s">
         <v>2021</v>
@@ -16203,7 +16203,7 @@
         <v>1660</v>
       </c>
       <c r="I218" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J218" t="s">
         <v>2027</v>
@@ -16483,7 +16483,7 @@
         <v>1660</v>
       </c>
       <c r="I226" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J226" t="s">
         <v>2035</v>
@@ -16518,7 +16518,7 @@
         <v>1660</v>
       </c>
       <c r="I227" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J227" t="s">
         <v>2036</v>
@@ -16553,7 +16553,7 @@
         <v>1660</v>
       </c>
       <c r="I228" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="J228" t="s">
         <v>1909</v>
@@ -16798,7 +16798,7 @@
         <v>1660</v>
       </c>
       <c r="I235" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="J235" t="s">
         <v>2042</v>
@@ -16871,7 +16871,7 @@
         <v>1569</v>
       </c>
       <c r="I237" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="J237" t="s">
         <v>2044</v>
@@ -16976,7 +16976,7 @@
         <v>1660</v>
       </c>
       <c r="I240" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J240" t="s">
         <v>2047</v>
@@ -17119,7 +17119,7 @@
         <v>1669</v>
       </c>
       <c r="I244" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="J244" t="s">
         <v>2051</v>
@@ -17259,7 +17259,7 @@
         <v>1662</v>
       </c>
       <c r="I248" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
       <c r="J248" t="s">
         <v>2055</v>
@@ -17434,7 +17434,7 @@
         <v>1660</v>
       </c>
       <c r="I253" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J253" t="s">
         <v>2060</v>
@@ -17504,7 +17504,7 @@
         <v>1660</v>
       </c>
       <c r="I255" t="s">
-        <v>1780</v>
+        <v>1779</v>
       </c>
       <c r="J255" t="s">
         <v>2062</v>
@@ -17539,7 +17539,7 @@
         <v>1660</v>
       </c>
       <c r="I256" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
       <c r="J256" t="s">
         <v>2063</v>
@@ -17574,7 +17574,7 @@
         <v>1660</v>
       </c>
       <c r="I257" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J257" t="s">
         <v>2064</v>
@@ -17644,7 +17644,7 @@
         <v>1660</v>
       </c>
       <c r="I259" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J259" t="s">
         <v>2066</v>
@@ -17714,7 +17714,7 @@
         <v>1660</v>
       </c>
       <c r="I261" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J261" t="s">
         <v>2068</v>
@@ -17959,7 +17959,7 @@
         <v>1660</v>
       </c>
       <c r="I268" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J268" t="s">
         <v>2075</v>
@@ -18064,7 +18064,7 @@
         <v>1660</v>
       </c>
       <c r="I271" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J271" t="s">
         <v>2078</v>
@@ -18344,7 +18344,7 @@
         <v>1660</v>
       </c>
       <c r="I279" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J279" t="s">
         <v>2085</v>
@@ -18379,7 +18379,7 @@
         <v>1660</v>
       </c>
       <c r="I280" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J280" t="s">
         <v>2086</v>
@@ -18907,7 +18907,7 @@
         <v>1660</v>
       </c>
       <c r="I295" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J295" t="s">
         <v>2101</v>
@@ -18942,7 +18942,7 @@
         <v>1660</v>
       </c>
       <c r="I296" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J296" t="s">
         <v>2102</v>
@@ -19467,7 +19467,7 @@
         <v>1660</v>
       </c>
       <c r="I311" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J311" t="s">
         <v>2117</v>
@@ -19537,7 +19537,7 @@
         <v>1660</v>
       </c>
       <c r="I313" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="J313" t="s">
         <v>2119</v>
@@ -19645,7 +19645,7 @@
         <v>1670</v>
       </c>
       <c r="I316" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J316" t="s">
         <v>2122</v>
@@ -19680,7 +19680,7 @@
         <v>1660</v>
       </c>
       <c r="I317" t="s">
-        <v>1780</v>
+        <v>1779</v>
       </c>
       <c r="J317" t="s">
         <v>2123</v>
@@ -19785,7 +19785,7 @@
         <v>1660</v>
       </c>
       <c r="I320" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J320" t="s">
         <v>2126</v>
@@ -19820,7 +19820,7 @@
         <v>1660</v>
       </c>
       <c r="I321" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J321" t="s">
         <v>2127</v>
@@ -19960,7 +19960,7 @@
         <v>1660</v>
       </c>
       <c r="I325" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J325" t="s">
         <v>2131</v>
@@ -19995,7 +19995,7 @@
         <v>1660</v>
       </c>
       <c r="I326" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J326" t="s">
         <v>2132</v>
@@ -20310,7 +20310,7 @@
         <v>1660</v>
       </c>
       <c r="I335" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J335" t="s">
         <v>2140</v>
@@ -20593,7 +20593,7 @@
         <v>1660</v>
       </c>
       <c r="I343" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J343" t="s">
         <v>2147</v>
@@ -20873,7 +20873,7 @@
         <v>1660</v>
       </c>
       <c r="I351" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J351" t="s">
         <v>2155</v>
@@ -20908,7 +20908,7 @@
         <v>1660</v>
       </c>
       <c r="I352" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J352" t="s">
         <v>2156</v>
@@ -21013,7 +21013,7 @@
         <v>1660</v>
       </c>
       <c r="I355" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J355" t="s">
         <v>2159</v>
@@ -21048,7 +21048,7 @@
         <v>1660</v>
       </c>
       <c r="I356" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J356" t="s">
         <v>2160</v>
@@ -21296,7 +21296,7 @@
         <v>1660</v>
       </c>
       <c r="I363" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J363" t="s">
         <v>2167</v>
@@ -21436,7 +21436,7 @@
         <v>1660</v>
       </c>
       <c r="I367" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J367" t="s">
         <v>2171</v>
@@ -21471,7 +21471,7 @@
         <v>1660</v>
       </c>
       <c r="I368" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J368" t="s">
         <v>2172</v>
@@ -21716,7 +21716,7 @@
         <v>1660</v>
       </c>
       <c r="I375" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J375" t="s">
         <v>2179</v>
@@ -21821,7 +21821,7 @@
         <v>1660</v>
       </c>
       <c r="I378" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J378" t="s">
         <v>2182</v>
@@ -21961,7 +21961,7 @@
         <v>1660</v>
       </c>
       <c r="I382" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J382" t="s">
         <v>2186</v>
@@ -21996,7 +21996,7 @@
         <v>1660</v>
       </c>
       <c r="I383" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J383" t="s">
         <v>2187</v>
@@ -22031,7 +22031,7 @@
         <v>1660</v>
       </c>
       <c r="I384" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J384" t="s">
         <v>2188</v>
@@ -22101,7 +22101,7 @@
         <v>1660</v>
       </c>
       <c r="I386" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J386" t="s">
         <v>2190</v>
@@ -22276,7 +22276,7 @@
         <v>1660</v>
       </c>
       <c r="I391" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J391" t="s">
         <v>2195</v>
@@ -22311,7 +22311,7 @@
         <v>1660</v>
       </c>
       <c r="I392" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J392" t="s">
         <v>2196</v>
@@ -22454,7 +22454,7 @@
         <v>1673</v>
       </c>
       <c r="I396" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J396" t="s">
         <v>2200</v>
@@ -22804,7 +22804,7 @@
         <v>1660</v>
       </c>
       <c r="I406" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J406" t="s">
         <v>2210</v>
@@ -22979,7 +22979,7 @@
         <v>1660</v>
       </c>
       <c r="I411" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J411" t="s">
         <v>2215</v>
@@ -23049,7 +23049,7 @@
         <v>1660</v>
       </c>
       <c r="I413" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J413" t="s">
         <v>2217</v>
@@ -23157,7 +23157,7 @@
         <v>1660</v>
       </c>
       <c r="I416" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J416" t="s">
         <v>2220</v>
@@ -23297,7 +23297,7 @@
         <v>1660</v>
       </c>
       <c r="I420" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J420" t="s">
         <v>2224</v>
@@ -23787,7 +23787,7 @@
         <v>1660</v>
       </c>
       <c r="I434" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J434" t="s">
         <v>2238</v>
@@ -24175,7 +24175,7 @@
         <v>1660</v>
       </c>
       <c r="I445" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="J445" t="s">
         <v>2119</v>
@@ -24245,7 +24245,7 @@
         <v>1660</v>
       </c>
       <c r="I447" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J447" t="s">
         <v>2250</v>
@@ -24770,7 +24770,7 @@
         <v>1660</v>
       </c>
       <c r="I462" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J462" t="s">
         <v>2264</v>
@@ -24983,7 +24983,7 @@
         <v>1660</v>
       </c>
       <c r="I468" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J468" t="s">
         <v>2269</v>
@@ -25053,7 +25053,7 @@
         <v>1660</v>
       </c>
       <c r="I470" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J470" t="s">
         <v>2271</v>
@@ -25088,7 +25088,7 @@
         <v>1660</v>
       </c>
       <c r="I471" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J471" t="s">
         <v>2272</v>
@@ -25193,7 +25193,7 @@
         <v>1660</v>
       </c>
       <c r="I474" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J474" t="s">
         <v>2275</v>
@@ -25228,7 +25228,7 @@
         <v>1660</v>
       </c>
       <c r="I475" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J475" t="s">
         <v>2276</v>
@@ -25473,7 +25473,7 @@
         <v>1660</v>
       </c>
       <c r="I482" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J482" t="s">
         <v>2283</v>
@@ -25508,7 +25508,7 @@
         <v>1660</v>
       </c>
       <c r="I483" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J483" t="s">
         <v>2284</v>
@@ -25753,7 +25753,7 @@
         <v>1660</v>
       </c>
       <c r="I490" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J490" t="s">
         <v>2291</v>
@@ -25788,7 +25788,7 @@
         <v>1660</v>
       </c>
       <c r="I491" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J491" t="s">
         <v>2292</v>
@@ -25858,7 +25858,7 @@
         <v>1660</v>
       </c>
       <c r="I493" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J493" t="s">
         <v>2294</v>
@@ -25966,7 +25966,7 @@
         <v>1660</v>
       </c>
       <c r="I496" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J496" t="s">
         <v>2297</v>
@@ -26036,7 +26036,7 @@
         <v>1660</v>
       </c>
       <c r="I498" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J498" t="s">
         <v>2299</v>
@@ -26144,7 +26144,7 @@
         <v>1660</v>
       </c>
       <c r="I501" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J501" t="s">
         <v>2302</v>
@@ -26392,7 +26392,7 @@
         <v>1660</v>
       </c>
       <c r="I508" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J508" t="s">
         <v>2309</v>
@@ -26427,7 +26427,7 @@
         <v>1660</v>
       </c>
       <c r="I509" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J509" t="s">
         <v>2310</v>
@@ -26602,7 +26602,7 @@
         <v>1660</v>
       </c>
       <c r="I514" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="J514" t="s">
         <v>2315</v>
@@ -26637,7 +26637,7 @@
         <v>1660</v>
       </c>
       <c r="I515" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J515" t="s">
         <v>2316</v>
@@ -26812,7 +26812,7 @@
         <v>1660</v>
       </c>
       <c r="I520" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="J520" t="s">
         <v>2321</v>
@@ -26987,7 +26987,7 @@
         <v>1660</v>
       </c>
       <c r="I525" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J525" t="s">
         <v>2326</v>
@@ -27022,7 +27022,7 @@
         <v>1660</v>
       </c>
       <c r="I526" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J526" t="s">
         <v>2327</v>
@@ -27302,7 +27302,7 @@
         <v>1660</v>
       </c>
       <c r="I534" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J534" t="s">
         <v>2335</v>
@@ -27477,7 +27477,7 @@
         <v>1660</v>
       </c>
       <c r="I539" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J539" t="s">
         <v>2340</v>
@@ -27547,7 +27547,7 @@
         <v>1660</v>
       </c>
       <c r="I541" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J541" t="s">
         <v>2342</v>
@@ -27757,7 +27757,7 @@
         <v>1660</v>
       </c>
       <c r="I547" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J547" t="s">
         <v>2348</v>
@@ -27792,7 +27792,7 @@
         <v>1660</v>
       </c>
       <c r="I548" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J548" t="s">
         <v>2349</v>
@@ -27865,7 +27865,7 @@
         <v>1660</v>
       </c>
       <c r="I550" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J550" t="s">
         <v>2351</v>
@@ -27900,7 +27900,7 @@
         <v>1660</v>
       </c>
       <c r="I551" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J551" t="s">
         <v>2352</v>
@@ -28145,7 +28145,7 @@
         <v>1660</v>
       </c>
       <c r="I558" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J558" t="s">
         <v>2359</v>
@@ -28215,7 +28215,7 @@
         <v>1660</v>
       </c>
       <c r="I560" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J560" t="s">
         <v>2361</v>
@@ -28740,7 +28740,7 @@
         <v>1660</v>
       </c>
       <c r="I575" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J575" t="s">
         <v>2376</v>
@@ -28845,7 +28845,7 @@
         <v>1660</v>
       </c>
       <c r="I578" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J578" t="s">
         <v>2378</v>
@@ -28880,7 +28880,7 @@
         <v>1660</v>
       </c>
       <c r="I579" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="J579" t="s">
         <v>2379</v>
@@ -29055,7 +29055,7 @@
         <v>1660</v>
       </c>
       <c r="I584" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J584" t="s">
         <v>2384</v>
@@ -29125,7 +29125,7 @@
         <v>1660</v>
       </c>
       <c r="I586" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J586" t="s">
         <v>2386</v>
@@ -29265,7 +29265,7 @@
         <v>1660</v>
       </c>
       <c r="I590" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J590" t="s">
         <v>2390</v>
@@ -29586,7 +29586,7 @@
         <v>1660</v>
       </c>
       <c r="I599" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J599" t="s">
         <v>2399</v>
@@ -29691,7 +29691,7 @@
         <v>1660</v>
       </c>
       <c r="I602" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J602" t="s">
         <v>2402</v>
@@ -29901,7 +29901,7 @@
         <v>1660</v>
       </c>
       <c r="I608" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J608" t="s">
         <v>2408</v>
@@ -30044,7 +30044,7 @@
         <v>1681</v>
       </c>
       <c r="I612" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J612" t="s">
         <v>2412</v>
@@ -30184,7 +30184,7 @@
         <v>1660</v>
       </c>
       <c r="I616" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J616" t="s">
         <v>2416</v>
@@ -30254,7 +30254,7 @@
         <v>1660</v>
       </c>
       <c r="I618" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J618" t="s">
         <v>2418</v>
@@ -30394,7 +30394,7 @@
         <v>1660</v>
       </c>
       <c r="I622" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J622" t="s">
         <v>2422</v>
@@ -30534,7 +30534,7 @@
         <v>1660</v>
       </c>
       <c r="I626" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J626" t="s">
         <v>2426</v>
@@ -30604,7 +30604,7 @@
         <v>1660</v>
       </c>
       <c r="I628" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J628" t="s">
         <v>2428</v>
@@ -30674,7 +30674,7 @@
         <v>1660</v>
       </c>
       <c r="I630" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J630" t="s">
         <v>2430</v>
@@ -30709,7 +30709,7 @@
         <v>1660</v>
       </c>
       <c r="I631" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J631" t="s">
         <v>2431</v>
@@ -30814,7 +30814,7 @@
         <v>1660</v>
       </c>
       <c r="I634" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J634" t="s">
         <v>2434</v>
@@ -30849,7 +30849,7 @@
         <v>1660</v>
       </c>
       <c r="I635" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J635" t="s">
         <v>2435</v>
@@ -30884,7 +30884,7 @@
         <v>1660</v>
       </c>
       <c r="I636" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J636" t="s">
         <v>2436</v>
@@ -30989,7 +30989,7 @@
         <v>1660</v>
       </c>
       <c r="I639" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J639" t="s">
         <v>2439</v>
@@ -31024,7 +31024,7 @@
         <v>1660</v>
       </c>
       <c r="I640" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J640" t="s">
         <v>2440</v>
@@ -31310,7 +31310,7 @@
         <v>1683</v>
       </c>
       <c r="I648" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J648" t="s">
         <v>2448</v>
@@ -31345,7 +31345,7 @@
         <v>1660</v>
       </c>
       <c r="I649" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J649" t="s">
         <v>2449</v>
@@ -31415,7 +31415,7 @@
         <v>1660</v>
       </c>
       <c r="I651" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J651" t="s">
         <v>2451</v>
@@ -31628,7 +31628,7 @@
         <v>1660</v>
       </c>
       <c r="I657" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J657" t="s">
         <v>2457</v>
@@ -31663,7 +31663,7 @@
         <v>1660</v>
       </c>
       <c r="I658" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J658" t="s">
         <v>2458</v>
@@ -31768,7 +31768,7 @@
         <v>1660</v>
       </c>
       <c r="I661" t="s">
-        <v>1759</v>
+        <v>1781</v>
       </c>
       <c r="J661" t="s">
         <v>2461</v>
@@ -31987,7 +31987,7 @@
         <v>1685</v>
       </c>
       <c r="I667" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J667" t="s">
         <v>2467</v>
@@ -32022,7 +32022,7 @@
         <v>1660</v>
       </c>
       <c r="I668" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J668" t="s">
         <v>2468</v>
@@ -32092,7 +32092,7 @@
         <v>1660</v>
       </c>
       <c r="I670" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J670" t="s">
         <v>2470</v>
@@ -32232,7 +32232,7 @@
         <v>1660</v>
       </c>
       <c r="I674" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J674" t="s">
         <v>2474</v>
@@ -32267,7 +32267,7 @@
         <v>1660</v>
       </c>
       <c r="I675" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J675" t="s">
         <v>2475</v>
@@ -32302,7 +32302,7 @@
         <v>1660</v>
       </c>
       <c r="I676" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J676" t="s">
         <v>2476</v>
@@ -32337,7 +32337,7 @@
         <v>1660</v>
       </c>
       <c r="I677" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J677" t="s">
         <v>2477</v>
@@ -32480,7 +32480,7 @@
         <v>1660</v>
       </c>
       <c r="I681" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
       <c r="J681" t="s">
         <v>2481</v>
@@ -32658,7 +32658,7 @@
         <v>1660</v>
       </c>
       <c r="I686" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J686" t="s">
         <v>2486</v>
@@ -32941,7 +32941,7 @@
         <v>1660</v>
       </c>
       <c r="I694" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J694" t="s">
         <v>2494</v>
@@ -32973,7 +32973,7 @@
         <v>1660</v>
       </c>
       <c r="I695" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J695" t="s">
         <v>2495</v>
@@ -33005,7 +33005,7 @@
         <v>1660</v>
       </c>
       <c r="I696" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="J696" t="s">
         <v>2496</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-15 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -32742,7 +32742,7 @@
     </row>
     <row r="689" spans="1:12">
       <c r="A689" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B689" t="s">
         <v>726</v>
@@ -32763,7 +32763,7 @@
         <v>1660</v>
       </c>
       <c r="I689" t="s">
-        <v>1697</v>
+        <v>1814</v>
       </c>
       <c r="J689" t="s">
         <v>2489</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-15 12:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7966,7 +7966,7 @@
     <t>BIOLOGIA,ECONOMIA,GEOTECNIA,URBANISMO</t>
   </si>
   <si>
-    <t>URBANISMO,ECONOMIA,BIOLOGIA,GEOTECNIA</t>
+    <t>GEOTECNIA,URBANISMO,BIOLOGIA,ECONOMIA</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS</t>
@@ -8113,33 +8113,36 @@
     <t>ENGENHARIA QUÍMICA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
+  </si>
+  <si>
+    <t>GEOTECNIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
-  </si>
-  <si>
-    <t>GEOTECNIA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
     <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
@@ -8155,7 +8158,7 @@
     <t>MOBILIDADE E TRANSPORTE,EDIFICAÇÕES</t>
   </si>
   <si>
-    <t>ENGENHARIA QUÍMICA,ENGENHARIA AMBIENTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+    <t>ENGENHARIA AMBIENTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA QUÍMICA</t>
   </si>
   <si>
     <t>BIOLOGIA,EDIFICAÇÕES</t>
@@ -8164,7 +8167,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
@@ -8173,10 +8176,7 @@
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ECONOMIA,URBANISMO,ORÇAMENTO,PSICOLOGIA,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ASSISTÊNCIA SOCIAL,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
+    <t>PSICOLOGIA,MOBILIDADE E TRANSPORTE,URBANISMO,ECONOMIA,ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ORÇAMENTO,SAÚDE MENTAL</t>
   </si>
 </sst>
 </file>
@@ -16398,7 +16398,7 @@
         <v>1657</v>
       </c>
       <c r="I224" t="s">
-        <v>1694</v>
+        <v>1766</v>
       </c>
       <c r="J224" t="s">
         <v>2027</v>
@@ -26561,7 +26561,7 @@
         <v>2558</v>
       </c>
       <c r="L513" t="s">
-        <v>2699</v>
+        <v>2708</v>
       </c>
     </row>
     <row r="514" spans="1:12">
@@ -26701,7 +26701,7 @@
         <v>2527</v>
       </c>
       <c r="L517" t="s">
-        <v>2708</v>
+        <v>2709</v>
       </c>
     </row>
     <row r="518" spans="1:12">
@@ -27899,7 +27899,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B552" t="s">
         <v>588</v>
@@ -27920,7 +27920,7 @@
         <v>1657</v>
       </c>
       <c r="I552" t="s">
-        <v>1690</v>
+        <v>1694</v>
       </c>
       <c r="J552" t="s">
         <v>2347</v>
@@ -27929,7 +27929,7 @@
         <v>2624</v>
       </c>
       <c r="L552" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -28314,7 +28314,7 @@
         <v>2626</v>
       </c>
       <c r="L563" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="564" spans="1:12">
@@ -28349,7 +28349,7 @@
         <v>2627</v>
       </c>
       <c r="L564" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -28515,7 +28515,7 @@
         <v>1657</v>
       </c>
       <c r="I569" t="s">
-        <v>1694</v>
+        <v>1805</v>
       </c>
       <c r="J569" t="s">
         <v>2364</v>
@@ -28524,7 +28524,7 @@
         <v>2551</v>
       </c>
       <c r="L569" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -28559,7 +28559,7 @@
         <v>2628</v>
       </c>
       <c r="L570" t="s">
-        <v>2710</v>
+        <v>2711</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28585,7 +28585,7 @@
         <v>1657</v>
       </c>
       <c r="I571" t="s">
-        <v>1694</v>
+        <v>1805</v>
       </c>
       <c r="J571" t="s">
         <v>2366</v>
@@ -28594,7 +28594,7 @@
         <v>2629</v>
       </c>
       <c r="L571" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="572" spans="1:12">
@@ -28629,7 +28629,7 @@
         <v>2630</v>
       </c>
       <c r="L572" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="573" spans="1:12">
@@ -28664,7 +28664,7 @@
         <v>2534</v>
       </c>
       <c r="L573" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="574" spans="1:12">
@@ -28699,7 +28699,7 @@
         <v>2579</v>
       </c>
       <c r="L574" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="575" spans="1:12">
@@ -28769,7 +28769,7 @@
         <v>2511</v>
       </c>
       <c r="L576" t="s">
-        <v>2711</v>
+        <v>2712</v>
       </c>
     </row>
     <row r="577" spans="1:12">
@@ -28804,7 +28804,7 @@
         <v>2511</v>
       </c>
       <c r="L577" t="s">
-        <v>2712</v>
+        <v>2713</v>
       </c>
     </row>
     <row r="578" spans="1:12">
@@ -29014,7 +29014,7 @@
         <v>2631</v>
       </c>
       <c r="L583" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="584" spans="1:12">
@@ -29084,7 +29084,7 @@
         <v>2629</v>
       </c>
       <c r="L585" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="586" spans="1:12">
@@ -29440,7 +29440,7 @@
         <v>2632</v>
       </c>
       <c r="L595" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -29475,7 +29475,7 @@
         <v>2633</v>
       </c>
       <c r="L596" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="597" spans="1:12">
@@ -29720,7 +29720,7 @@
         <v>2527</v>
       </c>
       <c r="L603" t="s">
-        <v>2713</v>
+        <v>2714</v>
       </c>
     </row>
     <row r="604" spans="1:12">
@@ -29860,7 +29860,7 @@
         <v>2547</v>
       </c>
       <c r="L607" t="s">
-        <v>2714</v>
+        <v>2715</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -30353,7 +30353,7 @@
         <v>2513</v>
       </c>
       <c r="L621" t="s">
-        <v>2715</v>
+        <v>2716</v>
       </c>
     </row>
     <row r="622" spans="1:12">
@@ -30563,7 +30563,7 @@
         <v>2493</v>
       </c>
       <c r="L627" t="s">
-        <v>2716</v>
+        <v>2717</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30773,7 +30773,7 @@
         <v>2638</v>
       </c>
       <c r="L633" t="s">
-        <v>2692</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -31479,7 +31479,7 @@
         <v>2550</v>
       </c>
       <c r="L653" t="s">
-        <v>2717</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="654" spans="1:12">
@@ -31514,7 +31514,7 @@
         <v>2640</v>
       </c>
       <c r="L654" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="655" spans="1:12">
@@ -31835,7 +31835,7 @@
         <v>2515</v>
       </c>
       <c r="L663" t="s">
-        <v>2718</v>
+        <v>2719</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -32967,7 +32967,7 @@
         <v>2643</v>
       </c>
       <c r="L695" t="s">
-        <v>2719</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="696" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-15 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -100,36 +100,36 @@
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
+    <t>NÚCLEO TÉCNICO DE CONTABILIDADE, NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS, NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE ECONOMIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE, ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE CONTABILIDADE, NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS, NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE ECONOMIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, NÚCLEO TÉCNICO DE CONTABILIDADE</t>
   </si>
   <si>
@@ -5230,100 +5230,100 @@
     <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
   </si>
   <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
+  </si>
+  <si>
+    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
     <t>HIAN GOMES DE OLIVEIRA DA COSTA, PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
-  </si>
-  <si>
-    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
   </si>
   <si>
     <t>GABRIEL GERON MOREIRA</t>
@@ -9683,7 +9683,7 @@
         <v>1657</v>
       </c>
       <c r="I33" t="s">
-        <v>1695</v>
+        <v>1691</v>
       </c>
       <c r="J33" t="s">
         <v>1842</v>
@@ -12798,7 +12798,7 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B122" t="s">
         <v>160</v>
@@ -13183,7 +13183,7 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B133" t="s">
         <v>171</v>
@@ -13393,7 +13393,7 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B139" t="s">
         <v>176</v>
@@ -14306,7 +14306,7 @@
     </row>
     <row r="165" spans="1:12">
       <c r="A165" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B165" t="s">
         <v>202</v>
@@ -14659,7 +14659,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B175" t="s">
         <v>212</v>
@@ -14694,7 +14694,7 @@
     </row>
     <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B176" t="s">
         <v>213</v>
@@ -14799,7 +14799,7 @@
     </row>
     <row r="179" spans="1:12">
       <c r="A179" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B179" t="s">
         <v>216</v>
@@ -15135,7 +15135,7 @@
         <v>1657</v>
       </c>
       <c r="I188" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J188" t="s">
         <v>1989</v>
@@ -15485,7 +15485,7 @@
         <v>1657</v>
       </c>
       <c r="I198" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J198" t="s">
         <v>1999</v>
@@ -15520,7 +15520,7 @@
         <v>1657</v>
       </c>
       <c r="I199" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J199" t="s">
         <v>2000</v>
@@ -15695,7 +15695,7 @@
         <v>1657</v>
       </c>
       <c r="I204" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="J204" t="s">
         <v>2005</v>
@@ -15765,7 +15765,7 @@
         <v>1657</v>
       </c>
       <c r="I206" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J206" t="s">
         <v>2007</v>
@@ -15779,7 +15779,7 @@
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B207" t="s">
         <v>244</v>
@@ -15814,7 +15814,7 @@
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B208" t="s">
         <v>245</v>
@@ -15835,7 +15835,7 @@
         <v>1657</v>
       </c>
       <c r="I208" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
       <c r="J208" t="s">
         <v>2009</v>
@@ -15870,7 +15870,7 @@
         <v>1657</v>
       </c>
       <c r="I209" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J209" t="s">
         <v>2010</v>
@@ -15989,7 +15989,7 @@
     </row>
     <row r="213" spans="1:12">
       <c r="A213" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B213" t="s">
         <v>250</v>
@@ -16234,7 +16234,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B220" t="s">
         <v>257</v>
@@ -16325,7 +16325,7 @@
         <v>1657</v>
       </c>
       <c r="I222" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J222" t="s">
         <v>2023</v>
@@ -16395,7 +16395,7 @@
         <v>1657</v>
       </c>
       <c r="I224" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J224" t="s">
         <v>2025</v>
@@ -16465,7 +16465,7 @@
         <v>1657</v>
       </c>
       <c r="I226" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J226" t="s">
         <v>1900</v>
@@ -16710,7 +16710,7 @@
         <v>1657</v>
       </c>
       <c r="I233" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
       <c r="J233" t="s">
         <v>2032</v>
@@ -16783,7 +16783,7 @@
         <v>1565</v>
       </c>
       <c r="I235" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J235" t="s">
         <v>2034</v>
@@ -16832,7 +16832,7 @@
     </row>
     <row r="237" spans="1:12">
       <c r="A237" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B237" t="s">
         <v>274</v>
@@ -16853,7 +16853,7 @@
         <v>1657</v>
       </c>
       <c r="I237" t="s">
-        <v>1738</v>
+        <v>1769</v>
       </c>
       <c r="J237" t="s">
         <v>2036</v>
@@ -17007,7 +17007,7 @@
     </row>
     <row r="242" spans="1:12">
       <c r="A242" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B242" t="s">
         <v>279</v>
@@ -17150,7 +17150,7 @@
     </row>
     <row r="246" spans="1:12">
       <c r="A246" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B246" t="s">
         <v>283</v>
@@ -17626,7 +17626,7 @@
         <v>1657</v>
       </c>
       <c r="I259" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J259" t="s">
         <v>2058</v>
@@ -17976,7 +17976,7 @@
         <v>1657</v>
       </c>
       <c r="I269" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J269" t="s">
         <v>2068</v>
@@ -18550,7 +18550,7 @@
     </row>
     <row r="286" spans="1:12">
       <c r="A286" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B286" t="s">
         <v>323</v>
@@ -18784,7 +18784,7 @@
         <v>1657</v>
       </c>
       <c r="I292" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J292" t="s">
         <v>2090</v>
@@ -19344,7 +19344,7 @@
         <v>1657</v>
       </c>
       <c r="I308" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J308" t="s">
         <v>2106</v>
@@ -19414,7 +19414,7 @@
         <v>1657</v>
       </c>
       <c r="I310" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J310" t="s">
         <v>2108</v>
@@ -19428,7 +19428,7 @@
     </row>
     <row r="311" spans="1:12">
       <c r="A311" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B311" t="s">
         <v>348</v>
@@ -19522,7 +19522,7 @@
         <v>1667</v>
       </c>
       <c r="I313" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J313" t="s">
         <v>2111</v>
@@ -19571,7 +19571,7 @@
     </row>
     <row r="315" spans="1:12">
       <c r="A315" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B315" t="s">
         <v>352</v>
@@ -19662,7 +19662,7 @@
         <v>1657</v>
       </c>
       <c r="I317" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J317" t="s">
         <v>2115</v>
@@ -19697,7 +19697,7 @@
         <v>1657</v>
       </c>
       <c r="I318" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J318" t="s">
         <v>2116</v>
@@ -19837,7 +19837,7 @@
         <v>1657</v>
       </c>
       <c r="I322" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J322" t="s">
         <v>2120</v>
@@ -20187,7 +20187,7 @@
         <v>1657</v>
       </c>
       <c r="I332" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J332" t="s">
         <v>2129</v>
@@ -20470,7 +20470,7 @@
         <v>1657</v>
       </c>
       <c r="I340" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J340" t="s">
         <v>2136</v>
@@ -20750,7 +20750,7 @@
         <v>1657</v>
       </c>
       <c r="I348" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J348" t="s">
         <v>2144</v>
@@ -20785,7 +20785,7 @@
         <v>1657</v>
       </c>
       <c r="I349" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J349" t="s">
         <v>2145</v>
@@ -20925,7 +20925,7 @@
         <v>1657</v>
       </c>
       <c r="I353" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J353" t="s">
         <v>2149</v>
@@ -21173,7 +21173,7 @@
         <v>1657</v>
       </c>
       <c r="I360" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J360" t="s">
         <v>2156</v>
@@ -21292,7 +21292,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B364" t="s">
         <v>401</v>
@@ -21313,7 +21313,7 @@
         <v>1657</v>
       </c>
       <c r="I364" t="s">
-        <v>1738</v>
+        <v>1769</v>
       </c>
       <c r="J364" t="s">
         <v>2160</v>
@@ -21838,7 +21838,7 @@
         <v>1657</v>
       </c>
       <c r="I379" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J379" t="s">
         <v>2175</v>
@@ -22153,7 +22153,7 @@
         <v>1657</v>
       </c>
       <c r="I388" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J388" t="s">
         <v>2184</v>
@@ -22188,7 +22188,7 @@
         <v>1657</v>
       </c>
       <c r="I389" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J389" t="s">
         <v>2185</v>
@@ -22681,7 +22681,7 @@
         <v>1657</v>
       </c>
       <c r="I403" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J403" t="s">
         <v>2199</v>
@@ -22856,7 +22856,7 @@
         <v>1657</v>
       </c>
       <c r="I408" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J408" t="s">
         <v>2204</v>
@@ -22926,7 +22926,7 @@
         <v>1657</v>
       </c>
       <c r="I410" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J410" t="s">
         <v>2206</v>
@@ -23034,7 +23034,7 @@
         <v>1657</v>
       </c>
       <c r="I413" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J413" t="s">
         <v>2209</v>
@@ -23664,7 +23664,7 @@
         <v>1657</v>
       </c>
       <c r="I431" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J431" t="s">
         <v>2227</v>
@@ -24090,7 +24090,7 @@
         <v>1657</v>
       </c>
       <c r="I443" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J443" t="s">
         <v>2108</v>
@@ -24685,7 +24685,7 @@
         <v>1657</v>
       </c>
       <c r="I460" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J460" t="s">
         <v>2253</v>
@@ -24898,7 +24898,7 @@
         <v>1657</v>
       </c>
       <c r="I466" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J466" t="s">
         <v>2258</v>
@@ -24912,7 +24912,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B467" t="s">
         <v>503</v>
@@ -24968,7 +24968,7 @@
         <v>1657</v>
       </c>
       <c r="I468" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J468" t="s">
         <v>2260</v>
@@ -25108,7 +25108,7 @@
         <v>1657</v>
       </c>
       <c r="I472" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J472" t="s">
         <v>2264</v>
@@ -25143,7 +25143,7 @@
         <v>1657</v>
       </c>
       <c r="I473" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J473" t="s">
         <v>2265</v>
@@ -25388,7 +25388,7 @@
         <v>1657</v>
       </c>
       <c r="I480" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J480" t="s">
         <v>2272</v>
@@ -25423,7 +25423,7 @@
         <v>1657</v>
       </c>
       <c r="I481" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J481" t="s">
         <v>2273</v>
@@ -25773,7 +25773,7 @@
         <v>1657</v>
       </c>
       <c r="I491" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J491" t="s">
         <v>2283</v>
@@ -26307,7 +26307,7 @@
         <v>1657</v>
       </c>
       <c r="I506" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J506" t="s">
         <v>2298</v>
@@ -26342,7 +26342,7 @@
         <v>1657</v>
       </c>
       <c r="I507" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J507" t="s">
         <v>2299</v>
@@ -26517,7 +26517,7 @@
         <v>1657</v>
       </c>
       <c r="I512" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J512" t="s">
         <v>2304</v>
@@ -26552,7 +26552,7 @@
         <v>1657</v>
       </c>
       <c r="I513" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J513" t="s">
         <v>2305</v>
@@ -26727,7 +26727,7 @@
         <v>1657</v>
       </c>
       <c r="I518" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J518" t="s">
         <v>2310</v>
@@ -26902,7 +26902,7 @@
         <v>1657</v>
       </c>
       <c r="I523" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J523" t="s">
         <v>2315</v>
@@ -27217,7 +27217,7 @@
         <v>1657</v>
       </c>
       <c r="I532" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J532" t="s">
         <v>2324</v>
@@ -27392,7 +27392,7 @@
         <v>1657</v>
       </c>
       <c r="I537" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J537" t="s">
         <v>2329</v>
@@ -27672,7 +27672,7 @@
         <v>1657</v>
       </c>
       <c r="I545" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J545" t="s">
         <v>2337</v>
@@ -27780,7 +27780,7 @@
         <v>1657</v>
       </c>
       <c r="I548" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J548" t="s">
         <v>2340</v>
@@ -28620,7 +28620,7 @@
         <v>1657</v>
       </c>
       <c r="I572" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J572" t="s">
         <v>2364</v>
@@ -28760,7 +28760,7 @@
         <v>1657</v>
       </c>
       <c r="I576" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J576" t="s">
         <v>2367</v>
@@ -28935,7 +28935,7 @@
         <v>1657</v>
       </c>
       <c r="I581" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J581" t="s">
         <v>2372</v>
@@ -29005,7 +29005,7 @@
         <v>1657</v>
       </c>
       <c r="I583" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J583" t="s">
         <v>2374</v>
@@ -29466,7 +29466,7 @@
         <v>1657</v>
       </c>
       <c r="I596" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J596" t="s">
         <v>2387</v>
@@ -29781,7 +29781,7 @@
         <v>1657</v>
       </c>
       <c r="I605" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J605" t="s">
         <v>2396</v>
@@ -30064,7 +30064,7 @@
         <v>1657</v>
       </c>
       <c r="I613" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J613" t="s">
         <v>2404</v>
@@ -30134,7 +30134,7 @@
         <v>1657</v>
       </c>
       <c r="I615" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J615" t="s">
         <v>2406</v>
@@ -30414,7 +30414,7 @@
         <v>1657</v>
       </c>
       <c r="I623" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J623" t="s">
         <v>2414</v>
@@ -30484,7 +30484,7 @@
         <v>1657</v>
       </c>
       <c r="I625" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J625" t="s">
         <v>2416</v>
@@ -30554,7 +30554,7 @@
         <v>1657</v>
       </c>
       <c r="I627" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J627" t="s">
         <v>2418</v>
@@ -30589,7 +30589,7 @@
         <v>1657</v>
       </c>
       <c r="I628" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J628" t="s">
         <v>2419</v>
@@ -30694,7 +30694,7 @@
         <v>1657</v>
       </c>
       <c r="I631" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J631" t="s">
         <v>2422</v>
@@ -30729,7 +30729,7 @@
         <v>1657</v>
       </c>
       <c r="I632" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J632" t="s">
         <v>2423</v>
@@ -30764,7 +30764,7 @@
         <v>1657</v>
       </c>
       <c r="I633" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J633" t="s">
         <v>2424</v>
@@ -30869,7 +30869,7 @@
         <v>1657</v>
       </c>
       <c r="I636" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J636" t="s">
         <v>2427</v>
@@ -31225,7 +31225,7 @@
         <v>1657</v>
       </c>
       <c r="I646" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J646" t="s">
         <v>2437</v>
@@ -31508,7 +31508,7 @@
         <v>1657</v>
       </c>
       <c r="I654" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J654" t="s">
         <v>2445</v>
@@ -31543,7 +31543,7 @@
         <v>1657</v>
       </c>
       <c r="I655" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J655" t="s">
         <v>2446</v>
@@ -31648,7 +31648,7 @@
         <v>1657</v>
       </c>
       <c r="I658" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J658" t="s">
         <v>2449</v>
@@ -32112,7 +32112,7 @@
         <v>1657</v>
       </c>
       <c r="I671" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J671" t="s">
         <v>2462</v>
@@ -32182,7 +32182,7 @@
         <v>1657</v>
       </c>
       <c r="I673" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J673" t="s">
         <v>2464</v>
@@ -32360,7 +32360,7 @@
         <v>1657</v>
       </c>
       <c r="I678" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J678" t="s">
         <v>2469</v>
@@ -32859,7 +32859,7 @@
         <v>1685</v>
       </c>
       <c r="I692" t="s">
-        <v>1695</v>
+        <v>1770</v>
       </c>
       <c r="J692" t="s">
         <v>2483</v>
@@ -32894,7 +32894,7 @@
         <v>1657</v>
       </c>
       <c r="I693" t="s">
-        <v>1760</v>
+        <v>1738</v>
       </c>
       <c r="J693" t="s">
         <v>2484</v>
@@ -32929,7 +32929,7 @@
         <v>1657</v>
       </c>
       <c r="I694" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J694" t="s">
         <v>2485</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-27 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -91,6 +91,9 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
   </si>
   <si>
@@ -101,9 +104,6 @@
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
-  </si>
-  <si>
-    <t>SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
@@ -10480,7 +10480,7 @@
     </row>
     <row r="58" spans="1:12">
       <c r="A58" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B58" t="s">
         <v>98</v>
@@ -10501,7 +10501,7 @@
         <v>1638</v>
       </c>
       <c r="I58" t="s">
-        <v>1696</v>
+        <v>1678</v>
       </c>
       <c r="J58" t="s">
         <v>1866</v>
@@ -10938,7 +10938,7 @@
     </row>
     <row r="71" spans="1:12">
       <c r="A71" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B71" t="s">
         <v>111</v>
@@ -11329,7 +11329,7 @@
     </row>
     <row r="82" spans="1:12">
       <c r="A82" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B82" t="s">
         <v>122</v>
@@ -11539,7 +11539,7 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B88" t="s">
         <v>128</v>
@@ -11574,7 +11574,7 @@
     </row>
     <row r="89" spans="1:12">
       <c r="A89" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B89" t="s">
         <v>129</v>
@@ -11679,7 +11679,7 @@
     </row>
     <row r="92" spans="1:12">
       <c r="A92" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B92" t="s">
         <v>132</v>
@@ -12105,7 +12105,7 @@
     </row>
     <row r="104" spans="1:12">
       <c r="A104" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B104" t="s">
         <v>144</v>
@@ -13570,7 +13570,7 @@
         <v>1818</v>
       </c>
       <c r="K145" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="L145" t="s">
         <v>2634</v>
@@ -13683,7 +13683,7 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B149" t="s">
         <v>189</v>
@@ -13966,7 +13966,7 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B157" t="s">
         <v>197</v>
@@ -14001,7 +14001,7 @@
     </row>
     <row r="158" spans="1:12">
       <c r="A158" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B158" t="s">
         <v>198</v>
@@ -14106,7 +14106,7 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B161" t="s">
         <v>201</v>
@@ -14246,7 +14246,7 @@
     </row>
     <row r="165" spans="1:12">
       <c r="A165" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B165" t="s">
         <v>205</v>
@@ -14456,7 +14456,7 @@
     </row>
     <row r="171" spans="1:12">
       <c r="A171" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B171" t="s">
         <v>211</v>
@@ -14596,7 +14596,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B175" t="s">
         <v>215</v>
@@ -14701,7 +14701,7 @@
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B178" t="s">
         <v>218</v>
@@ -14911,7 +14911,7 @@
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B184" t="s">
         <v>224</v>
@@ -14981,7 +14981,7 @@
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B186" t="s">
         <v>226</v>
@@ -15121,7 +15121,7 @@
     </row>
     <row r="190" spans="1:12">
       <c r="A190" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B190" t="s">
         <v>230</v>
@@ -15366,7 +15366,7 @@
     </row>
     <row r="197" spans="1:12">
       <c r="A197" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B197" t="s">
         <v>237</v>
@@ -15789,7 +15789,7 @@
     </row>
     <row r="209" spans="1:12">
       <c r="A209" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B209" t="s">
         <v>249</v>
@@ -15964,7 +15964,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B214" t="s">
         <v>254</v>
@@ -15999,7 +15999,7 @@
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B215" t="s">
         <v>255</v>
@@ -16034,7 +16034,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B216" t="s">
         <v>256</v>
@@ -16104,7 +16104,7 @@
     </row>
     <row r="218" spans="1:12">
       <c r="A218" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B218" t="s">
         <v>258</v>
@@ -16384,7 +16384,7 @@
     </row>
     <row r="226" spans="1:12">
       <c r="A226" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B226" t="s">
         <v>266</v>
@@ -16454,7 +16454,7 @@
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B228" t="s">
         <v>268</v>
@@ -16664,7 +16664,7 @@
     </row>
     <row r="234" spans="1:12">
       <c r="A234" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B234" t="s">
         <v>274</v>
@@ -16839,7 +16839,7 @@
     </row>
     <row r="239" spans="1:12">
       <c r="A239" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B239" t="s">
         <v>279</v>
@@ -16874,7 +16874,7 @@
     </row>
     <row r="240" spans="1:12">
       <c r="A240" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B240" t="s">
         <v>280</v>
@@ -16909,7 +16909,7 @@
     </row>
     <row r="241" spans="1:12">
       <c r="A241" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B241" t="s">
         <v>281</v>
@@ -17014,7 +17014,7 @@
     </row>
     <row r="244" spans="1:12">
       <c r="A244" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B244" t="s">
         <v>284</v>
@@ -17402,7 +17402,7 @@
     </row>
     <row r="255" spans="1:12">
       <c r="A255" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B255" t="s">
         <v>295</v>
@@ -17892,7 +17892,7 @@
     </row>
     <row r="269" spans="1:12">
       <c r="A269" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B269" t="s">
         <v>309</v>
@@ -17962,7 +17962,7 @@
     </row>
     <row r="271" spans="1:12">
       <c r="A271" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B271" t="s">
         <v>311</v>
@@ -18032,7 +18032,7 @@
     </row>
     <row r="273" spans="1:12">
       <c r="A273" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B273" t="s">
         <v>313</v>
@@ -18140,7 +18140,7 @@
     </row>
     <row r="276" spans="1:12">
       <c r="A276" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B276" t="s">
         <v>316</v>
@@ -18175,7 +18175,7 @@
     </row>
     <row r="277" spans="1:12">
       <c r="A277" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B277" t="s">
         <v>317</v>
@@ -18210,7 +18210,7 @@
     </row>
     <row r="278" spans="1:12">
       <c r="A278" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B278" t="s">
         <v>318</v>
@@ -18315,7 +18315,7 @@
     </row>
     <row r="281" spans="1:12">
       <c r="A281" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B281" t="s">
         <v>321</v>
@@ -18350,7 +18350,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B282" t="s">
         <v>322</v>
@@ -18560,7 +18560,7 @@
     </row>
     <row r="288" spans="1:12">
       <c r="A288" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B288" t="s">
         <v>328</v>
@@ -18808,7 +18808,7 @@
     </row>
     <row r="295" spans="1:12">
       <c r="A295" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B295" t="s">
         <v>335</v>
@@ -18843,7 +18843,7 @@
     </row>
     <row r="296" spans="1:12">
       <c r="A296" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B296" t="s">
         <v>336</v>
@@ -19123,7 +19123,7 @@
     </row>
     <row r="304" spans="1:12">
       <c r="A304" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B304" t="s">
         <v>344</v>
@@ -19193,7 +19193,7 @@
     </row>
     <row r="306" spans="1:12">
       <c r="A306" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B306" t="s">
         <v>346</v>
@@ -19263,7 +19263,7 @@
     </row>
     <row r="308" spans="1:12">
       <c r="A308" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B308" t="s">
         <v>348</v>
@@ -19298,7 +19298,7 @@
     </row>
     <row r="309" spans="1:12">
       <c r="A309" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B309" t="s">
         <v>349</v>
@@ -19721,7 +19721,7 @@
     </row>
     <row r="321" spans="1:12">
       <c r="A321" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B321" t="s">
         <v>361</v>
@@ -19756,7 +19756,7 @@
     </row>
     <row r="322" spans="1:12">
       <c r="A322" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B322" t="s">
         <v>362</v>
@@ -19791,7 +19791,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B323" t="s">
         <v>363</v>
@@ -20036,7 +20036,7 @@
     </row>
     <row r="330" spans="1:12">
       <c r="A330" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B330" t="s">
         <v>370</v>
@@ -20176,7 +20176,7 @@
     </row>
     <row r="334" spans="1:12">
       <c r="A334" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B334" t="s">
         <v>374</v>
@@ -20281,7 +20281,7 @@
     </row>
     <row r="337" spans="1:12">
       <c r="A337" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B337" t="s">
         <v>377</v>
@@ -20386,7 +20386,7 @@
     </row>
     <row r="340" spans="1:12">
       <c r="A340" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B340" t="s">
         <v>380</v>
@@ -20456,7 +20456,7 @@
     </row>
     <row r="342" spans="1:12">
       <c r="A342" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B342" t="s">
         <v>382</v>
@@ -20491,7 +20491,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B343" t="s">
         <v>383</v>
@@ -20561,7 +20561,7 @@
     </row>
     <row r="345" spans="1:12">
       <c r="A345" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B345" t="s">
         <v>385</v>
@@ -20631,7 +20631,7 @@
     </row>
     <row r="347" spans="1:12">
       <c r="A347" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B347" t="s">
         <v>387</v>
@@ -20739,7 +20739,7 @@
     </row>
     <row r="350" spans="1:12">
       <c r="A350" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B350" t="s">
         <v>390</v>
@@ -20879,7 +20879,7 @@
     </row>
     <row r="354" spans="1:12">
       <c r="A354" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B354" t="s">
         <v>394</v>
@@ -20949,7 +20949,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B356" t="s">
         <v>395</v>
@@ -21019,7 +21019,7 @@
     </row>
     <row r="358" spans="1:12">
       <c r="A358" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B358" t="s">
         <v>397</v>
@@ -21264,7 +21264,7 @@
     </row>
     <row r="365" spans="1:12">
       <c r="A365" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B365" t="s">
         <v>404</v>
@@ -21372,7 +21372,7 @@
     </row>
     <row r="368" spans="1:12">
       <c r="A368" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B368" t="s">
         <v>407</v>
@@ -21442,7 +21442,7 @@
     </row>
     <row r="370" spans="1:12">
       <c r="A370" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B370" t="s">
         <v>409</v>
@@ -21477,7 +21477,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B371" t="s">
         <v>410</v>
@@ -21512,7 +21512,7 @@
     </row>
     <row r="372" spans="1:12">
       <c r="A372" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B372" t="s">
         <v>411</v>
@@ -21827,7 +21827,7 @@
     </row>
     <row r="381" spans="1:12">
       <c r="A381" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B381" t="s">
         <v>420</v>
@@ -22002,7 +22002,7 @@
     </row>
     <row r="386" spans="1:12">
       <c r="A386" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B386" t="s">
         <v>425</v>
@@ -22072,7 +22072,7 @@
     </row>
     <row r="388" spans="1:12">
       <c r="A388" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B388" t="s">
         <v>427</v>
@@ -22212,7 +22212,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B392" t="s">
         <v>431</v>
@@ -22317,7 +22317,7 @@
     </row>
     <row r="395" spans="1:12">
       <c r="A395" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B395" t="s">
         <v>434</v>
@@ -22352,7 +22352,7 @@
     </row>
     <row r="396" spans="1:12">
       <c r="A396" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B396" t="s">
         <v>435</v>
@@ -22492,7 +22492,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B400" t="s">
         <v>439</v>
@@ -22527,7 +22527,7 @@
     </row>
     <row r="401" spans="1:12">
       <c r="A401" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B401" t="s">
         <v>440</v>
@@ -22772,7 +22772,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B408" t="s">
         <v>447</v>
@@ -22877,7 +22877,7 @@
     </row>
     <row r="411" spans="1:12">
       <c r="A411" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B411" t="s">
         <v>450</v>
@@ -22985,7 +22985,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B414" t="s">
         <v>453</v>
@@ -23055,7 +23055,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B416" t="s">
         <v>455</v>
@@ -23090,7 +23090,7 @@
     </row>
     <row r="417" spans="1:12">
       <c r="A417" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B417" t="s">
         <v>456</v>
@@ -23125,7 +23125,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B418" t="s">
         <v>457</v>
@@ -23160,7 +23160,7 @@
     </row>
     <row r="419" spans="1:12">
       <c r="A419" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B419" t="s">
         <v>458</v>
@@ -23195,7 +23195,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B420" t="s">
         <v>459</v>
@@ -23230,7 +23230,7 @@
     </row>
     <row r="421" spans="1:12">
       <c r="A421" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B421" t="s">
         <v>460</v>
@@ -23300,7 +23300,7 @@
     </row>
     <row r="423" spans="1:12">
       <c r="A423" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B423" t="s">
         <v>462</v>
@@ -23335,7 +23335,7 @@
     </row>
     <row r="424" spans="1:12">
       <c r="A424" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B424" t="s">
         <v>463</v>
@@ -23440,7 +23440,7 @@
     </row>
     <row r="427" spans="1:12">
       <c r="A427" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B427" t="s">
         <v>466</v>
@@ -23475,7 +23475,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B428" t="s">
         <v>467</v>
@@ -23510,7 +23510,7 @@
     </row>
     <row r="429" spans="1:12">
       <c r="A429" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B429" t="s">
         <v>468</v>
@@ -23580,7 +23580,7 @@
     </row>
     <row r="431" spans="1:12">
       <c r="A431" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B431" t="s">
         <v>470</v>
@@ -23650,7 +23650,7 @@
     </row>
     <row r="433" spans="1:12">
       <c r="A433" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B433" t="s">
         <v>472</v>
@@ -23685,7 +23685,7 @@
     </row>
     <row r="434" spans="1:12">
       <c r="A434" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B434" t="s">
         <v>473</v>
@@ -23755,7 +23755,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B436" t="s">
         <v>475</v>
@@ -23790,7 +23790,7 @@
     </row>
     <row r="437" spans="1:12">
       <c r="A437" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B437" t="s">
         <v>476</v>
@@ -23825,7 +23825,7 @@
     </row>
     <row r="438" spans="1:12">
       <c r="A438" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B438" t="s">
         <v>477</v>
@@ -23895,7 +23895,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B440" t="s">
         <v>479</v>
@@ -23965,7 +23965,7 @@
     </row>
     <row r="442" spans="1:12">
       <c r="A442" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B442" t="s">
         <v>481</v>
@@ -24000,7 +24000,7 @@
     </row>
     <row r="443" spans="1:12">
       <c r="A443" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B443" t="s">
         <v>482</v>
@@ -24035,7 +24035,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B444" t="s">
         <v>483</v>
@@ -24105,7 +24105,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B446" t="s">
         <v>485</v>
@@ -24248,7 +24248,7 @@
     </row>
     <row r="450" spans="1:12">
       <c r="A450" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B450" t="s">
         <v>489</v>
@@ -24318,7 +24318,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B452" t="s">
         <v>491</v>
@@ -24353,7 +24353,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B453" t="s">
         <v>492</v>
@@ -24388,7 +24388,7 @@
     </row>
     <row r="454" spans="1:12">
       <c r="A454" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B454" t="s">
         <v>493</v>
@@ -24528,7 +24528,7 @@
     </row>
     <row r="458" spans="1:12">
       <c r="A458" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B458" t="s">
         <v>497</v>
@@ -24598,7 +24598,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B460" t="s">
         <v>499</v>
@@ -24738,7 +24738,7 @@
     </row>
     <row r="464" spans="1:12">
       <c r="A464" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B464" t="s">
         <v>503</v>
@@ -24808,7 +24808,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B466" t="s">
         <v>505</v>
@@ -24913,7 +24913,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B469" t="s">
         <v>508</v>
@@ -24983,7 +24983,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B471" t="s">
         <v>510</v>
@@ -25018,7 +25018,7 @@
     </row>
     <row r="472" spans="1:12">
       <c r="A472" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B472" t="s">
         <v>511</v>
@@ -25088,7 +25088,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B474" t="s">
         <v>513</v>
@@ -25123,7 +25123,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B475" t="s">
         <v>514</v>
@@ -25158,7 +25158,7 @@
     </row>
     <row r="476" spans="1:12">
       <c r="A476" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B476" t="s">
         <v>515</v>
@@ -25263,7 +25263,7 @@
     </row>
     <row r="479" spans="1:12">
       <c r="A479" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B479" t="s">
         <v>518</v>
@@ -25403,7 +25403,7 @@
     </row>
     <row r="483" spans="1:12">
       <c r="A483" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B483" t="s">
         <v>522</v>
@@ -25438,7 +25438,7 @@
     </row>
     <row r="484" spans="1:12">
       <c r="A484" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B484" t="s">
         <v>523</v>
@@ -25473,7 +25473,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B485" t="s">
         <v>524</v>
@@ -25648,7 +25648,7 @@
     </row>
     <row r="490" spans="1:12">
       <c r="A490" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B490" t="s">
         <v>529</v>
@@ -25683,7 +25683,7 @@
     </row>
     <row r="491" spans="1:12">
       <c r="A491" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B491" t="s">
         <v>530</v>
@@ -25718,7 +25718,7 @@
     </row>
     <row r="492" spans="1:12">
       <c r="A492" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B492" t="s">
         <v>531</v>
@@ -25756,7 +25756,7 @@
     </row>
     <row r="493" spans="1:12">
       <c r="A493" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B493" t="s">
         <v>532</v>
@@ -25791,7 +25791,7 @@
     </row>
     <row r="494" spans="1:12">
       <c r="A494" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B494" t="s">
         <v>533</v>
@@ -26036,7 +26036,7 @@
     </row>
     <row r="501" spans="1:12">
       <c r="A501" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B501" t="s">
         <v>540</v>
@@ -26106,7 +26106,7 @@
     </row>
     <row r="503" spans="1:12">
       <c r="A503" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B503" t="s">
         <v>542</v>
@@ -26141,7 +26141,7 @@
     </row>
     <row r="504" spans="1:12">
       <c r="A504" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B504" t="s">
         <v>543</v>
@@ -26211,7 +26211,7 @@
     </row>
     <row r="506" spans="1:12">
       <c r="A506" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B506" t="s">
         <v>545</v>
@@ -26246,7 +26246,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B507" t="s">
         <v>546</v>
@@ -26526,7 +26526,7 @@
     </row>
     <row r="515" spans="1:12">
       <c r="A515" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B515" t="s">
         <v>554</v>
@@ -26596,7 +26596,7 @@
     </row>
     <row r="517" spans="1:12">
       <c r="A517" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B517" t="s">
         <v>556</v>
@@ -26666,7 +26666,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B519" t="s">
         <v>558</v>
@@ -26806,7 +26806,7 @@
     </row>
     <row r="523" spans="1:12">
       <c r="A523" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B523" t="s">
         <v>562</v>
@@ -26876,7 +26876,7 @@
     </row>
     <row r="525" spans="1:12">
       <c r="A525" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B525" t="s">
         <v>564</v>
@@ -26981,7 +26981,7 @@
     </row>
     <row r="528" spans="1:12">
       <c r="A528" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B528" t="s">
         <v>567</v>
@@ -27016,7 +27016,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B529" t="s">
         <v>568</v>
@@ -27194,7 +27194,7 @@
     </row>
     <row r="534" spans="1:12">
       <c r="A534" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B534" t="s">
         <v>573</v>
@@ -27229,7 +27229,7 @@
     </row>
     <row r="535" spans="1:12">
       <c r="A535" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B535" t="s">
         <v>574</v>
@@ -27299,7 +27299,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B537" t="s">
         <v>576</v>
@@ -27369,7 +27369,7 @@
     </row>
     <row r="539" spans="1:12">
       <c r="A539" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B539" t="s">
         <v>578</v>
@@ -27509,7 +27509,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B543" t="s">
         <v>582</v>
@@ -27544,7 +27544,7 @@
     </row>
     <row r="544" spans="1:12">
       <c r="A544" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B544" t="s">
         <v>583</v>
@@ -27579,7 +27579,7 @@
     </row>
     <row r="545" spans="1:12">
       <c r="A545" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B545" t="s">
         <v>584</v>
@@ -27614,7 +27614,7 @@
     </row>
     <row r="546" spans="1:12">
       <c r="A546" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B546" t="s">
         <v>585</v>
@@ -27649,7 +27649,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B547" t="s">
         <v>586</v>
@@ -27687,7 +27687,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B548" t="s">
         <v>587</v>
@@ -27722,7 +27722,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B549" t="s">
         <v>588</v>
@@ -27827,7 +27827,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B552" t="s">
         <v>591</v>
@@ -27862,7 +27862,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B553" t="s">
         <v>592</v>
@@ -28177,7 +28177,7 @@
     </row>
     <row r="562" spans="1:12">
       <c r="A562" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B562" t="s">
         <v>601</v>
@@ -28212,7 +28212,7 @@
     </row>
     <row r="563" spans="1:12">
       <c r="A563" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B563" t="s">
         <v>602</v>
@@ -28282,7 +28282,7 @@
     </row>
     <row r="565" spans="1:12">
       <c r="A565" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B565" t="s">
         <v>604</v>
@@ -28317,7 +28317,7 @@
     </row>
     <row r="566" spans="1:12">
       <c r="A566" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B566" t="s">
         <v>605</v>
@@ -28422,7 +28422,7 @@
     </row>
     <row r="569" spans="1:12">
       <c r="A569" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B569" t="s">
         <v>608</v>
@@ -28492,7 +28492,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B571" t="s">
         <v>610</v>
@@ -28527,7 +28527,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B572" t="s">
         <v>611</v>
@@ -28562,7 +28562,7 @@
     </row>
     <row r="573" spans="1:12">
       <c r="A573" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B573" t="s">
         <v>612</v>
@@ -28632,7 +28632,7 @@
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B575" t="s">
         <v>614</v>
@@ -28667,7 +28667,7 @@
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B576" t="s">
         <v>615</v>
@@ -28775,7 +28775,7 @@
     </row>
     <row r="579" spans="1:12">
       <c r="A579" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B579" t="s">
         <v>618</v>
@@ -28845,7 +28845,7 @@
     </row>
     <row r="581" spans="1:12">
       <c r="A581" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B581" t="s">
         <v>620</v>
@@ -28880,7 +28880,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B582" t="s">
         <v>621</v>
@@ -28915,7 +28915,7 @@
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B583" t="s">
         <v>622</v>
@@ -28953,7 +28953,7 @@
     </row>
     <row r="584" spans="1:12">
       <c r="A584" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B584" t="s">
         <v>623</v>
@@ -28988,7 +28988,7 @@
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B585" t="s">
         <v>624</v>
@@ -29023,7 +29023,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B586" t="s">
         <v>625</v>
@@ -29058,7 +29058,7 @@
     </row>
     <row r="587" spans="1:12">
       <c r="A587" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B587" t="s">
         <v>626</v>
@@ -29093,7 +29093,7 @@
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B588" t="s">
         <v>627</v>
@@ -29128,7 +29128,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B589" t="s">
         <v>628</v>
@@ -29163,7 +29163,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B590" t="s">
         <v>629</v>
@@ -29233,7 +29233,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B592" t="s">
         <v>631</v>
@@ -29268,7 +29268,7 @@
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B593" t="s">
         <v>632</v>
@@ -29303,7 +29303,7 @@
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B594" t="s">
         <v>633</v>
@@ -29373,7 +29373,7 @@
     </row>
     <row r="596" spans="1:12">
       <c r="A596" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B596" t="s">
         <v>635</v>
@@ -29446,7 +29446,7 @@
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B598" t="s">
         <v>637</v>
@@ -29481,7 +29481,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B599" t="s">
         <v>638</v>
@@ -29516,7 +29516,7 @@
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B600" t="s">
         <v>639</v>
@@ -29551,7 +29551,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B601" t="s">
         <v>640</v>
@@ -29586,7 +29586,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B602" t="s">
         <v>641</v>
@@ -29621,7 +29621,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B603" t="s">
         <v>642</v>
@@ -29656,7 +29656,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B604" t="s">
         <v>643</v>
@@ -29691,7 +29691,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B605" t="s">
         <v>644</v>
@@ -29761,7 +29761,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B607" t="s">
         <v>646</v>
@@ -29939,7 +29939,7 @@
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B612" t="s">
         <v>651</v>
@@ -30082,7 +30082,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B616" t="s">
         <v>655</v>
@@ -30117,7 +30117,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B617" t="s">
         <v>656</v>
@@ -30152,7 +30152,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B618" t="s">
         <v>657</v>
@@ -30225,7 +30225,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B620" t="s">
         <v>659</v>
@@ -30260,7 +30260,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B621" t="s">
         <v>660</v>
@@ -30295,7 +30295,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B622" t="s">
         <v>661</v>
@@ -30330,7 +30330,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B623" t="s">
         <v>662</v>
@@ -30403,7 +30403,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B625" t="s">
         <v>664</v>
@@ -30473,7 +30473,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B627" t="s">
         <v>666</v>
@@ -30581,7 +30581,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B630" t="s">
         <v>669</v>
@@ -30616,7 +30616,7 @@
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B631" t="s">
         <v>670</v>
@@ -30654,7 +30654,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B632" t="s">
         <v>671</v>
@@ -30689,7 +30689,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B633" t="s">
         <v>672</v>
@@ -30724,7 +30724,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B634" t="s">
         <v>673</v>
@@ -30797,7 +30797,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B636" t="s">
         <v>675</v>
@@ -30905,7 +30905,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B639" t="s">
         <v>678</v>
@@ -30940,7 +30940,7 @@
     </row>
     <row r="640" spans="1:12">
       <c r="A640" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B640" t="s">
         <v>679</v>
@@ -31200,7 +31200,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B647" t="s">
         <v>686</v>
@@ -31235,7 +31235,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B648" t="s">
         <v>687</v>
@@ -31270,7 +31270,7 @@
     </row>
     <row r="649" spans="1:12">
       <c r="A649" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B649" t="s">
         <v>688</v>
@@ -31448,7 +31448,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B654" t="s">
         <v>693</v>
@@ -31483,7 +31483,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B655" t="s">
         <v>694</v>
@@ -31518,7 +31518,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B656" t="s">
         <v>695</v>
@@ -31553,7 +31553,7 @@
     </row>
     <row r="657" spans="1:12">
       <c r="A657" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B657" t="s">
         <v>696</v>
@@ -31623,7 +31623,7 @@
     </row>
     <row r="659" spans="1:12">
       <c r="A659" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B659" t="s">
         <v>698</v>
@@ -31658,7 +31658,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B660" t="s">
         <v>699</v>
@@ -31693,7 +31693,7 @@
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B661" t="s">
         <v>700</v>
@@ -31728,7 +31728,7 @@
     </row>
     <row r="662" spans="1:12">
       <c r="A662" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B662" t="s">
         <v>701</v>
@@ -31763,7 +31763,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B663" t="s">
         <v>702</v>
@@ -31871,7 +31871,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B666" t="s">
         <v>705</v>
@@ -31906,7 +31906,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B667" t="s">
         <v>706</v>
@@ -31941,7 +31941,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B668" t="s">
         <v>707</v>
@@ -31979,7 +31979,7 @@
     </row>
     <row r="669" spans="1:12">
       <c r="A669" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B669" t="s">
         <v>708</v>
@@ -32017,7 +32017,7 @@
     </row>
     <row r="670" spans="1:12">
       <c r="A670" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B670" t="s">
         <v>709</v>
@@ -32128,7 +32128,7 @@
     </row>
     <row r="673" spans="1:12">
       <c r="A673" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B673" t="s">
         <v>712</v>
@@ -32201,7 +32201,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B675" t="s">
         <v>714</v>
@@ -32239,7 +32239,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B676" t="s">
         <v>715</v>
@@ -32274,7 +32274,7 @@
     </row>
     <row r="677" spans="1:12">
       <c r="A677" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B677" t="s">
         <v>716</v>
@@ -32309,7 +32309,7 @@
     </row>
     <row r="678" spans="1:12">
       <c r="A678" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B678" t="s">
         <v>717</v>
@@ -32347,7 +32347,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B679" t="s">
         <v>718</v>
@@ -32382,7 +32382,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B680" t="s">
         <v>719</v>
@@ -32417,7 +32417,7 @@
     </row>
     <row r="681" spans="1:12">
       <c r="A681" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B681" t="s">
         <v>720</v>
@@ -32452,7 +32452,7 @@
     </row>
     <row r="682" spans="1:12">
       <c r="A682" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B682" t="s">
         <v>721</v>
@@ -32487,7 +32487,7 @@
     </row>
     <row r="683" spans="1:12">
       <c r="A683" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B683" t="s">
         <v>722</v>
@@ -32522,7 +32522,7 @@
     </row>
     <row r="684" spans="1:12">
       <c r="A684" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B684" t="s">
         <v>723</v>
@@ -32554,7 +32554,7 @@
     </row>
     <row r="685" spans="1:12">
       <c r="A685" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B685" t="s">
         <v>724</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-28 12:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5104,6 +5104,9 @@
     <t>CELSO BARBOSA MONTENEGRO</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>ROSEMARY PROVENZANO THAMI</t>
   </si>
   <si>
@@ -5438,9 +5441,6 @@
   </si>
   <si>
     <t>DAGER SALLES AMARAL,EDUARDO COUTO SOLEDADE,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>PATRICIA FONTES ESTEVES</t>
@@ -10495,7 +10495,7 @@
         <v>1638</v>
       </c>
       <c r="I58" t="s">
-        <v>1678</v>
+        <v>1696</v>
       </c>
       <c r="J58" t="s">
         <v>1865</v>
@@ -10530,7 +10530,7 @@
         <v>1638</v>
       </c>
       <c r="I59" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J59" t="s">
         <v>1866</v>
@@ -10600,7 +10600,7 @@
         <v>1638</v>
       </c>
       <c r="I61" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J61" t="s">
         <v>1868</v>
@@ -10705,7 +10705,7 @@
         <v>1638</v>
       </c>
       <c r="I64" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J64" t="s">
         <v>1871</v>
@@ -10743,7 +10743,7 @@
         <v>1469</v>
       </c>
       <c r="I65" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J65" t="s">
         <v>1872</v>
@@ -10813,7 +10813,7 @@
         <v>1638</v>
       </c>
       <c r="I67" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="J67" t="s">
         <v>1874</v>
@@ -10848,7 +10848,7 @@
         <v>1638</v>
       </c>
       <c r="I68" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="J68" t="s">
         <v>1875</v>
@@ -10883,7 +10883,7 @@
         <v>1638</v>
       </c>
       <c r="I69" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="J69" t="s">
         <v>1876</v>
@@ -10991,7 +10991,7 @@
         <v>1638</v>
       </c>
       <c r="I72" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="J72" t="s">
         <v>1879</v>
@@ -11026,7 +11026,7 @@
         <v>1638</v>
       </c>
       <c r="I73" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J73" t="s">
         <v>1880</v>
@@ -11061,7 +11061,7 @@
         <v>1638</v>
       </c>
       <c r="I74" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="J74" t="s">
         <v>1881</v>
@@ -11166,7 +11166,7 @@
         <v>1638</v>
       </c>
       <c r="I77" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J77" t="s">
         <v>1884</v>
@@ -11201,7 +11201,7 @@
         <v>1638</v>
       </c>
       <c r="I78" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="J78" t="s">
         <v>1885</v>
@@ -11274,7 +11274,7 @@
         <v>1644</v>
       </c>
       <c r="I80" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J80" t="s">
         <v>1887</v>
@@ -11344,7 +11344,7 @@
         <v>1638</v>
       </c>
       <c r="I82" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J82" t="s">
         <v>1889</v>
@@ -11379,7 +11379,7 @@
         <v>1638</v>
       </c>
       <c r="I83" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J83" t="s">
         <v>1890</v>
@@ -11414,7 +11414,7 @@
         <v>1638</v>
       </c>
       <c r="I84" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="J84" t="s">
         <v>1891</v>
@@ -11519,7 +11519,7 @@
         <v>1638</v>
       </c>
       <c r="I87" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J87" t="s">
         <v>1894</v>
@@ -11554,7 +11554,7 @@
         <v>1638</v>
       </c>
       <c r="I88" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J88" t="s">
         <v>1895</v>
@@ -11589,7 +11589,7 @@
         <v>1638</v>
       </c>
       <c r="I89" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J89" t="s">
         <v>1895</v>
@@ -11694,7 +11694,7 @@
         <v>1638</v>
       </c>
       <c r="I92" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J92" t="s">
         <v>1897</v>
@@ -11729,7 +11729,7 @@
         <v>1638</v>
       </c>
       <c r="I93" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J93" t="s">
         <v>1898</v>
@@ -11767,7 +11767,7 @@
         <v>1645</v>
       </c>
       <c r="I94" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J94" t="s">
         <v>1899</v>
@@ -11805,7 +11805,7 @@
         <v>1645</v>
       </c>
       <c r="I95" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J95" t="s">
         <v>1899</v>
@@ -11875,7 +11875,7 @@
         <v>1638</v>
       </c>
       <c r="I97" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="J97" t="s">
         <v>1901</v>
@@ -12085,7 +12085,7 @@
         <v>1640</v>
       </c>
       <c r="I103" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J103" t="s">
         <v>1907</v>
@@ -12120,7 +12120,7 @@
         <v>1638</v>
       </c>
       <c r="I104" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J104" t="s">
         <v>1908</v>
@@ -12190,7 +12190,7 @@
         <v>1638</v>
       </c>
       <c r="I106" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J106" t="s">
         <v>1910</v>
@@ -12470,7 +12470,7 @@
         <v>1638</v>
       </c>
       <c r="I114" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J114" t="s">
         <v>1918</v>
@@ -12575,7 +12575,7 @@
         <v>1638</v>
       </c>
       <c r="I117" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J117" t="s">
         <v>1921</v>
@@ -12610,7 +12610,7 @@
         <v>1638</v>
       </c>
       <c r="I118" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J118" t="s">
         <v>1922</v>
@@ -12785,7 +12785,7 @@
         <v>1638</v>
       </c>
       <c r="I123" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J123" t="s">
         <v>1927</v>
@@ -12820,7 +12820,7 @@
         <v>1638</v>
       </c>
       <c r="I124" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J124" t="s">
         <v>1928</v>
@@ -12890,7 +12890,7 @@
         <v>1638</v>
       </c>
       <c r="I126" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J126" t="s">
         <v>1930</v>
@@ -12995,7 +12995,7 @@
         <v>1638</v>
       </c>
       <c r="I129" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J129" t="s">
         <v>1933</v>
@@ -13065,7 +13065,7 @@
         <v>1638</v>
       </c>
       <c r="I131" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J131" t="s">
         <v>1935</v>
@@ -13135,7 +13135,7 @@
         <v>1638</v>
       </c>
       <c r="I133" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J133" t="s">
         <v>1937</v>
@@ -13205,7 +13205,7 @@
         <v>1638</v>
       </c>
       <c r="I135" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="J135" t="s">
         <v>1939</v>
@@ -13348,7 +13348,7 @@
         <v>1638</v>
       </c>
       <c r="I139" t="s">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="J139" t="s">
         <v>1943</v>
@@ -13418,7 +13418,7 @@
         <v>1638</v>
       </c>
       <c r="I141" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="J141" t="s">
         <v>1944</v>
@@ -13453,7 +13453,7 @@
         <v>1638</v>
       </c>
       <c r="I142" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J142" t="s">
         <v>1945</v>
@@ -13523,7 +13523,7 @@
         <v>1638</v>
       </c>
       <c r="I144" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J144" t="s">
         <v>1947</v>
@@ -13698,7 +13698,7 @@
         <v>1638</v>
       </c>
       <c r="I149" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J149" t="s">
         <v>1951</v>
@@ -13733,7 +13733,7 @@
         <v>1638</v>
       </c>
       <c r="I150" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J150" t="s">
         <v>1952</v>
@@ -13876,7 +13876,7 @@
         <v>1638</v>
       </c>
       <c r="I154" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J154" t="s">
         <v>1955</v>
@@ -13911,7 +13911,7 @@
         <v>1638</v>
       </c>
       <c r="I155" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="J155" t="s">
         <v>1956</v>
@@ -13946,7 +13946,7 @@
         <v>1638</v>
       </c>
       <c r="I156" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J156" t="s">
         <v>1957</v>
@@ -14016,7 +14016,7 @@
         <v>1638</v>
       </c>
       <c r="I158" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J158" t="s">
         <v>1959</v>
@@ -14051,7 +14051,7 @@
         <v>1638</v>
       </c>
       <c r="I159" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="J159" t="s">
         <v>1960</v>
@@ -14121,7 +14121,7 @@
         <v>1638</v>
       </c>
       <c r="I161" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J161" t="s">
         <v>1962</v>
@@ -14261,7 +14261,7 @@
         <v>1638</v>
       </c>
       <c r="I165" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J165" t="s">
         <v>1966</v>
@@ -14331,7 +14331,7 @@
         <v>1638</v>
       </c>
       <c r="I167" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J167" t="s">
         <v>1968</v>
@@ -14611,7 +14611,7 @@
         <v>1638</v>
       </c>
       <c r="I175" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J175" t="s">
         <v>1976</v>
@@ -14646,7 +14646,7 @@
         <v>1638</v>
       </c>
       <c r="I176" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J176" t="s">
         <v>1977</v>
@@ -14716,7 +14716,7 @@
         <v>1638</v>
       </c>
       <c r="I178" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="J178" t="s">
         <v>1979</v>
@@ -14786,7 +14786,7 @@
         <v>1638</v>
       </c>
       <c r="I180" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="J180" t="s">
         <v>1981</v>
@@ -14891,7 +14891,7 @@
         <v>1638</v>
       </c>
       <c r="I183" t="s">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="J183" t="s">
         <v>1984</v>
@@ -14926,7 +14926,7 @@
         <v>1638</v>
       </c>
       <c r="I184" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J184" t="s">
         <v>1985</v>
@@ -14961,7 +14961,7 @@
         <v>1638</v>
       </c>
       <c r="I185" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J185" t="s">
         <v>1986</v>
@@ -14996,7 +14996,7 @@
         <v>1638</v>
       </c>
       <c r="I186" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J186" t="s">
         <v>1987</v>
@@ -15136,7 +15136,7 @@
         <v>1638</v>
       </c>
       <c r="I190" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J190" t="s">
         <v>1991</v>
@@ -15381,7 +15381,7 @@
         <v>1638</v>
       </c>
       <c r="I197" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J197" t="s">
         <v>1998</v>
@@ -15416,7 +15416,7 @@
         <v>1638</v>
       </c>
       <c r="I198" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J198" t="s">
         <v>1890</v>
@@ -15626,7 +15626,7 @@
         <v>1638</v>
       </c>
       <c r="I204" t="s">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="J204" t="s">
         <v>2003</v>
@@ -15699,7 +15699,7 @@
         <v>1543</v>
       </c>
       <c r="I206" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J206" t="s">
         <v>2005</v>
@@ -15769,7 +15769,7 @@
         <v>1638</v>
       </c>
       <c r="I208" t="s">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="J208" t="s">
         <v>2007</v>
@@ -15979,7 +15979,7 @@
         <v>1638</v>
       </c>
       <c r="I214" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J214" t="s">
         <v>2013</v>
@@ -16014,7 +16014,7 @@
         <v>1638</v>
       </c>
       <c r="I215" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J215" t="s">
         <v>2014</v>
@@ -16049,7 +16049,7 @@
         <v>1640</v>
       </c>
       <c r="I216" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J216" t="s">
         <v>2015</v>
@@ -16084,7 +16084,7 @@
         <v>1638</v>
       </c>
       <c r="I217" t="s">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="J217" t="s">
         <v>2016</v>
@@ -16119,7 +16119,7 @@
         <v>1638</v>
       </c>
       <c r="I218" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J218" t="s">
         <v>2017</v>
@@ -16154,7 +16154,7 @@
         <v>1638</v>
       </c>
       <c r="I219" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="J219" t="s">
         <v>2018</v>
@@ -16224,7 +16224,7 @@
         <v>1638</v>
       </c>
       <c r="I221" t="s">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="J221" t="s">
         <v>2020</v>
@@ -16259,7 +16259,7 @@
         <v>1638</v>
       </c>
       <c r="I222" t="s">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="J222" t="s">
         <v>2021</v>
@@ -16329,7 +16329,7 @@
         <v>1638</v>
       </c>
       <c r="I224" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="J224" t="s">
         <v>2023</v>
@@ -16399,7 +16399,7 @@
         <v>1638</v>
       </c>
       <c r="I226" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J226" t="s">
         <v>2025</v>
@@ -16434,7 +16434,7 @@
         <v>1638</v>
       </c>
       <c r="I227" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J227" t="s">
         <v>2026</v>
@@ -16469,7 +16469,7 @@
         <v>1638</v>
       </c>
       <c r="I228" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J228" t="s">
         <v>2027</v>
@@ -16609,7 +16609,7 @@
         <v>1638</v>
       </c>
       <c r="I232" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J232" t="s">
         <v>2031</v>
@@ -16679,7 +16679,7 @@
         <v>1638</v>
       </c>
       <c r="I234" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J234" t="s">
         <v>2033</v>
@@ -16819,7 +16819,7 @@
         <v>1638</v>
       </c>
       <c r="I238" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J238" t="s">
         <v>2037</v>
@@ -16854,7 +16854,7 @@
         <v>1638</v>
       </c>
       <c r="I239" t="s">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="J239" t="s">
         <v>1895</v>
@@ -16889,7 +16889,7 @@
         <v>1638</v>
       </c>
       <c r="I240" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J240" t="s">
         <v>2038</v>
@@ -16924,7 +16924,7 @@
         <v>1638</v>
       </c>
       <c r="I241" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J241" t="s">
         <v>2039</v>
@@ -16959,7 +16959,7 @@
         <v>1638</v>
       </c>
       <c r="I242" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="J242" t="s">
         <v>2040</v>
@@ -17204,7 +17204,7 @@
         <v>1638</v>
       </c>
       <c r="I249" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="J249" t="s">
         <v>2047</v>
@@ -17239,7 +17239,7 @@
         <v>1638</v>
       </c>
       <c r="I250" t="s">
-        <v>1758</v>
+        <v>1759</v>
       </c>
       <c r="J250" t="s">
         <v>2048</v>
@@ -17274,7 +17274,7 @@
         <v>1638</v>
       </c>
       <c r="I251" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J251" t="s">
         <v>2049</v>
@@ -17312,7 +17312,7 @@
         <v>1553</v>
       </c>
       <c r="I252" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="J252" t="s">
         <v>2050</v>
@@ -17417,7 +17417,7 @@
         <v>1638</v>
       </c>
       <c r="I255" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J255" t="s">
         <v>2053</v>
@@ -17487,7 +17487,7 @@
         <v>1638</v>
       </c>
       <c r="I257" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J257" t="s">
         <v>2055</v>
@@ -17592,7 +17592,7 @@
         <v>1638</v>
       </c>
       <c r="I260" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J260" t="s">
         <v>2058</v>
@@ -17732,7 +17732,7 @@
         <v>1638</v>
       </c>
       <c r="I264" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J264" t="s">
         <v>2062</v>
@@ -17837,7 +17837,7 @@
         <v>1638</v>
       </c>
       <c r="I267" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J267" t="s">
         <v>2065</v>
@@ -17907,7 +17907,7 @@
         <v>1638</v>
       </c>
       <c r="I269" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J269" t="s">
         <v>2067</v>
@@ -18050,7 +18050,7 @@
         <v>1647</v>
       </c>
       <c r="I273" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J273" t="s">
         <v>2071</v>
@@ -18155,7 +18155,7 @@
         <v>1638</v>
       </c>
       <c r="I276" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J276" t="s">
         <v>2074</v>
@@ -18190,7 +18190,7 @@
         <v>1638</v>
       </c>
       <c r="I277" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J277" t="s">
         <v>2075</v>
@@ -18225,7 +18225,7 @@
         <v>1638</v>
       </c>
       <c r="I278" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J278" t="s">
         <v>2076</v>
@@ -18295,7 +18295,7 @@
         <v>1638</v>
       </c>
       <c r="I280" t="s">
-        <v>1764</v>
+        <v>1765</v>
       </c>
       <c r="J280" t="s">
         <v>2078</v>
@@ -18330,7 +18330,7 @@
         <v>1638</v>
       </c>
       <c r="I281" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J281" t="s">
         <v>2079</v>
@@ -18365,7 +18365,7 @@
         <v>1638</v>
       </c>
       <c r="I282" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J282" t="s">
         <v>2080</v>
@@ -18400,7 +18400,7 @@
         <v>1638</v>
       </c>
       <c r="I283" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J283" t="s">
         <v>2081</v>
@@ -18540,7 +18540,7 @@
         <v>1638</v>
       </c>
       <c r="I287" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J287" t="s">
         <v>2084</v>
@@ -18575,7 +18575,7 @@
         <v>1638</v>
       </c>
       <c r="I288" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J288" t="s">
         <v>2085</v>
@@ -18645,7 +18645,7 @@
         <v>1638</v>
       </c>
       <c r="I290" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J290" t="s">
         <v>2087</v>
@@ -18680,7 +18680,7 @@
         <v>1638</v>
       </c>
       <c r="I291" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J291" t="s">
         <v>2088</v>
@@ -18718,7 +18718,7 @@
         <v>1648</v>
       </c>
       <c r="I292" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J292" t="s">
         <v>2089</v>
@@ -18858,7 +18858,7 @@
         <v>1638</v>
       </c>
       <c r="I296" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J296" t="s">
         <v>2092</v>
@@ -18893,7 +18893,7 @@
         <v>1638</v>
       </c>
       <c r="I297" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J297" t="s">
         <v>2093</v>
@@ -19138,7 +19138,7 @@
         <v>1638</v>
       </c>
       <c r="I304" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J304" t="s">
         <v>2100</v>
@@ -19208,7 +19208,7 @@
         <v>1638</v>
       </c>
       <c r="I306" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J306" t="s">
         <v>2102</v>
@@ -19278,7 +19278,7 @@
         <v>1638</v>
       </c>
       <c r="I308" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J308" t="s">
         <v>2104</v>
@@ -19313,7 +19313,7 @@
         <v>1638</v>
       </c>
       <c r="I309" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J309" t="s">
         <v>2105</v>
@@ -19526,7 +19526,7 @@
         <v>1638</v>
       </c>
       <c r="I315" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J315" t="s">
         <v>2111</v>
@@ -19561,7 +19561,7 @@
         <v>1638</v>
       </c>
       <c r="I316" t="s">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="J316" t="s">
         <v>2112</v>
@@ -19736,7 +19736,7 @@
         <v>1638</v>
       </c>
       <c r="I321" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J321" t="s">
         <v>2117</v>
@@ -19771,7 +19771,7 @@
         <v>1638</v>
       </c>
       <c r="I322" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J322" t="s">
         <v>2118</v>
@@ -19806,7 +19806,7 @@
         <v>1638</v>
       </c>
       <c r="I323" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="J323" t="s">
         <v>2119</v>
@@ -19911,7 +19911,7 @@
         <v>1638</v>
       </c>
       <c r="I326" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="J326" t="s">
         <v>2122</v>
@@ -19981,7 +19981,7 @@
         <v>1638</v>
       </c>
       <c r="I328" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
       <c r="J328" t="s">
         <v>2124</v>
@@ -20016,7 +20016,7 @@
         <v>1638</v>
       </c>
       <c r="I329" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="J329" t="s">
         <v>2125</v>
@@ -20051,7 +20051,7 @@
         <v>1638</v>
       </c>
       <c r="I330" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J330" t="s">
         <v>2126</v>
@@ -20191,7 +20191,7 @@
         <v>1638</v>
       </c>
       <c r="I334" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J334" t="s">
         <v>2130</v>
@@ -20226,7 +20226,7 @@
         <v>1638</v>
       </c>
       <c r="I335" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J335" t="s">
         <v>2131</v>
@@ -20296,7 +20296,7 @@
         <v>1638</v>
       </c>
       <c r="I337" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J337" t="s">
         <v>2133</v>
@@ -20401,7 +20401,7 @@
         <v>1638</v>
       </c>
       <c r="I340" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J340" t="s">
         <v>2136</v>
@@ -20436,7 +20436,7 @@
         <v>1638</v>
       </c>
       <c r="I341" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
       <c r="J341" t="s">
         <v>2137</v>
@@ -20471,7 +20471,7 @@
         <v>1638</v>
       </c>
       <c r="I342" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J342" t="s">
         <v>2138</v>
@@ -20506,7 +20506,7 @@
         <v>1638</v>
       </c>
       <c r="I343" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J343" t="s">
         <v>2139</v>
@@ -20576,7 +20576,7 @@
         <v>1638</v>
       </c>
       <c r="I345" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J345" t="s">
         <v>2141</v>
@@ -20611,7 +20611,7 @@
         <v>1638</v>
       </c>
       <c r="I346" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="J346" t="s">
         <v>2142</v>
@@ -20649,7 +20649,7 @@
         <v>1650</v>
       </c>
       <c r="I347" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J347" t="s">
         <v>2143</v>
@@ -20754,7 +20754,7 @@
         <v>1638</v>
       </c>
       <c r="I350" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J350" t="s">
         <v>2146</v>
@@ -20894,7 +20894,7 @@
         <v>1638</v>
       </c>
       <c r="I354" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J354" t="s">
         <v>2150</v>
@@ -20929,7 +20929,7 @@
         <v>1638</v>
       </c>
       <c r="I355" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
       <c r="J355" t="s">
         <v>2151</v>
@@ -20999,7 +20999,7 @@
         <v>1638</v>
       </c>
       <c r="I357" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J357" t="s">
         <v>2153</v>
@@ -21069,7 +21069,7 @@
         <v>1638</v>
       </c>
       <c r="I359" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="J359" t="s">
         <v>2155</v>
@@ -21104,7 +21104,7 @@
         <v>1638</v>
       </c>
       <c r="I360" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="J360" t="s">
         <v>2156</v>
@@ -21209,7 +21209,7 @@
         <v>1638</v>
       </c>
       <c r="I363" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
       <c r="J363" t="s">
         <v>2159</v>
@@ -21244,7 +21244,7 @@
         <v>1638</v>
       </c>
       <c r="I364" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J364" t="s">
         <v>2160</v>
@@ -21317,7 +21317,7 @@
         <v>1589</v>
       </c>
       <c r="I366" t="s">
-        <v>1778</v>
+        <v>1779</v>
       </c>
       <c r="J366" t="s">
         <v>2162</v>
@@ -21352,7 +21352,7 @@
         <v>1638</v>
       </c>
       <c r="I367" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J367" t="s">
         <v>2163</v>
@@ -21422,7 +21422,7 @@
         <v>1638</v>
       </c>
       <c r="I369" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J369" t="s">
         <v>2165</v>
@@ -21457,7 +21457,7 @@
         <v>1638</v>
       </c>
       <c r="I370" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J370" t="s">
         <v>2166</v>
@@ -21492,7 +21492,7 @@
         <v>1638</v>
       </c>
       <c r="I371" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J371" t="s">
         <v>2167</v>
@@ -21527,7 +21527,7 @@
         <v>1638</v>
       </c>
       <c r="I372" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
       <c r="J372" t="s">
         <v>2168</v>
@@ -21667,7 +21667,7 @@
         <v>1638</v>
       </c>
       <c r="I376" t="s">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="J376" t="s">
         <v>2172</v>
@@ -21737,7 +21737,7 @@
         <v>1638</v>
       </c>
       <c r="I378" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="J378" t="s">
         <v>2174</v>
@@ -21807,7 +21807,7 @@
         <v>1638</v>
       </c>
       <c r="I380" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J380" t="s">
         <v>2176</v>
@@ -21947,7 +21947,7 @@
         <v>1638</v>
       </c>
       <c r="I384" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J384" t="s">
         <v>2180</v>
@@ -21982,7 +21982,7 @@
         <v>1638</v>
       </c>
       <c r="I385" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J385" t="s">
         <v>2181</v>
@@ -22052,7 +22052,7 @@
         <v>1638</v>
       </c>
       <c r="I387" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J387" t="s">
         <v>2183</v>
@@ -22192,7 +22192,7 @@
         <v>1638</v>
       </c>
       <c r="I391" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J391" t="s">
         <v>2187</v>
@@ -22332,7 +22332,7 @@
         <v>1638</v>
       </c>
       <c r="I395" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J395" t="s">
         <v>2191</v>
@@ -22472,7 +22472,7 @@
         <v>1638</v>
       </c>
       <c r="I399" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J399" t="s">
         <v>2195</v>
@@ -22507,7 +22507,7 @@
         <v>1638</v>
       </c>
       <c r="I400" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J400" t="s">
         <v>2001</v>
@@ -22752,7 +22752,7 @@
         <v>1638</v>
       </c>
       <c r="I407" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J407" t="s">
         <v>2202</v>
@@ -22857,7 +22857,7 @@
         <v>1638</v>
       </c>
       <c r="I410" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J410" t="s">
         <v>2205</v>
@@ -22895,7 +22895,7 @@
         <v>1651</v>
       </c>
       <c r="I411" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J411" t="s">
         <v>2206</v>
@@ -22965,7 +22965,7 @@
         <v>1638</v>
       </c>
       <c r="I413" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J413" t="s">
         <v>2208</v>
@@ -23035,7 +23035,7 @@
         <v>1638</v>
       </c>
       <c r="I415" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J415" t="s">
         <v>2209</v>
@@ -23070,7 +23070,7 @@
         <v>1638</v>
       </c>
       <c r="I416" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J416" t="s">
         <v>2210</v>
@@ -23140,7 +23140,7 @@
         <v>1638</v>
       </c>
       <c r="I418" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J418" t="s">
         <v>2212</v>
@@ -23175,7 +23175,7 @@
         <v>1638</v>
       </c>
       <c r="I419" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J419" t="s">
         <v>2213</v>
@@ -23210,7 +23210,7 @@
         <v>1638</v>
       </c>
       <c r="I420" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J420" t="s">
         <v>2214</v>
@@ -23280,7 +23280,7 @@
         <v>1638</v>
       </c>
       <c r="I422" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J422" t="s">
         <v>2216</v>
@@ -23315,7 +23315,7 @@
         <v>1638</v>
       </c>
       <c r="I423" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J423" t="s">
         <v>2217</v>
@@ -23385,7 +23385,7 @@
         <v>1638</v>
       </c>
       <c r="I425" t="s">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="J425" t="s">
         <v>2219</v>
@@ -23420,7 +23420,7 @@
         <v>1638</v>
       </c>
       <c r="I426" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J426" t="s">
         <v>2220</v>
@@ -23455,7 +23455,7 @@
         <v>1638</v>
       </c>
       <c r="I427" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J427" t="s">
         <v>2221</v>
@@ -23560,7 +23560,7 @@
         <v>1638</v>
       </c>
       <c r="I430" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J430" t="s">
         <v>2224</v>
@@ -23665,7 +23665,7 @@
         <v>1638</v>
       </c>
       <c r="I433" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J433" t="s">
         <v>2227</v>
@@ -23735,7 +23735,7 @@
         <v>1638</v>
       </c>
       <c r="I435" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J435" t="s">
         <v>2229</v>
@@ -23770,7 +23770,7 @@
         <v>1638</v>
       </c>
       <c r="I436" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J436" t="s">
         <v>2230</v>
@@ -23805,7 +23805,7 @@
         <v>1638</v>
       </c>
       <c r="I437" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J437" t="s">
         <v>2231</v>
@@ -23875,7 +23875,7 @@
         <v>1638</v>
       </c>
       <c r="I439" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J439" t="s">
         <v>2233</v>
@@ -23945,7 +23945,7 @@
         <v>1638</v>
       </c>
       <c r="I441" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J441" t="s">
         <v>2235</v>
@@ -23980,7 +23980,7 @@
         <v>1638</v>
       </c>
       <c r="I442" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J442" t="s">
         <v>2236</v>
@@ -24015,7 +24015,7 @@
         <v>1638</v>
       </c>
       <c r="I443" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J443" t="s">
         <v>2237</v>
@@ -24085,7 +24085,7 @@
         <v>1638</v>
       </c>
       <c r="I445" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J445" t="s">
         <v>2239</v>
@@ -24193,7 +24193,7 @@
         <v>1652</v>
       </c>
       <c r="I448" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J448" t="s">
         <v>2242</v>
@@ -24228,7 +24228,7 @@
         <v>1638</v>
       </c>
       <c r="I449" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J449" t="s">
         <v>2243</v>
@@ -24333,7 +24333,7 @@
         <v>1638</v>
       </c>
       <c r="I452" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J452" t="s">
         <v>2246</v>
@@ -24368,7 +24368,7 @@
         <v>1638</v>
       </c>
       <c r="I453" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J453" t="s">
         <v>2247</v>
@@ -24438,7 +24438,7 @@
         <v>1638</v>
       </c>
       <c r="I455" t="s">
-        <v>1785</v>
+        <v>1786</v>
       </c>
       <c r="J455" t="s">
         <v>2249</v>
@@ -24508,7 +24508,7 @@
         <v>1638</v>
       </c>
       <c r="I457" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J457" t="s">
         <v>2251</v>
@@ -24543,7 +24543,7 @@
         <v>1638</v>
       </c>
       <c r="I458" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J458" t="s">
         <v>2252</v>
@@ -24578,7 +24578,7 @@
         <v>1638</v>
       </c>
       <c r="I459" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J459" t="s">
         <v>2253</v>
@@ -24648,7 +24648,7 @@
         <v>1638</v>
       </c>
       <c r="I461" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J461" t="s">
         <v>2255</v>
@@ -24718,7 +24718,7 @@
         <v>1638</v>
       </c>
       <c r="I463" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J463" t="s">
         <v>2257</v>
@@ -24753,7 +24753,7 @@
         <v>1638</v>
       </c>
       <c r="I464" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J464" t="s">
         <v>2258</v>
@@ -24788,7 +24788,7 @@
         <v>1638</v>
       </c>
       <c r="I465" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J465" t="s">
         <v>2259</v>
@@ -24893,7 +24893,7 @@
         <v>1638</v>
       </c>
       <c r="I468" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J468" t="s">
         <v>2262</v>
@@ -24928,7 +24928,7 @@
         <v>1638</v>
       </c>
       <c r="I469" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J469" t="s">
         <v>2263</v>
@@ -24963,7 +24963,7 @@
         <v>1638</v>
       </c>
       <c r="I470" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J470" t="s">
         <v>2264</v>
@@ -24998,7 +24998,7 @@
         <v>1638</v>
       </c>
       <c r="I471" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J471" t="s">
         <v>2265</v>
@@ -25033,7 +25033,7 @@
         <v>1638</v>
       </c>
       <c r="I472" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J472" t="s">
         <v>2266</v>
@@ -25068,7 +25068,7 @@
         <v>1638</v>
       </c>
       <c r="I473" t="s">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="J473" t="s">
         <v>2267</v>
@@ -25103,7 +25103,7 @@
         <v>1638</v>
       </c>
       <c r="I474" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J474" t="s">
         <v>2268</v>
@@ -25138,7 +25138,7 @@
         <v>1638</v>
       </c>
       <c r="I475" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J475" t="s">
         <v>2269</v>
@@ -25243,7 +25243,7 @@
         <v>1638</v>
       </c>
       <c r="I478" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J478" t="s">
         <v>2272</v>
@@ -25383,7 +25383,7 @@
         <v>1638</v>
       </c>
       <c r="I482" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J482" t="s">
         <v>2276</v>
@@ -25418,7 +25418,7 @@
         <v>1638</v>
       </c>
       <c r="I483" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J483" t="s">
         <v>2277</v>
@@ -25453,7 +25453,7 @@
         <v>1638</v>
       </c>
       <c r="I484" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J484" t="s">
         <v>2278</v>
@@ -25593,7 +25593,7 @@
         <v>1638</v>
       </c>
       <c r="I488" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="J488" t="s">
         <v>2282</v>
@@ -25628,7 +25628,7 @@
         <v>1638</v>
       </c>
       <c r="I489" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J489" t="s">
         <v>2283</v>
@@ -25663,7 +25663,7 @@
         <v>1638</v>
       </c>
       <c r="I490" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J490" t="s">
         <v>2284</v>
@@ -25701,7 +25701,7 @@
         <v>1653</v>
       </c>
       <c r="I491" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J491" t="s">
         <v>2285</v>
@@ -25736,7 +25736,7 @@
         <v>1638</v>
       </c>
       <c r="I492" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J492" t="s">
         <v>2286</v>
@@ -25771,7 +25771,7 @@
         <v>1638</v>
       </c>
       <c r="I493" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J493" t="s">
         <v>2287</v>
@@ -25981,7 +25981,7 @@
         <v>1638</v>
       </c>
       <c r="I499" t="s">
-        <v>1787</v>
+        <v>1788</v>
       </c>
       <c r="J499" t="s">
         <v>2293</v>
@@ -26016,7 +26016,7 @@
         <v>1638</v>
       </c>
       <c r="I500" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J500" t="s">
         <v>2294</v>
@@ -26086,7 +26086,7 @@
         <v>1638</v>
       </c>
       <c r="I502" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J502" t="s">
         <v>2296</v>
@@ -26121,7 +26121,7 @@
         <v>1638</v>
       </c>
       <c r="I503" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J503" t="s">
         <v>2297</v>
@@ -26191,7 +26191,7 @@
         <v>1638</v>
       </c>
       <c r="I505" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J505" t="s">
         <v>2299</v>
@@ -26226,7 +26226,7 @@
         <v>1638</v>
       </c>
       <c r="I506" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J506" t="s">
         <v>2300</v>
@@ -26331,7 +26331,7 @@
         <v>1638</v>
       </c>
       <c r="I509" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="J509" t="s">
         <v>2303</v>
@@ -26401,7 +26401,7 @@
         <v>1638</v>
       </c>
       <c r="I511" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="J511" t="s">
         <v>2305</v>
@@ -26506,7 +26506,7 @@
         <v>1638</v>
       </c>
       <c r="I514" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J514" t="s">
         <v>2308</v>
@@ -26541,7 +26541,7 @@
         <v>1638</v>
       </c>
       <c r="I515" t="s">
-        <v>1768</v>
+        <v>1746</v>
       </c>
       <c r="J515" t="s">
         <v>2309</v>
@@ -26576,7 +26576,7 @@
         <v>1638</v>
       </c>
       <c r="I516" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J516" t="s">
         <v>2310</v>
@@ -26611,7 +26611,7 @@
         <v>1638</v>
       </c>
       <c r="I517" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J517" t="s">
         <v>2311</v>
@@ -26646,7 +26646,7 @@
         <v>1638</v>
       </c>
       <c r="I518" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J518" t="s">
         <v>2312</v>
@@ -26681,7 +26681,7 @@
         <v>1638</v>
       </c>
       <c r="I519" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J519" t="s">
         <v>2313</v>
@@ -26716,7 +26716,7 @@
         <v>1638</v>
       </c>
       <c r="I520" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J520" t="s">
         <v>2314</v>
@@ -26786,7 +26786,7 @@
         <v>1638</v>
       </c>
       <c r="I522" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J522" t="s">
         <v>2316</v>
@@ -26856,7 +26856,7 @@
         <v>1638</v>
       </c>
       <c r="I524" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J524" t="s">
         <v>2318</v>
@@ -26961,7 +26961,7 @@
         <v>1638</v>
       </c>
       <c r="I527" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J527" t="s">
         <v>2321</v>
@@ -26996,7 +26996,7 @@
         <v>1638</v>
       </c>
       <c r="I528" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J528" t="s">
         <v>2322</v>
@@ -27031,7 +27031,7 @@
         <v>1638</v>
       </c>
       <c r="I529" t="s">
-        <v>1790</v>
+        <v>1791</v>
       </c>
       <c r="J529" t="s">
         <v>2323</v>
@@ -27174,7 +27174,7 @@
         <v>1638</v>
       </c>
       <c r="I533" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J533" t="s">
         <v>2327</v>
@@ -27209,7 +27209,7 @@
         <v>1638</v>
       </c>
       <c r="I534" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J534" t="s">
         <v>2328</v>
@@ -27244,7 +27244,7 @@
         <v>1638</v>
       </c>
       <c r="I535" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J535" t="s">
         <v>2329</v>
@@ -27279,7 +27279,7 @@
         <v>1638</v>
       </c>
       <c r="I536" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J536" t="s">
         <v>2330</v>
@@ -27349,7 +27349,7 @@
         <v>1638</v>
       </c>
       <c r="I538" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J538" t="s">
         <v>2332</v>
@@ -27384,7 +27384,7 @@
         <v>1638</v>
       </c>
       <c r="I539" t="s">
-        <v>1791</v>
+        <v>1792</v>
       </c>
       <c r="J539" t="s">
         <v>2333</v>
@@ -27454,7 +27454,7 @@
         <v>1638</v>
       </c>
       <c r="I541" t="s">
-        <v>1792</v>
+        <v>1793</v>
       </c>
       <c r="J541" t="s">
         <v>2335</v>
@@ -27489,7 +27489,7 @@
         <v>1638</v>
       </c>
       <c r="I542" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J542" t="s">
         <v>2336</v>
@@ -27632,7 +27632,7 @@
         <v>1655</v>
       </c>
       <c r="I546" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J546" t="s">
         <v>2340</v>
@@ -27667,7 +27667,7 @@
         <v>1638</v>
       </c>
       <c r="I547" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J547" t="s">
         <v>2341</v>
@@ -27702,7 +27702,7 @@
         <v>1638</v>
       </c>
       <c r="I548" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J548" t="s">
         <v>2342</v>
@@ -27807,7 +27807,7 @@
         <v>1638</v>
       </c>
       <c r="I551" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J551" t="s">
         <v>2345</v>
@@ -27842,7 +27842,7 @@
         <v>1638</v>
       </c>
       <c r="I552" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J552" t="s">
         <v>2346</v>
@@ -27982,7 +27982,7 @@
         <v>1638</v>
       </c>
       <c r="I556" t="s">
-        <v>1793</v>
+        <v>1794</v>
       </c>
       <c r="J556" t="s">
         <v>2350</v>
@@ -28122,7 +28122,7 @@
         <v>1638</v>
       </c>
       <c r="I560" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J560" t="s">
         <v>2354</v>
@@ -28157,7 +28157,7 @@
         <v>1638</v>
       </c>
       <c r="I561" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J561" t="s">
         <v>2355</v>
@@ -28192,7 +28192,7 @@
         <v>1638</v>
       </c>
       <c r="I562" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J562" t="s">
         <v>2356</v>
@@ -28262,7 +28262,7 @@
         <v>1638</v>
       </c>
       <c r="I564" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J564" t="s">
         <v>2358</v>
@@ -28297,7 +28297,7 @@
         <v>1638</v>
       </c>
       <c r="I565" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J565" t="s">
         <v>2359</v>
@@ -28332,7 +28332,7 @@
         <v>1638</v>
       </c>
       <c r="I566" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J566" t="s">
         <v>2360</v>
@@ -28367,7 +28367,7 @@
         <v>1638</v>
       </c>
       <c r="I567" t="s">
-        <v>1794</v>
+        <v>1795</v>
       </c>
       <c r="J567" t="s">
         <v>2361</v>
@@ -28402,7 +28402,7 @@
         <v>1638</v>
       </c>
       <c r="I568" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J568" t="s">
         <v>2362</v>
@@ -28437,7 +28437,7 @@
         <v>1638</v>
       </c>
       <c r="I569" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="J569" t="s">
         <v>2363</v>
@@ -28472,7 +28472,7 @@
         <v>1638</v>
       </c>
       <c r="I570" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J570" t="s">
         <v>2364</v>
@@ -28507,7 +28507,7 @@
         <v>1638</v>
       </c>
       <c r="I571" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J571" t="s">
         <v>2365</v>
@@ -28542,7 +28542,7 @@
         <v>1638</v>
       </c>
       <c r="I572" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J572" t="s">
         <v>2366</v>
@@ -28577,7 +28577,7 @@
         <v>1638</v>
       </c>
       <c r="I573" t="s">
-        <v>1795</v>
+        <v>1796</v>
       </c>
       <c r="J573" t="s">
         <v>2367</v>
@@ -28612,7 +28612,7 @@
         <v>1638</v>
       </c>
       <c r="I574" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J574" t="s">
         <v>2368</v>
@@ -28647,7 +28647,7 @@
         <v>1638</v>
       </c>
       <c r="I575" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J575" t="s">
         <v>2369</v>
@@ -28685,7 +28685,7 @@
         <v>1656</v>
       </c>
       <c r="I576" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J576" t="s">
         <v>2370</v>
@@ -28755,7 +28755,7 @@
         <v>1638</v>
       </c>
       <c r="I578" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J578" t="s">
         <v>2372</v>
@@ -28825,7 +28825,7 @@
         <v>1638</v>
       </c>
       <c r="I580" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J580" t="s">
         <v>2374</v>
@@ -28860,7 +28860,7 @@
         <v>1638</v>
       </c>
       <c r="I581" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J581" t="s">
         <v>2375</v>
@@ -28898,7 +28898,7 @@
         <v>1657</v>
       </c>
       <c r="I582" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J582" t="s">
         <v>2376</v>
@@ -28933,7 +28933,7 @@
         <v>1638</v>
       </c>
       <c r="I583" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J583" t="s">
         <v>2377</v>
@@ -28968,7 +28968,7 @@
         <v>1638</v>
       </c>
       <c r="I584" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J584" t="s">
         <v>2378</v>
@@ -29003,7 +29003,7 @@
         <v>1638</v>
       </c>
       <c r="I585" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J585" t="s">
         <v>2379</v>
@@ -29038,7 +29038,7 @@
         <v>1638</v>
       </c>
       <c r="I586" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J586" t="s">
         <v>2380</v>
@@ -29073,7 +29073,7 @@
         <v>1638</v>
       </c>
       <c r="I587" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J587" t="s">
         <v>2381</v>
@@ -29108,7 +29108,7 @@
         <v>1638</v>
       </c>
       <c r="I588" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J588" t="s">
         <v>2382</v>
@@ -29143,7 +29143,7 @@
         <v>1638</v>
       </c>
       <c r="I589" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J589" t="s">
         <v>2383</v>
@@ -29178,7 +29178,7 @@
         <v>1638</v>
       </c>
       <c r="I590" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J590" t="s">
         <v>2384</v>
@@ -29213,7 +29213,7 @@
         <v>1638</v>
       </c>
       <c r="I591" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J591" t="s">
         <v>2385</v>
@@ -29248,7 +29248,7 @@
         <v>1638</v>
       </c>
       <c r="I592" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J592" t="s">
         <v>2386</v>
@@ -29283,7 +29283,7 @@
         <v>1638</v>
       </c>
       <c r="I593" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J593" t="s">
         <v>2387</v>
@@ -29318,7 +29318,7 @@
         <v>1638</v>
       </c>
       <c r="I594" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J594" t="s">
         <v>2388</v>
@@ -29391,7 +29391,7 @@
         <v>1638</v>
       </c>
       <c r="I596" t="s">
-        <v>1796</v>
+        <v>1797</v>
       </c>
       <c r="J596" t="s">
         <v>2390</v>
@@ -29426,7 +29426,7 @@
         <v>1638</v>
       </c>
       <c r="I597" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J597" t="s">
         <v>2391</v>
@@ -29461,7 +29461,7 @@
         <v>1638</v>
       </c>
       <c r="I598" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J598" t="s">
         <v>2392</v>
@@ -29496,7 +29496,7 @@
         <v>1638</v>
       </c>
       <c r="I599" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J599" t="s">
         <v>2393</v>
@@ -29531,7 +29531,7 @@
         <v>1638</v>
       </c>
       <c r="I600" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J600" t="s">
         <v>2394</v>
@@ -29566,7 +29566,7 @@
         <v>1638</v>
       </c>
       <c r="I601" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J601" t="s">
         <v>2395</v>
@@ -29601,7 +29601,7 @@
         <v>1638</v>
       </c>
       <c r="I602" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J602" t="s">
         <v>2396</v>
@@ -29636,7 +29636,7 @@
         <v>1638</v>
       </c>
       <c r="I603" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J603" t="s">
         <v>2397</v>
@@ -29671,7 +29671,7 @@
         <v>1638</v>
       </c>
       <c r="I604" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J604" t="s">
         <v>2398</v>
@@ -29706,7 +29706,7 @@
         <v>1638</v>
       </c>
       <c r="I605" t="s">
-        <v>1797</v>
+        <v>1798</v>
       </c>
       <c r="J605" t="s">
         <v>2399</v>
@@ -29741,7 +29741,7 @@
         <v>1638</v>
       </c>
       <c r="I606" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J606" t="s">
         <v>2400</v>
@@ -29849,7 +29849,7 @@
         <v>1638</v>
       </c>
       <c r="I609" t="s">
-        <v>1798</v>
+        <v>1799</v>
       </c>
       <c r="J609" t="s">
         <v>2403</v>
@@ -29884,7 +29884,7 @@
         <v>1638</v>
       </c>
       <c r="I610" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J610" t="s">
         <v>2404</v>
@@ -29919,7 +29919,7 @@
         <v>1638</v>
       </c>
       <c r="I611" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J611" t="s">
         <v>2405</v>
@@ -30027,7 +30027,7 @@
         <v>1658</v>
       </c>
       <c r="I614" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J614" t="s">
         <v>2408</v>
@@ -30062,7 +30062,7 @@
         <v>1638</v>
       </c>
       <c r="I615" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J615" t="s">
         <v>2409</v>
@@ -30097,7 +30097,7 @@
         <v>1638</v>
       </c>
       <c r="I616" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J616" t="s">
         <v>2410</v>
@@ -30132,7 +30132,7 @@
         <v>1638</v>
       </c>
       <c r="I617" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J617" t="s">
         <v>2411</v>
@@ -30170,7 +30170,7 @@
         <v>1659</v>
       </c>
       <c r="I618" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J618" t="s">
         <v>2412</v>
@@ -30205,7 +30205,7 @@
         <v>1638</v>
       </c>
       <c r="I619" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J619" t="s">
         <v>2413</v>
@@ -30240,7 +30240,7 @@
         <v>1638</v>
       </c>
       <c r="I620" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J620" t="s">
         <v>2414</v>
@@ -30275,7 +30275,7 @@
         <v>1638</v>
       </c>
       <c r="I621" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J621" t="s">
         <v>2415</v>
@@ -30310,7 +30310,7 @@
         <v>1638</v>
       </c>
       <c r="I622" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J622" t="s">
         <v>2416</v>
@@ -30383,7 +30383,7 @@
         <v>1638</v>
       </c>
       <c r="I624" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J624" t="s">
         <v>2418</v>
@@ -30453,7 +30453,7 @@
         <v>1638</v>
       </c>
       <c r="I626" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J626" t="s">
         <v>2420</v>
@@ -30491,7 +30491,7 @@
         <v>1661</v>
       </c>
       <c r="I627" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="J627" t="s">
         <v>2421</v>
@@ -30526,7 +30526,7 @@
         <v>1638</v>
       </c>
       <c r="I628" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J628" t="s">
         <v>2422</v>
@@ -30561,7 +30561,7 @@
         <v>1638</v>
       </c>
       <c r="I629" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J629" t="s">
         <v>2423</v>
@@ -30599,7 +30599,7 @@
         <v>1662</v>
       </c>
       <c r="I630" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J630" t="s">
         <v>2424</v>
@@ -30634,7 +30634,7 @@
         <v>1638</v>
       </c>
       <c r="I631" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J631" t="s">
         <v>2425</v>
@@ -30669,7 +30669,7 @@
         <v>1638</v>
       </c>
       <c r="I632" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J632" t="s">
         <v>2426</v>
@@ -30704,7 +30704,7 @@
         <v>1638</v>
       </c>
       <c r="I633" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J633" t="s">
         <v>2427</v>
@@ -30742,7 +30742,7 @@
         <v>1661</v>
       </c>
       <c r="I634" t="s">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="J634" t="s">
         <v>2428</v>
@@ -30777,7 +30777,7 @@
         <v>1638</v>
       </c>
       <c r="I635" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J635" t="s">
         <v>2429</v>
@@ -30815,7 +30815,7 @@
         <v>1663</v>
       </c>
       <c r="I636" t="s">
-        <v>1802</v>
+        <v>1803</v>
       </c>
       <c r="J636" t="s">
         <v>2430</v>
@@ -30885,7 +30885,7 @@
         <v>1638</v>
       </c>
       <c r="I638" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J638" t="s">
         <v>2432</v>
@@ -30920,7 +30920,7 @@
         <v>1638</v>
       </c>
       <c r="I639" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J639" t="s">
         <v>2433</v>
@@ -30958,7 +30958,7 @@
         <v>1658</v>
       </c>
       <c r="I640" t="s">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="J640" t="s">
         <v>2434</v>
@@ -30993,7 +30993,7 @@
         <v>1638</v>
       </c>
       <c r="I641" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="J641" t="s">
         <v>2435</v>
@@ -31069,7 +31069,7 @@
         <v>1664</v>
       </c>
       <c r="I643" t="s">
-        <v>1803</v>
+        <v>1804</v>
       </c>
       <c r="J643" t="s">
         <v>2437</v>
@@ -31107,7 +31107,7 @@
         <v>1648</v>
       </c>
       <c r="I644" t="s">
-        <v>1804</v>
+        <v>1805</v>
       </c>
       <c r="J644" t="s">
         <v>2438</v>
@@ -31145,7 +31145,7 @@
         <v>1665</v>
       </c>
       <c r="I645" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="J645" t="s">
         <v>2439</v>
@@ -31180,7 +31180,7 @@
         <v>1638</v>
       </c>
       <c r="I646" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J646" t="s">
         <v>2440</v>
@@ -31215,7 +31215,7 @@
         <v>1638</v>
       </c>
       <c r="I647" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J647" t="s">
         <v>2441</v>
@@ -31250,7 +31250,7 @@
         <v>1638</v>
       </c>
       <c r="I648" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J648" t="s">
         <v>2442</v>
@@ -31288,7 +31288,7 @@
         <v>1658</v>
       </c>
       <c r="I649" t="s">
-        <v>1806</v>
+        <v>1807</v>
       </c>
       <c r="J649" t="s">
         <v>2443</v>
@@ -31428,7 +31428,7 @@
         <v>1638</v>
       </c>
       <c r="I653" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J653" t="s">
         <v>2447</v>
@@ -31463,7 +31463,7 @@
         <v>1638</v>
       </c>
       <c r="I654" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J654" t="s">
         <v>2448</v>
@@ -31498,7 +31498,7 @@
         <v>1638</v>
       </c>
       <c r="I655" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J655" t="s">
         <v>2449</v>
@@ -31533,7 +31533,7 @@
         <v>1638</v>
       </c>
       <c r="I656" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J656" t="s">
         <v>2450</v>
@@ -31568,7 +31568,7 @@
         <v>1638</v>
       </c>
       <c r="I657" t="s">
-        <v>1807</v>
+        <v>1808</v>
       </c>
       <c r="J657" t="s">
         <v>2451</v>
@@ -31603,7 +31603,7 @@
         <v>1638</v>
       </c>
       <c r="I658" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J658" t="s">
         <v>2452</v>
@@ -31638,7 +31638,7 @@
         <v>1638</v>
       </c>
       <c r="I659" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J659" t="s">
         <v>2453</v>
@@ -31673,7 +31673,7 @@
         <v>1638</v>
       </c>
       <c r="I660" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J660" t="s">
         <v>2454</v>
@@ -31708,7 +31708,7 @@
         <v>1638</v>
       </c>
       <c r="I661" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J661" t="s">
         <v>2455</v>
@@ -31743,7 +31743,7 @@
         <v>1638</v>
       </c>
       <c r="I662" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J662" t="s">
         <v>2456</v>
@@ -31781,7 +31781,7 @@
         <v>1666</v>
       </c>
       <c r="I663" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J663" t="s">
         <v>2457</v>
@@ -31851,7 +31851,7 @@
         <v>1638</v>
       </c>
       <c r="I665" t="s">
-        <v>1808</v>
+        <v>1696</v>
       </c>
       <c r="J665" t="s">
         <v>2459</v>
@@ -31886,7 +31886,7 @@
         <v>1638</v>
       </c>
       <c r="I666" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="J666" t="s">
         <v>2460</v>
@@ -31997,7 +31997,7 @@
         <v>1638</v>
       </c>
       <c r="I669" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J669" t="s">
         <v>2463</v>
@@ -32108,7 +32108,7 @@
         <v>1638</v>
       </c>
       <c r="I672" t="s">
-        <v>1808</v>
+        <v>1696</v>
       </c>
       <c r="J672" t="s">
         <v>2466</v>
@@ -32146,7 +32146,7 @@
         <v>1669</v>
       </c>
       <c r="I673" t="s">
-        <v>1678</v>
+        <v>1696</v>
       </c>
       <c r="J673" t="s">
         <v>2467</v>
@@ -32160,7 +32160,7 @@
     </row>
     <row r="674" spans="1:12">
       <c r="A674" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B674" t="s">
         <v>714</v>
@@ -32184,7 +32184,7 @@
         <v>1670</v>
       </c>
       <c r="I674" t="s">
-        <v>1678</v>
+        <v>1714</v>
       </c>
       <c r="J674" t="s">
         <v>2468</v>
@@ -32198,7 +32198,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B675" t="s">
         <v>715</v>
@@ -32219,7 +32219,7 @@
         <v>1638</v>
       </c>
       <c r="I675" t="s">
-        <v>1678</v>
+        <v>1783</v>
       </c>
       <c r="J675" t="s">
         <v>2469</v>
@@ -32233,7 +32233,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B676" t="s">
         <v>716</v>
@@ -32254,7 +32254,7 @@
         <v>1638</v>
       </c>
       <c r="I676" t="s">
-        <v>1678</v>
+        <v>1742</v>
       </c>
       <c r="J676" t="s">
         <v>2470</v>
@@ -32292,7 +32292,7 @@
         <v>1631</v>
       </c>
       <c r="I677" t="s">
-        <v>1678</v>
+        <v>1734</v>
       </c>
       <c r="J677" t="s">
         <v>2471</v>
@@ -32327,7 +32327,7 @@
         <v>1638</v>
       </c>
       <c r="I678" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J678" t="s">
         <v>2472</v>
@@ -32362,7 +32362,7 @@
         <v>1638</v>
       </c>
       <c r="I679" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J679" t="s">
         <v>2473</v>
@@ -32397,7 +32397,7 @@
         <v>1638</v>
       </c>
       <c r="I680" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J680" t="s">
         <v>2474</v>
@@ -32432,7 +32432,7 @@
         <v>1638</v>
       </c>
       <c r="I681" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J681" t="s">
         <v>2475</v>
@@ -32467,7 +32467,7 @@
         <v>1638</v>
       </c>
       <c r="I682" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J682" t="s">
         <v>2476</v>
@@ -32499,7 +32499,7 @@
         <v>1638</v>
       </c>
       <c r="I683" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J683" t="s">
         <v>2477</v>
@@ -32531,7 +32531,7 @@
         <v>1638</v>
       </c>
       <c r="I684" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J684" t="s">
         <v>2478</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-29 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -32368,7 +32368,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B679" t="s">
         <v>720</v>
@@ -32389,7 +32389,7 @@
         <v>1643</v>
       </c>
       <c r="I679" t="s">
-        <v>1683</v>
+        <v>1718</v>
       </c>
       <c r="J679" t="s">
         <v>2480</v>
@@ -32535,7 +32535,7 @@
         <v>1643</v>
       </c>
       <c r="I683" t="s">
-        <v>1683</v>
+        <v>1814</v>
       </c>
       <c r="J683" t="s">
         <v>2484</v>
@@ -32570,7 +32570,7 @@
         <v>1643</v>
       </c>
       <c r="I684" t="s">
-        <v>1683</v>
+        <v>1814</v>
       </c>
       <c r="J684" t="s">
         <v>2485</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-29 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -100,12 +100,12 @@
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
   </si>
   <si>
@@ -5212,69 +5212,69 @@
     <t>EDUARDO COUTO SOLEDADE</t>
   </si>
   <si>
+    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
     <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
   </si>
   <si>
-    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER</t>
   </si>
   <si>
@@ -5365,49 +5365,49 @@
     <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA, PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES, HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>PAULA DE ARAUJO CRUZ VIGIO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
+    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
     <t>DAGER SALLES AMARAL</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA, PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES, HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>PAULA DE ARAUJO CRUZ VIGIO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
-    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
   </si>
   <si>
     <t>GLAUCO CASTILHO DE ALMEIDA</t>
@@ -12014,7 +12014,7 @@
     </row>
     <row r="99" spans="1:12">
       <c r="A99" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B99" t="s">
         <v>139</v>
@@ -12035,7 +12035,7 @@
         <v>1656</v>
       </c>
       <c r="I99" t="s">
-        <v>1732</v>
+        <v>1695</v>
       </c>
       <c r="J99" t="s">
         <v>1922</v>
@@ -12070,7 +12070,7 @@
         <v>1654</v>
       </c>
       <c r="I100" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J100" t="s">
         <v>1923</v>
@@ -12420,7 +12420,7 @@
         <v>1654</v>
       </c>
       <c r="I110" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J110" t="s">
         <v>1933</v>
@@ -12525,7 +12525,7 @@
         <v>1654</v>
       </c>
       <c r="I113" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J113" t="s">
         <v>1936</v>
@@ -12560,7 +12560,7 @@
         <v>1654</v>
       </c>
       <c r="I114" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J114" t="s">
         <v>1937</v>
@@ -12770,7 +12770,7 @@
         <v>1654</v>
       </c>
       <c r="I120" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="J120" t="s">
         <v>1943</v>
@@ -12840,7 +12840,7 @@
         <v>1654</v>
       </c>
       <c r="I122" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J122" t="s">
         <v>1945</v>
@@ -12945,7 +12945,7 @@
         <v>1654</v>
       </c>
       <c r="I125" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J125" t="s">
         <v>1948</v>
@@ -13015,7 +13015,7 @@
         <v>1654</v>
       </c>
       <c r="I127" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
       <c r="J127" t="s">
         <v>1950</v>
@@ -13085,7 +13085,7 @@
         <v>1654</v>
       </c>
       <c r="I129" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="J129" t="s">
         <v>1952</v>
@@ -13155,7 +13155,7 @@
         <v>1654</v>
       </c>
       <c r="I131" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J131" t="s">
         <v>1954</v>
@@ -13298,7 +13298,7 @@
         <v>1654</v>
       </c>
       <c r="I135" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J135" t="s">
         <v>1958</v>
@@ -13368,7 +13368,7 @@
         <v>1654</v>
       </c>
       <c r="I137" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J137" t="s">
         <v>1959</v>
@@ -13473,7 +13473,7 @@
         <v>1654</v>
       </c>
       <c r="I140" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="J140" t="s">
         <v>1962</v>
@@ -13514,7 +13514,7 @@
         <v>1835</v>
       </c>
       <c r="K141" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L141" t="s">
         <v>2659</v>
@@ -13648,7 +13648,7 @@
         <v>1654</v>
       </c>
       <c r="I145" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="J145" t="s">
         <v>1966</v>
@@ -13826,7 +13826,7 @@
         <v>1654</v>
       </c>
       <c r="I150" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="J150" t="s">
         <v>1970</v>
@@ -13861,7 +13861,7 @@
         <v>1654</v>
       </c>
       <c r="I151" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J151" t="s">
         <v>1971</v>
@@ -13896,7 +13896,7 @@
         <v>1654</v>
       </c>
       <c r="I152" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J152" t="s">
         <v>1972</v>
@@ -13910,7 +13910,7 @@
     </row>
     <row r="153" spans="1:12">
       <c r="A153" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B153" t="s">
         <v>193</v>
@@ -13945,7 +13945,7 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B154" t="s">
         <v>194</v>
@@ -13966,7 +13966,7 @@
         <v>1654</v>
       </c>
       <c r="I154" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J154" t="s">
         <v>1974</v>
@@ -14001,7 +14001,7 @@
         <v>1654</v>
       </c>
       <c r="I155" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="J155" t="s">
         <v>1975</v>
@@ -14071,7 +14071,7 @@
         <v>1654</v>
       </c>
       <c r="I157" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J157" t="s">
         <v>1977</v>
@@ -14211,7 +14211,7 @@
         <v>1654</v>
       </c>
       <c r="I161" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J161" t="s">
         <v>1981</v>
@@ -14281,7 +14281,7 @@
         <v>1654</v>
       </c>
       <c r="I163" t="s">
-        <v>1732</v>
+        <v>1752</v>
       </c>
       <c r="J163" t="s">
         <v>1983</v>
@@ -14645,7 +14645,7 @@
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B174" t="s">
         <v>214</v>
@@ -15964,7 +15964,7 @@
         <v>1654</v>
       </c>
       <c r="I211" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J211" t="s">
         <v>2029</v>
@@ -16349,7 +16349,7 @@
         <v>1654</v>
       </c>
       <c r="I222" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J222" t="s">
         <v>2040</v>
@@ -16629,7 +16629,7 @@
         <v>1654</v>
       </c>
       <c r="I230" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J230" t="s">
         <v>2048</v>
@@ -17906,7 +17906,7 @@
     </row>
     <row r="267" spans="1:12">
       <c r="A267" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B267" t="s">
         <v>307</v>
@@ -18105,7 +18105,7 @@
         <v>1654</v>
       </c>
       <c r="I272" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J272" t="s">
         <v>2089</v>
@@ -18154,7 +18154,7 @@
     </row>
     <row r="274" spans="1:12">
       <c r="A274" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B274" t="s">
         <v>314</v>
@@ -18315,7 +18315,7 @@
         <v>1654</v>
       </c>
       <c r="I278" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="J278" t="s">
         <v>2095</v>
@@ -18469,7 +18469,7 @@
     </row>
     <row r="283" spans="1:12">
       <c r="A283" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B283" t="s">
         <v>323</v>
@@ -18490,7 +18490,7 @@
         <v>1654</v>
       </c>
       <c r="I283" t="s">
-        <v>1783</v>
+        <v>1695</v>
       </c>
       <c r="J283" t="s">
         <v>2099</v>
@@ -18525,7 +18525,7 @@
         <v>1654</v>
       </c>
       <c r="I284" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J284" t="s">
         <v>2100</v>
@@ -18668,7 +18668,7 @@
         <v>1664</v>
       </c>
       <c r="I288" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J288" t="s">
         <v>2104</v>
@@ -18808,7 +18808,7 @@
         <v>1654</v>
       </c>
       <c r="I292" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J292" t="s">
         <v>2107</v>
@@ -18843,7 +18843,7 @@
         <v>1654</v>
       </c>
       <c r="I293" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J293" t="s">
         <v>2108</v>
@@ -19441,7 +19441,7 @@
         <v>1654</v>
       </c>
       <c r="I310" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
       <c r="J310" t="s">
         <v>2125</v>
@@ -19665,7 +19665,7 @@
     </row>
     <row r="317" spans="1:12">
       <c r="A317" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B317" t="s">
         <v>357</v>
@@ -19721,7 +19721,7 @@
         <v>1654</v>
       </c>
       <c r="I318" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
       <c r="J318" t="s">
         <v>2133</v>
@@ -19826,7 +19826,7 @@
         <v>1654</v>
       </c>
       <c r="I321" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J321" t="s">
         <v>2136</v>
@@ -19896,7 +19896,7 @@
         <v>1654</v>
       </c>
       <c r="I323" t="s">
-        <v>1787</v>
+        <v>1786</v>
       </c>
       <c r="J323" t="s">
         <v>2138</v>
@@ -19931,7 +19931,7 @@
         <v>1654</v>
       </c>
       <c r="I324" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="J324" t="s">
         <v>2139</v>
@@ -20106,7 +20106,7 @@
         <v>1654</v>
       </c>
       <c r="I329" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J329" t="s">
         <v>2144</v>
@@ -20295,7 +20295,7 @@
     </row>
     <row r="335" spans="1:12">
       <c r="A335" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B335" t="s">
         <v>375</v>
@@ -20316,7 +20316,7 @@
         <v>1654</v>
       </c>
       <c r="I335" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J335" t="s">
         <v>2150</v>
@@ -20351,7 +20351,7 @@
         <v>1654</v>
       </c>
       <c r="I336" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="J336" t="s">
         <v>2151</v>
@@ -20386,7 +20386,7 @@
         <v>1654</v>
       </c>
       <c r="I337" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J337" t="s">
         <v>2152</v>
@@ -20491,7 +20491,7 @@
         <v>1654</v>
       </c>
       <c r="I340" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J340" t="s">
         <v>2155</v>
@@ -20526,7 +20526,7 @@
         <v>1654</v>
       </c>
       <c r="I341" t="s">
-        <v>1790</v>
+        <v>1789</v>
       </c>
       <c r="J341" t="s">
         <v>2156</v>
@@ -20809,7 +20809,7 @@
         <v>1654</v>
       </c>
       <c r="I349" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J349" t="s">
         <v>2164</v>
@@ -20844,7 +20844,7 @@
         <v>1654</v>
       </c>
       <c r="I350" t="s">
-        <v>1791</v>
+        <v>1790</v>
       </c>
       <c r="J350" t="s">
         <v>2165</v>
@@ -20914,7 +20914,7 @@
         <v>1654</v>
       </c>
       <c r="I352" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J352" t="s">
         <v>2167</v>
@@ -20963,7 +20963,7 @@
     </row>
     <row r="354" spans="1:12">
       <c r="A354" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B354" t="s">
         <v>394</v>
@@ -21019,7 +21019,7 @@
         <v>1654</v>
       </c>
       <c r="I355" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="J355" t="s">
         <v>2170</v>
@@ -21124,7 +21124,7 @@
         <v>1654</v>
       </c>
       <c r="I358" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="J358" t="s">
         <v>2173</v>
@@ -21232,7 +21232,7 @@
         <v>1603</v>
       </c>
       <c r="I361" t="s">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="J361" t="s">
         <v>2176</v>
@@ -21337,7 +21337,7 @@
         <v>1654</v>
       </c>
       <c r="I364" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J364" t="s">
         <v>2179</v>
@@ -21372,7 +21372,7 @@
         <v>1654</v>
       </c>
       <c r="I365" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J365" t="s">
         <v>2180</v>
@@ -21442,7 +21442,7 @@
         <v>1654</v>
       </c>
       <c r="I367" t="s">
-        <v>1794</v>
+        <v>1793</v>
       </c>
       <c r="J367" t="s">
         <v>2182</v>
@@ -21582,7 +21582,7 @@
         <v>1654</v>
       </c>
       <c r="I371" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="J371" t="s">
         <v>2186</v>
@@ -21652,7 +21652,7 @@
         <v>1654</v>
       </c>
       <c r="I373" t="s">
-        <v>1796</v>
+        <v>1795</v>
       </c>
       <c r="J373" t="s">
         <v>2188</v>
@@ -21722,7 +21722,7 @@
         <v>1654</v>
       </c>
       <c r="I375" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J375" t="s">
         <v>2190</v>
@@ -21862,7 +21862,7 @@
         <v>1654</v>
       </c>
       <c r="I379" t="s">
-        <v>1783</v>
+        <v>1797</v>
       </c>
       <c r="J379" t="s">
         <v>2194</v>
@@ -21897,7 +21897,7 @@
         <v>1654</v>
       </c>
       <c r="I380" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J380" t="s">
         <v>2195</v>
@@ -22107,7 +22107,7 @@
         <v>1654</v>
       </c>
       <c r="I386" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J386" t="s">
         <v>2201</v>
@@ -22352,7 +22352,7 @@
         <v>1654</v>
       </c>
       <c r="I393" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J393" t="s">
         <v>2208</v>
@@ -22611,7 +22611,7 @@
     </row>
     <row r="401" spans="1:12">
       <c r="A401" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B401" t="s">
         <v>441</v>
@@ -22632,7 +22632,7 @@
         <v>1654</v>
       </c>
       <c r="I401" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J401" t="s">
         <v>2215</v>
@@ -22737,7 +22737,7 @@
         <v>1654</v>
       </c>
       <c r="I404" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J404" t="s">
         <v>2218</v>
@@ -22824,7 +22824,7 @@
     </row>
     <row r="407" spans="1:12">
       <c r="A407" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B407" t="s">
         <v>447</v>
@@ -22964,7 +22964,7 @@
     </row>
     <row r="411" spans="1:12">
       <c r="A411" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B411" t="s">
         <v>451</v>
@@ -23090,7 +23090,7 @@
         <v>1654</v>
       </c>
       <c r="I414" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J414" t="s">
         <v>2227</v>
@@ -23195,7 +23195,7 @@
         <v>1654</v>
       </c>
       <c r="I417" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J417" t="s">
         <v>2230</v>
@@ -23279,7 +23279,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B420" t="s">
         <v>460</v>
@@ -23300,7 +23300,7 @@
         <v>1654</v>
       </c>
       <c r="I420" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J420" t="s">
         <v>2233</v>
@@ -23335,7 +23335,7 @@
         <v>1654</v>
       </c>
       <c r="I421" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J421" t="s">
         <v>2234</v>
@@ -23615,7 +23615,7 @@
         <v>1654</v>
       </c>
       <c r="I429" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J429" t="s">
         <v>2242</v>
@@ -23860,7 +23860,7 @@
         <v>1654</v>
       </c>
       <c r="I436" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J436" t="s">
         <v>2249</v>
@@ -24108,7 +24108,7 @@
         <v>1654</v>
       </c>
       <c r="I443" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J443" t="s">
         <v>2256</v>
@@ -24213,7 +24213,7 @@
         <v>1654</v>
       </c>
       <c r="I446" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J446" t="s">
         <v>2259</v>
@@ -24388,7 +24388,7 @@
         <v>1654</v>
       </c>
       <c r="I451" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J451" t="s">
         <v>2264</v>
@@ -24542,7 +24542,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B456" t="s">
         <v>495</v>
@@ -24633,7 +24633,7 @@
         <v>1654</v>
       </c>
       <c r="I458" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J458" t="s">
         <v>2270</v>
@@ -24787,7 +24787,7 @@
     </row>
     <row r="463" spans="1:12">
       <c r="A463" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B463" t="s">
         <v>502</v>
@@ -25018,7 +25018,7 @@
         <v>1654</v>
       </c>
       <c r="I469" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J469" t="s">
         <v>2281</v>
@@ -25053,7 +25053,7 @@
         <v>1654</v>
       </c>
       <c r="I470" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J470" t="s">
         <v>2282</v>
@@ -25333,7 +25333,7 @@
         <v>1654</v>
       </c>
       <c r="I478" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J478" t="s">
         <v>2290</v>
@@ -25543,7 +25543,7 @@
         <v>1654</v>
       </c>
       <c r="I484" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J484" t="s">
         <v>2296</v>
@@ -25578,7 +25578,7 @@
         <v>1654</v>
       </c>
       <c r="I485" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J485" t="s">
         <v>2297</v>
@@ -25616,7 +25616,7 @@
         <v>1669</v>
       </c>
       <c r="I486" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J486" t="s">
         <v>2298</v>
@@ -25651,7 +25651,7 @@
         <v>1654</v>
       </c>
       <c r="I487" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J487" t="s">
         <v>2299</v>
@@ -25931,7 +25931,7 @@
         <v>1654</v>
       </c>
       <c r="I495" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J495" t="s">
         <v>2307</v>
@@ -26036,7 +26036,7 @@
         <v>1654</v>
       </c>
       <c r="I498" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J498" t="s">
         <v>2310</v>
@@ -26106,7 +26106,7 @@
         <v>1654</v>
       </c>
       <c r="I500" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J500" t="s">
         <v>2312</v>
@@ -26141,7 +26141,7 @@
         <v>1654</v>
       </c>
       <c r="I501" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J501" t="s">
         <v>2313</v>
@@ -26561,7 +26561,7 @@
         <v>1654</v>
       </c>
       <c r="I513" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J513" t="s">
         <v>2325</v>
@@ -26631,7 +26631,7 @@
         <v>1654</v>
       </c>
       <c r="I515" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J515" t="s">
         <v>2327</v>
@@ -26701,7 +26701,7 @@
         <v>1654</v>
       </c>
       <c r="I517" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J517" t="s">
         <v>2329</v>
@@ -26771,7 +26771,7 @@
         <v>1654</v>
       </c>
       <c r="I519" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J519" t="s">
         <v>2331</v>
@@ -27089,7 +27089,7 @@
         <v>1654</v>
       </c>
       <c r="I528" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J528" t="s">
         <v>2340</v>
@@ -27103,7 +27103,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B529" t="s">
         <v>568</v>
@@ -27124,7 +27124,7 @@
         <v>1654</v>
       </c>
       <c r="I529" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J529" t="s">
         <v>2341</v>
@@ -27159,7 +27159,7 @@
         <v>1654</v>
       </c>
       <c r="I530" t="s">
-        <v>1783</v>
+        <v>1797</v>
       </c>
       <c r="J530" t="s">
         <v>2342</v>
@@ -27194,7 +27194,7 @@
         <v>1654</v>
       </c>
       <c r="I531" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J531" t="s">
         <v>2343</v>
@@ -27582,7 +27582,7 @@
         <v>1654</v>
       </c>
       <c r="I542" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J542" t="s">
         <v>2354</v>
@@ -27687,7 +27687,7 @@
         <v>1654</v>
       </c>
       <c r="I545" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J545" t="s">
         <v>2357</v>
@@ -27806,7 +27806,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B549" t="s">
         <v>588</v>
@@ -28002,7 +28002,7 @@
         <v>1654</v>
       </c>
       <c r="I554" t="s">
-        <v>1783</v>
+        <v>1797</v>
       </c>
       <c r="J554" t="s">
         <v>2366</v>
@@ -28037,7 +28037,7 @@
         <v>1654</v>
       </c>
       <c r="I555" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J555" t="s">
         <v>2367</v>
@@ -28072,7 +28072,7 @@
         <v>1654</v>
       </c>
       <c r="I556" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J556" t="s">
         <v>2368</v>
@@ -28212,7 +28212,7 @@
         <v>1654</v>
       </c>
       <c r="I560" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J560" t="s">
         <v>2372</v>
@@ -28282,7 +28282,7 @@
         <v>1654</v>
       </c>
       <c r="I562" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J562" t="s">
         <v>2374</v>
@@ -28352,7 +28352,7 @@
         <v>1654</v>
       </c>
       <c r="I564" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J564" t="s">
         <v>2376</v>
@@ -28387,7 +28387,7 @@
         <v>1654</v>
       </c>
       <c r="I565" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J565" t="s">
         <v>2377</v>
@@ -28422,7 +28422,7 @@
         <v>1654</v>
       </c>
       <c r="I566" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J566" t="s">
         <v>2378</v>
@@ -28565,7 +28565,7 @@
         <v>1672</v>
       </c>
       <c r="I570" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J570" t="s">
         <v>2382</v>
@@ -28635,7 +28635,7 @@
         <v>1654</v>
       </c>
       <c r="I572" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J572" t="s">
         <v>2384</v>
@@ -28705,7 +28705,7 @@
         <v>1654</v>
       </c>
       <c r="I574" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J574" t="s">
         <v>2386</v>
@@ -28740,7 +28740,7 @@
         <v>1654</v>
       </c>
       <c r="I575" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J575" t="s">
         <v>2387</v>
@@ -28848,7 +28848,7 @@
         <v>1654</v>
       </c>
       <c r="I578" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J578" t="s">
         <v>2390</v>
@@ -28918,7 +28918,7 @@
         <v>1654</v>
       </c>
       <c r="I580" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J580" t="s">
         <v>2392</v>
@@ -28953,7 +28953,7 @@
         <v>1654</v>
       </c>
       <c r="I581" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J581" t="s">
         <v>2393</v>
@@ -29128,7 +29128,7 @@
         <v>1654</v>
       </c>
       <c r="I586" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J586" t="s">
         <v>2398</v>
@@ -29163,7 +29163,7 @@
         <v>1654</v>
       </c>
       <c r="I587" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J587" t="s">
         <v>2399</v>
@@ -29198,7 +29198,7 @@
         <v>1654</v>
       </c>
       <c r="I588" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J588" t="s">
         <v>2400</v>
@@ -29236,7 +29236,7 @@
         <v>1645</v>
       </c>
       <c r="I589" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
       <c r="J589" t="s">
         <v>2401</v>
@@ -29341,7 +29341,7 @@
         <v>1654</v>
       </c>
       <c r="I592" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J592" t="s">
         <v>2404</v>
@@ -29446,7 +29446,7 @@
         <v>1654</v>
       </c>
       <c r="I595" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J595" t="s">
         <v>2407</v>
@@ -29764,7 +29764,7 @@
         <v>1654</v>
       </c>
       <c r="I604" t="s">
-        <v>1783</v>
+        <v>1797</v>
       </c>
       <c r="J604" t="s">
         <v>2416</v>
@@ -29799,7 +29799,7 @@
         <v>1654</v>
       </c>
       <c r="I605" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J605" t="s">
         <v>2417</v>
@@ -29907,7 +29907,7 @@
         <v>1674</v>
       </c>
       <c r="I608" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J608" t="s">
         <v>2420</v>
@@ -30085,7 +30085,7 @@
         <v>1654</v>
       </c>
       <c r="I613" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J613" t="s">
         <v>2425</v>
@@ -30190,7 +30190,7 @@
         <v>1654</v>
       </c>
       <c r="I616" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J616" t="s">
         <v>2428</v>
@@ -30263,7 +30263,7 @@
         <v>1654</v>
       </c>
       <c r="I618" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J618" t="s">
         <v>2430</v>
@@ -30333,7 +30333,7 @@
         <v>1654</v>
       </c>
       <c r="I620" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J620" t="s">
         <v>2432</v>
@@ -30511,7 +30511,7 @@
         <v>1654</v>
       </c>
       <c r="I625" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J625" t="s">
         <v>2437</v>
@@ -30546,7 +30546,7 @@
         <v>1654</v>
       </c>
       <c r="I626" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J626" t="s">
         <v>2438</v>
@@ -30619,7 +30619,7 @@
         <v>1654</v>
       </c>
       <c r="I628" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J628" t="s">
         <v>2440</v>
@@ -30727,7 +30727,7 @@
         <v>1654</v>
       </c>
       <c r="I631" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J631" t="s">
         <v>2443</v>
@@ -30741,7 +30741,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B632" t="s">
         <v>671</v>
@@ -30762,7 +30762,7 @@
         <v>1654</v>
       </c>
       <c r="I632" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J632" t="s">
         <v>2444</v>
@@ -31092,7 +31092,7 @@
         <v>1654</v>
       </c>
       <c r="I641" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J641" t="s">
         <v>2453</v>
@@ -31305,7 +31305,7 @@
         <v>1654</v>
       </c>
       <c r="I647" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J647" t="s">
         <v>2459</v>
@@ -31319,7 +31319,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B648" t="s">
         <v>687</v>
@@ -31375,7 +31375,7 @@
         <v>1654</v>
       </c>
       <c r="I649" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J649" t="s">
         <v>2461</v>
@@ -31424,7 +31424,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B651" t="s">
         <v>690</v>
@@ -31459,7 +31459,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B652" t="s">
         <v>691</v>
@@ -31550,7 +31550,7 @@
         <v>1654</v>
       </c>
       <c r="I654" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J654" t="s">
         <v>2466</v>
@@ -31672,7 +31672,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B658" t="s">
         <v>697</v>
@@ -31742,7 +31742,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B660" t="s">
         <v>699</v>
@@ -31818,7 +31818,7 @@
     </row>
     <row r="662" spans="1:12">
       <c r="A662" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B662" t="s">
         <v>701</v>
@@ -31929,7 +31929,7 @@
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B665" t="s">
         <v>704</v>
@@ -31964,7 +31964,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B666" t="s">
         <v>705</v>
@@ -31979,7 +31979,7 @@
         <v>2</v>
       </c>
       <c r="F666" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="G666" t="s">
         <v>1657</v>
@@ -31988,7 +31988,7 @@
         <v>1685</v>
       </c>
       <c r="I666" t="s">
-        <v>1729</v>
+        <v>1695</v>
       </c>
       <c r="J666" t="s">
         <v>2478</v>
@@ -32023,7 +32023,7 @@
         <v>1654</v>
       </c>
       <c r="I667" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J667" t="s">
         <v>2479</v>
@@ -32131,7 +32131,7 @@
         <v>1654</v>
       </c>
       <c r="I670" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J670" t="s">
         <v>2482</v>
@@ -32250,7 +32250,7 @@
     </row>
     <row r="674" spans="1:12">
       <c r="A674" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B674" t="s">
         <v>713</v>
@@ -32271,7 +32271,7 @@
         <v>1654</v>
       </c>
       <c r="I674" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J674" t="s">
         <v>2486</v>
@@ -32431,7 +32431,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B679" t="s">
         <v>718</v>
@@ -32466,7 +32466,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B680" t="s">
         <v>719</v>
@@ -32501,7 +32501,7 @@
     </row>
     <row r="681" spans="1:12">
       <c r="A681" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B681" t="s">
         <v>720</v>
@@ -32557,7 +32557,7 @@
         <v>1654</v>
       </c>
       <c r="I682" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
       <c r="J682" t="s">
         <v>2494</v>
@@ -32606,7 +32606,7 @@
     </row>
     <row r="684" spans="1:12">
       <c r="A684" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B684" t="s">
         <v>723</v>
@@ -32627,7 +32627,7 @@
         <v>1654</v>
       </c>
       <c r="I684" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J684" t="s">
         <v>2496</v>
@@ -32679,7 +32679,7 @@
     </row>
     <row r="686" spans="1:12">
       <c r="A686" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B686" t="s">
         <v>725</v>
@@ -32717,7 +32717,7 @@
     </row>
     <row r="687" spans="1:12">
       <c r="A687" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B687" t="s">
         <v>726</v>
@@ -32755,7 +32755,7 @@
     </row>
     <row r="688" spans="1:12">
       <c r="A688" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B688" t="s">
         <v>727</v>
@@ -32770,7 +32770,7 @@
         <v>0</v>
       </c>
       <c r="F688" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="G688" t="s">
         <v>1657</v>
@@ -32779,7 +32779,7 @@
         <v>1688</v>
       </c>
       <c r="I688" t="s">
-        <v>1780</v>
+        <v>1690</v>
       </c>
       <c r="J688" t="s">
         <v>2500</v>
@@ -32793,7 +32793,7 @@
     </row>
     <row r="689" spans="1:12">
       <c r="A689" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B689" t="s">
         <v>728</v>
@@ -32808,7 +32808,7 @@
         <v>0</v>
       </c>
       <c r="F689" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="G689" t="s">
         <v>1657</v>
@@ -32817,7 +32817,7 @@
         <v>1688</v>
       </c>
       <c r="I689" t="s">
-        <v>1780</v>
+        <v>1692</v>
       </c>
       <c r="J689" t="s">
         <v>2501</v>
@@ -32866,7 +32866,7 @@
     </row>
     <row r="691" spans="1:12">
       <c r="A691" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B691" t="s">
         <v>730</v>
@@ -32919,7 +32919,7 @@
         <v>1654</v>
       </c>
       <c r="I692" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J692" t="s">
         <v>2503</v>
@@ -32933,7 +32933,7 @@
     </row>
     <row r="693" spans="1:12">
       <c r="A693" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B693" t="s">
         <v>732</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-01 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5143,6 +5143,9 @@
     <t>MARCELO TEIXEIRA SANTANA,VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>RODRIGO VENTURA MARRA</t>
   </si>
   <si>
@@ -5158,6 +5161,9 @@
     <t>PEDRO MARCELO ROCHA GOMES</t>
   </si>
   <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
     <t>CELSO BARBOSA MONTENEGRO</t>
   </si>
   <si>
@@ -5269,9 +5275,6 @@
     <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
     <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
   </si>
   <si>
@@ -5498,9 +5501,6 @@
   </si>
   <si>
     <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>PATRICIA FONTES ESTEVES</t>
@@ -9576,7 +9576,7 @@
         <v>1657</v>
       </c>
       <c r="I29" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J29" t="s">
         <v>1857</v>
@@ -9611,7 +9611,7 @@
         <v>1657</v>
       </c>
       <c r="I30" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J30" t="s">
         <v>1858</v>
@@ -9681,7 +9681,7 @@
         <v>1657</v>
       </c>
       <c r="I32" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J32" t="s">
         <v>1860</v>
@@ -9891,7 +9891,7 @@
         <v>1657</v>
       </c>
       <c r="I38" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J38" t="s">
         <v>1866</v>
@@ -9999,7 +9999,7 @@
         <v>1661</v>
       </c>
       <c r="I41" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J41" t="s">
         <v>1869</v>
@@ -10142,7 +10142,7 @@
         <v>1662</v>
       </c>
       <c r="I45" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J45" t="s">
         <v>1873</v>
@@ -10387,7 +10387,7 @@
         <v>1657</v>
       </c>
       <c r="I52" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J52" t="s">
         <v>1880</v>
@@ -10436,7 +10436,7 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B54" t="s">
         <v>94</v>
@@ -10457,7 +10457,7 @@
         <v>1657</v>
       </c>
       <c r="I54" t="s">
-        <v>1707</v>
+        <v>1715</v>
       </c>
       <c r="J54" t="s">
         <v>1882</v>
@@ -10492,7 +10492,7 @@
         <v>1657</v>
       </c>
       <c r="I55" t="s">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="J55" t="s">
         <v>1883</v>
@@ -10527,7 +10527,7 @@
         <v>1657</v>
       </c>
       <c r="I56" t="s">
-        <v>1715</v>
+        <v>1717</v>
       </c>
       <c r="J56" t="s">
         <v>1884</v>
@@ -10597,7 +10597,7 @@
         <v>1657</v>
       </c>
       <c r="I58" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="J58" t="s">
         <v>1886</v>
@@ -10667,7 +10667,7 @@
         <v>1657</v>
       </c>
       <c r="I60" t="s">
-        <v>1717</v>
+        <v>1719</v>
       </c>
       <c r="J60" t="s">
         <v>1888</v>
@@ -10702,7 +10702,7 @@
         <v>1657</v>
       </c>
       <c r="I61" t="s">
-        <v>1718</v>
+        <v>1720</v>
       </c>
       <c r="J61" t="s">
         <v>1889</v>
@@ -10740,7 +10740,7 @@
         <v>1485</v>
       </c>
       <c r="I62" t="s">
-        <v>1719</v>
+        <v>1721</v>
       </c>
       <c r="J62" t="s">
         <v>1890</v>
@@ -10810,7 +10810,7 @@
         <v>1657</v>
       </c>
       <c r="I64" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="J64" t="s">
         <v>1892</v>
@@ -10845,7 +10845,7 @@
         <v>1657</v>
       </c>
       <c r="I65" t="s">
-        <v>1721</v>
+        <v>1723</v>
       </c>
       <c r="J65" t="s">
         <v>1893</v>
@@ -10880,7 +10880,7 @@
         <v>1657</v>
       </c>
       <c r="I66" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="J66" t="s">
         <v>1894</v>
@@ -10988,7 +10988,7 @@
         <v>1657</v>
       </c>
       <c r="I69" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J69" t="s">
         <v>1897</v>
@@ -11023,7 +11023,7 @@
         <v>1657</v>
       </c>
       <c r="I70" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="J70" t="s">
         <v>1898</v>
@@ -11058,7 +11058,7 @@
         <v>1657</v>
       </c>
       <c r="I71" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="J71" t="s">
         <v>1899</v>
@@ -11163,7 +11163,7 @@
         <v>1657</v>
       </c>
       <c r="I74" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="J74" t="s">
         <v>1902</v>
@@ -11198,7 +11198,7 @@
         <v>1657</v>
       </c>
       <c r="I75" t="s">
-        <v>1726</v>
+        <v>1728</v>
       </c>
       <c r="J75" t="s">
         <v>1903</v>
@@ -11271,7 +11271,7 @@
         <v>1663</v>
       </c>
       <c r="I77" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="J77" t="s">
         <v>1905</v>
@@ -11341,7 +11341,7 @@
         <v>1657</v>
       </c>
       <c r="I79" t="s">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="J79" t="s">
         <v>1907</v>
@@ -11376,7 +11376,7 @@
         <v>1657</v>
       </c>
       <c r="I80" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="J80" t="s">
         <v>1908</v>
@@ -11481,7 +11481,7 @@
         <v>1657</v>
       </c>
       <c r="I83" t="s">
-        <v>1729</v>
+        <v>1731</v>
       </c>
       <c r="J83" t="s">
         <v>1911</v>
@@ -11516,7 +11516,7 @@
         <v>1657</v>
       </c>
       <c r="I84" t="s">
-        <v>1730</v>
+        <v>1732</v>
       </c>
       <c r="J84" t="s">
         <v>1912</v>
@@ -11551,7 +11551,7 @@
         <v>1657</v>
       </c>
       <c r="I85" t="s">
-        <v>1730</v>
+        <v>1732</v>
       </c>
       <c r="J85" t="s">
         <v>1912</v>
@@ -11621,7 +11621,7 @@
         <v>1657</v>
       </c>
       <c r="I87" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J87" t="s">
         <v>1913</v>
@@ -11656,7 +11656,7 @@
         <v>1657</v>
       </c>
       <c r="I88" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J88" t="s">
         <v>1914</v>
@@ -11691,7 +11691,7 @@
         <v>1657</v>
       </c>
       <c r="I89" t="s">
-        <v>1732</v>
+        <v>1734</v>
       </c>
       <c r="J89" t="s">
         <v>1915</v>
@@ -11729,7 +11729,7 @@
         <v>1664</v>
       </c>
       <c r="I90" t="s">
-        <v>1733</v>
+        <v>1735</v>
       </c>
       <c r="J90" t="s">
         <v>1916</v>
@@ -11767,7 +11767,7 @@
         <v>1664</v>
       </c>
       <c r="I91" t="s">
-        <v>1733</v>
+        <v>1735</v>
       </c>
       <c r="J91" t="s">
         <v>1916</v>
@@ -11837,7 +11837,7 @@
         <v>1657</v>
       </c>
       <c r="I93" t="s">
-        <v>1734</v>
+        <v>1736</v>
       </c>
       <c r="J93" t="s">
         <v>1918</v>
@@ -11872,7 +11872,7 @@
         <v>1657</v>
       </c>
       <c r="I94" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J94" t="s">
         <v>1919</v>
@@ -12047,7 +12047,7 @@
         <v>1659</v>
       </c>
       <c r="I99" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J99" t="s">
         <v>1924</v>
@@ -12082,7 +12082,7 @@
         <v>1657</v>
       </c>
       <c r="I100" t="s">
-        <v>1735</v>
+        <v>1737</v>
       </c>
       <c r="J100" t="s">
         <v>1925</v>
@@ -12117,7 +12117,7 @@
         <v>1657</v>
       </c>
       <c r="I101" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J101" t="s">
         <v>1926</v>
@@ -12152,7 +12152,7 @@
         <v>1657</v>
       </c>
       <c r="I102" t="s">
-        <v>1732</v>
+        <v>1734</v>
       </c>
       <c r="J102" t="s">
         <v>1927</v>
@@ -12432,7 +12432,7 @@
         <v>1657</v>
       </c>
       <c r="I110" t="s">
-        <v>1736</v>
+        <v>1738</v>
       </c>
       <c r="J110" t="s">
         <v>1935</v>
@@ -12502,7 +12502,7 @@
         <v>1657</v>
       </c>
       <c r="I112" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="J112" t="s">
         <v>1937</v>
@@ -12537,7 +12537,7 @@
         <v>1657</v>
       </c>
       <c r="I113" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="J113" t="s">
         <v>1938</v>
@@ -12572,7 +12572,7 @@
         <v>1657</v>
       </c>
       <c r="I114" t="s">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="J114" t="s">
         <v>1939</v>
@@ -12747,7 +12747,7 @@
         <v>1657</v>
       </c>
       <c r="I119" t="s">
-        <v>1719</v>
+        <v>1721</v>
       </c>
       <c r="J119" t="s">
         <v>1944</v>
@@ -12782,7 +12782,7 @@
         <v>1657</v>
       </c>
       <c r="I120" t="s">
-        <v>1739</v>
+        <v>1741</v>
       </c>
       <c r="J120" t="s">
         <v>1945</v>
@@ -12852,7 +12852,7 @@
         <v>1657</v>
       </c>
       <c r="I122" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="J122" t="s">
         <v>1947</v>
@@ -12957,7 +12957,7 @@
         <v>1657</v>
       </c>
       <c r="I125" t="s">
-        <v>1740</v>
+        <v>1742</v>
       </c>
       <c r="J125" t="s">
         <v>1950</v>
@@ -13027,7 +13027,7 @@
         <v>1657</v>
       </c>
       <c r="I127" t="s">
-        <v>1741</v>
+        <v>1743</v>
       </c>
       <c r="J127" t="s">
         <v>1952</v>
@@ -13097,7 +13097,7 @@
         <v>1657</v>
       </c>
       <c r="I129" t="s">
-        <v>1742</v>
+        <v>1744</v>
       </c>
       <c r="J129" t="s">
         <v>1954</v>
@@ -13167,7 +13167,7 @@
         <v>1657</v>
       </c>
       <c r="I131" t="s">
-        <v>1743</v>
+        <v>1745</v>
       </c>
       <c r="J131" t="s">
         <v>1956</v>
@@ -13310,7 +13310,7 @@
         <v>1657</v>
       </c>
       <c r="I135" t="s">
-        <v>1744</v>
+        <v>1746</v>
       </c>
       <c r="J135" t="s">
         <v>1960</v>
@@ -13380,7 +13380,7 @@
         <v>1657</v>
       </c>
       <c r="I137" t="s">
-        <v>1745</v>
+        <v>1747</v>
       </c>
       <c r="J137" t="s">
         <v>1961</v>
@@ -13415,7 +13415,7 @@
         <v>1657</v>
       </c>
       <c r="I138" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="J138" t="s">
         <v>1962</v>
@@ -13485,7 +13485,7 @@
         <v>1657</v>
       </c>
       <c r="I140" t="s">
-        <v>1746</v>
+        <v>1748</v>
       </c>
       <c r="J140" t="s">
         <v>1964</v>
@@ -13660,7 +13660,7 @@
         <v>1657</v>
       </c>
       <c r="I145" t="s">
-        <v>1747</v>
+        <v>1749</v>
       </c>
       <c r="J145" t="s">
         <v>1968</v>
@@ -13695,7 +13695,7 @@
         <v>1657</v>
       </c>
       <c r="I146" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="J146" t="s">
         <v>1969</v>
@@ -13838,7 +13838,7 @@
         <v>1657</v>
       </c>
       <c r="I150" t="s">
-        <v>1748</v>
+        <v>1750</v>
       </c>
       <c r="J150" t="s">
         <v>1972</v>
@@ -13873,7 +13873,7 @@
         <v>1657</v>
       </c>
       <c r="I151" t="s">
-        <v>1749</v>
+        <v>1751</v>
       </c>
       <c r="J151" t="s">
         <v>1973</v>
@@ -13908,7 +13908,7 @@
         <v>1657</v>
       </c>
       <c r="I152" t="s">
-        <v>1750</v>
+        <v>1752</v>
       </c>
       <c r="J152" t="s">
         <v>1974</v>
@@ -13978,7 +13978,7 @@
         <v>1657</v>
       </c>
       <c r="I154" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J154" t="s">
         <v>1976</v>
@@ -14013,7 +14013,7 @@
         <v>1657</v>
       </c>
       <c r="I155" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="J155" t="s">
         <v>1977</v>
@@ -14083,7 +14083,7 @@
         <v>1657</v>
       </c>
       <c r="I157" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J157" t="s">
         <v>1979</v>
@@ -14223,7 +14223,7 @@
         <v>1657</v>
       </c>
       <c r="I161" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J161" t="s">
         <v>1983</v>
@@ -14293,7 +14293,7 @@
         <v>1657</v>
       </c>
       <c r="I163" t="s">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="J163" t="s">
         <v>1985</v>
@@ -14398,7 +14398,7 @@
         <v>1657</v>
       </c>
       <c r="I166" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="J166" t="s">
         <v>1988</v>
@@ -14573,7 +14573,7 @@
         <v>1657</v>
       </c>
       <c r="I171" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="J171" t="s">
         <v>1993</v>
@@ -14608,7 +14608,7 @@
         <v>1657</v>
       </c>
       <c r="I172" t="s">
-        <v>1758</v>
+        <v>1759</v>
       </c>
       <c r="J172" t="s">
         <v>1994</v>
@@ -14678,7 +14678,7 @@
         <v>1657</v>
       </c>
       <c r="I174" t="s">
-        <v>1726</v>
+        <v>1728</v>
       </c>
       <c r="J174" t="s">
         <v>1996</v>
@@ -14748,7 +14748,7 @@
         <v>1657</v>
       </c>
       <c r="I176" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="J176" t="s">
         <v>1998</v>
@@ -14853,7 +14853,7 @@
         <v>1657</v>
       </c>
       <c r="I179" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="J179" t="s">
         <v>2001</v>
@@ -14888,7 +14888,7 @@
         <v>1657</v>
       </c>
       <c r="I180" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J180" t="s">
         <v>2002</v>
@@ -14923,7 +14923,7 @@
         <v>1657</v>
       </c>
       <c r="I181" t="s">
-        <v>1715</v>
+        <v>1717</v>
       </c>
       <c r="J181" t="s">
         <v>2003</v>
@@ -14958,7 +14958,7 @@
         <v>1657</v>
       </c>
       <c r="I182" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J182" t="s">
         <v>2004</v>
@@ -15098,7 +15098,7 @@
         <v>1657</v>
       </c>
       <c r="I186" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J186" t="s">
         <v>2008</v>
@@ -15343,7 +15343,7 @@
         <v>1657</v>
       </c>
       <c r="I193" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J193" t="s">
         <v>2015</v>
@@ -15378,7 +15378,7 @@
         <v>1657</v>
       </c>
       <c r="I194" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J194" t="s">
         <v>1907</v>
@@ -15588,7 +15588,7 @@
         <v>1657</v>
       </c>
       <c r="I200" t="s">
-        <v>1764</v>
+        <v>1765</v>
       </c>
       <c r="J200" t="s">
         <v>2020</v>
@@ -15661,7 +15661,7 @@
         <v>1559</v>
       </c>
       <c r="I202" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J202" t="s">
         <v>2022</v>
@@ -15731,7 +15731,7 @@
         <v>1657</v>
       </c>
       <c r="I204" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="J204" t="s">
         <v>2024</v>
@@ -15941,7 +15941,7 @@
         <v>1657</v>
       </c>
       <c r="I210" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J210" t="s">
         <v>2030</v>
@@ -15976,7 +15976,7 @@
         <v>1657</v>
       </c>
       <c r="I211" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J211" t="s">
         <v>2031</v>
@@ -16011,7 +16011,7 @@
         <v>1659</v>
       </c>
       <c r="I212" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J212" t="s">
         <v>2032</v>
@@ -16046,7 +16046,7 @@
         <v>1657</v>
       </c>
       <c r="I213" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J213" t="s">
         <v>2033</v>
@@ -16081,7 +16081,7 @@
         <v>1657</v>
       </c>
       <c r="I214" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J214" t="s">
         <v>2034</v>
@@ -16116,7 +16116,7 @@
         <v>1657</v>
       </c>
       <c r="I215" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="J215" t="s">
         <v>2035</v>
@@ -16186,7 +16186,7 @@
         <v>1657</v>
       </c>
       <c r="I217" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="J217" t="s">
         <v>2037</v>
@@ -16221,7 +16221,7 @@
         <v>1657</v>
       </c>
       <c r="I218" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="J218" t="s">
         <v>2038</v>
@@ -16291,7 +16291,7 @@
         <v>1657</v>
       </c>
       <c r="I220" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J220" t="s">
         <v>2040</v>
@@ -16361,7 +16361,7 @@
         <v>1657</v>
       </c>
       <c r="I222" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J222" t="s">
         <v>2042</v>
@@ -16396,7 +16396,7 @@
         <v>1657</v>
       </c>
       <c r="I223" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
       <c r="J223" t="s">
         <v>2043</v>
@@ -16431,7 +16431,7 @@
         <v>1657</v>
       </c>
       <c r="I224" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J224" t="s">
         <v>2044</v>
@@ -16571,7 +16571,7 @@
         <v>1657</v>
       </c>
       <c r="I228" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="J228" t="s">
         <v>2048</v>
@@ -16641,7 +16641,7 @@
         <v>1657</v>
       </c>
       <c r="I230" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J230" t="s">
         <v>2050</v>
@@ -16781,7 +16781,7 @@
         <v>1657</v>
       </c>
       <c r="I234" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
       <c r="J234" t="s">
         <v>2054</v>
@@ -16816,7 +16816,7 @@
         <v>1657</v>
       </c>
       <c r="I235" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="J235" t="s">
         <v>1912</v>
@@ -16851,7 +16851,7 @@
         <v>1657</v>
       </c>
       <c r="I236" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J236" t="s">
         <v>2055</v>
@@ -16886,7 +16886,7 @@
         <v>1657</v>
       </c>
       <c r="I237" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J237" t="s">
         <v>2056</v>
@@ -16921,7 +16921,7 @@
         <v>1657</v>
       </c>
       <c r="I238" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
       <c r="J238" t="s">
         <v>2057</v>
@@ -17166,7 +17166,7 @@
         <v>1657</v>
       </c>
       <c r="I245" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="J245" t="s">
         <v>2064</v>
@@ -17201,7 +17201,7 @@
         <v>1657</v>
       </c>
       <c r="I246" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
       <c r="J246" t="s">
         <v>2065</v>
@@ -17236,7 +17236,7 @@
         <v>1657</v>
       </c>
       <c r="I247" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="J247" t="s">
         <v>2066</v>
@@ -17274,7 +17274,7 @@
         <v>1569</v>
       </c>
       <c r="I248" t="s">
-        <v>1778</v>
+        <v>1779</v>
       </c>
       <c r="J248" t="s">
         <v>2067</v>
@@ -17379,7 +17379,7 @@
         <v>1657</v>
       </c>
       <c r="I251" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J251" t="s">
         <v>2070</v>
@@ -17449,7 +17449,7 @@
         <v>1657</v>
       </c>
       <c r="I253" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
       <c r="J253" t="s">
         <v>2072</v>
@@ -17484,7 +17484,7 @@
         <v>1657</v>
       </c>
       <c r="I254" t="s">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="J254" t="s">
         <v>2073</v>
@@ -17554,7 +17554,7 @@
         <v>1657</v>
       </c>
       <c r="I256" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J256" t="s">
         <v>2075</v>
@@ -17694,7 +17694,7 @@
         <v>1657</v>
       </c>
       <c r="I260" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="J260" t="s">
         <v>2079</v>
@@ -17799,7 +17799,7 @@
         <v>1657</v>
       </c>
       <c r="I263" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="J263" t="s">
         <v>2082</v>
@@ -17869,7 +17869,7 @@
         <v>1657</v>
       </c>
       <c r="I265" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J265" t="s">
         <v>2084</v>
@@ -18012,7 +18012,7 @@
         <v>1666</v>
       </c>
       <c r="I269" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J269" t="s">
         <v>2088</v>
@@ -18117,7 +18117,7 @@
         <v>1657</v>
       </c>
       <c r="I272" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J272" t="s">
         <v>2091</v>
@@ -18152,7 +18152,7 @@
         <v>1657</v>
       </c>
       <c r="I273" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J273" t="s">
         <v>2092</v>
@@ -18187,7 +18187,7 @@
         <v>1657</v>
       </c>
       <c r="I274" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J274" t="s">
         <v>2093</v>
@@ -18257,7 +18257,7 @@
         <v>1657</v>
       </c>
       <c r="I276" t="s">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="J276" t="s">
         <v>2095</v>
@@ -18292,7 +18292,7 @@
         <v>1657</v>
       </c>
       <c r="I277" t="s">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="J277" t="s">
         <v>2096</v>
@@ -18327,7 +18327,7 @@
         <v>1657</v>
       </c>
       <c r="I278" t="s">
-        <v>1747</v>
+        <v>1749</v>
       </c>
       <c r="J278" t="s">
         <v>2097</v>
@@ -18362,7 +18362,7 @@
         <v>1657</v>
       </c>
       <c r="I279" t="s">
-        <v>1785</v>
+        <v>1786</v>
       </c>
       <c r="J279" t="s">
         <v>2098</v>
@@ -18432,7 +18432,7 @@
         <v>1657</v>
       </c>
       <c r="I281" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J281" t="s">
         <v>2100</v>
@@ -18502,7 +18502,7 @@
         <v>1657</v>
       </c>
       <c r="I283" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J283" t="s">
         <v>2101</v>
@@ -18537,7 +18537,7 @@
         <v>1657</v>
       </c>
       <c r="I284" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J284" t="s">
         <v>2102</v>
@@ -18607,7 +18607,7 @@
         <v>1657</v>
       </c>
       <c r="I286" t="s">
-        <v>1732</v>
+        <v>1734</v>
       </c>
       <c r="J286" t="s">
         <v>2104</v>
@@ -18680,7 +18680,7 @@
         <v>1667</v>
       </c>
       <c r="I288" t="s">
-        <v>1736</v>
+        <v>1738</v>
       </c>
       <c r="J288" t="s">
         <v>2106</v>
@@ -18820,7 +18820,7 @@
         <v>1657</v>
       </c>
       <c r="I292" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J292" t="s">
         <v>2109</v>
@@ -18855,7 +18855,7 @@
         <v>1657</v>
       </c>
       <c r="I293" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J293" t="s">
         <v>2110</v>
@@ -19100,7 +19100,7 @@
         <v>1657</v>
       </c>
       <c r="I300" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J300" t="s">
         <v>2117</v>
@@ -19205,7 +19205,7 @@
         <v>1657</v>
       </c>
       <c r="I303" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J303" t="s">
         <v>2120</v>
@@ -19240,7 +19240,7 @@
         <v>1657</v>
       </c>
       <c r="I304" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J304" t="s">
         <v>2121</v>
@@ -19453,7 +19453,7 @@
         <v>1657</v>
       </c>
       <c r="I310" t="s">
-        <v>1787</v>
+        <v>1788</v>
       </c>
       <c r="J310" t="s">
         <v>2127</v>
@@ -19488,7 +19488,7 @@
         <v>1657</v>
       </c>
       <c r="I311" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="J311" t="s">
         <v>2128</v>
@@ -19558,7 +19558,7 @@
         <v>1657</v>
       </c>
       <c r="I313" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="J313" t="s">
         <v>2130</v>
@@ -19698,7 +19698,7 @@
         <v>1657</v>
       </c>
       <c r="I317" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J317" t="s">
         <v>2134</v>
@@ -19733,7 +19733,7 @@
         <v>1657</v>
       </c>
       <c r="I318" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="J318" t="s">
         <v>2135</v>
@@ -19803,7 +19803,7 @@
         <v>1657</v>
       </c>
       <c r="I320" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J320" t="s">
         <v>2137</v>
@@ -19838,7 +19838,7 @@
         <v>1657</v>
       </c>
       <c r="I321" t="s">
-        <v>1749</v>
+        <v>1751</v>
       </c>
       <c r="J321" t="s">
         <v>2138</v>
@@ -19908,7 +19908,7 @@
         <v>1657</v>
       </c>
       <c r="I323" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="J323" t="s">
         <v>2140</v>
@@ -19943,7 +19943,7 @@
         <v>1657</v>
       </c>
       <c r="I324" t="s">
-        <v>1790</v>
+        <v>1791</v>
       </c>
       <c r="J324" t="s">
         <v>2141</v>
@@ -19978,7 +19978,7 @@
         <v>1657</v>
       </c>
       <c r="I325" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J325" t="s">
         <v>2142</v>
@@ -20118,7 +20118,7 @@
         <v>1657</v>
       </c>
       <c r="I329" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J329" t="s">
         <v>2146</v>
@@ -20153,7 +20153,7 @@
         <v>1657</v>
       </c>
       <c r="I330" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J330" t="s">
         <v>2147</v>
@@ -20223,7 +20223,7 @@
         <v>1657</v>
       </c>
       <c r="I332" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J332" t="s">
         <v>2149</v>
@@ -20328,7 +20328,7 @@
         <v>1657</v>
       </c>
       <c r="I335" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J335" t="s">
         <v>2152</v>
@@ -20363,7 +20363,7 @@
         <v>1657</v>
       </c>
       <c r="I336" t="s">
-        <v>1791</v>
+        <v>1792</v>
       </c>
       <c r="J336" t="s">
         <v>2153</v>
@@ -20398,7 +20398,7 @@
         <v>1657</v>
       </c>
       <c r="I337" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J337" t="s">
         <v>2154</v>
@@ -20433,7 +20433,7 @@
         <v>1657</v>
       </c>
       <c r="I338" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J338" t="s">
         <v>2155</v>
@@ -20503,7 +20503,7 @@
         <v>1657</v>
       </c>
       <c r="I340" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J340" t="s">
         <v>2157</v>
@@ -20538,7 +20538,7 @@
         <v>1657</v>
       </c>
       <c r="I341" t="s">
-        <v>1792</v>
+        <v>1793</v>
       </c>
       <c r="J341" t="s">
         <v>2158</v>
@@ -20576,7 +20576,7 @@
         <v>1669</v>
       </c>
       <c r="I342" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J342" t="s">
         <v>2159</v>
@@ -20611,7 +20611,7 @@
         <v>1657</v>
       </c>
       <c r="I343" t="s">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="J343" t="s">
         <v>2160</v>
@@ -20681,7 +20681,7 @@
         <v>1657</v>
       </c>
       <c r="I345" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J345" t="s">
         <v>2162</v>
@@ -20821,7 +20821,7 @@
         <v>1657</v>
       </c>
       <c r="I349" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J349" t="s">
         <v>2166</v>
@@ -20856,7 +20856,7 @@
         <v>1657</v>
       </c>
       <c r="I350" t="s">
-        <v>1793</v>
+        <v>1794</v>
       </c>
       <c r="J350" t="s">
         <v>2167</v>
@@ -20926,7 +20926,7 @@
         <v>1657</v>
       </c>
       <c r="I352" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J352" t="s">
         <v>2169</v>
@@ -20996,7 +20996,7 @@
         <v>1657</v>
       </c>
       <c r="I354" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J354" t="s">
         <v>2171</v>
@@ -21031,7 +21031,7 @@
         <v>1657</v>
       </c>
       <c r="I355" t="s">
-        <v>1790</v>
+        <v>1791</v>
       </c>
       <c r="J355" t="s">
         <v>2172</v>
@@ -21136,7 +21136,7 @@
         <v>1657</v>
       </c>
       <c r="I358" t="s">
-        <v>1794</v>
+        <v>1795</v>
       </c>
       <c r="J358" t="s">
         <v>2175</v>
@@ -21171,7 +21171,7 @@
         <v>1657</v>
       </c>
       <c r="I359" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J359" t="s">
         <v>2176</v>
@@ -21244,7 +21244,7 @@
         <v>1605</v>
       </c>
       <c r="I361" t="s">
-        <v>1795</v>
+        <v>1796</v>
       </c>
       <c r="J361" t="s">
         <v>2178</v>
@@ -21279,7 +21279,7 @@
         <v>1657</v>
       </c>
       <c r="I362" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J362" t="s">
         <v>2179</v>
@@ -21349,7 +21349,7 @@
         <v>1657</v>
       </c>
       <c r="I364" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J364" t="s">
         <v>2181</v>
@@ -21384,7 +21384,7 @@
         <v>1657</v>
       </c>
       <c r="I365" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J365" t="s">
         <v>2182</v>
@@ -21419,7 +21419,7 @@
         <v>1657</v>
       </c>
       <c r="I366" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J366" t="s">
         <v>2183</v>
@@ -21454,7 +21454,7 @@
         <v>1657</v>
       </c>
       <c r="I367" t="s">
-        <v>1796</v>
+        <v>1797</v>
       </c>
       <c r="J367" t="s">
         <v>2184</v>
@@ -21594,7 +21594,7 @@
         <v>1657</v>
       </c>
       <c r="I371" t="s">
-        <v>1797</v>
+        <v>1798</v>
       </c>
       <c r="J371" t="s">
         <v>2188</v>
@@ -21629,7 +21629,7 @@
         <v>1657</v>
       </c>
       <c r="I372" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J372" t="s">
         <v>2189</v>
@@ -21664,7 +21664,7 @@
         <v>1657</v>
       </c>
       <c r="I373" t="s">
-        <v>1798</v>
+        <v>1799</v>
       </c>
       <c r="J373" t="s">
         <v>2190</v>
@@ -21734,7 +21734,7 @@
         <v>1657</v>
       </c>
       <c r="I375" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J375" t="s">
         <v>2192</v>
@@ -21874,7 +21874,7 @@
         <v>1657</v>
       </c>
       <c r="I379" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="J379" t="s">
         <v>2196</v>
@@ -21909,7 +21909,7 @@
         <v>1657</v>
       </c>
       <c r="I380" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J380" t="s">
         <v>2197</v>
@@ -21979,7 +21979,7 @@
         <v>1657</v>
       </c>
       <c r="I382" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J382" t="s">
         <v>2199</v>
@@ -22119,7 +22119,7 @@
         <v>1657</v>
       </c>
       <c r="I386" t="s">
-        <v>1735</v>
+        <v>1737</v>
       </c>
       <c r="J386" t="s">
         <v>2203</v>
@@ -22189,7 +22189,7 @@
         <v>1657</v>
       </c>
       <c r="I388" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="J388" t="s">
         <v>2205</v>
@@ -22224,7 +22224,7 @@
         <v>1657</v>
       </c>
       <c r="I389" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J389" t="s">
         <v>2206</v>
@@ -22364,7 +22364,7 @@
         <v>1657</v>
       </c>
       <c r="I393" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J393" t="s">
         <v>2210</v>
@@ -22399,7 +22399,7 @@
         <v>1657</v>
       </c>
       <c r="I394" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J394" t="s">
         <v>2018</v>
@@ -22644,7 +22644,7 @@
         <v>1657</v>
       </c>
       <c r="I401" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J401" t="s">
         <v>2217</v>
@@ -22749,7 +22749,7 @@
         <v>1657</v>
       </c>
       <c r="I404" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J404" t="s">
         <v>2220</v>
@@ -22787,7 +22787,7 @@
         <v>1670</v>
       </c>
       <c r="I405" t="s">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="J405" t="s">
         <v>2221</v>
@@ -22857,7 +22857,7 @@
         <v>1657</v>
       </c>
       <c r="I407" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J407" t="s">
         <v>2223</v>
@@ -22927,7 +22927,7 @@
         <v>1657</v>
       </c>
       <c r="I409" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J409" t="s">
         <v>2224</v>
@@ -22962,7 +22962,7 @@
         <v>1657</v>
       </c>
       <c r="I410" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J410" t="s">
         <v>2225</v>
@@ -23032,7 +23032,7 @@
         <v>1657</v>
       </c>
       <c r="I412" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J412" t="s">
         <v>2227</v>
@@ -23067,7 +23067,7 @@
         <v>1657</v>
       </c>
       <c r="I413" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J413" t="s">
         <v>2228</v>
@@ -23102,7 +23102,7 @@
         <v>1657</v>
       </c>
       <c r="I414" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J414" t="s">
         <v>2229</v>
@@ -23172,7 +23172,7 @@
         <v>1657</v>
       </c>
       <c r="I416" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="J416" t="s">
         <v>2231</v>
@@ -23207,7 +23207,7 @@
         <v>1657</v>
       </c>
       <c r="I417" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J417" t="s">
         <v>2232</v>
@@ -23277,7 +23277,7 @@
         <v>1657</v>
       </c>
       <c r="I419" t="s">
-        <v>1802</v>
+        <v>1803</v>
       </c>
       <c r="J419" t="s">
         <v>2234</v>
@@ -23312,7 +23312,7 @@
         <v>1657</v>
       </c>
       <c r="I420" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J420" t="s">
         <v>2235</v>
@@ -23347,7 +23347,7 @@
         <v>1657</v>
       </c>
       <c r="I421" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J421" t="s">
         <v>2236</v>
@@ -23452,7 +23452,7 @@
         <v>1657</v>
       </c>
       <c r="I424" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J424" t="s">
         <v>2239</v>
@@ -23557,7 +23557,7 @@
         <v>1657</v>
       </c>
       <c r="I427" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J427" t="s">
         <v>2242</v>
@@ -23627,7 +23627,7 @@
         <v>1657</v>
       </c>
       <c r="I429" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J429" t="s">
         <v>2244</v>
@@ -23662,7 +23662,7 @@
         <v>1657</v>
       </c>
       <c r="I430" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J430" t="s">
         <v>2245</v>
@@ -23697,7 +23697,7 @@
         <v>1657</v>
       </c>
       <c r="I431" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J431" t="s">
         <v>2246</v>
@@ -23767,7 +23767,7 @@
         <v>1657</v>
       </c>
       <c r="I433" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J433" t="s">
         <v>2248</v>
@@ -23837,7 +23837,7 @@
         <v>1657</v>
       </c>
       <c r="I435" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J435" t="s">
         <v>2250</v>
@@ -23872,7 +23872,7 @@
         <v>1657</v>
       </c>
       <c r="I436" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J436" t="s">
         <v>2251</v>
@@ -23907,7 +23907,7 @@
         <v>1657</v>
       </c>
       <c r="I437" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J437" t="s">
         <v>2252</v>
@@ -23977,7 +23977,7 @@
         <v>1657</v>
       </c>
       <c r="I439" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J439" t="s">
         <v>2254</v>
@@ -24085,7 +24085,7 @@
         <v>1671</v>
       </c>
       <c r="I442" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="J442" t="s">
         <v>2257</v>
@@ -24120,7 +24120,7 @@
         <v>1657</v>
       </c>
       <c r="I443" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J443" t="s">
         <v>2258</v>
@@ -24225,7 +24225,7 @@
         <v>1657</v>
       </c>
       <c r="I446" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J446" t="s">
         <v>2261</v>
@@ -24260,7 +24260,7 @@
         <v>1657</v>
       </c>
       <c r="I447" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J447" t="s">
         <v>2262</v>
@@ -24330,7 +24330,7 @@
         <v>1657</v>
       </c>
       <c r="I449" t="s">
-        <v>1803</v>
+        <v>1804</v>
       </c>
       <c r="J449" t="s">
         <v>2264</v>
@@ -24400,7 +24400,7 @@
         <v>1657</v>
       </c>
       <c r="I451" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J451" t="s">
         <v>2266</v>
@@ -24435,7 +24435,7 @@
         <v>1657</v>
       </c>
       <c r="I452" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J452" t="s">
         <v>2267</v>
@@ -24470,7 +24470,7 @@
         <v>1657</v>
       </c>
       <c r="I453" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J453" t="s">
         <v>2268</v>
@@ -24540,7 +24540,7 @@
         <v>1657</v>
       </c>
       <c r="I455" t="s">
-        <v>1804</v>
+        <v>1805</v>
       </c>
       <c r="J455" t="s">
         <v>2270</v>
@@ -24575,7 +24575,7 @@
         <v>1657</v>
       </c>
       <c r="I456" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J456" t="s">
         <v>2270</v>
@@ -24645,7 +24645,7 @@
         <v>1657</v>
       </c>
       <c r="I458" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J458" t="s">
         <v>2272</v>
@@ -24680,7 +24680,7 @@
         <v>1657</v>
       </c>
       <c r="I459" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J459" t="s">
         <v>2273</v>
@@ -24715,7 +24715,7 @@
         <v>1657</v>
       </c>
       <c r="I460" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J460" t="s">
         <v>2274</v>
@@ -24820,7 +24820,7 @@
         <v>1657</v>
       </c>
       <c r="I463" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J463" t="s">
         <v>2277</v>
@@ -24855,7 +24855,7 @@
         <v>1657</v>
       </c>
       <c r="I464" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="J464" t="s">
         <v>2278</v>
@@ -24890,7 +24890,7 @@
         <v>1657</v>
       </c>
       <c r="I465" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J465" t="s">
         <v>2279</v>
@@ -24925,7 +24925,7 @@
         <v>1657</v>
       </c>
       <c r="I466" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J466" t="s">
         <v>2280</v>
@@ -24960,7 +24960,7 @@
         <v>1657</v>
       </c>
       <c r="I467" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="J467" t="s">
         <v>2281</v>
@@ -24995,7 +24995,7 @@
         <v>1657</v>
       </c>
       <c r="I468" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="J468" t="s">
         <v>2282</v>
@@ -25030,7 +25030,7 @@
         <v>1657</v>
       </c>
       <c r="I469" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J469" t="s">
         <v>2283</v>
@@ -25065,7 +25065,7 @@
         <v>1657</v>
       </c>
       <c r="I470" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J470" t="s">
         <v>2284</v>
@@ -25170,7 +25170,7 @@
         <v>1657</v>
       </c>
       <c r="I473" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J473" t="s">
         <v>2287</v>
@@ -25310,7 +25310,7 @@
         <v>1657</v>
       </c>
       <c r="I477" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J477" t="s">
         <v>2291</v>
@@ -25345,7 +25345,7 @@
         <v>1657</v>
       </c>
       <c r="I478" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J478" t="s">
         <v>2292</v>
@@ -25380,7 +25380,7 @@
         <v>1657</v>
       </c>
       <c r="I479" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J479" t="s">
         <v>2293</v>
@@ -25520,7 +25520,7 @@
         <v>1657</v>
       </c>
       <c r="I483" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="J483" t="s">
         <v>2297</v>
@@ -25555,7 +25555,7 @@
         <v>1657</v>
       </c>
       <c r="I484" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J484" t="s">
         <v>2298</v>
@@ -25590,7 +25590,7 @@
         <v>1657</v>
       </c>
       <c r="I485" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J485" t="s">
         <v>2299</v>
@@ -25628,7 +25628,7 @@
         <v>1672</v>
       </c>
       <c r="I486" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J486" t="s">
         <v>2300</v>
@@ -25663,7 +25663,7 @@
         <v>1657</v>
       </c>
       <c r="I487" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J487" t="s">
         <v>2301</v>
@@ -25698,7 +25698,7 @@
         <v>1657</v>
       </c>
       <c r="I488" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J488" t="s">
         <v>2302</v>
@@ -25908,7 +25908,7 @@
         <v>1657</v>
       </c>
       <c r="I494" t="s">
-        <v>1806</v>
+        <v>1807</v>
       </c>
       <c r="J494" t="s">
         <v>2308</v>
@@ -25943,7 +25943,7 @@
         <v>1657</v>
       </c>
       <c r="I495" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J495" t="s">
         <v>2309</v>
@@ -25978,7 +25978,7 @@
         <v>1657</v>
       </c>
       <c r="I496" t="s">
-        <v>1807</v>
+        <v>1808</v>
       </c>
       <c r="J496" t="s">
         <v>2310</v>
@@ -26013,7 +26013,7 @@
         <v>1657</v>
       </c>
       <c r="I497" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J497" t="s">
         <v>2311</v>
@@ -26048,7 +26048,7 @@
         <v>1657</v>
       </c>
       <c r="I498" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J498" t="s">
         <v>2312</v>
@@ -26118,7 +26118,7 @@
         <v>1657</v>
       </c>
       <c r="I500" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J500" t="s">
         <v>2314</v>
@@ -26153,7 +26153,7 @@
         <v>1657</v>
       </c>
       <c r="I501" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J501" t="s">
         <v>2315</v>
@@ -26258,7 +26258,7 @@
         <v>1657</v>
       </c>
       <c r="I504" t="s">
-        <v>1808</v>
+        <v>1809</v>
       </c>
       <c r="J504" t="s">
         <v>2318</v>
@@ -26328,7 +26328,7 @@
         <v>1657</v>
       </c>
       <c r="I506" t="s">
-        <v>1808</v>
+        <v>1809</v>
       </c>
       <c r="J506" t="s">
         <v>2320</v>
@@ -26433,7 +26433,7 @@
         <v>1657</v>
       </c>
       <c r="I509" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J509" t="s">
         <v>2323</v>
@@ -26468,7 +26468,7 @@
         <v>1657</v>
       </c>
       <c r="I510" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J510" t="s">
         <v>2324</v>
@@ -26503,7 +26503,7 @@
         <v>1657</v>
       </c>
       <c r="I511" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J511" t="s">
         <v>2325</v>
@@ -26538,7 +26538,7 @@
         <v>1657</v>
       </c>
       <c r="I512" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="J512" t="s">
         <v>2326</v>
@@ -26573,7 +26573,7 @@
         <v>1657</v>
       </c>
       <c r="I513" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J513" t="s">
         <v>2327</v>
@@ -26608,7 +26608,7 @@
         <v>1657</v>
       </c>
       <c r="I514" t="s">
-        <v>1718</v>
+        <v>1720</v>
       </c>
       <c r="J514" t="s">
         <v>2328</v>
@@ -26643,7 +26643,7 @@
         <v>1657</v>
       </c>
       <c r="I515" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J515" t="s">
         <v>2329</v>
@@ -26713,7 +26713,7 @@
         <v>1657</v>
       </c>
       <c r="I517" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J517" t="s">
         <v>2331</v>
@@ -26783,7 +26783,7 @@
         <v>1657</v>
       </c>
       <c r="I519" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J519" t="s">
         <v>2333</v>
@@ -26923,7 +26923,7 @@
         <v>1657</v>
       </c>
       <c r="I523" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J523" t="s">
         <v>2337</v>
@@ -26958,7 +26958,7 @@
         <v>1657</v>
       </c>
       <c r="I524" t="s">
-        <v>1809</v>
+        <v>1810</v>
       </c>
       <c r="J524" t="s">
         <v>2338</v>
@@ -27101,7 +27101,7 @@
         <v>1657</v>
       </c>
       <c r="I528" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J528" t="s">
         <v>2342</v>
@@ -27136,7 +27136,7 @@
         <v>1657</v>
       </c>
       <c r="I529" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J529" t="s">
         <v>2343</v>
@@ -27171,7 +27171,7 @@
         <v>1657</v>
       </c>
       <c r="I530" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="J530" t="s">
         <v>2344</v>
@@ -27206,7 +27206,7 @@
         <v>1657</v>
       </c>
       <c r="I531" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J531" t="s">
         <v>2345</v>
@@ -27276,7 +27276,7 @@
         <v>1657</v>
       </c>
       <c r="I533" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J533" t="s">
         <v>2347</v>
@@ -27311,7 +27311,7 @@
         <v>1657</v>
       </c>
       <c r="I534" t="s">
-        <v>1810</v>
+        <v>1811</v>
       </c>
       <c r="J534" t="s">
         <v>2348</v>
@@ -27381,7 +27381,7 @@
         <v>1657</v>
       </c>
       <c r="I536" t="s">
-        <v>1811</v>
+        <v>1812</v>
       </c>
       <c r="J536" t="s">
         <v>2350</v>
@@ -27416,7 +27416,7 @@
         <v>1657</v>
       </c>
       <c r="I537" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J537" t="s">
         <v>2351</v>
@@ -27559,7 +27559,7 @@
         <v>1674</v>
       </c>
       <c r="I541" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J541" t="s">
         <v>2355</v>
@@ -27594,7 +27594,7 @@
         <v>1657</v>
       </c>
       <c r="I542" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J542" t="s">
         <v>2356</v>
@@ -27699,7 +27699,7 @@
         <v>1657</v>
       </c>
       <c r="I545" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J545" t="s">
         <v>2359</v>
@@ -27734,7 +27734,7 @@
         <v>1657</v>
       </c>
       <c r="I546" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J546" t="s">
         <v>2360</v>
@@ -27874,7 +27874,7 @@
         <v>1657</v>
       </c>
       <c r="I550" t="s">
-        <v>1812</v>
+        <v>1813</v>
       </c>
       <c r="J550" t="s">
         <v>2364</v>
@@ -28014,7 +28014,7 @@
         <v>1657</v>
       </c>
       <c r="I554" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="J554" t="s">
         <v>2368</v>
@@ -28049,7 +28049,7 @@
         <v>1657</v>
       </c>
       <c r="I555" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J555" t="s">
         <v>2369</v>
@@ -28084,7 +28084,7 @@
         <v>1657</v>
       </c>
       <c r="I556" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J556" t="s">
         <v>2370</v>
@@ -28154,7 +28154,7 @@
         <v>1657</v>
       </c>
       <c r="I558" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J558" t="s">
         <v>2372</v>
@@ -28189,7 +28189,7 @@
         <v>1657</v>
       </c>
       <c r="I559" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J559" t="s">
         <v>2373</v>
@@ -28224,7 +28224,7 @@
         <v>1657</v>
       </c>
       <c r="I560" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J560" t="s">
         <v>2374</v>
@@ -28259,7 +28259,7 @@
         <v>1657</v>
       </c>
       <c r="I561" t="s">
-        <v>1813</v>
+        <v>1814</v>
       </c>
       <c r="J561" t="s">
         <v>2375</v>
@@ -28294,7 +28294,7 @@
         <v>1657</v>
       </c>
       <c r="I562" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J562" t="s">
         <v>2376</v>
@@ -28329,7 +28329,7 @@
         <v>1657</v>
       </c>
       <c r="I563" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="J563" t="s">
         <v>2377</v>
@@ -28364,7 +28364,7 @@
         <v>1657</v>
       </c>
       <c r="I564" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J564" t="s">
         <v>2378</v>
@@ -28399,7 +28399,7 @@
         <v>1657</v>
       </c>
       <c r="I565" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J565" t="s">
         <v>2379</v>
@@ -28434,7 +28434,7 @@
         <v>1657</v>
       </c>
       <c r="I566" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J566" t="s">
         <v>2380</v>
@@ -28469,7 +28469,7 @@
         <v>1657</v>
       </c>
       <c r="I567" t="s">
-        <v>1814</v>
+        <v>1815</v>
       </c>
       <c r="J567" t="s">
         <v>2381</v>
@@ -28504,7 +28504,7 @@
         <v>1657</v>
       </c>
       <c r="I568" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J568" t="s">
         <v>2382</v>
@@ -28539,7 +28539,7 @@
         <v>1657</v>
       </c>
       <c r="I569" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J569" t="s">
         <v>2383</v>
@@ -28577,7 +28577,7 @@
         <v>1675</v>
       </c>
       <c r="I570" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J570" t="s">
         <v>2384</v>
@@ -28647,7 +28647,7 @@
         <v>1657</v>
       </c>
       <c r="I572" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J572" t="s">
         <v>2386</v>
@@ -28717,7 +28717,7 @@
         <v>1657</v>
       </c>
       <c r="I574" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J574" t="s">
         <v>2388</v>
@@ -28752,7 +28752,7 @@
         <v>1657</v>
       </c>
       <c r="I575" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J575" t="s">
         <v>2389</v>
@@ -28790,7 +28790,7 @@
         <v>1676</v>
       </c>
       <c r="I576" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J576" t="s">
         <v>2390</v>
@@ -28825,7 +28825,7 @@
         <v>1657</v>
       </c>
       <c r="I577" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J577" t="s">
         <v>2391</v>
@@ -28860,7 +28860,7 @@
         <v>1657</v>
       </c>
       <c r="I578" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J578" t="s">
         <v>2392</v>
@@ -28895,7 +28895,7 @@
         <v>1657</v>
       </c>
       <c r="I579" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J579" t="s">
         <v>2393</v>
@@ -28930,7 +28930,7 @@
         <v>1657</v>
       </c>
       <c r="I580" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J580" t="s">
         <v>2394</v>
@@ -28965,7 +28965,7 @@
         <v>1657</v>
       </c>
       <c r="I581" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J581" t="s">
         <v>2395</v>
@@ -29000,7 +29000,7 @@
         <v>1657</v>
       </c>
       <c r="I582" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J582" t="s">
         <v>2396</v>
@@ -29035,7 +29035,7 @@
         <v>1657</v>
       </c>
       <c r="I583" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J583" t="s">
         <v>2397</v>
@@ -29070,7 +29070,7 @@
         <v>1657</v>
       </c>
       <c r="I584" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="J584" t="s">
         <v>2398</v>
@@ -29105,7 +29105,7 @@
         <v>1657</v>
       </c>
       <c r="I585" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J585" t="s">
         <v>2399</v>
@@ -29140,7 +29140,7 @@
         <v>1657</v>
       </c>
       <c r="I586" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J586" t="s">
         <v>2400</v>
@@ -29175,7 +29175,7 @@
         <v>1657</v>
       </c>
       <c r="I587" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J587" t="s">
         <v>2401</v>
@@ -29210,7 +29210,7 @@
         <v>1657</v>
       </c>
       <c r="I588" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J588" t="s">
         <v>2402</v>
@@ -29248,7 +29248,7 @@
         <v>1647</v>
       </c>
       <c r="I589" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="J589" t="s">
         <v>2403</v>
@@ -29283,7 +29283,7 @@
         <v>1657</v>
       </c>
       <c r="I590" t="s">
-        <v>1815</v>
+        <v>1816</v>
       </c>
       <c r="J590" t="s">
         <v>2404</v>
@@ -29353,7 +29353,7 @@
         <v>1657</v>
       </c>
       <c r="I592" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J592" t="s">
         <v>2406</v>
@@ -29423,7 +29423,7 @@
         <v>1657</v>
       </c>
       <c r="I594" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J594" t="s">
         <v>2408</v>
@@ -29458,7 +29458,7 @@
         <v>1657</v>
       </c>
       <c r="I595" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J595" t="s">
         <v>2409</v>
@@ -29493,7 +29493,7 @@
         <v>1657</v>
       </c>
       <c r="I596" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J596" t="s">
         <v>2410</v>
@@ -29528,7 +29528,7 @@
         <v>1657</v>
       </c>
       <c r="I597" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J597" t="s">
         <v>2411</v>
@@ -29563,7 +29563,7 @@
         <v>1657</v>
       </c>
       <c r="I598" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J598" t="s">
         <v>2412</v>
@@ -29598,7 +29598,7 @@
         <v>1657</v>
       </c>
       <c r="I599" t="s">
-        <v>1816</v>
+        <v>1817</v>
       </c>
       <c r="J599" t="s">
         <v>2413</v>
@@ -29633,7 +29633,7 @@
         <v>1657</v>
       </c>
       <c r="I600" t="s">
-        <v>1817</v>
+        <v>1818</v>
       </c>
       <c r="J600" t="s">
         <v>2414</v>
@@ -29671,7 +29671,7 @@
         <v>1677</v>
       </c>
       <c r="I601" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J601" t="s">
         <v>2415</v>
@@ -29741,7 +29741,7 @@
         <v>1657</v>
       </c>
       <c r="I603" t="s">
-        <v>1818</v>
+        <v>1819</v>
       </c>
       <c r="J603" t="s">
         <v>2417</v>
@@ -29776,7 +29776,7 @@
         <v>1657</v>
       </c>
       <c r="I604" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="J604" t="s">
         <v>2418</v>
@@ -29811,7 +29811,7 @@
         <v>1657</v>
       </c>
       <c r="I605" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J605" t="s">
         <v>2419</v>
@@ -29919,7 +29919,7 @@
         <v>1677</v>
       </c>
       <c r="I608" t="s">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="J608" t="s">
         <v>2422</v>
@@ -29989,7 +29989,7 @@
         <v>1657</v>
       </c>
       <c r="I610" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J610" t="s">
         <v>2424</v>
@@ -30024,7 +30024,7 @@
         <v>1657</v>
       </c>
       <c r="I611" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J611" t="s">
         <v>2425</v>
@@ -30062,7 +30062,7 @@
         <v>1678</v>
       </c>
       <c r="I612" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="J612" t="s">
         <v>2426</v>
@@ -30097,7 +30097,7 @@
         <v>1657</v>
       </c>
       <c r="I613" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J613" t="s">
         <v>2427</v>
@@ -30167,7 +30167,7 @@
         <v>1657</v>
       </c>
       <c r="I615" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J615" t="s">
         <v>2429</v>
@@ -30202,7 +30202,7 @@
         <v>1657</v>
       </c>
       <c r="I616" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J616" t="s">
         <v>2430</v>
@@ -30275,7 +30275,7 @@
         <v>1657</v>
       </c>
       <c r="I618" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J618" t="s">
         <v>2432</v>
@@ -30345,7 +30345,7 @@
         <v>1657</v>
       </c>
       <c r="I620" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J620" t="s">
         <v>2434</v>
@@ -30380,7 +30380,7 @@
         <v>1657</v>
       </c>
       <c r="I621" t="s">
-        <v>1779</v>
+        <v>1698</v>
       </c>
       <c r="J621" t="s">
         <v>2435</v>
@@ -30415,7 +30415,7 @@
         <v>1657</v>
       </c>
       <c r="I622" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J622" t="s">
         <v>2436</v>
@@ -30453,7 +30453,7 @@
         <v>1680</v>
       </c>
       <c r="I623" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J623" t="s">
         <v>2437</v>
@@ -30488,7 +30488,7 @@
         <v>1657</v>
       </c>
       <c r="I624" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J624" t="s">
         <v>2438</v>
@@ -30523,7 +30523,7 @@
         <v>1657</v>
       </c>
       <c r="I625" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J625" t="s">
         <v>2439</v>
@@ -30558,7 +30558,7 @@
         <v>1657</v>
       </c>
       <c r="I626" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J626" t="s">
         <v>2440</v>
@@ -30596,7 +30596,7 @@
         <v>1681</v>
       </c>
       <c r="I627" t="s">
-        <v>1749</v>
+        <v>1751</v>
       </c>
       <c r="J627" t="s">
         <v>2441</v>
@@ -30634,7 +30634,7 @@
         <v>1681</v>
       </c>
       <c r="I628" t="s">
-        <v>1698</v>
+        <v>1709</v>
       </c>
       <c r="J628" t="s">
         <v>2441</v>
@@ -30669,7 +30669,7 @@
         <v>1657</v>
       </c>
       <c r="I629" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J629" t="s">
         <v>2442</v>
@@ -30707,7 +30707,7 @@
         <v>1682</v>
       </c>
       <c r="I630" t="s">
-        <v>1820</v>
+        <v>1821</v>
       </c>
       <c r="J630" t="s">
         <v>2443</v>
@@ -30777,7 +30777,7 @@
         <v>1657</v>
       </c>
       <c r="I632" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J632" t="s">
         <v>2445</v>
@@ -30812,7 +30812,7 @@
         <v>1657</v>
       </c>
       <c r="I633" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J633" t="s">
         <v>2446</v>
@@ -30850,7 +30850,7 @@
         <v>1677</v>
       </c>
       <c r="I634" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="J634" t="s">
         <v>2447</v>
@@ -30885,7 +30885,7 @@
         <v>1657</v>
       </c>
       <c r="I635" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="J635" t="s">
         <v>2448</v>
@@ -30923,7 +30923,7 @@
         <v>1667</v>
       </c>
       <c r="I636" t="s">
-        <v>1821</v>
+        <v>1822</v>
       </c>
       <c r="J636" t="s">
         <v>2449</v>
@@ -30961,7 +30961,7 @@
         <v>1683</v>
       </c>
       <c r="I637" t="s">
-        <v>1822</v>
+        <v>1823</v>
       </c>
       <c r="J637" t="s">
         <v>2450</v>
@@ -30999,7 +30999,7 @@
         <v>1667</v>
       </c>
       <c r="I638" t="s">
-        <v>1823</v>
+        <v>1824</v>
       </c>
       <c r="J638" t="s">
         <v>2451</v>
@@ -31037,7 +31037,7 @@
         <v>1684</v>
       </c>
       <c r="I639" t="s">
-        <v>1824</v>
+        <v>1825</v>
       </c>
       <c r="J639" t="s">
         <v>2452</v>
@@ -31072,7 +31072,7 @@
         <v>1657</v>
       </c>
       <c r="I640" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J640" t="s">
         <v>2453</v>
@@ -31107,7 +31107,7 @@
         <v>1657</v>
       </c>
       <c r="I641" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J641" t="s">
         <v>2454</v>
@@ -31142,7 +31142,7 @@
         <v>1657</v>
       </c>
       <c r="I642" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J642" t="s">
         <v>2455</v>
@@ -31180,7 +31180,7 @@
         <v>1677</v>
       </c>
       <c r="I643" t="s">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="J643" t="s">
         <v>2456</v>
@@ -31355,7 +31355,7 @@
         <v>1657</v>
       </c>
       <c r="I648" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J648" t="s">
         <v>2461</v>
@@ -31390,7 +31390,7 @@
         <v>1657</v>
       </c>
       <c r="I649" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J649" t="s">
         <v>2462</v>
@@ -31425,7 +31425,7 @@
         <v>1657</v>
       </c>
       <c r="I650" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="J650" t="s">
         <v>2463</v>
@@ -31460,7 +31460,7 @@
         <v>1657</v>
       </c>
       <c r="I651" t="s">
-        <v>1826</v>
+        <v>1827</v>
       </c>
       <c r="J651" t="s">
         <v>2464</v>
@@ -31495,7 +31495,7 @@
         <v>1657</v>
       </c>
       <c r="I652" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J652" t="s">
         <v>2465</v>
@@ -31530,7 +31530,7 @@
         <v>1657</v>
       </c>
       <c r="I653" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J653" t="s">
         <v>2466</v>
@@ -31565,7 +31565,7 @@
         <v>1657</v>
       </c>
       <c r="I654" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J654" t="s">
         <v>2467</v>
@@ -31600,7 +31600,7 @@
         <v>1657</v>
       </c>
       <c r="I655" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="J655" t="s">
         <v>2468</v>
@@ -31635,7 +31635,7 @@
         <v>1657</v>
       </c>
       <c r="I656" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J656" t="s">
         <v>2469</v>
@@ -31673,7 +31673,7 @@
         <v>1685</v>
       </c>
       <c r="I657" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
       <c r="J657" t="s">
         <v>2470</v>
@@ -31708,7 +31708,7 @@
         <v>1657</v>
       </c>
       <c r="I658" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="J658" t="s">
         <v>2471</v>
@@ -31743,7 +31743,7 @@
         <v>1657</v>
       </c>
       <c r="I659" t="s">
-        <v>1828</v>
+        <v>1709</v>
       </c>
       <c r="J659" t="s">
         <v>2472</v>
@@ -31778,7 +31778,7 @@
         <v>1657</v>
       </c>
       <c r="I660" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J660" t="s">
         <v>2473</v>
@@ -31889,7 +31889,7 @@
         <v>1657</v>
       </c>
       <c r="I663" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J663" t="s">
         <v>2476</v>
@@ -32000,7 +32000,7 @@
         <v>1657</v>
       </c>
       <c r="I666" t="s">
-        <v>1828</v>
+        <v>1709</v>
       </c>
       <c r="J666" t="s">
         <v>2479</v>
@@ -32073,7 +32073,7 @@
         <v>1657</v>
       </c>
       <c r="I668" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J668" t="s">
         <v>2481</v>
@@ -32108,7 +32108,7 @@
         <v>1657</v>
       </c>
       <c r="I669" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J669" t="s">
         <v>2482</v>
@@ -32146,7 +32146,7 @@
         <v>1647</v>
       </c>
       <c r="I670" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J670" t="s">
         <v>2483</v>
@@ -32181,7 +32181,7 @@
         <v>1657</v>
       </c>
       <c r="I671" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J671" t="s">
         <v>2484</v>
@@ -32216,7 +32216,7 @@
         <v>1657</v>
       </c>
       <c r="I672" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J672" t="s">
         <v>2485</v>
@@ -32251,7 +32251,7 @@
         <v>1657</v>
       </c>
       <c r="I673" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J673" t="s">
         <v>2486</v>
@@ -32286,7 +32286,7 @@
         <v>1657</v>
       </c>
       <c r="I674" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J674" t="s">
         <v>2487</v>
@@ -32321,7 +32321,7 @@
         <v>1657</v>
       </c>
       <c r="I675" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J675" t="s">
         <v>2488</v>
@@ -32356,7 +32356,7 @@
         <v>1657</v>
       </c>
       <c r="I676" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J676" t="s">
         <v>2489</v>
@@ -32391,7 +32391,7 @@
         <v>1657</v>
       </c>
       <c r="I677" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J677" t="s">
         <v>2490</v>
@@ -32429,7 +32429,7 @@
         <v>1684</v>
       </c>
       <c r="I678" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="J678" t="s">
         <v>2491</v>
@@ -32467,7 +32467,7 @@
         <v>1689</v>
       </c>
       <c r="I679" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J679" t="s">
         <v>2492</v>
@@ -32502,7 +32502,7 @@
         <v>1657</v>
       </c>
       <c r="I680" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J680" t="s">
         <v>2493</v>
@@ -32537,7 +32537,7 @@
         <v>1657</v>
       </c>
       <c r="I681" t="s">
-        <v>1828</v>
+        <v>1709</v>
       </c>
       <c r="J681" t="s">
         <v>2494</v>
@@ -32572,7 +32572,7 @@
         <v>1657</v>
       </c>
       <c r="I682" t="s">
-        <v>1828</v>
+        <v>1709</v>
       </c>
       <c r="J682" t="s">
         <v>2495</v>
@@ -32607,7 +32607,7 @@
         <v>1657</v>
       </c>
       <c r="I683" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="J683" t="s">
         <v>2496</v>
@@ -32642,7 +32642,7 @@
         <v>1657</v>
       </c>
       <c r="I684" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="J684" t="s">
         <v>2497</v>
@@ -32677,7 +32677,7 @@
         <v>1657</v>
       </c>
       <c r="I685" t="s">
-        <v>1751</v>
+        <v>1715</v>
       </c>
       <c r="J685" t="s">
         <v>2498</v>
@@ -32715,7 +32715,7 @@
         <v>1690</v>
       </c>
       <c r="I686" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="J686" t="s">
         <v>2499</v>
@@ -32791,7 +32791,7 @@
         <v>1691</v>
       </c>
       <c r="I688" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="J688" t="s">
         <v>2501</v>
@@ -32902,7 +32902,7 @@
         <v>1657</v>
       </c>
       <c r="I691" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="J691" t="s">
         <v>1837</v>
@@ -32937,7 +32937,7 @@
         <v>1657</v>
       </c>
       <c r="I692" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="J692" t="s">
         <v>2504</v>
@@ -32975,7 +32975,7 @@
         <v>1691</v>
       </c>
       <c r="I693" t="s">
-        <v>1698</v>
+        <v>1829</v>
       </c>
       <c r="J693" t="s">
         <v>2505</v>
@@ -33007,7 +33007,7 @@
         <v>1657</v>
       </c>
       <c r="I694" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J694" t="s">
         <v>2506</v>
@@ -33039,7 +33039,7 @@
         <v>1657</v>
       </c>
       <c r="I695" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="J695" t="s">
         <v>2507</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-02 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -20745,7 +20745,7 @@
     </row>
     <row r="347" spans="1:12">
       <c r="A347" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B347" t="s">
         <v>386</v>
@@ -20766,7 +20766,7 @@
         <v>1659</v>
       </c>
       <c r="I347" t="s">
-        <v>1788</v>
+        <v>1754</v>
       </c>
       <c r="J347" t="s">
         <v>2166</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-02 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -97,21 +97,21 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
+  </si>
+  <si>
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
   </si>
   <si>
@@ -5131,102 +5131,102 @@
     <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
   </si>
   <si>
+    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
+    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
     <t>ANA LÍCIA SOUZA E SILVA</t>
   </si>
   <si>
-    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
-    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO, RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
     <t>LUIZ FRANCISCO PERALTA BRAGA</t>
   </si>
   <si>
@@ -5287,58 +5287,58 @@
     <t>FERNANDA TEIXEIRA ROSALBA</t>
   </si>
   <si>
+    <t>ANDRÉA DINIZ MATTOS</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES, HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
     <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
   </si>
   <si>
-    <t>ANDRÉA DINIZ MATTOS</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES, HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>DANIEL FONTANA OBERLING,EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
   </si>
   <si>
     <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>DANIEL FONTANA OBERLING,EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
   </si>
   <si>
     <t>VANESSA FERNANDES LEÃO</t>
@@ -11422,7 +11422,7 @@
     </row>
     <row r="85" spans="1:12">
       <c r="A85" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B85" t="s">
         <v>124</v>
@@ -11443,7 +11443,7 @@
         <v>1634</v>
       </c>
       <c r="I85" t="s">
-        <v>1705</v>
+        <v>1673</v>
       </c>
       <c r="J85" t="s">
         <v>1886</v>
@@ -11478,7 +11478,7 @@
         <v>1634</v>
       </c>
       <c r="I86" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="J86" t="s">
         <v>1887</v>
@@ -11492,7 +11492,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B87" t="s">
         <v>126</v>
@@ -11516,7 +11516,7 @@
         <v>1641</v>
       </c>
       <c r="I87" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J87" t="s">
         <v>1888</v>
@@ -11530,7 +11530,7 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B88" t="s">
         <v>127</v>
@@ -11554,7 +11554,7 @@
         <v>1641</v>
       </c>
       <c r="I88" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J88" t="s">
         <v>1888</v>
@@ -11624,7 +11624,7 @@
         <v>1634</v>
       </c>
       <c r="I90" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
       <c r="J90" t="s">
         <v>1890</v>
@@ -11834,7 +11834,7 @@
         <v>1634</v>
       </c>
       <c r="I96" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="J96" t="s">
         <v>1896</v>
@@ -11904,7 +11904,7 @@
         <v>1634</v>
       </c>
       <c r="I98" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="J98" t="s">
         <v>1898</v>
@@ -12184,7 +12184,7 @@
         <v>1634</v>
       </c>
       <c r="I106" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J106" t="s">
         <v>1906</v>
@@ -12289,7 +12289,7 @@
         <v>1634</v>
       </c>
       <c r="I109" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="J109" t="s">
         <v>1909</v>
@@ -12324,7 +12324,7 @@
         <v>1634</v>
       </c>
       <c r="I110" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="J110" t="s">
         <v>1910</v>
@@ -12534,7 +12534,7 @@
         <v>1634</v>
       </c>
       <c r="I116" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="J116" t="s">
         <v>1916</v>
@@ -12604,7 +12604,7 @@
         <v>1634</v>
       </c>
       <c r="I118" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="J118" t="s">
         <v>1918</v>
@@ -12709,7 +12709,7 @@
         <v>1634</v>
       </c>
       <c r="I121" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J121" t="s">
         <v>1921</v>
@@ -12779,7 +12779,7 @@
         <v>1634</v>
       </c>
       <c r="I123" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J123" t="s">
         <v>1923</v>
@@ -12849,7 +12849,7 @@
         <v>1634</v>
       </c>
       <c r="I125" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J125" t="s">
         <v>1925</v>
@@ -12898,7 +12898,7 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B127" t="s">
         <v>166</v>
@@ -12919,7 +12919,7 @@
         <v>1634</v>
       </c>
       <c r="I127" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J127" t="s">
         <v>1927</v>
@@ -12992,7 +12992,7 @@
         <v>1525</v>
       </c>
       <c r="I129" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="J129" t="s">
         <v>1929</v>
@@ -13062,7 +13062,7 @@
         <v>1634</v>
       </c>
       <c r="I131" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="J131" t="s">
         <v>1931</v>
@@ -13111,7 +13111,7 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B133" t="s">
         <v>172</v>
@@ -13132,7 +13132,7 @@
         <v>1634</v>
       </c>
       <c r="I133" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J133" t="s">
         <v>1932</v>
@@ -13237,7 +13237,7 @@
         <v>1634</v>
       </c>
       <c r="I136" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J136" t="s">
         <v>1935</v>
@@ -13278,7 +13278,7 @@
         <v>1812</v>
       </c>
       <c r="K137" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L137" t="s">
         <v>2625</v>
@@ -13412,7 +13412,7 @@
         <v>1634</v>
       </c>
       <c r="I141" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J141" t="s">
         <v>1939</v>
@@ -13555,7 +13555,7 @@
         <v>1642</v>
       </c>
       <c r="I145" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J145" t="s">
         <v>1812</v>
@@ -13590,7 +13590,7 @@
         <v>1634</v>
       </c>
       <c r="I146" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J146" t="s">
         <v>1943</v>
@@ -13625,7 +13625,7 @@
         <v>1634</v>
       </c>
       <c r="I147" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J147" t="s">
         <v>1944</v>
@@ -13660,7 +13660,7 @@
         <v>1634</v>
       </c>
       <c r="I148" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J148" t="s">
         <v>1945</v>
@@ -13674,7 +13674,7 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B149" t="s">
         <v>188</v>
@@ -13709,7 +13709,7 @@
     </row>
     <row r="150" spans="1:12">
       <c r="A150" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B150" t="s">
         <v>189</v>
@@ -13730,7 +13730,7 @@
         <v>1634</v>
       </c>
       <c r="I150" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J150" t="s">
         <v>1947</v>
@@ -13744,7 +13744,7 @@
     </row>
     <row r="151" spans="1:12">
       <c r="A151" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B151" t="s">
         <v>190</v>
@@ -13765,7 +13765,7 @@
         <v>1634</v>
       </c>
       <c r="I151" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J151" t="s">
         <v>1948</v>
@@ -13814,7 +13814,7 @@
     </row>
     <row r="153" spans="1:12">
       <c r="A153" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B153" t="s">
         <v>192</v>
@@ -13835,7 +13835,7 @@
         <v>1634</v>
       </c>
       <c r="I153" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J153" t="s">
         <v>1950</v>
@@ -13954,7 +13954,7 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B157" t="s">
         <v>196</v>
@@ -13975,7 +13975,7 @@
         <v>1634</v>
       </c>
       <c r="I157" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J157" t="s">
         <v>1954</v>
@@ -13989,7 +13989,7 @@
     </row>
     <row r="158" spans="1:12">
       <c r="A158" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B158" t="s">
         <v>197</v>
@@ -14010,7 +14010,7 @@
         <v>1634</v>
       </c>
       <c r="I158" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J158" t="s">
         <v>1955</v>
@@ -14045,7 +14045,7 @@
         <v>1634</v>
       </c>
       <c r="I159" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J159" t="s">
         <v>1956</v>
@@ -14150,7 +14150,7 @@
         <v>1634</v>
       </c>
       <c r="I162" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J162" t="s">
         <v>1959</v>
@@ -14325,7 +14325,7 @@
         <v>1634</v>
       </c>
       <c r="I167" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J167" t="s">
         <v>1964</v>
@@ -14374,7 +14374,7 @@
     </row>
     <row r="169" spans="1:12">
       <c r="A169" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B169" t="s">
         <v>208</v>
@@ -14395,7 +14395,7 @@
         <v>1634</v>
       </c>
       <c r="I169" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J169" t="s">
         <v>1966</v>
@@ -14465,7 +14465,7 @@
         <v>1634</v>
       </c>
       <c r="I171" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J171" t="s">
         <v>1968</v>
@@ -14570,7 +14570,7 @@
         <v>1634</v>
       </c>
       <c r="I174" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J174" t="s">
         <v>1971</v>
@@ -14584,7 +14584,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B175" t="s">
         <v>214</v>
@@ -14605,7 +14605,7 @@
         <v>1634</v>
       </c>
       <c r="I175" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J175" t="s">
         <v>1972</v>
@@ -14654,7 +14654,7 @@
     </row>
     <row r="177" spans="1:12">
       <c r="A177" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B177" t="s">
         <v>216</v>
@@ -14675,7 +14675,7 @@
         <v>1634</v>
       </c>
       <c r="I177" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J177" t="s">
         <v>1974</v>
@@ -14794,7 +14794,7 @@
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B181" t="s">
         <v>220</v>
@@ -14815,7 +14815,7 @@
         <v>1634</v>
       </c>
       <c r="I181" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J181" t="s">
         <v>1978</v>
@@ -15039,7 +15039,7 @@
     </row>
     <row r="188" spans="1:12">
       <c r="A188" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B188" t="s">
         <v>227</v>
@@ -15060,7 +15060,7 @@
         <v>1634</v>
       </c>
       <c r="I188" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J188" t="s">
         <v>1985</v>
@@ -15637,7 +15637,7 @@
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B205" t="s">
         <v>244</v>
@@ -15658,7 +15658,7 @@
         <v>1634</v>
       </c>
       <c r="I205" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J205" t="s">
         <v>2000</v>
@@ -15672,7 +15672,7 @@
     </row>
     <row r="206" spans="1:12">
       <c r="A206" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B206" t="s">
         <v>245</v>
@@ -15742,7 +15742,7 @@
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B208" t="s">
         <v>247</v>
@@ -15763,7 +15763,7 @@
         <v>1634</v>
       </c>
       <c r="I208" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J208" t="s">
         <v>2003</v>
@@ -15952,7 +15952,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B214" t="s">
         <v>253</v>
@@ -15973,7 +15973,7 @@
         <v>1634</v>
       </c>
       <c r="I214" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J214" t="s">
         <v>2009</v>
@@ -16022,7 +16022,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B216" t="s">
         <v>255</v>
@@ -16043,7 +16043,7 @@
         <v>1634</v>
       </c>
       <c r="I216" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J216" t="s">
         <v>2011</v>
@@ -16092,7 +16092,7 @@
     </row>
     <row r="218" spans="1:12">
       <c r="A218" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B218" t="s">
         <v>257</v>
@@ -16113,7 +16113,7 @@
         <v>1634</v>
       </c>
       <c r="I218" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J218" t="s">
         <v>2013</v>
@@ -16302,7 +16302,7 @@
     </row>
     <row r="224" spans="1:12">
       <c r="A224" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B224" t="s">
         <v>263</v>
@@ -16323,7 +16323,7 @@
         <v>1634</v>
       </c>
       <c r="I224" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J224" t="s">
         <v>2019</v>
@@ -16512,7 +16512,7 @@
     </row>
     <row r="230" spans="1:12">
       <c r="A230" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B230" t="s">
         <v>269</v>
@@ -16533,7 +16533,7 @@
         <v>1634</v>
       </c>
       <c r="I230" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J230" t="s">
         <v>2024</v>
@@ -16547,7 +16547,7 @@
     </row>
     <row r="231" spans="1:12">
       <c r="A231" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B231" t="s">
         <v>270</v>
@@ -16568,7 +16568,7 @@
         <v>1634</v>
       </c>
       <c r="I231" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J231" t="s">
         <v>2025</v>
@@ -17040,7 +17040,7 @@
     </row>
     <row r="245" spans="1:12">
       <c r="A245" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B245" t="s">
         <v>284</v>
@@ -17495,7 +17495,7 @@
     </row>
     <row r="258" spans="1:12">
       <c r="A258" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B258" t="s">
         <v>297</v>
@@ -17516,7 +17516,7 @@
         <v>1634</v>
       </c>
       <c r="I258" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J258" t="s">
         <v>2052</v>
@@ -17565,7 +17565,7 @@
     </row>
     <row r="260" spans="1:12">
       <c r="A260" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B260" t="s">
         <v>299</v>
@@ -17635,7 +17635,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B262" t="s">
         <v>301</v>
@@ -17659,7 +17659,7 @@
         <v>1643</v>
       </c>
       <c r="I262" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J262" t="s">
         <v>2056</v>
@@ -17743,7 +17743,7 @@
     </row>
     <row r="265" spans="1:12">
       <c r="A265" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B265" t="s">
         <v>304</v>
@@ -17764,7 +17764,7 @@
         <v>1634</v>
       </c>
       <c r="I265" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J265" t="s">
         <v>2059</v>
@@ -17778,7 +17778,7 @@
     </row>
     <row r="266" spans="1:12">
       <c r="A266" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B266" t="s">
         <v>305</v>
@@ -17799,7 +17799,7 @@
         <v>1634</v>
       </c>
       <c r="I266" t="s">
-        <v>1757</v>
+        <v>1673</v>
       </c>
       <c r="J266" t="s">
         <v>2060</v>
@@ -17869,7 +17869,7 @@
         <v>1634</v>
       </c>
       <c r="I268" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="J268" t="s">
         <v>2062</v>
@@ -17904,7 +17904,7 @@
         <v>1634</v>
       </c>
       <c r="I269" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="J269" t="s">
         <v>2063</v>
@@ -17939,7 +17939,7 @@
         <v>1634</v>
       </c>
       <c r="I270" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J270" t="s">
         <v>2064</v>
@@ -17974,7 +17974,7 @@
         <v>1634</v>
       </c>
       <c r="I271" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J271" t="s">
         <v>2065</v>
@@ -18149,7 +18149,7 @@
         <v>1634</v>
       </c>
       <c r="I276" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="J276" t="s">
         <v>2069</v>
@@ -18222,7 +18222,7 @@
         <v>1644</v>
       </c>
       <c r="I278" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="J278" t="s">
         <v>2071</v>
@@ -18341,7 +18341,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B282" t="s">
         <v>321</v>
@@ -18362,7 +18362,7 @@
         <v>1634</v>
       </c>
       <c r="I282" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J282" t="s">
         <v>2074</v>
@@ -18397,7 +18397,7 @@
         <v>1634</v>
       </c>
       <c r="I283" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J283" t="s">
         <v>2075</v>
@@ -18621,7 +18621,7 @@
     </row>
     <row r="290" spans="1:12">
       <c r="A290" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B290" t="s">
         <v>329</v>
@@ -18642,7 +18642,7 @@
         <v>1634</v>
       </c>
       <c r="I290" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J290" t="s">
         <v>2082</v>
@@ -18726,7 +18726,7 @@
     </row>
     <row r="293" spans="1:12">
       <c r="A293" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B293" t="s">
         <v>332</v>
@@ -18747,7 +18747,7 @@
         <v>1634</v>
       </c>
       <c r="I293" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J293" t="s">
         <v>2085</v>
@@ -18761,7 +18761,7 @@
     </row>
     <row r="294" spans="1:12">
       <c r="A294" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B294" t="s">
         <v>333</v>
@@ -18782,7 +18782,7 @@
         <v>1634</v>
       </c>
       <c r="I294" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J294" t="s">
         <v>2086</v>
@@ -18995,7 +18995,7 @@
         <v>1634</v>
       </c>
       <c r="I300" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="J300" t="s">
         <v>2092</v>
@@ -19065,7 +19065,7 @@
         <v>1634</v>
       </c>
       <c r="I302" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J302" t="s">
         <v>2094</v>
@@ -19205,7 +19205,7 @@
         <v>1634</v>
       </c>
       <c r="I306" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J306" t="s">
         <v>2098</v>
@@ -19310,7 +19310,7 @@
         <v>1634</v>
       </c>
       <c r="I309" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J309" t="s">
         <v>2101</v>
@@ -19359,7 +19359,7 @@
     </row>
     <row r="311" spans="1:12">
       <c r="A311" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B311" t="s">
         <v>350</v>
@@ -19380,7 +19380,7 @@
         <v>1634</v>
       </c>
       <c r="I311" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J311" t="s">
         <v>2103</v>
@@ -19415,7 +19415,7 @@
         <v>1634</v>
       </c>
       <c r="I312" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="J312" t="s">
         <v>2104</v>
@@ -19429,7 +19429,7 @@
     </row>
     <row r="313" spans="1:12">
       <c r="A313" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B313" t="s">
         <v>352</v>
@@ -19450,7 +19450,7 @@
         <v>1634</v>
       </c>
       <c r="I313" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J313" t="s">
         <v>2105</v>
@@ -19569,7 +19569,7 @@
     </row>
     <row r="317" spans="1:12">
       <c r="A317" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B317" t="s">
         <v>356</v>
@@ -19590,7 +19590,7 @@
         <v>1634</v>
       </c>
       <c r="I317" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J317" t="s">
         <v>2109</v>
@@ -19639,7 +19639,7 @@
     </row>
     <row r="319" spans="1:12">
       <c r="A319" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B319" t="s">
         <v>358</v>
@@ -19660,7 +19660,7 @@
         <v>1634</v>
       </c>
       <c r="I319" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J319" t="s">
         <v>2111</v>
@@ -19744,7 +19744,7 @@
     </row>
     <row r="322" spans="1:12">
       <c r="A322" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B322" t="s">
         <v>361</v>
@@ -19765,7 +19765,7 @@
         <v>1634</v>
       </c>
       <c r="I322" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J322" t="s">
         <v>2114</v>
@@ -19779,7 +19779,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B323" t="s">
         <v>362</v>
@@ -19800,7 +19800,7 @@
         <v>1634</v>
       </c>
       <c r="I323" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J323" t="s">
         <v>2115</v>
@@ -19814,7 +19814,7 @@
     </row>
     <row r="324" spans="1:12">
       <c r="A324" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B324" t="s">
         <v>363</v>
@@ -19835,7 +19835,7 @@
         <v>1634</v>
       </c>
       <c r="I324" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J324" t="s">
         <v>2116</v>
@@ -19905,7 +19905,7 @@
         <v>1634</v>
       </c>
       <c r="I326" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
       <c r="J326" t="s">
         <v>2118</v>
@@ -19919,7 +19919,7 @@
     </row>
     <row r="327" spans="1:12">
       <c r="A327" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B327" t="s">
         <v>366</v>
@@ -19943,7 +19943,7 @@
         <v>1646</v>
       </c>
       <c r="I327" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J327" t="s">
         <v>2119</v>
@@ -20167,7 +20167,7 @@
     </row>
     <row r="334" spans="1:12">
       <c r="A334" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B334" t="s">
         <v>373</v>
@@ -20188,7 +20188,7 @@
         <v>1634</v>
       </c>
       <c r="I334" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J334" t="s">
         <v>2126</v>
@@ -20202,7 +20202,7 @@
     </row>
     <row r="335" spans="1:12">
       <c r="A335" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B335" t="s">
         <v>374</v>
@@ -20223,7 +20223,7 @@
         <v>1634</v>
       </c>
       <c r="I335" t="s">
-        <v>1766</v>
+        <v>1765</v>
       </c>
       <c r="J335" t="s">
         <v>2127</v>
@@ -20272,7 +20272,7 @@
     </row>
     <row r="337" spans="1:12">
       <c r="A337" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B337" t="s">
         <v>376</v>
@@ -20293,7 +20293,7 @@
         <v>1634</v>
       </c>
       <c r="I337" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J337" t="s">
         <v>2129</v>
@@ -20342,7 +20342,7 @@
     </row>
     <row r="339" spans="1:12">
       <c r="A339" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B339" t="s">
         <v>378</v>
@@ -20363,7 +20363,7 @@
         <v>1634</v>
       </c>
       <c r="I339" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J339" t="s">
         <v>2131</v>
@@ -20468,7 +20468,7 @@
         <v>1634</v>
       </c>
       <c r="I342" t="s">
-        <v>1767</v>
+        <v>1766</v>
       </c>
       <c r="J342" t="s">
         <v>2134</v>
@@ -20482,7 +20482,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B343" t="s">
         <v>382</v>
@@ -20503,7 +20503,7 @@
         <v>1634</v>
       </c>
       <c r="I343" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J343" t="s">
         <v>2135</v>
@@ -20576,7 +20576,7 @@
         <v>1580</v>
       </c>
       <c r="I345" t="s">
-        <v>1768</v>
+        <v>1767</v>
       </c>
       <c r="J345" t="s">
         <v>2137</v>
@@ -20590,7 +20590,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B346" t="s">
         <v>385</v>
@@ -20611,7 +20611,7 @@
         <v>1634</v>
       </c>
       <c r="I346" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J346" t="s">
         <v>2138</v>
@@ -20660,7 +20660,7 @@
     </row>
     <row r="348" spans="1:12">
       <c r="A348" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B348" t="s">
         <v>387</v>
@@ -20681,7 +20681,7 @@
         <v>1634</v>
       </c>
       <c r="I348" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J348" t="s">
         <v>2140</v>
@@ -20695,7 +20695,7 @@
     </row>
     <row r="349" spans="1:12">
       <c r="A349" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B349" t="s">
         <v>388</v>
@@ -20716,7 +20716,7 @@
         <v>1634</v>
       </c>
       <c r="I349" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J349" t="s">
         <v>2141</v>
@@ -20751,7 +20751,7 @@
         <v>1634</v>
       </c>
       <c r="I350" t="s">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="J350" t="s">
         <v>2142</v>
@@ -20891,7 +20891,7 @@
         <v>1634</v>
       </c>
       <c r="I354" t="s">
-        <v>1770</v>
+        <v>1769</v>
       </c>
       <c r="J354" t="s">
         <v>2146</v>
@@ -20961,7 +20961,7 @@
         <v>1634</v>
       </c>
       <c r="I356" t="s">
-        <v>1771</v>
+        <v>1770</v>
       </c>
       <c r="J356" t="s">
         <v>2148</v>
@@ -21031,7 +21031,7 @@
         <v>1634</v>
       </c>
       <c r="I358" t="s">
-        <v>1772</v>
+        <v>1706</v>
       </c>
       <c r="J358" t="s">
         <v>2150</v>
@@ -21150,7 +21150,7 @@
     </row>
     <row r="362" spans="1:12">
       <c r="A362" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B362" t="s">
         <v>401</v>
@@ -21171,7 +21171,7 @@
         <v>1634</v>
       </c>
       <c r="I362" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J362" t="s">
         <v>2154</v>
@@ -21220,7 +21220,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B364" t="s">
         <v>403</v>
@@ -21381,7 +21381,7 @@
         <v>1634</v>
       </c>
       <c r="I368" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="J368" t="s">
         <v>2160</v>
@@ -21451,7 +21451,7 @@
         <v>1634</v>
       </c>
       <c r="I370" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J370" t="s">
         <v>2162</v>
@@ -21465,7 +21465,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B371" t="s">
         <v>410</v>
@@ -21486,7 +21486,7 @@
         <v>1634</v>
       </c>
       <c r="I371" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J371" t="s">
         <v>2163</v>
@@ -21605,7 +21605,7 @@
     </row>
     <row r="375" spans="1:12">
       <c r="A375" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B375" t="s">
         <v>414</v>
@@ -21850,7 +21850,7 @@
     </row>
     <row r="382" spans="1:12">
       <c r="A382" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B382" t="s">
         <v>421</v>
@@ -21871,7 +21871,7 @@
         <v>1634</v>
       </c>
       <c r="I382" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J382" t="s">
         <v>2173</v>
@@ -21955,7 +21955,7 @@
     </row>
     <row r="385" spans="1:12">
       <c r="A385" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B385" t="s">
         <v>424</v>
@@ -21976,7 +21976,7 @@
         <v>1634</v>
       </c>
       <c r="I385" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J385" t="s">
         <v>2176</v>
@@ -22025,7 +22025,7 @@
     </row>
     <row r="387" spans="1:12">
       <c r="A387" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B387" t="s">
         <v>426</v>
@@ -22046,7 +22046,7 @@
         <v>1634</v>
       </c>
       <c r="I387" t="s">
-        <v>1757</v>
+        <v>1771</v>
       </c>
       <c r="J387" t="s">
         <v>2178</v>
@@ -22095,7 +22095,7 @@
     </row>
     <row r="389" spans="1:12">
       <c r="A389" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B389" t="s">
         <v>428</v>
@@ -22130,7 +22130,7 @@
     </row>
     <row r="390" spans="1:12">
       <c r="A390" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B390" t="s">
         <v>429</v>
@@ -22165,7 +22165,7 @@
     </row>
     <row r="391" spans="1:12">
       <c r="A391" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B391" t="s">
         <v>430</v>
@@ -22186,7 +22186,7 @@
         <v>1634</v>
       </c>
       <c r="I391" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J391" t="s">
         <v>2181</v>
@@ -22200,7 +22200,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B392" t="s">
         <v>431</v>
@@ -22221,7 +22221,7 @@
         <v>1634</v>
       </c>
       <c r="I392" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J392" t="s">
         <v>2182</v>
@@ -22235,7 +22235,7 @@
     </row>
     <row r="393" spans="1:12">
       <c r="A393" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B393" t="s">
         <v>432</v>
@@ -22256,7 +22256,7 @@
         <v>1634</v>
       </c>
       <c r="I393" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J393" t="s">
         <v>2183</v>
@@ -22326,7 +22326,7 @@
         <v>1634</v>
       </c>
       <c r="I395" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
       <c r="J395" t="s">
         <v>2185</v>
@@ -22340,7 +22340,7 @@
     </row>
     <row r="396" spans="1:12">
       <c r="A396" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B396" t="s">
         <v>435</v>
@@ -22361,7 +22361,7 @@
         <v>1634</v>
       </c>
       <c r="I396" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J396" t="s">
         <v>2186</v>
@@ -22431,7 +22431,7 @@
         <v>1634</v>
       </c>
       <c r="I398" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="J398" t="s">
         <v>2188</v>
@@ -22445,7 +22445,7 @@
     </row>
     <row r="399" spans="1:12">
       <c r="A399" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B399" t="s">
         <v>438</v>
@@ -22466,7 +22466,7 @@
         <v>1634</v>
       </c>
       <c r="I399" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J399" t="s">
         <v>2189</v>
@@ -22480,7 +22480,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B400" t="s">
         <v>439</v>
@@ -22501,7 +22501,7 @@
         <v>1634</v>
       </c>
       <c r="I400" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J400" t="s">
         <v>2190</v>
@@ -22585,7 +22585,7 @@
     </row>
     <row r="403" spans="1:12">
       <c r="A403" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B403" t="s">
         <v>442</v>
@@ -22606,7 +22606,7 @@
         <v>1634</v>
       </c>
       <c r="I403" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J403" t="s">
         <v>2193</v>
@@ -22690,7 +22690,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B406" t="s">
         <v>445</v>
@@ -22711,7 +22711,7 @@
         <v>1634</v>
       </c>
       <c r="I406" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J406" t="s">
         <v>2196</v>
@@ -22760,7 +22760,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B408" t="s">
         <v>447</v>
@@ -22781,7 +22781,7 @@
         <v>1634</v>
       </c>
       <c r="I408" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J408" t="s">
         <v>2198</v>
@@ -22795,7 +22795,7 @@
     </row>
     <row r="409" spans="1:12">
       <c r="A409" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B409" t="s">
         <v>448</v>
@@ -22816,7 +22816,7 @@
         <v>1634</v>
       </c>
       <c r="I409" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J409" t="s">
         <v>2199</v>
@@ -22830,7 +22830,7 @@
     </row>
     <row r="410" spans="1:12">
       <c r="A410" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B410" t="s">
         <v>449</v>
@@ -22851,7 +22851,7 @@
         <v>1634</v>
       </c>
       <c r="I410" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J410" t="s">
         <v>2200</v>
@@ -22900,7 +22900,7 @@
     </row>
     <row r="412" spans="1:12">
       <c r="A412" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B412" t="s">
         <v>451</v>
@@ -22921,7 +22921,7 @@
         <v>1634</v>
       </c>
       <c r="I412" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J412" t="s">
         <v>2202</v>
@@ -22970,7 +22970,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B414" t="s">
         <v>453</v>
@@ -22991,7 +22991,7 @@
         <v>1634</v>
       </c>
       <c r="I414" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J414" t="s">
         <v>2204</v>
@@ -23005,7 +23005,7 @@
     </row>
     <row r="415" spans="1:12">
       <c r="A415" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B415" t="s">
         <v>454</v>
@@ -23026,7 +23026,7 @@
         <v>1634</v>
       </c>
       <c r="I415" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J415" t="s">
         <v>2205</v>
@@ -23040,7 +23040,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B416" t="s">
         <v>455</v>
@@ -23061,7 +23061,7 @@
         <v>1634</v>
       </c>
       <c r="I416" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J416" t="s">
         <v>2206</v>
@@ -23110,7 +23110,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B418" t="s">
         <v>457</v>
@@ -23131,7 +23131,7 @@
         <v>1634</v>
       </c>
       <c r="I418" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J418" t="s">
         <v>2208</v>
@@ -23253,7 +23253,7 @@
     </row>
     <row r="422" spans="1:12">
       <c r="A422" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B422" t="s">
         <v>461</v>
@@ -23274,7 +23274,7 @@
         <v>1634</v>
       </c>
       <c r="I422" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J422" t="s">
         <v>2212</v>
@@ -23358,7 +23358,7 @@
     </row>
     <row r="425" spans="1:12">
       <c r="A425" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B425" t="s">
         <v>464</v>
@@ -23379,7 +23379,7 @@
         <v>1634</v>
       </c>
       <c r="I425" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J425" t="s">
         <v>2215</v>
@@ -23393,7 +23393,7 @@
     </row>
     <row r="426" spans="1:12">
       <c r="A426" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B426" t="s">
         <v>465</v>
@@ -23414,7 +23414,7 @@
         <v>1634</v>
       </c>
       <c r="I426" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J426" t="s">
         <v>2216</v>
@@ -23533,7 +23533,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B430" t="s">
         <v>469</v>
@@ -23554,7 +23554,7 @@
         <v>1634</v>
       </c>
       <c r="I430" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J430" t="s">
         <v>2220</v>
@@ -23603,7 +23603,7 @@
     </row>
     <row r="432" spans="1:12">
       <c r="A432" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B432" t="s">
         <v>471</v>
@@ -23624,7 +23624,7 @@
         <v>1634</v>
       </c>
       <c r="I432" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J432" t="s">
         <v>2222</v>
@@ -23708,7 +23708,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B435" t="s">
         <v>473</v>
@@ -23729,7 +23729,7 @@
         <v>1634</v>
       </c>
       <c r="I435" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J435" t="s">
         <v>2224</v>
@@ -23778,7 +23778,7 @@
     </row>
     <row r="437" spans="1:12">
       <c r="A437" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B437" t="s">
         <v>475</v>
@@ -23799,7 +23799,7 @@
         <v>1634</v>
       </c>
       <c r="I437" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J437" t="s">
         <v>2226</v>
@@ -23848,7 +23848,7 @@
     </row>
     <row r="439" spans="1:12">
       <c r="A439" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B439" t="s">
         <v>477</v>
@@ -23953,7 +23953,7 @@
     </row>
     <row r="442" spans="1:12">
       <c r="A442" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B442" t="s">
         <v>480</v>
@@ -23974,7 +23974,7 @@
         <v>1634</v>
       </c>
       <c r="I442" t="s">
-        <v>1757</v>
+        <v>1673</v>
       </c>
       <c r="J442" t="s">
         <v>2231</v>
@@ -24023,7 +24023,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B444" t="s">
         <v>482</v>
@@ -24044,7 +24044,7 @@
         <v>1634</v>
       </c>
       <c r="I444" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J444" t="s">
         <v>2233</v>
@@ -24058,7 +24058,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B445" t="s">
         <v>483</v>
@@ -24163,7 +24163,7 @@
     </row>
     <row r="448" spans="1:12">
       <c r="A448" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B448" t="s">
         <v>486</v>
@@ -24184,7 +24184,7 @@
         <v>1634</v>
       </c>
       <c r="I448" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J448" t="s">
         <v>2237</v>
@@ -24198,7 +24198,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B449" t="s">
         <v>487</v>
@@ -24219,7 +24219,7 @@
         <v>1634</v>
       </c>
       <c r="I449" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J449" t="s">
         <v>2238</v>
@@ -24303,7 +24303,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B452" t="s">
         <v>490</v>
@@ -24324,7 +24324,7 @@
         <v>1634</v>
       </c>
       <c r="I452" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J452" t="s">
         <v>2241</v>
@@ -24443,7 +24443,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B456" t="s">
         <v>494</v>
@@ -24464,7 +24464,7 @@
         <v>1634</v>
       </c>
       <c r="I456" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J456" t="s">
         <v>2245</v>
@@ -24478,7 +24478,7 @@
     </row>
     <row r="457" spans="1:12">
       <c r="A457" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B457" t="s">
         <v>495</v>
@@ -24499,7 +24499,7 @@
         <v>1634</v>
       </c>
       <c r="I457" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J457" t="s">
         <v>2246</v>
@@ -24513,7 +24513,7 @@
     </row>
     <row r="458" spans="1:12">
       <c r="A458" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B458" t="s">
         <v>496</v>
@@ -24534,7 +24534,7 @@
         <v>1634</v>
       </c>
       <c r="I458" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J458" t="s">
         <v>2247</v>
@@ -24688,7 +24688,7 @@
     </row>
     <row r="463" spans="1:12">
       <c r="A463" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B463" t="s">
         <v>501</v>
@@ -24709,7 +24709,7 @@
         <v>1634</v>
       </c>
       <c r="I463" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J463" t="s">
         <v>2252</v>
@@ -24723,7 +24723,7 @@
     </row>
     <row r="464" spans="1:12">
       <c r="A464" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B464" t="s">
         <v>502</v>
@@ -24744,7 +24744,7 @@
         <v>1634</v>
       </c>
       <c r="I464" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J464" t="s">
         <v>2253</v>
@@ -24758,7 +24758,7 @@
     </row>
     <row r="465" spans="1:12">
       <c r="A465" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B465" t="s">
         <v>503</v>
@@ -24782,7 +24782,7 @@
         <v>1648</v>
       </c>
       <c r="I465" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J465" t="s">
         <v>2254</v>
@@ -24796,7 +24796,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B466" t="s">
         <v>504</v>
@@ -24817,7 +24817,7 @@
         <v>1634</v>
       </c>
       <c r="I466" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J466" t="s">
         <v>2255</v>
@@ -24831,7 +24831,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B467" t="s">
         <v>505</v>
@@ -24852,7 +24852,7 @@
         <v>1634</v>
       </c>
       <c r="I467" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J467" t="s">
         <v>2256</v>
@@ -25076,7 +25076,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B474" t="s">
         <v>512</v>
@@ -25097,7 +25097,7 @@
         <v>1634</v>
       </c>
       <c r="I474" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J474" t="s">
         <v>2263</v>
@@ -25146,7 +25146,7 @@
     </row>
     <row r="476" spans="1:12">
       <c r="A476" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B476" t="s">
         <v>514</v>
@@ -25167,7 +25167,7 @@
         <v>1634</v>
       </c>
       <c r="I476" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J476" t="s">
         <v>2265</v>
@@ -25181,7 +25181,7 @@
     </row>
     <row r="477" spans="1:12">
       <c r="A477" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B477" t="s">
         <v>515</v>
@@ -25202,7 +25202,7 @@
         <v>1634</v>
       </c>
       <c r="I477" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J477" t="s">
         <v>2266</v>
@@ -25251,7 +25251,7 @@
     </row>
     <row r="479" spans="1:12">
       <c r="A479" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B479" t="s">
         <v>517</v>
@@ -25272,7 +25272,7 @@
         <v>1634</v>
       </c>
       <c r="I479" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J479" t="s">
         <v>2268</v>
@@ -25286,7 +25286,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B480" t="s">
         <v>518</v>
@@ -25307,7 +25307,7 @@
         <v>1634</v>
       </c>
       <c r="I480" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J480" t="s">
         <v>2269</v>
@@ -25461,7 +25461,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B485" t="s">
         <v>523</v>
@@ -25482,7 +25482,7 @@
         <v>1634</v>
       </c>
       <c r="I485" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J485" t="s">
         <v>2274</v>
@@ -25566,7 +25566,7 @@
     </row>
     <row r="488" spans="1:12">
       <c r="A488" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B488" t="s">
         <v>526</v>
@@ -25587,7 +25587,7 @@
         <v>1634</v>
       </c>
       <c r="I488" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J488" t="s">
         <v>2277</v>
@@ -25636,7 +25636,7 @@
     </row>
     <row r="490" spans="1:12">
       <c r="A490" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B490" t="s">
         <v>528</v>
@@ -25657,7 +25657,7 @@
         <v>1634</v>
       </c>
       <c r="I490" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J490" t="s">
         <v>2279</v>
@@ -25706,7 +25706,7 @@
     </row>
     <row r="492" spans="1:12">
       <c r="A492" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B492" t="s">
         <v>530</v>
@@ -25727,7 +25727,7 @@
         <v>1634</v>
       </c>
       <c r="I492" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J492" t="s">
         <v>2281</v>
@@ -25797,7 +25797,7 @@
         <v>1634</v>
       </c>
       <c r="I494" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J494" t="s">
         <v>2283</v>
@@ -25846,7 +25846,7 @@
     </row>
     <row r="496" spans="1:12">
       <c r="A496" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B496" t="s">
         <v>534</v>
@@ -25867,7 +25867,7 @@
         <v>1634</v>
       </c>
       <c r="I496" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J496" t="s">
         <v>2285</v>
@@ -25916,7 +25916,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B498" t="s">
         <v>536</v>
@@ -25937,7 +25937,7 @@
         <v>1634</v>
       </c>
       <c r="I498" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J498" t="s">
         <v>2287</v>
@@ -26056,7 +26056,7 @@
     </row>
     <row r="502" spans="1:12">
       <c r="A502" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B502" t="s">
         <v>540</v>
@@ -26234,7 +26234,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B507" t="s">
         <v>545</v>
@@ -26255,7 +26255,7 @@
         <v>1634</v>
       </c>
       <c r="I507" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J507" t="s">
         <v>2296</v>
@@ -26269,7 +26269,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B508" t="s">
         <v>546</v>
@@ -26290,7 +26290,7 @@
         <v>1634</v>
       </c>
       <c r="I508" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J508" t="s">
         <v>2297</v>
@@ -26339,7 +26339,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B510" t="s">
         <v>548</v>
@@ -26360,7 +26360,7 @@
         <v>1634</v>
       </c>
       <c r="I510" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J510" t="s">
         <v>2299</v>
@@ -26409,7 +26409,7 @@
     </row>
     <row r="512" spans="1:12">
       <c r="A512" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B512" t="s">
         <v>550</v>
@@ -26430,7 +26430,7 @@
         <v>1634</v>
       </c>
       <c r="I512" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J512" t="s">
         <v>2301</v>
@@ -26549,7 +26549,7 @@
     </row>
     <row r="516" spans="1:12">
       <c r="A516" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B516" t="s">
         <v>554</v>
@@ -26570,7 +26570,7 @@
         <v>1634</v>
       </c>
       <c r="I516" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J516" t="s">
         <v>2305</v>
@@ -26689,7 +26689,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B520" t="s">
         <v>558</v>
@@ -26713,7 +26713,7 @@
         <v>1650</v>
       </c>
       <c r="I520" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J520" t="s">
         <v>2309</v>
@@ -26727,7 +26727,7 @@
     </row>
     <row r="521" spans="1:12">
       <c r="A521" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B521" t="s">
         <v>559</v>
@@ -26748,7 +26748,7 @@
         <v>1634</v>
       </c>
       <c r="I521" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J521" t="s">
         <v>2310</v>
@@ -26832,7 +26832,7 @@
     </row>
     <row r="524" spans="1:12">
       <c r="A524" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B524" t="s">
         <v>562</v>
@@ -26853,7 +26853,7 @@
         <v>1634</v>
       </c>
       <c r="I524" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J524" t="s">
         <v>2313</v>
@@ -26867,7 +26867,7 @@
     </row>
     <row r="525" spans="1:12">
       <c r="A525" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B525" t="s">
         <v>563</v>
@@ -26888,7 +26888,7 @@
         <v>1634</v>
       </c>
       <c r="I525" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J525" t="s">
         <v>2314</v>
@@ -26972,7 +26972,7 @@
     </row>
     <row r="528" spans="1:12">
       <c r="A528" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B528" t="s">
         <v>566</v>
@@ -27147,7 +27147,7 @@
     </row>
     <row r="533" spans="1:12">
       <c r="A533" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B533" t="s">
         <v>571</v>
@@ -27168,7 +27168,7 @@
         <v>1634</v>
       </c>
       <c r="I533" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J533" t="s">
         <v>2322</v>
@@ -27182,7 +27182,7 @@
     </row>
     <row r="534" spans="1:12">
       <c r="A534" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B534" t="s">
         <v>572</v>
@@ -27203,7 +27203,7 @@
         <v>1634</v>
       </c>
       <c r="I534" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J534" t="s">
         <v>2323</v>
@@ -27252,7 +27252,7 @@
     </row>
     <row r="536" spans="1:12">
       <c r="A536" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B536" t="s">
         <v>574</v>
@@ -27273,7 +27273,7 @@
         <v>1634</v>
       </c>
       <c r="I536" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J536" t="s">
         <v>2325</v>
@@ -27287,7 +27287,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B537" t="s">
         <v>575</v>
@@ -27308,7 +27308,7 @@
         <v>1634</v>
       </c>
       <c r="I537" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J537" t="s">
         <v>2326</v>
@@ -27343,7 +27343,7 @@
         <v>1634</v>
       </c>
       <c r="I538" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J538" t="s">
         <v>2327</v>
@@ -27392,7 +27392,7 @@
     </row>
     <row r="540" spans="1:12">
       <c r="A540" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B540" t="s">
         <v>578</v>
@@ -27413,7 +27413,7 @@
         <v>1634</v>
       </c>
       <c r="I540" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J540" t="s">
         <v>2329</v>
@@ -27448,7 +27448,7 @@
         <v>1634</v>
       </c>
       <c r="I541" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J541" t="s">
         <v>2330</v>
@@ -27462,7 +27462,7 @@
     </row>
     <row r="542" spans="1:12">
       <c r="A542" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B542" t="s">
         <v>580</v>
@@ -27483,7 +27483,7 @@
         <v>1634</v>
       </c>
       <c r="I542" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J542" t="s">
         <v>2331</v>
@@ -27497,7 +27497,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B543" t="s">
         <v>581</v>
@@ -27518,7 +27518,7 @@
         <v>1634</v>
       </c>
       <c r="I543" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J543" t="s">
         <v>2332</v>
@@ -27532,7 +27532,7 @@
     </row>
     <row r="544" spans="1:12">
       <c r="A544" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B544" t="s">
         <v>582</v>
@@ -27553,7 +27553,7 @@
         <v>1634</v>
       </c>
       <c r="I544" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J544" t="s">
         <v>2333</v>
@@ -27602,7 +27602,7 @@
     </row>
     <row r="546" spans="1:12">
       <c r="A546" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B546" t="s">
         <v>584</v>
@@ -27623,7 +27623,7 @@
         <v>1634</v>
       </c>
       <c r="I546" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J546" t="s">
         <v>2335</v>
@@ -27637,7 +27637,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B547" t="s">
         <v>585</v>
@@ -27696,7 +27696,7 @@
         <v>1651</v>
       </c>
       <c r="I548" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J548" t="s">
         <v>2337</v>
@@ -27745,7 +27745,7 @@
     </row>
     <row r="550" spans="1:12">
       <c r="A550" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B550" t="s">
         <v>588</v>
@@ -27766,7 +27766,7 @@
         <v>1634</v>
       </c>
       <c r="I550" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J550" t="s">
         <v>2339</v>
@@ -27815,7 +27815,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B552" t="s">
         <v>590</v>
@@ -27836,7 +27836,7 @@
         <v>1634</v>
       </c>
       <c r="I552" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J552" t="s">
         <v>2341</v>
@@ -27850,7 +27850,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B553" t="s">
         <v>591</v>
@@ -27871,7 +27871,7 @@
         <v>1634</v>
       </c>
       <c r="I553" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J553" t="s">
         <v>2342</v>
@@ -27885,7 +27885,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B554" t="s">
         <v>592</v>
@@ -27909,7 +27909,7 @@
         <v>1652</v>
       </c>
       <c r="I554" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J554" t="s">
         <v>2343</v>
@@ -27923,7 +27923,7 @@
     </row>
     <row r="555" spans="1:12">
       <c r="A555" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B555" t="s">
         <v>593</v>
@@ -27944,7 +27944,7 @@
         <v>1634</v>
       </c>
       <c r="I555" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J555" t="s">
         <v>2344</v>
@@ -27958,7 +27958,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B556" t="s">
         <v>594</v>
@@ -27979,7 +27979,7 @@
         <v>1634</v>
       </c>
       <c r="I556" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J556" t="s">
         <v>2345</v>
@@ -27993,7 +27993,7 @@
     </row>
     <row r="557" spans="1:12">
       <c r="A557" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B557" t="s">
         <v>595</v>
@@ -28014,7 +28014,7 @@
         <v>1634</v>
       </c>
       <c r="I557" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J557" t="s">
         <v>2346</v>
@@ -28028,7 +28028,7 @@
     </row>
     <row r="558" spans="1:12">
       <c r="A558" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B558" t="s">
         <v>596</v>
@@ -28049,7 +28049,7 @@
         <v>1634</v>
       </c>
       <c r="I558" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J558" t="s">
         <v>2347</v>
@@ -28063,7 +28063,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B559" t="s">
         <v>597</v>
@@ -28084,7 +28084,7 @@
         <v>1634</v>
       </c>
       <c r="I559" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J559" t="s">
         <v>2348</v>
@@ -28098,7 +28098,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B560" t="s">
         <v>598</v>
@@ -28119,7 +28119,7 @@
         <v>1634</v>
       </c>
       <c r="I560" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J560" t="s">
         <v>2349</v>
@@ -28133,7 +28133,7 @@
     </row>
     <row r="561" spans="1:12">
       <c r="A561" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B561" t="s">
         <v>599</v>
@@ -28154,7 +28154,7 @@
         <v>1634</v>
       </c>
       <c r="I561" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J561" t="s">
         <v>2350</v>
@@ -28203,7 +28203,7 @@
     </row>
     <row r="563" spans="1:12">
       <c r="A563" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B563" t="s">
         <v>601</v>
@@ -28238,7 +28238,7 @@
     </row>
     <row r="564" spans="1:12">
       <c r="A564" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B564" t="s">
         <v>602</v>
@@ -28259,7 +28259,7 @@
         <v>1634</v>
       </c>
       <c r="I564" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J564" t="s">
         <v>2353</v>
@@ -28294,7 +28294,7 @@
         <v>1634</v>
       </c>
       <c r="I565" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J565" t="s">
         <v>2354</v>
@@ -28332,7 +28332,7 @@
         <v>1622</v>
       </c>
       <c r="I566" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="J566" t="s">
         <v>2355</v>
@@ -28416,7 +28416,7 @@
     </row>
     <row r="569" spans="1:12">
       <c r="A569" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B569" t="s">
         <v>607</v>
@@ -28437,7 +28437,7 @@
         <v>1634</v>
       </c>
       <c r="I569" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J569" t="s">
         <v>2358</v>
@@ -28486,7 +28486,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B571" t="s">
         <v>609</v>
@@ -28521,7 +28521,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B572" t="s">
         <v>610</v>
@@ -28542,7 +28542,7 @@
         <v>1634</v>
       </c>
       <c r="I572" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J572" t="s">
         <v>2361</v>
@@ -28556,7 +28556,7 @@
     </row>
     <row r="573" spans="1:12">
       <c r="A573" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B573" t="s">
         <v>611</v>
@@ -28577,7 +28577,7 @@
         <v>1634</v>
       </c>
       <c r="I573" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J573" t="s">
         <v>2362</v>
@@ -28591,7 +28591,7 @@
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B574" t="s">
         <v>612</v>
@@ -28612,7 +28612,7 @@
         <v>1634</v>
       </c>
       <c r="I574" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J574" t="s">
         <v>2363</v>
@@ -28626,7 +28626,7 @@
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B575" t="s">
         <v>613</v>
@@ -28647,7 +28647,7 @@
         <v>1634</v>
       </c>
       <c r="I575" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J575" t="s">
         <v>2364</v>
@@ -28874,7 +28874,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B582" t="s">
         <v>620</v>
@@ -28895,7 +28895,7 @@
         <v>1634</v>
       </c>
       <c r="I582" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J582" t="s">
         <v>2371</v>
@@ -29003,7 +29003,7 @@
         <v>1653</v>
       </c>
       <c r="I585" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="J585" t="s">
         <v>2374</v>
@@ -29052,7 +29052,7 @@
     </row>
     <row r="587" spans="1:12">
       <c r="A587" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B587" t="s">
         <v>625</v>
@@ -29087,7 +29087,7 @@
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B588" t="s">
         <v>626</v>
@@ -29108,7 +29108,7 @@
         <v>1634</v>
       </c>
       <c r="I588" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J588" t="s">
         <v>2377</v>
@@ -29160,7 +29160,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B590" t="s">
         <v>628</v>
@@ -29181,7 +29181,7 @@
         <v>1634</v>
       </c>
       <c r="I590" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J590" t="s">
         <v>2379</v>
@@ -29230,7 +29230,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B592" t="s">
         <v>630</v>
@@ -29265,7 +29265,7 @@
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B593" t="s">
         <v>631</v>
@@ -29286,7 +29286,7 @@
         <v>1634</v>
       </c>
       <c r="I593" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J593" t="s">
         <v>2382</v>
@@ -29338,7 +29338,7 @@
     </row>
     <row r="595" spans="1:12">
       <c r="A595" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B595" t="s">
         <v>633</v>
@@ -29359,7 +29359,7 @@
         <v>1634</v>
       </c>
       <c r="I595" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J595" t="s">
         <v>2384</v>
@@ -29408,7 +29408,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B597" t="s">
         <v>635</v>
@@ -29429,7 +29429,7 @@
         <v>1634</v>
       </c>
       <c r="I597" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J597" t="s">
         <v>2386</v>
@@ -29478,7 +29478,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B599" t="s">
         <v>637</v>
@@ -29499,7 +29499,7 @@
         <v>1634</v>
       </c>
       <c r="I599" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J599" t="s">
         <v>2388</v>
@@ -29513,7 +29513,7 @@
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B600" t="s">
         <v>638</v>
@@ -29537,7 +29537,7 @@
         <v>1656</v>
       </c>
       <c r="I600" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J600" t="s">
         <v>2389</v>
@@ -29551,7 +29551,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -29586,7 +29586,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B602" t="s">
         <v>640</v>
@@ -29607,7 +29607,7 @@
         <v>1634</v>
       </c>
       <c r="I602" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J602" t="s">
         <v>2391</v>
@@ -29621,7 +29621,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B603" t="s">
         <v>641</v>
@@ -29642,7 +29642,7 @@
         <v>1634</v>
       </c>
       <c r="I603" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J603" t="s">
         <v>2392</v>
@@ -29656,7 +29656,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B604" t="s">
         <v>642</v>
@@ -29677,7 +29677,7 @@
         <v>1634</v>
       </c>
       <c r="I604" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J604" t="s">
         <v>2393</v>
@@ -29764,7 +29764,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B607" t="s">
         <v>645</v>
@@ -29785,7 +29785,7 @@
         <v>1634</v>
       </c>
       <c r="I607" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J607" t="s">
         <v>2396</v>
@@ -30024,7 +30024,7 @@
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B614" t="s">
         <v>652</v>
@@ -30059,7 +30059,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B615" t="s">
         <v>653</v>
@@ -30080,7 +30080,7 @@
         <v>1634</v>
       </c>
       <c r="I615" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J615" t="s">
         <v>2404</v>
@@ -30094,7 +30094,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B616" t="s">
         <v>654</v>
@@ -30115,7 +30115,7 @@
         <v>1634</v>
       </c>
       <c r="I616" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J616" t="s">
         <v>2405</v>
@@ -30307,7 +30307,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B622" t="s">
         <v>660</v>
@@ -30328,7 +30328,7 @@
         <v>1634</v>
       </c>
       <c r="I622" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J622" t="s">
         <v>2411</v>
@@ -30342,7 +30342,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B623" t="s">
         <v>661</v>
@@ -30363,7 +30363,7 @@
         <v>1634</v>
       </c>
       <c r="I623" t="s">
-        <v>1757</v>
+        <v>1771</v>
       </c>
       <c r="J623" t="s">
         <v>2412</v>
@@ -30377,7 +30377,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B624" t="s">
         <v>662</v>
@@ -30398,7 +30398,7 @@
         <v>1634</v>
       </c>
       <c r="I624" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J624" t="s">
         <v>2413</v>
@@ -30447,7 +30447,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B626" t="s">
         <v>664</v>
@@ -30468,7 +30468,7 @@
         <v>1634</v>
       </c>
       <c r="I626" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J626" t="s">
         <v>2415</v>
@@ -30482,7 +30482,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B627" t="s">
         <v>665</v>
@@ -30503,7 +30503,7 @@
         <v>1634</v>
       </c>
       <c r="I627" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J627" t="s">
         <v>2416</v>
@@ -30517,7 +30517,7 @@
     </row>
     <row r="628" spans="1:12">
       <c r="A628" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B628" t="s">
         <v>666</v>
@@ -30538,7 +30538,7 @@
         <v>1634</v>
       </c>
       <c r="I628" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J628" t="s">
         <v>2417</v>
@@ -30552,7 +30552,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B629" t="s">
         <v>667</v>
@@ -30573,7 +30573,7 @@
         <v>1634</v>
       </c>
       <c r="I629" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J629" t="s">
         <v>2418</v>
@@ -30587,7 +30587,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B630" t="s">
         <v>668</v>
@@ -30695,7 +30695,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B633" t="s">
         <v>671</v>
@@ -30716,7 +30716,7 @@
         <v>1634</v>
       </c>
       <c r="I633" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J633" t="s">
         <v>2422</v>
@@ -30730,7 +30730,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B634" t="s">
         <v>672</v>
@@ -30841,7 +30841,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B637" t="s">
         <v>675</v>
@@ -30862,7 +30862,7 @@
         <v>1634</v>
       </c>
       <c r="I637" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J637" t="s">
         <v>2426</v>
@@ -30952,7 +30952,7 @@
     </row>
     <row r="640" spans="1:12">
       <c r="A640" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B640" t="s">
         <v>678</v>
@@ -30973,7 +30973,7 @@
         <v>1634</v>
       </c>
       <c r="I640" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J640" t="s">
         <v>2429</v>
@@ -31025,7 +31025,7 @@
     </row>
     <row r="642" spans="1:12">
       <c r="A642" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B642" t="s">
         <v>680</v>
@@ -31046,7 +31046,7 @@
         <v>1634</v>
       </c>
       <c r="I642" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J642" t="s">
         <v>2431</v>
@@ -31060,7 +31060,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B643" t="s">
         <v>681</v>
@@ -31081,7 +31081,7 @@
         <v>1634</v>
       </c>
       <c r="I643" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J643" t="s">
         <v>2432</v>
@@ -31095,7 +31095,7 @@
     </row>
     <row r="644" spans="1:12">
       <c r="A644" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B644" t="s">
         <v>682</v>
@@ -31119,7 +31119,7 @@
         <v>1622</v>
       </c>
       <c r="I644" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J644" t="s">
         <v>2433</v>
@@ -31133,7 +31133,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B645" t="s">
         <v>683</v>
@@ -31154,7 +31154,7 @@
         <v>1634</v>
       </c>
       <c r="I645" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J645" t="s">
         <v>2434</v>
@@ -31168,7 +31168,7 @@
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B646" t="s">
         <v>684</v>
@@ -31189,7 +31189,7 @@
         <v>1634</v>
       </c>
       <c r="I646" t="s">
-        <v>1705</v>
+        <v>1736</v>
       </c>
       <c r="J646" t="s">
         <v>2435</v>
@@ -31203,7 +31203,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B647" t="s">
         <v>685</v>
@@ -31224,7 +31224,7 @@
         <v>1634</v>
       </c>
       <c r="I647" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J647" t="s">
         <v>2436</v>
@@ -31238,7 +31238,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B648" t="s">
         <v>686</v>
@@ -31259,7 +31259,7 @@
         <v>1634</v>
       </c>
       <c r="I648" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J648" t="s">
         <v>2437</v>
@@ -31273,7 +31273,7 @@
     </row>
     <row r="649" spans="1:12">
       <c r="A649" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B649" t="s">
         <v>687</v>
@@ -31294,7 +31294,7 @@
         <v>1634</v>
       </c>
       <c r="I649" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J649" t="s">
         <v>2438</v>
@@ -31308,7 +31308,7 @@
     </row>
     <row r="650" spans="1:12">
       <c r="A650" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B650" t="s">
         <v>688</v>
@@ -31329,7 +31329,7 @@
         <v>1634</v>
       </c>
       <c r="I650" t="s">
-        <v>1705</v>
+        <v>1673</v>
       </c>
       <c r="J650" t="s">
         <v>2439</v>
@@ -31378,7 +31378,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B652" t="s">
         <v>690</v>
@@ -31402,7 +31402,7 @@
         <v>1664</v>
       </c>
       <c r="I652" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J652" t="s">
         <v>2441</v>
@@ -31416,7 +31416,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B653" t="s">
         <v>691</v>
@@ -31437,7 +31437,7 @@
         <v>1634</v>
       </c>
       <c r="I653" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J653" t="s">
         <v>2442</v>
@@ -31451,7 +31451,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B654" t="s">
         <v>692</v>
@@ -31472,7 +31472,7 @@
         <v>1634</v>
       </c>
       <c r="I654" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J654" t="s">
         <v>2443</v>
@@ -31486,7 +31486,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B655" t="s">
         <v>693</v>
@@ -31507,7 +31507,7 @@
         <v>1634</v>
       </c>
       <c r="I655" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J655" t="s">
         <v>2444</v>
@@ -31580,7 +31580,7 @@
         <v>1665</v>
       </c>
       <c r="I657" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J657" t="s">
         <v>2446</v>
@@ -31632,7 +31632,7 @@
     </row>
     <row r="659" spans="1:12">
       <c r="A659" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B659" t="s">
         <v>696</v>
@@ -31656,7 +31656,7 @@
         <v>1654</v>
       </c>
       <c r="I659" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="J659" t="s">
         <v>2447</v>
@@ -31784,7 +31784,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B663" t="s">
         <v>700</v>
@@ -31805,7 +31805,7 @@
         <v>1634</v>
       </c>
       <c r="I663" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J663" t="s">
         <v>1812</v>
@@ -31819,7 +31819,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B664" t="s">
         <v>701</v>
@@ -31840,7 +31840,7 @@
         <v>1634</v>
       </c>
       <c r="I664" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J664" t="s">
         <v>2451</v>
@@ -31892,7 +31892,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B666" t="s">
         <v>703</v>
@@ -31913,7 +31913,7 @@
         <v>1634</v>
       </c>
       <c r="I666" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J666" t="s">
         <v>2453</v>
@@ -31927,7 +31927,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B667" t="s">
         <v>704</v>
@@ -31962,7 +31962,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B668" t="s">
         <v>705</v>
@@ -31983,7 +31983,7 @@
         <v>1634</v>
       </c>
       <c r="I668" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J668" t="s">
         <v>2455</v>
@@ -31997,7 +31997,7 @@
     </row>
     <row r="669" spans="1:12">
       <c r="A669" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B669" t="s">
         <v>706</v>
@@ -32018,7 +32018,7 @@
         <v>1634</v>
       </c>
       <c r="I669" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J669" t="s">
         <v>2456</v>
@@ -32032,7 +32032,7 @@
     </row>
     <row r="670" spans="1:12">
       <c r="A670" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B670" t="s">
         <v>707</v>
@@ -32053,7 +32053,7 @@
         <v>1634</v>
       </c>
       <c r="I670" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J670" t="s">
         <v>2457</v>
@@ -32067,7 +32067,7 @@
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B671" t="s">
         <v>708</v>
@@ -32088,7 +32088,7 @@
         <v>1634</v>
       </c>
       <c r="I671" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J671" t="s">
         <v>2458</v>
@@ -32102,7 +32102,7 @@
     </row>
     <row r="672" spans="1:12">
       <c r="A672" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B672" t="s">
         <v>709</v>
@@ -32123,7 +32123,7 @@
         <v>1634</v>
       </c>
       <c r="I672" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J672" t="s">
         <v>2459</v>
@@ -32137,7 +32137,7 @@
     </row>
     <row r="673" spans="1:12">
       <c r="A673" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B673" t="s">
         <v>710</v>
@@ -32158,7 +32158,7 @@
         <v>1634</v>
       </c>
       <c r="I673" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J673" t="s">
         <v>2460</v>
@@ -32172,7 +32172,7 @@
     </row>
     <row r="674" spans="1:12">
       <c r="A674" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B674" t="s">
         <v>711</v>
@@ -32193,7 +32193,7 @@
         <v>1634</v>
       </c>
       <c r="I674" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J674" t="s">
         <v>2461</v>
@@ -32207,7 +32207,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B675" t="s">
         <v>712</v>
@@ -32228,7 +32228,7 @@
         <v>1634</v>
       </c>
       <c r="I675" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J675" t="s">
         <v>2462</v>
@@ -32242,7 +32242,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B676" t="s">
         <v>713</v>
@@ -32263,7 +32263,7 @@
         <v>1634</v>
       </c>
       <c r="I676" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J676" t="s">
         <v>2463</v>
@@ -32315,7 +32315,7 @@
     </row>
     <row r="678" spans="1:12">
       <c r="A678" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B678" t="s">
         <v>715</v>
@@ -32336,7 +32336,7 @@
         <v>1634</v>
       </c>
       <c r="I678" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J678" t="s">
         <v>2465</v>
@@ -32350,7 +32350,7 @@
     </row>
     <row r="679" spans="1:12">
       <c r="A679" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B679" t="s">
         <v>716</v>
@@ -32374,7 +32374,7 @@
         <v>1666</v>
       </c>
       <c r="I679" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J679" t="s">
         <v>2466</v>
@@ -32388,7 +32388,7 @@
     </row>
     <row r="680" spans="1:12">
       <c r="A680" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B680" t="s">
         <v>717</v>
@@ -32409,7 +32409,7 @@
         <v>1634</v>
       </c>
       <c r="I680" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J680" t="s">
         <v>2467</v>
@@ -32423,7 +32423,7 @@
     </row>
     <row r="681" spans="1:12">
       <c r="A681" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B681" t="s">
         <v>718</v>
@@ -32444,7 +32444,7 @@
         <v>1634</v>
       </c>
       <c r="I681" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="J681" t="s">
         <v>2468</v>
@@ -32458,7 +32458,7 @@
     </row>
     <row r="682" spans="1:12">
       <c r="A682" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B682" t="s">
         <v>719</v>
@@ -32493,7 +32493,7 @@
     </row>
     <row r="683" spans="1:12">
       <c r="A683" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B683" t="s">
         <v>720</v>
@@ -32511,7 +32511,7 @@
         <v>1634</v>
       </c>
       <c r="I683" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J683" t="s">
         <v>2470</v>
@@ -32525,7 +32525,7 @@
     </row>
     <row r="684" spans="1:12">
       <c r="A684" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B684" t="s">
         <v>721</v>
@@ -32543,7 +32543,7 @@
         <v>1634</v>
       </c>
       <c r="I684" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J684" t="s">
         <v>2471</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-05 18:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -15580,7 +15580,7 @@
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B205" t="s">
         <v>243</v>
@@ -15601,7 +15601,7 @@
         <v>1629</v>
       </c>
       <c r="I205" t="s">
-        <v>1724</v>
+        <v>1667</v>
       </c>
       <c r="J205" t="s">
         <v>1989</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-08 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -8047,7 +8047,7 @@
     <t>ENGENHARIA FLORESTAL,ENGENHARIA QUÍMICA,GEOLOGIA</t>
   </si>
   <si>
-    <t>SAÚDE MENTAL,ASSISTÊNCIA SOCIAL</t>
+    <t>ASSISTÊNCIA SOCIAL,SAÚDE MENTAL</t>
   </si>
   <si>
     <t>SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,SAÚDE,ECONOMIA,URBANISMO,ORÇAMENTO,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL</t>
@@ -15510,7 +15510,7 @@
     </row>
     <row r="203" spans="1:12">
       <c r="A203" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B203" t="s">
         <v>241</v>
@@ -15531,7 +15531,7 @@
         <v>1629</v>
       </c>
       <c r="I203" t="s">
-        <v>1688</v>
+        <v>1667</v>
       </c>
       <c r="J203" t="s">
         <v>1987</v>
@@ -30075,7 +30075,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B617" t="s">
         <v>654</v>
@@ -30096,7 +30096,7 @@
         <v>1629</v>
       </c>
       <c r="I617" t="s">
-        <v>1713</v>
+        <v>1667</v>
       </c>
       <c r="J617" t="s">
         <v>2395</v>
@@ -31006,7 +31006,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B643" t="s">
         <v>680</v>
@@ -31027,7 +31027,7 @@
         <v>1629</v>
       </c>
       <c r="I643" t="s">
-        <v>1713</v>
+        <v>1667</v>
       </c>
       <c r="J643" t="s">
         <v>2421</v>
@@ -31721,7 +31721,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B663" t="s">
         <v>700</v>
@@ -31742,7 +31742,7 @@
         <v>1629</v>
       </c>
       <c r="I663" t="s">
-        <v>1713</v>
+        <v>1667</v>
       </c>
       <c r="J663" t="s">
         <v>2440</v>
@@ -31756,7 +31756,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B664" t="s">
         <v>701</v>
@@ -31777,7 +31777,7 @@
         <v>1629</v>
       </c>
       <c r="I664" t="s">
-        <v>1713</v>
+        <v>1667</v>
       </c>
       <c r="J664" t="s">
         <v>2441</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-08 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -30110,7 +30110,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B618" t="s">
         <v>655</v>
@@ -30131,7 +30131,7 @@
         <v>1629</v>
       </c>
       <c r="I618" t="s">
-        <v>1713</v>
+        <v>1667</v>
       </c>
       <c r="J618" t="s">
         <v>2396</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-08 16:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -82,6 +82,9 @@
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA</t>
   </si>
   <si>
@@ -94,9 +97,6 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -5008,6 +5008,9 @@
     <t>LILIAN ALVES DE ARAUJO,SERGIO PEDRO LOPES,VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>PEDRO MARCELO ROCHA GOMES</t>
   </si>
   <si>
@@ -5026,33 +5029,33 @@
     <t>DAYSE BARBOSA DE ARAÚJO GÓIS,SERGIO PEDRO LOPES</t>
   </si>
   <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
+    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA</t>
+  </si>
+  <si>
+    <t>DANIEL FONTANA OBERLING</t>
+  </si>
+  <si>
+    <t>MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
     <t>PATRICIA PASSARO DA SILVA TOLEDO</t>
   </si>
   <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>DANIEL FONTANA OBERLING</t>
-  </si>
-  <si>
-    <t>MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
     <t>ROSEMARY PROVENZANO THAMI,VICTOR AUGUSTO LOURO BERBARA</t>
   </si>
   <si>
@@ -5099,9 +5102,6 @@
   </si>
   <si>
     <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
@@ -9753,7 +9753,7 @@
     </row>
     <row r="41" spans="1:12">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
         <v>77</v>
@@ -9774,7 +9774,7 @@
         <v>1614</v>
       </c>
       <c r="I41" t="s">
-        <v>1659</v>
+        <v>1664</v>
       </c>
       <c r="J41" t="s">
         <v>1817</v>
@@ -9858,7 +9858,7 @@
     </row>
     <row r="44" spans="1:12">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
         <v>80</v>
@@ -9882,7 +9882,7 @@
         <v>1619</v>
       </c>
       <c r="I44" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J44" t="s">
         <v>1820</v>
@@ -10176,7 +10176,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B53" t="s">
         <v>89</v>
@@ -10197,7 +10197,7 @@
         <v>1614</v>
       </c>
       <c r="I53" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J53" t="s">
         <v>1829</v>
@@ -10267,7 +10267,7 @@
         <v>1614</v>
       </c>
       <c r="I55" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J55" t="s">
         <v>1831</v>
@@ -10337,7 +10337,7 @@
         <v>1614</v>
       </c>
       <c r="I57" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J57" t="s">
         <v>1833</v>
@@ -10372,7 +10372,7 @@
         <v>1614</v>
       </c>
       <c r="I58" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J58" t="s">
         <v>1834</v>
@@ -10410,7 +10410,7 @@
         <v>1441</v>
       </c>
       <c r="I59" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J59" t="s">
         <v>1835</v>
@@ -10459,7 +10459,7 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B61" t="s">
         <v>97</v>
@@ -10480,7 +10480,7 @@
         <v>1614</v>
       </c>
       <c r="I61" t="s">
-        <v>1670</v>
+        <v>1664</v>
       </c>
       <c r="J61" t="s">
         <v>1837</v>
@@ -10529,7 +10529,7 @@
     </row>
     <row r="63" spans="1:12">
       <c r="A63" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B63" t="s">
         <v>99</v>
@@ -10599,7 +10599,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B65" t="s">
         <v>101</v>
@@ -10672,7 +10672,7 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B67" t="s">
         <v>103</v>
@@ -10882,7 +10882,7 @@
     </row>
     <row r="73" spans="1:12">
       <c r="A73" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B73" t="s">
         <v>109</v>
@@ -10990,7 +10990,7 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B76" t="s">
         <v>112</v>
@@ -11011,7 +11011,7 @@
         <v>1614</v>
       </c>
       <c r="I76" t="s">
-        <v>1670</v>
+        <v>1679</v>
       </c>
       <c r="J76" t="s">
         <v>1852</v>
@@ -11095,7 +11095,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B79" t="s">
         <v>115</v>
@@ -11116,7 +11116,7 @@
         <v>1614</v>
       </c>
       <c r="I79" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="J79" t="s">
         <v>1855</v>
@@ -11130,7 +11130,7 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B80" t="s">
         <v>116</v>
@@ -11151,7 +11151,7 @@
         <v>1614</v>
       </c>
       <c r="I80" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J80" t="s">
         <v>1856</v>
@@ -11165,7 +11165,7 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B81" t="s">
         <v>117</v>
@@ -11186,7 +11186,7 @@
         <v>1614</v>
       </c>
       <c r="I81" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J81" t="s">
         <v>1856</v>
@@ -11235,7 +11235,7 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B83" t="s">
         <v>119</v>
@@ -11256,7 +11256,7 @@
         <v>1614</v>
       </c>
       <c r="I83" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J83" t="s">
         <v>1857</v>
@@ -11305,7 +11305,7 @@
     </row>
     <row r="85" spans="1:12">
       <c r="A85" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B85" t="s">
         <v>121</v>
@@ -11326,7 +11326,7 @@
         <v>1614</v>
       </c>
       <c r="I85" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J85" t="s">
         <v>1859</v>
@@ -11375,7 +11375,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B87" t="s">
         <v>123</v>
@@ -11396,7 +11396,7 @@
         <v>1614</v>
       </c>
       <c r="I87" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="J87" t="s">
         <v>1861</v>
@@ -11550,7 +11550,7 @@
     </row>
     <row r="92" spans="1:12">
       <c r="A92" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B92" t="s">
         <v>128</v>
@@ -11585,7 +11585,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B93" t="s">
         <v>129</v>
@@ -11606,7 +11606,7 @@
         <v>1614</v>
       </c>
       <c r="I93" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J93" t="s">
         <v>1867</v>
@@ -11655,7 +11655,7 @@
     </row>
     <row r="95" spans="1:12">
       <c r="A95" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B95" t="s">
         <v>131</v>
@@ -11676,7 +11676,7 @@
         <v>1614</v>
       </c>
       <c r="I95" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J95" t="s">
         <v>1869</v>
@@ -11725,7 +11725,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B97" t="s">
         <v>133</v>
@@ -11865,7 +11865,7 @@
     </row>
     <row r="101" spans="1:12">
       <c r="A101" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B101" t="s">
         <v>137</v>
@@ -11935,7 +11935,7 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B103" t="s">
         <v>139</v>
@@ -11956,7 +11956,7 @@
         <v>1614</v>
       </c>
       <c r="I103" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J103" t="s">
         <v>1877</v>
@@ -12040,7 +12040,7 @@
     </row>
     <row r="106" spans="1:12">
       <c r="A106" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B106" t="s">
         <v>142</v>
@@ -12061,7 +12061,7 @@
         <v>1614</v>
       </c>
       <c r="I106" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J106" t="s">
         <v>1880</v>
@@ -12096,7 +12096,7 @@
         <v>1614</v>
       </c>
       <c r="I107" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J107" t="s">
         <v>1881</v>
@@ -12271,7 +12271,7 @@
         <v>1614</v>
       </c>
       <c r="I112" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J112" t="s">
         <v>1886</v>
@@ -12285,7 +12285,7 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B113" t="s">
         <v>149</v>
@@ -12306,7 +12306,7 @@
         <v>1614</v>
       </c>
       <c r="I113" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="J113" t="s">
         <v>1887</v>
@@ -12355,7 +12355,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B115" t="s">
         <v>151</v>
@@ -12376,7 +12376,7 @@
         <v>1614</v>
       </c>
       <c r="I115" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J115" t="s">
         <v>1889</v>
@@ -12460,7 +12460,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B118" t="s">
         <v>154</v>
@@ -12481,7 +12481,7 @@
         <v>1614</v>
       </c>
       <c r="I118" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J118" t="s">
         <v>1892</v>
@@ -12530,7 +12530,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B120" t="s">
         <v>156</v>
@@ -12551,7 +12551,7 @@
         <v>1614</v>
       </c>
       <c r="I120" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J120" t="s">
         <v>1894</v>
@@ -12621,7 +12621,7 @@
         <v>1614</v>
       </c>
       <c r="I122" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="J122" t="s">
         <v>1896</v>
@@ -12670,7 +12670,7 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B124" t="s">
         <v>160</v>
@@ -12691,7 +12691,7 @@
         <v>1614</v>
       </c>
       <c r="I124" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J124" t="s">
         <v>1898</v>
@@ -12764,7 +12764,7 @@
         <v>1504</v>
       </c>
       <c r="I126" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J126" t="s">
         <v>1900</v>
@@ -12945,7 +12945,7 @@
         <v>1785</v>
       </c>
       <c r="K131" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="L131" t="s">
         <v>2586</v>
@@ -13058,7 +13058,7 @@
     </row>
     <row r="135" spans="1:12">
       <c r="A135" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B135" t="s">
         <v>171</v>
@@ -13079,7 +13079,7 @@
         <v>1614</v>
       </c>
       <c r="I135" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J135" t="s">
         <v>1907</v>
@@ -13114,7 +13114,7 @@
         <v>1614</v>
       </c>
       <c r="I136" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J136" t="s">
         <v>1908</v>
@@ -13163,7 +13163,7 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B138" t="s">
         <v>174</v>
@@ -13222,7 +13222,7 @@
         <v>1621</v>
       </c>
       <c r="I139" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J139" t="s">
         <v>1785</v>
@@ -13257,7 +13257,7 @@
         <v>1614</v>
       </c>
       <c r="I140" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J140" t="s">
         <v>1911</v>
@@ -13271,7 +13271,7 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B141" t="s">
         <v>177</v>
@@ -13292,7 +13292,7 @@
         <v>1614</v>
       </c>
       <c r="I141" t="s">
-        <v>1695</v>
+        <v>1664</v>
       </c>
       <c r="J141" t="s">
         <v>1912</v>
@@ -13376,7 +13376,7 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B144" t="s">
         <v>180</v>
@@ -13656,7 +13656,7 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B152" t="s">
         <v>188</v>
@@ -13726,7 +13726,7 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B154" t="s">
         <v>190</v>
@@ -13796,7 +13796,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B156" t="s">
         <v>192</v>
@@ -13901,7 +13901,7 @@
     </row>
     <row r="159" spans="1:12">
       <c r="A159" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B159" t="s">
         <v>195</v>
@@ -14181,7 +14181,7 @@
     </row>
     <row r="167" spans="1:12">
       <c r="A167" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B167" t="s">
         <v>203</v>
@@ -14286,7 +14286,7 @@
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B170" t="s">
         <v>206</v>
@@ -14391,7 +14391,7 @@
     </row>
     <row r="173" spans="1:12">
       <c r="A173" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B173" t="s">
         <v>209</v>
@@ -14426,7 +14426,7 @@
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B174" t="s">
         <v>210</v>
@@ -14461,7 +14461,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B175" t="s">
         <v>211</v>
@@ -14531,7 +14531,7 @@
     </row>
     <row r="177" spans="1:12">
       <c r="A177" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B177" t="s">
         <v>213</v>
@@ -14881,7 +14881,7 @@
     </row>
     <row r="187" spans="1:12">
       <c r="A187" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B187" t="s">
         <v>223</v>
@@ -15129,7 +15129,7 @@
     </row>
     <row r="194" spans="1:12">
       <c r="A194" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B194" t="s">
         <v>230</v>
@@ -15689,7 +15689,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B210" t="s">
         <v>246</v>
@@ -15794,7 +15794,7 @@
     </row>
     <row r="213" spans="1:12">
       <c r="A213" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B213" t="s">
         <v>249</v>
@@ -15899,7 +15899,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B216" t="s">
         <v>252</v>
@@ -16074,7 +16074,7 @@
     </row>
     <row r="221" spans="1:12">
       <c r="A221" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B221" t="s">
         <v>257</v>
@@ -16340,7 +16340,7 @@
         <v>1614</v>
       </c>
       <c r="I228" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J228" t="s">
         <v>1996</v>
@@ -16354,7 +16354,7 @@
     </row>
     <row r="229" spans="1:12">
       <c r="A229" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B229" t="s">
         <v>265</v>
@@ -16427,7 +16427,7 @@
     </row>
     <row r="231" spans="1:12">
       <c r="A231" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B231" t="s">
         <v>267</v>
@@ -16567,7 +16567,7 @@
     </row>
     <row r="235" spans="1:12">
       <c r="A235" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B235" t="s">
         <v>271</v>
@@ -16742,7 +16742,7 @@
     </row>
     <row r="240" spans="1:12">
       <c r="A240" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B240" t="s">
         <v>276</v>
@@ -16777,7 +16777,7 @@
     </row>
     <row r="241" spans="1:12">
       <c r="A241" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B241" t="s">
         <v>277</v>
@@ -16917,7 +16917,7 @@
     </row>
     <row r="245" spans="1:12">
       <c r="A245" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B245" t="s">
         <v>281</v>
@@ -16987,7 +16987,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B247" t="s">
         <v>283</v>
@@ -17095,7 +17095,7 @@
     </row>
     <row r="250" spans="1:12">
       <c r="A250" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B250" t="s">
         <v>286</v>
@@ -17235,7 +17235,7 @@
     </row>
     <row r="254" spans="1:12">
       <c r="A254" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B254" t="s">
         <v>290</v>
@@ -17270,7 +17270,7 @@
     </row>
     <row r="255" spans="1:12">
       <c r="A255" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B255" t="s">
         <v>291</v>
@@ -17305,7 +17305,7 @@
     </row>
     <row r="256" spans="1:12">
       <c r="A256" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B256" t="s">
         <v>292</v>
@@ -17326,7 +17326,7 @@
         <v>1614</v>
       </c>
       <c r="I256" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J256" t="s">
         <v>2024</v>
@@ -17515,7 +17515,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B262" t="s">
         <v>298</v>
@@ -17536,7 +17536,7 @@
         <v>1614</v>
       </c>
       <c r="I262" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J262" t="s">
         <v>2029</v>
@@ -17550,7 +17550,7 @@
     </row>
     <row r="263" spans="1:12">
       <c r="A263" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B263" t="s">
         <v>299</v>
@@ -17585,7 +17585,7 @@
     </row>
     <row r="264" spans="1:12">
       <c r="A264" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B264" t="s">
         <v>300</v>
@@ -17609,7 +17609,7 @@
         <v>1623</v>
       </c>
       <c r="I264" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J264" t="s">
         <v>2031</v>
@@ -17623,7 +17623,7 @@
     </row>
     <row r="265" spans="1:12">
       <c r="A265" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B265" t="s">
         <v>301</v>
@@ -17658,7 +17658,7 @@
     </row>
     <row r="266" spans="1:12">
       <c r="A266" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B266" t="s">
         <v>302</v>
@@ -17693,7 +17693,7 @@
     </row>
     <row r="267" spans="1:12">
       <c r="A267" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B267" t="s">
         <v>303</v>
@@ -17903,7 +17903,7 @@
     </row>
     <row r="273" spans="1:12">
       <c r="A273" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B273" t="s">
         <v>309</v>
@@ -18218,7 +18218,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B282" t="s">
         <v>318</v>
@@ -18396,7 +18396,7 @@
     </row>
     <row r="287" spans="1:12">
       <c r="A287" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B287" t="s">
         <v>323</v>
@@ -18466,7 +18466,7 @@
     </row>
     <row r="289" spans="1:12">
       <c r="A289" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B289" t="s">
         <v>325</v>
@@ -18571,7 +18571,7 @@
     </row>
     <row r="292" spans="1:12">
       <c r="A292" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B292" t="s">
         <v>328</v>
@@ -18886,7 +18886,7 @@
     </row>
     <row r="301" spans="1:12">
       <c r="A301" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B301" t="s">
         <v>337</v>
@@ -19131,7 +19131,7 @@
     </row>
     <row r="308" spans="1:12">
       <c r="A308" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B308" t="s">
         <v>344</v>
@@ -19187,7 +19187,7 @@
         <v>1614</v>
       </c>
       <c r="I309" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J309" t="s">
         <v>2075</v>
@@ -19379,7 +19379,7 @@
     </row>
     <row r="315" spans="1:12">
       <c r="A315" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B315" t="s">
         <v>351</v>
@@ -19400,7 +19400,7 @@
         <v>1614</v>
       </c>
       <c r="I315" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J315" t="s">
         <v>2081</v>
@@ -19519,7 +19519,7 @@
     </row>
     <row r="319" spans="1:12">
       <c r="A319" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B319" t="s">
         <v>355</v>
@@ -19624,7 +19624,7 @@
     </row>
     <row r="322" spans="1:12">
       <c r="A322" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B322" t="s">
         <v>358</v>
@@ -19939,7 +19939,7 @@
     </row>
     <row r="331" spans="1:12">
       <c r="A331" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B331" t="s">
         <v>367</v>
@@ -20187,7 +20187,7 @@
     </row>
     <row r="338" spans="1:12">
       <c r="A338" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B338" t="s">
         <v>374</v>
@@ -20222,7 +20222,7 @@
     </row>
     <row r="339" spans="1:12">
       <c r="A339" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B339" t="s">
         <v>375</v>
@@ -20257,7 +20257,7 @@
     </row>
     <row r="340" spans="1:12">
       <c r="A340" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B340" t="s">
         <v>376</v>
@@ -20397,7 +20397,7 @@
     </row>
     <row r="344" spans="1:12">
       <c r="A344" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B344" t="s">
         <v>380</v>
@@ -20432,7 +20432,7 @@
     </row>
     <row r="345" spans="1:12">
       <c r="A345" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B345" t="s">
         <v>381</v>
@@ -20537,7 +20537,7 @@
     </row>
     <row r="348" spans="1:12">
       <c r="A348" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B348" t="s">
         <v>384</v>
@@ -20712,7 +20712,7 @@
     </row>
     <row r="353" spans="1:12">
       <c r="A353" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B353" t="s">
         <v>389</v>
@@ -20733,7 +20733,7 @@
         <v>1614</v>
       </c>
       <c r="I353" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J353" t="s">
         <v>2119</v>
@@ -21062,7 +21062,7 @@
     </row>
     <row r="363" spans="1:12">
       <c r="A363" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B363" t="s">
         <v>399</v>
@@ -21132,7 +21132,7 @@
     </row>
     <row r="365" spans="1:12">
       <c r="A365" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B365" t="s">
         <v>401</v>
@@ -21167,7 +21167,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B366" t="s">
         <v>402</v>
@@ -21202,7 +21202,7 @@
     </row>
     <row r="367" spans="1:12">
       <c r="A367" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B367" t="s">
         <v>403</v>
@@ -21342,7 +21342,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B371" t="s">
         <v>407</v>
@@ -21377,7 +21377,7 @@
     </row>
     <row r="372" spans="1:12">
       <c r="A372" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B372" t="s">
         <v>408</v>
@@ -21657,7 +21657,7 @@
     </row>
     <row r="380" spans="1:12">
       <c r="A380" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B380" t="s">
         <v>416</v>
@@ -21867,7 +21867,7 @@
     </row>
     <row r="386" spans="1:12">
       <c r="A386" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B386" t="s">
         <v>422</v>
@@ -21972,7 +21972,7 @@
     </row>
     <row r="389" spans="1:12">
       <c r="A389" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B389" t="s">
         <v>425</v>
@@ -22007,7 +22007,7 @@
     </row>
     <row r="390" spans="1:12">
       <c r="A390" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B390" t="s">
         <v>426</v>
@@ -22591,7 +22591,7 @@
         <v>1626</v>
       </c>
       <c r="I406" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J406" t="s">
         <v>2170</v>
@@ -22640,7 +22640,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B408" t="s">
         <v>444</v>
@@ -22675,7 +22675,7 @@
     </row>
     <row r="409" spans="1:12">
       <c r="A409" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B409" t="s">
         <v>445</v>
@@ -22850,7 +22850,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B414" t="s">
         <v>450</v>
@@ -23060,7 +23060,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B420" t="s">
         <v>455</v>
@@ -23081,7 +23081,7 @@
         <v>1614</v>
       </c>
       <c r="I420" t="s">
-        <v>1695</v>
+        <v>1664</v>
       </c>
       <c r="J420" t="s">
         <v>2183</v>
@@ -23165,7 +23165,7 @@
     </row>
     <row r="423" spans="1:12">
       <c r="A423" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B423" t="s">
         <v>458</v>
@@ -23186,7 +23186,7 @@
         <v>1614</v>
       </c>
       <c r="I423" t="s">
-        <v>1710</v>
+        <v>1664</v>
       </c>
       <c r="J423" t="s">
         <v>2186</v>
@@ -23235,7 +23235,7 @@
     </row>
     <row r="425" spans="1:12">
       <c r="A425" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B425" t="s">
         <v>460</v>
@@ -23340,7 +23340,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B428" t="s">
         <v>463</v>
@@ -23466,7 +23466,7 @@
         <v>1614</v>
       </c>
       <c r="I431" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J431" t="s">
         <v>2194</v>
@@ -23480,7 +23480,7 @@
     </row>
     <row r="432" spans="1:12">
       <c r="A432" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B432" t="s">
         <v>467</v>
@@ -23760,7 +23760,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B440" t="s">
         <v>475</v>
@@ -24005,7 +24005,7 @@
     </row>
     <row r="447" spans="1:12">
       <c r="A447" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B447" t="s">
         <v>482</v>
@@ -24218,7 +24218,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B453" t="s">
         <v>488</v>
@@ -24253,7 +24253,7 @@
     </row>
     <row r="454" spans="1:12">
       <c r="A454" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B454" t="s">
         <v>489</v>
@@ -24288,7 +24288,7 @@
     </row>
     <row r="455" spans="1:12">
       <c r="A455" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B455" t="s">
         <v>490</v>
@@ -24463,7 +24463,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B460" t="s">
         <v>495</v>
@@ -24708,7 +24708,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B467" t="s">
         <v>502</v>
@@ -24743,7 +24743,7 @@
     </row>
     <row r="468" spans="1:12">
       <c r="A468" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B468" t="s">
         <v>503</v>
@@ -24778,7 +24778,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B469" t="s">
         <v>504</v>
@@ -24813,7 +24813,7 @@
     </row>
     <row r="470" spans="1:12">
       <c r="A470" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B470" t="s">
         <v>505</v>
@@ -25044,7 +25044,7 @@
         <v>1614</v>
       </c>
       <c r="I476" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J476" t="s">
         <v>2239</v>
@@ -25093,7 +25093,7 @@
     </row>
     <row r="478" spans="1:12">
       <c r="A478" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B478" t="s">
         <v>513</v>
@@ -25163,7 +25163,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B480" t="s">
         <v>515</v>
@@ -25446,7 +25446,7 @@
     </row>
     <row r="488" spans="1:12">
       <c r="A488" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B488" t="s">
         <v>523</v>
@@ -25481,7 +25481,7 @@
     </row>
     <row r="489" spans="1:12">
       <c r="A489" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B489" t="s">
         <v>524</v>
@@ -25551,7 +25551,7 @@
     </row>
     <row r="491" spans="1:12">
       <c r="A491" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B491" t="s">
         <v>526</v>
@@ -25866,7 +25866,7 @@
     </row>
     <row r="500" spans="1:12">
       <c r="A500" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B500" t="s">
         <v>535</v>
@@ -25901,7 +25901,7 @@
     </row>
     <row r="501" spans="1:12">
       <c r="A501" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B501" t="s">
         <v>536</v>
@@ -25936,7 +25936,7 @@
     </row>
     <row r="502" spans="1:12">
       <c r="A502" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B502" t="s">
         <v>537</v>
@@ -26044,7 +26044,7 @@
     </row>
     <row r="505" spans="1:12">
       <c r="A505" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B505" t="s">
         <v>540</v>
@@ -26289,7 +26289,7 @@
     </row>
     <row r="512" spans="1:12">
       <c r="A512" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B512" t="s">
         <v>547</v>
@@ -26324,7 +26324,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B513" t="s">
         <v>548</v>
@@ -26359,7 +26359,7 @@
     </row>
     <row r="514" spans="1:12">
       <c r="A514" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B514" t="s">
         <v>549</v>
@@ -26499,7 +26499,7 @@
     </row>
     <row r="518" spans="1:12">
       <c r="A518" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B518" t="s">
         <v>553</v>
@@ -26639,7 +26639,7 @@
     </row>
     <row r="522" spans="1:12">
       <c r="A522" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B522" t="s">
         <v>557</v>
@@ -27590,7 +27590,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B549" t="s">
         <v>584</v>
@@ -27663,7 +27663,7 @@
     </row>
     <row r="551" spans="1:12">
       <c r="A551" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B551" t="s">
         <v>586</v>
@@ -27733,7 +27733,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B553" t="s">
         <v>588</v>
@@ -27978,7 +27978,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B560" t="s">
         <v>595</v>
@@ -28285,7 +28285,7 @@
         <v>1632</v>
       </c>
       <c r="I568" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J568" t="s">
         <v>2331</v>
@@ -28299,7 +28299,7 @@
     </row>
     <row r="569" spans="1:12">
       <c r="A569" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B569" t="s">
         <v>604</v>
@@ -28477,7 +28477,7 @@
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B574" t="s">
         <v>609</v>
@@ -28582,7 +28582,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B577" t="s">
         <v>612</v>
@@ -29011,7 +29011,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B589" t="s">
         <v>624</v>
@@ -29554,7 +29554,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B604" t="s">
         <v>639</v>
@@ -29624,7 +29624,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B606" t="s">
         <v>641</v>
@@ -29729,7 +29729,7 @@
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B609" t="s">
         <v>644</v>
@@ -29764,7 +29764,7 @@
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B610" t="s">
         <v>645</v>
@@ -29942,7 +29942,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B615" t="s">
         <v>650</v>
@@ -29977,7 +29977,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B616" t="s">
         <v>651</v>
@@ -30085,7 +30085,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B619" t="s">
         <v>654</v>
@@ -30196,7 +30196,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B622" t="s">
         <v>657</v>
@@ -30217,7 +30217,7 @@
         <v>1614</v>
       </c>
       <c r="I622" t="s">
-        <v>1695</v>
+        <v>1664</v>
       </c>
       <c r="J622" t="s">
         <v>2385</v>
@@ -30660,7 +30660,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B635" t="s">
         <v>670</v>
@@ -30695,7 +30695,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B636" t="s">
         <v>671</v>
@@ -30716,7 +30716,7 @@
         <v>1614</v>
       </c>
       <c r="I636" t="s">
-        <v>1695</v>
+        <v>1664</v>
       </c>
       <c r="J636" t="s">
         <v>2399</v>
@@ -30862,7 +30862,7 @@
         <v>1633</v>
       </c>
       <c r="I640" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J640" t="s">
         <v>2403</v>
@@ -30952,7 +30952,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B643" t="s">
         <v>678</v>
@@ -31375,7 +31375,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B655" t="s">
         <v>690</v>
@@ -31410,7 +31410,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B656" t="s">
         <v>691</v>
@@ -31696,7 +31696,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B664" t="s">
         <v>699</v>
@@ -31731,7 +31731,7 @@
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B665" t="s">
         <v>700</v>
@@ -31769,7 +31769,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B666" t="s">
         <v>701</v>
@@ -31807,7 +31807,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B667" t="s">
         <v>702</v>
@@ -31842,7 +31842,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B668" t="s">
         <v>703</v>
@@ -31947,7 +31947,7 @@
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B671" t="s">
         <v>706</v>
@@ -32020,7 +32020,7 @@
     </row>
     <row r="673" spans="1:12">
       <c r="A673" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B673" t="s">
         <v>708</v>
@@ -32055,7 +32055,7 @@
     </row>
     <row r="674" spans="1:12">
       <c r="A674" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B674" t="s">
         <v>709</v>
@@ -32087,7 +32087,7 @@
     </row>
     <row r="675" spans="1:12">
       <c r="A675" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B675" t="s">
         <v>710</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-08 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6780" uniqueCount="2645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6780" uniqueCount="2646">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -5155,150 +5155,150 @@
     <t>GIULIANA DE ANDRADE CERVAI,HUDSON DE OLIVEIRA SACRAMENTO</t>
   </si>
   <si>
+    <t>GLAUCO CASTILHO DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>ANDRÉA DINIZ MATTOS</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
+    <t>RAQUEL SILVA FERNANDES LYRA</t>
+  </si>
+  <si>
+    <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>DANIEL FONTANA OBERLING,EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
+    <t>VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,FERNANDA FERREIRA FONTES</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,PATRÍCIA FINAMORE ARAÚJO,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA</t>
+  </si>
+  <si>
+    <t>MARCELO KOLBLINGER DE GODOY</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,LILIAN ALVES DE ARAUJO</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,EDIWAN SOUSA DA SILVA,JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>MARCELO KOLBLINGER DE GODOY,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>REINALDO DE SOUZA MACHADO,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,PATRÍCIA FINAMORE ARAÚJO</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA</t>
+  </si>
+  <si>
+    <t>SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>JORGE LUIS DANTAS BATISTA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>DAYSE BARBOSA DE ARAÚJO GÓIS,IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
     <t>REINALDO DE SOUZA MACHADO</t>
   </si>
   <si>
-    <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
-    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>ANDRÉA DINIZ MATTOS</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI,SEZISNANDO JOSE PRIMO PAES,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
-    <t>RAQUEL SILVA FERNANDES LYRA</t>
-  </si>
-  <si>
-    <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>DANIEL FONTANA OBERLING,EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
-    <t>VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,FERNANDA FERREIRA FONTES</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,PATRÍCIA FINAMORE ARAÚJO,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA</t>
-  </si>
-  <si>
-    <t>MARCELO KOLBLINGER DE GODOY</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,LILIAN ALVES DE ARAUJO</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,EDIWAN SOUSA DA SILVA,JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>MARCELO KOLBLINGER DE GODOY,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,PATRÍCIA FINAMORE ARAÚJO</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA</t>
-  </si>
-  <si>
-    <t>SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>JORGE LUIS DANTAS BATISTA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>DAYSE BARBOSA DE ARAÚJO GÓIS,IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
     <t>ERIKA CANTANHEDE WUILLAUME,MARCELO TEIXEIRA SANTANA,VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
@@ -7870,7 +7870,7 @@
     <t>BIOLOGIA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
+    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7882,7 +7882,7 @@
     <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA FLORESTAL,ENGENHARIA AMBIENTAL</t>
+    <t>ENGENHARIA AMBIENTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7948,7 +7948,10 @@
     <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ECONOMIA,URBANISMO,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL,ORÇAMENTO,SAÚDE</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ECONOMIA,ASSISTÊNCIA SOCIAL,SAÚDE,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,URBANISMO,PSICOLOGIA,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
 </sst>
 </file>
@@ -16391,7 +16394,7 @@
     </row>
     <row r="231" spans="1:12">
       <c r="A231" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B231" t="s">
         <v>266</v>
@@ -16412,7 +16415,7 @@
         <v>1607</v>
       </c>
       <c r="I231" t="s">
-        <v>1713</v>
+        <v>1645</v>
       </c>
       <c r="J231" t="s">
         <v>1989</v>
@@ -16552,7 +16555,7 @@
         <v>1607</v>
       </c>
       <c r="I235" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J235" t="s">
         <v>1993</v>
@@ -16657,7 +16660,7 @@
         <v>1607</v>
       </c>
       <c r="I238" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J238" t="s">
         <v>1996</v>
@@ -16762,7 +16765,7 @@
         <v>1607</v>
       </c>
       <c r="I241" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="J241" t="s">
         <v>1999</v>
@@ -17115,7 +17118,7 @@
         <v>1607</v>
       </c>
       <c r="I251" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="J251" t="s">
         <v>2009</v>
@@ -17150,7 +17153,7 @@
         <v>1607</v>
       </c>
       <c r="I252" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="J252" t="s">
         <v>2010</v>
@@ -17185,7 +17188,7 @@
         <v>1607</v>
       </c>
       <c r="I253" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="J253" t="s">
         <v>2011</v>
@@ -17255,7 +17258,7 @@
         <v>1607</v>
       </c>
       <c r="I255" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="J255" t="s">
         <v>2013</v>
@@ -17678,7 +17681,7 @@
         <v>1607</v>
       </c>
       <c r="I267" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J267" t="s">
         <v>2023</v>
@@ -18276,7 +18279,7 @@
         <v>1607</v>
       </c>
       <c r="I284" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J284" t="s">
         <v>2040</v>
@@ -18486,7 +18489,7 @@
         <v>1607</v>
       </c>
       <c r="I290" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J290" t="s">
         <v>2046</v>
@@ -18591,7 +18594,7 @@
         <v>1607</v>
       </c>
       <c r="I293" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J293" t="s">
         <v>2049</v>
@@ -19046,7 +19049,7 @@
         <v>1607</v>
       </c>
       <c r="I306" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J306" t="s">
         <v>2062</v>
@@ -19221,7 +19224,7 @@
         <v>1607</v>
       </c>
       <c r="I311" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J311" t="s">
         <v>2067</v>
@@ -19749,7 +19752,7 @@
         <v>1607</v>
       </c>
       <c r="I326" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J326" t="s">
         <v>2082</v>
@@ -19857,7 +19860,7 @@
         <v>1552</v>
       </c>
       <c r="I329" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J329" t="s">
         <v>2085</v>
@@ -20032,7 +20035,7 @@
         <v>1607</v>
       </c>
       <c r="I334" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J334" t="s">
         <v>2090</v>
@@ -20172,7 +20175,7 @@
         <v>1607</v>
       </c>
       <c r="I338" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="J338" t="s">
         <v>2094</v>
@@ -20242,7 +20245,7 @@
         <v>1607</v>
       </c>
       <c r="I340" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="J340" t="s">
         <v>2096</v>
@@ -20487,7 +20490,7 @@
         <v>1607</v>
       </c>
       <c r="I347" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J347" t="s">
         <v>2103</v>
@@ -20872,7 +20875,7 @@
         <v>1607</v>
       </c>
       <c r="I358" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J358" t="s">
         <v>1941</v>
@@ -21117,7 +21120,7 @@
         <v>1607</v>
       </c>
       <c r="I365" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J365" t="s">
         <v>2120</v>
@@ -21292,7 +21295,7 @@
         <v>1607</v>
       </c>
       <c r="I370" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J370" t="s">
         <v>2125</v>
@@ -21362,7 +21365,7 @@
         <v>1607</v>
       </c>
       <c r="I372" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J372" t="s">
         <v>2126</v>
@@ -21572,7 +21575,7 @@
         <v>1607</v>
       </c>
       <c r="I378" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="J378" t="s">
         <v>2132</v>
@@ -21677,7 +21680,7 @@
         <v>1607</v>
       </c>
       <c r="I381" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="J381" t="s">
         <v>2135</v>
@@ -22520,7 +22523,7 @@
         <v>1607</v>
       </c>
       <c r="I405" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J405" t="s">
         <v>2159</v>
@@ -22730,7 +22733,7 @@
         <v>1607</v>
       </c>
       <c r="I411" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="J411" t="s">
         <v>2165</v>
@@ -22940,7 +22943,7 @@
         <v>1607</v>
       </c>
       <c r="I417" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="J417" t="s">
         <v>2171</v>
@@ -23045,7 +23048,7 @@
         <v>1607</v>
       </c>
       <c r="I420" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J420" t="s">
         <v>2173</v>
@@ -23115,7 +23118,7 @@
         <v>1607</v>
       </c>
       <c r="I422" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J422" t="s">
         <v>2175</v>
@@ -23255,7 +23258,7 @@
         <v>1607</v>
       </c>
       <c r="I426" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J426" t="s">
         <v>2179</v>
@@ -23325,7 +23328,7 @@
         <v>1607</v>
       </c>
       <c r="I428" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J428" t="s">
         <v>2181</v>
@@ -23395,7 +23398,7 @@
         <v>1607</v>
       </c>
       <c r="I430" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J430" t="s">
         <v>2183</v>
@@ -23430,7 +23433,7 @@
         <v>1607</v>
       </c>
       <c r="I431" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J431" t="s">
         <v>2184</v>
@@ -23465,7 +23468,7 @@
         <v>1607</v>
       </c>
       <c r="I432" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J432" t="s">
         <v>2185</v>
@@ -24308,7 +24311,7 @@
         <v>1607</v>
       </c>
       <c r="I456" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
       <c r="J456" t="s">
         <v>2209</v>
@@ -24378,7 +24381,7 @@
         <v>1607</v>
       </c>
       <c r="I458" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="J458" t="s">
         <v>2211</v>
@@ -24518,7 +24521,7 @@
         <v>1607</v>
       </c>
       <c r="I462" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J462" t="s">
         <v>2215</v>
@@ -24553,7 +24556,7 @@
         <v>1607</v>
       </c>
       <c r="I463" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J463" t="s">
         <v>2216</v>
@@ -24658,7 +24661,7 @@
         <v>1607</v>
       </c>
       <c r="I466" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J466" t="s">
         <v>2219</v>
@@ -24868,7 +24871,7 @@
         <v>1607</v>
       </c>
       <c r="I472" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="J472" t="s">
         <v>2225</v>
@@ -24973,7 +24976,7 @@
         <v>1607</v>
       </c>
       <c r="I475" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J475" t="s">
         <v>2228</v>
@@ -25253,7 +25256,7 @@
         <v>1607</v>
       </c>
       <c r="I483" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J483" t="s">
         <v>2236</v>
@@ -25288,7 +25291,7 @@
         <v>1607</v>
       </c>
       <c r="I484" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="J484" t="s">
         <v>2237</v>
@@ -25361,7 +25364,7 @@
         <v>1607</v>
       </c>
       <c r="I486" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="J486" t="s">
         <v>2239</v>
@@ -25431,7 +25434,7 @@
         <v>1607</v>
       </c>
       <c r="I488" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J488" t="s">
         <v>2241</v>
@@ -25466,7 +25469,7 @@
         <v>1607</v>
       </c>
       <c r="I489" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J489" t="s">
         <v>2242</v>
@@ -25536,7 +25539,7 @@
         <v>1607</v>
       </c>
       <c r="I491" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J491" t="s">
         <v>2244</v>
@@ -25641,7 +25644,7 @@
         <v>1607</v>
       </c>
       <c r="I494" t="s">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="J494" t="s">
         <v>2247</v>
@@ -25711,7 +25714,7 @@
         <v>1607</v>
       </c>
       <c r="I496" t="s">
-        <v>1745</v>
+        <v>1744</v>
       </c>
       <c r="J496" t="s">
         <v>2249</v>
@@ -26029,7 +26032,7 @@
         <v>1607</v>
       </c>
       <c r="I505" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J505" t="s">
         <v>2258</v>
@@ -26204,7 +26207,7 @@
         <v>1607</v>
       </c>
       <c r="I510" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="J510" t="s">
         <v>2263</v>
@@ -26519,7 +26522,7 @@
         <v>1607</v>
       </c>
       <c r="I519" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J519" t="s">
         <v>2272</v>
@@ -26554,7 +26557,7 @@
         <v>1607</v>
       </c>
       <c r="I520" t="s">
-        <v>1747</v>
+        <v>1746</v>
       </c>
       <c r="J520" t="s">
         <v>2273</v>
@@ -26694,7 +26697,7 @@
         <v>1607</v>
       </c>
       <c r="I524" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J524" t="s">
         <v>2277</v>
@@ -26729,7 +26732,7 @@
         <v>1607</v>
       </c>
       <c r="I525" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J525" t="s">
         <v>2278</v>
@@ -26764,7 +26767,7 @@
         <v>1607</v>
       </c>
       <c r="I526" t="s">
-        <v>1748</v>
+        <v>1747</v>
       </c>
       <c r="J526" t="s">
         <v>2279</v>
@@ -26834,7 +26837,7 @@
         <v>1607</v>
       </c>
       <c r="I528" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J528" t="s">
         <v>2281</v>
@@ -26872,7 +26875,7 @@
         <v>1623</v>
       </c>
       <c r="I529" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J529" t="s">
         <v>2282</v>
@@ -26942,7 +26945,7 @@
         <v>1607</v>
       </c>
       <c r="I531" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J531" t="s">
         <v>2284</v>
@@ -27012,7 +27015,7 @@
         <v>1607</v>
       </c>
       <c r="I533" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J533" t="s">
         <v>2286</v>
@@ -27047,7 +27050,7 @@
         <v>1607</v>
       </c>
       <c r="I534" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J534" t="s">
         <v>2287</v>
@@ -27155,7 +27158,7 @@
         <v>1607</v>
       </c>
       <c r="I537" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J537" t="s">
         <v>2290</v>
@@ -27400,7 +27403,7 @@
         <v>1607</v>
       </c>
       <c r="I544" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J544" t="s">
         <v>2297</v>
@@ -27470,7 +27473,7 @@
         <v>1607</v>
       </c>
       <c r="I546" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="J546" t="s">
         <v>2299</v>
@@ -27508,7 +27511,7 @@
         <v>1594</v>
       </c>
       <c r="I547" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J547" t="s">
         <v>2300</v>
@@ -27543,7 +27546,7 @@
         <v>1607</v>
       </c>
       <c r="I548" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="J548" t="s">
         <v>2301</v>
@@ -27613,7 +27616,7 @@
         <v>1607</v>
       </c>
       <c r="I550" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J550" t="s">
         <v>2303</v>
@@ -27683,7 +27686,7 @@
         <v>1607</v>
       </c>
       <c r="I552" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J552" t="s">
         <v>2305</v>
@@ -27858,7 +27861,7 @@
         <v>1607</v>
       </c>
       <c r="I557" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="J557" t="s">
         <v>2310</v>
@@ -27893,7 +27896,7 @@
         <v>1607</v>
       </c>
       <c r="I558" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="J558" t="s">
         <v>2311</v>
@@ -28001,7 +28004,7 @@
         <v>1607</v>
       </c>
       <c r="I561" t="s">
-        <v>1752</v>
+        <v>1751</v>
       </c>
       <c r="J561" t="s">
         <v>2314</v>
@@ -28249,7 +28252,7 @@
         <v>1607</v>
       </c>
       <c r="I568" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J568" t="s">
         <v>2321</v>
@@ -28322,7 +28325,7 @@
         <v>1626</v>
       </c>
       <c r="I570" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="J570" t="s">
         <v>2323</v>
@@ -28357,7 +28360,7 @@
         <v>1607</v>
       </c>
       <c r="I571" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J571" t="s">
         <v>2324</v>
@@ -28427,7 +28430,7 @@
         <v>1607</v>
       </c>
       <c r="I573" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J573" t="s">
         <v>2326</v>
@@ -28748,7 +28751,7 @@
         <v>1607</v>
       </c>
       <c r="I582" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J582" t="s">
         <v>2335</v>
@@ -28783,7 +28786,7 @@
         <v>1607</v>
       </c>
       <c r="I583" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J583" t="s">
         <v>2336</v>
@@ -28818,7 +28821,7 @@
         <v>1607</v>
       </c>
       <c r="I584" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J584" t="s">
         <v>2337</v>
@@ -28853,7 +28856,7 @@
         <v>1607</v>
       </c>
       <c r="I585" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J585" t="s">
         <v>2338</v>
@@ -28891,7 +28894,7 @@
         <v>1629</v>
       </c>
       <c r="I586" t="s">
-        <v>1754</v>
+        <v>1753</v>
       </c>
       <c r="J586" t="s">
         <v>2339</v>
@@ -29072,7 +29075,7 @@
         <v>1616</v>
       </c>
       <c r="I591" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="J591" t="s">
         <v>2344</v>
@@ -29110,7 +29113,7 @@
         <v>1630</v>
       </c>
       <c r="I592" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="J592" t="s">
         <v>2345</v>
@@ -29148,7 +29151,7 @@
         <v>1616</v>
       </c>
       <c r="I593" t="s">
-        <v>1757</v>
+        <v>1756</v>
       </c>
       <c r="J593" t="s">
         <v>2346</v>
@@ -29186,7 +29189,7 @@
         <v>1631</v>
       </c>
       <c r="I594" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="J594" t="s">
         <v>2347</v>
@@ -29221,7 +29224,7 @@
         <v>1607</v>
       </c>
       <c r="I595" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J595" t="s">
         <v>2348</v>
@@ -29291,7 +29294,7 @@
         <v>1607</v>
       </c>
       <c r="I597" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J597" t="s">
         <v>2350</v>
@@ -29329,7 +29332,7 @@
         <v>1625</v>
       </c>
       <c r="I598" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="J598" t="s">
         <v>2351</v>
@@ -29539,7 +29542,7 @@
         <v>1607</v>
       </c>
       <c r="I604" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="J604" t="s">
         <v>2357</v>
@@ -29609,7 +29612,7 @@
         <v>1607</v>
       </c>
       <c r="I606" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="J606" t="s">
         <v>2359</v>
@@ -29784,7 +29787,7 @@
         <v>1607</v>
       </c>
       <c r="I611" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J611" t="s">
         <v>2364</v>
@@ -29822,7 +29825,7 @@
         <v>1632</v>
       </c>
       <c r="I612" t="s">
-        <v>1713</v>
+        <v>1760</v>
       </c>
       <c r="J612" t="s">
         <v>2365</v>
@@ -29857,7 +29860,7 @@
         <v>1607</v>
       </c>
       <c r="I613" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="J613" t="s">
         <v>2366</v>
@@ -29927,7 +29930,7 @@
         <v>1607</v>
       </c>
       <c r="I615" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J615" t="s">
         <v>2368</v>
@@ -30184,7 +30187,7 @@
         <v>1607</v>
       </c>
       <c r="I622" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J622" t="s">
         <v>2375</v>
@@ -30292,7 +30295,7 @@
         <v>1607</v>
       </c>
       <c r="I625" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J625" t="s">
         <v>2378</v>
@@ -30867,7 +30870,7 @@
         <v>1607</v>
       </c>
       <c r="I641" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J641" t="s">
         <v>1775</v>
@@ -30902,7 +30905,7 @@
         <v>1607</v>
       </c>
       <c r="I642" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J642" t="s">
         <v>2394</v>
@@ -31010,7 +31013,7 @@
         <v>1607</v>
       </c>
       <c r="I645" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J645" t="s">
         <v>2397</v>
@@ -31080,7 +31083,7 @@
         <v>1607</v>
       </c>
       <c r="I647" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J647" t="s">
         <v>2399</v>
@@ -31255,7 +31258,7 @@
         <v>1607</v>
       </c>
       <c r="I652" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J652" t="s">
         <v>2404</v>
@@ -31398,7 +31401,7 @@
         <v>1607</v>
       </c>
       <c r="I656" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J656" t="s">
         <v>2408</v>
@@ -31445,7 +31448,7 @@
         <v>2427</v>
       </c>
       <c r="L657" t="s">
-        <v>2606</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="658" spans="1:12">
@@ -31471,7 +31474,7 @@
         <v>1607</v>
       </c>
       <c r="I658" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J658" t="s">
         <v>2410</v>
@@ -31506,7 +31509,7 @@
         <v>1607</v>
       </c>
       <c r="I659" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J659" t="s">
         <v>2411</v>
@@ -31541,7 +31544,7 @@
         <v>1607</v>
       </c>
       <c r="I660" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J660" t="s">
         <v>2412</v>
@@ -31576,7 +31579,7 @@
         <v>1607</v>
       </c>
       <c r="I661" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="J661" t="s">
         <v>2413</v>
@@ -31611,7 +31614,7 @@
         <v>1607</v>
       </c>
       <c r="I662" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J662" t="s">
         <v>1862</v>
@@ -31649,7 +31652,7 @@
         <v>1616</v>
       </c>
       <c r="I663" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J663" t="s">
         <v>2414</v>
@@ -31722,7 +31725,7 @@
         <v>1607</v>
       </c>
       <c r="I665" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J665" t="s">
         <v>2416</v>
@@ -31976,7 +31979,7 @@
         <v>2568</v>
       </c>
       <c r="L672" t="s">
-        <v>2596</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="673" spans="1:12">
@@ -32008,7 +32011,7 @@
         <v>2568</v>
       </c>
       <c r="L673" t="s">
-        <v>2644</v>
+        <v>2645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-08 22:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7876,13 +7876,13 @@
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA FLORESTAL</t>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7909,10 +7909,10 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7936,7 +7936,7 @@
     <t>AVALIAÇÃO DE IMÓVEIS,URBANISMO</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,GEOTECNIA</t>
+    <t>GEOTECNIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,ENGENHARIA QUÍMICA,GEOLOGIA</t>
@@ -7945,13 +7945,13 @@
     <t>ASSISTÊNCIA SOCIAL,SAÚDE MENTAL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ECONOMIA,ASSISTÊNCIA SOCIAL,SAÚDE,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,URBANISMO,PSICOLOGIA,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS</t>
+    <t>PSICOLOGIA,SAÚDE,ECONOMICIDADE CONTÁBIL,SAÚDE MENTAL,URBANISMO,MOBILIDADE E TRANSPORTE,ECONOMIA,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,ASSISTÊNCIA SOCIAL</t>
   </si>
 </sst>
 </file>
@@ -31127,7 +31127,7 @@
         <v>2425</v>
       </c>
       <c r="L648" t="s">
-        <v>2606</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="649" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-09 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -19084,7 +19084,7 @@
     </row>
     <row r="307" spans="1:12">
       <c r="A307" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B307" t="s">
         <v>342</v>
@@ -19105,7 +19105,7 @@
         <v>1612</v>
       </c>
       <c r="I307" t="s">
-        <v>1689</v>
+        <v>1650</v>
       </c>
       <c r="J307" t="s">
         <v>2068</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-12 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -29991,7 +29991,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B620" t="s">
         <v>654</v>
@@ -30012,7 +30012,7 @@
         <v>1596</v>
       </c>
       <c r="I620" t="s">
-        <v>1692</v>
+        <v>1627</v>
       </c>
       <c r="J620" t="s">
         <v>2349</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-15 14:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5242,7 +5242,7 @@
     <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
-    <t>PATRICIA FONTES ESTEVES</t>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES, PATRICIA FONTES ESTEVES</t>
   </si>
   <si>
     <t>202200822461</t>
@@ -31411,7 +31411,7 @@
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B661" t="s">
         <v>697</v>
@@ -31426,7 +31426,7 @@
         <v>2</v>
       </c>
       <c r="F661" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="G661" t="s">
         <v>1599</v>
@@ -31470,7 +31470,7 @@
         <v>1597</v>
       </c>
       <c r="I662" t="s">
-        <v>1627</v>
+        <v>1741</v>
       </c>
       <c r="J662" t="s">
         <v>2388</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-16 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4873,189 +4873,192 @@
     <t>CELSO BARBOSA MONTENEGRO,PATRICIA PASSARO DA SILVA TOLEDO</t>
   </si>
   <si>
+    <t>EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>DAYSE BARBOSA DE ARAÚJO GÓIS,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
+    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA</t>
+  </si>
+  <si>
+    <t>DANIEL FONTANA OBERLING</t>
+  </si>
+  <si>
+    <t>MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>PATRICIA PASSARO DA SILVA TOLEDO</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
+  </si>
+  <si>
+    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
+  </si>
+  <si>
     <t>ROSEMARY PROVENZANO THAMI</t>
   </si>
   <si>
-    <t>EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>DAYSE BARBOSA DE ARAÚJO GÓIS,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER,SERGIO PEDRO LOPES,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI,MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>DANIEL FONTANA OBERLING</t>
-  </si>
-  <si>
-    <t>MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>PATRICIA PASSARO DA SILVA TOLEDO</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
-  </si>
-  <si>
-    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,RENATA PASCOAL FREIRE,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
-  </si>
-  <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER</t>
   </si>
   <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,RODRIGO VENTURA MARRA</t>
   </si>
   <si>
+    <t>DAGER SALLES AMARAL</t>
+  </si>
+  <si>
+    <t>ANA LÍCIA SOUZA E SILVA</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>NIVANA DANIELLE SILVA COSTA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
+  </si>
+  <si>
+    <t>RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI,HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>GLAUCO CASTILHO DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
+  </si>
+  <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
     <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
   </si>
   <si>
-    <t>ANA LÍCIA SOUZA E SILVA</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>NIVANA DANIELLE SILVA COSTA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI,HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
-    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
     <t>JOELSON SANTANA DE CARVALHO</t>
   </si>
   <si>
@@ -5099,9 +5102,6 @@
   </si>
   <si>
     <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
-    <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
   </si>
   <si>
     <t>RAQUEL SILVA FERNANDES LYRA</t>
@@ -9790,7 +9790,7 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B49" t="s">
         <v>84</v>
@@ -9811,7 +9811,7 @@
         <v>1575</v>
       </c>
       <c r="I49" t="s">
-        <v>1619</v>
+        <v>1606</v>
       </c>
       <c r="J49" t="s">
         <v>1772</v>
@@ -9881,7 +9881,7 @@
         <v>1575</v>
       </c>
       <c r="I51" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J51" t="s">
         <v>1774</v>
@@ -9986,7 +9986,7 @@
         <v>1575</v>
       </c>
       <c r="I54" t="s">
-        <v>1621</v>
+        <v>1620</v>
       </c>
       <c r="J54" t="s">
         <v>1777</v>
@@ -10024,7 +10024,7 @@
         <v>1396</v>
       </c>
       <c r="I55" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="J55" t="s">
         <v>1778</v>
@@ -10094,7 +10094,7 @@
         <v>1575</v>
       </c>
       <c r="I57" t="s">
-        <v>1623</v>
+        <v>1622</v>
       </c>
       <c r="J57" t="s">
         <v>1780</v>
@@ -10129,7 +10129,7 @@
         <v>1575</v>
       </c>
       <c r="I58" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="J58" t="s">
         <v>1781</v>
@@ -10237,7 +10237,7 @@
         <v>1575</v>
       </c>
       <c r="I61" t="s">
-        <v>1625</v>
+        <v>1624</v>
       </c>
       <c r="J61" t="s">
         <v>1784</v>
@@ -10272,7 +10272,7 @@
         <v>1575</v>
       </c>
       <c r="I62" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
       <c r="J62" t="s">
         <v>1785</v>
@@ -10377,7 +10377,7 @@
         <v>1575</v>
       </c>
       <c r="I65" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="J65" t="s">
         <v>1788</v>
@@ -10412,7 +10412,7 @@
         <v>1575</v>
       </c>
       <c r="I66" t="s">
-        <v>1628</v>
+        <v>1627</v>
       </c>
       <c r="J66" t="s">
         <v>1789</v>
@@ -10485,7 +10485,7 @@
         <v>1579</v>
       </c>
       <c r="I68" t="s">
-        <v>1629</v>
+        <v>1628</v>
       </c>
       <c r="J68" t="s">
         <v>1791</v>
@@ -10520,7 +10520,7 @@
         <v>1575</v>
       </c>
       <c r="I69" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J69" t="s">
         <v>1792</v>
@@ -10555,7 +10555,7 @@
         <v>1575</v>
       </c>
       <c r="I70" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J70" t="s">
         <v>1793</v>
@@ -10660,7 +10660,7 @@
         <v>1575</v>
       </c>
       <c r="I73" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="J73" t="s">
         <v>1796</v>
@@ -10695,7 +10695,7 @@
         <v>1575</v>
       </c>
       <c r="I74" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="J74" t="s">
         <v>1797</v>
@@ -10730,7 +10730,7 @@
         <v>1575</v>
       </c>
       <c r="I75" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="J75" t="s">
         <v>1797</v>
@@ -10870,7 +10870,7 @@
         <v>1575</v>
       </c>
       <c r="I79" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="J79" t="s">
         <v>1800</v>
@@ -10940,7 +10940,7 @@
         <v>1575</v>
       </c>
       <c r="I81" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="J81" t="s">
         <v>1802</v>
@@ -11115,7 +11115,7 @@
         <v>1575</v>
       </c>
       <c r="I86" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J86" t="s">
         <v>1807</v>
@@ -11185,7 +11185,7 @@
         <v>1575</v>
       </c>
       <c r="I88" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="J88" t="s">
         <v>1809</v>
@@ -11255,7 +11255,7 @@
         <v>1575</v>
       </c>
       <c r="I90" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="J90" t="s">
         <v>1811</v>
@@ -11360,7 +11360,7 @@
         <v>1575</v>
       </c>
       <c r="I93" t="s">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="J93" t="s">
         <v>1814</v>
@@ -11395,7 +11395,7 @@
         <v>1575</v>
       </c>
       <c r="I94" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="J94" t="s">
         <v>1815</v>
@@ -11430,7 +11430,7 @@
         <v>1575</v>
       </c>
       <c r="I95" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J95" t="s">
         <v>1816</v>
@@ -11465,7 +11465,7 @@
         <v>1575</v>
       </c>
       <c r="I96" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="J96" t="s">
         <v>1817</v>
@@ -11535,7 +11535,7 @@
         <v>1575</v>
       </c>
       <c r="I98" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="J98" t="s">
         <v>1819</v>
@@ -11570,7 +11570,7 @@
         <v>1575</v>
       </c>
       <c r="I99" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="J99" t="s">
         <v>1820</v>
@@ -11710,7 +11710,7 @@
         <v>1575</v>
       </c>
       <c r="I103" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J103" t="s">
         <v>1824</v>
@@ -11745,7 +11745,7 @@
         <v>1575</v>
       </c>
       <c r="I104" t="s">
-        <v>1643</v>
+        <v>1642</v>
       </c>
       <c r="J104" t="s">
         <v>1825</v>
@@ -11815,7 +11815,7 @@
         <v>1575</v>
       </c>
       <c r="I106" t="s">
-        <v>1644</v>
+        <v>1643</v>
       </c>
       <c r="J106" t="s">
         <v>1827</v>
@@ -11920,7 +11920,7 @@
         <v>1575</v>
       </c>
       <c r="I109" t="s">
-        <v>1645</v>
+        <v>1644</v>
       </c>
       <c r="J109" t="s">
         <v>1830</v>
@@ -11990,7 +11990,7 @@
         <v>1575</v>
       </c>
       <c r="I111" t="s">
-        <v>1646</v>
+        <v>1645</v>
       </c>
       <c r="J111" t="s">
         <v>1832</v>
@@ -12025,7 +12025,7 @@
         <v>1575</v>
       </c>
       <c r="I112" t="s">
-        <v>1647</v>
+        <v>1646</v>
       </c>
       <c r="J112" t="s">
         <v>1833</v>
@@ -12060,7 +12060,7 @@
         <v>1575</v>
       </c>
       <c r="I113" t="s">
-        <v>1648</v>
+        <v>1647</v>
       </c>
       <c r="J113" t="s">
         <v>1834</v>
@@ -12130,7 +12130,7 @@
         <v>1575</v>
       </c>
       <c r="I115" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="J115" t="s">
         <v>1836</v>
@@ -12203,7 +12203,7 @@
         <v>1580</v>
       </c>
       <c r="I117" t="s">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="J117" t="s">
         <v>1838</v>
@@ -12273,7 +12273,7 @@
         <v>1575</v>
       </c>
       <c r="I119" t="s">
-        <v>1650</v>
+        <v>1649</v>
       </c>
       <c r="J119" t="s">
         <v>1732</v>
@@ -12308,7 +12308,7 @@
         <v>1575</v>
       </c>
       <c r="I120" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="J120" t="s">
         <v>1840</v>
@@ -12518,7 +12518,7 @@
         <v>1575</v>
       </c>
       <c r="I126" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J126" t="s">
         <v>1845</v>
@@ -12553,7 +12553,7 @@
         <v>1575</v>
       </c>
       <c r="I127" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J127" t="s">
         <v>1846</v>
@@ -12588,7 +12588,7 @@
         <v>1575</v>
       </c>
       <c r="I128" t="s">
-        <v>1643</v>
+        <v>1642</v>
       </c>
       <c r="J128" t="s">
         <v>1847</v>
@@ -12623,7 +12623,7 @@
         <v>1575</v>
       </c>
       <c r="I129" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J129" t="s">
         <v>1848</v>
@@ -12661,7 +12661,7 @@
         <v>1581</v>
       </c>
       <c r="I130" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="J130" t="s">
         <v>1732</v>
@@ -12696,7 +12696,7 @@
         <v>1575</v>
       </c>
       <c r="I131" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J131" t="s">
         <v>1849</v>
@@ -12731,7 +12731,7 @@
         <v>1575</v>
       </c>
       <c r="I132" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="J132" t="s">
         <v>1850</v>
@@ -12801,7 +12801,7 @@
         <v>1575</v>
       </c>
       <c r="I134" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J134" t="s">
         <v>1852</v>
@@ -12871,7 +12871,7 @@
         <v>1575</v>
       </c>
       <c r="I136" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J136" t="s">
         <v>1854</v>
@@ -12976,7 +12976,7 @@
         <v>1575</v>
       </c>
       <c r="I139" t="s">
-        <v>1657</v>
+        <v>1656</v>
       </c>
       <c r="J139" t="s">
         <v>1857</v>
@@ -13011,7 +13011,7 @@
         <v>1575</v>
       </c>
       <c r="I140" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J140" t="s">
         <v>1858</v>
@@ -13081,7 +13081,7 @@
         <v>1575</v>
       </c>
       <c r="I142" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="J142" t="s">
         <v>1860</v>
@@ -13151,7 +13151,7 @@
         <v>1575</v>
       </c>
       <c r="I144" t="s">
-        <v>1619</v>
+        <v>1659</v>
       </c>
       <c r="J144" t="s">
         <v>1862</v>
@@ -13326,7 +13326,7 @@
         <v>1575</v>
       </c>
       <c r="I149" t="s">
-        <v>1619</v>
+        <v>1659</v>
       </c>
       <c r="J149" t="s">
         <v>1867</v>
@@ -13431,7 +13431,7 @@
         <v>1575</v>
       </c>
       <c r="I152" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J152" t="s">
         <v>1870</v>
@@ -13550,7 +13550,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B156" t="s">
         <v>191</v>
@@ -13606,7 +13606,7 @@
         <v>1575</v>
       </c>
       <c r="I157" t="s">
-        <v>1619</v>
+        <v>1659</v>
       </c>
       <c r="J157" t="s">
         <v>1875</v>
@@ -13711,7 +13711,7 @@
         <v>1575</v>
       </c>
       <c r="I160" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="J160" t="s">
         <v>1878</v>
@@ -14414,7 +14414,7 @@
         <v>1575</v>
       </c>
       <c r="I180" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J180" t="s">
         <v>1897</v>
@@ -14799,7 +14799,7 @@
         <v>1575</v>
       </c>
       <c r="I191" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J191" t="s">
         <v>1908</v>
@@ -15079,7 +15079,7 @@
         <v>1575</v>
       </c>
       <c r="I199" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J199" t="s">
         <v>1916</v>
@@ -15604,7 +15604,7 @@
         <v>1575</v>
       </c>
       <c r="I214" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J214" t="s">
         <v>1930</v>
@@ -15639,7 +15639,7 @@
         <v>1575</v>
       </c>
       <c r="I215" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J215" t="s">
         <v>1931</v>
@@ -16167,7 +16167,7 @@
         <v>1575</v>
       </c>
       <c r="I230" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J230" t="s">
         <v>1946</v>
@@ -16310,7 +16310,7 @@
         <v>1582</v>
       </c>
       <c r="I234" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J234" t="s">
         <v>1950</v>
@@ -16450,7 +16450,7 @@
         <v>1575</v>
       </c>
       <c r="I238" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J238" t="s">
         <v>1954</v>
@@ -16485,7 +16485,7 @@
         <v>1575</v>
       </c>
       <c r="I239" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J239" t="s">
         <v>1955</v>
@@ -16520,7 +16520,7 @@
         <v>1575</v>
       </c>
       <c r="I240" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J240" t="s">
         <v>1956</v>
@@ -16555,7 +16555,7 @@
         <v>1575</v>
       </c>
       <c r="I241" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J241" t="s">
         <v>1957</v>
@@ -16590,7 +16590,7 @@
         <v>1575</v>
       </c>
       <c r="I242" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="J242" t="s">
         <v>1958</v>
@@ -16765,7 +16765,7 @@
         <v>1575</v>
       </c>
       <c r="I247" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="J247" t="s">
         <v>1962</v>
@@ -16838,7 +16838,7 @@
         <v>1583</v>
       </c>
       <c r="I249" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="J249" t="s">
         <v>1964</v>
@@ -16978,7 +16978,7 @@
         <v>1575</v>
       </c>
       <c r="I253" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J253" t="s">
         <v>1967</v>
@@ -17013,7 +17013,7 @@
         <v>1575</v>
       </c>
       <c r="I254" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J254" t="s">
         <v>1968</v>
@@ -17258,7 +17258,7 @@
         <v>1575</v>
       </c>
       <c r="I261" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J261" t="s">
         <v>1975</v>
@@ -17293,7 +17293,7 @@
         <v>1575</v>
       </c>
       <c r="I262" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J262" t="s">
         <v>1976</v>
@@ -17398,7 +17398,7 @@
         <v>1575</v>
       </c>
       <c r="I265" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J265" t="s">
         <v>1979</v>
@@ -17611,7 +17611,7 @@
         <v>1575</v>
       </c>
       <c r="I271" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J271" t="s">
         <v>1985</v>
@@ -17821,7 +17821,7 @@
         <v>1575</v>
       </c>
       <c r="I277" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J277" t="s">
         <v>1991</v>
@@ -17926,7 +17926,7 @@
         <v>1575</v>
       </c>
       <c r="I280" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="J280" t="s">
         <v>1994</v>
@@ -18276,7 +18276,7 @@
         <v>1575</v>
       </c>
       <c r="I290" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J290" t="s">
         <v>2004</v>
@@ -18311,7 +18311,7 @@
         <v>1575</v>
       </c>
       <c r="I291" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J291" t="s">
         <v>2005</v>
@@ -18346,7 +18346,7 @@
         <v>1575</v>
       </c>
       <c r="I292" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J292" t="s">
         <v>2006</v>
@@ -18416,7 +18416,7 @@
         <v>1575</v>
       </c>
       <c r="I294" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J294" t="s">
         <v>2008</v>
@@ -18804,7 +18804,7 @@
         <v>1575</v>
       </c>
       <c r="I305" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J305" t="s">
         <v>2019</v>
@@ -18944,7 +18944,7 @@
         <v>1575</v>
       </c>
       <c r="I309" t="s">
-        <v>1657</v>
+        <v>1656</v>
       </c>
       <c r="J309" t="s">
         <v>2023</v>
@@ -18979,7 +18979,7 @@
         <v>1575</v>
       </c>
       <c r="I310" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J310" t="s">
         <v>2024</v>
@@ -19052,7 +19052,7 @@
         <v>1512</v>
       </c>
       <c r="I312" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="J312" t="s">
         <v>2026</v>
@@ -19087,7 +19087,7 @@
         <v>1575</v>
       </c>
       <c r="I313" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J313" t="s">
         <v>2027</v>
@@ -19157,7 +19157,7 @@
         <v>1575</v>
       </c>
       <c r="I315" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J315" t="s">
         <v>2029</v>
@@ -19227,7 +19227,7 @@
         <v>1575</v>
       </c>
       <c r="I317" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J317" t="s">
         <v>2031</v>
@@ -19367,7 +19367,7 @@
         <v>1575</v>
       </c>
       <c r="I321" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J321" t="s">
         <v>2035</v>
@@ -19437,7 +19437,7 @@
         <v>1575</v>
       </c>
       <c r="I323" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J323" t="s">
         <v>2037</v>
@@ -19647,7 +19647,7 @@
         <v>1575</v>
       </c>
       <c r="I329" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J329" t="s">
         <v>2043</v>
@@ -19787,7 +19787,7 @@
         <v>1575</v>
       </c>
       <c r="I333" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J333" t="s">
         <v>2047</v>
@@ -20277,7 +20277,7 @@
         <v>1575</v>
       </c>
       <c r="I347" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J347" t="s">
         <v>2060</v>
@@ -20382,7 +20382,7 @@
         <v>1575</v>
       </c>
       <c r="I350" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J350" t="s">
         <v>2063</v>
@@ -20431,7 +20431,7 @@
     </row>
     <row r="352" spans="1:12">
       <c r="A352" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B352" t="s">
         <v>387</v>
@@ -20452,7 +20452,7 @@
         <v>1575</v>
       </c>
       <c r="I352" t="s">
-        <v>1695</v>
+        <v>1606</v>
       </c>
       <c r="J352" t="s">
         <v>2065</v>
@@ -20592,7 +20592,7 @@
         <v>1575</v>
       </c>
       <c r="I356" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J356" t="s">
         <v>2068</v>
@@ -20662,7 +20662,7 @@
         <v>1575</v>
       </c>
       <c r="I358" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J358" t="s">
         <v>2070</v>
@@ -20767,7 +20767,7 @@
         <v>1575</v>
       </c>
       <c r="I361" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J361" t="s">
         <v>2073</v>
@@ -20977,7 +20977,7 @@
         <v>1575</v>
       </c>
       <c r="I367" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J367" t="s">
         <v>2079</v>
@@ -21152,7 +21152,7 @@
         <v>1575</v>
       </c>
       <c r="I372" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J372" t="s">
         <v>2084</v>
@@ -21292,7 +21292,7 @@
         <v>1575</v>
       </c>
       <c r="I376" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J376" t="s">
         <v>2088</v>
@@ -21397,7 +21397,7 @@
         <v>1575</v>
       </c>
       <c r="I379" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J379" t="s">
         <v>2091</v>
@@ -21712,7 +21712,7 @@
         <v>1575</v>
       </c>
       <c r="I388" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J388" t="s">
         <v>2100</v>
@@ -21747,7 +21747,7 @@
         <v>1575</v>
       </c>
       <c r="I389" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J389" t="s">
         <v>2101</v>
@@ -21817,7 +21817,7 @@
         <v>1575</v>
       </c>
       <c r="I391" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J391" t="s">
         <v>2103</v>
@@ -22307,7 +22307,7 @@
         <v>1575</v>
       </c>
       <c r="I405" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J405" t="s">
         <v>2117</v>
@@ -22517,7 +22517,7 @@
         <v>1575</v>
       </c>
       <c r="I411" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J411" t="s">
         <v>2123</v>
@@ -22657,7 +22657,7 @@
         <v>1575</v>
       </c>
       <c r="I415" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J415" t="s">
         <v>2127</v>
@@ -22692,7 +22692,7 @@
         <v>1575</v>
       </c>
       <c r="I416" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J416" t="s">
         <v>2128</v>
@@ -22867,7 +22867,7 @@
         <v>1575</v>
       </c>
       <c r="I421" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="J421" t="s">
         <v>2133</v>
@@ -22902,7 +22902,7 @@
         <v>1575</v>
       </c>
       <c r="I422" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J422" t="s">
         <v>2134</v>
@@ -22937,7 +22937,7 @@
         <v>1575</v>
       </c>
       <c r="I423" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J423" t="s">
         <v>2135</v>
@@ -23217,7 +23217,7 @@
         <v>1575</v>
       </c>
       <c r="I431" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J431" t="s">
         <v>2143</v>
@@ -23602,7 +23602,7 @@
         <v>1575</v>
       </c>
       <c r="I442" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J442" t="s">
         <v>2154</v>
@@ -23742,7 +23742,7 @@
         <v>1575</v>
       </c>
       <c r="I446" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J446" t="s">
         <v>2158</v>
@@ -23777,7 +23777,7 @@
         <v>1575</v>
       </c>
       <c r="I447" t="s">
-        <v>1621</v>
+        <v>1620</v>
       </c>
       <c r="J447" t="s">
         <v>2159</v>
@@ -23812,7 +23812,7 @@
         <v>1575</v>
       </c>
       <c r="I448" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J448" t="s">
         <v>2160</v>
@@ -23882,7 +23882,7 @@
         <v>1575</v>
       </c>
       <c r="I450" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J450" t="s">
         <v>2162</v>
@@ -23952,7 +23952,7 @@
         <v>1575</v>
       </c>
       <c r="I452" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J452" t="s">
         <v>2164</v>
@@ -24305,7 +24305,7 @@
         <v>1575</v>
       </c>
       <c r="I462" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J462" t="s">
         <v>2174</v>
@@ -24585,7 +24585,7 @@
         <v>1575</v>
       </c>
       <c r="I470" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J470" t="s">
         <v>2182</v>
@@ -24763,7 +24763,7 @@
         <v>1575</v>
       </c>
       <c r="I475" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J475" t="s">
         <v>2187</v>
@@ -24903,7 +24903,7 @@
         <v>1575</v>
       </c>
       <c r="I479" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J479" t="s">
         <v>2191</v>
@@ -25148,7 +25148,7 @@
         <v>1575</v>
       </c>
       <c r="I486" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J486" t="s">
         <v>2198</v>
@@ -25183,7 +25183,7 @@
         <v>1575</v>
       </c>
       <c r="I487" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J487" t="s">
         <v>2199</v>
@@ -25253,7 +25253,7 @@
         <v>1575</v>
       </c>
       <c r="I489" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J489" t="s">
         <v>2201</v>
@@ -25288,7 +25288,7 @@
         <v>1575</v>
       </c>
       <c r="I490" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J490" t="s">
         <v>2202</v>
@@ -25323,7 +25323,7 @@
         <v>1575</v>
       </c>
       <c r="I491" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J491" t="s">
         <v>2203</v>
@@ -25358,7 +25358,7 @@
         <v>1575</v>
       </c>
       <c r="I492" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J492" t="s">
         <v>2204</v>
@@ -25428,7 +25428,7 @@
         <v>1575</v>
       </c>
       <c r="I494" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J494" t="s">
         <v>2206</v>
@@ -25641,7 +25641,7 @@
         <v>1588</v>
       </c>
       <c r="I500" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J500" t="s">
         <v>2212</v>
@@ -25854,7 +25854,7 @@
         <v>1589</v>
       </c>
       <c r="I506" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="J506" t="s">
         <v>2218</v>
@@ -25889,7 +25889,7 @@
         <v>1575</v>
       </c>
       <c r="I507" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J507" t="s">
         <v>2219</v>
@@ -25994,7 +25994,7 @@
         <v>1575</v>
       </c>
       <c r="I510" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J510" t="s">
         <v>2222</v>
@@ -26029,7 +26029,7 @@
         <v>1575</v>
       </c>
       <c r="I511" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J511" t="s">
         <v>2223</v>
@@ -26064,7 +26064,7 @@
         <v>1575</v>
       </c>
       <c r="I512" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J512" t="s">
         <v>2224</v>
@@ -26099,7 +26099,7 @@
         <v>1575</v>
       </c>
       <c r="I513" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J513" t="s">
         <v>2225</v>
@@ -26204,7 +26204,7 @@
         <v>1575</v>
       </c>
       <c r="I516" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J516" t="s">
         <v>2228</v>
@@ -26239,7 +26239,7 @@
         <v>1575</v>
       </c>
       <c r="I517" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J517" t="s">
         <v>2229</v>
@@ -26449,7 +26449,7 @@
         <v>1575</v>
       </c>
       <c r="I523" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J523" t="s">
         <v>2235</v>
@@ -26519,7 +26519,7 @@
         <v>1575</v>
       </c>
       <c r="I525" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J525" t="s">
         <v>2237</v>
@@ -26802,7 +26802,7 @@
         <v>1575</v>
       </c>
       <c r="I533" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J533" t="s">
         <v>2245</v>
@@ -27012,7 +27012,7 @@
         <v>1575</v>
       </c>
       <c r="I539" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J539" t="s">
         <v>2251</v>
@@ -27117,7 +27117,7 @@
         <v>1575</v>
       </c>
       <c r="I542" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J542" t="s">
         <v>2254</v>
@@ -27190,7 +27190,7 @@
         <v>1575</v>
       </c>
       <c r="I544" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J544" t="s">
         <v>2256</v>
@@ -27260,7 +27260,7 @@
         <v>1575</v>
       </c>
       <c r="I546" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J546" t="s">
         <v>2258</v>
@@ -27330,7 +27330,7 @@
         <v>1575</v>
       </c>
       <c r="I548" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J548" t="s">
         <v>2260</v>
@@ -27578,7 +27578,7 @@
         <v>1575</v>
       </c>
       <c r="I555" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J555" t="s">
         <v>2267</v>
@@ -27972,7 +27972,7 @@
         <v>1575</v>
       </c>
       <c r="I566" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J566" t="s">
         <v>2278</v>
@@ -27986,7 +27986,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B567" t="s">
         <v>602</v>
@@ -28001,13 +28001,13 @@
         <v>25</v>
       </c>
       <c r="F567" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="G567" t="s">
         <v>1575</v>
       </c>
       <c r="I567" t="s">
-        <v>1695</v>
+        <v>1606</v>
       </c>
       <c r="J567" t="s">
         <v>2279</v>
@@ -28147,7 +28147,7 @@
         <v>1575</v>
       </c>
       <c r="I571" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J571" t="s">
         <v>2283</v>
@@ -28287,7 +28287,7 @@
         <v>1575</v>
       </c>
       <c r="I575" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J575" t="s">
         <v>2287</v>
@@ -28611,7 +28611,7 @@
         <v>1575</v>
       </c>
       <c r="I584" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J584" t="s">
         <v>2296</v>
@@ -28646,7 +28646,7 @@
         <v>1575</v>
       </c>
       <c r="I585" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J585" t="s">
         <v>2297</v>
@@ -28765,7 +28765,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B589" t="s">
         <v>624</v>
@@ -28780,7 +28780,7 @@
         <v>19</v>
       </c>
       <c r="F589" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="G589" t="s">
         <v>1577</v>
@@ -28789,7 +28789,7 @@
         <v>1594</v>
       </c>
       <c r="I589" t="s">
-        <v>1662</v>
+        <v>1606</v>
       </c>
       <c r="J589" t="s">
         <v>2301</v>
@@ -29116,7 +29116,7 @@
         <v>1575</v>
       </c>
       <c r="I598" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J598" t="s">
         <v>2310</v>
@@ -29130,7 +29130,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B599" t="s">
         <v>634</v>
@@ -29151,7 +29151,7 @@
         <v>1575</v>
       </c>
       <c r="I599" t="s">
-        <v>1696</v>
+        <v>1676</v>
       </c>
       <c r="J599" t="s">
         <v>2311</v>
@@ -29186,7 +29186,7 @@
         <v>1575</v>
       </c>
       <c r="I600" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J600" t="s">
         <v>2312</v>
@@ -29221,7 +29221,7 @@
         <v>1575</v>
       </c>
       <c r="I601" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J601" t="s">
         <v>2313</v>
@@ -29256,7 +29256,7 @@
         <v>1575</v>
       </c>
       <c r="I602" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J602" t="s">
         <v>2314</v>
@@ -29326,7 +29326,7 @@
         <v>1575</v>
       </c>
       <c r="I604" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J604" t="s">
         <v>2316</v>
@@ -29717,7 +29717,7 @@
         <v>1575</v>
       </c>
       <c r="I615" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J615" t="s">
         <v>2327</v>
@@ -29752,7 +29752,7 @@
         <v>1575</v>
       </c>
       <c r="I616" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J616" t="s">
         <v>2328</v>
@@ -29895,7 +29895,7 @@
         <v>1575</v>
       </c>
       <c r="I620" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J620" t="s">
         <v>2331</v>
@@ -30000,7 +30000,7 @@
         <v>1575</v>
       </c>
       <c r="I623" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J623" t="s">
         <v>2334</v>
@@ -30105,7 +30105,7 @@
         <v>1575</v>
       </c>
       <c r="I626" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J626" t="s">
         <v>2337</v>
@@ -30210,7 +30210,7 @@
         <v>1575</v>
       </c>
       <c r="I629" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J629" t="s">
         <v>2340</v>
@@ -30297,7 +30297,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B632" t="s">
         <v>667</v>
@@ -30312,13 +30312,13 @@
         <v>6</v>
       </c>
       <c r="F632" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="G632" t="s">
         <v>1575</v>
       </c>
       <c r="I632" t="s">
-        <v>1662</v>
+        <v>1606</v>
       </c>
       <c r="J632" t="s">
         <v>2343</v>
@@ -30388,7 +30388,7 @@
         <v>1575</v>
       </c>
       <c r="I634" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J634" t="s">
         <v>2345</v>
@@ -30458,7 +30458,7 @@
         <v>1575</v>
       </c>
       <c r="I636" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J636" t="s">
         <v>2347</v>
@@ -30493,7 +30493,7 @@
         <v>1575</v>
       </c>
       <c r="I637" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J637" t="s">
         <v>2348</v>
@@ -30563,7 +30563,7 @@
         <v>1575</v>
       </c>
       <c r="I639" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J639" t="s">
         <v>2350</v>
@@ -30668,7 +30668,7 @@
         <v>1575</v>
       </c>
       <c r="I642" t="s">
-        <v>1662</v>
+        <v>1680</v>
       </c>
       <c r="J642" t="s">
         <v>2353</v>
@@ -30738,7 +30738,7 @@
         <v>1575</v>
       </c>
       <c r="I644" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J644" t="s">
         <v>1852</v>
@@ -30846,7 +30846,7 @@
         <v>1575</v>
       </c>
       <c r="I647" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J647" t="s">
         <v>2357</v>
@@ -31059,7 +31059,7 @@
         <v>1575</v>
       </c>
       <c r="I653" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J653" t="s">
         <v>2362</v>
@@ -31091,7 +31091,7 @@
         <v>1575</v>
       </c>
       <c r="I654" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J654" t="s">
         <v>2363</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-18 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -16623,7 +16623,7 @@
     </row>
     <row r="242" spans="1:12">
       <c r="A242" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="B242" t="s">
         <v>279</v>
@@ -16647,7 +16647,7 @@
         <v>1590</v>
       </c>
       <c r="I242" t="s">
-        <v>1650</v>
+        <v>1618</v>
       </c>
       <c r="J242" t="s">
         <v>1972</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-25 08:30:01
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6636" uniqueCount="2585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6636" uniqueCount="2582">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7639,6 +7639,9 @@
     <t>ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
+    <t>### SEM TEMA ###</t>
+  </si>
+  <si>
     <t>ENGENHARIA QUÍMICA</t>
   </si>
   <si>
@@ -7681,9 +7684,6 @@
     <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
     <t>FARMÁCIA</t>
   </si>
   <si>
@@ -7696,7 +7696,7 @@
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
+    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7732,13 +7732,13 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>URBANISMO,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,ENGENHARIA FLORESTAL,GEOTECNIA,BIOLOGIA,RESÍDUOS SÓLIDOS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>RECURSOS HÍDRICOS,URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,BIOLOGIA,GEOTECNIA,ENGENHARIA FLORESTAL,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
@@ -7756,19 +7756,10 @@
     <t>ASSISTÊNCIA SOCIAL,SAÚDE MENTAL</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,GEOTECNIA</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,URBANISMO,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL,SAÚDE,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,ORÇAMENTO,ECONOMIA,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
 </sst>
 </file>
@@ -11921,7 +11912,7 @@
         <v>2409</v>
       </c>
       <c r="L108" t="s">
-        <v>2531</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="109" spans="1:12">
@@ -11991,7 +11982,7 @@
         <v>2377</v>
       </c>
       <c r="L110" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="111" spans="1:12">
@@ -12236,7 +12227,7 @@
         <v>2419</v>
       </c>
       <c r="L117" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="118" spans="1:12">
@@ -12271,7 +12262,7 @@
         <v>2427</v>
       </c>
       <c r="L118" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="119" spans="1:12">
@@ -12449,7 +12440,7 @@
         <v>2387</v>
       </c>
       <c r="L123" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="124" spans="1:12">
@@ -12519,7 +12510,7 @@
         <v>2395</v>
       </c>
       <c r="L125" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="126" spans="1:12">
@@ -12694,7 +12685,7 @@
         <v>2427</v>
       </c>
       <c r="L130" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="131" spans="1:12">
@@ -13149,7 +13140,7 @@
         <v>2418</v>
       </c>
       <c r="L143" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="144" spans="1:12">
@@ -13324,7 +13315,7 @@
         <v>2426</v>
       </c>
       <c r="L148" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="149" spans="1:12">
@@ -13639,7 +13630,7 @@
         <v>2390</v>
       </c>
       <c r="L157" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="158" spans="1:12">
@@ -13779,7 +13770,7 @@
         <v>2445</v>
       </c>
       <c r="L161" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="162" spans="1:12">
@@ -13919,7 +13910,7 @@
         <v>2385</v>
       </c>
       <c r="L165" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="166" spans="1:12">
@@ -14132,7 +14123,7 @@
         <v>2426</v>
       </c>
       <c r="L171" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="172" spans="1:12">
@@ -14307,7 +14298,7 @@
         <v>2437</v>
       </c>
       <c r="L176" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="177" spans="1:12">
@@ -14447,7 +14438,7 @@
         <v>2387</v>
       </c>
       <c r="L180" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="181" spans="1:12">
@@ -14587,7 +14578,7 @@
         <v>2404</v>
       </c>
       <c r="L184" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="185" spans="1:12">
@@ -14937,7 +14928,7 @@
         <v>2407</v>
       </c>
       <c r="L194" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -15042,7 +15033,7 @@
         <v>2426</v>
       </c>
       <c r="L197" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -15147,7 +15138,7 @@
         <v>2451</v>
       </c>
       <c r="L200" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -15182,7 +15173,7 @@
         <v>2385</v>
       </c>
       <c r="L201" t="s">
-        <v>2552</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -15252,7 +15243,7 @@
         <v>2395</v>
       </c>
       <c r="L203" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="204" spans="1:12">
@@ -15290,7 +15281,7 @@
         <v>2378</v>
       </c>
       <c r="L204" t="s">
-        <v>2515</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="205" spans="1:12">
@@ -15570,7 +15561,7 @@
         <v>2452</v>
       </c>
       <c r="L212" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="213" spans="1:12">
@@ -15640,7 +15631,7 @@
         <v>2397</v>
       </c>
       <c r="L214" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="215" spans="1:12">
@@ -15783,7 +15774,7 @@
         <v>2454</v>
       </c>
       <c r="L218" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="219" spans="1:12">
@@ -15923,7 +15914,7 @@
         <v>2455</v>
       </c>
       <c r="L222" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="223" spans="1:12">
@@ -16028,7 +16019,7 @@
         <v>2409</v>
       </c>
       <c r="L225" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="226" spans="1:12">
@@ -16063,7 +16054,7 @@
         <v>2456</v>
       </c>
       <c r="L226" t="s">
-        <v>2553</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="227" spans="1:12">
@@ -16098,7 +16089,7 @@
         <v>2391</v>
       </c>
       <c r="L227" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="228" spans="1:12">
@@ -16203,7 +16194,7 @@
         <v>2457</v>
       </c>
       <c r="L230" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="231" spans="1:12">
@@ -16658,7 +16649,7 @@
         <v>2462</v>
       </c>
       <c r="L243" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="244" spans="1:12">
@@ -16693,7 +16684,7 @@
         <v>2453</v>
       </c>
       <c r="L244" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="245" spans="1:12">
@@ -16798,7 +16789,7 @@
         <v>2416</v>
       </c>
       <c r="L247" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="248" spans="1:12">
@@ -16833,7 +16824,7 @@
         <v>2463</v>
       </c>
       <c r="L248" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="249" spans="1:12">
@@ -16938,7 +16929,7 @@
         <v>2465</v>
       </c>
       <c r="L251" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="252" spans="1:12">
@@ -17011,7 +17002,7 @@
         <v>2419</v>
       </c>
       <c r="L253" t="s">
-        <v>2555</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="254" spans="1:12">
@@ -17221,7 +17212,7 @@
         <v>2390</v>
       </c>
       <c r="L259" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="260" spans="1:12">
@@ -17256,7 +17247,7 @@
         <v>2462</v>
       </c>
       <c r="L260" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="261" spans="1:12">
@@ -17361,7 +17352,7 @@
         <v>2466</v>
       </c>
       <c r="L263" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="264" spans="1:12">
@@ -17501,7 +17492,7 @@
         <v>2390</v>
       </c>
       <c r="L267" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="268" spans="1:12">
@@ -17746,7 +17737,7 @@
         <v>2395</v>
       </c>
       <c r="L274" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="275" spans="1:12">
@@ -17781,7 +17772,7 @@
         <v>2437</v>
       </c>
       <c r="L275" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -17889,7 +17880,7 @@
         <v>2386</v>
       </c>
       <c r="L278" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="279" spans="1:12">
@@ -17924,7 +17915,7 @@
         <v>2469</v>
       </c>
       <c r="L279" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="280" spans="1:12">
@@ -18029,7 +18020,7 @@
         <v>2432</v>
       </c>
       <c r="L282" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="283" spans="1:12">
@@ -18134,7 +18125,7 @@
         <v>2471</v>
       </c>
       <c r="L285" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="286" spans="1:12">
@@ -18204,7 +18195,7 @@
         <v>2440</v>
       </c>
       <c r="L287" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -18239,7 +18230,7 @@
         <v>2455</v>
       </c>
       <c r="L288" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="289" spans="1:12">
@@ -18274,7 +18265,7 @@
         <v>2455</v>
       </c>
       <c r="L289" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="290" spans="1:12">
@@ -18309,7 +18300,7 @@
         <v>2417</v>
       </c>
       <c r="L290" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="291" spans="1:12">
@@ -18417,7 +18408,7 @@
         <v>2390</v>
       </c>
       <c r="L293" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="294" spans="1:12">
@@ -18592,7 +18583,7 @@
         <v>2465</v>
       </c>
       <c r="L298" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="299" spans="1:12">
@@ -18977,7 +18968,7 @@
         <v>2468</v>
       </c>
       <c r="L309" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="310" spans="1:12">
@@ -19082,7 +19073,7 @@
         <v>2376</v>
       </c>
       <c r="L312" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="313" spans="1:12">
@@ -19537,7 +19528,7 @@
         <v>2379</v>
       </c>
       <c r="L325" t="s">
-        <v>2522</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="326" spans="1:12">
@@ -19572,7 +19563,7 @@
         <v>2379</v>
       </c>
       <c r="L326" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="327" spans="1:12">
@@ -19782,7 +19773,7 @@
         <v>2398</v>
       </c>
       <c r="L332" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="333" spans="1:12">
@@ -19852,7 +19843,7 @@
         <v>2422</v>
       </c>
       <c r="L334" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="335" spans="1:12">
@@ -19957,7 +19948,7 @@
         <v>2395</v>
       </c>
       <c r="L337" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="338" spans="1:12">
@@ -20167,7 +20158,7 @@
         <v>2395</v>
       </c>
       <c r="L343" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="344" spans="1:12">
@@ -20202,7 +20193,7 @@
         <v>2390</v>
       </c>
       <c r="L344" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="345" spans="1:12">
@@ -20272,7 +20263,7 @@
         <v>2479</v>
       </c>
       <c r="L346" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="347" spans="1:12">
@@ -20517,7 +20508,7 @@
         <v>2481</v>
       </c>
       <c r="L353" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="354" spans="1:12">
@@ -20692,7 +20683,7 @@
         <v>2418</v>
       </c>
       <c r="L358" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20797,7 +20788,7 @@
         <v>2398</v>
       </c>
       <c r="L361" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="362" spans="1:12">
@@ -20902,7 +20893,7 @@
         <v>2461</v>
       </c>
       <c r="L364" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="365" spans="1:12">
@@ -20972,7 +20963,7 @@
         <v>2378</v>
       </c>
       <c r="L366" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="367" spans="1:12">
@@ -21287,7 +21278,7 @@
         <v>2467</v>
       </c>
       <c r="L375" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="376" spans="1:12">
@@ -21462,7 +21453,7 @@
         <v>2375</v>
       </c>
       <c r="L380" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="381" spans="1:12">
@@ -21497,7 +21488,7 @@
         <v>2395</v>
       </c>
       <c r="L381" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="382" spans="1:12">
@@ -21672,7 +21663,7 @@
         <v>2436</v>
       </c>
       <c r="L386" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="387" spans="1:12">
@@ -21707,7 +21698,7 @@
         <v>2422</v>
       </c>
       <c r="L387" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="388" spans="1:12">
@@ -21777,7 +21768,7 @@
         <v>2484</v>
       </c>
       <c r="L389" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="390" spans="1:12">
@@ -21847,7 +21838,7 @@
         <v>2395</v>
       </c>
       <c r="L391" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="392" spans="1:12">
@@ -21952,7 +21943,7 @@
         <v>2440</v>
       </c>
       <c r="L394" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="395" spans="1:12">
@@ -21987,7 +21978,7 @@
         <v>2465</v>
       </c>
       <c r="L395" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="396" spans="1:12">
@@ -22022,7 +22013,7 @@
         <v>2485</v>
       </c>
       <c r="L396" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="397" spans="1:12">
@@ -22337,7 +22328,7 @@
         <v>2417</v>
       </c>
       <c r="L405" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="406" spans="1:12">
@@ -22512,7 +22503,7 @@
         <v>2433</v>
       </c>
       <c r="L410" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="411" spans="1:12">
@@ -22722,7 +22713,7 @@
         <v>2436</v>
       </c>
       <c r="L416" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="417" spans="1:12">
@@ -23142,7 +23133,7 @@
         <v>2453</v>
       </c>
       <c r="L428" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="429" spans="1:12">
@@ -23282,7 +23273,7 @@
         <v>2373</v>
       </c>
       <c r="L432" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="433" spans="1:12">
@@ -23457,7 +23448,7 @@
         <v>2440</v>
       </c>
       <c r="L437" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="438" spans="1:12">
@@ -23527,7 +23518,7 @@
         <v>2416</v>
       </c>
       <c r="L439" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="440" spans="1:12">
@@ -23562,7 +23553,7 @@
         <v>2479</v>
       </c>
       <c r="L440" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="441" spans="1:12">
@@ -23632,7 +23623,7 @@
         <v>2479</v>
       </c>
       <c r="L442" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="443" spans="1:12">
@@ -23845,7 +23836,7 @@
         <v>2407</v>
       </c>
       <c r="L448" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="449" spans="1:12">
@@ -23915,7 +23906,7 @@
         <v>2440</v>
       </c>
       <c r="L450" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="451" spans="1:12">
@@ -24195,7 +24186,7 @@
         <v>2395</v>
       </c>
       <c r="L458" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24230,7 +24221,7 @@
         <v>2478</v>
       </c>
       <c r="L459" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="460" spans="1:12">
@@ -24335,7 +24326,7 @@
         <v>2421</v>
       </c>
       <c r="L462" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="463" spans="1:12">
@@ -24475,7 +24466,7 @@
         <v>2496</v>
       </c>
       <c r="L466" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="467" spans="1:12">
@@ -24545,7 +24536,7 @@
         <v>2422</v>
       </c>
       <c r="L468" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="469" spans="1:12">
@@ -24618,7 +24609,7 @@
         <v>2399</v>
       </c>
       <c r="L470" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="471" spans="1:12">
@@ -24688,7 +24679,7 @@
         <v>2395</v>
       </c>
       <c r="L472" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="473" spans="1:12">
@@ -24723,7 +24714,7 @@
         <v>2395</v>
       </c>
       <c r="L473" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="474" spans="1:12">
@@ -24796,7 +24787,7 @@
         <v>2421</v>
       </c>
       <c r="L475" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="476" spans="1:12">
@@ -24971,7 +24962,7 @@
         <v>2432</v>
       </c>
       <c r="L480" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="481" spans="1:12">
@@ -25006,7 +24997,7 @@
         <v>2432</v>
       </c>
       <c r="L481" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="482" spans="1:12">
@@ -25041,7 +25032,7 @@
         <v>2432</v>
       </c>
       <c r="L482" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="483" spans="1:12">
@@ -25076,7 +25067,7 @@
         <v>2498</v>
       </c>
       <c r="L483" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="484" spans="1:12">
@@ -25216,7 +25207,7 @@
         <v>2499</v>
       </c>
       <c r="L487" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="488" spans="1:12">
@@ -25251,7 +25242,7 @@
         <v>2378</v>
       </c>
       <c r="L488" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="489" spans="1:12">
@@ -25286,7 +25277,7 @@
         <v>2499</v>
       </c>
       <c r="L489" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="490" spans="1:12">
@@ -25321,7 +25312,7 @@
         <v>2390</v>
       </c>
       <c r="L490" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="491" spans="1:12">
@@ -25461,7 +25452,7 @@
         <v>2390</v>
       </c>
       <c r="L494" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="495" spans="1:12">
@@ -25531,7 +25522,7 @@
         <v>2410</v>
       </c>
       <c r="L496" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="497" spans="1:12">
@@ -25706,7 +25697,7 @@
         <v>2422</v>
       </c>
       <c r="L501" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="502" spans="1:12">
@@ -25776,7 +25767,7 @@
         <v>2391</v>
       </c>
       <c r="L503" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -25954,7 +25945,7 @@
         <v>2498</v>
       </c>
       <c r="L508" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="509" spans="1:12">
@@ -26024,7 +26015,7 @@
         <v>2481</v>
       </c>
       <c r="L510" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="511" spans="1:12">
@@ -26059,7 +26050,7 @@
         <v>2453</v>
       </c>
       <c r="L511" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="512" spans="1:12">
@@ -26132,7 +26123,7 @@
         <v>2433</v>
       </c>
       <c r="L513" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="514" spans="1:12">
@@ -26167,7 +26158,7 @@
         <v>2395</v>
       </c>
       <c r="L514" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="515" spans="1:12">
@@ -26307,7 +26298,7 @@
         <v>2497</v>
       </c>
       <c r="L518" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="519" spans="1:12">
@@ -26415,7 +26406,7 @@
         <v>2437</v>
       </c>
       <c r="L521" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="522" spans="1:12">
@@ -26555,7 +26546,7 @@
         <v>2409</v>
       </c>
       <c r="L525" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="526" spans="1:12">
@@ -26625,7 +26616,7 @@
         <v>2497</v>
       </c>
       <c r="L527" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="528" spans="1:12">
@@ -26695,7 +26686,7 @@
         <v>2395</v>
       </c>
       <c r="L529" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="530" spans="1:12">
@@ -26765,7 +26756,7 @@
         <v>2398</v>
       </c>
       <c r="L531" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="532" spans="1:12">
@@ -26870,7 +26861,7 @@
         <v>2399</v>
       </c>
       <c r="L534" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="535" spans="1:12">
@@ -27048,7 +27039,7 @@
         <v>2469</v>
       </c>
       <c r="L539" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="540" spans="1:12">
@@ -27086,7 +27077,7 @@
         <v>2469</v>
       </c>
       <c r="L540" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27121,7 +27112,7 @@
         <v>2395</v>
       </c>
       <c r="L541" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="542" spans="1:12">
@@ -27191,7 +27182,7 @@
         <v>2453</v>
       </c>
       <c r="L543" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="544" spans="1:12">
@@ -27226,7 +27217,7 @@
         <v>2398</v>
       </c>
       <c r="L544" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="545" spans="1:12">
@@ -27261,7 +27252,7 @@
         <v>2379</v>
       </c>
       <c r="L545" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="546" spans="1:12">
@@ -27369,7 +27360,7 @@
         <v>2409</v>
       </c>
       <c r="L548" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="549" spans="1:12">
@@ -27620,7 +27611,7 @@
         <v>2373</v>
       </c>
       <c r="L555" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="556" spans="1:12">
@@ -27655,7 +27646,7 @@
         <v>2462</v>
       </c>
       <c r="L556" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="557" spans="1:12">
@@ -27690,7 +27681,7 @@
         <v>2468</v>
       </c>
       <c r="L557" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="558" spans="1:12">
@@ -27725,7 +27716,7 @@
         <v>2374</v>
       </c>
       <c r="L558" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="559" spans="1:12">
@@ -27760,7 +27751,7 @@
         <v>2374</v>
       </c>
       <c r="L559" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="560" spans="1:12">
@@ -27795,7 +27786,7 @@
         <v>2398</v>
       </c>
       <c r="L560" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="561" spans="1:12">
@@ -27830,7 +27821,7 @@
         <v>2497</v>
       </c>
       <c r="L561" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="562" spans="1:12">
@@ -28075,7 +28066,7 @@
         <v>2422</v>
       </c>
       <c r="L568" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="569" spans="1:12">
@@ -28110,7 +28101,7 @@
         <v>2382</v>
       </c>
       <c r="L569" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -28145,7 +28136,7 @@
         <v>2478</v>
       </c>
       <c r="L570" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28285,7 +28276,7 @@
         <v>2422</v>
       </c>
       <c r="L574" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="575" spans="1:12">
@@ -28355,7 +28346,7 @@
         <v>2407</v>
       </c>
       <c r="L576" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="577" spans="1:12">
@@ -28495,7 +28486,7 @@
         <v>2494</v>
       </c>
       <c r="L580" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28708,7 +28699,7 @@
         <v>2421</v>
       </c>
       <c r="L586" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28743,7 +28734,7 @@
         <v>2421</v>
       </c>
       <c r="L587" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="588" spans="1:12">
@@ -28918,7 +28909,7 @@
         <v>2410</v>
       </c>
       <c r="L592" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="593" spans="1:12">
@@ -28953,7 +28944,7 @@
         <v>2395</v>
       </c>
       <c r="L593" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -28988,7 +28979,7 @@
         <v>2395</v>
       </c>
       <c r="L594" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -29023,7 +29014,7 @@
         <v>2455</v>
       </c>
       <c r="L595" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -29058,7 +29049,7 @@
         <v>2485</v>
       </c>
       <c r="L596" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="597" spans="1:12">
@@ -29093,7 +29084,7 @@
         <v>2395</v>
       </c>
       <c r="L597" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="598" spans="1:12">
@@ -29128,7 +29119,7 @@
         <v>2456</v>
       </c>
       <c r="L598" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="599" spans="1:12">
@@ -29312,7 +29303,7 @@
         <v>2395</v>
       </c>
       <c r="L603" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="604" spans="1:12">
@@ -29560,7 +29551,7 @@
         <v>2462</v>
       </c>
       <c r="L610" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="611" spans="1:12">
@@ -29595,7 +29586,7 @@
         <v>2472</v>
       </c>
       <c r="L611" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="612" spans="1:12">
@@ -29706,7 +29697,7 @@
         <v>2496</v>
       </c>
       <c r="L614" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="615" spans="1:12">
@@ -29741,7 +29732,7 @@
         <v>2390</v>
       </c>
       <c r="L615" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="616" spans="1:12">
@@ -29811,7 +29802,7 @@
         <v>2390</v>
       </c>
       <c r="L617" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29951,7 +29942,7 @@
         <v>2390</v>
       </c>
       <c r="L621" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="622" spans="1:12">
@@ -30056,7 +30047,7 @@
         <v>2403</v>
       </c>
       <c r="L624" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="625" spans="1:12">
@@ -30161,7 +30152,7 @@
         <v>2379</v>
       </c>
       <c r="L627" t="s">
-        <v>2582</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30196,7 +30187,7 @@
         <v>2416</v>
       </c>
       <c r="L628" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30231,7 +30222,7 @@
         <v>2416</v>
       </c>
       <c r="L629" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="630" spans="1:12">
@@ -30339,7 +30330,7 @@
         <v>2390</v>
       </c>
       <c r="L632" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30377,7 +30368,7 @@
         <v>2390</v>
       </c>
       <c r="L633" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30520,7 +30511,7 @@
         <v>2422</v>
       </c>
       <c r="L637" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30555,7 +30546,7 @@
         <v>2390</v>
       </c>
       <c r="L638" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30590,7 +30581,7 @@
         <v>2390</v>
       </c>
       <c r="L639" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="640" spans="1:12">
@@ -30695,7 +30686,7 @@
         <v>2417</v>
       </c>
       <c r="L642" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="643" spans="1:12">
@@ -30879,7 +30870,7 @@
         <v>2378</v>
       </c>
       <c r="L647" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="648" spans="1:12">
@@ -30984,7 +30975,7 @@
         <v>2398</v>
       </c>
       <c r="L650" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31019,7 +31010,7 @@
         <v>2398</v>
       </c>
       <c r="L651" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31054,7 +31045,7 @@
         <v>2391</v>
       </c>
       <c r="L652" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31092,7 +31083,7 @@
         <v>2494</v>
       </c>
       <c r="L653" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="654" spans="1:12">
@@ -31127,7 +31118,7 @@
         <v>2416</v>
       </c>
       <c r="L654" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="655" spans="1:12">
@@ -31162,7 +31153,7 @@
         <v>2453</v>
       </c>
       <c r="L655" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31197,7 +31188,7 @@
         <v>2379</v>
       </c>
       <c r="L656" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="657" spans="1:12">
@@ -31232,7 +31223,7 @@
         <v>2378</v>
       </c>
       <c r="L657" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="658" spans="1:12">
@@ -31267,7 +31258,7 @@
         <v>2374</v>
       </c>
       <c r="L658" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="659" spans="1:12">
@@ -31299,7 +31290,7 @@
         <v>2510</v>
       </c>
       <c r="L659" t="s">
-        <v>2583</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="660" spans="1:12">
@@ -31331,7 +31322,7 @@
         <v>2510</v>
       </c>
       <c r="L660" t="s">
-        <v>2584</v>
+        <v>2546</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-25 14:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -27412,7 +27412,7 @@
         <v>1578</v>
       </c>
       <c r="I550" t="s">
-        <v>1613</v>
+        <v>1702</v>
       </c>
       <c r="J550" t="s">
         <v>2263</v>
@@ -28856,7 +28856,7 @@
         <v>1578</v>
       </c>
       <c r="I591" t="s">
-        <v>1639</v>
+        <v>1613</v>
       </c>
       <c r="J591" t="s">
         <v>2303</v>
@@ -30735,7 +30735,7 @@
         <v>2</v>
       </c>
       <c r="F644" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="G644" t="s">
         <v>1580</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-29 08:30:02
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6656" uniqueCount="2587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6656" uniqueCount="2586">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7642,6 +7642,9 @@
     <t>ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
+    <t>### SEM TEMA ###</t>
+  </si>
+  <si>
     <t>ENGENHARIA QUÍMICA</t>
   </si>
   <si>
@@ -7684,9 +7687,6 @@
     <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
     <t>FARMÁCIA</t>
   </si>
   <si>
@@ -7699,7 +7699,7 @@
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
+    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7741,10 +7741,10 @@
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
   </si>
   <si>
-    <t>RESÍDUOS SÓLIDOS,GEOTECNIA,BIOLOGIA,ENGENHARIA FLORESTAL,ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+    <t>ENGENHARIA QUÍMICA,BIOLOGIA,ENGENHARIA FLORESTAL,GEOTECNIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7759,7 +7759,7 @@
     <t>GEOTECNIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
+    <t>MEDICINA LEGAL,EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
@@ -7768,13 +7768,10 @@
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ENGENHARIA CIVIL,PATRIMÔNIO HISTÓRICO E CULTURAL,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ASSISTÊNCIA SOCIAL,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,SAÚDE MENTAL,URBANISMO,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,SAÚDE,MOBILIDADE E TRANSPORTE</t>
   </si>
 </sst>
 </file>
@@ -11892,7 +11889,7 @@
         <v>2411</v>
       </c>
       <c r="L107" t="s">
-        <v>2532</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="108" spans="1:12">
@@ -11962,7 +11959,7 @@
         <v>2379</v>
       </c>
       <c r="L109" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="110" spans="1:12">
@@ -12207,7 +12204,7 @@
         <v>2421</v>
       </c>
       <c r="L116" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="117" spans="1:12">
@@ -12242,7 +12239,7 @@
         <v>2429</v>
       </c>
       <c r="L117" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="118" spans="1:12">
@@ -12420,7 +12417,7 @@
         <v>2389</v>
       </c>
       <c r="L122" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="123" spans="1:12">
@@ -12490,7 +12487,7 @@
         <v>2397</v>
       </c>
       <c r="L124" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="125" spans="1:12">
@@ -12665,7 +12662,7 @@
         <v>2429</v>
       </c>
       <c r="L129" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="130" spans="1:12">
@@ -13085,7 +13082,7 @@
         <v>2420</v>
       </c>
       <c r="L141" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="142" spans="1:12">
@@ -13260,7 +13257,7 @@
         <v>2428</v>
       </c>
       <c r="L146" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="147" spans="1:12">
@@ -13575,7 +13572,7 @@
         <v>2392</v>
       </c>
       <c r="L155" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="156" spans="1:12">
@@ -13715,7 +13712,7 @@
         <v>2447</v>
       </c>
       <c r="L159" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="160" spans="1:12">
@@ -13855,7 +13852,7 @@
         <v>2387</v>
       </c>
       <c r="L163" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -14030,7 +14027,7 @@
         <v>2428</v>
       </c>
       <c r="L168" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="169" spans="1:12">
@@ -14205,7 +14202,7 @@
         <v>2439</v>
       </c>
       <c r="L173" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="174" spans="1:12">
@@ -14345,7 +14342,7 @@
         <v>2389</v>
       </c>
       <c r="L177" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="178" spans="1:12">
@@ -14485,7 +14482,7 @@
         <v>2406</v>
       </c>
       <c r="L181" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="182" spans="1:12">
@@ -14835,7 +14832,7 @@
         <v>2409</v>
       </c>
       <c r="L191" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -14940,7 +14937,7 @@
         <v>2428</v>
       </c>
       <c r="L194" t="s">
-        <v>2552</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -15045,7 +15042,7 @@
         <v>2452</v>
       </c>
       <c r="L197" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -15080,7 +15077,7 @@
         <v>2387</v>
       </c>
       <c r="L198" t="s">
-        <v>2553</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="199" spans="1:12">
@@ -15150,7 +15147,7 @@
         <v>2397</v>
       </c>
       <c r="L200" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -15188,7 +15185,7 @@
         <v>2380</v>
       </c>
       <c r="L201" t="s">
-        <v>2516</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -15468,7 +15465,7 @@
         <v>2453</v>
       </c>
       <c r="L209" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="210" spans="1:12">
@@ -15538,7 +15535,7 @@
         <v>2399</v>
       </c>
       <c r="L211" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="212" spans="1:12">
@@ -15681,7 +15678,7 @@
         <v>2455</v>
       </c>
       <c r="L215" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="216" spans="1:12">
@@ -15821,7 +15818,7 @@
         <v>2456</v>
       </c>
       <c r="L219" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="220" spans="1:12">
@@ -15926,7 +15923,7 @@
         <v>2411</v>
       </c>
       <c r="L222" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="223" spans="1:12">
@@ -15961,7 +15958,7 @@
         <v>2457</v>
       </c>
       <c r="L223" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="224" spans="1:12">
@@ -15996,7 +15993,7 @@
         <v>2393</v>
       </c>
       <c r="L224" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="225" spans="1:12">
@@ -16101,7 +16098,7 @@
         <v>2458</v>
       </c>
       <c r="L227" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="228" spans="1:12">
@@ -16556,7 +16553,7 @@
         <v>2463</v>
       </c>
       <c r="L240" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="241" spans="1:12">
@@ -16591,7 +16588,7 @@
         <v>2454</v>
       </c>
       <c r="L241" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="242" spans="1:12">
@@ -16696,7 +16693,7 @@
         <v>2418</v>
       </c>
       <c r="L244" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="245" spans="1:12">
@@ -16731,7 +16728,7 @@
         <v>2464</v>
       </c>
       <c r="L245" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="246" spans="1:12">
@@ -16836,7 +16833,7 @@
         <v>2466</v>
       </c>
       <c r="L248" t="s">
-        <v>2555</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="249" spans="1:12">
@@ -16909,7 +16906,7 @@
         <v>2421</v>
       </c>
       <c r="L250" t="s">
-        <v>2556</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="251" spans="1:12">
@@ -17119,7 +17116,7 @@
         <v>2392</v>
       </c>
       <c r="L256" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="257" spans="1:12">
@@ -17154,7 +17151,7 @@
         <v>2463</v>
       </c>
       <c r="L257" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="258" spans="1:12">
@@ -17259,7 +17256,7 @@
         <v>2467</v>
       </c>
       <c r="L260" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="261" spans="1:12">
@@ -17399,7 +17396,7 @@
         <v>2392</v>
       </c>
       <c r="L264" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="265" spans="1:12">
@@ -17644,7 +17641,7 @@
         <v>2397</v>
       </c>
       <c r="L271" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="272" spans="1:12">
@@ -17679,7 +17676,7 @@
         <v>2439</v>
       </c>
       <c r="L272" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="273" spans="1:12">
@@ -17787,7 +17784,7 @@
         <v>2388</v>
       </c>
       <c r="L275" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -17822,7 +17819,7 @@
         <v>2470</v>
       </c>
       <c r="L276" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="277" spans="1:12">
@@ -17927,7 +17924,7 @@
         <v>2434</v>
       </c>
       <c r="L279" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="280" spans="1:12">
@@ -18032,7 +18029,7 @@
         <v>2472</v>
       </c>
       <c r="L282" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="283" spans="1:12">
@@ -18102,7 +18099,7 @@
         <v>2442</v>
       </c>
       <c r="L284" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="285" spans="1:12">
@@ -18137,7 +18134,7 @@
         <v>2456</v>
       </c>
       <c r="L285" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="286" spans="1:12">
@@ -18172,7 +18169,7 @@
         <v>2456</v>
       </c>
       <c r="L286" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="287" spans="1:12">
@@ -18207,7 +18204,7 @@
         <v>2419</v>
       </c>
       <c r="L287" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -18315,7 +18312,7 @@
         <v>2392</v>
       </c>
       <c r="L290" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="291" spans="1:12">
@@ -18490,7 +18487,7 @@
         <v>2466</v>
       </c>
       <c r="L295" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="296" spans="1:12">
@@ -18875,7 +18872,7 @@
         <v>2469</v>
       </c>
       <c r="L306" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="307" spans="1:12">
@@ -18980,7 +18977,7 @@
         <v>2378</v>
       </c>
       <c r="L309" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="310" spans="1:12">
@@ -19435,7 +19432,7 @@
         <v>2381</v>
       </c>
       <c r="L322" t="s">
-        <v>2523</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="323" spans="1:12">
@@ -19470,7 +19467,7 @@
         <v>2381</v>
       </c>
       <c r="L323" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="324" spans="1:12">
@@ -19680,7 +19677,7 @@
         <v>2400</v>
       </c>
       <c r="L329" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="330" spans="1:12">
@@ -19750,7 +19747,7 @@
         <v>2424</v>
       </c>
       <c r="L331" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="332" spans="1:12">
@@ -19855,7 +19852,7 @@
         <v>2397</v>
       </c>
       <c r="L334" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="335" spans="1:12">
@@ -20065,7 +20062,7 @@
         <v>2397</v>
       </c>
       <c r="L340" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="341" spans="1:12">
@@ -20100,7 +20097,7 @@
         <v>2392</v>
       </c>
       <c r="L341" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="342" spans="1:12">
@@ -20170,7 +20167,7 @@
         <v>2480</v>
       </c>
       <c r="L343" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="344" spans="1:12">
@@ -20415,7 +20412,7 @@
         <v>2482</v>
       </c>
       <c r="L350" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="351" spans="1:12">
@@ -20590,7 +20587,7 @@
         <v>2420</v>
       </c>
       <c r="L355" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="356" spans="1:12">
@@ -20695,7 +20692,7 @@
         <v>2400</v>
       </c>
       <c r="L358" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20800,7 +20797,7 @@
         <v>2462</v>
       </c>
       <c r="L361" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="362" spans="1:12">
@@ -20870,7 +20867,7 @@
         <v>2380</v>
       </c>
       <c r="L363" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="364" spans="1:12">
@@ -21185,7 +21182,7 @@
         <v>2468</v>
       </c>
       <c r="L372" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="373" spans="1:12">
@@ -21360,7 +21357,7 @@
         <v>2377</v>
       </c>
       <c r="L377" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="378" spans="1:12">
@@ -21395,7 +21392,7 @@
         <v>2397</v>
       </c>
       <c r="L378" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="379" spans="1:12">
@@ -21570,7 +21567,7 @@
         <v>2438</v>
       </c>
       <c r="L383" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -21605,7 +21602,7 @@
         <v>2424</v>
       </c>
       <c r="L384" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="385" spans="1:12">
@@ -21675,7 +21672,7 @@
         <v>2485</v>
       </c>
       <c r="L386" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="387" spans="1:12">
@@ -21745,7 +21742,7 @@
         <v>2397</v>
       </c>
       <c r="L388" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="389" spans="1:12">
@@ -21850,7 +21847,7 @@
         <v>2442</v>
       </c>
       <c r="L391" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="392" spans="1:12">
@@ -21885,7 +21882,7 @@
         <v>2466</v>
       </c>
       <c r="L392" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="393" spans="1:12">
@@ -21920,7 +21917,7 @@
         <v>2486</v>
       </c>
       <c r="L393" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="394" spans="1:12">
@@ -22235,7 +22232,7 @@
         <v>2419</v>
       </c>
       <c r="L402" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="403" spans="1:12">
@@ -22410,7 +22407,7 @@
         <v>2435</v>
       </c>
       <c r="L407" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22620,7 +22617,7 @@
         <v>2438</v>
       </c>
       <c r="L413" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="414" spans="1:12">
@@ -23145,7 +23142,7 @@
         <v>2375</v>
       </c>
       <c r="L428" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="429" spans="1:12">
@@ -23320,7 +23317,7 @@
         <v>2442</v>
       </c>
       <c r="L433" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="434" spans="1:12">
@@ -23390,7 +23387,7 @@
         <v>2418</v>
       </c>
       <c r="L435" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="436" spans="1:12">
@@ -23425,7 +23422,7 @@
         <v>2480</v>
       </c>
       <c r="L436" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="437" spans="1:12">
@@ -23495,7 +23492,7 @@
         <v>2480</v>
       </c>
       <c r="L438" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="439" spans="1:12">
@@ -23708,7 +23705,7 @@
         <v>2409</v>
       </c>
       <c r="L444" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="445" spans="1:12">
@@ -23778,7 +23775,7 @@
         <v>2442</v>
       </c>
       <c r="L446" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="447" spans="1:12">
@@ -24058,7 +24055,7 @@
         <v>2397</v>
       </c>
       <c r="L454" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="455" spans="1:12">
@@ -24093,7 +24090,7 @@
         <v>2479</v>
       </c>
       <c r="L455" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -24198,7 +24195,7 @@
         <v>2423</v>
       </c>
       <c r="L458" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24338,7 +24335,7 @@
         <v>2497</v>
       </c>
       <c r="L462" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="463" spans="1:12">
@@ -24446,7 +24443,7 @@
         <v>2401</v>
       </c>
       <c r="L465" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="466" spans="1:12">
@@ -24516,7 +24513,7 @@
         <v>2397</v>
       </c>
       <c r="L467" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -24551,7 +24548,7 @@
         <v>2397</v>
       </c>
       <c r="L468" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="469" spans="1:12">
@@ -24624,7 +24621,7 @@
         <v>2423</v>
       </c>
       <c r="L470" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="471" spans="1:12">
@@ -24799,7 +24796,7 @@
         <v>2434</v>
       </c>
       <c r="L475" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="476" spans="1:12">
@@ -24834,7 +24831,7 @@
         <v>2434</v>
       </c>
       <c r="L476" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="477" spans="1:12">
@@ -24869,7 +24866,7 @@
         <v>2434</v>
       </c>
       <c r="L477" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="478" spans="1:12">
@@ -24904,7 +24901,7 @@
         <v>2499</v>
       </c>
       <c r="L478" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -25044,7 +25041,7 @@
         <v>2500</v>
       </c>
       <c r="L482" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="483" spans="1:12">
@@ -25079,7 +25076,7 @@
         <v>2380</v>
       </c>
       <c r="L483" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="484" spans="1:12">
@@ -25114,7 +25111,7 @@
         <v>2500</v>
       </c>
       <c r="L484" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="485" spans="1:12">
@@ -25149,7 +25146,7 @@
         <v>2392</v>
       </c>
       <c r="L485" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25289,7 +25286,7 @@
         <v>2392</v>
       </c>
       <c r="L489" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="490" spans="1:12">
@@ -25359,7 +25356,7 @@
         <v>2412</v>
       </c>
       <c r="L491" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="492" spans="1:12">
@@ -25534,7 +25531,7 @@
         <v>2424</v>
       </c>
       <c r="L496" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="497" spans="1:12">
@@ -25604,7 +25601,7 @@
         <v>2393</v>
       </c>
       <c r="L498" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="499" spans="1:12">
@@ -25782,7 +25779,7 @@
         <v>2499</v>
       </c>
       <c r="L503" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -25852,7 +25849,7 @@
         <v>2482</v>
       </c>
       <c r="L505" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="506" spans="1:12">
@@ -25887,7 +25884,7 @@
         <v>2454</v>
       </c>
       <c r="L506" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25960,7 +25957,7 @@
         <v>2435</v>
       </c>
       <c r="L508" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="509" spans="1:12">
@@ -25995,7 +25992,7 @@
         <v>2397</v>
       </c>
       <c r="L509" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="510" spans="1:12">
@@ -26135,7 +26132,7 @@
         <v>2498</v>
       </c>
       <c r="L513" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="514" spans="1:12">
@@ -26243,7 +26240,7 @@
         <v>2439</v>
       </c>
       <c r="L516" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="517" spans="1:12">
@@ -26383,7 +26380,7 @@
         <v>2411</v>
       </c>
       <c r="L520" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="521" spans="1:12">
@@ -26453,7 +26450,7 @@
         <v>2498</v>
       </c>
       <c r="L522" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="523" spans="1:12">
@@ -26523,7 +26520,7 @@
         <v>2397</v>
       </c>
       <c r="L524" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="525" spans="1:12">
@@ -26593,7 +26590,7 @@
         <v>2400</v>
       </c>
       <c r="L526" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="527" spans="1:12">
@@ -26698,7 +26695,7 @@
         <v>2401</v>
       </c>
       <c r="L529" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="530" spans="1:12">
@@ -26876,7 +26873,7 @@
         <v>2470</v>
       </c>
       <c r="L534" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="535" spans="1:12">
@@ -26914,7 +26911,7 @@
         <v>2470</v>
       </c>
       <c r="L535" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="536" spans="1:12">
@@ -26949,7 +26946,7 @@
         <v>2397</v>
       </c>
       <c r="L536" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="537" spans="1:12">
@@ -27019,7 +27016,7 @@
         <v>2454</v>
       </c>
       <c r="L538" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -27054,7 +27051,7 @@
         <v>2400</v>
       </c>
       <c r="L539" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="540" spans="1:12">
@@ -27089,7 +27086,7 @@
         <v>2381</v>
       </c>
       <c r="L540" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27197,7 +27194,7 @@
         <v>2411</v>
       </c>
       <c r="L543" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="544" spans="1:12">
@@ -27486,7 +27483,7 @@
         <v>2375</v>
       </c>
       <c r="L551" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="552" spans="1:12">
@@ -27521,7 +27518,7 @@
         <v>2463</v>
       </c>
       <c r="L552" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27556,7 +27553,7 @@
         <v>2469</v>
       </c>
       <c r="L553" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -27591,7 +27588,7 @@
         <v>2376</v>
       </c>
       <c r="L554" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="555" spans="1:12">
@@ -27626,7 +27623,7 @@
         <v>2376</v>
       </c>
       <c r="L555" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="556" spans="1:12">
@@ -27661,7 +27658,7 @@
         <v>2400</v>
       </c>
       <c r="L556" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="557" spans="1:12">
@@ -27696,7 +27693,7 @@
         <v>2498</v>
       </c>
       <c r="L557" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="558" spans="1:12">
@@ -27906,7 +27903,7 @@
         <v>2424</v>
       </c>
       <c r="L563" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="564" spans="1:12">
@@ -27941,7 +27938,7 @@
         <v>2384</v>
       </c>
       <c r="L564" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -28116,7 +28113,7 @@
         <v>2424</v>
       </c>
       <c r="L569" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -28151,7 +28148,7 @@
         <v>2409</v>
       </c>
       <c r="L570" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28291,7 +28288,7 @@
         <v>2495</v>
       </c>
       <c r="L574" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="575" spans="1:12">
@@ -28504,7 +28501,7 @@
         <v>2423</v>
       </c>
       <c r="L580" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28539,7 +28536,7 @@
         <v>2423</v>
       </c>
       <c r="L581" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="582" spans="1:12">
@@ -28714,7 +28711,7 @@
         <v>2412</v>
       </c>
       <c r="L586" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28749,7 +28746,7 @@
         <v>2397</v>
       </c>
       <c r="L587" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="588" spans="1:12">
@@ -28784,7 +28781,7 @@
         <v>2456</v>
       </c>
       <c r="L588" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -28819,7 +28816,7 @@
         <v>2397</v>
       </c>
       <c r="L589" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="590" spans="1:12">
@@ -28854,7 +28851,7 @@
         <v>2457</v>
       </c>
       <c r="L590" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="591" spans="1:12">
@@ -29000,7 +28997,7 @@
         <v>2397</v>
       </c>
       <c r="L594" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -29248,7 +29245,7 @@
         <v>2463</v>
       </c>
       <c r="L601" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="602" spans="1:12">
@@ -29283,7 +29280,7 @@
         <v>2473</v>
       </c>
       <c r="L602" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29391,7 +29388,7 @@
         <v>2392</v>
       </c>
       <c r="L605" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="606" spans="1:12">
@@ -29461,7 +29458,7 @@
         <v>2392</v>
       </c>
       <c r="L607" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29601,7 +29598,7 @@
         <v>2392</v>
       </c>
       <c r="L611" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="612" spans="1:12">
@@ -29706,7 +29703,7 @@
         <v>2405</v>
       </c>
       <c r="L614" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="615" spans="1:12">
@@ -29811,7 +29808,7 @@
         <v>2381</v>
       </c>
       <c r="L617" t="s">
-        <v>2528</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29846,7 +29843,7 @@
         <v>2418</v>
       </c>
       <c r="L618" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29881,7 +29878,7 @@
         <v>2418</v>
       </c>
       <c r="L619" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29989,7 +29986,7 @@
         <v>2392</v>
       </c>
       <c r="L622" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="623" spans="1:12">
@@ -30027,7 +30024,7 @@
         <v>2392</v>
       </c>
       <c r="L623" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="624" spans="1:12">
@@ -30170,7 +30167,7 @@
         <v>2424</v>
       </c>
       <c r="L627" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30205,7 +30202,7 @@
         <v>2392</v>
       </c>
       <c r="L628" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30240,7 +30237,7 @@
         <v>2392</v>
       </c>
       <c r="L629" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="630" spans="1:12">
@@ -30380,7 +30377,7 @@
         <v>2419</v>
       </c>
       <c r="L633" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30529,7 +30526,7 @@
         <v>2389</v>
       </c>
       <c r="L637" t="s">
-        <v>2584</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30564,7 +30561,7 @@
         <v>2380</v>
       </c>
       <c r="L638" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30634,7 +30631,7 @@
         <v>2400</v>
       </c>
       <c r="L640" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -30669,7 +30666,7 @@
         <v>2400</v>
       </c>
       <c r="L641" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30704,7 +30701,7 @@
         <v>2393</v>
       </c>
       <c r="L642" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="643" spans="1:12">
@@ -30742,7 +30739,7 @@
         <v>2495</v>
       </c>
       <c r="L643" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="644" spans="1:12">
@@ -30777,7 +30774,7 @@
         <v>2418</v>
       </c>
       <c r="L644" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="645" spans="1:12">
@@ -30812,7 +30809,7 @@
         <v>2454</v>
       </c>
       <c r="L645" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -30847,7 +30844,7 @@
         <v>2381</v>
       </c>
       <c r="L646" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="647" spans="1:12">
@@ -30882,7 +30879,7 @@
         <v>2380</v>
       </c>
       <c r="L647" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="648" spans="1:12">
@@ -30917,7 +30914,7 @@
         <v>2376</v>
       </c>
       <c r="L648" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="649" spans="1:12">
@@ -30987,7 +30984,7 @@
         <v>2466</v>
       </c>
       <c r="L650" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31022,7 +31019,7 @@
         <v>2510</v>
       </c>
       <c r="L651" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31060,7 +31057,7 @@
         <v>2415</v>
       </c>
       <c r="L652" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31133,7 +31130,7 @@
         <v>2400</v>
       </c>
       <c r="L654" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="655" spans="1:12">
@@ -31168,7 +31165,7 @@
         <v>2400</v>
       </c>
       <c r="L655" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31238,7 +31235,7 @@
         <v>2466</v>
       </c>
       <c r="L657" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="658" spans="1:12">
@@ -31343,7 +31340,7 @@
         <v>2405</v>
       </c>
       <c r="L660" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="661" spans="1:12">
@@ -31375,7 +31372,7 @@
         <v>2511</v>
       </c>
       <c r="L661" t="s">
-        <v>2585</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="662" spans="1:12">
@@ -31407,7 +31404,7 @@
         <v>2511</v>
       </c>
       <c r="L662" t="s">
-        <v>2586</v>
+        <v>2547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-29 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6656" uniqueCount="2586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6656" uniqueCount="2587">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7642,9 +7642,6 @@
     <t>ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>### SEM TEMA ###</t>
-  </si>
-  <si>
     <t>ENGENHARIA QUÍMICA</t>
   </si>
   <si>
@@ -7687,6 +7684,9 @@
     <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
+    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
     <t>FARMÁCIA</t>
   </si>
   <si>
@@ -7699,7 +7699,7 @@
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7741,10 +7741,10 @@
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
   </si>
   <si>
-    <t>ENGENHARIA QUÍMICA,BIOLOGIA,ENGENHARIA FLORESTAL,GEOTECNIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+    <t>RESÍDUOS SÓLIDOS,GEOTECNIA,BIOLOGIA,ENGENHARIA FLORESTAL,ENGENHARIA QUÍMICA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7759,7 +7759,7 @@
     <t>GEOTECNIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>MEDICINA LEGAL,EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
@@ -7768,10 +7768,13 @@
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
-  </si>
-  <si>
     <t>ENGENHARIA CIVIL,PATRIMÔNIO HISTÓRICO E CULTURAL,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ASSISTÊNCIA SOCIAL,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,SAÚDE MENTAL,URBANISMO,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,SAÚDE,MOBILIDADE E TRANSPORTE</t>
   </si>
 </sst>
 </file>
@@ -11889,7 +11892,7 @@
         <v>2411</v>
       </c>
       <c r="L107" t="s">
-        <v>2542</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="108" spans="1:12">
@@ -11959,7 +11962,7 @@
         <v>2379</v>
       </c>
       <c r="L109" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="110" spans="1:12">
@@ -12204,7 +12207,7 @@
         <v>2421</v>
       </c>
       <c r="L116" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="117" spans="1:12">
@@ -12239,7 +12242,7 @@
         <v>2429</v>
       </c>
       <c r="L117" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="118" spans="1:12">
@@ -12417,7 +12420,7 @@
         <v>2389</v>
       </c>
       <c r="L122" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="123" spans="1:12">
@@ -12487,7 +12490,7 @@
         <v>2397</v>
       </c>
       <c r="L124" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="125" spans="1:12">
@@ -12662,7 +12665,7 @@
         <v>2429</v>
       </c>
       <c r="L129" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="130" spans="1:12">
@@ -13082,7 +13085,7 @@
         <v>2420</v>
       </c>
       <c r="L141" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="142" spans="1:12">
@@ -13257,7 +13260,7 @@
         <v>2428</v>
       </c>
       <c r="L146" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="147" spans="1:12">
@@ -13572,7 +13575,7 @@
         <v>2392</v>
       </c>
       <c r="L155" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="156" spans="1:12">
@@ -13712,7 +13715,7 @@
         <v>2447</v>
       </c>
       <c r="L159" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="160" spans="1:12">
@@ -13852,7 +13855,7 @@
         <v>2387</v>
       </c>
       <c r="L163" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -14027,7 +14030,7 @@
         <v>2428</v>
       </c>
       <c r="L168" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="169" spans="1:12">
@@ -14202,7 +14205,7 @@
         <v>2439</v>
       </c>
       <c r="L173" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="174" spans="1:12">
@@ -14342,7 +14345,7 @@
         <v>2389</v>
       </c>
       <c r="L177" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="178" spans="1:12">
@@ -14482,7 +14485,7 @@
         <v>2406</v>
       </c>
       <c r="L181" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="182" spans="1:12">
@@ -14832,7 +14835,7 @@
         <v>2409</v>
       </c>
       <c r="L191" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -14937,7 +14940,7 @@
         <v>2428</v>
       </c>
       <c r="L194" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -15042,7 +15045,7 @@
         <v>2452</v>
       </c>
       <c r="L197" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -15077,7 +15080,7 @@
         <v>2387</v>
       </c>
       <c r="L198" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="199" spans="1:12">
@@ -15147,7 +15150,7 @@
         <v>2397</v>
       </c>
       <c r="L200" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -15185,7 +15188,7 @@
         <v>2380</v>
       </c>
       <c r="L201" t="s">
-        <v>2547</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -15465,7 +15468,7 @@
         <v>2453</v>
       </c>
       <c r="L209" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="210" spans="1:12">
@@ -15535,7 +15538,7 @@
         <v>2399</v>
       </c>
       <c r="L211" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="212" spans="1:12">
@@ -15678,7 +15681,7 @@
         <v>2455</v>
       </c>
       <c r="L215" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="216" spans="1:12">
@@ -15818,7 +15821,7 @@
         <v>2456</v>
       </c>
       <c r="L219" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="220" spans="1:12">
@@ -15923,7 +15926,7 @@
         <v>2411</v>
       </c>
       <c r="L222" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="223" spans="1:12">
@@ -15958,7 +15961,7 @@
         <v>2457</v>
       </c>
       <c r="L223" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="224" spans="1:12">
@@ -15993,7 +15996,7 @@
         <v>2393</v>
       </c>
       <c r="L224" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="225" spans="1:12">
@@ -16098,7 +16101,7 @@
         <v>2458</v>
       </c>
       <c r="L227" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="228" spans="1:12">
@@ -16553,7 +16556,7 @@
         <v>2463</v>
       </c>
       <c r="L240" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="241" spans="1:12">
@@ -16588,7 +16591,7 @@
         <v>2454</v>
       </c>
       <c r="L241" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="242" spans="1:12">
@@ -16693,7 +16696,7 @@
         <v>2418</v>
       </c>
       <c r="L244" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="245" spans="1:12">
@@ -16728,7 +16731,7 @@
         <v>2464</v>
       </c>
       <c r="L245" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="246" spans="1:12">
@@ -16833,7 +16836,7 @@
         <v>2466</v>
       </c>
       <c r="L248" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="249" spans="1:12">
@@ -16906,7 +16909,7 @@
         <v>2421</v>
       </c>
       <c r="L250" t="s">
-        <v>2542</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="251" spans="1:12">
@@ -17116,7 +17119,7 @@
         <v>2392</v>
       </c>
       <c r="L256" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="257" spans="1:12">
@@ -17151,7 +17154,7 @@
         <v>2463</v>
       </c>
       <c r="L257" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="258" spans="1:12">
@@ -17256,7 +17259,7 @@
         <v>2467</v>
       </c>
       <c r="L260" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="261" spans="1:12">
@@ -17396,7 +17399,7 @@
         <v>2392</v>
       </c>
       <c r="L264" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="265" spans="1:12">
@@ -17641,7 +17644,7 @@
         <v>2397</v>
       </c>
       <c r="L271" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="272" spans="1:12">
@@ -17676,7 +17679,7 @@
         <v>2439</v>
       </c>
       <c r="L272" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="273" spans="1:12">
@@ -17784,7 +17787,7 @@
         <v>2388</v>
       </c>
       <c r="L275" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="276" spans="1:12">
@@ -17819,7 +17822,7 @@
         <v>2470</v>
       </c>
       <c r="L276" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="277" spans="1:12">
@@ -17924,7 +17927,7 @@
         <v>2434</v>
       </c>
       <c r="L279" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="280" spans="1:12">
@@ -18029,7 +18032,7 @@
         <v>2472</v>
       </c>
       <c r="L282" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="283" spans="1:12">
@@ -18099,7 +18102,7 @@
         <v>2442</v>
       </c>
       <c r="L284" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="285" spans="1:12">
@@ -18134,7 +18137,7 @@
         <v>2456</v>
       </c>
       <c r="L285" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="286" spans="1:12">
@@ -18169,7 +18172,7 @@
         <v>2456</v>
       </c>
       <c r="L286" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="287" spans="1:12">
@@ -18204,7 +18207,7 @@
         <v>2419</v>
       </c>
       <c r="L287" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="288" spans="1:12">
@@ -18312,7 +18315,7 @@
         <v>2392</v>
       </c>
       <c r="L290" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="291" spans="1:12">
@@ -18487,7 +18490,7 @@
         <v>2466</v>
       </c>
       <c r="L295" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="296" spans="1:12">
@@ -18872,7 +18875,7 @@
         <v>2469</v>
       </c>
       <c r="L306" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="307" spans="1:12">
@@ -18977,7 +18980,7 @@
         <v>2378</v>
       </c>
       <c r="L309" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="310" spans="1:12">
@@ -19432,7 +19435,7 @@
         <v>2381</v>
       </c>
       <c r="L322" t="s">
-        <v>2547</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="323" spans="1:12">
@@ -19467,7 +19470,7 @@
         <v>2381</v>
       </c>
       <c r="L323" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="324" spans="1:12">
@@ -19677,7 +19680,7 @@
         <v>2400</v>
       </c>
       <c r="L329" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="330" spans="1:12">
@@ -19747,7 +19750,7 @@
         <v>2424</v>
       </c>
       <c r="L331" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="332" spans="1:12">
@@ -19852,7 +19855,7 @@
         <v>2397</v>
       </c>
       <c r="L334" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="335" spans="1:12">
@@ -20062,7 +20065,7 @@
         <v>2397</v>
       </c>
       <c r="L340" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="341" spans="1:12">
@@ -20097,7 +20100,7 @@
         <v>2392</v>
       </c>
       <c r="L341" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="342" spans="1:12">
@@ -20167,7 +20170,7 @@
         <v>2480</v>
       </c>
       <c r="L343" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="344" spans="1:12">
@@ -20412,7 +20415,7 @@
         <v>2482</v>
       </c>
       <c r="L350" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="351" spans="1:12">
@@ -20587,7 +20590,7 @@
         <v>2420</v>
       </c>
       <c r="L355" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="356" spans="1:12">
@@ -20692,7 +20695,7 @@
         <v>2400</v>
       </c>
       <c r="L358" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20797,7 +20800,7 @@
         <v>2462</v>
       </c>
       <c r="L361" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="362" spans="1:12">
@@ -20867,7 +20870,7 @@
         <v>2380</v>
       </c>
       <c r="L363" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="364" spans="1:12">
@@ -21182,7 +21185,7 @@
         <v>2468</v>
       </c>
       <c r="L372" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="373" spans="1:12">
@@ -21357,7 +21360,7 @@
         <v>2377</v>
       </c>
       <c r="L377" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="378" spans="1:12">
@@ -21392,7 +21395,7 @@
         <v>2397</v>
       </c>
       <c r="L378" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="379" spans="1:12">
@@ -21567,7 +21570,7 @@
         <v>2438</v>
       </c>
       <c r="L383" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -21602,7 +21605,7 @@
         <v>2424</v>
       </c>
       <c r="L384" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="385" spans="1:12">
@@ -21672,7 +21675,7 @@
         <v>2485</v>
       </c>
       <c r="L386" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="387" spans="1:12">
@@ -21742,7 +21745,7 @@
         <v>2397</v>
       </c>
       <c r="L388" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="389" spans="1:12">
@@ -21847,7 +21850,7 @@
         <v>2442</v>
       </c>
       <c r="L391" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="392" spans="1:12">
@@ -21882,7 +21885,7 @@
         <v>2466</v>
       </c>
       <c r="L392" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="393" spans="1:12">
@@ -21917,7 +21920,7 @@
         <v>2486</v>
       </c>
       <c r="L393" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="394" spans="1:12">
@@ -22232,7 +22235,7 @@
         <v>2419</v>
       </c>
       <c r="L402" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="403" spans="1:12">
@@ -22407,7 +22410,7 @@
         <v>2435</v>
       </c>
       <c r="L407" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22617,7 +22620,7 @@
         <v>2438</v>
       </c>
       <c r="L413" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="414" spans="1:12">
@@ -23142,7 +23145,7 @@
         <v>2375</v>
       </c>
       <c r="L428" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="429" spans="1:12">
@@ -23317,7 +23320,7 @@
         <v>2442</v>
       </c>
       <c r="L433" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="434" spans="1:12">
@@ -23387,7 +23390,7 @@
         <v>2418</v>
       </c>
       <c r="L435" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="436" spans="1:12">
@@ -23422,7 +23425,7 @@
         <v>2480</v>
       </c>
       <c r="L436" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="437" spans="1:12">
@@ -23492,7 +23495,7 @@
         <v>2480</v>
       </c>
       <c r="L438" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="439" spans="1:12">
@@ -23705,7 +23708,7 @@
         <v>2409</v>
       </c>
       <c r="L444" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="445" spans="1:12">
@@ -23775,7 +23778,7 @@
         <v>2442</v>
       </c>
       <c r="L446" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="447" spans="1:12">
@@ -24055,7 +24058,7 @@
         <v>2397</v>
       </c>
       <c r="L454" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="455" spans="1:12">
@@ -24090,7 +24093,7 @@
         <v>2479</v>
       </c>
       <c r="L455" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -24195,7 +24198,7 @@
         <v>2423</v>
       </c>
       <c r="L458" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24335,7 +24338,7 @@
         <v>2497</v>
       </c>
       <c r="L462" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="463" spans="1:12">
@@ -24443,7 +24446,7 @@
         <v>2401</v>
       </c>
       <c r="L465" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="466" spans="1:12">
@@ -24513,7 +24516,7 @@
         <v>2397</v>
       </c>
       <c r="L467" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -24548,7 +24551,7 @@
         <v>2397</v>
       </c>
       <c r="L468" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="469" spans="1:12">
@@ -24621,7 +24624,7 @@
         <v>2423</v>
       </c>
       <c r="L470" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="471" spans="1:12">
@@ -24796,7 +24799,7 @@
         <v>2434</v>
       </c>
       <c r="L475" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="476" spans="1:12">
@@ -24831,7 +24834,7 @@
         <v>2434</v>
       </c>
       <c r="L476" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="477" spans="1:12">
@@ -24866,7 +24869,7 @@
         <v>2434</v>
       </c>
       <c r="L477" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="478" spans="1:12">
@@ -24901,7 +24904,7 @@
         <v>2499</v>
       </c>
       <c r="L478" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -25041,7 +25044,7 @@
         <v>2500</v>
       </c>
       <c r="L482" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="483" spans="1:12">
@@ -25076,7 +25079,7 @@
         <v>2380</v>
       </c>
       <c r="L483" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="484" spans="1:12">
@@ -25111,7 +25114,7 @@
         <v>2500</v>
       </c>
       <c r="L484" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="485" spans="1:12">
@@ -25146,7 +25149,7 @@
         <v>2392</v>
       </c>
       <c r="L485" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25286,7 +25289,7 @@
         <v>2392</v>
       </c>
       <c r="L489" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="490" spans="1:12">
@@ -25356,7 +25359,7 @@
         <v>2412</v>
       </c>
       <c r="L491" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="492" spans="1:12">
@@ -25531,7 +25534,7 @@
         <v>2424</v>
       </c>
       <c r="L496" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="497" spans="1:12">
@@ -25601,7 +25604,7 @@
         <v>2393</v>
       </c>
       <c r="L498" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="499" spans="1:12">
@@ -25779,7 +25782,7 @@
         <v>2499</v>
       </c>
       <c r="L503" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -25849,7 +25852,7 @@
         <v>2482</v>
       </c>
       <c r="L505" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="506" spans="1:12">
@@ -25884,7 +25887,7 @@
         <v>2454</v>
       </c>
       <c r="L506" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25957,7 +25960,7 @@
         <v>2435</v>
       </c>
       <c r="L508" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="509" spans="1:12">
@@ -25992,7 +25995,7 @@
         <v>2397</v>
       </c>
       <c r="L509" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="510" spans="1:12">
@@ -26132,7 +26135,7 @@
         <v>2498</v>
       </c>
       <c r="L513" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="514" spans="1:12">
@@ -26240,7 +26243,7 @@
         <v>2439</v>
       </c>
       <c r="L516" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="517" spans="1:12">
@@ -26380,7 +26383,7 @@
         <v>2411</v>
       </c>
       <c r="L520" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="521" spans="1:12">
@@ -26450,7 +26453,7 @@
         <v>2498</v>
       </c>
       <c r="L522" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="523" spans="1:12">
@@ -26520,7 +26523,7 @@
         <v>2397</v>
       </c>
       <c r="L524" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="525" spans="1:12">
@@ -26590,7 +26593,7 @@
         <v>2400</v>
       </c>
       <c r="L526" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="527" spans="1:12">
@@ -26695,7 +26698,7 @@
         <v>2401</v>
       </c>
       <c r="L529" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="530" spans="1:12">
@@ -26873,7 +26876,7 @@
         <v>2470</v>
       </c>
       <c r="L534" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="535" spans="1:12">
@@ -26911,7 +26914,7 @@
         <v>2470</v>
       </c>
       <c r="L535" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="536" spans="1:12">
@@ -26946,7 +26949,7 @@
         <v>2397</v>
       </c>
       <c r="L536" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="537" spans="1:12">
@@ -27016,7 +27019,7 @@
         <v>2454</v>
       </c>
       <c r="L538" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -27051,7 +27054,7 @@
         <v>2400</v>
       </c>
       <c r="L539" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="540" spans="1:12">
@@ -27086,7 +27089,7 @@
         <v>2381</v>
       </c>
       <c r="L540" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27194,7 +27197,7 @@
         <v>2411</v>
       </c>
       <c r="L543" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="544" spans="1:12">
@@ -27483,7 +27486,7 @@
         <v>2375</v>
       </c>
       <c r="L551" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="552" spans="1:12">
@@ -27518,7 +27521,7 @@
         <v>2463</v>
       </c>
       <c r="L552" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27553,7 +27556,7 @@
         <v>2469</v>
       </c>
       <c r="L553" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -27588,7 +27591,7 @@
         <v>2376</v>
       </c>
       <c r="L554" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="555" spans="1:12">
@@ -27623,7 +27626,7 @@
         <v>2376</v>
       </c>
       <c r="L555" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="556" spans="1:12">
@@ -27658,7 +27661,7 @@
         <v>2400</v>
       </c>
       <c r="L556" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="557" spans="1:12">
@@ -27693,7 +27696,7 @@
         <v>2498</v>
       </c>
       <c r="L557" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="558" spans="1:12">
@@ -27903,7 +27906,7 @@
         <v>2424</v>
       </c>
       <c r="L563" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="564" spans="1:12">
@@ -27938,7 +27941,7 @@
         <v>2384</v>
       </c>
       <c r="L564" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -28113,7 +28116,7 @@
         <v>2424</v>
       </c>
       <c r="L569" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -28148,7 +28151,7 @@
         <v>2409</v>
       </c>
       <c r="L570" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28288,7 +28291,7 @@
         <v>2495</v>
       </c>
       <c r="L574" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="575" spans="1:12">
@@ -28501,7 +28504,7 @@
         <v>2423</v>
       </c>
       <c r="L580" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28536,7 +28539,7 @@
         <v>2423</v>
       </c>
       <c r="L581" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="582" spans="1:12">
@@ -28711,7 +28714,7 @@
         <v>2412</v>
       </c>
       <c r="L586" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28746,7 +28749,7 @@
         <v>2397</v>
       </c>
       <c r="L587" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="588" spans="1:12">
@@ -28781,7 +28784,7 @@
         <v>2456</v>
       </c>
       <c r="L588" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -28816,7 +28819,7 @@
         <v>2397</v>
       </c>
       <c r="L589" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="590" spans="1:12">
@@ -28851,7 +28854,7 @@
         <v>2457</v>
       </c>
       <c r="L590" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="591" spans="1:12">
@@ -28997,7 +29000,7 @@
         <v>2397</v>
       </c>
       <c r="L594" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -29245,7 +29248,7 @@
         <v>2463</v>
       </c>
       <c r="L601" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="602" spans="1:12">
@@ -29280,7 +29283,7 @@
         <v>2473</v>
       </c>
       <c r="L602" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29388,7 +29391,7 @@
         <v>2392</v>
       </c>
       <c r="L605" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="606" spans="1:12">
@@ -29458,7 +29461,7 @@
         <v>2392</v>
       </c>
       <c r="L607" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29598,7 +29601,7 @@
         <v>2392</v>
       </c>
       <c r="L611" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="612" spans="1:12">
@@ -29703,7 +29706,7 @@
         <v>2405</v>
       </c>
       <c r="L614" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="615" spans="1:12">
@@ -29808,7 +29811,7 @@
         <v>2381</v>
       </c>
       <c r="L617" t="s">
-        <v>2584</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29843,7 +29846,7 @@
         <v>2418</v>
       </c>
       <c r="L618" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29878,7 +29881,7 @@
         <v>2418</v>
       </c>
       <c r="L619" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29986,7 +29989,7 @@
         <v>2392</v>
       </c>
       <c r="L622" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="623" spans="1:12">
@@ -30024,7 +30027,7 @@
         <v>2392</v>
       </c>
       <c r="L623" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="624" spans="1:12">
@@ -30167,7 +30170,7 @@
         <v>2424</v>
       </c>
       <c r="L627" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30202,7 +30205,7 @@
         <v>2392</v>
       </c>
       <c r="L628" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30237,7 +30240,7 @@
         <v>2392</v>
       </c>
       <c r="L629" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="630" spans="1:12">
@@ -30377,7 +30380,7 @@
         <v>2419</v>
       </c>
       <c r="L633" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30526,7 +30529,7 @@
         <v>2389</v>
       </c>
       <c r="L637" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30561,7 +30564,7 @@
         <v>2380</v>
       </c>
       <c r="L638" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30631,7 +30634,7 @@
         <v>2400</v>
       </c>
       <c r="L640" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -30666,7 +30669,7 @@
         <v>2400</v>
       </c>
       <c r="L641" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30701,7 +30704,7 @@
         <v>2393</v>
       </c>
       <c r="L642" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="643" spans="1:12">
@@ -30739,7 +30742,7 @@
         <v>2495</v>
       </c>
       <c r="L643" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="644" spans="1:12">
@@ -30774,7 +30777,7 @@
         <v>2418</v>
       </c>
       <c r="L644" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="645" spans="1:12">
@@ -30809,7 +30812,7 @@
         <v>2454</v>
       </c>
       <c r="L645" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -30844,7 +30847,7 @@
         <v>2381</v>
       </c>
       <c r="L646" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="647" spans="1:12">
@@ -30879,7 +30882,7 @@
         <v>2380</v>
       </c>
       <c r="L647" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="648" spans="1:12">
@@ -30914,7 +30917,7 @@
         <v>2376</v>
       </c>
       <c r="L648" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="649" spans="1:12">
@@ -30984,7 +30987,7 @@
         <v>2466</v>
       </c>
       <c r="L650" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31019,7 +31022,7 @@
         <v>2510</v>
       </c>
       <c r="L651" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31057,7 +31060,7 @@
         <v>2415</v>
       </c>
       <c r="L652" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31130,7 +31133,7 @@
         <v>2400</v>
       </c>
       <c r="L654" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="655" spans="1:12">
@@ -31165,7 +31168,7 @@
         <v>2400</v>
       </c>
       <c r="L655" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31235,7 +31238,7 @@
         <v>2466</v>
       </c>
       <c r="L657" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="658" spans="1:12">
@@ -31340,7 +31343,7 @@
         <v>2405</v>
       </c>
       <c r="L660" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="661" spans="1:12">
@@ -31372,7 +31375,7 @@
         <v>2511</v>
       </c>
       <c r="L661" t="s">
-        <v>2547</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="662" spans="1:12">
@@ -31404,7 +31407,7 @@
         <v>2511</v>
       </c>
       <c r="L662" t="s">
-        <v>2547</v>
+        <v>2586</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-01 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6678" uniqueCount="2592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6678" uniqueCount="2593">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7711,7 +7711,7 @@
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>GEOLOGIA,BIOLOGIA,URBANISMO</t>
+    <t>BIOLOGIA,URBANISMO,GEOLOGIA</t>
   </si>
   <si>
     <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
@@ -7747,16 +7747,16 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
   </si>
   <si>
-    <t>ENGENHARIA FLORESTAL,GEOTECNIA,RESÍDUOS SÓLIDOS,BIOLOGIA,ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+    <t>BIOLOGIA,GEOTECNIA,ENGENHARIA FLORESTAL,RESÍDUOS SÓLIDOS,ENGENHARIA QUÍMICA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7780,6 +7780,9 @@
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ENGENHARIA CIVIL,PATRIMÔNIO HISTÓRICO E CULTURAL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
@@ -7789,7 +7792,7 @@
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>SAÚDE,ECONOMICIDADE CONTÁBIL,ORÇAMENTO,URBANISMO,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,MOBILIDADE E TRANSPORTE,ECONOMIA,SAÚDE MENTAL</t>
+    <t>ASSISTÊNCIA SOCIAL,ECONOMICIDADE CONTÁBIL,SAÚDE,URBANISMO,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ECONOMIA,SAÚDE MENTAL,MOBILIDADE E TRANSPORTE</t>
   </si>
 </sst>
 </file>
@@ -29502,7 +29505,7 @@
         <v>2423</v>
       </c>
       <c r="L608" t="s">
-        <v>2530</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="609" spans="1:12">
@@ -30220,7 +30223,7 @@
         <v>2390</v>
       </c>
       <c r="L628" t="s">
-        <v>2588</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -31180,7 +31183,7 @@
         <v>2397</v>
       </c>
       <c r="L655" t="s">
-        <v>2589</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31466,7 +31469,7 @@
         <v>2514</v>
       </c>
       <c r="L663" t="s">
-        <v>2590</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -31498,7 +31501,7 @@
         <v>2514</v>
       </c>
       <c r="L664" t="s">
-        <v>2591</v>
+        <v>2592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-02 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6549" uniqueCount="2558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6549" uniqueCount="2559">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7606,7 +7606,7 @@
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>BIOLOGIA,URBANISMO,GEOLOGIA</t>
+    <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
   </si>
   <si>
     <t>VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7651,7 +7651,7 @@
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
   </si>
   <si>
-    <t>ENGENHARIA QUÍMICA,BIOLOGIA,GEOTECNIA,ENGENHARIA FLORESTAL,RESÍDUOS SÓLIDOS</t>
+    <t>RESÍDUOS SÓLIDOS,BIOLOGIA,ENGENHARIA QUÍMICA,GEOTECNIA,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7669,25 +7669,28 @@
     <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
+    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ENGENHARIA CIVIL,PATRIMÔNIO HISTÓRICO E CULTURAL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>GEOLOGIA,ENGENHARIA QUÍMICA</t>
   </si>
   <si>
-    <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
+    <t>RECURSOS HÍDRICOS,BIOLOGIA</t>
   </si>
   <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>PSICOLOGIA,ASSISTÊNCIA SOCIAL,MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL,ECONOMIA,SAÚDE,AVALIAÇÃO DE IMÓVEIS,URBANISMO,SAÚDE MENTAL,ORÇAMENTO</t>
+    <t>SAÚDE,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL,PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,URBANISMO,ECONOMIA,ORÇAMENTO,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -28875,7 +28878,7 @@
         <v>2389</v>
       </c>
       <c r="L593" t="s">
-        <v>2497</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -29558,7 +29561,7 @@
         <v>2358</v>
       </c>
       <c r="L612" t="s">
-        <v>2553</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="613" spans="1:12">
@@ -30337,7 +30340,7 @@
         <v>2433</v>
       </c>
       <c r="L634" t="s">
-        <v>2487</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="635" spans="1:12">
@@ -30480,7 +30483,7 @@
         <v>2479</v>
       </c>
       <c r="L638" t="s">
-        <v>2514</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30556,7 +30559,7 @@
         <v>2365</v>
       </c>
       <c r="L640" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -30594,7 +30597,7 @@
         <v>2365</v>
       </c>
       <c r="L641" t="s">
-        <v>2555</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30912,7 +30915,7 @@
         <v>2481</v>
       </c>
       <c r="L650" t="s">
-        <v>2556</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -30944,7 +30947,7 @@
         <v>2481</v>
       </c>
       <c r="L651" t="s">
-        <v>2557</v>
+        <v>2558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-02 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -30818,7 +30818,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B648" t="s">
         <v>685</v>
@@ -30839,7 +30839,7 @@
         <v>1564</v>
       </c>
       <c r="I648" t="s">
-        <v>1598</v>
+        <v>1709</v>
       </c>
       <c r="J648" t="s">
         <v>2341</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-03 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7594,13 +7594,13 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
   </si>
   <si>
-    <t>RESÍDUOS SÓLIDOS,ENGENHARIA QUÍMICA,BIOLOGIA</t>
+    <t>RESÍDUOS SÓLIDOS,BIOLOGIA,ENGENHARIA QUÍMICA</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
@@ -7630,7 +7630,7 @@
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,ECONOMIA,PSICOLOGIA,SAÚDE,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ORÇAMENTO,URBANISMO,AVALIAÇÃO DE IMÓVEIS</t>
+    <t>ECONOMIA,SAÚDE,PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,ASSISTÊNCIA SOCIAL,URBANISMO,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
   </si>
 </sst>
 </file>
@@ -18943,7 +18943,7 @@
     </row>
     <row r="313" spans="1:12">
       <c r="A313" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B313" t="s">
         <v>351</v>
@@ -18964,7 +18964,7 @@
         <v>1555</v>
       </c>
       <c r="I313" t="s">
-        <v>1632</v>
+        <v>1588</v>
       </c>
       <c r="J313" t="s">
         <v>2000</v>
@@ -30566,7 +30566,7 @@
         <v>2392</v>
       </c>
       <c r="L642" t="s">
-        <v>2498</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="643" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-07 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5035,6 +5035,9 @@
     <t>DANIEL FONTANA OBERLING,EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
   </si>
   <si>
+    <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
+  </si>
+  <si>
     <t>ANA LÍCIA SOUZA E SILVA</t>
   </si>
   <si>
@@ -5114,9 +5117,6 @@
   </si>
   <si>
     <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
   </si>
   <si>
     <t>LEONARDO ARAÚJO DE SOUZA,RENATA DE ARAUJO RIOS</t>
@@ -19178,7 +19178,7 @@
         <v>1566</v>
       </c>
       <c r="I318" t="s">
-        <v>1598</v>
+        <v>1673</v>
       </c>
       <c r="J318" t="s">
         <v>2017</v>
@@ -19213,7 +19213,7 @@
         <v>1566</v>
       </c>
       <c r="I319" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J319" t="s">
         <v>2018</v>
@@ -20193,7 +20193,7 @@
         <v>1566</v>
       </c>
       <c r="I347" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J347" t="s">
         <v>2046</v>
@@ -20438,7 +20438,7 @@
         <v>1566</v>
       </c>
       <c r="I354" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="J354" t="s">
         <v>2053</v>
@@ -20473,7 +20473,7 @@
         <v>1566</v>
       </c>
       <c r="I355" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J355" t="s">
         <v>2054</v>
@@ -20508,7 +20508,7 @@
         <v>1566</v>
       </c>
       <c r="I356" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="J356" t="s">
         <v>2055</v>
@@ -20928,7 +20928,7 @@
         <v>1566</v>
       </c>
       <c r="I368" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="J368" t="s">
         <v>2067</v>
@@ -21103,7 +21103,7 @@
         <v>1566</v>
       </c>
       <c r="I373" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="J373" t="s">
         <v>2072</v>
@@ -21243,7 +21243,7 @@
         <v>1566</v>
       </c>
       <c r="I377" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J377" t="s">
         <v>2076</v>
@@ -21488,7 +21488,7 @@
         <v>1566</v>
       </c>
       <c r="I384" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J384" t="s">
         <v>2083</v>
@@ -21663,7 +21663,7 @@
         <v>1566</v>
       </c>
       <c r="I389" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J389" t="s">
         <v>2088</v>
@@ -21908,7 +21908,7 @@
         <v>1566</v>
       </c>
       <c r="I396" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="J396" t="s">
         <v>2095</v>
@@ -22188,7 +22188,7 @@
         <v>1566</v>
       </c>
       <c r="I404" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J404" t="s">
         <v>2103</v>
@@ -23066,7 +23066,7 @@
         <v>1566</v>
       </c>
       <c r="I429" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J429" t="s">
         <v>2128</v>
@@ -23101,7 +23101,7 @@
         <v>1566</v>
       </c>
       <c r="I430" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J430" t="s">
         <v>2129</v>
@@ -23136,7 +23136,7 @@
         <v>1566</v>
       </c>
       <c r="I431" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J431" t="s">
         <v>2130</v>
@@ -23419,7 +23419,7 @@
         <v>1566</v>
       </c>
       <c r="I439" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J439" t="s">
         <v>2138</v>
@@ -23629,7 +23629,7 @@
         <v>1566</v>
       </c>
       <c r="I445" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J445" t="s">
         <v>2144</v>
@@ -23734,7 +23734,7 @@
         <v>1566</v>
       </c>
       <c r="I448" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J448" t="s">
         <v>2147</v>
@@ -23874,7 +23874,7 @@
         <v>1566</v>
       </c>
       <c r="I452" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J452" t="s">
         <v>2151</v>
@@ -23979,7 +23979,7 @@
         <v>1566</v>
       </c>
       <c r="I455" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="J455" t="s">
         <v>2154</v>
@@ -24224,7 +24224,7 @@
         <v>1566</v>
       </c>
       <c r="I462" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J462" t="s">
         <v>2161</v>
@@ -24294,7 +24294,7 @@
         <v>1566</v>
       </c>
       <c r="I464" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J464" t="s">
         <v>2163</v>
@@ -24329,7 +24329,7 @@
         <v>1566</v>
       </c>
       <c r="I465" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J465" t="s">
         <v>2164</v>
@@ -24828,7 +24828,7 @@
         <v>1557</v>
       </c>
       <c r="I479" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="J479" t="s">
         <v>2178</v>
@@ -25003,7 +25003,7 @@
         <v>1566</v>
       </c>
       <c r="I484" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J484" t="s">
         <v>2183</v>
@@ -25178,7 +25178,7 @@
         <v>1566</v>
       </c>
       <c r="I489" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="J489" t="s">
         <v>2188</v>
@@ -25356,7 +25356,7 @@
         <v>1578</v>
       </c>
       <c r="I494" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J494" t="s">
         <v>2193</v>
@@ -25426,7 +25426,7 @@
         <v>1566</v>
       </c>
       <c r="I496" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J496" t="s">
         <v>2195</v>
@@ -25499,7 +25499,7 @@
         <v>1531</v>
       </c>
       <c r="I498" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J498" t="s">
         <v>2197</v>
@@ -25569,7 +25569,7 @@
         <v>1566</v>
       </c>
       <c r="I500" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J500" t="s">
         <v>2199</v>
@@ -25782,7 +25782,7 @@
         <v>1579</v>
       </c>
       <c r="I506" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J506" t="s">
         <v>2205</v>
@@ -25852,7 +25852,7 @@
         <v>1566</v>
       </c>
       <c r="I508" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="J508" t="s">
         <v>2207</v>
@@ -25925,7 +25925,7 @@
         <v>1551</v>
       </c>
       <c r="I510" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J510" t="s">
         <v>2209</v>
@@ -26275,7 +26275,7 @@
         <v>1566</v>
       </c>
       <c r="I520" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J520" t="s">
         <v>2219</v>
@@ -26345,7 +26345,7 @@
         <v>1566</v>
       </c>
       <c r="I522" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J522" t="s">
         <v>2221</v>
@@ -26380,7 +26380,7 @@
         <v>1566</v>
       </c>
       <c r="I523" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J523" t="s">
         <v>2222</v>
@@ -26415,7 +26415,7 @@
         <v>1566</v>
       </c>
       <c r="I524" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J524" t="s">
         <v>2223</v>
@@ -26520,7 +26520,7 @@
         <v>1566</v>
       </c>
       <c r="I527" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="J527" t="s">
         <v>1888</v>
@@ -26555,7 +26555,7 @@
         <v>1566</v>
       </c>
       <c r="I528" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="J528" t="s">
         <v>2226</v>
@@ -26625,7 +26625,7 @@
         <v>1566</v>
       </c>
       <c r="I530" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J530" t="s">
         <v>2228</v>
@@ -26695,7 +26695,7 @@
         <v>1566</v>
       </c>
       <c r="I532" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J532" t="s">
         <v>2230</v>
@@ -26730,7 +26730,7 @@
         <v>1566</v>
       </c>
       <c r="I533" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J533" t="s">
         <v>2231</v>
@@ -26905,7 +26905,7 @@
         <v>1566</v>
       </c>
       <c r="I538" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J538" t="s">
         <v>2236</v>
@@ -26940,7 +26940,7 @@
         <v>1566</v>
       </c>
       <c r="I539" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="J539" t="s">
         <v>2237</v>
@@ -27045,7 +27045,7 @@
         <v>1566</v>
       </c>
       <c r="I542" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J542" t="s">
         <v>2240</v>
@@ -27255,7 +27255,7 @@
         <v>1566</v>
       </c>
       <c r="I548" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J548" t="s">
         <v>2245</v>
@@ -27328,7 +27328,7 @@
         <v>1566</v>
       </c>
       <c r="I550" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J550" t="s">
         <v>2247</v>
@@ -27363,7 +27363,7 @@
         <v>1566</v>
       </c>
       <c r="I551" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J551" t="s">
         <v>2248</v>
@@ -27398,7 +27398,7 @@
         <v>1566</v>
       </c>
       <c r="I552" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J552" t="s">
         <v>2249</v>
@@ -27471,7 +27471,7 @@
         <v>1581</v>
       </c>
       <c r="I554" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J554" t="s">
         <v>2251</v>
@@ -27506,7 +27506,7 @@
         <v>1566</v>
       </c>
       <c r="I555" t="s">
-        <v>1700</v>
+        <v>1673</v>
       </c>
       <c r="J555" t="s">
         <v>2252</v>
@@ -27541,7 +27541,7 @@
         <v>1566</v>
       </c>
       <c r="I556" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J556" t="s">
         <v>2253</v>
@@ -27754,7 +27754,7 @@
         <v>1566</v>
       </c>
       <c r="I562" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J562" t="s">
         <v>2258</v>
@@ -27894,7 +27894,7 @@
         <v>1566</v>
       </c>
       <c r="I566" t="s">
-        <v>1700</v>
+        <v>1673</v>
       </c>
       <c r="J566" t="s">
         <v>2262</v>
@@ -27964,7 +27964,7 @@
         <v>1566</v>
       </c>
       <c r="I568" t="s">
-        <v>1700</v>
+        <v>1673</v>
       </c>
       <c r="J568" t="s">
         <v>2264</v>
@@ -28139,7 +28139,7 @@
         <v>1566</v>
       </c>
       <c r="I573" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J573" t="s">
         <v>2269</v>
@@ -28209,7 +28209,7 @@
         <v>1566</v>
       </c>
       <c r="I575" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J575" t="s">
         <v>2271</v>
@@ -28244,7 +28244,7 @@
         <v>1566</v>
       </c>
       <c r="I576" t="s">
-        <v>1700</v>
+        <v>1673</v>
       </c>
       <c r="J576" t="s">
         <v>2272</v>
@@ -28495,7 +28495,7 @@
         <v>1566</v>
       </c>
       <c r="I583" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J583" t="s">
         <v>2278</v>
@@ -28565,7 +28565,7 @@
         <v>1566</v>
       </c>
       <c r="I585" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J585" t="s">
         <v>2280</v>
@@ -28705,7 +28705,7 @@
         <v>1566</v>
       </c>
       <c r="I589" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J589" t="s">
         <v>2283</v>
@@ -28778,7 +28778,7 @@
         <v>1566</v>
       </c>
       <c r="I591" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J591" t="s">
         <v>2285</v>
@@ -28883,7 +28883,7 @@
         <v>1566</v>
       </c>
       <c r="I594" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J594" t="s">
         <v>2288</v>
@@ -28918,7 +28918,7 @@
         <v>1566</v>
       </c>
       <c r="I595" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J595" t="s">
         <v>2289</v>
@@ -28953,7 +28953,7 @@
         <v>1566</v>
       </c>
       <c r="I596" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J596" t="s">
         <v>2290</v>
@@ -29061,7 +29061,7 @@
         <v>1566</v>
       </c>
       <c r="I599" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J599" t="s">
         <v>2293</v>
@@ -29096,7 +29096,7 @@
         <v>1566</v>
       </c>
       <c r="I600" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J600" t="s">
         <v>2294</v>
@@ -29131,7 +29131,7 @@
         <v>1566</v>
       </c>
       <c r="I601" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J601" t="s">
         <v>2295</v>
@@ -29271,7 +29271,7 @@
         <v>1566</v>
       </c>
       <c r="I605" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="J605" t="s">
         <v>2299</v>
@@ -29382,7 +29382,7 @@
         <v>1566</v>
       </c>
       <c r="I608" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J608" t="s">
         <v>2302</v>
@@ -29417,7 +29417,7 @@
         <v>1566</v>
       </c>
       <c r="I609" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J609" t="s">
         <v>2303</v>
@@ -29452,7 +29452,7 @@
         <v>1566</v>
       </c>
       <c r="I610" t="s">
-        <v>1700</v>
+        <v>1673</v>
       </c>
       <c r="J610" t="s">
         <v>2304</v>
@@ -29627,7 +29627,7 @@
         <v>1566</v>
       </c>
       <c r="I615" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J615" t="s">
         <v>2309</v>
@@ -29884,7 +29884,7 @@
         <v>1566</v>
       </c>
       <c r="I622" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J622" t="s">
         <v>2316</v>
@@ -29989,7 +29989,7 @@
         <v>1566</v>
       </c>
       <c r="I625" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J625" t="s">
         <v>2319</v>
@@ -30024,7 +30024,7 @@
         <v>1566</v>
       </c>
       <c r="I626" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J626" t="s">
         <v>2320</v>
@@ -30059,7 +30059,7 @@
         <v>1566</v>
       </c>
       <c r="I627" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J627" t="s">
         <v>2321</v>
@@ -30234,7 +30234,7 @@
         <v>1566</v>
       </c>
       <c r="I632" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J632" t="s">
         <v>2326</v>
@@ -30342,7 +30342,7 @@
         <v>1586</v>
       </c>
       <c r="I635" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J635" t="s">
         <v>2329</v>
@@ -30380,7 +30380,7 @@
         <v>1586</v>
       </c>
       <c r="I636" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J636" t="s">
         <v>2330</v>
@@ -30450,7 +30450,7 @@
         <v>1566</v>
       </c>
       <c r="I638" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J638" t="s">
         <v>2332</v>
@@ -30558,7 +30558,7 @@
         <v>1566</v>
       </c>
       <c r="I641" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J641" t="s">
         <v>2335</v>
@@ -30680,7 +30680,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B645" t="s">
         <v>683</v>
@@ -30704,7 +30704,7 @@
         <v>1588</v>
       </c>
       <c r="I645" t="s">
-        <v>1598</v>
+        <v>1708</v>
       </c>
       <c r="J645" t="s">
         <v>2339</v>
@@ -30739,7 +30739,7 @@
         <v>1566</v>
       </c>
       <c r="I646" t="s">
-        <v>1598</v>
+        <v>1704</v>
       </c>
       <c r="J646" t="s">
         <v>2340</v>
@@ -30774,7 +30774,7 @@
         <v>1566</v>
       </c>
       <c r="I647" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J647" t="s">
         <v>2341</v>
@@ -30788,7 +30788,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B648" t="s">
         <v>686</v>
@@ -30809,7 +30809,7 @@
         <v>1566</v>
       </c>
       <c r="I648" t="s">
-        <v>1598</v>
+        <v>1708</v>
       </c>
       <c r="J648" t="s">
         <v>2342</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-08 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -109,6 +109,9 @@
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
+    <t>NÚCLEO TÉCNICO DE ENGENHARIA, SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE ECONOMIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -128,9 +131,6 @@
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE CONTABILIDADE, NÚCLEO TÉCNICO DE CONTABILIDADE</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE ENGENHARIA, SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE</t>
@@ -12078,7 +12078,7 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B116" t="s">
         <v>155</v>
@@ -12533,7 +12533,7 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B129" t="s">
         <v>168</v>
@@ -12778,7 +12778,7 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B136" t="s">
         <v>175</v>
@@ -14248,7 +14248,7 @@
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B178" t="s">
         <v>217</v>
@@ -18460,7 +18460,7 @@
     </row>
     <row r="298" spans="1:12">
       <c r="A298" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B298" t="s">
         <v>337</v>
@@ -18635,7 +18635,7 @@
     </row>
     <row r="303" spans="1:12">
       <c r="A303" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B303" t="s">
         <v>342</v>
@@ -21890,7 +21890,7 @@
     </row>
     <row r="396" spans="1:12">
       <c r="A396" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B396" t="s">
         <v>435</v>
@@ -22978,7 +22978,7 @@
     </row>
     <row r="427" spans="1:12">
       <c r="A427" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B427" t="s">
         <v>466</v>
@@ -23821,7 +23821,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B451" t="s">
         <v>490</v>
@@ -25764,7 +25764,7 @@
     </row>
     <row r="506" spans="1:12">
       <c r="A506" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B506" t="s">
         <v>545</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-13 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4855,7 +4855,7 @@
     <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
-    <t>MANOELA DE MORAES SILVA, _SEM USUARIO ATRIBUIDO</t>
+    <t>MANOELA DE MORAES SILVA, VÍTOR MENDONÇA CELANE PINHEIRO</t>
   </si>
   <si>
     <t>MARCELO TEIXEIRA SANTANA</t>
@@ -13890,7 +13890,7 @@
         <v>1568</v>
       </c>
       <c r="I167" t="s">
-        <v>1601</v>
+        <v>1598</v>
       </c>
       <c r="J167" t="s">
         <v>1871</v>
@@ -30537,7 +30537,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B641" t="s">
         <v>680</v>
@@ -30558,7 +30558,7 @@
         <v>1568</v>
       </c>
       <c r="I641" t="s">
-        <v>1601</v>
+        <v>1679</v>
       </c>
       <c r="J641" t="s">
         <v>2338</v>
@@ -30596,7 +30596,7 @@
         <v>1591</v>
       </c>
       <c r="I642" t="s">
-        <v>1601</v>
+        <v>1707</v>
       </c>
       <c r="J642" t="s">
         <v>2339</v>
@@ -30634,7 +30634,7 @@
         <v>1591</v>
       </c>
       <c r="I643" t="s">
-        <v>1601</v>
+        <v>1707</v>
       </c>
       <c r="J643" t="s">
         <v>2340</v>
@@ -30672,7 +30672,7 @@
         <v>1591</v>
       </c>
       <c r="I644" t="s">
-        <v>1601</v>
+        <v>1707</v>
       </c>
       <c r="J644" t="s">
         <v>2341</v>
@@ -30686,7 +30686,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B645" t="s">
         <v>684</v>
@@ -30707,7 +30707,7 @@
         <v>1568</v>
       </c>
       <c r="I645" t="s">
-        <v>1601</v>
+        <v>1679</v>
       </c>
       <c r="J645" t="s">
         <v>2342</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-15 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -22828,7 +22828,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B430" t="s">
         <v>468</v>
@@ -22843,13 +22843,13 @@
         <v>62</v>
       </c>
       <c r="F430" t="s">
-        <v>1515</v>
+        <v>1514</v>
       </c>
       <c r="G430" t="s">
         <v>1519</v>
       </c>
       <c r="I430" t="s">
-        <v>1594</v>
+        <v>1630</v>
       </c>
       <c r="J430" t="s">
         <v>2073</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-15 14:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -115,6 +115,9 @@
     <t>NÚCLEO TÉCNICO DE CONTABILIDADE,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
   </si>
   <si>
@@ -133,9 +136,6 @@
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO, SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>20.22.0001.0070364.2024-27</t>
   </si>
   <si>
@@ -4822,52 +4822,52 @@
     <t>GLAUCO CASTILHO DE ALMEIDA</t>
   </si>
   <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>ANDRÉA DINIZ MATTOS</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>REINALDO DE SOUZA MACHADO</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>PAULA DE ARAUJO CRUZ VIGIO</t>
+  </si>
+  <si>
     <t>NIVANA DANIELLE SILVA COSTA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>ANDRÉA DINIZ MATTOS</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>PAULA DE ARAUJO CRUZ VIGIO</t>
   </si>
   <si>
     <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
@@ -10902,7 +10902,7 @@
         <v>1657</v>
       </c>
       <c r="K89" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="L89" t="s">
         <v>2402</v>
@@ -14063,7 +14063,7 @@
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B180" t="s">
         <v>218</v>
@@ -14087,7 +14087,7 @@
         <v>1525</v>
       </c>
       <c r="I180" t="s">
-        <v>1602</v>
+        <v>1549</v>
       </c>
       <c r="J180" t="s">
         <v>1827</v>
@@ -14227,7 +14227,7 @@
         <v>1519</v>
       </c>
       <c r="I184" t="s">
-        <v>1603</v>
+        <v>1602</v>
       </c>
       <c r="J184" t="s">
         <v>1831</v>
@@ -14262,7 +14262,7 @@
         <v>1519</v>
       </c>
       <c r="I185" t="s">
-        <v>1604</v>
+        <v>1603</v>
       </c>
       <c r="J185" t="s">
         <v>1832</v>
@@ -14332,7 +14332,7 @@
         <v>1519</v>
       </c>
       <c r="I187" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J187" t="s">
         <v>1834</v>
@@ -14682,7 +14682,7 @@
         <v>1519</v>
       </c>
       <c r="I197" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="J197" t="s">
         <v>1842</v>
@@ -14927,7 +14927,7 @@
         <v>1519</v>
       </c>
       <c r="I204" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="J204" t="s">
         <v>1849</v>
@@ -14997,7 +14997,7 @@
         <v>1519</v>
       </c>
       <c r="I206" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J206" t="s">
         <v>1851</v>
@@ -15032,7 +15032,7 @@
         <v>1519</v>
       </c>
       <c r="I207" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="J207" t="s">
         <v>1852</v>
@@ -15102,7 +15102,7 @@
         <v>1519</v>
       </c>
       <c r="I209" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="J209" t="s">
         <v>1854</v>
@@ -15280,7 +15280,7 @@
         <v>1519</v>
       </c>
       <c r="I214" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J214" t="s">
         <v>1859</v>
@@ -15385,7 +15385,7 @@
         <v>1519</v>
       </c>
       <c r="I217" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="J217" t="s">
         <v>1862</v>
@@ -15490,7 +15490,7 @@
         <v>1519</v>
       </c>
       <c r="I220" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J220" t="s">
         <v>1865</v>
@@ -15700,7 +15700,7 @@
         <v>1519</v>
       </c>
       <c r="I226" t="s">
-        <v>1614</v>
+        <v>1613</v>
       </c>
       <c r="J226" t="s">
         <v>1871</v>
@@ -15910,7 +15910,7 @@
         <v>1519</v>
       </c>
       <c r="I232" t="s">
-        <v>1615</v>
+        <v>1614</v>
       </c>
       <c r="J232" t="s">
         <v>1877</v>
@@ -16053,7 +16053,7 @@
         <v>1519</v>
       </c>
       <c r="I236" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="J236" t="s">
         <v>1881</v>
@@ -16158,7 +16158,7 @@
         <v>1519</v>
       </c>
       <c r="I239" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="J239" t="s">
         <v>1884</v>
@@ -16263,7 +16263,7 @@
         <v>1519</v>
       </c>
       <c r="I242" t="s">
-        <v>1549</v>
+        <v>1617</v>
       </c>
       <c r="J242" t="s">
         <v>1887</v>
@@ -16438,7 +16438,7 @@
         <v>1519</v>
       </c>
       <c r="I247" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J247" t="s">
         <v>1892</v>
@@ -16508,7 +16508,7 @@
         <v>1519</v>
       </c>
       <c r="I249" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J249" t="s">
         <v>1894</v>
@@ -16613,7 +16613,7 @@
         <v>1519</v>
       </c>
       <c r="I252" t="s">
-        <v>1614</v>
+        <v>1613</v>
       </c>
       <c r="J252" t="s">
         <v>1897</v>
@@ -17208,7 +17208,7 @@
         <v>1519</v>
       </c>
       <c r="I269" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J269" t="s">
         <v>1914</v>
@@ -17747,7 +17747,7 @@
     </row>
     <row r="285" spans="1:12">
       <c r="A285" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B285" t="s">
         <v>323</v>
@@ -18363,7 +18363,7 @@
         <v>1519</v>
       </c>
       <c r="I302" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J302" t="s">
         <v>1945</v>
@@ -18783,7 +18783,7 @@
         <v>1519</v>
       </c>
       <c r="I314" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J314" t="s">
         <v>1957</v>
@@ -19483,7 +19483,7 @@
         <v>1519</v>
       </c>
       <c r="I334" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J334" t="s">
         <v>1977</v>
@@ -19623,7 +19623,7 @@
         <v>1519</v>
       </c>
       <c r="I338" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J338" t="s">
         <v>1981</v>
@@ -20288,7 +20288,7 @@
         <v>1519</v>
       </c>
       <c r="I357" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J357" t="s">
         <v>2000</v>
@@ -20393,7 +20393,7 @@
         <v>1519</v>
       </c>
       <c r="I360" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="J360" t="s">
         <v>2003</v>
@@ -20757,7 +20757,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B371" t="s">
         <v>409</v>
@@ -20953,7 +20953,7 @@
         <v>1519</v>
       </c>
       <c r="I376" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J376" t="s">
         <v>2019</v>
@@ -21236,7 +21236,7 @@
         <v>1519</v>
       </c>
       <c r="I384" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J384" t="s">
         <v>2027</v>
@@ -21586,7 +21586,7 @@
         <v>1519</v>
       </c>
       <c r="I394" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J394" t="s">
         <v>2037</v>
@@ -21621,7 +21621,7 @@
         <v>1519</v>
       </c>
       <c r="I395" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J395" t="s">
         <v>2038</v>
@@ -21656,7 +21656,7 @@
         <v>1519</v>
       </c>
       <c r="I396" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="J396" t="s">
         <v>2039</v>
@@ -21845,7 +21845,7 @@
     </row>
     <row r="402" spans="1:12">
       <c r="A402" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B402" t="s">
         <v>440</v>
@@ -22114,7 +22114,7 @@
         <v>1519</v>
       </c>
       <c r="I409" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J409" t="s">
         <v>2052</v>
@@ -22219,7 +22219,7 @@
         <v>1519</v>
       </c>
       <c r="I412" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J412" t="s">
         <v>2055</v>
@@ -22254,7 +22254,7 @@
         <v>1519</v>
       </c>
       <c r="I413" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J413" t="s">
         <v>2056</v>
@@ -22499,7 +22499,7 @@
         <v>1519</v>
       </c>
       <c r="I420" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J420" t="s">
         <v>2063</v>
@@ -22548,7 +22548,7 @@
     </row>
     <row r="422" spans="1:12">
       <c r="A422" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B422" t="s">
         <v>460</v>
@@ -23027,7 +23027,7 @@
         <v>1519</v>
       </c>
       <c r="I435" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J435" t="s">
         <v>2078</v>
@@ -23453,7 +23453,7 @@
         <v>1519</v>
       </c>
       <c r="I447" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="J447" t="s">
         <v>2090</v>
@@ -23978,7 +23978,7 @@
         <v>1519</v>
       </c>
       <c r="I462" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J462" t="s">
         <v>2105</v>
@@ -24013,7 +24013,7 @@
         <v>1519</v>
       </c>
       <c r="I463" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J463" t="s">
         <v>2106</v>
@@ -24401,7 +24401,7 @@
         <v>1519</v>
       </c>
       <c r="I474" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J474" t="s">
         <v>2117</v>
@@ -24471,7 +24471,7 @@
         <v>1519</v>
       </c>
       <c r="I476" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J476" t="s">
         <v>2119</v>
@@ -24541,7 +24541,7 @@
         <v>1519</v>
       </c>
       <c r="I478" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J478" t="s">
         <v>2121</v>
@@ -24765,7 +24765,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B485" t="s">
         <v>523</v>
@@ -24835,7 +24835,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B487" t="s">
         <v>525</v>
@@ -24891,7 +24891,7 @@
         <v>1519</v>
       </c>
       <c r="I488" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J488" t="s">
         <v>2131</v>
@@ -25381,7 +25381,7 @@
         <v>1519</v>
       </c>
       <c r="I502" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J502" t="s">
         <v>2145</v>
@@ -25804,7 +25804,7 @@
         <v>1519</v>
       </c>
       <c r="I514" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J514" t="s">
         <v>2157</v>
@@ -25874,7 +25874,7 @@
         <v>1519</v>
       </c>
       <c r="I516" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J516" t="s">
         <v>2159</v>
@@ -25888,7 +25888,7 @@
     </row>
     <row r="517" spans="1:12">
       <c r="A517" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B517" t="s">
         <v>555</v>
@@ -25958,7 +25958,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B519" t="s">
         <v>557</v>
@@ -26203,7 +26203,7 @@
     </row>
     <row r="526" spans="1:12">
       <c r="A526" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B526" t="s">
         <v>564</v>
@@ -26434,7 +26434,7 @@
         <v>1519</v>
       </c>
       <c r="I532" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J532" t="s">
         <v>2175</v>
@@ -26825,7 +26825,7 @@
         <v>1534</v>
       </c>
       <c r="I543" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J543" t="s">
         <v>2186</v>
@@ -26860,7 +26860,7 @@
         <v>1519</v>
       </c>
       <c r="I544" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J544" t="s">
         <v>2187</v>
@@ -27000,7 +27000,7 @@
         <v>1519</v>
       </c>
       <c r="I548" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J548" t="s">
         <v>2191</v>
@@ -27192,7 +27192,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B554" t="s">
         <v>592</v>
@@ -27248,7 +27248,7 @@
         <v>1519</v>
       </c>
       <c r="I555" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J555" t="s">
         <v>2198</v>
@@ -27402,7 +27402,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B560" t="s">
         <v>598</v>
@@ -27706,7 +27706,7 @@
         <v>1519</v>
       </c>
       <c r="I568" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J568" t="s">
         <v>2211</v>
@@ -27811,7 +27811,7 @@
         <v>1519</v>
       </c>
       <c r="I571" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J571" t="s">
         <v>2214</v>
@@ -28027,7 +28027,7 @@
         <v>1519</v>
       </c>
       <c r="I577" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J577" t="s">
         <v>2220</v>
@@ -28132,7 +28132,7 @@
         <v>1519</v>
       </c>
       <c r="I580" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J580" t="s">
         <v>2223</v>
@@ -28415,7 +28415,7 @@
         <v>1519</v>
       </c>
       <c r="I588" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J588" t="s">
         <v>2231</v>
@@ -28485,7 +28485,7 @@
         <v>1519</v>
       </c>
       <c r="I590" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J590" t="s">
         <v>2233</v>
@@ -28663,7 +28663,7 @@
         <v>1519</v>
       </c>
       <c r="I595" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J595" t="s">
         <v>2238</v>
@@ -28733,7 +28733,7 @@
         <v>1519</v>
       </c>
       <c r="I597" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J597" t="s">
         <v>2240</v>
@@ -29027,7 +29027,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B606" t="s">
         <v>644</v>
@@ -29413,7 +29413,7 @@
         <v>1521</v>
       </c>
       <c r="I616" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J616" t="s">
         <v>2258</v>
@@ -29462,7 +29462,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B618" t="s">
         <v>656</v>
@@ -29602,7 +29602,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B622" t="s">
         <v>659</v>
@@ -29731,7 +29731,7 @@
         <v>1519</v>
       </c>
       <c r="I625" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J625" t="s">
         <v>2266</v>
@@ -29745,7 +29745,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B626" t="s">
         <v>663</v>
@@ -29766,7 +29766,7 @@
         <v>1519</v>
       </c>
       <c r="I626" t="s">
-        <v>1592</v>
+        <v>1644</v>
       </c>
       <c r="J626" t="s">
         <v>2267</v>
@@ -29853,7 +29853,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B629" t="s">
         <v>666</v>
@@ -29885,7 +29885,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B630" t="s">
         <v>667</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-17 12:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6367" uniqueCount="2482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6367" uniqueCount="2481">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7393,7 +7393,7 @@
     <t>VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7420,7 +7420,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7441,7 +7441,7 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
@@ -7450,16 +7450,13 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ORÇAMENTO,ECONOMIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,ASSISTÊNCIA SOCIAL,SAÚDE,ECONOMICIDADE CONTÁBIL,URBANISMO,PSICOLOGIA,SAÚDE MENTAL</t>
+    <t>ASSISTÊNCIA SOCIAL,ECONOMIA,MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL,URBANISMO,SAÚDE MENTAL,PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -13122,7 +13119,7 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B152" t="s">
         <v>189</v>
@@ -13143,7 +13140,7 @@
         <v>1528</v>
       </c>
       <c r="I152" t="s">
-        <v>1594</v>
+        <v>1556</v>
       </c>
       <c r="J152" t="s">
         <v>1810</v>
@@ -14592,7 +14589,7 @@
     </row>
     <row r="194" spans="1:12">
       <c r="A194" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B194" t="s">
         <v>231</v>
@@ -14613,7 +14610,7 @@
         <v>1528</v>
       </c>
       <c r="I194" t="s">
-        <v>1594</v>
+        <v>1556</v>
       </c>
       <c r="J194" t="s">
         <v>1850</v>
@@ -16243,7 +16240,7 @@
     </row>
     <row r="241" spans="1:12">
       <c r="A241" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B241" t="s">
         <v>278</v>
@@ -16264,7 +16261,7 @@
         <v>1528</v>
       </c>
       <c r="I241" t="s">
-        <v>1594</v>
+        <v>1556</v>
       </c>
       <c r="J241" t="s">
         <v>1897</v>
@@ -17643,7 +17640,7 @@
     </row>
     <row r="281" spans="1:12">
       <c r="A281" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B281" t="s">
         <v>318</v>
@@ -17664,7 +17661,7 @@
         <v>1528</v>
       </c>
       <c r="I281" t="s">
-        <v>1594</v>
+        <v>1556</v>
       </c>
       <c r="J281" t="s">
         <v>1936</v>
@@ -23363,7 +23360,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B444" t="s">
         <v>481</v>
@@ -23384,7 +23381,7 @@
         <v>1528</v>
       </c>
       <c r="I444" t="s">
-        <v>1628</v>
+        <v>1633</v>
       </c>
       <c r="J444" t="s">
         <v>2098</v>
@@ -24857,7 +24854,7 @@
         <v>1528</v>
       </c>
       <c r="I486" t="s">
-        <v>1556</v>
+        <v>1598</v>
       </c>
       <c r="J486" t="s">
         <v>2140</v>
@@ -26840,7 +26837,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B543" t="s">
         <v>580</v>
@@ -26861,7 +26858,7 @@
         <v>1528</v>
       </c>
       <c r="I543" t="s">
-        <v>1594</v>
+        <v>1556</v>
       </c>
       <c r="J543" t="s">
         <v>2197</v>
@@ -29881,7 +29878,7 @@
         <v>2343</v>
       </c>
       <c r="L628" t="s">
-        <v>2471</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30021,7 +30018,7 @@
         <v>2329</v>
       </c>
       <c r="L632" t="s">
-        <v>2471</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30053,7 +30050,7 @@
         <v>2410</v>
       </c>
       <c r="L633" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30085,7 +30082,7 @@
         <v>2410</v>
       </c>
       <c r="L634" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-20 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7435,7 +7435,7 @@
     <t>VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7483,7 +7483,7 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
@@ -7492,7 +7492,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
@@ -7504,10 +7504,10 @@
     <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>BIOLOGIA,RESÍDUOS SÓLIDOS,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>ASSISTÊNCIA SOCIAL,PSICOLOGIA,ECONOMIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,URBANISMO,SAÚDE,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL</t>
+    <t>RESÍDUOS SÓLIDOS,ENGENHARIA AMBIENTAL,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,ECONOMIA,PSICOLOGIA,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,MOBILIDADE E TRANSPORTE,URBANISMO,SAÚDE</t>
   </si>
 </sst>
 </file>
@@ -30171,7 +30171,7 @@
         <v>2364</v>
       </c>
       <c r="L635" t="s">
-        <v>2485</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="636" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-21 04:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4969,6 +4969,9 @@
     <t>SERGIO PEDRO LOPES</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>JULIANA BUSTAMANTE DE MONTI SOUZA,JULIANA MARTINS BAHIENSE,RODRIGO VENTURA MARRA</t>
   </si>
   <si>
@@ -5033,9 +5036,6 @@
   </si>
   <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA, PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
@@ -21862,7 +21862,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B400" t="s">
         <v>439</v>
@@ -21883,7 +21883,7 @@
         <v>1540</v>
       </c>
       <c r="I400" t="s">
-        <v>1626</v>
+        <v>1651</v>
       </c>
       <c r="J400" t="s">
         <v>2065</v>
@@ -22093,7 +22093,7 @@
         <v>1540</v>
       </c>
       <c r="I406" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J406" t="s">
         <v>2071</v>
@@ -22338,7 +22338,7 @@
         <v>1540</v>
       </c>
       <c r="I413" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J413" t="s">
         <v>2078</v>
@@ -22583,7 +22583,7 @@
         <v>1540</v>
       </c>
       <c r="I420" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J420" t="s">
         <v>2085</v>
@@ -23082,7 +23082,7 @@
         <v>1523</v>
       </c>
       <c r="I434" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J434" t="s">
         <v>2099</v>
@@ -23362,7 +23362,7 @@
         <v>1540</v>
       </c>
       <c r="I442" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J442" t="s">
         <v>2107</v>
@@ -23642,7 +23642,7 @@
         <v>1540</v>
       </c>
       <c r="I450" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J450" t="s">
         <v>2115</v>
@@ -23656,7 +23656,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B451" t="s">
         <v>490</v>
@@ -23677,7 +23677,7 @@
         <v>1540</v>
       </c>
       <c r="I451" t="s">
-        <v>1626</v>
+        <v>1651</v>
       </c>
       <c r="J451" t="s">
         <v>2116</v>
@@ -23855,7 +23855,7 @@
         <v>1551</v>
       </c>
       <c r="I456" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J456" t="s">
         <v>2121</v>
@@ -23925,7 +23925,7 @@
         <v>1540</v>
       </c>
       <c r="I458" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J458" t="s">
         <v>2123</v>
@@ -24310,7 +24310,7 @@
         <v>1540</v>
       </c>
       <c r="I469" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J469" t="s">
         <v>2134</v>
@@ -24380,7 +24380,7 @@
         <v>1540</v>
       </c>
       <c r="I471" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J471" t="s">
         <v>2136</v>
@@ -24450,7 +24450,7 @@
         <v>1540</v>
       </c>
       <c r="I473" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J473" t="s">
         <v>2138</v>
@@ -24555,7 +24555,7 @@
         <v>1540</v>
       </c>
       <c r="I476" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J476" t="s">
         <v>2141</v>
@@ -24625,7 +24625,7 @@
         <v>1540</v>
       </c>
       <c r="I478" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J478" t="s">
         <v>2143</v>
@@ -24695,7 +24695,7 @@
         <v>1540</v>
       </c>
       <c r="I480" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J480" t="s">
         <v>2145</v>
@@ -24730,7 +24730,7 @@
         <v>1540</v>
       </c>
       <c r="I481" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J481" t="s">
         <v>2146</v>
@@ -25115,7 +25115,7 @@
         <v>1540</v>
       </c>
       <c r="I492" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J492" t="s">
         <v>2157</v>
@@ -25150,7 +25150,7 @@
         <v>1540</v>
       </c>
       <c r="I493" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J493" t="s">
         <v>2158</v>
@@ -25185,7 +25185,7 @@
         <v>1540</v>
       </c>
       <c r="I494" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J494" t="s">
         <v>2159</v>
@@ -25258,7 +25258,7 @@
         <v>1552</v>
       </c>
       <c r="I496" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J496" t="s">
         <v>2161</v>
@@ -25328,7 +25328,7 @@
         <v>1540</v>
       </c>
       <c r="I498" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J498" t="s">
         <v>2163</v>
@@ -25433,7 +25433,7 @@
         <v>1540</v>
       </c>
       <c r="I501" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J501" t="s">
         <v>2166</v>
@@ -25853,7 +25853,7 @@
         <v>1540</v>
       </c>
       <c r="I513" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J513" t="s">
         <v>2178</v>
@@ -26098,7 +26098,7 @@
         <v>1540</v>
       </c>
       <c r="I520" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J520" t="s">
         <v>2185</v>
@@ -26241,7 +26241,7 @@
         <v>1540</v>
       </c>
       <c r="I524" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J524" t="s">
         <v>2189</v>
@@ -26346,7 +26346,7 @@
         <v>1540</v>
       </c>
       <c r="I527" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J527" t="s">
         <v>2192</v>
@@ -26381,7 +26381,7 @@
         <v>1540</v>
       </c>
       <c r="I528" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J528" t="s">
         <v>2193</v>
@@ -26416,7 +26416,7 @@
         <v>1540</v>
       </c>
       <c r="I529" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J529" t="s">
         <v>2194</v>
@@ -26594,7 +26594,7 @@
         <v>1540</v>
       </c>
       <c r="I534" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J534" t="s">
         <v>2199</v>
@@ -26734,7 +26734,7 @@
         <v>1540</v>
       </c>
       <c r="I538" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J538" t="s">
         <v>2203</v>
@@ -26769,7 +26769,7 @@
         <v>1540</v>
       </c>
       <c r="I539" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J539" t="s">
         <v>2204</v>
@@ -26979,7 +26979,7 @@
         <v>1540</v>
       </c>
       <c r="I545" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J545" t="s">
         <v>2210</v>
@@ -27017,7 +27017,7 @@
         <v>1532</v>
       </c>
       <c r="I546" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J546" t="s">
         <v>2211</v>
@@ -27087,7 +27087,7 @@
         <v>1540</v>
       </c>
       <c r="I548" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J548" t="s">
         <v>2213</v>
@@ -27192,7 +27192,7 @@
         <v>1540</v>
       </c>
       <c r="I551" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J551" t="s">
         <v>2216</v>
@@ -27472,7 +27472,7 @@
         <v>1540</v>
       </c>
       <c r="I559" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J559" t="s">
         <v>2224</v>
@@ -27580,7 +27580,7 @@
         <v>1540</v>
       </c>
       <c r="I562" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J562" t="s">
         <v>2227</v>
@@ -27863,7 +27863,7 @@
         <v>1540</v>
       </c>
       <c r="I570" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J570" t="s">
         <v>2235</v>
@@ -27898,7 +27898,7 @@
         <v>1540</v>
       </c>
       <c r="I571" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J571" t="s">
         <v>2236</v>
@@ -28111,7 +28111,7 @@
         <v>1540</v>
       </c>
       <c r="I577" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J577" t="s">
         <v>2242</v>
@@ -28216,7 +28216,7 @@
         <v>1540</v>
       </c>
       <c r="I580" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J580" t="s">
         <v>2245</v>
@@ -28286,7 +28286,7 @@
         <v>1540</v>
       </c>
       <c r="I582" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J582" t="s">
         <v>2246</v>
@@ -28321,7 +28321,7 @@
         <v>1540</v>
       </c>
       <c r="I583" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J583" t="s">
         <v>2247</v>
@@ -28391,7 +28391,7 @@
         <v>1540</v>
       </c>
       <c r="I585" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J585" t="s">
         <v>2249</v>
@@ -28426,7 +28426,7 @@
         <v>1540</v>
       </c>
       <c r="I586" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J586" t="s">
         <v>2250</v>
@@ -28496,7 +28496,7 @@
         <v>1540</v>
       </c>
       <c r="I588" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J588" t="s">
         <v>2252</v>
@@ -28636,7 +28636,7 @@
         <v>1540</v>
       </c>
       <c r="I592" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J592" t="s">
         <v>2256</v>
@@ -28674,7 +28674,7 @@
         <v>1556</v>
       </c>
       <c r="I593" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J593" t="s">
         <v>2257</v>
@@ -28712,7 +28712,7 @@
         <v>1556</v>
       </c>
       <c r="I594" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J594" t="s">
         <v>2258</v>
@@ -28750,7 +28750,7 @@
         <v>1556</v>
       </c>
       <c r="I595" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J595" t="s">
         <v>2259</v>
@@ -28785,7 +28785,7 @@
         <v>1540</v>
       </c>
       <c r="I596" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J596" t="s">
         <v>2260</v>
@@ -28928,7 +28928,7 @@
         <v>1540</v>
       </c>
       <c r="I600" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J600" t="s">
         <v>2264</v>
@@ -28963,7 +28963,7 @@
         <v>1540</v>
       </c>
       <c r="I601" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J601" t="s">
         <v>2265</v>
@@ -29033,7 +29033,7 @@
         <v>1540</v>
       </c>
       <c r="I603" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J603" t="s">
         <v>2266</v>
@@ -29103,7 +29103,7 @@
         <v>1540</v>
       </c>
       <c r="I605" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J605" t="s">
         <v>2268</v>
@@ -29138,7 +29138,7 @@
         <v>1540</v>
       </c>
       <c r="I606" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J606" t="s">
         <v>2269</v>
@@ -29208,7 +29208,7 @@
         <v>1540</v>
       </c>
       <c r="I608" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J608" t="s">
         <v>2271</v>
@@ -29243,7 +29243,7 @@
         <v>1540</v>
       </c>
       <c r="I609" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J609" t="s">
         <v>2272</v>
@@ -29278,7 +29278,7 @@
         <v>1540</v>
       </c>
       <c r="I610" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J610" t="s">
         <v>2273</v>
@@ -29348,7 +29348,7 @@
         <v>1540</v>
       </c>
       <c r="I612" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J612" t="s">
         <v>2275</v>
@@ -29418,7 +29418,7 @@
         <v>1540</v>
       </c>
       <c r="I614" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J614" t="s">
         <v>2276</v>
@@ -29523,7 +29523,7 @@
         <v>1540</v>
       </c>
       <c r="I617" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J617" t="s">
         <v>2279</v>
@@ -29666,7 +29666,7 @@
         <v>1540</v>
       </c>
       <c r="I621" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J621" t="s">
         <v>2282</v>
@@ -29736,7 +29736,7 @@
         <v>1540</v>
       </c>
       <c r="I623" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J623" t="s">
         <v>2284</v>
@@ -29774,7 +29774,7 @@
         <v>1558</v>
       </c>
       <c r="I624" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="J624" t="s">
         <v>2285</v>
@@ -29809,7 +29809,7 @@
         <v>1540</v>
       </c>
       <c r="I625" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J625" t="s">
         <v>2286</v>
@@ -29847,7 +29847,7 @@
         <v>1559</v>
       </c>
       <c r="I626" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J626" t="s">
         <v>2287</v>
@@ -29882,7 +29882,7 @@
         <v>1540</v>
       </c>
       <c r="I627" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J627" t="s">
         <v>2288</v>
@@ -29917,7 +29917,7 @@
         <v>1540</v>
       </c>
       <c r="I628" t="s">
-        <v>1673</v>
+        <v>1651</v>
       </c>
       <c r="J628" t="s">
         <v>2289</v>
@@ -29952,7 +29952,7 @@
         <v>1540</v>
       </c>
       <c r="I629" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J629" t="s">
         <v>2290</v>
@@ -30022,7 +30022,7 @@
         <v>1540</v>
       </c>
       <c r="I631" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J631" t="s">
         <v>2292</v>
@@ -30057,7 +30057,7 @@
         <v>1540</v>
       </c>
       <c r="I632" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J632" t="s">
         <v>2293</v>
@@ -30127,7 +30127,7 @@
         <v>1540</v>
       </c>
       <c r="I634" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J634" t="s">
         <v>2295</v>
@@ -30162,7 +30162,7 @@
         <v>1540</v>
       </c>
       <c r="I635" t="s">
-        <v>1673</v>
+        <v>1651</v>
       </c>
       <c r="J635" t="s">
         <v>2296</v>
@@ -30197,7 +30197,7 @@
         <v>1540</v>
       </c>
       <c r="I636" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J636" t="s">
         <v>2297</v>
@@ -30267,7 +30267,7 @@
         <v>1540</v>
       </c>
       <c r="I638" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J638" t="s">
         <v>2299</v>
@@ -30299,7 +30299,7 @@
         <v>1540</v>
       </c>
       <c r="I639" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J639" t="s">
         <v>2300</v>
@@ -30331,7 +30331,7 @@
         <v>1540</v>
       </c>
       <c r="I640" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J640" t="s">
         <v>2301</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-22 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4768,7 +4768,7 @@
     <t>MARCELO TEIXEIRA SANTANA</t>
   </si>
   <si>
-    <t>MAYRA LIMA VERISSIMO RAMOS MUNIVE, _SEM USUARIO ATRIBUIDO</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
   </si>
   <si>
     <t>PEDRO MARCELO ROCHA GOMES</t>
@@ -4900,6 +4900,9 @@
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
   </si>
   <si>
@@ -4919,9 +4922,6 @@
   </si>
   <si>
     <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>GLAUCO CASTILHO DE ALMEIDA</t>
@@ -13895,7 +13895,7 @@
         <v>1546</v>
       </c>
       <c r="I171" t="s">
-        <v>1574</v>
+        <v>1628</v>
       </c>
       <c r="J171" t="s">
         <v>1846</v>
@@ -13930,7 +13930,7 @@
         <v>1546</v>
       </c>
       <c r="I172" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J172" t="s">
         <v>1847</v>
@@ -14175,7 +14175,7 @@
         <v>1546</v>
       </c>
       <c r="I179" t="s">
-        <v>1574</v>
+        <v>1628</v>
       </c>
       <c r="J179" t="s">
         <v>1854</v>
@@ -14210,7 +14210,7 @@
         <v>1546</v>
       </c>
       <c r="I180" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J180" t="s">
         <v>1855</v>
@@ -14280,7 +14280,7 @@
         <v>1546</v>
       </c>
       <c r="I182" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J182" t="s">
         <v>1857</v>
@@ -14630,7 +14630,7 @@
         <v>1546</v>
       </c>
       <c r="I192" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J192" t="s">
         <v>1865</v>
@@ -14875,7 +14875,7 @@
         <v>1546</v>
       </c>
       <c r="I199" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="J199" t="s">
         <v>1872</v>
@@ -14945,7 +14945,7 @@
         <v>1546</v>
       </c>
       <c r="I201" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J201" t="s">
         <v>1874</v>
@@ -14980,7 +14980,7 @@
         <v>1546</v>
       </c>
       <c r="I202" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="J202" t="s">
         <v>1875</v>
@@ -15050,7 +15050,7 @@
         <v>1546</v>
       </c>
       <c r="I204" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
       <c r="J204" t="s">
         <v>1877</v>
@@ -16386,7 +16386,7 @@
         <v>1546</v>
       </c>
       <c r="I242" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J242" t="s">
         <v>1915</v>
@@ -16456,7 +16456,7 @@
         <v>1546</v>
       </c>
       <c r="I244" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J244" t="s">
         <v>1917</v>
@@ -18276,7 +18276,7 @@
         <v>1546</v>
       </c>
       <c r="I296" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J296" t="s">
         <v>1967</v>
@@ -18696,7 +18696,7 @@
         <v>1546</v>
       </c>
       <c r="I308" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J308" t="s">
         <v>1979</v>
@@ -19396,7 +19396,7 @@
         <v>1546</v>
       </c>
       <c r="I328" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J328" t="s">
         <v>1999</v>
@@ -19536,7 +19536,7 @@
         <v>1546</v>
       </c>
       <c r="I332" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J332" t="s">
         <v>2003</v>
@@ -20166,7 +20166,7 @@
         <v>1546</v>
       </c>
       <c r="I350" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J350" t="s">
         <v>2021</v>
@@ -20271,7 +20271,7 @@
         <v>1546</v>
       </c>
       <c r="I353" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J353" t="s">
         <v>2024</v>
@@ -20831,7 +20831,7 @@
         <v>1546</v>
       </c>
       <c r="I369" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J369" t="s">
         <v>2040</v>
@@ -21079,7 +21079,7 @@
         <v>1546</v>
       </c>
       <c r="I376" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J376" t="s">
         <v>2047</v>
@@ -21429,7 +21429,7 @@
         <v>1546</v>
       </c>
       <c r="I386" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J386" t="s">
         <v>2057</v>
@@ -21464,7 +21464,7 @@
         <v>1546</v>
       </c>
       <c r="I387" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J387" t="s">
         <v>2058</v>
@@ -21499,7 +21499,7 @@
         <v>1546</v>
       </c>
       <c r="I388" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J388" t="s">
         <v>2059</v>
@@ -21992,7 +21992,7 @@
         <v>1546</v>
       </c>
       <c r="I402" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J402" t="s">
         <v>2073</v>
@@ -22027,7 +22027,7 @@
         <v>1546</v>
       </c>
       <c r="I403" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J403" t="s">
         <v>2074</v>
@@ -22272,7 +22272,7 @@
         <v>1546</v>
       </c>
       <c r="I410" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J410" t="s">
         <v>2081</v>
@@ -22800,7 +22800,7 @@
         <v>1546</v>
       </c>
       <c r="I425" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J425" t="s">
         <v>2096</v>
@@ -23681,7 +23681,7 @@
         <v>1546</v>
       </c>
       <c r="I450" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J450" t="s">
         <v>2121</v>
@@ -24069,7 +24069,7 @@
         <v>1546</v>
       </c>
       <c r="I461" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J461" t="s">
         <v>2132</v>
@@ -24139,7 +24139,7 @@
         <v>1546</v>
       </c>
       <c r="I463" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J463" t="s">
         <v>2134</v>
@@ -24209,7 +24209,7 @@
         <v>1546</v>
       </c>
       <c r="I465" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J465" t="s">
         <v>2136</v>
@@ -24559,7 +24559,7 @@
         <v>1546</v>
       </c>
       <c r="I475" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J475" t="s">
         <v>2146</v>
@@ -25014,7 +25014,7 @@
         <v>1546</v>
       </c>
       <c r="I488" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J488" t="s">
         <v>2159</v>
@@ -25437,7 +25437,7 @@
         <v>1546</v>
       </c>
       <c r="I500" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J500" t="s">
         <v>2171</v>
@@ -25507,7 +25507,7 @@
         <v>1546</v>
       </c>
       <c r="I502" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J502" t="s">
         <v>2173</v>
@@ -26032,7 +26032,7 @@
         <v>1546</v>
       </c>
       <c r="I517" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J517" t="s">
         <v>2188</v>
@@ -26423,7 +26423,7 @@
         <v>1559</v>
       </c>
       <c r="I528" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J528" t="s">
         <v>2199</v>
@@ -26458,7 +26458,7 @@
         <v>1546</v>
       </c>
       <c r="I529" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J529" t="s">
         <v>2200</v>
@@ -26598,7 +26598,7 @@
         <v>1546</v>
       </c>
       <c r="I533" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J533" t="s">
         <v>2204</v>
@@ -26773,7 +26773,7 @@
         <v>1546</v>
       </c>
       <c r="I538" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J538" t="s">
         <v>2209</v>
@@ -26986,7 +26986,7 @@
         <v>1537</v>
       </c>
       <c r="I544" t="s">
-        <v>1574</v>
+        <v>1628</v>
       </c>
       <c r="J544" t="s">
         <v>2215</v>
@@ -27196,7 +27196,7 @@
         <v>1546</v>
       </c>
       <c r="I550" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J550" t="s">
         <v>2221</v>
@@ -27301,7 +27301,7 @@
         <v>1546</v>
       </c>
       <c r="I553" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J553" t="s">
         <v>2224</v>
@@ -27479,7 +27479,7 @@
         <v>1546</v>
       </c>
       <c r="I558" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J558" t="s">
         <v>2229</v>
@@ -27584,7 +27584,7 @@
         <v>1546</v>
       </c>
       <c r="I561" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J561" t="s">
         <v>2232</v>
@@ -27867,7 +27867,7 @@
         <v>1546</v>
       </c>
       <c r="I569" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J569" t="s">
         <v>2240</v>
@@ -27937,7 +27937,7 @@
         <v>1546</v>
       </c>
       <c r="I571" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J571" t="s">
         <v>2242</v>
@@ -28115,7 +28115,7 @@
         <v>1546</v>
       </c>
       <c r="I576" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J576" t="s">
         <v>2247</v>
@@ -28185,7 +28185,7 @@
         <v>1546</v>
       </c>
       <c r="I578" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J578" t="s">
         <v>2249</v>
@@ -28535,7 +28535,7 @@
         <v>1546</v>
       </c>
       <c r="I588" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J588" t="s">
         <v>2258</v>
@@ -28827,7 +28827,7 @@
         <v>1548</v>
       </c>
       <c r="I596" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J596" t="s">
         <v>2266</v>
@@ -29107,7 +29107,7 @@
         <v>1546</v>
       </c>
       <c r="I604" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J604" t="s">
         <v>2273</v>
@@ -29247,7 +29247,7 @@
         <v>1546</v>
       </c>
       <c r="I608" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J608" t="s">
         <v>2277</v>
@@ -29851,7 +29851,7 @@
         <v>1546</v>
       </c>
       <c r="I625" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
       <c r="J625" t="s">
         <v>2292</v>
@@ -30096,7 +30096,7 @@
         <v>1546</v>
       </c>
       <c r="I632" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
       <c r="J632" t="s">
         <v>2299</v>
@@ -30236,7 +30236,7 @@
         <v>1546</v>
       </c>
       <c r="I636" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J636" t="s">
         <v>2303</v>
@@ -30271,7 +30271,7 @@
         <v>1546</v>
       </c>
       <c r="I637" t="s">
-        <v>1574</v>
+        <v>1671</v>
       </c>
       <c r="J637" t="s">
         <v>2304</v>
@@ -30306,7 +30306,7 @@
         <v>1546</v>
       </c>
       <c r="I638" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J638" t="s">
         <v>2305</v>
@@ -30376,7 +30376,7 @@
         <v>1546</v>
       </c>
       <c r="I640" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
       <c r="J640" t="s">
         <v>2307</v>
@@ -30414,7 +30414,7 @@
         <v>1566</v>
       </c>
       <c r="I641" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J641" t="s">
         <v>2308</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-23 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -30263,7 +30263,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B636" t="s">
         <v>673</v>
@@ -30287,7 +30287,7 @@
         <v>1577</v>
       </c>
       <c r="I636" t="s">
-        <v>1691</v>
+        <v>1685</v>
       </c>
       <c r="J636" t="s">
         <v>2314</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-23 14:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5056,33 +5056,33 @@
     <t>RAQUEL SILVA FERNANDES LYRA</t>
   </si>
   <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,ERIKA CANTANHEDE WUILLAUME</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>GABRIEL GERON MOREIRA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
+  </si>
+  <si>
     <t>FLAVIA REIS RIBEIRO BASTOS, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,ERIKA CANTANHEDE WUILLAUME</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS</t>
-  </si>
-  <si>
     <t>JULIANA MARTINS BAHIENSE,SIMONE MANNHEIMER DE ALVARENGA</t>
   </si>
   <si>
@@ -7522,7 +7522,7 @@
     <t>VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -7570,22 +7570,25 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
+    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
@@ -7594,10 +7597,7 @@
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ECONOMIA,SAÚDE MENTAL,URBANISMO,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,SAÚDE,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL</t>
+    <t>URBANISMO,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL,PSICOLOGIA,MOBILIDADE E TRANSPORTE,SAÚDE,ECONOMIA,ORÇAMENTO,ASSISTÊNCIA SOCIAL</t>
   </si>
 </sst>
 </file>
@@ -24344,7 +24344,7 @@
     </row>
     <row r="468" spans="1:12">
       <c r="A468" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B468" t="s">
         <v>507</v>
@@ -25672,7 +25672,7 @@
         <v>2366</v>
       </c>
       <c r="L505" t="s">
-        <v>2480</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="506" spans="1:12">
@@ -26483,7 +26483,7 @@
         <v>2374</v>
       </c>
       <c r="L528" t="s">
-        <v>2520</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="529" spans="1:12">
@@ -27361,7 +27361,7 @@
         <v>2382</v>
       </c>
       <c r="L553" t="s">
-        <v>2521</v>
+        <v>2522</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -28458,7 +28458,7 @@
         <v>2337</v>
       </c>
       <c r="L584" t="s">
-        <v>2522</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="585" spans="1:12">
@@ -28566,7 +28566,7 @@
         <v>2374</v>
       </c>
       <c r="L587" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="588" spans="1:12">
@@ -28662,7 +28662,7 @@
         <v>1556</v>
       </c>
       <c r="I590" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J590" t="s">
         <v>2273</v>
@@ -28781,7 +28781,7 @@
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B594" t="s">
         <v>632</v>
@@ -28811,7 +28811,7 @@
         <v>2365</v>
       </c>
       <c r="L594" t="s">
-        <v>2514</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28921,7 +28921,7 @@
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B598" t="s">
         <v>636</v>
@@ -28951,7 +28951,7 @@
         <v>2447</v>
       </c>
       <c r="L598" t="s">
-        <v>2514</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="599" spans="1:12">
@@ -29026,7 +29026,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -29056,7 +29056,7 @@
         <v>2448</v>
       </c>
       <c r="L601" t="s">
-        <v>2514</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="602" spans="1:12">
@@ -29482,7 +29482,7 @@
         <v>2345</v>
       </c>
       <c r="L613" t="s">
-        <v>2524</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="614" spans="1:12">
@@ -29517,7 +29517,7 @@
         <v>2423</v>
       </c>
       <c r="L614" t="s">
-        <v>2525</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="615" spans="1:12">
@@ -29560,7 +29560,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B616" t="s">
         <v>653</v>
@@ -29590,7 +29590,7 @@
         <v>2365</v>
       </c>
       <c r="L616" t="s">
-        <v>2514</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="617" spans="1:12">
@@ -29630,7 +29630,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B618" t="s">
         <v>655</v>
@@ -29660,7 +29660,7 @@
         <v>2365</v>
       </c>
       <c r="L618" t="s">
-        <v>2514</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29721,7 +29721,7 @@
         <v>1556</v>
       </c>
       <c r="I620" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J620" t="s">
         <v>2300</v>
@@ -30252,7 +30252,7 @@
         <v>1576</v>
       </c>
       <c r="I635" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J635" t="s">
         <v>2315</v>
@@ -30430,7 +30430,7 @@
         <v>1577</v>
       </c>
       <c r="I640" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J640" t="s">
         <v>2320</v>
@@ -30576,7 +30576,7 @@
         <v>1568</v>
       </c>
       <c r="I644" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J644" t="s">
         <v>2324</v>
@@ -30652,7 +30652,7 @@
         <v>1573</v>
       </c>
       <c r="I646" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
       <c r="J646" t="s">
         <v>2325</v>
@@ -30693,7 +30693,7 @@
         <v>2453</v>
       </c>
       <c r="L647" t="s">
-        <v>2526</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="648" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-27 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -24365,7 +24365,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B471" t="s">
         <v>509</v>
@@ -24386,7 +24386,7 @@
         <v>1542</v>
       </c>
       <c r="I471" t="s">
-        <v>1627</v>
+        <v>1570</v>
       </c>
       <c r="J471" t="s">
         <v>2138</v>
@@ -27285,7 +27285,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B554" t="s">
         <v>592</v>
@@ -27309,7 +27309,7 @@
         <v>1555</v>
       </c>
       <c r="I554" t="s">
-        <v>1584</v>
+        <v>1570</v>
       </c>
       <c r="J554" t="s">
         <v>2221</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-27 12:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4858,6 +4858,9 @@
     <t>ERIKA SILVEIRA PAES BARRETO ALVES,SUZAN NIGRI</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
   </si>
   <si>
@@ -5018,9 +5021,6 @@
   </si>
   <si>
     <t>GABRIEL GERON MOREIRA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>ROSEMARY RODRIGUES CRUZ</t>
@@ -13249,7 +13249,7 @@
         <v>1538</v>
       </c>
       <c r="I154" t="s">
-        <v>1565</v>
+        <v>1614</v>
       </c>
       <c r="J154" t="s">
         <v>1820</v>
@@ -13284,7 +13284,7 @@
         <v>1538</v>
       </c>
       <c r="I155" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="J155" t="s">
         <v>1821</v>
@@ -13319,7 +13319,7 @@
         <v>1538</v>
       </c>
       <c r="I156" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J156" t="s">
         <v>1822</v>
@@ -13599,7 +13599,7 @@
         <v>1538</v>
       </c>
       <c r="I164" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="J164" t="s">
         <v>1830</v>
@@ -13634,7 +13634,7 @@
         <v>1538</v>
       </c>
       <c r="I165" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J165" t="s">
         <v>1831</v>
@@ -13844,7 +13844,7 @@
         <v>1538</v>
       </c>
       <c r="I171" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J171" t="s">
         <v>1837</v>
@@ -13914,7 +13914,7 @@
         <v>1538</v>
       </c>
       <c r="I173" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="J173" t="s">
         <v>1839</v>
@@ -14264,7 +14264,7 @@
         <v>1538</v>
       </c>
       <c r="I183" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J183" t="s">
         <v>1847</v>
@@ -14509,7 +14509,7 @@
         <v>1538</v>
       </c>
       <c r="I190" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J190" t="s">
         <v>1854</v>
@@ -14579,7 +14579,7 @@
         <v>1538</v>
       </c>
       <c r="I192" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J192" t="s">
         <v>1856</v>
@@ -14614,7 +14614,7 @@
         <v>1538</v>
       </c>
       <c r="I193" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J193" t="s">
         <v>1857</v>
@@ -14789,7 +14789,7 @@
         <v>1538</v>
       </c>
       <c r="I198" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J198" t="s">
         <v>1862</v>
@@ -14894,7 +14894,7 @@
         <v>1538</v>
       </c>
       <c r="I201" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J201" t="s">
         <v>1865</v>
@@ -14999,7 +14999,7 @@
         <v>1538</v>
       </c>
       <c r="I204" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J204" t="s">
         <v>1868</v>
@@ -15069,7 +15069,7 @@
         <v>1538</v>
       </c>
       <c r="I206" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J206" t="s">
         <v>1870</v>
@@ -15209,7 +15209,7 @@
         <v>1538</v>
       </c>
       <c r="I210" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J210" t="s">
         <v>1874</v>
@@ -15244,7 +15244,7 @@
         <v>1538</v>
       </c>
       <c r="I211" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J211" t="s">
         <v>1875</v>
@@ -15419,7 +15419,7 @@
         <v>1538</v>
       </c>
       <c r="I216" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J216" t="s">
         <v>1880</v>
@@ -15457,7 +15457,7 @@
         <v>1543</v>
       </c>
       <c r="I217" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J217" t="s">
         <v>1881</v>
@@ -15492,7 +15492,7 @@
         <v>1538</v>
       </c>
       <c r="I218" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J218" t="s">
         <v>1882</v>
@@ -15562,7 +15562,7 @@
         <v>1538</v>
       </c>
       <c r="I220" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J220" t="s">
         <v>1884</v>
@@ -15667,7 +15667,7 @@
         <v>1538</v>
       </c>
       <c r="I223" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J223" t="s">
         <v>1887</v>
@@ -15737,7 +15737,7 @@
         <v>1538</v>
       </c>
       <c r="I225" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="J225" t="s">
         <v>1889</v>
@@ -15807,7 +15807,7 @@
         <v>1538</v>
       </c>
       <c r="I227" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J227" t="s">
         <v>1891</v>
@@ -15842,7 +15842,7 @@
         <v>1538</v>
       </c>
       <c r="I228" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="J228" t="s">
         <v>1892</v>
@@ -15877,7 +15877,7 @@
         <v>1538</v>
       </c>
       <c r="I229" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="J229" t="s">
         <v>1893</v>
@@ -15947,7 +15947,7 @@
         <v>1538</v>
       </c>
       <c r="I231" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J231" t="s">
         <v>1895</v>
@@ -16052,7 +16052,7 @@
         <v>1538</v>
       </c>
       <c r="I234" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J234" t="s">
         <v>1898</v>
@@ -16087,7 +16087,7 @@
         <v>1538</v>
       </c>
       <c r="I235" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="J235" t="s">
         <v>1899</v>
@@ -16227,7 +16227,7 @@
         <v>1538</v>
       </c>
       <c r="I239" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J239" t="s">
         <v>1903</v>
@@ -16612,7 +16612,7 @@
         <v>1538</v>
       </c>
       <c r="I250" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J250" t="s">
         <v>1914</v>
@@ -16647,7 +16647,7 @@
         <v>1538</v>
       </c>
       <c r="I251" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J251" t="s">
         <v>1915</v>
@@ -17277,7 +17277,7 @@
         <v>1538</v>
       </c>
       <c r="I269" t="s">
-        <v>1565</v>
+        <v>1633</v>
       </c>
       <c r="J269" t="s">
         <v>1931</v>
@@ -17662,7 +17662,7 @@
         <v>1538</v>
       </c>
       <c r="I280" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J280" t="s">
         <v>1942</v>
@@ -17732,7 +17732,7 @@
         <v>1538</v>
       </c>
       <c r="I282" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J282" t="s">
         <v>1944</v>
@@ -17802,7 +17802,7 @@
         <v>1538</v>
       </c>
       <c r="I284" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J284" t="s">
         <v>1946</v>
@@ -17872,7 +17872,7 @@
         <v>1538</v>
       </c>
       <c r="I286" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J286" t="s">
         <v>1948</v>
@@ -18082,7 +18082,7 @@
         <v>1538</v>
       </c>
       <c r="I292" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J292" t="s">
         <v>1954</v>
@@ -18152,7 +18152,7 @@
         <v>1538</v>
       </c>
       <c r="I294" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J294" t="s">
         <v>1956</v>
@@ -18222,7 +18222,7 @@
         <v>1538</v>
       </c>
       <c r="I296" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J296" t="s">
         <v>1958</v>
@@ -18607,7 +18607,7 @@
         <v>1538</v>
       </c>
       <c r="I307" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J307" t="s">
         <v>1969</v>
@@ -18747,7 +18747,7 @@
         <v>1538</v>
       </c>
       <c r="I311" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J311" t="s">
         <v>1973</v>
@@ -18852,7 +18852,7 @@
         <v>1538</v>
       </c>
       <c r="I314" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J314" t="s">
         <v>1976</v>
@@ -18992,7 +18992,7 @@
         <v>1538</v>
       </c>
       <c r="I318" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J318" t="s">
         <v>1980</v>
@@ -19027,7 +19027,7 @@
         <v>1538</v>
       </c>
       <c r="I319" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J319" t="s">
         <v>1981</v>
@@ -19237,7 +19237,7 @@
         <v>1538</v>
       </c>
       <c r="I325" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J325" t="s">
         <v>1987</v>
@@ -19377,7 +19377,7 @@
         <v>1538</v>
       </c>
       <c r="I329" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="J329" t="s">
         <v>1991</v>
@@ -19622,7 +19622,7 @@
         <v>1538</v>
       </c>
       <c r="I336" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J336" t="s">
         <v>1998</v>
@@ -19692,7 +19692,7 @@
         <v>1538</v>
       </c>
       <c r="I338" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J338" t="s">
         <v>2000</v>
@@ -19727,7 +19727,7 @@
         <v>1538</v>
       </c>
       <c r="I339" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J339" t="s">
         <v>2001</v>
@@ -19762,7 +19762,7 @@
         <v>1538</v>
       </c>
       <c r="I340" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J340" t="s">
         <v>2002</v>
@@ -19832,7 +19832,7 @@
         <v>1538</v>
       </c>
       <c r="I342" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J342" t="s">
         <v>2004</v>
@@ -20007,7 +20007,7 @@
         <v>1538</v>
       </c>
       <c r="I347" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J347" t="s">
         <v>2009</v>
@@ -20182,7 +20182,7 @@
         <v>1538</v>
       </c>
       <c r="I352" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J352" t="s">
         <v>2014</v>
@@ -20252,7 +20252,7 @@
         <v>1538</v>
       </c>
       <c r="I354" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="J354" t="s">
         <v>2016</v>
@@ -20287,7 +20287,7 @@
         <v>1538</v>
       </c>
       <c r="I355" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J355" t="s">
         <v>2017</v>
@@ -20430,7 +20430,7 @@
         <v>1544</v>
       </c>
       <c r="I359" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J359" t="s">
         <v>2021</v>
@@ -20535,7 +20535,7 @@
         <v>1538</v>
       </c>
       <c r="I362" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J362" t="s">
         <v>2024</v>
@@ -20885,7 +20885,7 @@
         <v>1538</v>
       </c>
       <c r="I372" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J372" t="s">
         <v>2034</v>
@@ -20920,7 +20920,7 @@
         <v>1538</v>
       </c>
       <c r="I373" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J373" t="s">
         <v>2035</v>
@@ -20955,7 +20955,7 @@
         <v>1538</v>
       </c>
       <c r="I374" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J374" t="s">
         <v>2036</v>
@@ -21095,7 +21095,7 @@
         <v>1538</v>
       </c>
       <c r="I378" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J378" t="s">
         <v>2040</v>
@@ -21165,7 +21165,7 @@
         <v>1538</v>
       </c>
       <c r="I380" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J380" t="s">
         <v>2042</v>
@@ -21343,7 +21343,7 @@
         <v>1545</v>
       </c>
       <c r="I385" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J385" t="s">
         <v>2047</v>
@@ -21413,7 +21413,7 @@
         <v>1538</v>
       </c>
       <c r="I387" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J387" t="s">
         <v>2049</v>
@@ -21448,7 +21448,7 @@
         <v>1538</v>
       </c>
       <c r="I388" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J388" t="s">
         <v>2050</v>
@@ -21483,7 +21483,7 @@
         <v>1538</v>
       </c>
       <c r="I389" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J389" t="s">
         <v>2051</v>
@@ -21553,7 +21553,7 @@
         <v>1538</v>
       </c>
       <c r="I391" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="J391" t="s">
         <v>2053</v>
@@ -21728,7 +21728,7 @@
         <v>1538</v>
       </c>
       <c r="I396" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J396" t="s">
         <v>2058</v>
@@ -21763,7 +21763,7 @@
         <v>1538</v>
       </c>
       <c r="I397" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J397" t="s">
         <v>2059</v>
@@ -21798,7 +21798,7 @@
         <v>1538</v>
       </c>
       <c r="I398" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J398" t="s">
         <v>2060</v>
@@ -22008,7 +22008,7 @@
         <v>1538</v>
       </c>
       <c r="I404" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J404" t="s">
         <v>2066</v>
@@ -22043,7 +22043,7 @@
         <v>1538</v>
       </c>
       <c r="I405" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="J405" t="s">
         <v>2067</v>
@@ -22221,7 +22221,7 @@
         <v>1538</v>
       </c>
       <c r="I410" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J410" t="s">
         <v>2072</v>
@@ -22259,7 +22259,7 @@
         <v>1546</v>
       </c>
       <c r="I411" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J411" t="s">
         <v>2073</v>
@@ -22504,7 +22504,7 @@
         <v>1538</v>
       </c>
       <c r="I418" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J418" t="s">
         <v>2080</v>
@@ -22749,7 +22749,7 @@
         <v>1538</v>
       </c>
       <c r="I425" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J425" t="s">
         <v>2087</v>
@@ -22784,7 +22784,7 @@
         <v>1538</v>
       </c>
       <c r="I426" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J426" t="s">
         <v>2088</v>
@@ -23064,7 +23064,7 @@
         <v>1538</v>
       </c>
       <c r="I434" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J434" t="s">
         <v>2096</v>
@@ -23207,7 +23207,7 @@
         <v>1547</v>
       </c>
       <c r="I438" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J438" t="s">
         <v>2100</v>
@@ -23277,7 +23277,7 @@
         <v>1538</v>
       </c>
       <c r="I440" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J440" t="s">
         <v>2102</v>
@@ -23312,7 +23312,7 @@
         <v>1538</v>
       </c>
       <c r="I441" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J441" t="s">
         <v>2103</v>
@@ -23452,7 +23452,7 @@
         <v>1538</v>
       </c>
       <c r="I445" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J445" t="s">
         <v>2107</v>
@@ -23522,7 +23522,7 @@
         <v>1538</v>
       </c>
       <c r="I447" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J447" t="s">
         <v>2109</v>
@@ -23557,7 +23557,7 @@
         <v>1538</v>
       </c>
       <c r="I448" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J448" t="s">
         <v>2110</v>
@@ -23592,7 +23592,7 @@
         <v>1538</v>
       </c>
       <c r="I449" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J449" t="s">
         <v>2111</v>
@@ -23662,7 +23662,7 @@
         <v>1538</v>
       </c>
       <c r="I451" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J451" t="s">
         <v>2113</v>
@@ -23732,7 +23732,7 @@
         <v>1538</v>
       </c>
       <c r="I453" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J453" t="s">
         <v>2115</v>
@@ -23802,7 +23802,7 @@
         <v>1538</v>
       </c>
       <c r="I455" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J455" t="s">
         <v>2117</v>
@@ -23907,7 +23907,7 @@
         <v>1538</v>
       </c>
       <c r="I458" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J458" t="s">
         <v>2120</v>
@@ -23942,7 +23942,7 @@
         <v>1538</v>
       </c>
       <c r="I459" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J459" t="s">
         <v>2121</v>
@@ -24012,7 +24012,7 @@
         <v>1538</v>
       </c>
       <c r="I461" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J461" t="s">
         <v>2123</v>
@@ -24047,7 +24047,7 @@
         <v>1538</v>
       </c>
       <c r="I462" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J462" t="s">
         <v>2124</v>
@@ -24117,7 +24117,7 @@
         <v>1538</v>
       </c>
       <c r="I464" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J464" t="s">
         <v>2126</v>
@@ -24432,7 +24432,7 @@
         <v>1538</v>
       </c>
       <c r="I473" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J473" t="s">
         <v>2135</v>
@@ -24467,7 +24467,7 @@
         <v>1538</v>
       </c>
       <c r="I474" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J474" t="s">
         <v>2136</v>
@@ -24502,7 +24502,7 @@
         <v>1538</v>
       </c>
       <c r="I475" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J475" t="s">
         <v>2137</v>
@@ -24607,7 +24607,7 @@
         <v>1538</v>
       </c>
       <c r="I478" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J478" t="s">
         <v>2140</v>
@@ -24712,7 +24712,7 @@
         <v>1538</v>
       </c>
       <c r="I481" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J481" t="s">
         <v>2143</v>
@@ -24747,7 +24747,7 @@
         <v>1538</v>
       </c>
       <c r="I482" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J482" t="s">
         <v>2144</v>
@@ -24782,7 +24782,7 @@
         <v>1538</v>
       </c>
       <c r="I483" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J483" t="s">
         <v>2145</v>
@@ -24817,7 +24817,7 @@
         <v>1538</v>
       </c>
       <c r="I484" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J484" t="s">
         <v>2146</v>
@@ -25132,7 +25132,7 @@
         <v>1538</v>
       </c>
       <c r="I493" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J493" t="s">
         <v>2155</v>
@@ -25342,7 +25342,7 @@
         <v>1538</v>
       </c>
       <c r="I499" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J499" t="s">
         <v>2161</v>
@@ -25377,7 +25377,7 @@
         <v>1538</v>
       </c>
       <c r="I500" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J500" t="s">
         <v>2162</v>
@@ -25520,7 +25520,7 @@
         <v>1538</v>
       </c>
       <c r="I504" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J504" t="s">
         <v>2166</v>
@@ -25590,7 +25590,7 @@
         <v>1538</v>
       </c>
       <c r="I506" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J506" t="s">
         <v>2168</v>
@@ -25625,7 +25625,7 @@
         <v>1538</v>
       </c>
       <c r="I507" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J507" t="s">
         <v>2169</v>
@@ -25660,7 +25660,7 @@
         <v>1538</v>
       </c>
       <c r="I508" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J508" t="s">
         <v>2170</v>
@@ -25695,7 +25695,7 @@
         <v>1538</v>
       </c>
       <c r="I509" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J509" t="s">
         <v>2171</v>
@@ -25733,7 +25733,7 @@
         <v>1548</v>
       </c>
       <c r="I510" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J510" t="s">
         <v>2172</v>
@@ -25768,7 +25768,7 @@
         <v>1538</v>
       </c>
       <c r="I511" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J511" t="s">
         <v>2173</v>
@@ -25873,7 +25873,7 @@
         <v>1538</v>
       </c>
       <c r="I514" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J514" t="s">
         <v>2176</v>
@@ -25908,7 +25908,7 @@
         <v>1538</v>
       </c>
       <c r="I515" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J515" t="s">
         <v>2177</v>
@@ -26013,7 +26013,7 @@
         <v>1538</v>
       </c>
       <c r="I518" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J518" t="s">
         <v>2180</v>
@@ -26048,7 +26048,7 @@
         <v>1538</v>
       </c>
       <c r="I519" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J519" t="s">
         <v>2181</v>
@@ -26083,7 +26083,7 @@
         <v>1538</v>
       </c>
       <c r="I520" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J520" t="s">
         <v>2182</v>
@@ -26188,7 +26188,7 @@
         <v>1538</v>
       </c>
       <c r="I523" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J523" t="s">
         <v>2185</v>
@@ -26258,7 +26258,7 @@
         <v>1538</v>
       </c>
       <c r="I525" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J525" t="s">
         <v>2187</v>
@@ -26363,7 +26363,7 @@
         <v>1538</v>
       </c>
       <c r="I528" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J528" t="s">
         <v>2190</v>
@@ -26433,7 +26433,7 @@
         <v>1538</v>
       </c>
       <c r="I530" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J530" t="s">
         <v>2192</v>
@@ -26538,7 +26538,7 @@
         <v>1538</v>
       </c>
       <c r="I533" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J533" t="s">
         <v>2195</v>
@@ -26643,7 +26643,7 @@
         <v>1538</v>
       </c>
       <c r="I536" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J536" t="s">
         <v>2198</v>
@@ -26716,7 +26716,7 @@
         <v>1538</v>
       </c>
       <c r="I538" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J538" t="s">
         <v>2200</v>
@@ -26751,7 +26751,7 @@
         <v>1538</v>
       </c>
       <c r="I539" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J539" t="s">
         <v>2201</v>
@@ -26821,7 +26821,7 @@
         <v>1538</v>
       </c>
       <c r="I541" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J541" t="s">
         <v>2203</v>
@@ -26929,7 +26929,7 @@
         <v>1538</v>
       </c>
       <c r="I544" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J544" t="s">
         <v>2206</v>
@@ -26964,7 +26964,7 @@
         <v>1538</v>
       </c>
       <c r="I545" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J545" t="s">
         <v>2207</v>
@@ -27034,7 +27034,7 @@
         <v>1538</v>
       </c>
       <c r="I547" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J547" t="s">
         <v>2209</v>
@@ -27069,7 +27069,7 @@
         <v>1538</v>
       </c>
       <c r="I548" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J548" t="s">
         <v>2210</v>
@@ -27104,7 +27104,7 @@
         <v>1538</v>
       </c>
       <c r="I549" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J549" t="s">
         <v>2211</v>
@@ -27139,7 +27139,7 @@
         <v>1538</v>
       </c>
       <c r="I550" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J550" t="s">
         <v>2212</v>
@@ -27174,7 +27174,7 @@
         <v>1538</v>
       </c>
       <c r="I551" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J551" t="s">
         <v>2213</v>
@@ -27244,7 +27244,7 @@
         <v>1538</v>
       </c>
       <c r="I553" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J553" t="s">
         <v>2215</v>
@@ -27314,7 +27314,7 @@
         <v>1538</v>
       </c>
       <c r="I555" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J555" t="s">
         <v>2217</v>
@@ -27349,7 +27349,7 @@
         <v>1538</v>
       </c>
       <c r="I556" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J556" t="s">
         <v>2218</v>
@@ -27384,7 +27384,7 @@
         <v>1538</v>
       </c>
       <c r="I557" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J557" t="s">
         <v>2219</v>
@@ -27419,7 +27419,7 @@
         <v>1538</v>
       </c>
       <c r="I558" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J558" t="s">
         <v>2219</v>
@@ -27489,7 +27489,7 @@
         <v>1538</v>
       </c>
       <c r="I560" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J560" t="s">
         <v>2221</v>
@@ -27524,7 +27524,7 @@
         <v>1538</v>
       </c>
       <c r="I561" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J561" t="s">
         <v>2222</v>
@@ -27559,7 +27559,7 @@
         <v>1538</v>
       </c>
       <c r="I562" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J562" t="s">
         <v>2223</v>
@@ -27594,7 +27594,7 @@
         <v>1538</v>
       </c>
       <c r="I563" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J563" t="s">
         <v>2224</v>
@@ -27629,7 +27629,7 @@
         <v>1538</v>
       </c>
       <c r="I564" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J564" t="s">
         <v>2225</v>
@@ -27734,7 +27734,7 @@
         <v>1538</v>
       </c>
       <c r="I567" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J567" t="s">
         <v>2228</v>
@@ -27769,7 +27769,7 @@
         <v>1538</v>
       </c>
       <c r="I568" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J568" t="s">
         <v>2229</v>
@@ -27807,7 +27807,7 @@
         <v>1551</v>
       </c>
       <c r="I569" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J569" t="s">
         <v>2230</v>
@@ -27845,7 +27845,7 @@
         <v>1551</v>
       </c>
       <c r="I570" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J570" t="s">
         <v>2231</v>
@@ -27883,7 +27883,7 @@
         <v>1551</v>
       </c>
       <c r="I571" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J571" t="s">
         <v>2232</v>
@@ -27918,7 +27918,7 @@
         <v>1538</v>
       </c>
       <c r="I572" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J572" t="s">
         <v>2233</v>
@@ -27988,7 +27988,7 @@
         <v>1540</v>
       </c>
       <c r="I574" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J574" t="s">
         <v>2235</v>
@@ -28023,7 +28023,7 @@
         <v>1538</v>
       </c>
       <c r="I575" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J575" t="s">
         <v>2236</v>
@@ -28093,7 +28093,7 @@
         <v>1538</v>
       </c>
       <c r="I577" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J577" t="s">
         <v>2238</v>
@@ -28163,7 +28163,7 @@
         <v>1538</v>
       </c>
       <c r="I579" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J579" t="s">
         <v>2240</v>
@@ -28233,7 +28233,7 @@
         <v>1538</v>
       </c>
       <c r="I581" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J581" t="s">
         <v>2242</v>
@@ -28268,7 +28268,7 @@
         <v>1538</v>
       </c>
       <c r="I582" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J582" t="s">
         <v>2243</v>
@@ -28303,7 +28303,7 @@
         <v>1538</v>
       </c>
       <c r="I583" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J583" t="s">
         <v>2244</v>
@@ -28338,7 +28338,7 @@
         <v>1538</v>
       </c>
       <c r="I584" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J584" t="s">
         <v>2245</v>
@@ -28373,7 +28373,7 @@
         <v>1538</v>
       </c>
       <c r="I585" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J585" t="s">
         <v>2246</v>
@@ -28408,7 +28408,7 @@
         <v>1538</v>
       </c>
       <c r="I586" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J586" t="s">
         <v>2247</v>
@@ -28583,7 +28583,7 @@
         <v>1538</v>
       </c>
       <c r="I591" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J591" t="s">
         <v>2251</v>
@@ -28726,7 +28726,7 @@
         <v>1538</v>
       </c>
       <c r="I595" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J595" t="s">
         <v>2254</v>
@@ -28761,7 +28761,7 @@
         <v>1538</v>
       </c>
       <c r="I596" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J596" t="s">
         <v>2255</v>
@@ -28796,7 +28796,7 @@
         <v>1538</v>
       </c>
       <c r="I597" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J597" t="s">
         <v>2256</v>
@@ -28834,7 +28834,7 @@
         <v>1552</v>
       </c>
       <c r="I598" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J598" t="s">
         <v>2257</v>
@@ -28869,7 +28869,7 @@
         <v>1538</v>
       </c>
       <c r="I599" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J599" t="s">
         <v>2258</v>
@@ -28904,7 +28904,7 @@
         <v>1538</v>
       </c>
       <c r="I600" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J600" t="s">
         <v>2259</v>
@@ -28974,7 +28974,7 @@
         <v>1538</v>
       </c>
       <c r="I602" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J602" t="s">
         <v>2261</v>
@@ -29044,7 +29044,7 @@
         <v>1538</v>
       </c>
       <c r="I604" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J604" t="s">
         <v>2263</v>
@@ -29079,7 +29079,7 @@
         <v>1538</v>
       </c>
       <c r="I605" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J605" t="s">
         <v>2264</v>
@@ -29149,7 +29149,7 @@
         <v>1538</v>
       </c>
       <c r="I607" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J607" t="s">
         <v>2266</v>
@@ -29219,7 +29219,7 @@
         <v>1538</v>
       </c>
       <c r="I609" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J609" t="s">
         <v>2268</v>
@@ -29324,7 +29324,7 @@
         <v>1538</v>
       </c>
       <c r="I612" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J612" t="s">
         <v>2271</v>
@@ -29359,7 +29359,7 @@
         <v>1538</v>
       </c>
       <c r="I613" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J613" t="s">
         <v>2272</v>
@@ -29394,7 +29394,7 @@
         <v>1538</v>
       </c>
       <c r="I614" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J614" t="s">
         <v>2273</v>
@@ -29464,7 +29464,7 @@
         <v>1538</v>
       </c>
       <c r="I616" t="s">
-        <v>1668</v>
+        <v>1614</v>
       </c>
       <c r="J616" t="s">
         <v>2275</v>
@@ -29502,7 +29502,7 @@
         <v>1553</v>
       </c>
       <c r="I617" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J617" t="s">
         <v>2276</v>
@@ -29610,7 +29610,7 @@
         <v>1538</v>
       </c>
       <c r="I620" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J620" t="s">
         <v>2279</v>
@@ -29645,7 +29645,7 @@
         <v>1538</v>
       </c>
       <c r="I621" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J621" t="s">
         <v>2280</v>
@@ -29680,7 +29680,7 @@
         <v>1538</v>
       </c>
       <c r="I622" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J622" t="s">
         <v>2281</v>
@@ -29715,7 +29715,7 @@
         <v>1538</v>
       </c>
       <c r="I623" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J623" t="s">
         <v>2282</v>
@@ -29788,7 +29788,7 @@
         <v>1538</v>
       </c>
       <c r="I625" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J625" t="s">
         <v>2284</v>
@@ -29861,7 +29861,7 @@
         <v>1538</v>
       </c>
       <c r="I627" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J627" t="s">
         <v>2286</v>
@@ -29899,7 +29899,7 @@
         <v>1552</v>
       </c>
       <c r="I628" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J628" t="s">
         <v>2287</v>
@@ -29972,7 +29972,7 @@
         <v>1538</v>
       </c>
       <c r="I630" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J630" t="s">
         <v>2289</v>
@@ -30077,7 +30077,7 @@
         <v>1538</v>
       </c>
       <c r="I633" t="s">
-        <v>1668</v>
+        <v>1614</v>
       </c>
       <c r="J633" t="s">
         <v>2292</v>
@@ -30112,7 +30112,7 @@
         <v>1538</v>
       </c>
       <c r="I634" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J634" t="s">
         <v>2293</v>
@@ -30182,7 +30182,7 @@
         <v>1538</v>
       </c>
       <c r="I636" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J636" t="s">
         <v>2295</v>
@@ -30214,7 +30214,7 @@
         <v>1538</v>
       </c>
       <c r="I637" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J637" t="s">
         <v>2296</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-30 12:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6497" uniqueCount="2533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6497" uniqueCount="2534">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -4885,6 +4885,9 @@
     <t>CARLOS FELIPE DA GRAÇA SILVA,RODRIGO VALENTE SERRA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>PATRICIA PASSARO DA SILVA TOLEDO</t>
   </si>
   <si>
@@ -4912,9 +4915,6 @@
     <t>PABLO GINIO VIMERCATI SIMAS</t>
   </si>
   <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
     <t>FERNANDA FERREIRA FONTES,MARCELO TEIXEIRA SANTANA</t>
   </si>
   <si>
@@ -7585,19 +7585,22 @@
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
+    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
+    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>SAÚDE,SAÚDE MENTAL</t>
@@ -7612,7 +7615,7 @@
     <t>MEDICINA LEGAL,SAÚDE</t>
   </si>
   <si>
-    <t>SAÚDE,ASSISTÊNCIA SOCIAL,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ECONOMIA,PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,SAÚDE MENTAL,URBANISMO</t>
+    <t>SAÚDE,ECONOMIA,ECONOMICIDADE CONTÁBIL,URBANISMO,PSICOLOGIA,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,SAÚDE MENTAL</t>
   </si>
 </sst>
 </file>
@@ -11680,7 +11683,7 @@
         <v>1560</v>
       </c>
       <c r="I106" t="s">
-        <v>1589</v>
+        <v>1623</v>
       </c>
       <c r="J106" t="s">
         <v>1797</v>
@@ -11715,7 +11718,7 @@
         <v>1560</v>
       </c>
       <c r="I107" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J107" t="s">
         <v>1798</v>
@@ -11785,7 +11788,7 @@
         <v>1560</v>
       </c>
       <c r="I109" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J109" t="s">
         <v>1800</v>
@@ -11855,7 +11858,7 @@
         <v>1560</v>
       </c>
       <c r="I111" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J111" t="s">
         <v>1802</v>
@@ -11890,7 +11893,7 @@
         <v>1560</v>
       </c>
       <c r="I112" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J112" t="s">
         <v>1803</v>
@@ -11925,7 +11928,7 @@
         <v>1560</v>
       </c>
       <c r="I113" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J113" t="s">
         <v>1804</v>
@@ -11960,7 +11963,7 @@
         <v>1560</v>
       </c>
       <c r="I114" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J114" t="s">
         <v>1805</v>
@@ -12135,7 +12138,7 @@
         <v>1560</v>
       </c>
       <c r="I119" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J119" t="s">
         <v>1810</v>
@@ -12170,7 +12173,7 @@
         <v>1560</v>
       </c>
       <c r="I120" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J120" t="s">
         <v>1811</v>
@@ -12205,7 +12208,7 @@
         <v>1560</v>
       </c>
       <c r="I121" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J121" t="s">
         <v>1812</v>
@@ -12240,7 +12243,7 @@
         <v>1560</v>
       </c>
       <c r="I122" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J122" t="s">
         <v>1813</v>
@@ -12380,7 +12383,7 @@
         <v>1560</v>
       </c>
       <c r="I126" t="s">
-        <v>1632</v>
+        <v>1623</v>
       </c>
       <c r="J126" t="s">
         <v>1817</v>
@@ -12555,7 +12558,7 @@
         <v>1560</v>
       </c>
       <c r="I131" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J131" t="s">
         <v>1822</v>
@@ -14550,7 +14553,7 @@
         <v>1560</v>
       </c>
       <c r="I188" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J188" t="s">
         <v>1877</v>
@@ -15145,7 +15148,7 @@
         <v>1560</v>
       </c>
       <c r="I205" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J205" t="s">
         <v>1894</v>
@@ -15533,7 +15536,7 @@
         <v>1560</v>
       </c>
       <c r="I216" t="s">
-        <v>1632</v>
+        <v>1623</v>
       </c>
       <c r="J216" t="s">
         <v>1905</v>
@@ -15652,7 +15655,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B220" t="s">
         <v>259</v>
@@ -15673,7 +15676,7 @@
         <v>1560</v>
       </c>
       <c r="I220" t="s">
-        <v>1583</v>
+        <v>1623</v>
       </c>
       <c r="J220" t="s">
         <v>1909</v>
@@ -15778,7 +15781,7 @@
         <v>1560</v>
       </c>
       <c r="I223" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J223" t="s">
         <v>1912</v>
@@ -17143,7 +17146,7 @@
         <v>1560</v>
       </c>
       <c r="I262" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J262" t="s">
         <v>1949</v>
@@ -17913,7 +17916,7 @@
         <v>1560</v>
       </c>
       <c r="I284" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J284" t="s">
         <v>1971</v>
@@ -19558,7 +19561,7 @@
         <v>1560</v>
       </c>
       <c r="I331" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J331" t="s">
         <v>2018</v>
@@ -19593,7 +19596,7 @@
         <v>1560</v>
       </c>
       <c r="I332" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J332" t="s">
         <v>2019</v>
@@ -20541,7 +20544,7 @@
         <v>1560</v>
       </c>
       <c r="I359" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J359" t="s">
         <v>2046</v>
@@ -20786,7 +20789,7 @@
         <v>1560</v>
       </c>
       <c r="I366" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J366" t="s">
         <v>2053</v>
@@ -22157,7 +22160,7 @@
         <v>1560</v>
       </c>
       <c r="I405" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J405" t="s">
         <v>2092</v>
@@ -23945,7 +23948,7 @@
         <v>1560</v>
       </c>
       <c r="I456" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J456" t="s">
         <v>2143</v>
@@ -24575,7 +24578,7 @@
         <v>1560</v>
       </c>
       <c r="I474" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J474" t="s">
         <v>2161</v>
@@ -24829,7 +24832,7 @@
         <v>2369</v>
       </c>
       <c r="L481" t="s">
-        <v>2484</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="482" spans="1:12">
@@ -25065,7 +25068,7 @@
         <v>1560</v>
       </c>
       <c r="I488" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J488" t="s">
         <v>2175</v>
@@ -25605,7 +25608,7 @@
         <v>2376</v>
       </c>
       <c r="L503" t="s">
-        <v>2524</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -25806,7 +25809,7 @@
         <v>1560</v>
       </c>
       <c r="I509" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J509" t="s">
         <v>2196</v>
@@ -25946,7 +25949,7 @@
         <v>1560</v>
       </c>
       <c r="I513" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J513" t="s">
         <v>2200</v>
@@ -26051,7 +26054,7 @@
         <v>1560</v>
       </c>
       <c r="I516" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J516" t="s">
         <v>2203</v>
@@ -26226,7 +26229,7 @@
         <v>1560</v>
       </c>
       <c r="I521" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J521" t="s">
         <v>2208</v>
@@ -26448,7 +26451,7 @@
         <v>2383</v>
       </c>
       <c r="L527" t="s">
-        <v>2525</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="528" spans="1:12">
@@ -26512,7 +26515,7 @@
         <v>1570</v>
       </c>
       <c r="I529" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J529" t="s">
         <v>2216</v>
@@ -26932,7 +26935,7 @@
         <v>1560</v>
       </c>
       <c r="I541" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J541" t="s">
         <v>2228</v>
@@ -27507,7 +27510,7 @@
         <v>2341</v>
       </c>
       <c r="L557" t="s">
-        <v>2526</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="558" spans="1:12">
@@ -27606,7 +27609,7 @@
         <v>1560</v>
       </c>
       <c r="I560" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J560" t="s">
         <v>2246</v>
@@ -27615,7 +27618,7 @@
         <v>2376</v>
       </c>
       <c r="L560" t="s">
-        <v>2527</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="561" spans="1:12">
@@ -28140,7 +28143,7 @@
         <v>2417</v>
       </c>
       <c r="L575" t="s">
-        <v>2528</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="576" spans="1:12">
@@ -28166,7 +28169,7 @@
         <v>1560</v>
       </c>
       <c r="I576" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J576" t="s">
         <v>2261</v>
@@ -28201,7 +28204,7 @@
         <v>1560</v>
       </c>
       <c r="I577" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J577" t="s">
         <v>2262</v>
@@ -28496,7 +28499,7 @@
         <v>2349</v>
       </c>
       <c r="L585" t="s">
-        <v>2529</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="586" spans="1:12">
@@ -28531,7 +28534,7 @@
         <v>2425</v>
       </c>
       <c r="L586" t="s">
-        <v>2530</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28907,7 +28910,7 @@
         <v>1560</v>
       </c>
       <c r="I597" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J597" t="s">
         <v>2281</v>
@@ -29091,7 +29094,7 @@
         <v>2414</v>
       </c>
       <c r="L602" t="s">
-        <v>2531</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29117,7 +29120,7 @@
         <v>1560</v>
       </c>
       <c r="I603" t="s">
-        <v>1632</v>
+        <v>1623</v>
       </c>
       <c r="J603" t="s">
         <v>2287</v>
@@ -29528,7 +29531,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B615" t="s">
         <v>653</v>
@@ -29552,7 +29555,7 @@
         <v>1552</v>
       </c>
       <c r="I615" t="s">
-        <v>1664</v>
+        <v>1589</v>
       </c>
       <c r="J615" t="s">
         <v>2299</v>
@@ -29622,7 +29625,7 @@
         <v>1560</v>
       </c>
       <c r="I617" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J617" t="s">
         <v>2301</v>
@@ -29692,7 +29695,7 @@
         <v>1560</v>
       </c>
       <c r="I619" t="s">
-        <v>1632</v>
+        <v>1623</v>
       </c>
       <c r="J619" t="s">
         <v>2303</v>
@@ -29981,7 +29984,7 @@
         <v>1560</v>
       </c>
       <c r="I627" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J627" t="s">
         <v>2311</v>
@@ -30243,7 +30246,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B635" t="s">
         <v>673</v>
@@ -30264,7 +30267,7 @@
         <v>1560</v>
       </c>
       <c r="I635" t="s">
-        <v>1589</v>
+        <v>1679</v>
       </c>
       <c r="J635" t="s">
         <v>2319</v>
@@ -30273,7 +30276,7 @@
         <v>2364</v>
       </c>
       <c r="L635" t="s">
-        <v>2519</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30299,7 +30302,7 @@
         <v>1560</v>
       </c>
       <c r="I636" t="s">
-        <v>1589</v>
+        <v>1623</v>
       </c>
       <c r="J636" t="s">
         <v>2320</v>
@@ -30369,7 +30372,7 @@
         <v>1560</v>
       </c>
       <c r="I638" t="s">
-        <v>1589</v>
+        <v>1623</v>
       </c>
       <c r="J638" t="s">
         <v>2322</v>
@@ -30404,7 +30407,7 @@
         <v>1560</v>
       </c>
       <c r="I639" t="s">
-        <v>1589</v>
+        <v>1692</v>
       </c>
       <c r="J639" t="s">
         <v>2323</v>
@@ -30661,7 +30664,7 @@
         <v>2457</v>
       </c>
       <c r="L646" t="s">
-        <v>2526</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="647" spans="1:12">
@@ -30693,7 +30696,7 @@
         <v>2457</v>
       </c>
       <c r="L647" t="s">
-        <v>2532</v>
+        <v>2533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-31 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6426" uniqueCount="2507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6426" uniqueCount="2508">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -103,7 +103,7 @@
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE ENGENHARIA, SECRETARIA GERAL DO GATE</t>
+    <t>ADMISSIBILIDADE DA SECRETARIA DO GATE, NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
@@ -4825,6 +4825,9 @@
     <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA,EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
@@ -5020,9 +5023,6 @@
     <t>FERNANDA FERREIRA FONTES</t>
   </si>
   <si>
-    <t>LEONARDO ARAÚJO DE SOUZA</t>
-  </si>
-  <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA</t>
   </si>
   <si>
@@ -7510,10 +7510,13 @@
     <t>ENGENHARIA CIVIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
@@ -7534,7 +7537,7 @@
     <t>MEDICINA LEGAL,SAÚDE</t>
   </si>
   <si>
-    <t>URBANISMO,SAÚDE,ECONOMIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL</t>
+    <t>URBANISMO,SAÚDE,ECONOMICIDADE CONTÁBIL,ECONOMIA,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE MENTAL,MOBILIDADE E TRANSPORTE,PSICOLOGIA,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -11077,7 +11080,7 @@
         <v>1546</v>
       </c>
       <c r="I91" t="s">
-        <v>1575</v>
+        <v>1603</v>
       </c>
       <c r="J91" t="s">
         <v>1767</v>
@@ -11112,7 +11115,7 @@
         <v>1546</v>
       </c>
       <c r="I92" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="J92" t="s">
         <v>1768</v>
@@ -11217,7 +11220,7 @@
         <v>1546</v>
       </c>
       <c r="I95" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J95" t="s">
         <v>1771</v>
@@ -11287,7 +11290,7 @@
         <v>1546</v>
       </c>
       <c r="I97" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J97" t="s">
         <v>1773</v>
@@ -11462,7 +11465,7 @@
         <v>1546</v>
       </c>
       <c r="I102" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="J102" t="s">
         <v>1778</v>
@@ -11532,7 +11535,7 @@
         <v>1546</v>
       </c>
       <c r="I104" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="J104" t="s">
         <v>1780</v>
@@ -11602,7 +11605,7 @@
         <v>1546</v>
       </c>
       <c r="I106" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="J106" t="s">
         <v>1782</v>
@@ -11672,7 +11675,7 @@
         <v>1546</v>
       </c>
       <c r="I108" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J108" t="s">
         <v>1784</v>
@@ -11707,7 +11710,7 @@
         <v>1546</v>
       </c>
       <c r="I109" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="J109" t="s">
         <v>1785</v>
@@ -11742,7 +11745,7 @@
         <v>1546</v>
       </c>
       <c r="I110" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="J110" t="s">
         <v>1786</v>
@@ -11777,7 +11780,7 @@
         <v>1546</v>
       </c>
       <c r="I111" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="J111" t="s">
         <v>1787</v>
@@ -11952,7 +11955,7 @@
         <v>1546</v>
       </c>
       <c r="I116" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J116" t="s">
         <v>1792</v>
@@ -11987,7 +11990,7 @@
         <v>1546</v>
       </c>
       <c r="I117" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="J117" t="s">
         <v>1793</v>
@@ -12022,7 +12025,7 @@
         <v>1546</v>
       </c>
       <c r="I118" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="J118" t="s">
         <v>1794</v>
@@ -12057,7 +12060,7 @@
         <v>1546</v>
       </c>
       <c r="I119" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J119" t="s">
         <v>1795</v>
@@ -12337,7 +12340,7 @@
         <v>1546</v>
       </c>
       <c r="I127" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J127" t="s">
         <v>1803</v>
@@ -12372,7 +12375,7 @@
         <v>1546</v>
       </c>
       <c r="I128" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="J128" t="s">
         <v>1804</v>
@@ -12547,7 +12550,7 @@
         <v>1546</v>
       </c>
       <c r="I133" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J133" t="s">
         <v>1809</v>
@@ -12687,7 +12690,7 @@
         <v>1546</v>
       </c>
       <c r="I137" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J137" t="s">
         <v>1813</v>
@@ -12722,7 +12725,7 @@
         <v>1546</v>
       </c>
       <c r="I138" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J138" t="s">
         <v>1814</v>
@@ -12932,7 +12935,7 @@
         <v>1546</v>
       </c>
       <c r="I144" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="J144" t="s">
         <v>1820</v>
@@ -12967,7 +12970,7 @@
         <v>1546</v>
       </c>
       <c r="I145" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J145" t="s">
         <v>1821</v>
@@ -13177,7 +13180,7 @@
         <v>1546</v>
       </c>
       <c r="I151" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J151" t="s">
         <v>1827</v>
@@ -13247,7 +13250,7 @@
         <v>1546</v>
       </c>
       <c r="I153" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J153" t="s">
         <v>1829</v>
@@ -13282,7 +13285,7 @@
         <v>1546</v>
       </c>
       <c r="I154" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J154" t="s">
         <v>1830</v>
@@ -13492,7 +13495,7 @@
         <v>1546</v>
       </c>
       <c r="I160" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J160" t="s">
         <v>1836</v>
@@ -13527,7 +13530,7 @@
         <v>1546</v>
       </c>
       <c r="I161" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J161" t="s">
         <v>1837</v>
@@ -13632,7 +13635,7 @@
         <v>1546</v>
       </c>
       <c r="I164" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J164" t="s">
         <v>1840</v>
@@ -13877,7 +13880,7 @@
         <v>1546</v>
       </c>
       <c r="I171" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J171" t="s">
         <v>1845</v>
@@ -13912,7 +13915,7 @@
         <v>1546</v>
       </c>
       <c r="I172" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J172" t="s">
         <v>1846</v>
@@ -14227,7 +14230,7 @@
         <v>1546</v>
       </c>
       <c r="I181" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J181" t="s">
         <v>1855</v>
@@ -14332,7 +14335,7 @@
         <v>1546</v>
       </c>
       <c r="I184" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="J184" t="s">
         <v>1858</v>
@@ -14402,7 +14405,7 @@
         <v>1546</v>
       </c>
       <c r="I186" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J186" t="s">
         <v>1860</v>
@@ -14507,7 +14510,7 @@
         <v>1546</v>
       </c>
       <c r="I189" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J189" t="s">
         <v>1863</v>
@@ -14612,7 +14615,7 @@
         <v>1546</v>
       </c>
       <c r="I192" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="J192" t="s">
         <v>1866</v>
@@ -14682,7 +14685,7 @@
         <v>1546</v>
       </c>
       <c r="I194" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J194" t="s">
         <v>1868</v>
@@ -14822,7 +14825,7 @@
         <v>1546</v>
       </c>
       <c r="I198" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J198" t="s">
         <v>1872</v>
@@ -14927,7 +14930,7 @@
         <v>1546</v>
       </c>
       <c r="I201" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J201" t="s">
         <v>1875</v>
@@ -14997,7 +15000,7 @@
         <v>1546</v>
       </c>
       <c r="I203" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="J203" t="s">
         <v>1877</v>
@@ -15035,7 +15038,7 @@
         <v>1550</v>
       </c>
       <c r="I204" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J204" t="s">
         <v>1878</v>
@@ -15070,7 +15073,7 @@
         <v>1546</v>
       </c>
       <c r="I205" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="J205" t="s">
         <v>1879</v>
@@ -15140,7 +15143,7 @@
         <v>1546</v>
       </c>
       <c r="I207" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="J207" t="s">
         <v>1881</v>
@@ -15245,7 +15248,7 @@
         <v>1546</v>
       </c>
       <c r="I210" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J210" t="s">
         <v>1884</v>
@@ -15315,7 +15318,7 @@
         <v>1546</v>
       </c>
       <c r="I212" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J212" t="s">
         <v>1886</v>
@@ -15350,7 +15353,7 @@
         <v>1546</v>
       </c>
       <c r="I213" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J213" t="s">
         <v>1887</v>
@@ -15385,7 +15388,7 @@
         <v>1546</v>
       </c>
       <c r="I214" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J214" t="s">
         <v>1888</v>
@@ -15490,7 +15493,7 @@
         <v>1546</v>
       </c>
       <c r="I217" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="J217" t="s">
         <v>1891</v>
@@ -15525,7 +15528,7 @@
         <v>1546</v>
       </c>
       <c r="I218" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J218" t="s">
         <v>1892</v>
@@ -15560,7 +15563,7 @@
         <v>1546</v>
       </c>
       <c r="I219" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J219" t="s">
         <v>1893</v>
@@ -15595,7 +15598,7 @@
         <v>1546</v>
       </c>
       <c r="I220" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J220" t="s">
         <v>1894</v>
@@ -15735,7 +15738,7 @@
         <v>1546</v>
       </c>
       <c r="I224" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="J224" t="s">
         <v>1898</v>
@@ -16120,7 +16123,7 @@
         <v>1546</v>
       </c>
       <c r="I235" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J235" t="s">
         <v>1909</v>
@@ -16155,7 +16158,7 @@
         <v>1546</v>
       </c>
       <c r="I236" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J236" t="s">
         <v>1910</v>
@@ -16785,7 +16788,7 @@
         <v>1546</v>
       </c>
       <c r="I254" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J254" t="s">
         <v>1926</v>
@@ -16855,7 +16858,7 @@
         <v>1546</v>
       </c>
       <c r="I256" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="J256" t="s">
         <v>1928</v>
@@ -17170,7 +17173,7 @@
         <v>1546</v>
       </c>
       <c r="I265" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J265" t="s">
         <v>1937</v>
@@ -17310,7 +17313,7 @@
         <v>1546</v>
       </c>
       <c r="I269" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J269" t="s">
         <v>1941</v>
@@ -17380,7 +17383,7 @@
         <v>1546</v>
       </c>
       <c r="I271" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J271" t="s">
         <v>1943</v>
@@ -17590,7 +17593,7 @@
         <v>1546</v>
       </c>
       <c r="I277" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J277" t="s">
         <v>1949</v>
@@ -17625,7 +17628,7 @@
         <v>1546</v>
       </c>
       <c r="I278" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J278" t="s">
         <v>1950</v>
@@ -17660,7 +17663,7 @@
         <v>1546</v>
       </c>
       <c r="I279" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J279" t="s">
         <v>1951</v>
@@ -17730,7 +17733,7 @@
         <v>1546</v>
       </c>
       <c r="I281" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="J281" t="s">
         <v>1953</v>
@@ -18115,7 +18118,7 @@
         <v>1546</v>
       </c>
       <c r="I292" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J292" t="s">
         <v>1964</v>
@@ -18150,7 +18153,7 @@
         <v>1546</v>
       </c>
       <c r="I293" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J293" t="s">
         <v>1965</v>
@@ -18255,7 +18258,7 @@
         <v>1546</v>
       </c>
       <c r="I296" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="J296" t="s">
         <v>1968</v>
@@ -18360,7 +18363,7 @@
         <v>1546</v>
       </c>
       <c r="I299" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J299" t="s">
         <v>1971</v>
@@ -18500,7 +18503,7 @@
         <v>1546</v>
       </c>
       <c r="I303" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J303" t="s">
         <v>1975</v>
@@ -18535,7 +18538,7 @@
         <v>1546</v>
       </c>
       <c r="I304" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J304" t="s">
         <v>1976</v>
@@ -18710,7 +18713,7 @@
         <v>1546</v>
       </c>
       <c r="I309" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J309" t="s">
         <v>1981</v>
@@ -18850,7 +18853,7 @@
         <v>1546</v>
       </c>
       <c r="I313" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J313" t="s">
         <v>1985</v>
@@ -18885,7 +18888,7 @@
         <v>1546</v>
       </c>
       <c r="I314" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J314" t="s">
         <v>1986</v>
@@ -19095,7 +19098,7 @@
         <v>1546</v>
       </c>
       <c r="I320" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J320" t="s">
         <v>1992</v>
@@ -19165,7 +19168,7 @@
         <v>1546</v>
       </c>
       <c r="I322" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J322" t="s">
         <v>1994</v>
@@ -19200,7 +19203,7 @@
         <v>1546</v>
       </c>
       <c r="I323" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J323" t="s">
         <v>1995</v>
@@ -19235,7 +19238,7 @@
         <v>1546</v>
       </c>
       <c r="I324" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J324" t="s">
         <v>1996</v>
@@ -19270,7 +19273,7 @@
         <v>1546</v>
       </c>
       <c r="I325" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J325" t="s">
         <v>1997</v>
@@ -19410,7 +19413,7 @@
         <v>1546</v>
       </c>
       <c r="I329" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J329" t="s">
         <v>2001</v>
@@ -19585,7 +19588,7 @@
         <v>1546</v>
       </c>
       <c r="I334" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J334" t="s">
         <v>2006</v>
@@ -19655,7 +19658,7 @@
         <v>1546</v>
       </c>
       <c r="I336" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J336" t="s">
         <v>2008</v>
@@ -19690,7 +19693,7 @@
         <v>1546</v>
       </c>
       <c r="I337" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J337" t="s">
         <v>2009</v>
@@ -19833,7 +19836,7 @@
         <v>1551</v>
       </c>
       <c r="I341" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J341" t="s">
         <v>2013</v>
@@ -19938,7 +19941,7 @@
         <v>1546</v>
       </c>
       <c r="I344" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J344" t="s">
         <v>2016</v>
@@ -20183,7 +20186,7 @@
         <v>1546</v>
       </c>
       <c r="I351" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J351" t="s">
         <v>2023</v>
@@ -20218,7 +20221,7 @@
         <v>1546</v>
       </c>
       <c r="I352" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J352" t="s">
         <v>2024</v>
@@ -20288,7 +20291,7 @@
         <v>1546</v>
       </c>
       <c r="I354" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J354" t="s">
         <v>2026</v>
@@ -20323,7 +20326,7 @@
         <v>1546</v>
       </c>
       <c r="I355" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J355" t="s">
         <v>2027</v>
@@ -20358,7 +20361,7 @@
         <v>1546</v>
       </c>
       <c r="I356" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J356" t="s">
         <v>2028</v>
@@ -20463,7 +20466,7 @@
         <v>1546</v>
       </c>
       <c r="I359" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J359" t="s">
         <v>2031</v>
@@ -20498,7 +20501,7 @@
         <v>1546</v>
       </c>
       <c r="I360" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J360" t="s">
         <v>2032</v>
@@ -20568,7 +20571,7 @@
         <v>1546</v>
       </c>
       <c r="I362" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J362" t="s">
         <v>2034</v>
@@ -20778,7 +20781,7 @@
         <v>1546</v>
       </c>
       <c r="I368" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J368" t="s">
         <v>2040</v>
@@ -20813,7 +20816,7 @@
         <v>1546</v>
       </c>
       <c r="I369" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J369" t="s">
         <v>2041</v>
@@ -20848,7 +20851,7 @@
         <v>1546</v>
       </c>
       <c r="I370" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J370" t="s">
         <v>2042</v>
@@ -20918,7 +20921,7 @@
         <v>1546</v>
       </c>
       <c r="I372" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J372" t="s">
         <v>2044</v>
@@ -20953,7 +20956,7 @@
         <v>1546</v>
       </c>
       <c r="I373" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J373" t="s">
         <v>2045</v>
@@ -21023,7 +21026,7 @@
         <v>1546</v>
       </c>
       <c r="I375" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J375" t="s">
         <v>2047</v>
@@ -21093,7 +21096,7 @@
         <v>1546</v>
       </c>
       <c r="I377" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J377" t="s">
         <v>2049</v>
@@ -21128,7 +21131,7 @@
         <v>1546</v>
       </c>
       <c r="I378" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J378" t="s">
         <v>2050</v>
@@ -21163,7 +21166,7 @@
         <v>1546</v>
       </c>
       <c r="I379" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J379" t="s">
         <v>2051</v>
@@ -21373,7 +21376,7 @@
         <v>1546</v>
       </c>
       <c r="I385" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J385" t="s">
         <v>2057</v>
@@ -21408,7 +21411,7 @@
         <v>1546</v>
       </c>
       <c r="I386" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J386" t="s">
         <v>2058</v>
@@ -21516,7 +21519,7 @@
         <v>1546</v>
       </c>
       <c r="I389" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J389" t="s">
         <v>2061</v>
@@ -21586,7 +21589,7 @@
         <v>1546</v>
       </c>
       <c r="I391" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J391" t="s">
         <v>2063</v>
@@ -21624,7 +21627,7 @@
         <v>1552</v>
       </c>
       <c r="I392" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J392" t="s">
         <v>2064</v>
@@ -21834,7 +21837,7 @@
         <v>1546</v>
       </c>
       <c r="I398" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J398" t="s">
         <v>2070</v>
@@ -21869,7 +21872,7 @@
         <v>1546</v>
       </c>
       <c r="I399" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J399" t="s">
         <v>2071</v>
@@ -22009,7 +22012,7 @@
         <v>1546</v>
       </c>
       <c r="I403" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J403" t="s">
         <v>2075</v>
@@ -22114,7 +22117,7 @@
         <v>1546</v>
       </c>
       <c r="I406" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J406" t="s">
         <v>2078</v>
@@ -22149,7 +22152,7 @@
         <v>1546</v>
       </c>
       <c r="I407" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J407" t="s">
         <v>2079</v>
@@ -22429,7 +22432,7 @@
         <v>1546</v>
       </c>
       <c r="I415" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J415" t="s">
         <v>2087</v>
@@ -22572,7 +22575,7 @@
         <v>1553</v>
       </c>
       <c r="I419" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J419" t="s">
         <v>2091</v>
@@ -22642,7 +22645,7 @@
         <v>1546</v>
       </c>
       <c r="I421" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J421" t="s">
         <v>2093</v>
@@ -22677,7 +22680,7 @@
         <v>1546</v>
       </c>
       <c r="I422" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J422" t="s">
         <v>2094</v>
@@ -22747,7 +22750,7 @@
         <v>1546</v>
       </c>
       <c r="I424" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J424" t="s">
         <v>2096</v>
@@ -22817,7 +22820,7 @@
         <v>1546</v>
       </c>
       <c r="I426" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J426" t="s">
         <v>2098</v>
@@ -22887,7 +22890,7 @@
         <v>1546</v>
       </c>
       <c r="I428" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J428" t="s">
         <v>2100</v>
@@ -22922,7 +22925,7 @@
         <v>1546</v>
       </c>
       <c r="I429" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J429" t="s">
         <v>2101</v>
@@ -22957,7 +22960,7 @@
         <v>1546</v>
       </c>
       <c r="I430" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J430" t="s">
         <v>2102</v>
@@ -23097,7 +23100,7 @@
         <v>1546</v>
       </c>
       <c r="I434" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J434" t="s">
         <v>2106</v>
@@ -23167,7 +23170,7 @@
         <v>1546</v>
       </c>
       <c r="I436" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J436" t="s">
         <v>2108</v>
@@ -23272,7 +23275,7 @@
         <v>1546</v>
       </c>
       <c r="I439" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J439" t="s">
         <v>2111</v>
@@ -23307,7 +23310,7 @@
         <v>1546</v>
       </c>
       <c r="I440" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J440" t="s">
         <v>2112</v>
@@ -23342,7 +23345,7 @@
         <v>1546</v>
       </c>
       <c r="I441" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J441" t="s">
         <v>2113</v>
@@ -23377,7 +23380,7 @@
         <v>1546</v>
       </c>
       <c r="I442" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J442" t="s">
         <v>2114</v>
@@ -23447,7 +23450,7 @@
         <v>1546</v>
       </c>
       <c r="I444" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J444" t="s">
         <v>2116</v>
@@ -23587,7 +23590,7 @@
         <v>1546</v>
       </c>
       <c r="I448" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J448" t="s">
         <v>2120</v>
@@ -23762,7 +23765,7 @@
         <v>1546</v>
       </c>
       <c r="I453" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J453" t="s">
         <v>2125</v>
@@ -23797,7 +23800,7 @@
         <v>1546</v>
       </c>
       <c r="I454" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J454" t="s">
         <v>2126</v>
@@ -23832,7 +23835,7 @@
         <v>1546</v>
       </c>
       <c r="I455" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J455" t="s">
         <v>2127</v>
@@ -23937,7 +23940,7 @@
         <v>1546</v>
       </c>
       <c r="I458" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J458" t="s">
         <v>2130</v>
@@ -24042,7 +24045,7 @@
         <v>1546</v>
       </c>
       <c r="I461" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J461" t="s">
         <v>2133</v>
@@ -24077,7 +24080,7 @@
         <v>1546</v>
       </c>
       <c r="I462" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J462" t="s">
         <v>2134</v>
@@ -24112,7 +24115,7 @@
         <v>1546</v>
       </c>
       <c r="I463" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J463" t="s">
         <v>2135</v>
@@ -24147,7 +24150,7 @@
         <v>1546</v>
       </c>
       <c r="I464" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J464" t="s">
         <v>2136</v>
@@ -24217,7 +24220,7 @@
         <v>1546</v>
       </c>
       <c r="I466" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J466" t="s">
         <v>2138</v>
@@ -24427,7 +24430,7 @@
         <v>1546</v>
       </c>
       <c r="I472" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J472" t="s">
         <v>2144</v>
@@ -24462,7 +24465,7 @@
         <v>1546</v>
       </c>
       <c r="I473" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J473" t="s">
         <v>2145</v>
@@ -24471,7 +24474,7 @@
         <v>2347</v>
       </c>
       <c r="L473" t="s">
-        <v>2459</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="474" spans="1:12">
@@ -24637,7 +24640,7 @@
         <v>1546</v>
       </c>
       <c r="I478" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J478" t="s">
         <v>2150</v>
@@ -24672,7 +24675,7 @@
         <v>1546</v>
       </c>
       <c r="I479" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J479" t="s">
         <v>2151</v>
@@ -24707,7 +24710,7 @@
         <v>1546</v>
       </c>
       <c r="I480" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J480" t="s">
         <v>2152</v>
@@ -24885,7 +24888,7 @@
         <v>1546</v>
       </c>
       <c r="I485" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J485" t="s">
         <v>2157</v>
@@ -24920,7 +24923,7 @@
         <v>1546</v>
       </c>
       <c r="I486" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J486" t="s">
         <v>2158</v>
@@ -24955,7 +24958,7 @@
         <v>1546</v>
       </c>
       <c r="I487" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J487" t="s">
         <v>2159</v>
@@ -24990,7 +24993,7 @@
         <v>1546</v>
       </c>
       <c r="I488" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J488" t="s">
         <v>2160</v>
@@ -25028,7 +25031,7 @@
         <v>1554</v>
       </c>
       <c r="I489" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J489" t="s">
         <v>2161</v>
@@ -25063,7 +25066,7 @@
         <v>1546</v>
       </c>
       <c r="I490" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J490" t="s">
         <v>2162</v>
@@ -25168,7 +25171,7 @@
         <v>1546</v>
       </c>
       <c r="I493" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J493" t="s">
         <v>2165</v>
@@ -25247,7 +25250,7 @@
         <v>2354</v>
       </c>
       <c r="L495" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="496" spans="1:12">
@@ -25308,7 +25311,7 @@
         <v>1546</v>
       </c>
       <c r="I497" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J497" t="s">
         <v>2169</v>
@@ -25343,7 +25346,7 @@
         <v>1546</v>
       </c>
       <c r="I498" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J498" t="s">
         <v>2170</v>
@@ -25378,7 +25381,7 @@
         <v>1546</v>
       </c>
       <c r="I499" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J499" t="s">
         <v>2171</v>
@@ -25448,7 +25451,7 @@
         <v>1546</v>
       </c>
       <c r="I501" t="s">
-        <v>1575</v>
+        <v>1595</v>
       </c>
       <c r="J501" t="s">
         <v>2173</v>
@@ -25483,7 +25486,7 @@
         <v>1546</v>
       </c>
       <c r="I502" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J502" t="s">
         <v>2174</v>
@@ -25553,7 +25556,7 @@
         <v>1546</v>
       </c>
       <c r="I504" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J504" t="s">
         <v>2176</v>
@@ -25658,7 +25661,7 @@
         <v>1546</v>
       </c>
       <c r="I507" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J507" t="s">
         <v>2179</v>
@@ -25728,7 +25731,7 @@
         <v>1546</v>
       </c>
       <c r="I509" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J509" t="s">
         <v>2181</v>
@@ -25763,7 +25766,7 @@
         <v>1546</v>
       </c>
       <c r="I510" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J510" t="s">
         <v>2182</v>
@@ -25833,7 +25836,7 @@
         <v>1546</v>
       </c>
       <c r="I512" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J512" t="s">
         <v>2184</v>
@@ -25868,7 +25871,7 @@
         <v>1546</v>
       </c>
       <c r="I513" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J513" t="s">
         <v>2185</v>
@@ -25903,7 +25906,7 @@
         <v>1546</v>
       </c>
       <c r="I514" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J514" t="s">
         <v>2186</v>
@@ -25938,7 +25941,7 @@
         <v>1546</v>
       </c>
       <c r="I515" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J515" t="s">
         <v>2187</v>
@@ -26011,7 +26014,7 @@
         <v>1546</v>
       </c>
       <c r="I517" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J517" t="s">
         <v>2189</v>
@@ -26046,7 +26049,7 @@
         <v>1546</v>
       </c>
       <c r="I518" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J518" t="s">
         <v>2190</v>
@@ -26081,7 +26084,7 @@
         <v>1546</v>
       </c>
       <c r="I519" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J519" t="s">
         <v>2191</v>
@@ -26090,7 +26093,7 @@
         <v>2360</v>
       </c>
       <c r="L519" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="520" spans="1:12">
@@ -26116,7 +26119,7 @@
         <v>1546</v>
       </c>
       <c r="I520" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J520" t="s">
         <v>2192</v>
@@ -26154,7 +26157,7 @@
         <v>1556</v>
       </c>
       <c r="I521" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J521" t="s">
         <v>2193</v>
@@ -26189,7 +26192,7 @@
         <v>1546</v>
       </c>
       <c r="I522" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J522" t="s">
         <v>2194</v>
@@ -26224,7 +26227,7 @@
         <v>1546</v>
       </c>
       <c r="I523" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J523" t="s">
         <v>2195</v>
@@ -26259,7 +26262,7 @@
         <v>1546</v>
       </c>
       <c r="I524" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J524" t="s">
         <v>2196</v>
@@ -26294,7 +26297,7 @@
         <v>1546</v>
       </c>
       <c r="I525" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J525" t="s">
         <v>2197</v>
@@ -26329,7 +26332,7 @@
         <v>1546</v>
       </c>
       <c r="I526" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J526" t="s">
         <v>2198</v>
@@ -26364,7 +26367,7 @@
         <v>1546</v>
       </c>
       <c r="I527" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J527" t="s">
         <v>2199</v>
@@ -26399,7 +26402,7 @@
         <v>1546</v>
       </c>
       <c r="I528" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J528" t="s">
         <v>2200</v>
@@ -26434,7 +26437,7 @@
         <v>1546</v>
       </c>
       <c r="I529" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J529" t="s">
         <v>2201</v>
@@ -26469,7 +26472,7 @@
         <v>1546</v>
       </c>
       <c r="I530" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J530" t="s">
         <v>2202</v>
@@ -26483,7 +26486,7 @@
     </row>
     <row r="531" spans="1:12">
       <c r="A531" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B531" t="s">
         <v>571</v>
@@ -26504,7 +26507,7 @@
         <v>1546</v>
       </c>
       <c r="I531" t="s">
-        <v>1668</v>
+        <v>1575</v>
       </c>
       <c r="J531" t="s">
         <v>2203</v>
@@ -26539,7 +26542,7 @@
         <v>1546</v>
       </c>
       <c r="I532" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J532" t="s">
         <v>2204</v>
@@ -26574,7 +26577,7 @@
         <v>1546</v>
       </c>
       <c r="I533" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J533" t="s">
         <v>2205</v>
@@ -26609,7 +26612,7 @@
         <v>1546</v>
       </c>
       <c r="I534" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J534" t="s">
         <v>2206</v>
@@ -26644,7 +26647,7 @@
         <v>1546</v>
       </c>
       <c r="I535" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J535" t="s">
         <v>2207</v>
@@ -26679,7 +26682,7 @@
         <v>1546</v>
       </c>
       <c r="I536" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J536" t="s">
         <v>2208</v>
@@ -26714,7 +26717,7 @@
         <v>1546</v>
       </c>
       <c r="I537" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J537" t="s">
         <v>2208</v>
@@ -26784,7 +26787,7 @@
         <v>1546</v>
       </c>
       <c r="I539" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J539" t="s">
         <v>2210</v>
@@ -26819,7 +26822,7 @@
         <v>1546</v>
       </c>
       <c r="I540" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J540" t="s">
         <v>2211</v>
@@ -26854,7 +26857,7 @@
         <v>1546</v>
       </c>
       <c r="I541" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J541" t="s">
         <v>2212</v>
@@ -26889,7 +26892,7 @@
         <v>1546</v>
       </c>
       <c r="I542" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J542" t="s">
         <v>2213</v>
@@ -26924,7 +26927,7 @@
         <v>1546</v>
       </c>
       <c r="I543" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J543" t="s">
         <v>2214</v>
@@ -26959,7 +26962,7 @@
         <v>1546</v>
       </c>
       <c r="I544" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J544" t="s">
         <v>2215</v>
@@ -27029,7 +27032,7 @@
         <v>1546</v>
       </c>
       <c r="I546" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J546" t="s">
         <v>2217</v>
@@ -27064,7 +27067,7 @@
         <v>1546</v>
       </c>
       <c r="I547" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J547" t="s">
         <v>2218</v>
@@ -27149,7 +27152,7 @@
         <v>2319</v>
       </c>
       <c r="L549" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="550" spans="1:12">
@@ -27213,7 +27216,7 @@
         <v>1546</v>
       </c>
       <c r="I551" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J551" t="s">
         <v>2222</v>
@@ -27248,7 +27251,7 @@
         <v>1546</v>
       </c>
       <c r="I552" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J552" t="s">
         <v>2223</v>
@@ -27257,7 +27260,7 @@
         <v>2354</v>
       </c>
       <c r="L552" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27283,7 +27286,7 @@
         <v>1548</v>
       </c>
       <c r="I553" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J553" t="s">
         <v>2224</v>
@@ -27388,7 +27391,7 @@
         <v>1546</v>
       </c>
       <c r="I556" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J556" t="s">
         <v>2227</v>
@@ -27528,7 +27531,7 @@
         <v>1546</v>
       </c>
       <c r="I560" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J560" t="s">
         <v>2231</v>
@@ -27563,7 +27566,7 @@
         <v>1546</v>
       </c>
       <c r="I561" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J561" t="s">
         <v>2232</v>
@@ -27633,7 +27636,7 @@
         <v>1546</v>
       </c>
       <c r="I563" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J563" t="s">
         <v>2234</v>
@@ -27668,7 +27671,7 @@
         <v>1546</v>
       </c>
       <c r="I564" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J564" t="s">
         <v>2235</v>
@@ -27782,7 +27785,7 @@
         <v>2393</v>
       </c>
       <c r="L567" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="568" spans="1:12">
@@ -27808,7 +27811,7 @@
         <v>1546</v>
       </c>
       <c r="I568" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J568" t="s">
         <v>2238</v>
@@ -27843,7 +27846,7 @@
         <v>1546</v>
       </c>
       <c r="I569" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J569" t="s">
         <v>2239</v>
@@ -27878,7 +27881,7 @@
         <v>1546</v>
       </c>
       <c r="I570" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J570" t="s">
         <v>2240</v>
@@ -28021,7 +28024,7 @@
         <v>1546</v>
       </c>
       <c r="I574" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J574" t="s">
         <v>2243</v>
@@ -28056,7 +28059,7 @@
         <v>1546</v>
       </c>
       <c r="I575" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J575" t="s">
         <v>2244</v>
@@ -28091,7 +28094,7 @@
         <v>1546</v>
       </c>
       <c r="I576" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J576" t="s">
         <v>2245</v>
@@ -28138,7 +28141,7 @@
         <v>2327</v>
       </c>
       <c r="L577" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="578" spans="1:12">
@@ -28173,7 +28176,7 @@
         <v>2401</v>
       </c>
       <c r="L578" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="579" spans="1:12">
@@ -28374,7 +28377,7 @@
         <v>1546</v>
       </c>
       <c r="I584" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J584" t="s">
         <v>2253</v>
@@ -28549,7 +28552,7 @@
         <v>1546</v>
       </c>
       <c r="I589" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J589" t="s">
         <v>2258</v>
@@ -28619,7 +28622,7 @@
         <v>1546</v>
       </c>
       <c r="I591" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J591" t="s">
         <v>2260</v>
@@ -28689,7 +28692,7 @@
         <v>1546</v>
       </c>
       <c r="I593" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J593" t="s">
         <v>2262</v>
@@ -28733,7 +28736,7 @@
         <v>2390</v>
       </c>
       <c r="L594" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28797,7 +28800,7 @@
         <v>1558</v>
       </c>
       <c r="I596" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J596" t="s">
         <v>2265</v>
@@ -28905,7 +28908,7 @@
         <v>1546</v>
       </c>
       <c r="I599" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J599" t="s">
         <v>2268</v>
@@ -28940,7 +28943,7 @@
         <v>1546</v>
       </c>
       <c r="I600" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J600" t="s">
         <v>2269</v>
@@ -28975,7 +28978,7 @@
         <v>1546</v>
       </c>
       <c r="I601" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J601" t="s">
         <v>2270</v>
@@ -29010,7 +29013,7 @@
         <v>1546</v>
       </c>
       <c r="I602" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J602" t="s">
         <v>2271</v>
@@ -29048,7 +29051,7 @@
         <v>1560</v>
       </c>
       <c r="I603" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J603" t="s">
         <v>2272</v>
@@ -29083,7 +29086,7 @@
         <v>1546</v>
       </c>
       <c r="I604" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J604" t="s">
         <v>2273</v>
@@ -29191,7 +29194,7 @@
         <v>1546</v>
       </c>
       <c r="I607" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J607" t="s">
         <v>2276</v>
@@ -29226,7 +29229,7 @@
         <v>1546</v>
       </c>
       <c r="I608" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J608" t="s">
         <v>2277</v>
@@ -29261,7 +29264,7 @@
         <v>1546</v>
       </c>
       <c r="I609" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J609" t="s">
         <v>2278</v>
@@ -29331,7 +29334,7 @@
         <v>1546</v>
       </c>
       <c r="I611" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J611" t="s">
         <v>2280</v>
@@ -29404,7 +29407,7 @@
         <v>1546</v>
       </c>
       <c r="I613" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J613" t="s">
         <v>2282</v>
@@ -29439,7 +29442,7 @@
         <v>1546</v>
       </c>
       <c r="I614" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J614" t="s">
         <v>2283</v>
@@ -29477,7 +29480,7 @@
         <v>1562</v>
       </c>
       <c r="I615" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J615" t="s">
         <v>2284</v>
@@ -29585,7 +29588,7 @@
         <v>1546</v>
       </c>
       <c r="I618" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J618" t="s">
         <v>2287</v>
@@ -29620,7 +29623,7 @@
         <v>1546</v>
       </c>
       <c r="I619" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J619" t="s">
         <v>2288</v>
@@ -29725,7 +29728,7 @@
         <v>1546</v>
       </c>
       <c r="I622" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J622" t="s">
         <v>2291</v>
@@ -29763,7 +29766,7 @@
         <v>1564</v>
       </c>
       <c r="I623" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J623" t="s">
         <v>2292</v>
@@ -29798,7 +29801,7 @@
         <v>1546</v>
       </c>
       <c r="I624" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J624" t="s">
         <v>2293</v>
@@ -29833,7 +29836,7 @@
         <v>1546</v>
       </c>
       <c r="I625" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J625" t="s">
         <v>2294</v>
@@ -29868,7 +29871,7 @@
         <v>1546</v>
       </c>
       <c r="I626" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J626" t="s">
         <v>2295</v>
@@ -29938,7 +29941,7 @@
         <v>1546</v>
       </c>
       <c r="I628" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J628" t="s">
         <v>2297</v>
@@ -30043,7 +30046,7 @@
         <v>1546</v>
       </c>
       <c r="I631" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J631" t="s">
         <v>2300</v>
@@ -30081,7 +30084,7 @@
         <v>1565</v>
       </c>
       <c r="I632" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J632" t="s">
         <v>2301</v>
@@ -30154,7 +30157,7 @@
         <v>1546</v>
       </c>
       <c r="I634" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J634" t="s">
         <v>2303</v>
@@ -30224,7 +30227,7 @@
         <v>1546</v>
       </c>
       <c r="I636" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J636" t="s">
         <v>2305</v>
@@ -30259,7 +30262,7 @@
         <v>1546</v>
       </c>
       <c r="I637" t="s">
-        <v>1678</v>
+        <v>1606</v>
       </c>
       <c r="J637" t="s">
         <v>2306</v>
@@ -30268,7 +30271,7 @@
         <v>2364</v>
       </c>
       <c r="L637" t="s">
-        <v>2493</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30294,7 +30297,7 @@
         <v>1546</v>
       </c>
       <c r="I638" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J638" t="s">
         <v>2307</v>
@@ -30335,7 +30338,7 @@
         <v>2432</v>
       </c>
       <c r="L639" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="640" spans="1:12">
@@ -30367,7 +30370,7 @@
         <v>2432</v>
       </c>
       <c r="L640" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-03 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7453,7 +7453,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7483,7 +7483,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
@@ -7501,7 +7501,7 @@
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,PSICOLOGIA,ECONOMIA,ORÇAMENTO,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,URBANISMO,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ASSISTÊNCIA SOCIAL</t>
+    <t>SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ORÇAMENTO,MOBILIDADE E TRANSPORTE,URBANISMO,ECONOMIA,PSICOLOGIA</t>
   </si>
 </sst>
 </file>
@@ -23253,7 +23253,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B440" t="s">
         <v>479</v>
@@ -30089,7 +30089,7 @@
         <v>2304</v>
       </c>
       <c r="L633" t="s">
-        <v>2482</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="634" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-04 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4891,61 +4891,61 @@
     <t>ITAMAR COSTA KALIL</t>
   </si>
   <si>
+    <t>FERNANDA TEIXEIRA ROSALBA</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>PAULA DE ARAUJO CRUZ VIGIO</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>NIVANA DANIELLE SILVA COSTA</t>
+  </si>
+  <si>
+    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
     <t>REINALDO DE SOUZA MACHADO</t>
-  </si>
-  <si>
-    <t>FERNANDA TEIXEIRA ROSALBA</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>PAULA DE ARAUJO CRUZ VIGIO</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>NIVANA DANIELLE SILVA COSTA</t>
-  </si>
-  <si>
-    <t>JULIANA BUSTAMANTE DE MONTI SOUZA</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,SIMONE MANNHEIMER DE ALVARENGA</t>
@@ -13940,7 +13940,7 @@
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B174" t="s">
         <v>213</v>
@@ -13961,7 +13961,7 @@
         <v>1542</v>
       </c>
       <c r="I174" t="s">
-        <v>1625</v>
+        <v>1569</v>
       </c>
       <c r="J174" t="s">
         <v>1843</v>
@@ -14031,7 +14031,7 @@
         <v>1542</v>
       </c>
       <c r="I176" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
       <c r="J176" t="s">
         <v>1845</v>
@@ -14066,7 +14066,7 @@
         <v>1542</v>
       </c>
       <c r="I177" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="J177" t="s">
         <v>1846</v>
@@ -14241,7 +14241,7 @@
         <v>1542</v>
       </c>
       <c r="I182" t="s">
-        <v>1628</v>
+        <v>1627</v>
       </c>
       <c r="J182" t="s">
         <v>1851</v>
@@ -14346,7 +14346,7 @@
         <v>1542</v>
       </c>
       <c r="I185" t="s">
-        <v>1629</v>
+        <v>1628</v>
       </c>
       <c r="J185" t="s">
         <v>1854</v>
@@ -14451,7 +14451,7 @@
         <v>1542</v>
       </c>
       <c r="I188" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J188" t="s">
         <v>1857</v>
@@ -14521,7 +14521,7 @@
         <v>1542</v>
       </c>
       <c r="I190" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J190" t="s">
         <v>1859</v>
@@ -14661,7 +14661,7 @@
         <v>1542</v>
       </c>
       <c r="I194" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J194" t="s">
         <v>1863</v>
@@ -14836,7 +14836,7 @@
         <v>1542</v>
       </c>
       <c r="I199" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="J199" t="s">
         <v>1868</v>
@@ -14874,7 +14874,7 @@
         <v>1546</v>
       </c>
       <c r="I200" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J200" t="s">
         <v>1869</v>
@@ -14944,7 +14944,7 @@
         <v>1542</v>
       </c>
       <c r="I202" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="J202" t="s">
         <v>1871</v>
@@ -15119,7 +15119,7 @@
         <v>1542</v>
       </c>
       <c r="I207" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="J207" t="s">
         <v>1876</v>
@@ -15154,7 +15154,7 @@
         <v>1542</v>
       </c>
       <c r="I208" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="J208" t="s">
         <v>1877</v>
@@ -15189,7 +15189,7 @@
         <v>1542</v>
       </c>
       <c r="I209" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="J209" t="s">
         <v>1878</v>
@@ -15364,7 +15364,7 @@
         <v>1542</v>
       </c>
       <c r="I214" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="J214" t="s">
         <v>1883</v>
@@ -15399,7 +15399,7 @@
         <v>1542</v>
       </c>
       <c r="I215" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="J215" t="s">
         <v>1884</v>
@@ -15539,7 +15539,7 @@
         <v>1542</v>
       </c>
       <c r="I219" t="s">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="J219" t="s">
         <v>1888</v>
@@ -15924,7 +15924,7 @@
         <v>1542</v>
       </c>
       <c r="I230" t="s">
-        <v>1628</v>
+        <v>1627</v>
       </c>
       <c r="J230" t="s">
         <v>1899</v>
@@ -16554,7 +16554,7 @@
         <v>1542</v>
       </c>
       <c r="I248" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="J248" t="s">
         <v>1915</v>
@@ -16624,7 +16624,7 @@
         <v>1542</v>
       </c>
       <c r="I250" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="J250" t="s">
         <v>1917</v>
@@ -16939,7 +16939,7 @@
         <v>1542</v>
       </c>
       <c r="I259" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J259" t="s">
         <v>1926</v>
@@ -17079,7 +17079,7 @@
         <v>1542</v>
       </c>
       <c r="I263" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J263" t="s">
         <v>1930</v>
@@ -17149,7 +17149,7 @@
         <v>1542</v>
       </c>
       <c r="I265" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J265" t="s">
         <v>1932</v>
@@ -17394,7 +17394,7 @@
         <v>1542</v>
       </c>
       <c r="I272" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J272" t="s">
         <v>1939</v>
@@ -17464,7 +17464,7 @@
         <v>1542</v>
       </c>
       <c r="I274" t="s">
-        <v>1643</v>
+        <v>1642</v>
       </c>
       <c r="J274" t="s">
         <v>1941</v>
@@ -17849,7 +17849,7 @@
         <v>1542</v>
       </c>
       <c r="I285" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J285" t="s">
         <v>1952</v>
@@ -17884,7 +17884,7 @@
         <v>1542</v>
       </c>
       <c r="I286" t="s">
-        <v>1625</v>
+        <v>1643</v>
       </c>
       <c r="J286" t="s">
         <v>1953</v>
@@ -18094,7 +18094,7 @@
         <v>1542</v>
       </c>
       <c r="I292" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J292" t="s">
         <v>1959</v>
@@ -18234,7 +18234,7 @@
         <v>1542</v>
       </c>
       <c r="I296" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J296" t="s">
         <v>1963</v>
@@ -18269,7 +18269,7 @@
         <v>1542</v>
       </c>
       <c r="I297" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J297" t="s">
         <v>1964</v>
@@ -18444,7 +18444,7 @@
         <v>1542</v>
       </c>
       <c r="I302" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J302" t="s">
         <v>1969</v>
@@ -18829,7 +18829,7 @@
         <v>1542</v>
       </c>
       <c r="I313" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J313" t="s">
         <v>1980</v>
@@ -19319,7 +19319,7 @@
         <v>1542</v>
       </c>
       <c r="I327" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J327" t="s">
         <v>1994</v>
@@ -19424,7 +19424,7 @@
         <v>1542</v>
       </c>
       <c r="I330" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J330" t="s">
         <v>1997</v>
@@ -19567,7 +19567,7 @@
         <v>1547</v>
       </c>
       <c r="I334" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J334" t="s">
         <v>2001</v>
@@ -19672,7 +19672,7 @@
         <v>1542</v>
       </c>
       <c r="I337" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J337" t="s">
         <v>2004</v>
@@ -20022,7 +20022,7 @@
         <v>1542</v>
       </c>
       <c r="I347" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J347" t="s">
         <v>2014</v>
@@ -20057,7 +20057,7 @@
         <v>1542</v>
       </c>
       <c r="I348" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J348" t="s">
         <v>2015</v>
@@ -20302,7 +20302,7 @@
         <v>1542</v>
       </c>
       <c r="I355" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J355" t="s">
         <v>2022</v>
@@ -20512,7 +20512,7 @@
         <v>1542</v>
       </c>
       <c r="I361" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J361" t="s">
         <v>2028</v>
@@ -20547,7 +20547,7 @@
         <v>1542</v>
       </c>
       <c r="I362" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J362" t="s">
         <v>2029</v>
@@ -20582,7 +20582,7 @@
         <v>1542</v>
       </c>
       <c r="I363" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J363" t="s">
         <v>2030</v>
@@ -20827,7 +20827,7 @@
         <v>1542</v>
       </c>
       <c r="I370" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J370" t="s">
         <v>2037</v>
@@ -20862,7 +20862,7 @@
         <v>1542</v>
       </c>
       <c r="I371" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J371" t="s">
         <v>2038</v>
@@ -21107,7 +21107,7 @@
         <v>1542</v>
       </c>
       <c r="I378" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J378" t="s">
         <v>2045</v>
@@ -21320,7 +21320,7 @@
         <v>1542</v>
       </c>
       <c r="I384" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J384" t="s">
         <v>2051</v>
@@ -21358,7 +21358,7 @@
         <v>1548</v>
       </c>
       <c r="I385" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J385" t="s">
         <v>2052</v>
@@ -21603,7 +21603,7 @@
         <v>1542</v>
       </c>
       <c r="I392" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J392" t="s">
         <v>2059</v>
@@ -21883,7 +21883,7 @@
         <v>1542</v>
       </c>
       <c r="I400" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J400" t="s">
         <v>2067</v>
@@ -22163,7 +22163,7 @@
         <v>1542</v>
       </c>
       <c r="I408" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J408" t="s">
         <v>2075</v>
@@ -22411,7 +22411,7 @@
         <v>1542</v>
       </c>
       <c r="I415" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J415" t="s">
         <v>2082</v>
@@ -22551,7 +22551,7 @@
         <v>1542</v>
       </c>
       <c r="I419" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J419" t="s">
         <v>2086</v>
@@ -22621,7 +22621,7 @@
         <v>1542</v>
       </c>
       <c r="I421" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J421" t="s">
         <v>2088</v>
@@ -22656,7 +22656,7 @@
         <v>1542</v>
       </c>
       <c r="I422" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J422" t="s">
         <v>2089</v>
@@ -22691,7 +22691,7 @@
         <v>1542</v>
       </c>
       <c r="I423" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J423" t="s">
         <v>2090</v>
@@ -23006,7 +23006,7 @@
         <v>1542</v>
       </c>
       <c r="I432" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J432" t="s">
         <v>2099</v>
@@ -23181,7 +23181,7 @@
         <v>1542</v>
       </c>
       <c r="I437" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J437" t="s">
         <v>2104</v>
@@ -23811,7 +23811,7 @@
         <v>1542</v>
       </c>
       <c r="I455" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J455" t="s">
         <v>2122</v>
@@ -23846,7 +23846,7 @@
         <v>1542</v>
       </c>
       <c r="I456" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J456" t="s">
         <v>2123</v>
@@ -23881,7 +23881,7 @@
         <v>1542</v>
       </c>
       <c r="I457" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J457" t="s">
         <v>2124</v>
@@ -24371,7 +24371,7 @@
         <v>1542</v>
       </c>
       <c r="I471" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J471" t="s">
         <v>2138</v>
@@ -24619,7 +24619,7 @@
         <v>1542</v>
       </c>
       <c r="I478" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J478" t="s">
         <v>2145</v>
@@ -24762,7 +24762,7 @@
         <v>1550</v>
       </c>
       <c r="I482" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J482" t="s">
         <v>2149</v>
@@ -24797,7 +24797,7 @@
         <v>1542</v>
       </c>
       <c r="I483" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J483" t="s">
         <v>2150</v>
@@ -25112,7 +25112,7 @@
         <v>1542</v>
       </c>
       <c r="I492" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J492" t="s">
         <v>2159</v>
@@ -25182,7 +25182,7 @@
         <v>1542</v>
       </c>
       <c r="I494" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J494" t="s">
         <v>2161</v>
@@ -25427,7 +25427,7 @@
         <v>1542</v>
       </c>
       <c r="I501" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J501" t="s">
         <v>2168</v>
@@ -25532,7 +25532,7 @@
         <v>1542</v>
       </c>
       <c r="I504" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J504" t="s">
         <v>2171</v>
@@ -25672,7 +25672,7 @@
         <v>1542</v>
       </c>
       <c r="I508" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J508" t="s">
         <v>2175</v>
@@ -25777,7 +25777,7 @@
         <v>1542</v>
       </c>
       <c r="I511" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J511" t="s">
         <v>2178</v>
@@ -25885,7 +25885,7 @@
         <v>1542</v>
       </c>
       <c r="I514" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J514" t="s">
         <v>2181</v>
@@ -25920,7 +25920,7 @@
         <v>1542</v>
       </c>
       <c r="I515" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J515" t="s">
         <v>2182</v>
@@ -26025,7 +26025,7 @@
         <v>1542</v>
       </c>
       <c r="I518" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J518" t="s">
         <v>2185</v>
@@ -26060,7 +26060,7 @@
         <v>1542</v>
       </c>
       <c r="I519" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J519" t="s">
         <v>2186</v>
@@ -26095,7 +26095,7 @@
         <v>1542</v>
       </c>
       <c r="I520" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J520" t="s">
         <v>2187</v>
@@ -26200,7 +26200,7 @@
         <v>1542</v>
       </c>
       <c r="I523" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J523" t="s">
         <v>2190</v>
@@ -26270,7 +26270,7 @@
         <v>1542</v>
       </c>
       <c r="I525" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J525" t="s">
         <v>2192</v>
@@ -26375,7 +26375,7 @@
         <v>1542</v>
       </c>
       <c r="I528" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J528" t="s">
         <v>2194</v>
@@ -26480,7 +26480,7 @@
         <v>1542</v>
       </c>
       <c r="I531" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J531" t="s">
         <v>2197</v>
@@ -26620,7 +26620,7 @@
         <v>1542</v>
       </c>
       <c r="I535" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J535" t="s">
         <v>2201</v>
@@ -26798,7 +26798,7 @@
         <v>1544</v>
       </c>
       <c r="I540" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J540" t="s">
         <v>2206</v>
@@ -27043,7 +27043,7 @@
         <v>1542</v>
       </c>
       <c r="I547" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J547" t="s">
         <v>2213</v>
@@ -27571,7 +27571,7 @@
         <v>1542</v>
       </c>
       <c r="I562" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J562" t="s">
         <v>2226</v>
@@ -28096,7 +28096,7 @@
         <v>1542</v>
       </c>
       <c r="I577" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J577" t="s">
         <v>2241</v>
@@ -28166,7 +28166,7 @@
         <v>1542</v>
       </c>
       <c r="I579" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="J579" t="s">
         <v>2243</v>
@@ -28274,7 +28274,7 @@
         <v>1553</v>
       </c>
       <c r="I582" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J582" t="s">
         <v>2246</v>
@@ -28344,7 +28344,7 @@
         <v>1542</v>
       </c>
       <c r="I584" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J584" t="s">
         <v>2248</v>
@@ -28414,7 +28414,7 @@
         <v>1542</v>
       </c>
       <c r="I586" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J586" t="s">
         <v>2250</v>
@@ -28522,7 +28522,7 @@
         <v>1542</v>
       </c>
       <c r="I589" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J589" t="s">
         <v>2253</v>
@@ -28770,7 +28770,7 @@
         <v>1542</v>
       </c>
       <c r="I596" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J596" t="s">
         <v>2260</v>
@@ -29202,7 +29202,7 @@
         <v>1557</v>
       </c>
       <c r="I608" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="J608" t="s">
         <v>2272</v>
@@ -29593,7 +29593,7 @@
         <v>1542</v>
       </c>
       <c r="I619" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J619" t="s">
         <v>2283</v>
@@ -29663,7 +29663,7 @@
         <v>1542</v>
       </c>
       <c r="I621" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J621" t="s">
         <v>2285</v>
@@ -29768,7 +29768,7 @@
         <v>1542</v>
       </c>
       <c r="I624" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J624" t="s">
         <v>2288</v>
@@ -29949,7 +29949,7 @@
         <v>1542</v>
       </c>
       <c r="I629" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J629" t="s">
         <v>2292</v>
@@ -30095,7 +30095,7 @@
         <v>1560</v>
       </c>
       <c r="I633" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="J633" t="s">
         <v>2296</v>
@@ -30200,7 +30200,7 @@
         <v>1542</v>
       </c>
       <c r="I636" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="J636" t="s">
         <v>2299</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-05 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -28078,7 +28078,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B577" t="s">
         <v>614</v>
@@ -28102,7 +28102,7 @@
         <v>1549</v>
       </c>
       <c r="I577" t="s">
-        <v>1589</v>
+        <v>1565</v>
       </c>
       <c r="J577" t="s">
         <v>2244</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-06 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6373" uniqueCount="2498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6372" uniqueCount="2498">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -1879,9 +1879,6 @@
     <t>20.22.0001.0051719.2026-06</t>
   </si>
   <si>
-    <t>20.22.0001.0051626.2026-92</t>
-  </si>
-  <si>
     <t>20.22.0001.0052338.2026-74</t>
   </si>
   <si>
@@ -1948,6 +1945,9 @@
     <t>20.22.0001.0052762.2026-72</t>
   </si>
   <si>
+    <t>20.22.0001.0052761.2026-02</t>
+  </si>
+  <si>
     <t>20.22.0001.0052726.2026-74</t>
   </si>
   <si>
@@ -3778,9 +3778,6 @@
     <t>2026.0862</t>
   </si>
   <si>
-    <t>2026.0861</t>
-  </si>
-  <si>
     <t>2026.0869</t>
   </si>
   <si>
@@ -3847,6 +3844,9 @@
     <t>2026.0880</t>
   </si>
   <si>
+    <t>2026.0879</t>
+  </si>
+  <si>
     <t>2026.0878</t>
   </si>
   <si>
@@ -6763,9 +6763,6 @@
     <t>202600352229</t>
   </si>
   <si>
-    <t>202000803701</t>
-  </si>
-  <si>
     <t>202300121607</t>
   </si>
   <si>
@@ -6830,6 +6827,9 @@
   </si>
   <si>
     <t>202501160489</t>
+  </si>
+  <si>
+    <t>201900913020</t>
   </si>
   <si>
     <t>202500416795</t>
@@ -28282,7 +28282,7 @@
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B583" t="s">
         <v>621</v>
@@ -28291,31 +28291,28 @@
         <v>1254</v>
       </c>
       <c r="D583" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="E583">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F583" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="G583" t="s">
-        <v>1536</v>
-      </c>
-      <c r="H583" t="s">
-        <v>1525</v>
+        <v>1535</v>
       </c>
       <c r="I583" t="s">
-        <v>1628</v>
+        <v>1659</v>
       </c>
       <c r="J583" t="s">
         <v>2249</v>
       </c>
       <c r="K583" t="s">
-        <v>2337</v>
+        <v>2375</v>
       </c>
       <c r="L583" t="s">
-        <v>2429</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="584" spans="1:12">
@@ -28347,7 +28344,7 @@
         <v>2250</v>
       </c>
       <c r="K584" t="s">
-        <v>2375</v>
+        <v>2395</v>
       </c>
       <c r="L584" t="s">
         <v>2425</v>
@@ -28355,7 +28352,7 @@
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B585" t="s">
         <v>623</v>
@@ -28370,19 +28367,22 @@
         <v>10</v>
       </c>
       <c r="F585" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="G585" t="s">
-        <v>1535</v>
+        <v>1536</v>
+      </c>
+      <c r="H585" t="s">
+        <v>1548</v>
       </c>
       <c r="I585" t="s">
-        <v>1659</v>
+        <v>1558</v>
       </c>
       <c r="J585" t="s">
         <v>2251</v>
       </c>
       <c r="K585" t="s">
-        <v>2395</v>
+        <v>2318</v>
       </c>
       <c r="L585" t="s">
         <v>2425</v>
@@ -28390,7 +28390,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B586" t="s">
         <v>624</v>
@@ -28411,19 +28411,19 @@
         <v>1536</v>
       </c>
       <c r="H586" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="I586" t="s">
-        <v>1558</v>
+        <v>1666</v>
       </c>
       <c r="J586" t="s">
         <v>2252</v>
       </c>
       <c r="K586" t="s">
-        <v>2318</v>
+        <v>2417</v>
       </c>
       <c r="L586" t="s">
-        <v>2425</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28443,30 +28443,27 @@
         <v>10</v>
       </c>
       <c r="F587" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="G587" t="s">
-        <v>1536</v>
-      </c>
-      <c r="H587" t="s">
-        <v>1549</v>
+        <v>1535</v>
       </c>
       <c r="I587" t="s">
-        <v>1666</v>
+        <v>1598</v>
       </c>
       <c r="J587" t="s">
         <v>2253</v>
       </c>
       <c r="K587" t="s">
-        <v>2417</v>
+        <v>2331</v>
       </c>
       <c r="L587" t="s">
-        <v>2456</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B588" t="s">
         <v>626</v>
@@ -28487,16 +28484,16 @@
         <v>1535</v>
       </c>
       <c r="I588" t="s">
-        <v>1598</v>
+        <v>1606</v>
       </c>
       <c r="J588" t="s">
         <v>2254</v>
       </c>
       <c r="K588" t="s">
-        <v>2331</v>
+        <v>2343</v>
       </c>
       <c r="L588" t="s">
-        <v>2439</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -28522,21 +28519,21 @@
         <v>1535</v>
       </c>
       <c r="I589" t="s">
-        <v>1606</v>
+        <v>1655</v>
       </c>
       <c r="J589" t="s">
         <v>2255</v>
       </c>
       <c r="K589" t="s">
-        <v>2343</v>
+        <v>2337</v>
       </c>
       <c r="L589" t="s">
-        <v>2427</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B590" t="s">
         <v>628</v>
@@ -28545,10 +28542,10 @@
         <v>1261</v>
       </c>
       <c r="D590" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
       <c r="E590">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F590" t="s">
         <v>1531</v>
@@ -28557,16 +28554,16 @@
         <v>1535</v>
       </c>
       <c r="I590" t="s">
-        <v>1655</v>
+        <v>1563</v>
       </c>
       <c r="J590" t="s">
         <v>2256</v>
       </c>
       <c r="K590" t="s">
-        <v>2337</v>
+        <v>2366</v>
       </c>
       <c r="L590" t="s">
-        <v>2484</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="591" spans="1:12">
@@ -28598,7 +28595,7 @@
         <v>2257</v>
       </c>
       <c r="K591" t="s">
-        <v>2366</v>
+        <v>2306</v>
       </c>
       <c r="L591" t="s">
         <v>2439</v>
@@ -28606,7 +28603,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B592" t="s">
         <v>630</v>
@@ -28627,21 +28624,21 @@
         <v>1535</v>
       </c>
       <c r="I592" t="s">
-        <v>1563</v>
+        <v>1655</v>
       </c>
       <c r="J592" t="s">
         <v>2258</v>
       </c>
       <c r="K592" t="s">
-        <v>2306</v>
+        <v>2349</v>
       </c>
       <c r="L592" t="s">
-        <v>2439</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B593" t="s">
         <v>631</v>
@@ -28656,27 +28653,30 @@
         <v>9</v>
       </c>
       <c r="F593" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="G593" t="s">
-        <v>1535</v>
+        <v>1536</v>
+      </c>
+      <c r="H593" t="s">
+        <v>1550</v>
       </c>
       <c r="I593" t="s">
-        <v>1655</v>
+        <v>1638</v>
       </c>
       <c r="J593" t="s">
         <v>2259</v>
       </c>
       <c r="K593" t="s">
-        <v>2349</v>
+        <v>2340</v>
       </c>
       <c r="L593" t="s">
-        <v>2484</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B594" t="s">
         <v>632</v>
@@ -28691,22 +28691,19 @@
         <v>9</v>
       </c>
       <c r="F594" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="G594" t="s">
-        <v>1536</v>
-      </c>
-      <c r="H594" t="s">
-        <v>1550</v>
+        <v>1535</v>
       </c>
       <c r="I594" t="s">
-        <v>1638</v>
+        <v>1659</v>
       </c>
       <c r="J594" t="s">
         <v>2260</v>
       </c>
       <c r="K594" t="s">
-        <v>2340</v>
+        <v>2376</v>
       </c>
       <c r="L594" t="s">
         <v>2425</v>
@@ -28735,16 +28732,16 @@
         <v>1535</v>
       </c>
       <c r="I595" t="s">
-        <v>1659</v>
+        <v>1655</v>
       </c>
       <c r="J595" t="s">
         <v>2261</v>
       </c>
       <c r="K595" t="s">
-        <v>2376</v>
+        <v>2357</v>
       </c>
       <c r="L595" t="s">
-        <v>2425</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -28758,10 +28755,10 @@
         <v>1267</v>
       </c>
       <c r="D596" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="E596">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F596" t="s">
         <v>1531</v>
@@ -28770,21 +28767,21 @@
         <v>1535</v>
       </c>
       <c r="I596" t="s">
-        <v>1655</v>
+        <v>1659</v>
       </c>
       <c r="J596" t="s">
         <v>2262</v>
       </c>
       <c r="K596" t="s">
-        <v>2357</v>
+        <v>2332</v>
       </c>
       <c r="L596" t="s">
-        <v>2484</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B597" t="s">
         <v>635</v>
@@ -28805,21 +28802,21 @@
         <v>1535</v>
       </c>
       <c r="I597" t="s">
-        <v>1659</v>
+        <v>1667</v>
       </c>
       <c r="J597" t="s">
         <v>2263</v>
       </c>
       <c r="K597" t="s">
-        <v>2332</v>
+        <v>2418</v>
       </c>
       <c r="L597" t="s">
-        <v>2425</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B598" t="s">
         <v>636</v>
@@ -28840,21 +28837,21 @@
         <v>1535</v>
       </c>
       <c r="I598" t="s">
-        <v>1667</v>
+        <v>1659</v>
       </c>
       <c r="J598" t="s">
         <v>2264</v>
       </c>
       <c r="K598" t="s">
-        <v>2418</v>
+        <v>2419</v>
       </c>
       <c r="L598" t="s">
-        <v>2477</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B599" t="s">
         <v>637</v>
@@ -28875,21 +28872,21 @@
         <v>1535</v>
       </c>
       <c r="I599" t="s">
-        <v>1659</v>
+        <v>1667</v>
       </c>
       <c r="J599" t="s">
         <v>2265</v>
       </c>
       <c r="K599" t="s">
-        <v>2419</v>
+        <v>2418</v>
       </c>
       <c r="L599" t="s">
-        <v>2425</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B600" t="s">
         <v>638</v>
@@ -28904,27 +28901,27 @@
         <v>8</v>
       </c>
       <c r="F600" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="G600" t="s">
         <v>1535</v>
       </c>
       <c r="I600" t="s">
-        <v>1667</v>
+        <v>1563</v>
       </c>
       <c r="J600" t="s">
         <v>2266</v>
       </c>
       <c r="K600" t="s">
-        <v>2418</v>
+        <v>2419</v>
       </c>
       <c r="L600" t="s">
-        <v>2477</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -28939,27 +28936,27 @@
         <v>8</v>
       </c>
       <c r="F601" t="s">
-        <v>1534</v>
+        <v>1531</v>
       </c>
       <c r="G601" t="s">
         <v>1535</v>
       </c>
       <c r="I601" t="s">
-        <v>1563</v>
+        <v>1659</v>
       </c>
       <c r="J601" t="s">
         <v>2267</v>
       </c>
       <c r="K601" t="s">
-        <v>2419</v>
+        <v>2374</v>
       </c>
       <c r="L601" t="s">
-        <v>2461</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B602" t="s">
         <v>640</v>
@@ -28974,27 +28971,30 @@
         <v>8</v>
       </c>
       <c r="F602" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="G602" t="s">
-        <v>1535</v>
+        <v>1536</v>
+      </c>
+      <c r="H602" t="s">
+        <v>1551</v>
       </c>
       <c r="I602" t="s">
-        <v>1659</v>
+        <v>1590</v>
       </c>
       <c r="J602" t="s">
         <v>2268</v>
       </c>
       <c r="K602" t="s">
-        <v>2374</v>
+        <v>2381</v>
       </c>
       <c r="L602" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B603" t="s">
         <v>641</v>
@@ -29015,24 +29015,24 @@
         <v>1536</v>
       </c>
       <c r="H603" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="I603" t="s">
-        <v>1590</v>
+        <v>1670</v>
       </c>
       <c r="J603" t="s">
         <v>2269</v>
       </c>
       <c r="K603" t="s">
-        <v>2381</v>
+        <v>2331</v>
       </c>
       <c r="L603" t="s">
-        <v>2427</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B604" t="s">
         <v>642</v>
@@ -29047,30 +29047,27 @@
         <v>8</v>
       </c>
       <c r="F604" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="G604" t="s">
-        <v>1536</v>
-      </c>
-      <c r="H604" t="s">
-        <v>1552</v>
+        <v>1535</v>
       </c>
       <c r="I604" t="s">
-        <v>1670</v>
+        <v>1641</v>
       </c>
       <c r="J604" t="s">
         <v>2270</v>
       </c>
       <c r="K604" t="s">
-        <v>2331</v>
+        <v>2313</v>
       </c>
       <c r="L604" t="s">
-        <v>2455</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B605" t="s">
         <v>643</v>
@@ -29091,7 +29088,7 @@
         <v>1535</v>
       </c>
       <c r="I605" t="s">
-        <v>1641</v>
+        <v>1651</v>
       </c>
       <c r="J605" t="s">
         <v>2271</v>
@@ -29100,7 +29097,7 @@
         <v>2313</v>
       </c>
       <c r="L605" t="s">
-        <v>2425</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="606" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-06 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -28058,7 +28058,7 @@
         <v>1547</v>
       </c>
       <c r="I576" t="s">
-        <v>1563</v>
+        <v>1667</v>
       </c>
       <c r="J576" t="s">
         <v>2242</v>
@@ -29919,7 +29919,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B629" t="s">
         <v>667</v>
@@ -29940,7 +29940,7 @@
         <v>1535</v>
       </c>
       <c r="I629" t="s">
-        <v>1563</v>
+        <v>1674</v>
       </c>
       <c r="J629" t="s">
         <v>2294</v>
@@ -29954,7 +29954,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B630" t="s">
         <v>668</v>
@@ -29975,7 +29975,7 @@
         <v>1535</v>
       </c>
       <c r="I630" t="s">
-        <v>1563</v>
+        <v>1674</v>
       </c>
       <c r="J630" t="s">
         <v>2295</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-07 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4795,7 +4795,7 @@
     <t>JORGE LUIS DANTAS BATISTA</t>
   </si>
   <si>
-    <t>CHRISTIANA ROSA FERREIRA, _SEM USUARIO ATRIBUIDO</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, CHRISTIANA ROSA FERREIRA</t>
   </si>
   <si>
     <t>VANESSA FERNANDES LEÃO</t>
@@ -7540,7 +7540,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
@@ -7558,7 +7558,7 @@
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,URBANISMO,SAÚDE MENTAL,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,SAÚDE,ECONOMIA,PSICOLOGIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS</t>
+    <t>URBANISMO,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,SAÚDE,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ORÇAMENTO,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,ECONOMIA</t>
   </si>
 </sst>
 </file>
@@ -29996,7 +29996,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B630" t="s">
         <v>669</v>
@@ -30017,7 +30017,7 @@
         <v>1548</v>
       </c>
       <c r="I630" t="s">
-        <v>1574</v>
+        <v>1653</v>
       </c>
       <c r="J630" t="s">
         <v>2306</v>
@@ -30026,12 +30026,12 @@
         <v>2393</v>
       </c>
       <c r="L630" t="s">
-        <v>2501</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B631" t="s">
         <v>670</v>
@@ -30052,7 +30052,7 @@
         <v>1548</v>
       </c>
       <c r="I631" t="s">
-        <v>1574</v>
+        <v>1618</v>
       </c>
       <c r="J631" t="s">
         <v>2307</v>
@@ -30061,7 +30061,7 @@
         <v>2393</v>
       </c>
       <c r="L631" t="s">
-        <v>2501</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="632" spans="1:12">
@@ -30087,7 +30087,7 @@
         <v>1548</v>
       </c>
       <c r="I632" t="s">
-        <v>1685</v>
+        <v>1670</v>
       </c>
       <c r="J632" t="s">
         <v>2308</v>
@@ -30096,7 +30096,7 @@
         <v>2345</v>
       </c>
       <c r="L632" t="s">
-        <v>2501</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30157,7 +30157,7 @@
         <v>1548</v>
       </c>
       <c r="I634" t="s">
-        <v>1685</v>
+        <v>1653</v>
       </c>
       <c r="J634" t="s">
         <v>2310</v>
@@ -30166,7 +30166,7 @@
         <v>2329</v>
       </c>
       <c r="L634" t="s">
-        <v>2501</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="635" spans="1:12">
@@ -30192,7 +30192,7 @@
         <v>1548</v>
       </c>
       <c r="I635" t="s">
-        <v>1685</v>
+        <v>1607</v>
       </c>
       <c r="J635" t="s">
         <v>2311</v>
@@ -30201,7 +30201,7 @@
         <v>2329</v>
       </c>
       <c r="L635" t="s">
-        <v>2501</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30303,7 +30303,7 @@
         <v>1567</v>
       </c>
       <c r="I638" t="s">
-        <v>1574</v>
+        <v>1682</v>
       </c>
       <c r="J638" t="s">
         <v>2314</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-10 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -112,12 +112,12 @@
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
   </si>
   <si>
@@ -5017,7 +5017,7 @@
     <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
   </si>
   <si>
-    <t>RENATA PASCOAL FREIRE,VICTOR AUGUSTO LOURO BERBARA</t>
+    <t>_SEM USUARIO ATRIBUIDO, VICTOR AUGUSTO LOURO BERBARA</t>
   </si>
   <si>
     <t>CASSIA CRISTINA DA SILVA</t>
@@ -13203,7 +13203,7 @@
     </row>
     <row r="146" spans="1:12">
       <c r="A146" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B146" t="s">
         <v>186</v>
@@ -15481,7 +15481,7 @@
     </row>
     <row r="211" spans="1:12">
       <c r="A211" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B211" t="s">
         <v>251</v>
@@ -15586,7 +15586,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B214" t="s">
         <v>254</v>
@@ -16111,7 +16111,7 @@
     </row>
     <row r="229" spans="1:12">
       <c r="A229" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B229" t="s">
         <v>269</v>
@@ -17021,7 +17021,7 @@
     </row>
     <row r="255" spans="1:12">
       <c r="A255" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B255" t="s">
         <v>295</v>
@@ -17581,7 +17581,7 @@
     </row>
     <row r="271" spans="1:12">
       <c r="A271" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B271" t="s">
         <v>311</v>
@@ -19331,7 +19331,7 @@
     </row>
     <row r="321" spans="1:12">
       <c r="A321" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B321" t="s">
         <v>361</v>
@@ -19544,7 +19544,7 @@
     </row>
     <row r="327" spans="1:12">
       <c r="A327" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B327" t="s">
         <v>367</v>
@@ -19579,7 +19579,7 @@
     </row>
     <row r="328" spans="1:12">
       <c r="A328" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B328" t="s">
         <v>368</v>
@@ -23085,7 +23085,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B428" t="s">
         <v>468</v>
@@ -23820,7 +23820,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B449" t="s">
         <v>489</v>
@@ -26737,7 +26737,7 @@
     </row>
     <row r="532" spans="1:12">
       <c r="A532" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B532" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-10 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4891,6 +4891,9 @@
     <t>DAYSE BARBOSA DE ARAÚJO GÓIS,SERGIO PEDRO LOPES</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
@@ -5017,7 +5020,7 @@
     <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
   </si>
   <si>
-    <t>_SEM USUARIO ATRIBUIDO, VICTOR AUGUSTO LOURO BERBARA</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, VICTOR AUGUSTO LOURO BERBARA</t>
   </si>
   <si>
     <t>CASSIA CRISTINA DA SILVA</t>
@@ -5086,7 +5089,7 @@
     <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
   </si>
   <si>
-    <t>CLAUDIA DA SILVA LUNARDI,SEZISNANDO JOSE PRIMO PAES, _SEM USUARIO ATRIBUIDO</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, CLAUDIA DA SILVA LUNARDI,SEZISNANDO JOSE PRIMO PAES</t>
   </si>
   <si>
     <t>NIVANA DANIELLE SILVA COSTA</t>
@@ -5174,9 +5177,6 @@
   </si>
   <si>
     <t>LEONARDO ARAÚJO DE SOUZA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>DAGER SALLES AMARAL</t>
@@ -9371,7 +9371,7 @@
         <v>1593</v>
       </c>
       <c r="I36" t="s">
-        <v>1618</v>
+        <v>1625</v>
       </c>
       <c r="J36" t="s">
         <v>1761</v>
@@ -9444,7 +9444,7 @@
         <v>1593</v>
       </c>
       <c r="I38" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J38" t="s">
         <v>1763</v>
@@ -9549,7 +9549,7 @@
         <v>1593</v>
       </c>
       <c r="I41" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J41" t="s">
         <v>1766</v>
@@ -9724,7 +9724,7 @@
         <v>1593</v>
       </c>
       <c r="I46" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J46" t="s">
         <v>1770</v>
@@ -9794,7 +9794,7 @@
         <v>1593</v>
       </c>
       <c r="I48" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J48" t="s">
         <v>1772</v>
@@ -9829,7 +9829,7 @@
         <v>1593</v>
       </c>
       <c r="I49" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J49" t="s">
         <v>1773</v>
@@ -9934,7 +9934,7 @@
         <v>1593</v>
       </c>
       <c r="I52" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J52" t="s">
         <v>1776</v>
@@ -9969,7 +9969,7 @@
         <v>1593</v>
       </c>
       <c r="I53" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J53" t="s">
         <v>1777</v>
@@ -10039,7 +10039,7 @@
         <v>1593</v>
       </c>
       <c r="I55" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="J55" t="s">
         <v>1779</v>
@@ -10074,7 +10074,7 @@
         <v>1593</v>
       </c>
       <c r="I56" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J56" t="s">
         <v>1780</v>
@@ -10109,7 +10109,7 @@
         <v>1593</v>
       </c>
       <c r="I57" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="J57" t="s">
         <v>1781</v>
@@ -10179,7 +10179,7 @@
         <v>1593</v>
       </c>
       <c r="I59" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J59" t="s">
         <v>1783</v>
@@ -10249,7 +10249,7 @@
         <v>1593</v>
       </c>
       <c r="I61" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="J61" t="s">
         <v>1785</v>
@@ -10319,7 +10319,7 @@
         <v>1593</v>
       </c>
       <c r="I63" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="J63" t="s">
         <v>1787</v>
@@ -10529,7 +10529,7 @@
         <v>1593</v>
       </c>
       <c r="I69" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="J69" t="s">
         <v>1793</v>
@@ -10564,7 +10564,7 @@
         <v>1593</v>
       </c>
       <c r="I70" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J70" t="s">
         <v>1794</v>
@@ -10669,7 +10669,7 @@
         <v>1593</v>
       </c>
       <c r="I73" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="J73" t="s">
         <v>1796</v>
@@ -10704,7 +10704,7 @@
         <v>1593</v>
       </c>
       <c r="I74" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J74" t="s">
         <v>1797</v>
@@ -10774,7 +10774,7 @@
         <v>1593</v>
       </c>
       <c r="I76" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J76" t="s">
         <v>1799</v>
@@ -10809,7 +10809,7 @@
         <v>1593</v>
       </c>
       <c r="I77" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J77" t="s">
         <v>1800</v>
@@ -10844,7 +10844,7 @@
         <v>1593</v>
       </c>
       <c r="I78" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J78" t="s">
         <v>1801</v>
@@ -10879,7 +10879,7 @@
         <v>1593</v>
       </c>
       <c r="I79" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J79" t="s">
         <v>1802</v>
@@ -10914,7 +10914,7 @@
         <v>1593</v>
       </c>
       <c r="I80" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="J80" t="s">
         <v>1803</v>
@@ -10949,7 +10949,7 @@
         <v>1593</v>
       </c>
       <c r="I81" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J81" t="s">
         <v>1804</v>
@@ -11019,7 +11019,7 @@
         <v>1593</v>
       </c>
       <c r="I83" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J83" t="s">
         <v>1806</v>
@@ -11054,7 +11054,7 @@
         <v>1593</v>
       </c>
       <c r="I84" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="J84" t="s">
         <v>1807</v>
@@ -11089,7 +11089,7 @@
         <v>1593</v>
       </c>
       <c r="I85" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J85" t="s">
         <v>1808</v>
@@ -11124,7 +11124,7 @@
         <v>1593</v>
       </c>
       <c r="I86" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J86" t="s">
         <v>1809</v>
@@ -11229,7 +11229,7 @@
         <v>1593</v>
       </c>
       <c r="I89" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="J89" t="s">
         <v>1812</v>
@@ -11299,7 +11299,7 @@
         <v>1593</v>
       </c>
       <c r="I91" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J91" t="s">
         <v>1814</v>
@@ -11404,7 +11404,7 @@
         <v>1593</v>
       </c>
       <c r="I94" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="J94" t="s">
         <v>1817</v>
@@ -11474,7 +11474,7 @@
         <v>1593</v>
       </c>
       <c r="I96" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J96" t="s">
         <v>1819</v>
@@ -11544,7 +11544,7 @@
         <v>1593</v>
       </c>
       <c r="I98" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J98" t="s">
         <v>1821</v>
@@ -11579,7 +11579,7 @@
         <v>1593</v>
       </c>
       <c r="I99" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J99" t="s">
         <v>1822</v>
@@ -11614,7 +11614,7 @@
         <v>1593</v>
       </c>
       <c r="I100" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J100" t="s">
         <v>1823</v>
@@ -11684,7 +11684,7 @@
         <v>1593</v>
       </c>
       <c r="I102" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J102" t="s">
         <v>1825</v>
@@ -11719,7 +11719,7 @@
         <v>1593</v>
       </c>
       <c r="I103" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J103" t="s">
         <v>1826</v>
@@ -11894,7 +11894,7 @@
         <v>1593</v>
       </c>
       <c r="I108" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J108" t="s">
         <v>1831</v>
@@ -11929,7 +11929,7 @@
         <v>1593</v>
       </c>
       <c r="I109" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J109" t="s">
         <v>1832</v>
@@ -11964,7 +11964,7 @@
         <v>1593</v>
       </c>
       <c r="I110" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J110" t="s">
         <v>1833</v>
@@ -11999,7 +11999,7 @@
         <v>1593</v>
       </c>
       <c r="I111" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J111" t="s">
         <v>1834</v>
@@ -12034,7 +12034,7 @@
         <v>1593</v>
       </c>
       <c r="I112" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J112" t="s">
         <v>1835</v>
@@ -12209,7 +12209,7 @@
         <v>1593</v>
       </c>
       <c r="I117" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J117" t="s">
         <v>1840</v>
@@ -12279,7 +12279,7 @@
         <v>1593</v>
       </c>
       <c r="I119" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J119" t="s">
         <v>1842</v>
@@ -12314,7 +12314,7 @@
         <v>1593</v>
       </c>
       <c r="I120" t="s">
-        <v>1618</v>
+        <v>1625</v>
       </c>
       <c r="J120" t="s">
         <v>1843</v>
@@ -12489,7 +12489,7 @@
         <v>1593</v>
       </c>
       <c r="I125" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J125" t="s">
         <v>1848</v>
@@ -12629,7 +12629,7 @@
         <v>1593</v>
       </c>
       <c r="I129" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J129" t="s">
         <v>1852</v>
@@ -12664,7 +12664,7 @@
         <v>1593</v>
       </c>
       <c r="I130" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J130" t="s">
         <v>1853</v>
@@ -12874,7 +12874,7 @@
         <v>1593</v>
       </c>
       <c r="I136" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J136" t="s">
         <v>1859</v>
@@ -12909,7 +12909,7 @@
         <v>1593</v>
       </c>
       <c r="I137" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J137" t="s">
         <v>1860</v>
@@ -13119,7 +13119,7 @@
         <v>1593</v>
       </c>
       <c r="I143" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J143" t="s">
         <v>1866</v>
@@ -13189,7 +13189,7 @@
         <v>1593</v>
       </c>
       <c r="I145" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J145" t="s">
         <v>1868</v>
@@ -13224,7 +13224,7 @@
         <v>1593</v>
       </c>
       <c r="I146" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J146" t="s">
         <v>1869</v>
@@ -13399,7 +13399,7 @@
         <v>1593</v>
       </c>
       <c r="I151" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J151" t="s">
         <v>1874</v>
@@ -13434,7 +13434,7 @@
         <v>1593</v>
       </c>
       <c r="I152" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J152" t="s">
         <v>1875</v>
@@ -13539,7 +13539,7 @@
         <v>1593</v>
       </c>
       <c r="I155" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J155" t="s">
         <v>1878</v>
@@ -13749,7 +13749,7 @@
         <v>1593</v>
       </c>
       <c r="I161" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="J161" t="s">
         <v>1883</v>
@@ -13784,7 +13784,7 @@
         <v>1593</v>
       </c>
       <c r="I162" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J162" t="s">
         <v>1884</v>
@@ -13854,7 +13854,7 @@
         <v>1593</v>
       </c>
       <c r="I164" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J164" t="s">
         <v>1886</v>
@@ -13994,7 +13994,7 @@
         <v>1593</v>
       </c>
       <c r="I168" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J168" t="s">
         <v>1890</v>
@@ -14064,7 +14064,7 @@
         <v>1593</v>
       </c>
       <c r="I170" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="J170" t="s">
         <v>1892</v>
@@ -14099,7 +14099,7 @@
         <v>1593</v>
       </c>
       <c r="I171" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J171" t="s">
         <v>1893</v>
@@ -14204,7 +14204,7 @@
         <v>1593</v>
       </c>
       <c r="I174" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="J174" t="s">
         <v>1896</v>
@@ -14274,7 +14274,7 @@
         <v>1593</v>
       </c>
       <c r="I176" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="J176" t="s">
         <v>1898</v>
@@ -14344,7 +14344,7 @@
         <v>1593</v>
       </c>
       <c r="I178" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J178" t="s">
         <v>1900</v>
@@ -14379,7 +14379,7 @@
         <v>1593</v>
       </c>
       <c r="I179" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="J179" t="s">
         <v>1901</v>
@@ -14449,7 +14449,7 @@
         <v>1593</v>
       </c>
       <c r="I181" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J181" t="s">
         <v>1903</v>
@@ -14484,7 +14484,7 @@
         <v>1593</v>
       </c>
       <c r="I182" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J182" t="s">
         <v>1904</v>
@@ -14554,7 +14554,7 @@
         <v>1593</v>
       </c>
       <c r="I184" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J184" t="s">
         <v>1906</v>
@@ -14694,7 +14694,7 @@
         <v>1593</v>
       </c>
       <c r="I188" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J188" t="s">
         <v>1910</v>
@@ -14799,7 +14799,7 @@
         <v>1593</v>
       </c>
       <c r="I191" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J191" t="s">
         <v>1913</v>
@@ -14869,7 +14869,7 @@
         <v>1593</v>
       </c>
       <c r="I193" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="J193" t="s">
         <v>1915</v>
@@ -14907,7 +14907,7 @@
         <v>1597</v>
       </c>
       <c r="I194" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J194" t="s">
         <v>1916</v>
@@ -14977,7 +14977,7 @@
         <v>1593</v>
       </c>
       <c r="I196" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J196" t="s">
         <v>1918</v>
@@ -15082,7 +15082,7 @@
         <v>1593</v>
       </c>
       <c r="I199" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J199" t="s">
         <v>1921</v>
@@ -15152,7 +15152,7 @@
         <v>1593</v>
       </c>
       <c r="I201" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J201" t="s">
         <v>1923</v>
@@ -15187,7 +15187,7 @@
         <v>1593</v>
       </c>
       <c r="I202" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J202" t="s">
         <v>1924</v>
@@ -15222,7 +15222,7 @@
         <v>1593</v>
       </c>
       <c r="I203" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J203" t="s">
         <v>1925</v>
@@ -15327,7 +15327,7 @@
         <v>1593</v>
       </c>
       <c r="I206" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="J206" t="s">
         <v>1928</v>
@@ -15362,7 +15362,7 @@
         <v>1593</v>
       </c>
       <c r="I207" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J207" t="s">
         <v>1929</v>
@@ -15397,7 +15397,7 @@
         <v>1593</v>
       </c>
       <c r="I208" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J208" t="s">
         <v>1930</v>
@@ -15432,7 +15432,7 @@
         <v>1593</v>
       </c>
       <c r="I209" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J209" t="s">
         <v>1931</v>
@@ -15467,7 +15467,7 @@
         <v>1593</v>
       </c>
       <c r="I210" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J210" t="s">
         <v>1932</v>
@@ -15607,7 +15607,7 @@
         <v>1593</v>
       </c>
       <c r="I214" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="J214" t="s">
         <v>1936</v>
@@ -15642,7 +15642,7 @@
         <v>1593</v>
       </c>
       <c r="I215" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="J215" t="s">
         <v>1937</v>
@@ -15992,7 +15992,7 @@
         <v>1593</v>
       </c>
       <c r="I225" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="J225" t="s">
         <v>1947</v>
@@ -16622,7 +16622,7 @@
         <v>1593</v>
       </c>
       <c r="I243" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J243" t="s">
         <v>1963</v>
@@ -16692,7 +16692,7 @@
         <v>1593</v>
       </c>
       <c r="I245" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J245" t="s">
         <v>1965</v>
@@ -17007,7 +17007,7 @@
         <v>1593</v>
       </c>
       <c r="I254" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J254" t="s">
         <v>1974</v>
@@ -17077,7 +17077,7 @@
         <v>1593</v>
       </c>
       <c r="I256" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J256" t="s">
         <v>1976</v>
@@ -17147,7 +17147,7 @@
         <v>1593</v>
       </c>
       <c r="I258" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J258" t="s">
         <v>1978</v>
@@ -17217,7 +17217,7 @@
         <v>1593</v>
       </c>
       <c r="I260" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J260" t="s">
         <v>1980</v>
@@ -17427,7 +17427,7 @@
         <v>1593</v>
       </c>
       <c r="I266" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J266" t="s">
         <v>1986</v>
@@ -17497,7 +17497,7 @@
         <v>1593</v>
       </c>
       <c r="I268" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="J268" t="s">
         <v>1988</v>
@@ -17567,7 +17567,7 @@
         <v>1593</v>
       </c>
       <c r="I270" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J270" t="s">
         <v>1990</v>
@@ -17882,7 +17882,7 @@
         <v>1593</v>
       </c>
       <c r="I279" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J279" t="s">
         <v>1999</v>
@@ -17917,7 +17917,7 @@
         <v>1593</v>
       </c>
       <c r="I280" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J280" t="s">
         <v>2000</v>
@@ -17987,7 +17987,7 @@
         <v>1593</v>
       </c>
       <c r="I282" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J282" t="s">
         <v>2002</v>
@@ -18232,7 +18232,7 @@
         <v>1593</v>
       </c>
       <c r="I289" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J289" t="s">
         <v>2009</v>
@@ -18407,7 +18407,7 @@
         <v>1593</v>
       </c>
       <c r="I294" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J294" t="s">
         <v>2014</v>
@@ -18547,7 +18547,7 @@
         <v>1593</v>
       </c>
       <c r="I298" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="J298" t="s">
         <v>2018</v>
@@ -18582,7 +18582,7 @@
         <v>1593</v>
       </c>
       <c r="I299" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J299" t="s">
         <v>2019</v>
@@ -18792,7 +18792,7 @@
         <v>1593</v>
       </c>
       <c r="I305" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J305" t="s">
         <v>2025</v>
@@ -18862,7 +18862,7 @@
         <v>1593</v>
       </c>
       <c r="I307" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J307" t="s">
         <v>2027</v>
@@ -18897,7 +18897,7 @@
         <v>1593</v>
       </c>
       <c r="I308" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J308" t="s">
         <v>2028</v>
@@ -19072,7 +19072,7 @@
         <v>1593</v>
       </c>
       <c r="I313" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J313" t="s">
         <v>2033</v>
@@ -19107,7 +19107,7 @@
         <v>1593</v>
       </c>
       <c r="I314" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J314" t="s">
         <v>2034</v>
@@ -19121,7 +19121,7 @@
     </row>
     <row r="315" spans="1:12">
       <c r="A315" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B315" t="s">
         <v>355</v>
@@ -19142,7 +19142,7 @@
         <v>1593</v>
       </c>
       <c r="I315" t="s">
-        <v>1618</v>
+        <v>1625</v>
       </c>
       <c r="J315" t="s">
         <v>2035</v>
@@ -19247,7 +19247,7 @@
         <v>1593</v>
       </c>
       <c r="I318" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J318" t="s">
         <v>2038</v>
@@ -19317,7 +19317,7 @@
         <v>1593</v>
       </c>
       <c r="I320" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J320" t="s">
         <v>2040</v>
@@ -19387,7 +19387,7 @@
         <v>1593</v>
       </c>
       <c r="I322" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="J322" t="s">
         <v>2042</v>
@@ -19457,7 +19457,7 @@
         <v>1593</v>
       </c>
       <c r="I324" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="J324" t="s">
         <v>2044</v>
@@ -19495,7 +19495,7 @@
         <v>1598</v>
       </c>
       <c r="I325" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J325" t="s">
         <v>2045</v>
@@ -19845,7 +19845,7 @@
         <v>1593</v>
       </c>
       <c r="I335" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J335" t="s">
         <v>2055</v>
@@ -19880,7 +19880,7 @@
         <v>1593</v>
       </c>
       <c r="I336" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J336" t="s">
         <v>2056</v>
@@ -19915,7 +19915,7 @@
         <v>1593</v>
       </c>
       <c r="I337" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="J337" t="s">
         <v>2057</v>
@@ -19950,7 +19950,7 @@
         <v>1593</v>
       </c>
       <c r="I338" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J338" t="s">
         <v>2058</v>
@@ -19985,7 +19985,7 @@
         <v>1593</v>
       </c>
       <c r="I339" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J339" t="s">
         <v>2059</v>
@@ -20020,7 +20020,7 @@
         <v>1593</v>
       </c>
       <c r="I340" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J340" t="s">
         <v>2060</v>
@@ -20125,7 +20125,7 @@
         <v>1593</v>
       </c>
       <c r="I343" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J343" t="s">
         <v>2063</v>
@@ -20160,7 +20160,7 @@
         <v>1593</v>
       </c>
       <c r="I344" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="J344" t="s">
         <v>2064</v>
@@ -20230,7 +20230,7 @@
         <v>1593</v>
       </c>
       <c r="I346" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J346" t="s">
         <v>2066</v>
@@ -20440,7 +20440,7 @@
         <v>1593</v>
       </c>
       <c r="I352" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J352" t="s">
         <v>2072</v>
@@ -20475,7 +20475,7 @@
         <v>1593</v>
       </c>
       <c r="I353" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J353" t="s">
         <v>2073</v>
@@ -20580,7 +20580,7 @@
         <v>1593</v>
       </c>
       <c r="I356" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="J356" t="s">
         <v>2076</v>
@@ -20615,7 +20615,7 @@
         <v>1593</v>
       </c>
       <c r="I357" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J357" t="s">
         <v>2077</v>
@@ -20685,7 +20685,7 @@
         <v>1593</v>
       </c>
       <c r="I359" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J359" t="s">
         <v>2079</v>
@@ -20755,7 +20755,7 @@
         <v>1593</v>
       </c>
       <c r="I361" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J361" t="s">
         <v>2081</v>
@@ -20790,7 +20790,7 @@
         <v>1593</v>
       </c>
       <c r="I362" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J362" t="s">
         <v>2082</v>
@@ -20825,7 +20825,7 @@
         <v>1593</v>
       </c>
       <c r="I363" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="J363" t="s">
         <v>2083</v>
@@ -21000,7 +21000,7 @@
         <v>1593</v>
       </c>
       <c r="I368" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J368" t="s">
         <v>2088</v>
@@ -21035,7 +21035,7 @@
         <v>1593</v>
       </c>
       <c r="I369" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J369" t="s">
         <v>2089</v>
@@ -21143,7 +21143,7 @@
         <v>1593</v>
       </c>
       <c r="I372" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J372" t="s">
         <v>2092</v>
@@ -21213,7 +21213,7 @@
         <v>1593</v>
       </c>
       <c r="I374" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J374" t="s">
         <v>2094</v>
@@ -21251,7 +21251,7 @@
         <v>1599</v>
       </c>
       <c r="I375" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J375" t="s">
         <v>2095</v>
@@ -21426,7 +21426,7 @@
         <v>1593</v>
       </c>
       <c r="I380" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J380" t="s">
         <v>2100</v>
@@ -21461,7 +21461,7 @@
         <v>1593</v>
       </c>
       <c r="I381" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J381" t="s">
         <v>2101</v>
@@ -21496,7 +21496,7 @@
         <v>1593</v>
       </c>
       <c r="I382" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J382" t="s">
         <v>2102</v>
@@ -21636,7 +21636,7 @@
         <v>1593</v>
       </c>
       <c r="I386" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J386" t="s">
         <v>2106</v>
@@ -21741,7 +21741,7 @@
         <v>1593</v>
       </c>
       <c r="I389" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J389" t="s">
         <v>2109</v>
@@ -21776,7 +21776,7 @@
         <v>1593</v>
       </c>
       <c r="I390" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J390" t="s">
         <v>2110</v>
@@ -22056,7 +22056,7 @@
         <v>1593</v>
       </c>
       <c r="I398" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J398" t="s">
         <v>2118</v>
@@ -22231,7 +22231,7 @@
         <v>1593</v>
       </c>
       <c r="I403" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="J403" t="s">
         <v>2123</v>
@@ -22266,7 +22266,7 @@
         <v>1593</v>
       </c>
       <c r="I404" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J404" t="s">
         <v>2124</v>
@@ -22336,7 +22336,7 @@
         <v>1593</v>
       </c>
       <c r="I406" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J406" t="s">
         <v>2126</v>
@@ -22406,7 +22406,7 @@
         <v>1593</v>
       </c>
       <c r="I408" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J408" t="s">
         <v>2128</v>
@@ -22476,7 +22476,7 @@
         <v>1593</v>
       </c>
       <c r="I410" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J410" t="s">
         <v>2130</v>
@@ -22511,7 +22511,7 @@
         <v>1593</v>
       </c>
       <c r="I411" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J411" t="s">
         <v>2131</v>
@@ -22791,7 +22791,7 @@
         <v>1593</v>
       </c>
       <c r="I419" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J419" t="s">
         <v>2139</v>
@@ -22826,7 +22826,7 @@
         <v>1593</v>
       </c>
       <c r="I420" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J420" t="s">
         <v>2140</v>
@@ -22861,7 +22861,7 @@
         <v>1593</v>
       </c>
       <c r="I421" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J421" t="s">
         <v>2141</v>
@@ -22896,7 +22896,7 @@
         <v>1593</v>
       </c>
       <c r="I422" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J422" t="s">
         <v>2142</v>
@@ -22966,7 +22966,7 @@
         <v>1593</v>
       </c>
       <c r="I424" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J424" t="s">
         <v>2144</v>
@@ -23071,7 +23071,7 @@
         <v>1593</v>
       </c>
       <c r="I427" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J427" t="s">
         <v>2147</v>
@@ -23246,7 +23246,7 @@
         <v>1593</v>
       </c>
       <c r="I432" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J432" t="s">
         <v>2152</v>
@@ -23316,7 +23316,7 @@
         <v>1593</v>
       </c>
       <c r="I434" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J434" t="s">
         <v>2154</v>
@@ -23421,7 +23421,7 @@
         <v>1593</v>
       </c>
       <c r="I437" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J437" t="s">
         <v>2157</v>
@@ -23526,7 +23526,7 @@
         <v>1593</v>
       </c>
       <c r="I440" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J440" t="s">
         <v>2160</v>
@@ -23561,7 +23561,7 @@
         <v>1593</v>
       </c>
       <c r="I441" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J441" t="s">
         <v>2161</v>
@@ -23596,7 +23596,7 @@
         <v>1593</v>
       </c>
       <c r="I442" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J442" t="s">
         <v>2162</v>
@@ -23631,7 +23631,7 @@
         <v>1593</v>
       </c>
       <c r="I443" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J443" t="s">
         <v>2163</v>
@@ -23701,7 +23701,7 @@
         <v>1593</v>
       </c>
       <c r="I445" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J445" t="s">
         <v>2165</v>
@@ -23911,7 +23911,7 @@
         <v>1593</v>
       </c>
       <c r="I451" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J451" t="s">
         <v>2171</v>
@@ -24121,7 +24121,7 @@
         <v>1593</v>
       </c>
       <c r="I457" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J457" t="s">
         <v>2177</v>
@@ -24156,7 +24156,7 @@
         <v>1593</v>
       </c>
       <c r="I458" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J458" t="s">
         <v>2178</v>
@@ -24191,7 +24191,7 @@
         <v>1593</v>
       </c>
       <c r="I459" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J459" t="s">
         <v>2179</v>
@@ -24264,7 +24264,7 @@
         <v>1570</v>
       </c>
       <c r="I461" t="s">
-        <v>1629</v>
+        <v>1673</v>
       </c>
       <c r="J461" t="s">
         <v>2181</v>
@@ -24369,7 +24369,7 @@
         <v>1593</v>
       </c>
       <c r="I464" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J464" t="s">
         <v>2184</v>
@@ -24404,7 +24404,7 @@
         <v>1593</v>
       </c>
       <c r="I465" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J465" t="s">
         <v>2185</v>
@@ -24439,7 +24439,7 @@
         <v>1593</v>
       </c>
       <c r="I466" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J466" t="s">
         <v>2186</v>
@@ -24477,7 +24477,7 @@
         <v>1600</v>
       </c>
       <c r="I467" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J467" t="s">
         <v>2187</v>
@@ -24617,7 +24617,7 @@
         <v>1593</v>
       </c>
       <c r="I471" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J471" t="s">
         <v>2191</v>
@@ -24757,7 +24757,7 @@
         <v>1593</v>
       </c>
       <c r="I475" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J475" t="s">
         <v>2195</v>
@@ -24827,7 +24827,7 @@
         <v>1593</v>
       </c>
       <c r="I477" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J477" t="s">
         <v>2197</v>
@@ -24897,7 +24897,7 @@
         <v>1593</v>
       </c>
       <c r="I479" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J479" t="s">
         <v>2199</v>
@@ -25002,7 +25002,7 @@
         <v>1593</v>
       </c>
       <c r="I482" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J482" t="s">
         <v>2202</v>
@@ -25037,7 +25037,7 @@
         <v>1593</v>
       </c>
       <c r="I483" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J483" t="s">
         <v>2203</v>
@@ -25072,7 +25072,7 @@
         <v>1593</v>
       </c>
       <c r="I484" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J484" t="s">
         <v>2204</v>
@@ -25107,7 +25107,7 @@
         <v>1593</v>
       </c>
       <c r="I485" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J485" t="s">
         <v>2205</v>
@@ -25177,7 +25177,7 @@
         <v>1593</v>
       </c>
       <c r="I487" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J487" t="s">
         <v>2207</v>
@@ -25212,7 +25212,7 @@
         <v>1593</v>
       </c>
       <c r="I488" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J488" t="s">
         <v>2208</v>
@@ -25247,7 +25247,7 @@
         <v>1593</v>
       </c>
       <c r="I489" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J489" t="s">
         <v>2209</v>
@@ -25282,7 +25282,7 @@
         <v>1593</v>
       </c>
       <c r="I490" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J490" t="s">
         <v>2210</v>
@@ -25317,7 +25317,7 @@
         <v>1593</v>
       </c>
       <c r="I491" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J491" t="s">
         <v>2211</v>
@@ -25352,7 +25352,7 @@
         <v>1593</v>
       </c>
       <c r="I492" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J492" t="s">
         <v>2212</v>
@@ -25387,7 +25387,7 @@
         <v>1593</v>
       </c>
       <c r="I493" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J493" t="s">
         <v>2213</v>
@@ -25422,7 +25422,7 @@
         <v>1593</v>
       </c>
       <c r="I494" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J494" t="s">
         <v>2214</v>
@@ -25460,7 +25460,7 @@
         <v>1601</v>
       </c>
       <c r="I495" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J495" t="s">
         <v>2215</v>
@@ -25495,7 +25495,7 @@
         <v>1593</v>
       </c>
       <c r="I496" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J496" t="s">
         <v>2216</v>
@@ -25530,7 +25530,7 @@
         <v>1593</v>
       </c>
       <c r="I497" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J497" t="s">
         <v>2217</v>
@@ -25565,7 +25565,7 @@
         <v>1593</v>
       </c>
       <c r="I498" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J498" t="s">
         <v>2218</v>
@@ -25600,7 +25600,7 @@
         <v>1593</v>
       </c>
       <c r="I499" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J499" t="s">
         <v>2219</v>
@@ -25635,7 +25635,7 @@
         <v>1593</v>
       </c>
       <c r="I500" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J500" t="s">
         <v>2220</v>
@@ -25670,7 +25670,7 @@
         <v>1593</v>
       </c>
       <c r="I501" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J501" t="s">
         <v>2221</v>
@@ -25705,7 +25705,7 @@
         <v>1593</v>
       </c>
       <c r="I502" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J502" t="s">
         <v>2222</v>
@@ -25740,7 +25740,7 @@
         <v>1593</v>
       </c>
       <c r="I503" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J503" t="s">
         <v>2223</v>
@@ -25775,7 +25775,7 @@
         <v>1593</v>
       </c>
       <c r="I504" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J504" t="s">
         <v>2224</v>
@@ -25810,7 +25810,7 @@
         <v>1593</v>
       </c>
       <c r="I505" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J505" t="s">
         <v>2225</v>
@@ -25845,7 +25845,7 @@
         <v>1593</v>
       </c>
       <c r="I506" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J506" t="s">
         <v>2226</v>
@@ -25880,7 +25880,7 @@
         <v>1593</v>
       </c>
       <c r="I507" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J507" t="s">
         <v>2227</v>
@@ -25915,7 +25915,7 @@
         <v>1593</v>
       </c>
       <c r="I508" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J508" t="s">
         <v>2228</v>
@@ -25985,7 +25985,7 @@
         <v>1593</v>
       </c>
       <c r="I510" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J510" t="s">
         <v>2230</v>
@@ -26020,7 +26020,7 @@
         <v>1593</v>
       </c>
       <c r="I511" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J511" t="s">
         <v>2231</v>
@@ -26055,7 +26055,7 @@
         <v>1593</v>
       </c>
       <c r="I512" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J512" t="s">
         <v>2232</v>
@@ -26090,7 +26090,7 @@
         <v>1593</v>
       </c>
       <c r="I513" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J513" t="s">
         <v>2233</v>
@@ -26125,7 +26125,7 @@
         <v>1593</v>
       </c>
       <c r="I514" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J514" t="s">
         <v>2234</v>
@@ -26160,7 +26160,7 @@
         <v>1593</v>
       </c>
       <c r="I515" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J515" t="s">
         <v>2235</v>
@@ -26265,7 +26265,7 @@
         <v>1593</v>
       </c>
       <c r="I518" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J518" t="s">
         <v>2238</v>
@@ -26303,7 +26303,7 @@
         <v>1602</v>
       </c>
       <c r="I519" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J519" t="s">
         <v>2239</v>
@@ -26408,7 +26408,7 @@
         <v>1595</v>
       </c>
       <c r="I522" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J522" t="s">
         <v>2242</v>
@@ -26443,7 +26443,7 @@
         <v>1593</v>
       </c>
       <c r="I523" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J523" t="s">
         <v>2243</v>
@@ -26513,7 +26513,7 @@
         <v>1593</v>
       </c>
       <c r="I525" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J525" t="s">
         <v>2245</v>
@@ -26653,7 +26653,7 @@
         <v>1593</v>
       </c>
       <c r="I529" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J529" t="s">
         <v>2249</v>
@@ -26688,7 +26688,7 @@
         <v>1593</v>
       </c>
       <c r="I530" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J530" t="s">
         <v>2250</v>
@@ -26723,7 +26723,7 @@
         <v>1593</v>
       </c>
       <c r="I531" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J531" t="s">
         <v>2251</v>
@@ -26793,7 +26793,7 @@
         <v>1593</v>
       </c>
       <c r="I533" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J533" t="s">
         <v>2253</v>
@@ -26898,7 +26898,7 @@
         <v>1593</v>
       </c>
       <c r="I536" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J536" t="s">
         <v>2255</v>
@@ -26933,7 +26933,7 @@
         <v>1593</v>
       </c>
       <c r="I537" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J537" t="s">
         <v>2256</v>
@@ -26968,7 +26968,7 @@
         <v>1593</v>
       </c>
       <c r="I538" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J538" t="s">
         <v>2257</v>
@@ -27006,7 +27006,7 @@
         <v>1603</v>
       </c>
       <c r="I539" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J539" t="s">
         <v>2258</v>
@@ -27041,7 +27041,7 @@
         <v>1593</v>
       </c>
       <c r="I540" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J540" t="s">
         <v>2259</v>
@@ -27076,7 +27076,7 @@
         <v>1593</v>
       </c>
       <c r="I541" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J541" t="s">
         <v>2259</v>
@@ -27111,7 +27111,7 @@
         <v>1593</v>
       </c>
       <c r="I542" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J542" t="s">
         <v>2260</v>
@@ -27146,7 +27146,7 @@
         <v>1593</v>
       </c>
       <c r="I543" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J543" t="s">
         <v>2261</v>
@@ -27181,7 +27181,7 @@
         <v>1593</v>
       </c>
       <c r="I544" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J544" t="s">
         <v>2262</v>
@@ -27216,7 +27216,7 @@
         <v>1593</v>
       </c>
       <c r="I545" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J545" t="s">
         <v>2263</v>
@@ -27356,7 +27356,7 @@
         <v>1593</v>
       </c>
       <c r="I549" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J549" t="s">
         <v>2267</v>
@@ -27391,7 +27391,7 @@
         <v>1593</v>
       </c>
       <c r="I550" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J550" t="s">
         <v>2268</v>
@@ -27426,7 +27426,7 @@
         <v>1593</v>
       </c>
       <c r="I551" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J551" t="s">
         <v>2269</v>
@@ -27566,7 +27566,7 @@
         <v>1593</v>
       </c>
       <c r="I555" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J555" t="s">
         <v>2273</v>
@@ -27601,7 +27601,7 @@
         <v>1593</v>
       </c>
       <c r="I556" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J556" t="s">
         <v>2274</v>
@@ -27671,7 +27671,7 @@
         <v>1593</v>
       </c>
       <c r="I558" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J558" t="s">
         <v>2276</v>
@@ -27706,7 +27706,7 @@
         <v>1593</v>
       </c>
       <c r="I559" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J559" t="s">
         <v>2277</v>
@@ -27741,7 +27741,7 @@
         <v>1593</v>
       </c>
       <c r="I560" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J560" t="s">
         <v>2278</v>
@@ -27811,7 +27811,7 @@
         <v>1593</v>
       </c>
       <c r="I562" t="s">
-        <v>1720</v>
+        <v>1625</v>
       </c>
       <c r="J562" t="s">
         <v>2280</v>
@@ -27849,7 +27849,7 @@
         <v>1604</v>
       </c>
       <c r="I563" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J563" t="s">
         <v>2281</v>
@@ -27919,7 +27919,7 @@
         <v>1593</v>
       </c>
       <c r="I565" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J565" t="s">
         <v>2283</v>
@@ -27954,7 +27954,7 @@
         <v>1593</v>
       </c>
       <c r="I566" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J566" t="s">
         <v>2284</v>
@@ -27989,7 +27989,7 @@
         <v>1593</v>
       </c>
       <c r="I567" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J567" t="s">
         <v>2285</v>
@@ -28024,7 +28024,7 @@
         <v>1593</v>
       </c>
       <c r="I568" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J568" t="s">
         <v>2286</v>
@@ -28059,7 +28059,7 @@
         <v>1593</v>
       </c>
       <c r="I569" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J569" t="s">
         <v>2287</v>
@@ -28129,7 +28129,7 @@
         <v>1593</v>
       </c>
       <c r="I571" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J571" t="s">
         <v>2289</v>
@@ -28164,7 +28164,7 @@
         <v>1593</v>
       </c>
       <c r="I572" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J572" t="s">
         <v>2290</v>
@@ -28199,7 +28199,7 @@
         <v>1593</v>
       </c>
       <c r="I573" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J573" t="s">
         <v>2291</v>
@@ -28234,7 +28234,7 @@
         <v>1593</v>
       </c>
       <c r="I574" t="s">
-        <v>1720</v>
+        <v>1625</v>
       </c>
       <c r="J574" t="s">
         <v>2292</v>
@@ -28269,7 +28269,7 @@
         <v>1593</v>
       </c>
       <c r="I575" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J575" t="s">
         <v>2293</v>
@@ -28304,7 +28304,7 @@
         <v>1593</v>
       </c>
       <c r="I576" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J576" t="s">
         <v>2294</v>
@@ -28339,7 +28339,7 @@
         <v>1593</v>
       </c>
       <c r="I577" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J577" t="s">
         <v>2295</v>
@@ -28412,7 +28412,7 @@
         <v>1593</v>
       </c>
       <c r="I579" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J579" t="s">
         <v>2297</v>
@@ -28447,7 +28447,7 @@
         <v>1593</v>
       </c>
       <c r="I580" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J580" t="s">
         <v>2298</v>
@@ -28482,7 +28482,7 @@
         <v>1593</v>
       </c>
       <c r="I581" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J581" t="s">
         <v>2299</v>
@@ -28587,7 +28587,7 @@
         <v>1593</v>
       </c>
       <c r="I584" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J584" t="s">
         <v>2302</v>
@@ -28622,7 +28622,7 @@
         <v>1593</v>
       </c>
       <c r="I585" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J585" t="s">
         <v>2303</v>
@@ -28657,7 +28657,7 @@
         <v>1593</v>
       </c>
       <c r="I586" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J586" t="s">
         <v>2304</v>
@@ -28692,7 +28692,7 @@
         <v>1593</v>
       </c>
       <c r="I587" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J587" t="s">
         <v>2305</v>
@@ -28727,7 +28727,7 @@
         <v>1593</v>
       </c>
       <c r="I588" t="s">
-        <v>1720</v>
+        <v>1625</v>
       </c>
       <c r="J588" t="s">
         <v>2306</v>
@@ -28762,7 +28762,7 @@
         <v>1593</v>
       </c>
       <c r="I589" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J589" t="s">
         <v>2307</v>
@@ -28797,7 +28797,7 @@
         <v>1593</v>
       </c>
       <c r="I590" t="s">
-        <v>1720</v>
+        <v>1625</v>
       </c>
       <c r="J590" t="s">
         <v>2308</v>
@@ -28867,7 +28867,7 @@
         <v>1593</v>
       </c>
       <c r="I592" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J592" t="s">
         <v>2310</v>
@@ -28905,7 +28905,7 @@
         <v>1606</v>
       </c>
       <c r="I593" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J593" t="s">
         <v>2311</v>
@@ -28940,7 +28940,7 @@
         <v>1593</v>
       </c>
       <c r="I594" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J594" t="s">
         <v>2312</v>
@@ -28975,7 +28975,7 @@
         <v>1593</v>
       </c>
       <c r="I595" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J595" t="s">
         <v>2313</v>
@@ -29010,7 +29010,7 @@
         <v>1593</v>
       </c>
       <c r="I596" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J596" t="s">
         <v>2314</v>
@@ -29045,7 +29045,7 @@
         <v>1593</v>
       </c>
       <c r="I597" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J597" t="s">
         <v>2315</v>
@@ -29080,7 +29080,7 @@
         <v>1593</v>
       </c>
       <c r="I598" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J598" t="s">
         <v>2316</v>
@@ -29115,7 +29115,7 @@
         <v>1593</v>
       </c>
       <c r="I599" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J599" t="s">
         <v>2317</v>
@@ -29150,7 +29150,7 @@
         <v>1593</v>
       </c>
       <c r="I600" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J600" t="s">
         <v>2274</v>
@@ -29185,7 +29185,7 @@
         <v>1593</v>
       </c>
       <c r="I601" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J601" t="s">
         <v>2318</v>
@@ -29223,7 +29223,7 @@
         <v>1607</v>
       </c>
       <c r="I602" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J602" t="s">
         <v>2319</v>
@@ -29258,7 +29258,7 @@
         <v>1593</v>
       </c>
       <c r="I603" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J603" t="s">
         <v>2320</v>
@@ -29293,7 +29293,7 @@
         <v>1593</v>
       </c>
       <c r="I604" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J604" t="s">
         <v>2321</v>
@@ -29404,7 +29404,7 @@
         <v>1609</v>
       </c>
       <c r="I607" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J607" t="s">
         <v>2324</v>
@@ -29509,7 +29509,7 @@
         <v>1593</v>
       </c>
       <c r="I610" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J610" t="s">
         <v>2327</v>
@@ -29544,7 +29544,7 @@
         <v>1593</v>
       </c>
       <c r="I611" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J611" t="s">
         <v>2328</v>
@@ -29579,7 +29579,7 @@
         <v>1593</v>
       </c>
       <c r="I612" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J612" t="s">
         <v>2329</v>
@@ -29617,7 +29617,7 @@
         <v>1610</v>
       </c>
       <c r="I613" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J613" t="s">
         <v>2330</v>
@@ -29652,7 +29652,7 @@
         <v>1593</v>
       </c>
       <c r="I614" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J614" t="s">
         <v>2331</v>
@@ -29687,7 +29687,7 @@
         <v>1593</v>
       </c>
       <c r="I615" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J615" t="s">
         <v>2332</v>
@@ -29722,7 +29722,7 @@
         <v>1593</v>
       </c>
       <c r="I616" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J616" t="s">
         <v>2333</v>
@@ -29757,7 +29757,7 @@
         <v>1593</v>
       </c>
       <c r="I617" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J617" t="s">
         <v>2334</v>
@@ -29792,7 +29792,7 @@
         <v>1593</v>
       </c>
       <c r="I618" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J618" t="s">
         <v>2335</v>
@@ -29827,7 +29827,7 @@
         <v>1593</v>
       </c>
       <c r="I619" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J619" t="s">
         <v>2336</v>
@@ -29876,7 +29876,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B621" t="s">
         <v>660</v>
@@ -29897,7 +29897,7 @@
         <v>1593</v>
       </c>
       <c r="I621" t="s">
-        <v>1659</v>
+        <v>1669</v>
       </c>
       <c r="J621" t="s">
         <v>2338</v>
@@ -29932,7 +29932,7 @@
         <v>1593</v>
       </c>
       <c r="I622" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J622" t="s">
         <v>2339</v>
@@ -29967,7 +29967,7 @@
         <v>1593</v>
       </c>
       <c r="I623" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J623" t="s">
         <v>2340</v>
@@ -30002,7 +30002,7 @@
         <v>1593</v>
       </c>
       <c r="I624" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J624" t="s">
         <v>2341</v>
@@ -30037,7 +30037,7 @@
         <v>1593</v>
       </c>
       <c r="I625" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J625" t="s">
         <v>2342</v>
@@ -30072,7 +30072,7 @@
         <v>1593</v>
       </c>
       <c r="I626" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J626" t="s">
         <v>2343</v>
@@ -30107,7 +30107,7 @@
         <v>1593</v>
       </c>
       <c r="I627" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J627" t="s">
         <v>2344</v>
@@ -30142,7 +30142,7 @@
         <v>1593</v>
       </c>
       <c r="I628" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J628" t="s">
         <v>2345</v>
@@ -30177,7 +30177,7 @@
         <v>1593</v>
       </c>
       <c r="I629" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J629" t="s">
         <v>2346</v>
@@ -30250,7 +30250,7 @@
         <v>1593</v>
       </c>
       <c r="I631" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J631" t="s">
         <v>2348</v>
@@ -30285,7 +30285,7 @@
         <v>1593</v>
       </c>
       <c r="I632" t="s">
-        <v>1720</v>
+        <v>1625</v>
       </c>
       <c r="J632" t="s">
         <v>2349</v>
@@ -30299,7 +30299,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B633" t="s">
         <v>672</v>
@@ -30320,7 +30320,7 @@
         <v>1593</v>
       </c>
       <c r="I633" t="s">
-        <v>1618</v>
+        <v>1713</v>
       </c>
       <c r="J633" t="s">
         <v>2350</v>
@@ -30334,7 +30334,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B634" t="s">
         <v>673</v>
@@ -30355,7 +30355,7 @@
         <v>1593</v>
       </c>
       <c r="I634" t="s">
-        <v>1618</v>
+        <v>1725</v>
       </c>
       <c r="J634" t="s">
         <v>2351</v>
@@ -30369,7 +30369,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B635" t="s">
         <v>674</v>
@@ -30390,7 +30390,7 @@
         <v>1593</v>
       </c>
       <c r="I635" t="s">
-        <v>1618</v>
+        <v>1725</v>
       </c>
       <c r="J635" t="s">
         <v>2352</v>
@@ -30404,7 +30404,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B636" t="s">
         <v>675</v>
@@ -30425,7 +30425,7 @@
         <v>1593</v>
       </c>
       <c r="I636" t="s">
-        <v>1618</v>
+        <v>1725</v>
       </c>
       <c r="J636" t="s">
         <v>2353</v>
@@ -30439,7 +30439,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B637" t="s">
         <v>676</v>
@@ -30460,7 +30460,7 @@
         <v>1593</v>
       </c>
       <c r="I637" t="s">
-        <v>1618</v>
+        <v>1725</v>
       </c>
       <c r="J637" t="s">
         <v>2354</v>
@@ -30474,7 +30474,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B638" t="s">
         <v>677</v>
@@ -30495,7 +30495,7 @@
         <v>1593</v>
       </c>
       <c r="I638" t="s">
-        <v>1618</v>
+        <v>1725</v>
       </c>
       <c r="J638" t="s">
         <v>2355</v>
@@ -30530,7 +30530,7 @@
         <v>1593</v>
       </c>
       <c r="I639" t="s">
-        <v>1618</v>
+        <v>1723</v>
       </c>
       <c r="J639" t="s">
         <v>2356</v>
@@ -30565,7 +30565,7 @@
         <v>1593</v>
       </c>
       <c r="I640" t="s">
-        <v>1618</v>
+        <v>1723</v>
       </c>
       <c r="J640" t="s">
         <v>2357</v>
@@ -30600,7 +30600,7 @@
         <v>1593</v>
       </c>
       <c r="I641" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J641" t="s">
         <v>2358</v>
@@ -30635,7 +30635,7 @@
         <v>1593</v>
       </c>
       <c r="I642" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J642" t="s">
         <v>2359</v>
@@ -30670,7 +30670,7 @@
         <v>1593</v>
       </c>
       <c r="I643" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J643" t="s">
         <v>2360</v>
@@ -30705,7 +30705,7 @@
         <v>1593</v>
       </c>
       <c r="I644" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J644" t="s">
         <v>2361</v>
@@ -30740,7 +30740,7 @@
         <v>1593</v>
       </c>
       <c r="I645" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J645" t="s">
         <v>2362</v>
@@ -30775,7 +30775,7 @@
         <v>1593</v>
       </c>
       <c r="I646" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J646" t="s">
         <v>2363</v>
@@ -30810,7 +30810,7 @@
         <v>1593</v>
       </c>
       <c r="I647" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J647" t="s">
         <v>2364</v>
@@ -30845,7 +30845,7 @@
         <v>1593</v>
       </c>
       <c r="I648" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J648" t="s">
         <v>2365</v>
@@ -30880,7 +30880,7 @@
         <v>1593</v>
       </c>
       <c r="I649" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J649" t="s">
         <v>2366</v>
@@ -30915,7 +30915,7 @@
         <v>1593</v>
       </c>
       <c r="I650" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J650" t="s">
         <v>2367</v>
@@ -30950,7 +30950,7 @@
         <v>1593</v>
       </c>
       <c r="I651" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J651" t="s">
         <v>2368</v>
@@ -30985,7 +30985,7 @@
         <v>1593</v>
       </c>
       <c r="I652" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J652" t="s">
         <v>2369</v>
@@ -31020,7 +31020,7 @@
         <v>1593</v>
       </c>
       <c r="I653" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J653" t="s">
         <v>2370</v>
@@ -31055,7 +31055,7 @@
         <v>1593</v>
       </c>
       <c r="I654" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J654" t="s">
         <v>2371</v>
@@ -31090,7 +31090,7 @@
         <v>1593</v>
       </c>
       <c r="I655" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J655" t="s">
         <v>2372</v>
@@ -31125,7 +31125,7 @@
         <v>1593</v>
       </c>
       <c r="I656" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J656" t="s">
         <v>2373</v>
@@ -31160,7 +31160,7 @@
         <v>1593</v>
       </c>
       <c r="I657" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J657" t="s">
         <v>2374</v>
@@ -31195,7 +31195,7 @@
         <v>1593</v>
       </c>
       <c r="I658" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J658" t="s">
         <v>2375</v>
@@ -31230,7 +31230,7 @@
         <v>1593</v>
       </c>
       <c r="I659" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J659" t="s">
         <v>2376</v>
@@ -31265,7 +31265,7 @@
         <v>1593</v>
       </c>
       <c r="I660" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J660" t="s">
         <v>2377</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-10 22:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6691" uniqueCount="2586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6691" uniqueCount="2588">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7564,72 +7564,84 @@
     <t>RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,FENOMENOS DE ENERGIA E INFORMAÇÃO,VALORAÇÃO DANOS AMBIENTAIS</t>
+    <t>ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ORÇAMENTO</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,URBANISMO</t>
+  </si>
+  <si>
+    <t>PATRIMÔNIO HISTÓRICO E CULTURAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>PATRIMÔNIO HISTÓRICO E CULTURAL</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE,URBANISMO</t>
+  </si>
+  <si>
+    <t>ECONOMIA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,ENGENHARIA QUÍMICA</t>
+  </si>
+  <si>
+    <t>GEOLOGIA</t>
+  </si>
+  <si>
+    <t>SAÚDE</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES,PEDAGOGIA</t>
+  </si>
+  <si>
+    <t>BIOLOGIA</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES</t>
+  </si>
+  <si>
+    <t>RECURSOS HÍDRICOS,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>URBANISMO</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
     <t>### SEM TEMA ###</t>
   </si>
   <si>
-    <t>ORÇAMENTO</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,URBANISMO</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,PATRIMÔNIO HISTÓRICO E CULTURAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>PATRIMÔNIO HISTÓRICO E CULTURAL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,URBANISMO</t>
-  </si>
-  <si>
-    <t>ECONOMIA</t>
+    <t>ENGENHARIA QUÍMICA,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA</t>
   </si>
   <si>
-    <t>GEOLOGIA</t>
-  </si>
-  <si>
-    <t>SAÚDE</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES</t>
-  </si>
-  <si>
-    <t>BIOLOGIA</t>
-  </si>
-  <si>
-    <t>URBANISMO</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
-    <t>ECONOMIA,ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
     <t>RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
@@ -7639,7 +7651,7 @@
     <t>ENGENHARIA CIVIL,GEOTECNIA,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
   </si>
   <si>
-    <t>GEOTECNIA,VALORAÇÃO DANOS AMBIENTAIS</t>
+    <t>GEOTECNIA,ORÇAMENTO,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
     <t>ENGENHARIA AMBIENTAL</t>
@@ -7654,63 +7666,63 @@
     <t>ENGENHARIA QUÍMICA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
+    <t>ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
     <t>ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
     <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
+    <t>FARMÁCIA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
     <t>GEOTECNIA</t>
   </si>
   <si>
-    <t>GEOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>FARMÁCIA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,SAÚDE</t>
+    <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOTECNIA</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOTECNIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>MEDICINA LEGAL</t>
+  </si>
+  <si>
+    <t>ECONOMIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,EDIFICAÇÕES</t>
   </si>
   <si>
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,GEOTECNIA</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>MEDICINA LEGAL</t>
-  </si>
-  <si>
-    <t>ECONOMIA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>RECURSOS HÍDRICOS,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
     <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
@@ -7720,9 +7732,6 @@
     <t>BIOLOGIA,ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
@@ -7747,19 +7756,16 @@
     <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>PATRIMÔNIO HISTÓRICO E CULTURAL,URBANISMO</t>
-  </si>
-  <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>SAÚDE,SAÚDE MENTAL</t>
   </si>
   <si>
+    <t>BIOLOGIA,ENGENHARIA AMBIENTAL,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
     <t>MEDICINA LEGAL,SAÚDE</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ECONOMIA</t>
   </si>
   <si>
     <t>AVALIAÇÃO DE IMÓVEIS,AVALIAÇÃO DE IMÓVEIS</t>
@@ -8377,7 +8383,7 @@
         <v>2391</v>
       </c>
       <c r="L7" t="s">
-        <v>2517</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -8412,7 +8418,7 @@
         <v>2392</v>
       </c>
       <c r="L8" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -8447,7 +8453,7 @@
         <v>2393</v>
       </c>
       <c r="L9" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -8482,7 +8488,7 @@
         <v>2394</v>
       </c>
       <c r="L10" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -8517,7 +8523,7 @@
         <v>2395</v>
       </c>
       <c r="L11" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -8552,7 +8558,7 @@
         <v>2396</v>
       </c>
       <c r="L12" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -8587,7 +8593,7 @@
         <v>2396</v>
       </c>
       <c r="L13" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -8657,7 +8663,7 @@
         <v>2398</v>
       </c>
       <c r="L15" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -8727,7 +8733,7 @@
         <v>2400</v>
       </c>
       <c r="L17" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -8832,7 +8838,7 @@
         <v>2403</v>
       </c>
       <c r="L20" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -8902,7 +8908,7 @@
         <v>2405</v>
       </c>
       <c r="L22" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -8937,7 +8943,7 @@
         <v>2406</v>
       </c>
       <c r="L23" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -8972,7 +8978,7 @@
         <v>2406</v>
       </c>
       <c r="L24" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -9007,7 +9013,7 @@
         <v>2400</v>
       </c>
       <c r="L25" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -9042,7 +9048,7 @@
         <v>2400</v>
       </c>
       <c r="L26" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -9147,7 +9153,7 @@
         <v>2407</v>
       </c>
       <c r="L29" t="s">
-        <v>2517</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -9252,7 +9258,7 @@
         <v>2395</v>
       </c>
       <c r="L32" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -9287,7 +9293,7 @@
         <v>2411</v>
       </c>
       <c r="L33" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -9360,7 +9366,7 @@
         <v>2413</v>
       </c>
       <c r="L35" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -9608,7 +9614,7 @@
         <v>2413</v>
       </c>
       <c r="L42" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -9678,7 +9684,7 @@
         <v>2406</v>
       </c>
       <c r="L44" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -9853,7 +9859,7 @@
         <v>2421</v>
       </c>
       <c r="L49" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -10028,7 +10034,7 @@
         <v>2424</v>
       </c>
       <c r="L54" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -10063,7 +10069,7 @@
         <v>2425</v>
       </c>
       <c r="L55" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -10238,7 +10244,7 @@
         <v>2395</v>
       </c>
       <c r="L60" t="s">
-        <v>2515</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -10273,7 +10279,7 @@
         <v>2405</v>
       </c>
       <c r="L61" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -10308,7 +10314,7 @@
         <v>2423</v>
       </c>
       <c r="L62" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -10343,7 +10349,7 @@
         <v>2400</v>
       </c>
       <c r="L63" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -10413,7 +10419,7 @@
         <v>2406</v>
       </c>
       <c r="L65" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -10483,7 +10489,7 @@
         <v>2407</v>
       </c>
       <c r="L67" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -10623,7 +10629,7 @@
         <v>21</v>
       </c>
       <c r="L71" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -10693,7 +10699,7 @@
         <v>2395</v>
       </c>
       <c r="L73" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -10763,7 +10769,7 @@
         <v>2429</v>
       </c>
       <c r="L75" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -10798,7 +10804,7 @@
         <v>2430</v>
       </c>
       <c r="L76" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -10868,7 +10874,7 @@
         <v>2396</v>
       </c>
       <c r="L78" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -10903,7 +10909,7 @@
         <v>2418</v>
       </c>
       <c r="L79" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="80" spans="1:12">
@@ -10973,7 +10979,7 @@
         <v>2432</v>
       </c>
       <c r="L81" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="82" spans="1:12">
@@ -11008,7 +11014,7 @@
         <v>2433</v>
       </c>
       <c r="L82" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="83" spans="1:12">
@@ -11043,7 +11049,7 @@
         <v>2434</v>
       </c>
       <c r="L83" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="84" spans="1:12">
@@ -11113,7 +11119,7 @@
         <v>2401</v>
       </c>
       <c r="L85" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="86" spans="1:12">
@@ -11148,7 +11154,7 @@
         <v>2435</v>
       </c>
       <c r="L86" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="87" spans="1:12">
@@ -11183,7 +11189,7 @@
         <v>2436</v>
       </c>
       <c r="L87" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="88" spans="1:12">
@@ -11288,7 +11294,7 @@
         <v>2421</v>
       </c>
       <c r="L90" t="s">
-        <v>2517</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="91" spans="1:12">
@@ -11393,7 +11399,7 @@
         <v>2436</v>
       </c>
       <c r="L93" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="94" spans="1:12">
@@ -11428,7 +11434,7 @@
         <v>2407</v>
       </c>
       <c r="L94" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="95" spans="1:12">
@@ -11463,7 +11469,7 @@
         <v>2428</v>
       </c>
       <c r="L95" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="96" spans="1:12">
@@ -11708,7 +11714,7 @@
         <v>2424</v>
       </c>
       <c r="L102" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="103" spans="1:12">
@@ -11743,7 +11749,7 @@
         <v>2396</v>
       </c>
       <c r="L103" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="104" spans="1:12">
@@ -11813,7 +11819,7 @@
         <v>2415</v>
       </c>
       <c r="L105" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="106" spans="1:12">
@@ -11883,7 +11889,7 @@
         <v>2397</v>
       </c>
       <c r="L107" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="108" spans="1:12">
@@ -11953,7 +11959,7 @@
         <v>2444</v>
       </c>
       <c r="L109" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="110" spans="1:12">
@@ -11988,7 +11994,7 @@
         <v>2436</v>
       </c>
       <c r="L110" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="111" spans="1:12">
@@ -12023,7 +12029,7 @@
         <v>2414</v>
       </c>
       <c r="L111" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="112" spans="1:12">
@@ -12058,7 +12064,7 @@
         <v>2428</v>
       </c>
       <c r="L112" t="s">
-        <v>2525</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="113" spans="1:12">
@@ -12163,7 +12169,7 @@
         <v>2420</v>
       </c>
       <c r="L115" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="116" spans="1:12">
@@ -12198,7 +12204,7 @@
         <v>2436</v>
       </c>
       <c r="L116" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="117" spans="1:12">
@@ -12233,7 +12239,7 @@
         <v>2405</v>
       </c>
       <c r="L117" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="118" spans="1:12">
@@ -12268,7 +12274,7 @@
         <v>2400</v>
       </c>
       <c r="L118" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="119" spans="1:12">
@@ -12338,7 +12344,7 @@
         <v>2412</v>
       </c>
       <c r="L120" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="121" spans="1:12">
@@ -12373,7 +12379,7 @@
         <v>2412</v>
       </c>
       <c r="L121" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="122" spans="1:12">
@@ -12443,7 +12449,7 @@
         <v>2409</v>
       </c>
       <c r="L123" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="124" spans="1:12">
@@ -12478,7 +12484,7 @@
         <v>2421</v>
       </c>
       <c r="L124" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="125" spans="1:12">
@@ -12548,7 +12554,7 @@
         <v>2395</v>
       </c>
       <c r="L126" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="127" spans="1:12">
@@ -12583,7 +12589,7 @@
         <v>2424</v>
       </c>
       <c r="L127" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="128" spans="1:12">
@@ -12618,7 +12624,7 @@
         <v>2424</v>
       </c>
       <c r="L128" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="129" spans="1:12">
@@ -12653,7 +12659,7 @@
         <v>2435</v>
       </c>
       <c r="L129" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="130" spans="1:12">
@@ -12688,7 +12694,7 @@
         <v>2435</v>
       </c>
       <c r="L130" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="131" spans="1:12">
@@ -12723,7 +12729,7 @@
         <v>2428</v>
       </c>
       <c r="L131" t="s">
-        <v>2540</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="132" spans="1:12">
@@ -12828,7 +12834,7 @@
         <v>2397</v>
       </c>
       <c r="L134" t="s">
-        <v>2541</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="135" spans="1:12">
@@ -12863,7 +12869,7 @@
         <v>2407</v>
       </c>
       <c r="L135" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="136" spans="1:12">
@@ -12968,7 +12974,7 @@
         <v>2402</v>
       </c>
       <c r="L138" t="s">
-        <v>2542</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="139" spans="1:12">
@@ -13003,7 +13009,7 @@
         <v>2444</v>
       </c>
       <c r="L139" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="140" spans="1:12">
@@ -13073,7 +13079,7 @@
         <v>2404</v>
       </c>
       <c r="L141" t="s">
-        <v>2543</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="142" spans="1:12">
@@ -13108,7 +13114,7 @@
         <v>2423</v>
       </c>
       <c r="L142" t="s">
-        <v>2542</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="143" spans="1:12">
@@ -13283,7 +13289,7 @@
         <v>2417</v>
       </c>
       <c r="L147" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="148" spans="1:12">
@@ -13353,7 +13359,7 @@
         <v>2435</v>
       </c>
       <c r="L149" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="150" spans="1:12">
@@ -13388,7 +13394,7 @@
         <v>2414</v>
       </c>
       <c r="L150" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="151" spans="1:12">
@@ -13423,7 +13429,7 @@
         <v>2446</v>
       </c>
       <c r="L151" t="s">
-        <v>2545</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="152" spans="1:12">
@@ -13458,7 +13464,7 @@
         <v>2401</v>
       </c>
       <c r="L152" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="153" spans="1:12">
@@ -13493,7 +13499,7 @@
         <v>2401</v>
       </c>
       <c r="L153" t="s">
-        <v>2534</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="154" spans="1:12">
@@ -13528,7 +13534,7 @@
         <v>2397</v>
       </c>
       <c r="L154" t="s">
-        <v>2546</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="155" spans="1:12">
@@ -13668,7 +13674,7 @@
         <v>2440</v>
       </c>
       <c r="L158" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="159" spans="1:12">
@@ -13703,7 +13709,7 @@
         <v>2447</v>
       </c>
       <c r="L159" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="160" spans="1:12">
@@ -13738,7 +13744,7 @@
         <v>2448</v>
       </c>
       <c r="L160" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="161" spans="1:12">
@@ -13773,7 +13779,7 @@
         <v>2395</v>
       </c>
       <c r="L161" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="162" spans="1:12">
@@ -13808,7 +13814,7 @@
         <v>2388</v>
       </c>
       <c r="L162" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="163" spans="1:12">
@@ -13843,7 +13849,7 @@
         <v>2449</v>
       </c>
       <c r="L163" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -13913,7 +13919,7 @@
         <v>2450</v>
       </c>
       <c r="L165" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="166" spans="1:12">
@@ -14123,7 +14129,7 @@
         <v>2454</v>
       </c>
       <c r="L171" t="s">
-        <v>2548</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="172" spans="1:12">
@@ -14158,7 +14164,7 @@
         <v>2422</v>
       </c>
       <c r="L172" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="173" spans="1:12">
@@ -14228,7 +14234,7 @@
         <v>2454</v>
       </c>
       <c r="L174" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="175" spans="1:12">
@@ -14298,7 +14304,7 @@
         <v>2409</v>
       </c>
       <c r="L176" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="177" spans="1:12">
@@ -14333,7 +14339,7 @@
         <v>2400</v>
       </c>
       <c r="L177" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="178" spans="1:12">
@@ -14438,7 +14444,7 @@
         <v>2423</v>
       </c>
       <c r="L180" t="s">
-        <v>2549</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="181" spans="1:12">
@@ -14473,7 +14479,7 @@
         <v>2456</v>
       </c>
       <c r="L181" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="182" spans="1:12">
@@ -14508,7 +14514,7 @@
         <v>2421</v>
       </c>
       <c r="L182" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="183" spans="1:12">
@@ -14578,7 +14584,7 @@
         <v>2400</v>
       </c>
       <c r="L184" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="185" spans="1:12">
@@ -14613,7 +14619,7 @@
         <v>2447</v>
       </c>
       <c r="L185" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="186" spans="1:12">
@@ -14648,7 +14654,7 @@
         <v>2457</v>
       </c>
       <c r="L186" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="187" spans="1:12">
@@ -14683,7 +14689,7 @@
         <v>2458</v>
       </c>
       <c r="L187" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="188" spans="1:12">
@@ -14718,7 +14724,7 @@
         <v>2459</v>
       </c>
       <c r="L188" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="189" spans="1:12">
@@ -14753,7 +14759,7 @@
         <v>2405</v>
       </c>
       <c r="L189" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="190" spans="1:12">
@@ -14788,7 +14794,7 @@
         <v>2436</v>
       </c>
       <c r="L190" t="s">
-        <v>2550</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="191" spans="1:12">
@@ -14826,7 +14832,7 @@
         <v>2447</v>
       </c>
       <c r="L191" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -14861,7 +14867,7 @@
         <v>2395</v>
       </c>
       <c r="L192" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="193" spans="1:12">
@@ -14931,7 +14937,7 @@
         <v>2460</v>
       </c>
       <c r="L194" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -14966,7 +14972,7 @@
         <v>2412</v>
       </c>
       <c r="L195" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="196" spans="1:12">
@@ -15001,7 +15007,7 @@
         <v>2433</v>
       </c>
       <c r="L196" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="197" spans="1:12">
@@ -15036,7 +15042,7 @@
         <v>2461</v>
       </c>
       <c r="L197" t="s">
-        <v>2552</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -15071,7 +15077,7 @@
         <v>2389</v>
       </c>
       <c r="L198" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="199" spans="1:12">
@@ -15246,7 +15252,7 @@
         <v>2400</v>
       </c>
       <c r="L203" t="s">
-        <v>2517</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="204" spans="1:12">
@@ -15281,7 +15287,7 @@
         <v>2400</v>
       </c>
       <c r="L204" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="205" spans="1:12">
@@ -15316,7 +15322,7 @@
         <v>2400</v>
       </c>
       <c r="L205" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="206" spans="1:12">
@@ -15351,7 +15357,7 @@
         <v>2400</v>
       </c>
       <c r="L206" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="207" spans="1:12">
@@ -15386,7 +15392,7 @@
         <v>2418</v>
       </c>
       <c r="L207" t="s">
-        <v>2553</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="208" spans="1:12">
@@ -15736,7 +15742,7 @@
         <v>2396</v>
       </c>
       <c r="L217" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="218" spans="1:12">
@@ -15911,7 +15917,7 @@
         <v>2446</v>
       </c>
       <c r="L222" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="223" spans="1:12">
@@ -15981,7 +15987,7 @@
         <v>2436</v>
       </c>
       <c r="L224" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="225" spans="1:12">
@@ -16016,7 +16022,7 @@
         <v>2413</v>
       </c>
       <c r="L225" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="226" spans="1:12">
@@ -16086,7 +16092,7 @@
         <v>2423</v>
       </c>
       <c r="L227" t="s">
-        <v>2546</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="228" spans="1:12">
@@ -16156,7 +16162,7 @@
         <v>2405</v>
       </c>
       <c r="L229" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="230" spans="1:12">
@@ -16191,7 +16197,7 @@
         <v>2466</v>
       </c>
       <c r="L230" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="231" spans="1:12">
@@ -16226,7 +16232,7 @@
         <v>2467</v>
       </c>
       <c r="L231" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="232" spans="1:12">
@@ -16261,7 +16267,7 @@
         <v>2467</v>
       </c>
       <c r="L232" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="233" spans="1:12">
@@ -16296,7 +16302,7 @@
         <v>2423</v>
       </c>
       <c r="L233" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="234" spans="1:12">
@@ -16331,7 +16337,7 @@
         <v>2423</v>
       </c>
       <c r="L234" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="235" spans="1:12">
@@ -16366,7 +16372,7 @@
         <v>2423</v>
       </c>
       <c r="L235" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="236" spans="1:12">
@@ -16401,7 +16407,7 @@
         <v>2435</v>
       </c>
       <c r="L236" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="237" spans="1:12">
@@ -16506,7 +16512,7 @@
         <v>2468</v>
       </c>
       <c r="L239" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="240" spans="1:12">
@@ -16611,7 +16617,7 @@
         <v>2429</v>
       </c>
       <c r="L242" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="243" spans="1:12">
@@ -16646,7 +16652,7 @@
         <v>2405</v>
       </c>
       <c r="L243" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="244" spans="1:12">
@@ -16681,7 +16687,7 @@
         <v>2441</v>
       </c>
       <c r="L244" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="245" spans="1:12">
@@ -16716,7 +16722,7 @@
         <v>2423</v>
       </c>
       <c r="L245" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="246" spans="1:12">
@@ -16751,7 +16757,7 @@
         <v>2469</v>
       </c>
       <c r="L246" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="247" spans="1:12">
@@ -16786,7 +16792,7 @@
         <v>2405</v>
       </c>
       <c r="L247" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="248" spans="1:12">
@@ -16856,7 +16862,7 @@
         <v>2461</v>
       </c>
       <c r="L249" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="250" spans="1:12">
@@ -16891,7 +16897,7 @@
         <v>2426</v>
       </c>
       <c r="L250" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="251" spans="1:12">
@@ -16926,7 +16932,7 @@
         <v>2430</v>
       </c>
       <c r="L251" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="252" spans="1:12">
@@ -17066,7 +17072,7 @@
         <v>2421</v>
       </c>
       <c r="L255" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="256" spans="1:12">
@@ -17101,7 +17107,7 @@
         <v>2458</v>
       </c>
       <c r="L256" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="257" spans="1:12">
@@ -17136,7 +17142,7 @@
         <v>2439</v>
       </c>
       <c r="L257" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="258" spans="1:12">
@@ -17206,7 +17212,7 @@
         <v>2407</v>
       </c>
       <c r="L259" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="260" spans="1:12">
@@ -17346,7 +17352,7 @@
         <v>2389</v>
       </c>
       <c r="L263" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="264" spans="1:12">
@@ -17381,7 +17387,7 @@
         <v>2471</v>
       </c>
       <c r="L264" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="265" spans="1:12">
@@ -17486,7 +17492,7 @@
         <v>2448</v>
       </c>
       <c r="L267" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="268" spans="1:12">
@@ -17521,7 +17527,7 @@
         <v>2472</v>
       </c>
       <c r="L268" t="s">
-        <v>2558</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="269" spans="1:12">
@@ -17556,7 +17562,7 @@
         <v>2472</v>
       </c>
       <c r="L269" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="270" spans="1:12">
@@ -17591,7 +17597,7 @@
         <v>2411</v>
       </c>
       <c r="L270" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="271" spans="1:12">
@@ -17626,7 +17632,7 @@
         <v>2436</v>
       </c>
       <c r="L271" t="s">
-        <v>2559</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="272" spans="1:12">
@@ -17801,7 +17807,7 @@
         <v>2416</v>
       </c>
       <c r="L276" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="277" spans="1:12">
@@ -17836,7 +17842,7 @@
         <v>2405</v>
       </c>
       <c r="L277" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="278" spans="1:12">
@@ -17871,7 +17877,7 @@
         <v>2417</v>
       </c>
       <c r="L278" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="279" spans="1:12">
@@ -17906,7 +17912,7 @@
         <v>2404</v>
       </c>
       <c r="L279" t="s">
-        <v>2560</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="280" spans="1:12">
@@ -17941,7 +17947,7 @@
         <v>2469</v>
       </c>
       <c r="L280" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="281" spans="1:12">
@@ -18046,7 +18052,7 @@
         <v>2389</v>
       </c>
       <c r="L283" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="284" spans="1:12">
@@ -18116,7 +18122,7 @@
         <v>2450</v>
       </c>
       <c r="L285" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="286" spans="1:12">
@@ -18151,7 +18157,7 @@
         <v>2451</v>
       </c>
       <c r="L286" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="287" spans="1:12">
@@ -18291,7 +18297,7 @@
         <v>2389</v>
       </c>
       <c r="L290" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="291" spans="1:12">
@@ -18326,7 +18332,7 @@
         <v>2447</v>
       </c>
       <c r="L291" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="292" spans="1:12">
@@ -18396,7 +18402,7 @@
         <v>2412</v>
       </c>
       <c r="L293" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="294" spans="1:12">
@@ -18466,7 +18472,7 @@
         <v>2474</v>
       </c>
       <c r="L295" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="296" spans="1:12">
@@ -18501,7 +18507,7 @@
         <v>2447</v>
       </c>
       <c r="L296" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="297" spans="1:12">
@@ -18536,7 +18542,7 @@
         <v>2409</v>
       </c>
       <c r="L297" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="298" spans="1:12">
@@ -18641,7 +18647,7 @@
         <v>2450</v>
       </c>
       <c r="L300" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="301" spans="1:12">
@@ -18746,7 +18752,7 @@
         <v>2400</v>
       </c>
       <c r="L303" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="304" spans="1:12">
@@ -18781,7 +18787,7 @@
         <v>2422</v>
       </c>
       <c r="L304" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="305" spans="1:12">
@@ -18816,7 +18822,7 @@
         <v>2459</v>
       </c>
       <c r="L305" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="306" spans="1:12">
@@ -18851,7 +18857,7 @@
         <v>2388</v>
       </c>
       <c r="L306" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="307" spans="1:12">
@@ -18956,7 +18962,7 @@
         <v>2445</v>
       </c>
       <c r="L309" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="310" spans="1:12">
@@ -19026,7 +19032,7 @@
         <v>2475</v>
       </c>
       <c r="L311" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="312" spans="1:12">
@@ -19061,7 +19067,7 @@
         <v>2417</v>
       </c>
       <c r="L312" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="313" spans="1:12">
@@ -19096,7 +19102,7 @@
         <v>2437</v>
       </c>
       <c r="L313" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="314" spans="1:12">
@@ -19131,7 +19137,7 @@
         <v>2411</v>
       </c>
       <c r="L314" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="315" spans="1:12">
@@ -19201,7 +19207,7 @@
         <v>2424</v>
       </c>
       <c r="L316" t="s">
-        <v>2529</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="317" spans="1:12">
@@ -19271,7 +19277,7 @@
         <v>2476</v>
       </c>
       <c r="L318" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="319" spans="1:12">
@@ -19306,7 +19312,7 @@
         <v>2476</v>
       </c>
       <c r="L319" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="320" spans="1:12">
@@ -19341,7 +19347,7 @@
         <v>2476</v>
       </c>
       <c r="L320" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="321" spans="1:12">
@@ -19379,7 +19385,7 @@
         <v>2477</v>
       </c>
       <c r="L321" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="322" spans="1:12">
@@ -19519,7 +19525,7 @@
         <v>2395</v>
       </c>
       <c r="L325" t="s">
-        <v>2564</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="326" spans="1:12">
@@ -19589,7 +19595,7 @@
         <v>2402</v>
       </c>
       <c r="L327" t="s">
-        <v>2553</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="328" spans="1:12">
@@ -19729,7 +19735,7 @@
         <v>2479</v>
       </c>
       <c r="L331" t="s">
-        <v>2565</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="332" spans="1:12">
@@ -19764,7 +19770,7 @@
         <v>2479</v>
       </c>
       <c r="L332" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="333" spans="1:12">
@@ -19799,7 +19805,7 @@
         <v>2440</v>
       </c>
       <c r="L333" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="334" spans="1:12">
@@ -19904,7 +19910,7 @@
         <v>2422</v>
       </c>
       <c r="L336" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="337" spans="1:12">
@@ -19939,7 +19945,7 @@
         <v>2426</v>
       </c>
       <c r="L337" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="338" spans="1:12">
@@ -20009,7 +20015,7 @@
         <v>2432</v>
       </c>
       <c r="L339" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="340" spans="1:12">
@@ -20044,7 +20050,7 @@
         <v>2435</v>
       </c>
       <c r="L340" t="s">
-        <v>2566</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="341" spans="1:12">
@@ -20079,7 +20085,7 @@
         <v>2418</v>
       </c>
       <c r="L341" t="s">
-        <v>2567</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="342" spans="1:12">
@@ -20114,7 +20120,7 @@
         <v>2480</v>
       </c>
       <c r="L342" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="343" spans="1:12">
@@ -20184,7 +20190,7 @@
         <v>2422</v>
       </c>
       <c r="L344" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="345" spans="1:12">
@@ -20219,7 +20225,7 @@
         <v>2405</v>
       </c>
       <c r="L345" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="346" spans="1:12">
@@ -20254,7 +20260,7 @@
         <v>2405</v>
       </c>
       <c r="L346" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="347" spans="1:12">
@@ -20289,7 +20295,7 @@
         <v>2423</v>
       </c>
       <c r="L347" t="s">
-        <v>2546</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -20324,7 +20330,7 @@
         <v>2469</v>
       </c>
       <c r="L348" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="349" spans="1:12">
@@ -20464,7 +20470,7 @@
         <v>2397</v>
       </c>
       <c r="L352" t="s">
-        <v>2568</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="353" spans="1:12">
@@ -20499,7 +20505,7 @@
         <v>2481</v>
       </c>
       <c r="L353" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="354" spans="1:12">
@@ -20534,7 +20540,7 @@
         <v>2391</v>
       </c>
       <c r="L354" t="s">
-        <v>2525</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="355" spans="1:12">
@@ -20569,7 +20575,7 @@
         <v>2481</v>
       </c>
       <c r="L355" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="356" spans="1:12">
@@ -20674,7 +20680,7 @@
         <v>2400</v>
       </c>
       <c r="L358" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20779,7 +20785,7 @@
         <v>2422</v>
       </c>
       <c r="L361" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="362" spans="1:12">
@@ -20814,7 +20820,7 @@
         <v>2422</v>
       </c>
       <c r="L362" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="363" spans="1:12">
@@ -20849,7 +20855,7 @@
         <v>2450</v>
       </c>
       <c r="L363" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="364" spans="1:12">
@@ -20884,7 +20890,7 @@
         <v>2405</v>
       </c>
       <c r="L364" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="365" spans="1:12">
@@ -20919,7 +20925,7 @@
         <v>2482</v>
       </c>
       <c r="L365" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="366" spans="1:12">
@@ -21027,7 +21033,7 @@
         <v>2415</v>
       </c>
       <c r="L368" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="369" spans="1:12">
@@ -21135,7 +21141,7 @@
         <v>2414</v>
       </c>
       <c r="L371" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="372" spans="1:12">
@@ -21205,7 +21211,7 @@
         <v>2405</v>
       </c>
       <c r="L373" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="374" spans="1:12">
@@ -21240,7 +21246,7 @@
         <v>2429</v>
       </c>
       <c r="L374" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="375" spans="1:12">
@@ -21275,7 +21281,7 @@
         <v>2429</v>
       </c>
       <c r="L375" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="376" spans="1:12">
@@ -21310,7 +21316,7 @@
         <v>2485</v>
       </c>
       <c r="L376" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="377" spans="1:12">
@@ -21345,7 +21351,7 @@
         <v>2480</v>
       </c>
       <c r="L377" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="378" spans="1:12">
@@ -21380,7 +21386,7 @@
         <v>2432</v>
       </c>
       <c r="L378" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="379" spans="1:12">
@@ -21415,7 +21421,7 @@
         <v>2420</v>
       </c>
       <c r="L379" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="380" spans="1:12">
@@ -21450,7 +21456,7 @@
         <v>2471</v>
       </c>
       <c r="L380" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="381" spans="1:12">
@@ -21485,7 +21491,7 @@
         <v>2483</v>
       </c>
       <c r="L381" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="382" spans="1:12">
@@ -21520,7 +21526,7 @@
         <v>2480</v>
       </c>
       <c r="L382" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="383" spans="1:12">
@@ -21590,7 +21596,7 @@
         <v>2405</v>
       </c>
       <c r="L384" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="385" spans="1:12">
@@ -21625,7 +21631,7 @@
         <v>2486</v>
       </c>
       <c r="L385" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="386" spans="1:12">
@@ -21660,7 +21666,7 @@
         <v>2407</v>
       </c>
       <c r="L386" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="387" spans="1:12">
@@ -21695,7 +21701,7 @@
         <v>2487</v>
       </c>
       <c r="L387" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="388" spans="1:12">
@@ -21730,7 +21736,7 @@
         <v>2488</v>
       </c>
       <c r="L388" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="389" spans="1:12">
@@ -21765,7 +21771,7 @@
         <v>2489</v>
       </c>
       <c r="L389" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="390" spans="1:12">
@@ -21870,7 +21876,7 @@
         <v>2405</v>
       </c>
       <c r="L392" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="393" spans="1:12">
@@ -21905,7 +21911,7 @@
         <v>2436</v>
       </c>
       <c r="L393" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="394" spans="1:12">
@@ -21975,7 +21981,7 @@
         <v>2423</v>
       </c>
       <c r="L395" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="396" spans="1:12">
@@ -22010,7 +22016,7 @@
         <v>2413</v>
       </c>
       <c r="L396" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="397" spans="1:12">
@@ -22045,7 +22051,7 @@
         <v>2471</v>
       </c>
       <c r="L397" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="398" spans="1:12">
@@ -22115,7 +22121,7 @@
         <v>2490</v>
       </c>
       <c r="L399" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="400" spans="1:12">
@@ -22150,7 +22156,7 @@
         <v>2435</v>
       </c>
       <c r="L400" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="401" spans="1:12">
@@ -22185,7 +22191,7 @@
         <v>2446</v>
       </c>
       <c r="L401" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="402" spans="1:12">
@@ -22220,7 +22226,7 @@
         <v>2388</v>
       </c>
       <c r="L402" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="403" spans="1:12">
@@ -22395,7 +22401,7 @@
         <v>2407</v>
       </c>
       <c r="L407" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22605,7 +22611,7 @@
         <v>2469</v>
       </c>
       <c r="L413" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="414" spans="1:12">
@@ -22640,7 +22646,7 @@
         <v>2440</v>
       </c>
       <c r="L414" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="415" spans="1:12">
@@ -22710,7 +22716,7 @@
         <v>2418</v>
       </c>
       <c r="L416" t="s">
-        <v>2525</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="417" spans="1:12">
@@ -22745,7 +22751,7 @@
         <v>2410</v>
       </c>
       <c r="L417" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="418" spans="1:12">
@@ -22850,7 +22856,7 @@
         <v>2407</v>
       </c>
       <c r="L420" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="421" spans="1:12">
@@ -22920,7 +22926,7 @@
         <v>2423</v>
       </c>
       <c r="L422" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="423" spans="1:12">
@@ -22955,7 +22961,7 @@
         <v>2462</v>
       </c>
       <c r="L423" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="424" spans="1:12">
@@ -23025,7 +23031,7 @@
         <v>2405</v>
       </c>
       <c r="L425" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="426" spans="1:12">
@@ -23095,7 +23101,7 @@
         <v>2405</v>
       </c>
       <c r="L427" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="428" spans="1:12">
@@ -23130,7 +23136,7 @@
         <v>2446</v>
       </c>
       <c r="L428" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="429" spans="1:12">
@@ -23165,7 +23171,7 @@
         <v>2417</v>
       </c>
       <c r="L429" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="430" spans="1:12">
@@ -23200,7 +23206,7 @@
         <v>2405</v>
       </c>
       <c r="L430" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="431" spans="1:12">
@@ -23235,7 +23241,7 @@
         <v>2435</v>
       </c>
       <c r="L431" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -23305,7 +23311,7 @@
         <v>2461</v>
       </c>
       <c r="L433" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="434" spans="1:12">
@@ -23410,7 +23416,7 @@
         <v>2417</v>
       </c>
       <c r="L436" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="437" spans="1:12">
@@ -23480,7 +23486,7 @@
         <v>2400</v>
       </c>
       <c r="L438" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="439" spans="1:12">
@@ -23585,7 +23591,7 @@
         <v>2400</v>
       </c>
       <c r="L441" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="442" spans="1:12">
@@ -23655,7 +23661,7 @@
         <v>2400</v>
       </c>
       <c r="L443" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -23760,7 +23766,7 @@
         <v>2456</v>
       </c>
       <c r="L446" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="447" spans="1:12">
@@ -23795,7 +23801,7 @@
         <v>2391</v>
       </c>
       <c r="L447" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="448" spans="1:12">
@@ -23830,7 +23836,7 @@
         <v>2423</v>
       </c>
       <c r="L448" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="449" spans="1:12">
@@ -23900,7 +23906,7 @@
         <v>2491</v>
       </c>
       <c r="L450" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="451" spans="1:12">
@@ -24075,7 +24081,7 @@
         <v>2400</v>
       </c>
       <c r="L455" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -24148,7 +24154,7 @@
         <v>2422</v>
       </c>
       <c r="L457" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="458" spans="1:12">
@@ -24183,7 +24189,7 @@
         <v>2423</v>
       </c>
       <c r="L458" t="s">
-        <v>2564</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24253,7 +24259,7 @@
         <v>2389</v>
       </c>
       <c r="L460" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="461" spans="1:12">
@@ -24466,7 +24472,7 @@
         <v>2423</v>
       </c>
       <c r="L466" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="467" spans="1:12">
@@ -24571,7 +24577,7 @@
         <v>2429</v>
       </c>
       <c r="L469" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="470" spans="1:12">
@@ -24676,7 +24682,7 @@
         <v>2448</v>
       </c>
       <c r="L472" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="473" spans="1:12">
@@ -24711,7 +24717,7 @@
         <v>2411</v>
       </c>
       <c r="L473" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="474" spans="1:12">
@@ -24746,7 +24752,7 @@
         <v>2388</v>
       </c>
       <c r="L474" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="475" spans="1:12">
@@ -24816,7 +24822,7 @@
         <v>2426</v>
       </c>
       <c r="L476" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="477" spans="1:12">
@@ -24851,7 +24857,7 @@
         <v>2427</v>
       </c>
       <c r="L477" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="478" spans="1:12">
@@ -24921,7 +24927,7 @@
         <v>2420</v>
       </c>
       <c r="L479" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -24991,7 +24997,7 @@
         <v>2436</v>
       </c>
       <c r="L481" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="482" spans="1:12">
@@ -25026,7 +25032,7 @@
         <v>2397</v>
       </c>
       <c r="L482" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="483" spans="1:12">
@@ -25096,7 +25102,7 @@
         <v>2415</v>
       </c>
       <c r="L484" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="485" spans="1:12">
@@ -25131,7 +25137,7 @@
         <v>2400</v>
       </c>
       <c r="L485" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25271,7 +25277,7 @@
         <v>2435</v>
       </c>
       <c r="L489" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="490" spans="1:12">
@@ -25344,7 +25350,7 @@
         <v>2477</v>
       </c>
       <c r="L491" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="492" spans="1:12">
@@ -25379,7 +25385,7 @@
         <v>2437</v>
       </c>
       <c r="L492" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="493" spans="1:12">
@@ -25414,7 +25420,7 @@
         <v>2411</v>
       </c>
       <c r="L493" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="494" spans="1:12">
@@ -25449,7 +25455,7 @@
         <v>2480</v>
       </c>
       <c r="L494" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="495" spans="1:12">
@@ -25484,7 +25490,7 @@
         <v>2420</v>
       </c>
       <c r="L495" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="496" spans="1:12">
@@ -25519,7 +25525,7 @@
         <v>2395</v>
       </c>
       <c r="L496" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="497" spans="1:12">
@@ -25589,7 +25595,7 @@
         <v>2388</v>
       </c>
       <c r="L498" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="499" spans="1:12">
@@ -25694,7 +25700,7 @@
         <v>2421</v>
       </c>
       <c r="L501" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="502" spans="1:12">
@@ -25764,7 +25770,7 @@
         <v>2442</v>
       </c>
       <c r="L503" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -25834,7 +25840,7 @@
         <v>2391</v>
       </c>
       <c r="L505" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="506" spans="1:12">
@@ -25869,7 +25875,7 @@
         <v>2391</v>
       </c>
       <c r="L506" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25939,7 +25945,7 @@
         <v>2391</v>
       </c>
       <c r="L508" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="509" spans="1:12">
@@ -25974,7 +25980,7 @@
         <v>2391</v>
       </c>
       <c r="L509" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="510" spans="1:12">
@@ -26044,7 +26050,7 @@
         <v>2477</v>
       </c>
       <c r="L511" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="512" spans="1:12">
@@ -26149,7 +26155,7 @@
         <v>2396</v>
       </c>
       <c r="L514" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="515" spans="1:12">
@@ -26187,7 +26193,7 @@
         <v>2396</v>
       </c>
       <c r="L515" t="s">
-        <v>2549</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="516" spans="1:12">
@@ -26222,7 +26228,7 @@
         <v>2396</v>
       </c>
       <c r="L516" t="s">
-        <v>2577</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="517" spans="1:12">
@@ -26257,7 +26263,7 @@
         <v>2429</v>
       </c>
       <c r="L517" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="518" spans="1:12">
@@ -26327,7 +26333,7 @@
         <v>2396</v>
       </c>
       <c r="L519" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="520" spans="1:12">
@@ -26362,7 +26368,7 @@
         <v>2415</v>
       </c>
       <c r="L520" t="s">
-        <v>2558</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="521" spans="1:12">
@@ -26397,7 +26403,7 @@
         <v>2415</v>
       </c>
       <c r="L521" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="522" spans="1:12">
@@ -26467,7 +26473,7 @@
         <v>2422</v>
       </c>
       <c r="L523" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="524" spans="1:12">
@@ -26502,7 +26508,7 @@
         <v>2437</v>
       </c>
       <c r="L524" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="525" spans="1:12">
@@ -26572,7 +26578,7 @@
         <v>2493</v>
       </c>
       <c r="L526" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="527" spans="1:12">
@@ -26677,7 +26683,7 @@
         <v>2494</v>
       </c>
       <c r="L529" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="530" spans="1:12">
@@ -26712,7 +26718,7 @@
         <v>2481</v>
       </c>
       <c r="L530" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="531" spans="1:12">
@@ -26747,7 +26753,7 @@
         <v>2466</v>
       </c>
       <c r="L531" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="532" spans="1:12">
@@ -26782,7 +26788,7 @@
         <v>2495</v>
       </c>
       <c r="L532" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="533" spans="1:12">
@@ -26817,7 +26823,7 @@
         <v>2388</v>
       </c>
       <c r="L533" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="534" spans="1:12">
@@ -26925,7 +26931,7 @@
         <v>2397</v>
       </c>
       <c r="L536" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="537" spans="1:12">
@@ -26960,7 +26966,7 @@
         <v>2397</v>
       </c>
       <c r="L537" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="538" spans="1:12">
@@ -26995,7 +27001,7 @@
         <v>2399</v>
       </c>
       <c r="L538" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -27030,7 +27036,7 @@
         <v>2426</v>
       </c>
       <c r="L539" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="540" spans="1:12">
@@ -27065,7 +27071,7 @@
         <v>2402</v>
       </c>
       <c r="L540" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27100,7 +27106,7 @@
         <v>2474</v>
       </c>
       <c r="L541" t="s">
-        <v>2553</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="542" spans="1:12">
@@ -27135,7 +27141,7 @@
         <v>2422</v>
       </c>
       <c r="L542" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="543" spans="1:12">
@@ -27170,7 +27176,7 @@
         <v>2496</v>
       </c>
       <c r="L543" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="544" spans="1:12">
@@ -27205,7 +27211,7 @@
         <v>2422</v>
       </c>
       <c r="L544" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="545" spans="1:12">
@@ -27275,7 +27281,7 @@
         <v>2450</v>
       </c>
       <c r="L546" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="547" spans="1:12">
@@ -27415,7 +27421,7 @@
         <v>2443</v>
       </c>
       <c r="L550" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="551" spans="1:12">
@@ -27485,7 +27491,7 @@
         <v>2434</v>
       </c>
       <c r="L552" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27520,7 +27526,7 @@
         <v>2442</v>
       </c>
       <c r="L553" t="s">
-        <v>2517</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -27590,7 +27596,7 @@
         <v>2497</v>
       </c>
       <c r="L555" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="556" spans="1:12">
@@ -27660,7 +27666,7 @@
         <v>2463</v>
       </c>
       <c r="L557" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="558" spans="1:12">
@@ -27695,7 +27701,7 @@
         <v>2498</v>
       </c>
       <c r="L558" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="559" spans="1:12">
@@ -27838,7 +27844,7 @@
         <v>2428</v>
       </c>
       <c r="L562" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="563" spans="1:12">
@@ -27978,7 +27984,7 @@
         <v>2401</v>
       </c>
       <c r="L566" t="s">
-        <v>2581</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="567" spans="1:12">
@@ -28013,7 +28019,7 @@
         <v>2429</v>
       </c>
       <c r="L567" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="568" spans="1:12">
@@ -28048,7 +28054,7 @@
         <v>2447</v>
       </c>
       <c r="L568" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="569" spans="1:12">
@@ -28083,7 +28089,7 @@
         <v>2447</v>
       </c>
       <c r="L569" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -28118,7 +28124,7 @@
         <v>2501</v>
       </c>
       <c r="L570" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28331,7 +28337,7 @@
         <v>2429</v>
       </c>
       <c r="L576" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="577" spans="1:12">
@@ -28366,7 +28372,7 @@
         <v>2423</v>
       </c>
       <c r="L577" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="578" spans="1:12">
@@ -28471,7 +28477,7 @@
         <v>2435</v>
       </c>
       <c r="L580" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28541,7 +28547,7 @@
         <v>2442</v>
       </c>
       <c r="L582" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="583" spans="1:12">
@@ -28611,7 +28617,7 @@
         <v>2502</v>
       </c>
       <c r="L584" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="585" spans="1:12">
@@ -28681,7 +28687,7 @@
         <v>2502</v>
       </c>
       <c r="L586" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28716,7 +28722,7 @@
         <v>2503</v>
       </c>
       <c r="L587" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="588" spans="1:12">
@@ -28789,7 +28795,7 @@
         <v>2465</v>
       </c>
       <c r="L589" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="590" spans="1:12">
@@ -28859,7 +28865,7 @@
         <v>2400</v>
       </c>
       <c r="L591" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="592" spans="1:12">
@@ -28894,7 +28900,7 @@
         <v>2411</v>
       </c>
       <c r="L592" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="593" spans="1:12">
@@ -28929,7 +28935,7 @@
         <v>2439</v>
       </c>
       <c r="L593" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -28964,7 +28970,7 @@
         <v>2414</v>
       </c>
       <c r="L594" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28999,7 +29005,7 @@
         <v>2418</v>
       </c>
       <c r="L595" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -29034,7 +29040,7 @@
         <v>2434</v>
       </c>
       <c r="L596" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="597" spans="1:12">
@@ -29069,7 +29075,7 @@
         <v>2404</v>
       </c>
       <c r="L597" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="598" spans="1:12">
@@ -29107,7 +29113,7 @@
         <v>2414</v>
       </c>
       <c r="L598" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="599" spans="1:12">
@@ -29177,7 +29183,7 @@
         <v>2397</v>
       </c>
       <c r="L600" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="601" spans="1:12">
@@ -29212,7 +29218,7 @@
         <v>2443</v>
       </c>
       <c r="L601" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="602" spans="1:12">
@@ -29250,7 +29256,7 @@
         <v>2428</v>
       </c>
       <c r="L602" t="s">
-        <v>2525</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29393,7 +29399,7 @@
         <v>2447</v>
       </c>
       <c r="L606" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="607" spans="1:12">
@@ -29428,7 +29434,7 @@
         <v>2447</v>
       </c>
       <c r="L607" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29463,7 +29469,7 @@
         <v>2439</v>
       </c>
       <c r="L608" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="609" spans="1:12">
@@ -29501,7 +29507,7 @@
         <v>2395</v>
       </c>
       <c r="L609" t="s">
-        <v>2542</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="610" spans="1:12">
@@ -29536,7 +29542,7 @@
         <v>2471</v>
       </c>
       <c r="L610" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="611" spans="1:12">
@@ -29606,7 +29612,7 @@
         <v>2444</v>
       </c>
       <c r="L612" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="613" spans="1:12">
@@ -29641,7 +29647,7 @@
         <v>2459</v>
       </c>
       <c r="L613" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="614" spans="1:12">
@@ -29711,7 +29717,7 @@
         <v>2400</v>
       </c>
       <c r="L615" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="616" spans="1:12">
@@ -29746,7 +29752,7 @@
         <v>2506</v>
       </c>
       <c r="L616" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="617" spans="1:12">
@@ -29781,7 +29787,7 @@
         <v>2432</v>
       </c>
       <c r="L617" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29816,7 +29822,7 @@
         <v>2424</v>
       </c>
       <c r="L618" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29851,7 +29857,7 @@
         <v>2405</v>
       </c>
       <c r="L619" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29921,7 +29927,7 @@
         <v>2460</v>
       </c>
       <c r="L621" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="622" spans="1:12">
@@ -29956,7 +29962,7 @@
         <v>2415</v>
       </c>
       <c r="L622" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="623" spans="1:12">
@@ -29991,7 +29997,7 @@
         <v>2415</v>
       </c>
       <c r="L623" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="624" spans="1:12">
@@ -30061,7 +30067,7 @@
         <v>2400</v>
       </c>
       <c r="L625" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -30099,7 +30105,7 @@
         <v>2507</v>
       </c>
       <c r="L626" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="627" spans="1:12">
@@ -30169,7 +30175,7 @@
         <v>2508</v>
       </c>
       <c r="L628" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30414,7 +30420,7 @@
         <v>2400</v>
       </c>
       <c r="L635" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30449,7 +30455,7 @@
         <v>2422</v>
       </c>
       <c r="L636" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="637" spans="1:12">
@@ -30519,7 +30525,7 @@
         <v>2469</v>
       </c>
       <c r="L638" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30554,7 +30560,7 @@
         <v>2510</v>
       </c>
       <c r="L639" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="640" spans="1:12">
@@ -30589,7 +30595,7 @@
         <v>2510</v>
       </c>
       <c r="L640" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -30624,7 +30630,7 @@
         <v>2510</v>
       </c>
       <c r="L641" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30659,7 +30665,7 @@
         <v>2510</v>
       </c>
       <c r="L642" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="643" spans="1:12">
@@ -30694,7 +30700,7 @@
         <v>2510</v>
       </c>
       <c r="L643" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="644" spans="1:12">
@@ -30729,7 +30735,7 @@
         <v>2510</v>
       </c>
       <c r="L644" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="645" spans="1:12">
@@ -30764,7 +30770,7 @@
         <v>2510</v>
       </c>
       <c r="L645" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -30799,7 +30805,7 @@
         <v>2510</v>
       </c>
       <c r="L646" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="647" spans="1:12">
@@ -30834,7 +30840,7 @@
         <v>2510</v>
       </c>
       <c r="L647" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="648" spans="1:12">
@@ -30869,7 +30875,7 @@
         <v>2510</v>
       </c>
       <c r="L648" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="649" spans="1:12">
@@ -30904,7 +30910,7 @@
         <v>2510</v>
       </c>
       <c r="L649" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="650" spans="1:12">
@@ -30939,7 +30945,7 @@
         <v>2510</v>
       </c>
       <c r="L650" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -30974,7 +30980,7 @@
         <v>2510</v>
       </c>
       <c r="L651" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31009,7 +31015,7 @@
         <v>2510</v>
       </c>
       <c r="L652" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31044,7 +31050,7 @@
         <v>2510</v>
       </c>
       <c r="L653" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="654" spans="1:12">
@@ -31079,7 +31085,7 @@
         <v>2510</v>
       </c>
       <c r="L654" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="655" spans="1:12">
@@ -31114,7 +31120,7 @@
         <v>2510</v>
       </c>
       <c r="L655" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31149,7 +31155,7 @@
         <v>2510</v>
       </c>
       <c r="L656" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="657" spans="1:12">
@@ -31187,7 +31193,7 @@
         <v>2511</v>
       </c>
       <c r="L657" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="658" spans="1:12">
@@ -31222,7 +31228,7 @@
         <v>2447</v>
       </c>
       <c r="L658" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="659" spans="1:12">
@@ -31257,7 +31263,7 @@
         <v>2404</v>
       </c>
       <c r="L659" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="660" spans="1:12">
@@ -31295,7 +31301,7 @@
         <v>2404</v>
       </c>
       <c r="L660" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="661" spans="1:12">
@@ -31330,7 +31336,7 @@
         <v>2495</v>
       </c>
       <c r="L661" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="662" spans="1:12">
@@ -31365,7 +31371,7 @@
         <v>2495</v>
       </c>
       <c r="L662" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="663" spans="1:12">
@@ -31400,7 +31406,7 @@
         <v>2495</v>
       </c>
       <c r="L663" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -31435,7 +31441,7 @@
         <v>2397</v>
       </c>
       <c r="L664" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="665" spans="1:12">
@@ -31467,7 +31473,7 @@
         <v>2512</v>
       </c>
       <c r="L665" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="666" spans="1:12">
@@ -31499,7 +31505,7 @@
         <v>2512</v>
       </c>
       <c r="L666" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="667" spans="1:12">
@@ -31534,7 +31540,7 @@
         <v>2447</v>
       </c>
       <c r="L667" t="s">
-        <v>2533</v>
+        <v>2516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-11 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -23188,7 +23188,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B430" t="s">
         <v>468</v>
@@ -23209,7 +23209,7 @@
         <v>1601</v>
       </c>
       <c r="I430" t="s">
-        <v>1717</v>
+        <v>1645</v>
       </c>
       <c r="J430" t="s">
         <v>2157</v>
@@ -24311,7 +24311,7 @@
     </row>
     <row r="462" spans="1:12">
       <c r="A462" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B462" t="s">
         <v>500</v>
@@ -24332,7 +24332,7 @@
         <v>1601</v>
       </c>
       <c r="I462" t="s">
-        <v>1717</v>
+        <v>1638</v>
       </c>
       <c r="J462" t="s">
         <v>2189</v>
@@ -24769,7 +24769,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B475" t="s">
         <v>513</v>
@@ -24790,7 +24790,7 @@
         <v>1601</v>
       </c>
       <c r="I475" t="s">
-        <v>1717</v>
+        <v>1626</v>
       </c>
       <c r="J475" t="s">
         <v>2202</v>
@@ -25892,7 +25892,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B507" t="s">
         <v>545</v>
@@ -25913,7 +25913,7 @@
         <v>1601</v>
       </c>
       <c r="I507" t="s">
-        <v>1717</v>
+        <v>1626</v>
       </c>
       <c r="J507" t="s">
         <v>2234</v>
@@ -25927,7 +25927,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B508" t="s">
         <v>546</v>
@@ -25948,7 +25948,7 @@
         <v>1601</v>
       </c>
       <c r="I508" t="s">
-        <v>1717</v>
+        <v>1626</v>
       </c>
       <c r="J508" t="s">
         <v>2235</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-12 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5152,13 +5152,13 @@
     <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>RAQUEL SILVA FERNANDES LYRA</t>
   </si>
   <si>
     <t>FERNANDA ZUCOLOTTO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
@@ -23345,7 +23345,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B435" t="s">
         <v>472</v>
@@ -23366,7 +23366,7 @@
         <v>1591</v>
       </c>
       <c r="I435" t="s">
-        <v>1653</v>
+        <v>1712</v>
       </c>
       <c r="J435" t="s">
         <v>2159</v>
@@ -23821,7 +23821,7 @@
         <v>1591</v>
       </c>
       <c r="I448" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J448" t="s">
         <v>2172</v>
@@ -23929,7 +23929,7 @@
         <v>1565</v>
       </c>
       <c r="I451" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J451" t="s">
         <v>2175</v>
@@ -24069,7 +24069,7 @@
         <v>1591</v>
       </c>
       <c r="I455" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J455" t="s">
         <v>2179</v>
@@ -24282,7 +24282,7 @@
         <v>1591</v>
       </c>
       <c r="I461" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J461" t="s">
         <v>2185</v>
@@ -24422,7 +24422,7 @@
         <v>1591</v>
       </c>
       <c r="I465" t="s">
-        <v>1714</v>
+        <v>1712</v>
       </c>
       <c r="J465" t="s">
         <v>2189</v>
@@ -24667,7 +24667,7 @@
         <v>1591</v>
       </c>
       <c r="I472" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J472" t="s">
         <v>2196</v>
@@ -24947,7 +24947,7 @@
         <v>1591</v>
       </c>
       <c r="I480" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J480" t="s">
         <v>2204</v>
@@ -25017,7 +25017,7 @@
         <v>1591</v>
       </c>
       <c r="I482" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J482" t="s">
         <v>2206</v>
@@ -25440,7 +25440,7 @@
         <v>1591</v>
       </c>
       <c r="I494" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J494" t="s">
         <v>2218</v>
@@ -26388,7 +26388,7 @@
         <v>1591</v>
       </c>
       <c r="I521" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J521" t="s">
         <v>2245</v>
@@ -26633,7 +26633,7 @@
         <v>1591</v>
       </c>
       <c r="I528" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J528" t="s">
         <v>2251</v>
@@ -27091,7 +27091,7 @@
         <v>1591</v>
       </c>
       <c r="I541" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J541" t="s">
         <v>2263</v>
@@ -27689,7 +27689,7 @@
         <v>1591</v>
       </c>
       <c r="I558" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J558" t="s">
         <v>2280</v>
@@ -27969,7 +27969,7 @@
         <v>1591</v>
       </c>
       <c r="I566" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J566" t="s">
         <v>2288</v>
@@ -28004,7 +28004,7 @@
         <v>1591</v>
       </c>
       <c r="I567" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J567" t="s">
         <v>2289</v>
@@ -28287,7 +28287,7 @@
         <v>1591</v>
       </c>
       <c r="I575" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J575" t="s">
         <v>2297</v>
@@ -28357,7 +28357,7 @@
         <v>1591</v>
       </c>
       <c r="I577" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J577" t="s">
         <v>2299</v>
@@ -28427,7 +28427,7 @@
         <v>1591</v>
       </c>
       <c r="I579" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J579" t="s">
         <v>2301</v>
@@ -28497,7 +28497,7 @@
         <v>1591</v>
       </c>
       <c r="I581" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J581" t="s">
         <v>2303</v>
@@ -29279,7 +29279,7 @@
         <v>1591</v>
       </c>
       <c r="I603" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J603" t="s">
         <v>2324</v>
@@ -29842,7 +29842,7 @@
         <v>1591</v>
       </c>
       <c r="I619" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J619" t="s">
         <v>2340</v>
@@ -29877,7 +29877,7 @@
         <v>1591</v>
       </c>
       <c r="I620" t="s">
-        <v>1714</v>
+        <v>1712</v>
       </c>
       <c r="J620" t="s">
         <v>2341</v>
@@ -29912,7 +29912,7 @@
         <v>1591</v>
       </c>
       <c r="I621" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J621" t="s">
         <v>2342</v>
@@ -30017,7 +30017,7 @@
         <v>1591</v>
       </c>
       <c r="I624" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J624" t="s">
         <v>2345</v>
@@ -30052,7 +30052,7 @@
         <v>1591</v>
       </c>
       <c r="I625" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J625" t="s">
         <v>2346</v>
@@ -30192,7 +30192,7 @@
         <v>1591</v>
       </c>
       <c r="I629" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J629" t="s">
         <v>2350</v>
@@ -30965,7 +30965,7 @@
         <v>1591</v>
       </c>
       <c r="I651" t="s">
-        <v>1714</v>
+        <v>1712</v>
       </c>
       <c r="J651" t="s">
         <v>2372</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-12 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -18138,7 +18138,7 @@
     </row>
     <row r="287" spans="1:12">
       <c r="A287" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B287" t="s">
         <v>325</v>
@@ -18159,7 +18159,7 @@
         <v>1584</v>
       </c>
       <c r="I287" t="s">
-        <v>1637</v>
+        <v>1675</v>
       </c>
       <c r="J287" t="s">
         <v>2007</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-13 04:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -97,6 +97,9 @@
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
   </si>
   <si>
@@ -106,9 +109,6 @@
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
@@ -4963,6 +4963,9 @@
     <t>SERGIO PEDRO LOPES</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>VICTOR AUGUSTO LOURO BERBARA</t>
   </si>
   <si>
@@ -5039,9 +5042,6 @@
   </si>
   <si>
     <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>REINALDO DE SOUZA MACHADO</t>
@@ -10532,7 +10532,7 @@
         <v>1729</v>
       </c>
       <c r="K69" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="L69" t="s">
         <v>2507</v>
@@ -12045,7 +12045,7 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B113" t="s">
         <v>151</v>
@@ -12066,7 +12066,7 @@
         <v>1584</v>
       </c>
       <c r="I113" t="s">
-        <v>1647</v>
+        <v>1649</v>
       </c>
       <c r="J113" t="s">
         <v>1836</v>
@@ -12206,7 +12206,7 @@
         <v>1584</v>
       </c>
       <c r="I117" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J117" t="s">
         <v>1840</v>
@@ -12220,7 +12220,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B118" t="s">
         <v>156</v>
@@ -12241,7 +12241,7 @@
         <v>1584</v>
       </c>
       <c r="I118" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="J118" t="s">
         <v>1841</v>
@@ -12381,7 +12381,7 @@
         <v>1584</v>
       </c>
       <c r="I122" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J122" t="s">
         <v>1845</v>
@@ -12416,7 +12416,7 @@
         <v>1584</v>
       </c>
       <c r="I123" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J123" t="s">
         <v>1846</v>
@@ -12605,7 +12605,7 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B129" t="s">
         <v>167</v>
@@ -12626,7 +12626,7 @@
         <v>1584</v>
       </c>
       <c r="I129" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J129" t="s">
         <v>1852</v>
@@ -12661,7 +12661,7 @@
         <v>1584</v>
       </c>
       <c r="I130" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J130" t="s">
         <v>1853</v>
@@ -12731,7 +12731,7 @@
         <v>1584</v>
       </c>
       <c r="I132" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J132" t="s">
         <v>1855</v>
@@ -12745,7 +12745,7 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B133" t="s">
         <v>171</v>
@@ -12871,7 +12871,7 @@
         <v>1584</v>
       </c>
       <c r="I136" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J136" t="s">
         <v>1859</v>
@@ -12941,7 +12941,7 @@
         <v>1584</v>
       </c>
       <c r="I138" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J138" t="s">
         <v>1861</v>
@@ -12955,7 +12955,7 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B139" t="s">
         <v>177</v>
@@ -13116,7 +13116,7 @@
         <v>1584</v>
       </c>
       <c r="I143" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J143" t="s">
         <v>1866</v>
@@ -13151,7 +13151,7 @@
         <v>1584</v>
       </c>
       <c r="I144" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J144" t="s">
         <v>1867</v>
@@ -13256,7 +13256,7 @@
         <v>1584</v>
       </c>
       <c r="I147" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J147" t="s">
         <v>1870</v>
@@ -13466,7 +13466,7 @@
         <v>1584</v>
       </c>
       <c r="I153" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J153" t="s">
         <v>1875</v>
@@ -13501,7 +13501,7 @@
         <v>1584</v>
       </c>
       <c r="I154" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J154" t="s">
         <v>1876</v>
@@ -13571,7 +13571,7 @@
         <v>1584</v>
       </c>
       <c r="I156" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J156" t="s">
         <v>1878</v>
@@ -13711,7 +13711,7 @@
         <v>1584</v>
       </c>
       <c r="I160" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J160" t="s">
         <v>1882</v>
@@ -13746,7 +13746,7 @@
         <v>1584</v>
       </c>
       <c r="I161" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J161" t="s">
         <v>1883</v>
@@ -13781,7 +13781,7 @@
         <v>1584</v>
       </c>
       <c r="I162" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J162" t="s">
         <v>1884</v>
@@ -13886,7 +13886,7 @@
         <v>1584</v>
       </c>
       <c r="I165" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J165" t="s">
         <v>1887</v>
@@ -13956,7 +13956,7 @@
         <v>1584</v>
       </c>
       <c r="I167" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J167" t="s">
         <v>1889</v>
@@ -14061,7 +14061,7 @@
         <v>1584</v>
       </c>
       <c r="I170" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J170" t="s">
         <v>1892</v>
@@ -14166,7 +14166,7 @@
         <v>1584</v>
       </c>
       <c r="I173" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J173" t="s">
         <v>1895</v>
@@ -14341,7 +14341,7 @@
         <v>1584</v>
       </c>
       <c r="I178" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J178" t="s">
         <v>1900</v>
@@ -14516,7 +14516,7 @@
         <v>1584</v>
       </c>
       <c r="I183" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J183" t="s">
         <v>1905</v>
@@ -14554,7 +14554,7 @@
         <v>1588</v>
       </c>
       <c r="I184" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J184" t="s">
         <v>1906</v>
@@ -14624,7 +14624,7 @@
         <v>1584</v>
       </c>
       <c r="I186" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="J186" t="s">
         <v>1908</v>
@@ -14694,7 +14694,7 @@
         <v>1584</v>
       </c>
       <c r="I188" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J188" t="s">
         <v>1910</v>
@@ -14764,7 +14764,7 @@
         <v>1584</v>
       </c>
       <c r="I190" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J190" t="s">
         <v>1912</v>
@@ -14799,7 +14799,7 @@
         <v>1584</v>
       </c>
       <c r="I191" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J191" t="s">
         <v>1913</v>
@@ -14834,7 +14834,7 @@
         <v>1584</v>
       </c>
       <c r="I192" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J192" t="s">
         <v>1914</v>
@@ -14848,7 +14848,7 @@
     </row>
     <row r="193" spans="1:12">
       <c r="A193" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B193" t="s">
         <v>231</v>
@@ -14869,7 +14869,7 @@
         <v>1584</v>
       </c>
       <c r="I193" t="s">
-        <v>1675</v>
+        <v>1649</v>
       </c>
       <c r="J193" t="s">
         <v>1915</v>
@@ -15429,7 +15429,7 @@
         <v>1584</v>
       </c>
       <c r="I209" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J209" t="s">
         <v>1931</v>
@@ -15604,7 +15604,7 @@
         <v>1584</v>
       </c>
       <c r="I214" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J214" t="s">
         <v>1936</v>
@@ -16213,7 +16213,7 @@
     </row>
     <row r="232" spans="1:12">
       <c r="A232" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B232" t="s">
         <v>270</v>
@@ -16584,7 +16584,7 @@
         <v>1584</v>
       </c>
       <c r="I242" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J242" t="s">
         <v>1962</v>
@@ -16724,7 +16724,7 @@
         <v>1584</v>
       </c>
       <c r="I246" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J246" t="s">
         <v>1966</v>
@@ -16794,7 +16794,7 @@
         <v>1584</v>
       </c>
       <c r="I248" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J248" t="s">
         <v>1968</v>
@@ -17459,7 +17459,7 @@
         <v>1584</v>
       </c>
       <c r="I267" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J267" t="s">
         <v>1987</v>
@@ -17809,7 +17809,7 @@
         <v>1584</v>
       </c>
       <c r="I277" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J277" t="s">
         <v>1997</v>
@@ -17984,7 +17984,7 @@
         <v>1584</v>
       </c>
       <c r="I282" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J282" t="s">
         <v>2002</v>
@@ -18138,7 +18138,7 @@
     </row>
     <row r="287" spans="1:12">
       <c r="A287" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B287" t="s">
         <v>325</v>
@@ -18159,7 +18159,7 @@
         <v>1584</v>
       </c>
       <c r="I287" t="s">
-        <v>1675</v>
+        <v>1649</v>
       </c>
       <c r="J287" t="s">
         <v>2007</v>
@@ -18439,7 +18439,7 @@
         <v>1584</v>
       </c>
       <c r="I295" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J295" t="s">
         <v>2015</v>
@@ -18789,7 +18789,7 @@
         <v>1584</v>
       </c>
       <c r="I305" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J305" t="s">
         <v>2025</v>
@@ -19037,7 +19037,7 @@
         <v>1589</v>
       </c>
       <c r="I312" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J312" t="s">
         <v>2032</v>
@@ -19226,7 +19226,7 @@
     </row>
     <row r="318" spans="1:12">
       <c r="A318" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B318" t="s">
         <v>356</v>
@@ -19527,7 +19527,7 @@
         <v>1584</v>
       </c>
       <c r="I326" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J326" t="s">
         <v>2046</v>
@@ -19737,7 +19737,7 @@
         <v>1584</v>
       </c>
       <c r="I332" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J332" t="s">
         <v>2052</v>
@@ -19947,7 +19947,7 @@
         <v>1584</v>
       </c>
       <c r="I338" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J338" t="s">
         <v>2058</v>
@@ -20297,7 +20297,7 @@
         <v>1584</v>
       </c>
       <c r="I348" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J348" t="s">
         <v>2068</v>
@@ -20507,7 +20507,7 @@
         <v>1584</v>
       </c>
       <c r="I354" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J354" t="s">
         <v>2074</v>
@@ -20536,7 +20536,7 @@
         <v>91</v>
       </c>
       <c r="F355" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="G355" t="s">
         <v>1584</v>
@@ -20758,7 +20758,7 @@
         <v>1590</v>
       </c>
       <c r="I361" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J361" t="s">
         <v>2081</v>
@@ -20968,7 +20968,7 @@
         <v>1584</v>
       </c>
       <c r="I367" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J367" t="s">
         <v>2087</v>
@@ -21248,7 +21248,7 @@
         <v>1584</v>
       </c>
       <c r="I375" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J375" t="s">
         <v>2095</v>
@@ -21738,7 +21738,7 @@
         <v>1584</v>
       </c>
       <c r="I389" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J389" t="s">
         <v>2109</v>
@@ -21983,7 +21983,7 @@
         <v>1584</v>
       </c>
       <c r="I396" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J396" t="s">
         <v>2116</v>
@@ -22438,7 +22438,7 @@
         <v>1584</v>
       </c>
       <c r="I409" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J409" t="s">
         <v>2129</v>
@@ -22998,7 +22998,7 @@
         <v>1584</v>
       </c>
       <c r="I425" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J425" t="s">
         <v>2145</v>
@@ -23068,7 +23068,7 @@
         <v>1584</v>
       </c>
       <c r="I427" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J427" t="s">
         <v>2147</v>
@@ -23806,7 +23806,7 @@
         <v>1584</v>
       </c>
       <c r="I448" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J448" t="s">
         <v>2168</v>
@@ -24229,7 +24229,7 @@
         <v>1584</v>
       </c>
       <c r="I460" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J460" t="s">
         <v>2180</v>
@@ -24897,7 +24897,7 @@
         <v>1584</v>
       </c>
       <c r="I479" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J479" t="s">
         <v>2199</v>
@@ -24932,7 +24932,7 @@
         <v>1584</v>
       </c>
       <c r="I480" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J480" t="s">
         <v>2200</v>
@@ -24967,7 +24967,7 @@
         <v>1584</v>
       </c>
       <c r="I481" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J481" t="s">
         <v>2201</v>
@@ -25037,7 +25037,7 @@
         <v>1584</v>
       </c>
       <c r="I483" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J483" t="s">
         <v>2203</v>
@@ -25072,7 +25072,7 @@
         <v>1584</v>
       </c>
       <c r="I484" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J484" t="s">
         <v>2204</v>
@@ -25107,7 +25107,7 @@
         <v>1584</v>
       </c>
       <c r="I485" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J485" t="s">
         <v>2205</v>
@@ -25387,7 +25387,7 @@
         <v>1584</v>
       </c>
       <c r="I493" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J493" t="s">
         <v>2213</v>
@@ -25492,7 +25492,7 @@
         <v>1584</v>
       </c>
       <c r="I496" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J496" t="s">
         <v>2216</v>
@@ -26055,7 +26055,7 @@
         <v>1584</v>
       </c>
       <c r="I512" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J512" t="s">
         <v>2232</v>
@@ -26443,7 +26443,7 @@
         <v>1584</v>
       </c>
       <c r="I523" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J523" t="s">
         <v>2242</v>
@@ -26478,7 +26478,7 @@
         <v>1584</v>
       </c>
       <c r="I524" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J524" t="s">
         <v>2242</v>
@@ -26548,7 +26548,7 @@
         <v>1584</v>
       </c>
       <c r="I526" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J526" t="s">
         <v>2244</v>
@@ -26772,7 +26772,7 @@
     </row>
     <row r="533" spans="1:12">
       <c r="A533" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B533" t="s">
         <v>570</v>
@@ -27265,7 +27265,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B547" t="s">
         <v>584</v>
@@ -27286,7 +27286,7 @@
         <v>1584</v>
       </c>
       <c r="I547" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J547" t="s">
         <v>2265</v>
@@ -28339,7 +28339,7 @@
         <v>1584</v>
       </c>
       <c r="I577" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J577" t="s">
         <v>2295</v>
@@ -28444,7 +28444,7 @@
         <v>1584</v>
       </c>
       <c r="I580" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J580" t="s">
         <v>2298</v>
@@ -28838,7 +28838,7 @@
         <v>1584</v>
       </c>
       <c r="I591" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J591" t="s">
         <v>2308</v>
@@ -29156,7 +29156,7 @@
         <v>1584</v>
       </c>
       <c r="I600" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J600" t="s">
         <v>2317</v>
@@ -29170,7 +29170,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B601" t="s">
         <v>638</v>
@@ -29226,7 +29226,7 @@
         <v>1584</v>
       </c>
       <c r="I602" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J602" t="s">
         <v>2319</v>
@@ -29261,7 +29261,7 @@
         <v>1584</v>
       </c>
       <c r="I603" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J603" t="s">
         <v>2320</v>
@@ -29593,7 +29593,7 @@
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B613" t="s">
         <v>650</v>
@@ -29614,7 +29614,7 @@
         <v>1584</v>
       </c>
       <c r="I613" t="s">
-        <v>1675</v>
+        <v>1649</v>
       </c>
       <c r="J613" t="s">
         <v>2330</v>
@@ -29838,7 +29838,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B620" t="s">
         <v>657</v>
@@ -29873,7 +29873,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B621" t="s">
         <v>658</v>
@@ -29943,7 +29943,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B623" t="s">
         <v>660</v>
@@ -29978,7 +29978,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B624" t="s">
         <v>661</v>
@@ -30013,7 +30013,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B625" t="s">
         <v>662</v>
@@ -30048,7 +30048,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B626" t="s">
         <v>663</v>
@@ -30083,7 +30083,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B627" t="s">
         <v>664</v>
@@ -30118,7 +30118,7 @@
     </row>
     <row r="628" spans="1:12">
       <c r="A628" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B628" t="s">
         <v>665</v>
@@ -30153,7 +30153,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B629" t="s">
         <v>666</v>
@@ -30188,7 +30188,7 @@
     </row>
     <row r="630" spans="1:12">
       <c r="A630" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B630" t="s">
         <v>667</v>
@@ -30223,7 +30223,7 @@
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B631" t="s">
         <v>668</v>
@@ -30258,7 +30258,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B632" t="s">
         <v>669</v>
@@ -30293,7 +30293,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B633" t="s">
         <v>670</v>
@@ -30328,7 +30328,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B634" t="s">
         <v>671</v>
@@ -30363,7 +30363,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B635" t="s">
         <v>672</v>
@@ -30398,7 +30398,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B636" t="s">
         <v>673</v>
@@ -30433,7 +30433,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B637" t="s">
         <v>674</v>
@@ -30468,7 +30468,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B638" t="s">
         <v>675</v>
@@ -30503,7 +30503,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B639" t="s">
         <v>676</v>
@@ -30538,7 +30538,7 @@
     </row>
     <row r="640" spans="1:12">
       <c r="A640" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B640" t="s">
         <v>677</v>
@@ -30573,7 +30573,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B641" t="s">
         <v>678</v>
@@ -30667,7 +30667,7 @@
         <v>1584</v>
       </c>
       <c r="I643" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J643" t="s">
         <v>2360</v>
@@ -30681,7 +30681,7 @@
     </row>
     <row r="644" spans="1:12">
       <c r="A644" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B644" t="s">
         <v>681</v>
@@ -30702,7 +30702,7 @@
         <v>1584</v>
       </c>
       <c r="I644" t="s">
-        <v>1675</v>
+        <v>1649</v>
       </c>
       <c r="J644" t="s">
         <v>2361</v>
@@ -30964,7 +30964,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B652" t="s">
         <v>689</v>
@@ -30999,7 +30999,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B653" t="s">
         <v>690</v>
@@ -31107,7 +31107,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B656" t="s">
         <v>693</v>
@@ -31145,7 +31145,7 @@
     </row>
     <row r="657" spans="1:12">
       <c r="A657" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B657" t="s">
         <v>694</v>
@@ -31166,7 +31166,7 @@
         <v>1584</v>
       </c>
       <c r="I657" t="s">
-        <v>1675</v>
+        <v>1649</v>
       </c>
       <c r="J657" t="s">
         <v>2372</v>
@@ -31215,7 +31215,7 @@
     </row>
     <row r="659" spans="1:12">
       <c r="A659" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B659" t="s">
         <v>696</v>
@@ -31247,7 +31247,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B660" t="s">
         <v>697</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-14 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -31057,7 +31057,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B652" t="s">
         <v>689</v>
@@ -31081,7 +31081,7 @@
         <v>1622</v>
       </c>
       <c r="I652" t="s">
-        <v>1630</v>
+        <v>1710</v>
       </c>
       <c r="J652" t="s">
         <v>2389</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-14 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6728" uniqueCount="2610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6728" uniqueCount="2609">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7813,7 +7813,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
@@ -7831,19 +7831,16 @@
     <t>AVALIAÇÃO DE IMÓVEIS,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ECONOMIA</t>
-  </si>
-  <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMIA,SAÚDE MENTAL,PSICOLOGIA,ORÇAMENTO,URBANISMO,SAÚDE,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>ASSISTÊNCIA SOCIAL,ORÇAMENTO,SAÚDE,PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,URBANISMO,MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ECONOMIA,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -31090,7 +31087,7 @@
         <v>2496</v>
       </c>
       <c r="L652" t="s">
-        <v>2592</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31700,7 +31697,7 @@
         <v>2532</v>
       </c>
       <c r="L669" t="s">
-        <v>2608</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="670" spans="1:12">
@@ -31732,7 +31729,7 @@
         <v>2532</v>
       </c>
       <c r="L670" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-14 16:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6757" uniqueCount="2620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6757" uniqueCount="2621">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7864,16 +7864,19 @@
     <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>ECONOMIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,PSICOLOGIA,SAÚDE,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,URBANISMO,ECONOMIA,SAÚDE MENTAL,ORÇAMENTO</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,SAÚDE MENTAL,SAÚDE,ORÇAMENTO,URBANISMO,ASSISTÊNCIA SOCIAL,ECONOMIA</t>
   </si>
 </sst>
 </file>
@@ -28756,7 +28759,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B586" t="s">
         <v>624</v>
@@ -28777,7 +28780,7 @@
         <v>1611</v>
       </c>
       <c r="I586" t="s">
-        <v>1733</v>
+        <v>1637</v>
       </c>
       <c r="J586" t="s">
         <v>2332</v>
@@ -31047,7 +31050,7 @@
         <v>2424</v>
       </c>
       <c r="L650" t="s">
-        <v>2602</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31552,7 +31555,7 @@
         <v>2496</v>
       </c>
       <c r="L664" t="s">
-        <v>2602</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="665" spans="1:12">
@@ -31832,7 +31835,7 @@
         <v>2542</v>
       </c>
       <c r="L672" t="s">
-        <v>2618</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="673" spans="1:12">
@@ -31864,7 +31867,7 @@
         <v>2542</v>
       </c>
       <c r="L673" t="s">
-        <v>2619</v>
+        <v>2620</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-14 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6748" uniqueCount="2617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6748" uniqueCount="2616">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -4927,6 +4927,9 @@
     <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,MARINA DE AQUINO PARREIRA XAVIER,PEDRO DE OLIVEIRA PERES</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>JULIANA MARTINS BAHIENSE</t>
   </si>
   <si>
@@ -4990,7 +4993,7 @@
     <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
   </si>
   <si>
-    <t>EDIWAN SOUSA DA SILVA, _SEM USUARIO ATRIBUIDO</t>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
     <t>ROSEMARY PROVENZANO THAMI</t>
@@ -5251,9 +5254,6 @@
     <t>IZABELLA KRAICHETE LENTINO BARANDIER</t>
   </si>
   <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
     <t>GABRIEL GERON MOREIRA</t>
   </si>
   <si>
@@ -7801,7 +7801,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7861,10 +7861,7 @@
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ORÇAMENTO,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,URBANISMO,AVALIAÇÃO DE IMÓVEIS,ASSISTÊNCIA SOCIAL,ECONOMIA,MOBILIDADE E TRANSPORTE,SAÚDE,PSICOLOGIA</t>
+    <t>ECONOMIA,SAÚDE,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,PSICOLOGIA,SAÚDE MENTAL,URBANISMO,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -8601,7 +8598,7 @@
         <v>1607</v>
       </c>
       <c r="I11" t="s">
-        <v>1634</v>
+        <v>1637</v>
       </c>
       <c r="J11" t="s">
         <v>1762</v>
@@ -8636,7 +8633,7 @@
         <v>1607</v>
       </c>
       <c r="I12" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J12" t="s">
         <v>1763</v>
@@ -8706,7 +8703,7 @@
         <v>1607</v>
       </c>
       <c r="I14" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J14" t="s">
         <v>1765</v>
@@ -8776,7 +8773,7 @@
         <v>1607</v>
       </c>
       <c r="I16" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J16" t="s">
         <v>1767</v>
@@ -9091,7 +9088,7 @@
         <v>1607</v>
       </c>
       <c r="I25" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J25" t="s">
         <v>1776</v>
@@ -9161,7 +9158,7 @@
         <v>1607</v>
       </c>
       <c r="I27" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="J27" t="s">
         <v>1778</v>
@@ -9409,7 +9406,7 @@
         <v>1607</v>
       </c>
       <c r="I34" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J34" t="s">
         <v>1785</v>
@@ -9514,7 +9511,7 @@
         <v>1607</v>
       </c>
       <c r="I37" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J37" t="s">
         <v>1788</v>
@@ -9689,7 +9686,7 @@
         <v>1607</v>
       </c>
       <c r="I42" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="J42" t="s">
         <v>1792</v>
@@ -9759,7 +9756,7 @@
         <v>1607</v>
       </c>
       <c r="I44" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J44" t="s">
         <v>1794</v>
@@ -9829,7 +9826,7 @@
         <v>1607</v>
       </c>
       <c r="I46" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J46" t="s">
         <v>1796</v>
@@ -9864,7 +9861,7 @@
         <v>1607</v>
       </c>
       <c r="I47" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="J47" t="s">
         <v>1797</v>
@@ -9934,7 +9931,7 @@
         <v>1607</v>
       </c>
       <c r="I49" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="J49" t="s">
         <v>1799</v>
@@ -9969,7 +9966,7 @@
         <v>1607</v>
       </c>
       <c r="I50" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J50" t="s">
         <v>1800</v>
@@ -10004,7 +10001,7 @@
         <v>1607</v>
       </c>
       <c r="I51" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="J51" t="s">
         <v>1801</v>
@@ -10074,7 +10071,7 @@
         <v>1607</v>
       </c>
       <c r="I53" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J53" t="s">
         <v>1803</v>
@@ -10109,7 +10106,7 @@
         <v>1607</v>
       </c>
       <c r="I54" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J54" t="s">
         <v>1804</v>
@@ -10144,7 +10141,7 @@
         <v>1607</v>
       </c>
       <c r="I55" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="J55" t="s">
         <v>1805</v>
@@ -10214,7 +10211,7 @@
         <v>1607</v>
       </c>
       <c r="I57" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J57" t="s">
         <v>1807</v>
@@ -10424,7 +10421,7 @@
         <v>1607</v>
       </c>
       <c r="I63" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="J63" t="s">
         <v>1813</v>
@@ -10459,7 +10456,7 @@
         <v>1607</v>
       </c>
       <c r="I64" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="J64" t="s">
         <v>1814</v>
@@ -10494,7 +10491,7 @@
         <v>1607</v>
       </c>
       <c r="I65" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J65" t="s">
         <v>1815</v>
@@ -10564,7 +10561,7 @@
         <v>1607</v>
       </c>
       <c r="I67" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J67" t="s">
         <v>1816</v>
@@ -10599,7 +10596,7 @@
         <v>1607</v>
       </c>
       <c r="I68" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="J68" t="s">
         <v>1817</v>
@@ -10669,7 +10666,7 @@
         <v>1607</v>
       </c>
       <c r="I70" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J70" t="s">
         <v>1819</v>
@@ -10704,7 +10701,7 @@
         <v>1607</v>
       </c>
       <c r="I71" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J71" t="s">
         <v>1820</v>
@@ -10739,7 +10736,7 @@
         <v>1607</v>
       </c>
       <c r="I72" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J72" t="s">
         <v>1821</v>
@@ -10774,7 +10771,7 @@
         <v>1607</v>
       </c>
       <c r="I73" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="J73" t="s">
         <v>1822</v>
@@ -10809,7 +10806,7 @@
         <v>1607</v>
       </c>
       <c r="I74" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="J74" t="s">
         <v>1823</v>
@@ -10844,7 +10841,7 @@
         <v>1607</v>
       </c>
       <c r="I75" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="J75" t="s">
         <v>1824</v>
@@ -10914,7 +10911,7 @@
         <v>1607</v>
       </c>
       <c r="I77" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J77" t="s">
         <v>1826</v>
@@ -10949,7 +10946,7 @@
         <v>1607</v>
       </c>
       <c r="I78" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="J78" t="s">
         <v>1827</v>
@@ -11089,7 +11086,7 @@
         <v>1607</v>
       </c>
       <c r="I82" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J82" t="s">
         <v>1831</v>
@@ -11159,7 +11156,7 @@
         <v>1607</v>
       </c>
       <c r="I84" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J84" t="s">
         <v>1833</v>
@@ -11264,7 +11261,7 @@
         <v>1607</v>
       </c>
       <c r="I87" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="J87" t="s">
         <v>1836</v>
@@ -11334,7 +11331,7 @@
         <v>1607</v>
       </c>
       <c r="I89" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="J89" t="s">
         <v>1838</v>
@@ -11404,7 +11401,7 @@
         <v>1607</v>
       </c>
       <c r="I91" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J91" t="s">
         <v>1840</v>
@@ -11439,7 +11436,7 @@
         <v>1607</v>
       </c>
       <c r="I92" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="J92" t="s">
         <v>1841</v>
@@ -11474,7 +11471,7 @@
         <v>1607</v>
       </c>
       <c r="I93" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J93" t="s">
         <v>1842</v>
@@ -11509,7 +11506,7 @@
         <v>1607</v>
       </c>
       <c r="I94" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="J94" t="s">
         <v>1843</v>
@@ -11544,7 +11541,7 @@
         <v>1607</v>
       </c>
       <c r="I95" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J95" t="s">
         <v>1844</v>
@@ -11579,7 +11576,7 @@
         <v>1607</v>
       </c>
       <c r="I96" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="J96" t="s">
         <v>1845</v>
@@ -11614,7 +11611,7 @@
         <v>1607</v>
       </c>
       <c r="I97" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J97" t="s">
         <v>1846</v>
@@ -11684,7 +11681,7 @@
         <v>1607</v>
       </c>
       <c r="I99" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J99" t="s">
         <v>1848</v>
@@ -11719,7 +11716,7 @@
         <v>1607</v>
       </c>
       <c r="I100" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="J100" t="s">
         <v>1849</v>
@@ -11754,7 +11751,7 @@
         <v>1607</v>
       </c>
       <c r="I101" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="J101" t="s">
         <v>1850</v>
@@ -11789,7 +11786,7 @@
         <v>1607</v>
       </c>
       <c r="I102" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J102" t="s">
         <v>1851</v>
@@ -11824,7 +11821,7 @@
         <v>1607</v>
       </c>
       <c r="I103" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="J103" t="s">
         <v>1852</v>
@@ -11894,7 +11891,7 @@
         <v>1607</v>
       </c>
       <c r="I105" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J105" t="s">
         <v>1854</v>
@@ -11964,7 +11961,7 @@
         <v>1607</v>
       </c>
       <c r="I107" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="J107" t="s">
         <v>1856</v>
@@ -12139,7 +12136,7 @@
         <v>1607</v>
       </c>
       <c r="I112" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J112" t="s">
         <v>1861</v>
@@ -12174,7 +12171,7 @@
         <v>1607</v>
       </c>
       <c r="I113" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="J113" t="s">
         <v>1862</v>
@@ -12314,7 +12311,7 @@
         <v>1607</v>
       </c>
       <c r="I117" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J117" t="s">
         <v>1866</v>
@@ -12349,7 +12346,7 @@
         <v>1607</v>
       </c>
       <c r="I118" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="J118" t="s">
         <v>1867</v>
@@ -12454,7 +12451,7 @@
         <v>1607</v>
       </c>
       <c r="I121" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="J121" t="s">
         <v>1870</v>
@@ -12524,7 +12521,7 @@
         <v>1607</v>
       </c>
       <c r="I123" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J123" t="s">
         <v>1872</v>
@@ -12559,7 +12556,7 @@
         <v>1607</v>
       </c>
       <c r="I124" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="J124" t="s">
         <v>1873</v>
@@ -12594,7 +12591,7 @@
         <v>1607</v>
       </c>
       <c r="I125" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="J125" t="s">
         <v>1874</v>
@@ -12664,7 +12661,7 @@
         <v>1607</v>
       </c>
       <c r="I127" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="J127" t="s">
         <v>1876</v>
@@ -12804,7 +12801,7 @@
         <v>1607</v>
       </c>
       <c r="I131" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="J131" t="s">
         <v>1880</v>
@@ -12874,7 +12871,7 @@
         <v>1607</v>
       </c>
       <c r="I133" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="J133" t="s">
         <v>1882</v>
@@ -13049,7 +13046,7 @@
         <v>1607</v>
       </c>
       <c r="I138" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J138" t="s">
         <v>1887</v>
@@ -13084,7 +13081,7 @@
         <v>1607</v>
       </c>
       <c r="I139" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J139" t="s">
         <v>1888</v>
@@ -13119,7 +13116,7 @@
         <v>1607</v>
       </c>
       <c r="I140" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="J140" t="s">
         <v>1889</v>
@@ -13189,7 +13186,7 @@
         <v>1607</v>
       </c>
       <c r="I142" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="J142" t="s">
         <v>1891</v>
@@ -13399,7 +13396,7 @@
         <v>1607</v>
       </c>
       <c r="I148" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="J148" t="s">
         <v>1896</v>
@@ -13434,7 +13431,7 @@
         <v>1607</v>
       </c>
       <c r="I149" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J149" t="s">
         <v>1897</v>
@@ -13504,7 +13501,7 @@
         <v>1607</v>
       </c>
       <c r="I151" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J151" t="s">
         <v>1899</v>
@@ -13644,7 +13641,7 @@
         <v>1607</v>
       </c>
       <c r="I155" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="J155" t="s">
         <v>1903</v>
@@ -13679,7 +13676,7 @@
         <v>1607</v>
       </c>
       <c r="I156" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="J156" t="s">
         <v>1904</v>
@@ -13784,7 +13781,7 @@
         <v>1607</v>
       </c>
       <c r="I159" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="J159" t="s">
         <v>1907</v>
@@ -13854,7 +13851,7 @@
         <v>1607</v>
       </c>
       <c r="I161" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J161" t="s">
         <v>1909</v>
@@ -13924,7 +13921,7 @@
         <v>1607</v>
       </c>
       <c r="I163" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="J163" t="s">
         <v>1911</v>
@@ -13959,7 +13956,7 @@
         <v>1607</v>
       </c>
       <c r="I164" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="J164" t="s">
         <v>1912</v>
@@ -14029,7 +14026,7 @@
         <v>1607</v>
       </c>
       <c r="I166" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J166" t="s">
         <v>1914</v>
@@ -14064,7 +14061,7 @@
         <v>1607</v>
       </c>
       <c r="I167" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J167" t="s">
         <v>1915</v>
@@ -14239,7 +14236,7 @@
         <v>1607</v>
       </c>
       <c r="I172" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J172" t="s">
         <v>1920</v>
@@ -14344,7 +14341,7 @@
         <v>1607</v>
       </c>
       <c r="I175" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J175" t="s">
         <v>1923</v>
@@ -14414,7 +14411,7 @@
         <v>1607</v>
       </c>
       <c r="I177" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="J177" t="s">
         <v>1925</v>
@@ -14452,7 +14449,7 @@
         <v>1610</v>
       </c>
       <c r="I178" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J178" t="s">
         <v>1926</v>
@@ -14522,7 +14519,7 @@
         <v>1607</v>
       </c>
       <c r="I180" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="J180" t="s">
         <v>1928</v>
@@ -14592,7 +14589,7 @@
         <v>1607</v>
       </c>
       <c r="I182" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="J182" t="s">
         <v>1930</v>
@@ -14662,7 +14659,7 @@
         <v>1607</v>
       </c>
       <c r="I184" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="J184" t="s">
         <v>1932</v>
@@ -14697,7 +14694,7 @@
         <v>1607</v>
       </c>
       <c r="I185" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J185" t="s">
         <v>1933</v>
@@ -14732,7 +14729,7 @@
         <v>1607</v>
       </c>
       <c r="I186" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="J186" t="s">
         <v>1934</v>
@@ -14767,7 +14764,7 @@
         <v>1607</v>
       </c>
       <c r="I187" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J187" t="s">
         <v>1935</v>
@@ -14802,7 +14799,7 @@
         <v>1607</v>
       </c>
       <c r="I188" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J188" t="s">
         <v>1936</v>
@@ -14837,7 +14834,7 @@
         <v>1607</v>
       </c>
       <c r="I189" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="J189" t="s">
         <v>1937</v>
@@ -14872,7 +14869,7 @@
         <v>1607</v>
       </c>
       <c r="I190" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J190" t="s">
         <v>1938</v>
@@ -14907,7 +14904,7 @@
         <v>1607</v>
       </c>
       <c r="I191" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J191" t="s">
         <v>1939</v>
@@ -14942,7 +14939,7 @@
         <v>1607</v>
       </c>
       <c r="I192" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="J192" t="s">
         <v>1940</v>
@@ -15082,7 +15079,7 @@
         <v>1607</v>
       </c>
       <c r="I196" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="J196" t="s">
         <v>1944</v>
@@ -15117,7 +15114,7 @@
         <v>1607</v>
       </c>
       <c r="I197" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J197" t="s">
         <v>1945</v>
@@ -15152,7 +15149,7 @@
         <v>1607</v>
       </c>
       <c r="I198" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="J198" t="s">
         <v>1946</v>
@@ -15292,7 +15289,7 @@
         <v>1607</v>
       </c>
       <c r="I202" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="J202" t="s">
         <v>1950</v>
@@ -15397,7 +15394,7 @@
         <v>1607</v>
       </c>
       <c r="I205" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="J205" t="s">
         <v>1953</v>
@@ -15432,7 +15429,7 @@
         <v>1607</v>
       </c>
       <c r="I206" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="J206" t="s">
         <v>1954</v>
@@ -15467,7 +15464,7 @@
         <v>1607</v>
       </c>
       <c r="I207" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="J207" t="s">
         <v>1955</v>
@@ -16062,7 +16059,7 @@
         <v>1607</v>
       </c>
       <c r="I224" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J224" t="s">
         <v>1755</v>
@@ -16132,7 +16129,7 @@
         <v>1607</v>
       </c>
       <c r="I226" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="J226" t="s">
         <v>1972</v>
@@ -16447,7 +16444,7 @@
         <v>1607</v>
       </c>
       <c r="I235" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J235" t="s">
         <v>1981</v>
@@ -16517,7 +16514,7 @@
         <v>1607</v>
       </c>
       <c r="I237" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J237" t="s">
         <v>1983</v>
@@ -16587,7 +16584,7 @@
         <v>1607</v>
       </c>
       <c r="I239" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J239" t="s">
         <v>1985</v>
@@ -16622,7 +16619,7 @@
         <v>1607</v>
       </c>
       <c r="I240" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J240" t="s">
         <v>1986</v>
@@ -16657,7 +16654,7 @@
         <v>1607</v>
       </c>
       <c r="I241" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J241" t="s">
         <v>1987</v>
@@ -16727,7 +16724,7 @@
         <v>1607</v>
       </c>
       <c r="I243" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="J243" t="s">
         <v>1989</v>
@@ -16867,7 +16864,7 @@
         <v>1607</v>
       </c>
       <c r="I247" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J247" t="s">
         <v>1993</v>
@@ -16937,7 +16934,7 @@
         <v>1607</v>
       </c>
       <c r="I249" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="J249" t="s">
         <v>1995</v>
@@ -17007,7 +17004,7 @@
         <v>1607</v>
       </c>
       <c r="I251" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="J251" t="s">
         <v>1997</v>
@@ -17357,7 +17354,7 @@
         <v>1607</v>
       </c>
       <c r="I261" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J261" t="s">
         <v>2007</v>
@@ -17427,7 +17424,7 @@
         <v>1607</v>
       </c>
       <c r="I263" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="J263" t="s">
         <v>2009</v>
@@ -17497,7 +17494,7 @@
         <v>1607</v>
       </c>
       <c r="I265" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J265" t="s">
         <v>2011</v>
@@ -17532,7 +17529,7 @@
         <v>1607</v>
       </c>
       <c r="I266" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J266" t="s">
         <v>2012</v>
@@ -17567,7 +17564,7 @@
         <v>1607</v>
       </c>
       <c r="I267" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="J267" t="s">
         <v>2013</v>
@@ -17602,7 +17599,7 @@
         <v>1607</v>
       </c>
       <c r="I268" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="J268" t="s">
         <v>2014</v>
@@ -17672,7 +17669,7 @@
         <v>1607</v>
       </c>
       <c r="I270" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J270" t="s">
         <v>2016</v>
@@ -17847,7 +17844,7 @@
         <v>1607</v>
       </c>
       <c r="I275" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J275" t="s">
         <v>2021</v>
@@ -17987,7 +17984,7 @@
         <v>1607</v>
       </c>
       <c r="I279" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="J279" t="s">
         <v>2025</v>
@@ -18197,7 +18194,7 @@
         <v>1607</v>
       </c>
       <c r="I285" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J285" t="s">
         <v>2031</v>
@@ -18267,7 +18264,7 @@
         <v>1607</v>
       </c>
       <c r="I287" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J287" t="s">
         <v>2033</v>
@@ -18302,7 +18299,7 @@
         <v>1607</v>
       </c>
       <c r="I288" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J288" t="s">
         <v>2034</v>
@@ -18337,7 +18334,7 @@
         <v>1607</v>
       </c>
       <c r="I289" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J289" t="s">
         <v>2035</v>
@@ -18477,7 +18474,7 @@
         <v>1607</v>
       </c>
       <c r="I293" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="J293" t="s">
         <v>2039</v>
@@ -18512,7 +18509,7 @@
         <v>1607</v>
       </c>
       <c r="I294" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="J294" t="s">
         <v>2040</v>
@@ -18547,7 +18544,7 @@
         <v>1607</v>
       </c>
       <c r="I295" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="J295" t="s">
         <v>2041</v>
@@ -18617,7 +18614,7 @@
         <v>1607</v>
       </c>
       <c r="I297" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J297" t="s">
         <v>2043</v>
@@ -18687,7 +18684,7 @@
         <v>1607</v>
       </c>
       <c r="I299" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="J299" t="s">
         <v>2045</v>
@@ -18757,7 +18754,7 @@
         <v>1607</v>
       </c>
       <c r="I301" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J301" t="s">
         <v>2047</v>
@@ -18827,7 +18824,7 @@
         <v>1607</v>
       </c>
       <c r="I303" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="J303" t="s">
         <v>2049</v>
@@ -18865,7 +18862,7 @@
         <v>1611</v>
       </c>
       <c r="I304" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J304" t="s">
         <v>2050</v>
@@ -19005,7 +19002,7 @@
         <v>1607</v>
       </c>
       <c r="I308" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="J308" t="s">
         <v>2054</v>
@@ -19180,7 +19177,7 @@
         <v>1607</v>
       </c>
       <c r="I313" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J313" t="s">
         <v>2059</v>
@@ -19215,7 +19212,7 @@
         <v>1607</v>
       </c>
       <c r="I314" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J314" t="s">
         <v>2060</v>
@@ -19250,7 +19247,7 @@
         <v>1607</v>
       </c>
       <c r="I315" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="J315" t="s">
         <v>2061</v>
@@ -19285,7 +19282,7 @@
         <v>1607</v>
       </c>
       <c r="I316" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J316" t="s">
         <v>2062</v>
@@ -19320,7 +19317,7 @@
         <v>1607</v>
       </c>
       <c r="I317" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J317" t="s">
         <v>2063</v>
@@ -19355,7 +19352,7 @@
         <v>1607</v>
       </c>
       <c r="I318" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="J318" t="s">
         <v>2064</v>
@@ -19460,7 +19457,7 @@
         <v>1607</v>
       </c>
       <c r="I321" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J321" t="s">
         <v>2067</v>
@@ -19495,7 +19492,7 @@
         <v>1607</v>
       </c>
       <c r="I322" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="J322" t="s">
         <v>2068</v>
@@ -19565,7 +19562,7 @@
         <v>1607</v>
       </c>
       <c r="I324" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J324" t="s">
         <v>2070</v>
@@ -19775,7 +19772,7 @@
         <v>1607</v>
       </c>
       <c r="I330" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J330" t="s">
         <v>2076</v>
@@ -19810,7 +19807,7 @@
         <v>1607</v>
       </c>
       <c r="I331" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J331" t="s">
         <v>2077</v>
@@ -19915,7 +19912,7 @@
         <v>1607</v>
       </c>
       <c r="I334" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="J334" t="s">
         <v>2080</v>
@@ -19950,7 +19947,7 @@
         <v>1607</v>
       </c>
       <c r="I335" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J335" t="s">
         <v>2081</v>
@@ -20020,7 +20017,7 @@
         <v>1607</v>
       </c>
       <c r="I337" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J337" t="s">
         <v>2083</v>
@@ -20090,7 +20087,7 @@
         <v>1607</v>
       </c>
       <c r="I339" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J339" t="s">
         <v>2085</v>
@@ -20125,7 +20122,7 @@
         <v>1607</v>
       </c>
       <c r="I340" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J340" t="s">
         <v>2086</v>
@@ -20160,7 +20157,7 @@
         <v>1607</v>
       </c>
       <c r="I341" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="J341" t="s">
         <v>2087</v>
@@ -20335,7 +20332,7 @@
         <v>1607</v>
       </c>
       <c r="I346" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J346" t="s">
         <v>2092</v>
@@ -20370,7 +20367,7 @@
         <v>1607</v>
       </c>
       <c r="I347" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="J347" t="s">
         <v>2093</v>
@@ -20478,7 +20475,7 @@
         <v>1607</v>
       </c>
       <c r="I350" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J350" t="s">
         <v>2096</v>
@@ -20548,7 +20545,7 @@
         <v>1607</v>
       </c>
       <c r="I352" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J352" t="s">
         <v>2098</v>
@@ -20586,7 +20583,7 @@
         <v>1612</v>
       </c>
       <c r="I353" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J353" t="s">
         <v>2099</v>
@@ -20761,7 +20758,7 @@
         <v>1607</v>
       </c>
       <c r="I358" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J358" t="s">
         <v>2104</v>
@@ -20796,7 +20793,7 @@
         <v>1607</v>
       </c>
       <c r="I359" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J359" t="s">
         <v>2105</v>
@@ -20936,7 +20933,7 @@
         <v>1607</v>
       </c>
       <c r="I363" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J363" t="s">
         <v>2109</v>
@@ -21041,7 +21038,7 @@
         <v>1607</v>
       </c>
       <c r="I366" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="J366" t="s">
         <v>2112</v>
@@ -21076,7 +21073,7 @@
         <v>1607</v>
       </c>
       <c r="I367" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J367" t="s">
         <v>2113</v>
@@ -21356,7 +21353,7 @@
         <v>1607</v>
       </c>
       <c r="I375" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J375" t="s">
         <v>2121</v>
@@ -21531,7 +21528,7 @@
         <v>1607</v>
       </c>
       <c r="I380" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="J380" t="s">
         <v>2126</v>
@@ -21566,7 +21563,7 @@
         <v>1607</v>
       </c>
       <c r="I381" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J381" t="s">
         <v>2127</v>
@@ -21636,7 +21633,7 @@
         <v>1607</v>
       </c>
       <c r="I383" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J383" t="s">
         <v>2129</v>
@@ -21706,7 +21703,7 @@
         <v>1607</v>
       </c>
       <c r="I385" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J385" t="s">
         <v>2131</v>
@@ -21776,7 +21773,7 @@
         <v>1607</v>
       </c>
       <c r="I387" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J387" t="s">
         <v>2133</v>
@@ -21811,7 +21808,7 @@
         <v>1607</v>
       </c>
       <c r="I388" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J388" t="s">
         <v>2134</v>
@@ -22056,7 +22053,7 @@
         <v>1607</v>
       </c>
       <c r="I395" t="s">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="J395" t="s">
         <v>2141</v>
@@ -22091,7 +22088,7 @@
         <v>1607</v>
       </c>
       <c r="I396" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J396" t="s">
         <v>2142</v>
@@ -22126,7 +22123,7 @@
         <v>1607</v>
       </c>
       <c r="I397" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="J397" t="s">
         <v>2143</v>
@@ -22161,7 +22158,7 @@
         <v>1607</v>
       </c>
       <c r="I398" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="J398" t="s">
         <v>2144</v>
@@ -22266,7 +22263,7 @@
         <v>1607</v>
       </c>
       <c r="I401" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J401" t="s">
         <v>2147</v>
@@ -22371,7 +22368,7 @@
         <v>1607</v>
       </c>
       <c r="I404" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J404" t="s">
         <v>2150</v>
@@ -22546,7 +22543,7 @@
         <v>1607</v>
       </c>
       <c r="I409" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J409" t="s">
         <v>2155</v>
@@ -22616,7 +22613,7 @@
         <v>1607</v>
       </c>
       <c r="I411" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="J411" t="s">
         <v>2157</v>
@@ -22826,7 +22823,7 @@
         <v>1607</v>
       </c>
       <c r="I417" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J417" t="s">
         <v>2163</v>
@@ -22861,7 +22858,7 @@
         <v>1607</v>
       </c>
       <c r="I418" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J418" t="s">
         <v>2164</v>
@@ -22896,7 +22893,7 @@
         <v>1607</v>
       </c>
       <c r="I419" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J419" t="s">
         <v>2165</v>
@@ -22931,7 +22928,7 @@
         <v>1607</v>
       </c>
       <c r="I420" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J420" t="s">
         <v>2166</v>
@@ -23176,7 +23173,7 @@
         <v>1607</v>
       </c>
       <c r="I427" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J427" t="s">
         <v>2173</v>
@@ -23386,7 +23383,7 @@
         <v>1607</v>
       </c>
       <c r="I433" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J433" t="s">
         <v>2179</v>
@@ -23421,7 +23418,7 @@
         <v>1607</v>
       </c>
       <c r="I434" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J434" t="s">
         <v>2180</v>
@@ -23456,7 +23453,7 @@
         <v>1607</v>
       </c>
       <c r="I435" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J435" t="s">
         <v>2181</v>
@@ -23529,7 +23526,7 @@
         <v>1579</v>
       </c>
       <c r="I437" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="J437" t="s">
         <v>2183</v>
@@ -23634,7 +23631,7 @@
         <v>1607</v>
       </c>
       <c r="I440" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J440" t="s">
         <v>2186</v>
@@ -23669,7 +23666,7 @@
         <v>1607</v>
       </c>
       <c r="I441" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J441" t="s">
         <v>2187</v>
@@ -23704,7 +23701,7 @@
         <v>1607</v>
       </c>
       <c r="I442" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="J442" t="s">
         <v>2188</v>
@@ -23742,7 +23739,7 @@
         <v>1613</v>
       </c>
       <c r="I443" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J443" t="s">
         <v>2189</v>
@@ -24057,7 +24054,7 @@
         <v>1607</v>
       </c>
       <c r="I452" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J452" t="s">
         <v>2198</v>
@@ -24232,7 +24229,7 @@
         <v>1607</v>
       </c>
       <c r="I457" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="J457" t="s">
         <v>2203</v>
@@ -24267,7 +24264,7 @@
         <v>1607</v>
       </c>
       <c r="I458" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J458" t="s">
         <v>2204</v>
@@ -24302,7 +24299,7 @@
         <v>1607</v>
       </c>
       <c r="I459" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J459" t="s">
         <v>2205</v>
@@ -24372,7 +24369,7 @@
         <v>1607</v>
       </c>
       <c r="I461" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J461" t="s">
         <v>2207</v>
@@ -24407,7 +24404,7 @@
         <v>1607</v>
       </c>
       <c r="I462" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J462" t="s">
         <v>2208</v>
@@ -24442,7 +24439,7 @@
         <v>1607</v>
       </c>
       <c r="I463" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J463" t="s">
         <v>2209</v>
@@ -24477,7 +24474,7 @@
         <v>1607</v>
       </c>
       <c r="I464" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J464" t="s">
         <v>2210</v>
@@ -24512,7 +24509,7 @@
         <v>1607</v>
       </c>
       <c r="I465" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J465" t="s">
         <v>2211</v>
@@ -24547,7 +24544,7 @@
         <v>1607</v>
       </c>
       <c r="I466" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J466" t="s">
         <v>2212</v>
@@ -24582,7 +24579,7 @@
         <v>1607</v>
       </c>
       <c r="I467" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J467" t="s">
         <v>2213</v>
@@ -24617,7 +24614,7 @@
         <v>1607</v>
       </c>
       <c r="I468" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J468" t="s">
         <v>2214</v>
@@ -24655,7 +24652,7 @@
         <v>1614</v>
       </c>
       <c r="I469" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J469" t="s">
         <v>2215</v>
@@ -24690,7 +24687,7 @@
         <v>1607</v>
       </c>
       <c r="I470" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="J470" t="s">
         <v>2216</v>
@@ -24725,7 +24722,7 @@
         <v>1607</v>
       </c>
       <c r="I471" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J471" t="s">
         <v>2217</v>
@@ -24760,7 +24757,7 @@
         <v>1607</v>
       </c>
       <c r="I472" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J472" t="s">
         <v>2218</v>
@@ -24795,7 +24792,7 @@
         <v>1607</v>
       </c>
       <c r="I473" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J473" t="s">
         <v>2219</v>
@@ -24865,7 +24862,7 @@
         <v>1607</v>
       </c>
       <c r="I475" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J475" t="s">
         <v>2221</v>
@@ -24900,7 +24897,7 @@
         <v>1607</v>
       </c>
       <c r="I476" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J476" t="s">
         <v>2222</v>
@@ -24935,7 +24932,7 @@
         <v>1607</v>
       </c>
       <c r="I477" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J477" t="s">
         <v>2223</v>
@@ -24970,7 +24967,7 @@
         <v>1607</v>
       </c>
       <c r="I478" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J478" t="s">
         <v>2224</v>
@@ -25005,7 +25002,7 @@
         <v>1607</v>
       </c>
       <c r="I479" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J479" t="s">
         <v>2225</v>
@@ -25040,7 +25037,7 @@
         <v>1607</v>
       </c>
       <c r="I480" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J480" t="s">
         <v>2226</v>
@@ -25075,7 +25072,7 @@
         <v>1607</v>
       </c>
       <c r="I481" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J481" t="s">
         <v>2227</v>
@@ -25145,7 +25142,7 @@
         <v>1607</v>
       </c>
       <c r="I483" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J483" t="s">
         <v>2229</v>
@@ -25250,7 +25247,7 @@
         <v>1607</v>
       </c>
       <c r="I486" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J486" t="s">
         <v>2232</v>
@@ -25285,7 +25282,7 @@
         <v>1607</v>
       </c>
       <c r="I487" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J487" t="s">
         <v>2233</v>
@@ -25320,7 +25317,7 @@
         <v>1607</v>
       </c>
       <c r="I488" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J488" t="s">
         <v>2234</v>
@@ -25425,7 +25422,7 @@
         <v>1607</v>
       </c>
       <c r="I491" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J491" t="s">
         <v>2237</v>
@@ -25530,7 +25527,7 @@
         <v>1609</v>
       </c>
       <c r="I494" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J494" t="s">
         <v>2240</v>
@@ -25565,7 +25562,7 @@
         <v>1607</v>
       </c>
       <c r="I495" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="J495" t="s">
         <v>2241</v>
@@ -25635,7 +25632,7 @@
         <v>1607</v>
       </c>
       <c r="I497" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J497" t="s">
         <v>2243</v>
@@ -25775,7 +25772,7 @@
         <v>1607</v>
       </c>
       <c r="I501" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="J501" t="s">
         <v>2247</v>
@@ -25810,7 +25807,7 @@
         <v>1607</v>
       </c>
       <c r="I502" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J502" t="s">
         <v>2248</v>
@@ -25845,7 +25842,7 @@
         <v>1607</v>
       </c>
       <c r="I503" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J503" t="s">
         <v>2249</v>
@@ -25915,7 +25912,7 @@
         <v>1607</v>
       </c>
       <c r="I505" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J505" t="s">
         <v>2251</v>
@@ -26055,7 +26052,7 @@
         <v>1607</v>
       </c>
       <c r="I509" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J509" t="s">
         <v>2254</v>
@@ -26090,7 +26087,7 @@
         <v>1607</v>
       </c>
       <c r="I510" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J510" t="s">
         <v>2255</v>
@@ -26128,7 +26125,7 @@
         <v>1615</v>
       </c>
       <c r="I511" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="J511" t="s">
         <v>2256</v>
@@ -26163,7 +26160,7 @@
         <v>1607</v>
       </c>
       <c r="I512" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J512" t="s">
         <v>2257</v>
@@ -26198,7 +26195,7 @@
         <v>1607</v>
       </c>
       <c r="I513" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="J513" t="s">
         <v>2257</v>
@@ -26233,7 +26230,7 @@
         <v>1607</v>
       </c>
       <c r="I514" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J514" t="s">
         <v>2258</v>
@@ -26268,7 +26265,7 @@
         <v>1607</v>
       </c>
       <c r="I515" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J515" t="s">
         <v>2259</v>
@@ -26303,7 +26300,7 @@
         <v>1607</v>
       </c>
       <c r="I516" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J516" t="s">
         <v>2260</v>
@@ -26338,7 +26335,7 @@
         <v>1607</v>
       </c>
       <c r="I517" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="J517" t="s">
         <v>2261</v>
@@ -26478,7 +26475,7 @@
         <v>1607</v>
       </c>
       <c r="I521" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="J521" t="s">
         <v>2265</v>
@@ -26513,7 +26510,7 @@
         <v>1607</v>
       </c>
       <c r="I522" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J522" t="s">
         <v>2266</v>
@@ -26653,7 +26650,7 @@
         <v>1607</v>
       </c>
       <c r="I526" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J526" t="s">
         <v>2270</v>
@@ -26688,7 +26685,7 @@
         <v>1607</v>
       </c>
       <c r="I527" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J527" t="s">
         <v>2271</v>
@@ -26723,7 +26720,7 @@
         <v>1607</v>
       </c>
       <c r="I528" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="J528" t="s">
         <v>2272</v>
@@ -26758,7 +26755,7 @@
         <v>1607</v>
       </c>
       <c r="I529" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J529" t="s">
         <v>2273</v>
@@ -26793,7 +26790,7 @@
         <v>1607</v>
       </c>
       <c r="I530" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J530" t="s">
         <v>2274</v>
@@ -26828,7 +26825,7 @@
         <v>1607</v>
       </c>
       <c r="I531" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="J531" t="s">
         <v>2275</v>
@@ -26936,7 +26933,7 @@
         <v>1616</v>
       </c>
       <c r="I534" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J534" t="s">
         <v>2278</v>
@@ -26971,7 +26968,7 @@
         <v>1607</v>
       </c>
       <c r="I535" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="J535" t="s">
         <v>2279</v>
@@ -27006,7 +27003,7 @@
         <v>1607</v>
       </c>
       <c r="I536" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J536" t="s">
         <v>2280</v>
@@ -27041,7 +27038,7 @@
         <v>1607</v>
       </c>
       <c r="I537" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J537" t="s">
         <v>2281</v>
@@ -27076,7 +27073,7 @@
         <v>1607</v>
       </c>
       <c r="I538" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J538" t="s">
         <v>2282</v>
@@ -27111,7 +27108,7 @@
         <v>1607</v>
       </c>
       <c r="I539" t="s">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="J539" t="s">
         <v>2283</v>
@@ -27146,7 +27143,7 @@
         <v>1607</v>
       </c>
       <c r="I540" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J540" t="s">
         <v>2284</v>
@@ -27181,7 +27178,7 @@
         <v>1607</v>
       </c>
       <c r="I541" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="J541" t="s">
         <v>2285</v>
@@ -27216,7 +27213,7 @@
         <v>1607</v>
       </c>
       <c r="I542" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J542" t="s">
         <v>2286</v>
@@ -27251,7 +27248,7 @@
         <v>1607</v>
       </c>
       <c r="I543" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J543" t="s">
         <v>2287</v>
@@ -27286,7 +27283,7 @@
         <v>1607</v>
       </c>
       <c r="I544" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J544" t="s">
         <v>2288</v>
@@ -27356,7 +27353,7 @@
         <v>1607</v>
       </c>
       <c r="I546" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J546" t="s">
         <v>2290</v>
@@ -27391,7 +27388,7 @@
         <v>1607</v>
       </c>
       <c r="I547" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J547" t="s">
         <v>2291</v>
@@ -27426,7 +27423,7 @@
         <v>1607</v>
       </c>
       <c r="I548" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J548" t="s">
         <v>2292</v>
@@ -27499,7 +27496,7 @@
         <v>1607</v>
       </c>
       <c r="I550" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J550" t="s">
         <v>2294</v>
@@ -27534,7 +27531,7 @@
         <v>1607</v>
       </c>
       <c r="I551" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J551" t="s">
         <v>2295</v>
@@ -27569,7 +27566,7 @@
         <v>1607</v>
       </c>
       <c r="I552" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J552" t="s">
         <v>2296</v>
@@ -27674,7 +27671,7 @@
         <v>1607</v>
       </c>
       <c r="I555" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J555" t="s">
         <v>2299</v>
@@ -27709,7 +27706,7 @@
         <v>1607</v>
       </c>
       <c r="I556" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="J556" t="s">
         <v>2300</v>
@@ -27744,7 +27741,7 @@
         <v>1607</v>
       </c>
       <c r="I557" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J557" t="s">
         <v>2301</v>
@@ -27779,7 +27776,7 @@
         <v>1607</v>
       </c>
       <c r="I558" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J558" t="s">
         <v>2302</v>
@@ -27849,7 +27846,7 @@
         <v>1607</v>
       </c>
       <c r="I560" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J560" t="s">
         <v>2304</v>
@@ -27919,7 +27916,7 @@
         <v>1607</v>
       </c>
       <c r="I562" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J562" t="s">
         <v>2306</v>
@@ -27954,7 +27951,7 @@
         <v>1607</v>
       </c>
       <c r="I563" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J563" t="s">
         <v>2307</v>
@@ -27989,7 +27986,7 @@
         <v>1607</v>
       </c>
       <c r="I564" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="J564" t="s">
         <v>2308</v>
@@ -28024,7 +28021,7 @@
         <v>1607</v>
       </c>
       <c r="I565" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J565" t="s">
         <v>2309</v>
@@ -28059,7 +28056,7 @@
         <v>1607</v>
       </c>
       <c r="I566" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J566" t="s">
         <v>2310</v>
@@ -28094,7 +28091,7 @@
         <v>1607</v>
       </c>
       <c r="I567" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J567" t="s">
         <v>2311</v>
@@ -28129,7 +28126,7 @@
         <v>1607</v>
       </c>
       <c r="I568" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J568" t="s">
         <v>2312</v>
@@ -28164,7 +28161,7 @@
         <v>1607</v>
       </c>
       <c r="I569" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J569" t="s">
         <v>2271</v>
@@ -28199,7 +28196,7 @@
         <v>1607</v>
       </c>
       <c r="I570" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J570" t="s">
         <v>2313</v>
@@ -28272,7 +28269,7 @@
         <v>1607</v>
       </c>
       <c r="I572" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J572" t="s">
         <v>2315</v>
@@ -28380,7 +28377,7 @@
         <v>1619</v>
       </c>
       <c r="I575" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="J575" t="s">
         <v>2318</v>
@@ -28418,7 +28415,7 @@
         <v>1620</v>
       </c>
       <c r="I576" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="J576" t="s">
         <v>2319</v>
@@ -28523,7 +28520,7 @@
         <v>1607</v>
       </c>
       <c r="I579" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J579" t="s">
         <v>2322</v>
@@ -28558,7 +28555,7 @@
         <v>1607</v>
       </c>
       <c r="I580" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J580" t="s">
         <v>2323</v>
@@ -28593,7 +28590,7 @@
         <v>1607</v>
       </c>
       <c r="I581" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J581" t="s">
         <v>2324</v>
@@ -28628,7 +28625,7 @@
         <v>1607</v>
       </c>
       <c r="I582" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J582" t="s">
         <v>2325</v>
@@ -28698,7 +28695,7 @@
         <v>1607</v>
       </c>
       <c r="I584" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="J584" t="s">
         <v>2327</v>
@@ -28733,7 +28730,7 @@
         <v>1607</v>
       </c>
       <c r="I585" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J585" t="s">
         <v>2328</v>
@@ -28768,7 +28765,7 @@
         <v>1607</v>
       </c>
       <c r="I586" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J586" t="s">
         <v>2329</v>
@@ -28803,7 +28800,7 @@
         <v>1607</v>
       </c>
       <c r="I587" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J587" t="s">
         <v>2330</v>
@@ -28838,7 +28835,7 @@
         <v>1607</v>
       </c>
       <c r="I588" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J588" t="s">
         <v>2331</v>
@@ -28873,7 +28870,7 @@
         <v>1607</v>
       </c>
       <c r="I589" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="J589" t="s">
         <v>2332</v>
@@ -28908,7 +28905,7 @@
         <v>1607</v>
       </c>
       <c r="I590" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J590" t="s">
         <v>2333</v>
@@ -28943,7 +28940,7 @@
         <v>1607</v>
       </c>
       <c r="I591" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J591" t="s">
         <v>2334</v>
@@ -28978,7 +28975,7 @@
         <v>1607</v>
       </c>
       <c r="I592" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J592" t="s">
         <v>2335</v>
@@ -29013,7 +29010,7 @@
         <v>1607</v>
       </c>
       <c r="I593" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J593" t="s">
         <v>2336</v>
@@ -29048,7 +29045,7 @@
         <v>1607</v>
       </c>
       <c r="I594" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J594" t="s">
         <v>2337</v>
@@ -29083,7 +29080,7 @@
         <v>1607</v>
       </c>
       <c r="I595" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J595" t="s">
         <v>2338</v>
@@ -29118,7 +29115,7 @@
         <v>1607</v>
       </c>
       <c r="I596" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J596" t="s">
         <v>2339</v>
@@ -29153,7 +29150,7 @@
         <v>1607</v>
       </c>
       <c r="I597" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J597" t="s">
         <v>2340</v>
@@ -29191,7 +29188,7 @@
         <v>1619</v>
       </c>
       <c r="I598" t="s">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="J598" t="s">
         <v>2341</v>
@@ -29226,7 +29223,7 @@
         <v>1607</v>
       </c>
       <c r="I599" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J599" t="s">
         <v>2342</v>
@@ -29261,7 +29258,7 @@
         <v>1607</v>
       </c>
       <c r="I600" t="s">
-        <v>1745</v>
+        <v>1637</v>
       </c>
       <c r="J600" t="s">
         <v>2343</v>
@@ -29331,7 +29328,7 @@
         <v>1607</v>
       </c>
       <c r="I602" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J602" t="s">
         <v>2345</v>
@@ -29366,7 +29363,7 @@
         <v>1607</v>
       </c>
       <c r="I603" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J603" t="s">
         <v>2346</v>
@@ -29401,7 +29398,7 @@
         <v>1607</v>
       </c>
       <c r="I604" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J604" t="s">
         <v>2347</v>
@@ -29436,7 +29433,7 @@
         <v>1607</v>
       </c>
       <c r="I605" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="J605" t="s">
         <v>2348</v>
@@ -29471,7 +29468,7 @@
         <v>1607</v>
       </c>
       <c r="I606" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J606" t="s">
         <v>2349</v>
@@ -29576,7 +29573,7 @@
         <v>1607</v>
       </c>
       <c r="I609" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J609" t="s">
         <v>2352</v>
@@ -30279,7 +30276,7 @@
         <v>1621</v>
       </c>
       <c r="I629" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="J629" t="s">
         <v>2372</v>
@@ -30314,7 +30311,7 @@
         <v>1607</v>
       </c>
       <c r="I630" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J630" t="s">
         <v>2373</v>
@@ -30349,7 +30346,7 @@
         <v>1607</v>
       </c>
       <c r="I631" t="s">
-        <v>1745</v>
+        <v>1637</v>
       </c>
       <c r="J631" t="s">
         <v>2374</v>
@@ -30384,7 +30381,7 @@
         <v>1607</v>
       </c>
       <c r="I632" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="J632" t="s">
         <v>2375</v>
@@ -30457,7 +30454,7 @@
         <v>1607</v>
       </c>
       <c r="I634" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J634" t="s">
         <v>2377</v>
@@ -30492,7 +30489,7 @@
         <v>1607</v>
       </c>
       <c r="I635" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="J635" t="s">
         <v>2377</v>
@@ -30527,7 +30524,7 @@
         <v>1607</v>
       </c>
       <c r="I636" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J636" t="s">
         <v>2377</v>
@@ -30562,7 +30559,7 @@
         <v>1607</v>
       </c>
       <c r="I637" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J637" t="s">
         <v>2378</v>
@@ -30597,7 +30594,7 @@
         <v>1607</v>
       </c>
       <c r="I638" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="J638" t="s">
         <v>2379</v>
@@ -30702,7 +30699,7 @@
         <v>1607</v>
       </c>
       <c r="I641" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J641" t="s">
         <v>2382</v>
@@ -30816,7 +30813,7 @@
         <v>1623</v>
       </c>
       <c r="I644" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J644" t="s">
         <v>2385</v>
@@ -30886,7 +30883,7 @@
         <v>1607</v>
       </c>
       <c r="I646" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J646" t="s">
         <v>2386</v>
@@ -30997,7 +30994,7 @@
         <v>1607</v>
       </c>
       <c r="I649" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J649" t="s">
         <v>2389</v>
@@ -31041,7 +31038,7 @@
         <v>2462</v>
       </c>
       <c r="L650" t="s">
-        <v>2598</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31143,7 +31140,7 @@
         <v>1607</v>
       </c>
       <c r="I653" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J653" t="s">
         <v>2393</v>
@@ -31181,7 +31178,7 @@
         <v>1626</v>
       </c>
       <c r="I654" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="J654" t="s">
         <v>2394</v>
@@ -31225,7 +31222,7 @@
         <v>2419</v>
       </c>
       <c r="L655" t="s">
-        <v>2557</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="656" spans="1:12">
@@ -31251,7 +31248,7 @@
         <v>1607</v>
       </c>
       <c r="I656" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="J656" t="s">
         <v>2396</v>
@@ -31286,7 +31283,7 @@
         <v>1607</v>
       </c>
       <c r="I657" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="J657" t="s">
         <v>2397</v>
@@ -31432,7 +31429,7 @@
         <v>1627</v>
       </c>
       <c r="I661" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J661" t="s">
         <v>2401</v>
@@ -31537,7 +31534,7 @@
         <v>1607</v>
       </c>
       <c r="I664" t="s">
-        <v>1745</v>
+        <v>1637</v>
       </c>
       <c r="J664" t="s">
         <v>2404</v>
@@ -31575,7 +31572,7 @@
         <v>1628</v>
       </c>
       <c r="I665" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J665" t="s">
         <v>2405</v>
@@ -31610,7 +31607,7 @@
         <v>1607</v>
       </c>
       <c r="I666" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J666" t="s">
         <v>2406</v>
@@ -31645,7 +31642,7 @@
         <v>1607</v>
       </c>
       <c r="I667" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="J667" t="s">
         <v>2407</v>
@@ -31680,7 +31677,7 @@
         <v>1607</v>
       </c>
       <c r="I668" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="J668" t="s">
         <v>2408</v>
@@ -31715,7 +31712,7 @@
         <v>1607</v>
       </c>
       <c r="I669" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="J669" t="s">
         <v>2409</v>
@@ -31750,7 +31747,7 @@
         <v>1607</v>
       </c>
       <c r="I670" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="J670" t="s">
         <v>2410</v>
@@ -31791,7 +31788,7 @@
         <v>2538</v>
       </c>
       <c r="L671" t="s">
-        <v>2615</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="672" spans="1:12">
@@ -31823,7 +31820,7 @@
         <v>2538</v>
       </c>
       <c r="L672" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-17 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -29412,7 +29412,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B605" t="s">
         <v>642</v>
@@ -29433,7 +29433,7 @@
         <v>1607</v>
       </c>
       <c r="I605" t="s">
-        <v>1735</v>
+        <v>1634</v>
       </c>
       <c r="J605" t="s">
         <v>2348</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-19 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6726" uniqueCount="2606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6726" uniqueCount="2607">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7669,7 +7669,7 @@
     <t>### SEM TEMA ###</t>
   </si>
   <si>
-    <t>VALORAÇÃO DANOS AMBIENTAIS,ENGENHARIA QUÍMICA</t>
+    <t>ENGENHARIA QUÍMICA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
     <t>MOBILIDADE E TRANSPORTE,URBANISMO</t>
@@ -7768,7 +7768,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7816,10 +7816,10 @@
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,ENGENHARIA CIVIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ECONOMIA,RECURSOS HÍDRICOS</t>
@@ -7828,10 +7828,13 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
+    <t>RECURSOS HÍDRICOS,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL,URBANISMO,MOBILIDADE E TRANSPORTE,ORÇAMENTO,ASSISTÊNCIA SOCIAL,SAÚDE,ECONOMIA,PSICOLOGIA,SAÚDE MENTAL</t>
+    <t>PSICOLOGIA,SAÚDE MENTAL,URBANISMO,MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,ASSISTÊNCIA SOCIAL,ORÇAMENTO,SAÚDE</t>
   </si>
 </sst>
 </file>
@@ -31267,7 +31270,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B658" t="s">
         <v>694</v>
@@ -31288,7 +31291,7 @@
         <v>1602</v>
       </c>
       <c r="I658" t="s">
-        <v>1628</v>
+        <v>1744</v>
       </c>
       <c r="J658" t="s">
         <v>2389</v>
@@ -31326,7 +31329,7 @@
         <v>1622</v>
       </c>
       <c r="I659" t="s">
-        <v>1628</v>
+        <v>1738</v>
       </c>
       <c r="J659" t="s">
         <v>2390</v>
@@ -31335,7 +31338,7 @@
         <v>2413</v>
       </c>
       <c r="L659" t="s">
-        <v>2587</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="660" spans="1:12">
@@ -31682,7 +31685,7 @@
         <v>2527</v>
       </c>
       <c r="L669" t="s">
-        <v>2604</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="670" spans="1:12">
@@ -31714,7 +31717,7 @@
         <v>2527</v>
       </c>
       <c r="L670" t="s">
-        <v>2605</v>
+        <v>2606</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-20 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -79,15 +79,18 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
+  </si>
+  <si>
+    <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
-  </si>
-  <si>
-    <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
-  </si>
-  <si>
     <t>ECONOMICIDADE DE OBRAS E SERVIÇOS DE ENGENHARIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -115,9 +118,6 @@
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE ECONOMIA,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -4966,106 +4966,106 @@
     <t>EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
+    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>REGINA SILBERSTEIN RACHEVSKY</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES,MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,PATRICIA PASSARO DA SILVA TOLEDO</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
+  </si>
+  <si>
+    <t>PEDRO MARCELO ROCHA GOMES</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
+  </si>
+  <si>
+    <t>CASSIA CRISTINA DA SILVA</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
     <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>REGINA SILBERSTEIN RACHEVSKY</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES,MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,PATRICIA PASSARO DA SILVA TOLEDO</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
-  </si>
-  <si>
-    <t>PEDRO MARCELO ROCHA GOMES</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
-  </si>
-  <si>
-    <t>CASSIA CRISTINA DA SILVA</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
   </si>
   <si>
     <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
@@ -10468,7 +10468,7 @@
         <v>1754</v>
       </c>
       <c r="K64" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="L64" t="s">
         <v>2542</v>
@@ -10637,7 +10637,7 @@
         <v>1607</v>
       </c>
       <c r="I69" t="s">
-        <v>1650</v>
+        <v>1633</v>
       </c>
       <c r="J69" t="s">
         <v>1817</v>
@@ -10672,7 +10672,7 @@
         <v>1607</v>
       </c>
       <c r="I70" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J70" t="s">
         <v>1818</v>
@@ -10707,7 +10707,7 @@
         <v>1607</v>
       </c>
       <c r="I71" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="J71" t="s">
         <v>1819</v>
@@ -10742,7 +10742,7 @@
         <v>1607</v>
       </c>
       <c r="I72" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J72" t="s">
         <v>1820</v>
@@ -10777,7 +10777,7 @@
         <v>1607</v>
       </c>
       <c r="I73" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="J73" t="s">
         <v>1821</v>
@@ -10826,7 +10826,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B75" t="s">
         <v>114</v>
@@ -10847,7 +10847,7 @@
         <v>1607</v>
       </c>
       <c r="I75" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J75" t="s">
         <v>1823</v>
@@ -10952,7 +10952,7 @@
         <v>1607</v>
       </c>
       <c r="I78" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J78" t="s">
         <v>1826</v>
@@ -11001,7 +11001,7 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B80" t="s">
         <v>119</v>
@@ -11022,7 +11022,7 @@
         <v>1607</v>
       </c>
       <c r="I80" t="s">
-        <v>1657</v>
+        <v>1656</v>
       </c>
       <c r="J80" t="s">
         <v>1828</v>
@@ -11127,7 +11127,7 @@
         <v>1607</v>
       </c>
       <c r="I83" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J83" t="s">
         <v>1831</v>
@@ -11232,7 +11232,7 @@
         <v>1607</v>
       </c>
       <c r="I86" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="J86" t="s">
         <v>1834</v>
@@ -11267,7 +11267,7 @@
         <v>1607</v>
       </c>
       <c r="I87" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="J87" t="s">
         <v>1835</v>
@@ -11302,7 +11302,7 @@
         <v>1607</v>
       </c>
       <c r="I88" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="J88" t="s">
         <v>1836</v>
@@ -11337,7 +11337,7 @@
         <v>1607</v>
       </c>
       <c r="I89" t="s">
-        <v>1661</v>
+        <v>1660</v>
       </c>
       <c r="J89" t="s">
         <v>1837</v>
@@ -11351,7 +11351,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B90" t="s">
         <v>129</v>
@@ -11372,7 +11372,7 @@
         <v>1607</v>
       </c>
       <c r="I90" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J90" t="s">
         <v>1838</v>
@@ -11512,7 +11512,7 @@
         <v>1607</v>
       </c>
       <c r="I94" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="J94" t="s">
         <v>1842</v>
@@ -11547,7 +11547,7 @@
         <v>1607</v>
       </c>
       <c r="I95" t="s">
-        <v>1664</v>
+        <v>1663</v>
       </c>
       <c r="J95" t="s">
         <v>1843</v>
@@ -11561,7 +11561,7 @@
     </row>
     <row r="96" spans="1:12">
       <c r="A96" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B96" t="s">
         <v>135</v>
@@ -11582,7 +11582,7 @@
         <v>1607</v>
       </c>
       <c r="I96" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J96" t="s">
         <v>1844</v>
@@ -11757,7 +11757,7 @@
         <v>1607</v>
       </c>
       <c r="I101" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="J101" t="s">
         <v>1849</v>
@@ -11897,7 +11897,7 @@
         <v>1607</v>
       </c>
       <c r="I105" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="J105" t="s">
         <v>1853</v>
@@ -11932,7 +11932,7 @@
         <v>1607</v>
       </c>
       <c r="I106" t="s">
-        <v>1668</v>
+        <v>1667</v>
       </c>
       <c r="J106" t="s">
         <v>1854</v>
@@ -11946,7 +11946,7 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B107" t="s">
         <v>146</v>
@@ -11967,7 +11967,7 @@
         <v>1607</v>
       </c>
       <c r="I107" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
       <c r="J107" t="s">
         <v>1855</v>
@@ -12086,7 +12086,7 @@
     </row>
     <row r="111" spans="1:12">
       <c r="A111" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B111" t="s">
         <v>150</v>
@@ -12107,7 +12107,7 @@
         <v>1607</v>
       </c>
       <c r="I111" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="J111" t="s">
         <v>1859</v>
@@ -12121,7 +12121,7 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B112" t="s">
         <v>151</v>
@@ -12142,7 +12142,7 @@
         <v>1607</v>
       </c>
       <c r="I112" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="J112" t="s">
         <v>1860</v>
@@ -12226,7 +12226,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B115" t="s">
         <v>154</v>
@@ -12247,7 +12247,7 @@
         <v>1607</v>
       </c>
       <c r="I115" t="s">
-        <v>1671</v>
+        <v>1670</v>
       </c>
       <c r="J115" t="s">
         <v>1863</v>
@@ -12331,7 +12331,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B118" t="s">
         <v>157</v>
@@ -12352,7 +12352,7 @@
         <v>1607</v>
       </c>
       <c r="I118" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J118" t="s">
         <v>1866</v>
@@ -12366,7 +12366,7 @@
     </row>
     <row r="119" spans="1:12">
       <c r="A119" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B119" t="s">
         <v>158</v>
@@ -12387,7 +12387,7 @@
         <v>1607</v>
       </c>
       <c r="I119" t="s">
-        <v>1673</v>
+        <v>1672</v>
       </c>
       <c r="J119" t="s">
         <v>1867</v>
@@ -12436,7 +12436,7 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B121" t="s">
         <v>160</v>
@@ -12562,7 +12562,7 @@
         <v>1607</v>
       </c>
       <c r="I124" t="s">
-        <v>1674</v>
+        <v>1673</v>
       </c>
       <c r="J124" t="s">
         <v>1872</v>
@@ -12632,7 +12632,7 @@
         <v>1607</v>
       </c>
       <c r="I126" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="J126" t="s">
         <v>1874</v>
@@ -12646,7 +12646,7 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B127" t="s">
         <v>166</v>
@@ -12807,7 +12807,7 @@
         <v>1607</v>
       </c>
       <c r="I131" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J131" t="s">
         <v>1879</v>
@@ -12842,7 +12842,7 @@
         <v>1607</v>
       </c>
       <c r="I132" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
       <c r="J132" t="s">
         <v>1880</v>
@@ -13122,7 +13122,7 @@
         <v>1607</v>
       </c>
       <c r="I140" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
       <c r="J140" t="s">
         <v>1887</v>
@@ -13157,7 +13157,7 @@
         <v>1607</v>
       </c>
       <c r="I141" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="J141" t="s">
         <v>1888</v>
@@ -13227,7 +13227,7 @@
         <v>1607</v>
       </c>
       <c r="I143" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J143" t="s">
         <v>1890</v>
@@ -13367,7 +13367,7 @@
         <v>1607</v>
       </c>
       <c r="I147" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J147" t="s">
         <v>1894</v>
@@ -13472,7 +13472,7 @@
         <v>1607</v>
       </c>
       <c r="I150" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="J150" t="s">
         <v>1897</v>
@@ -13542,7 +13542,7 @@
         <v>1607</v>
       </c>
       <c r="I152" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J152" t="s">
         <v>1899</v>
@@ -13591,7 +13591,7 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B154" t="s">
         <v>193</v>
@@ -13612,7 +13612,7 @@
         <v>1607</v>
       </c>
       <c r="I154" t="s">
-        <v>1650</v>
+        <v>1683</v>
       </c>
       <c r="J154" t="s">
         <v>1901</v>
@@ -13661,7 +13661,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B156" t="s">
         <v>195</v>
@@ -13717,7 +13717,7 @@
         <v>1607</v>
       </c>
       <c r="I157" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="J157" t="s">
         <v>1904</v>
@@ -13906,7 +13906,7 @@
     </row>
     <row r="163" spans="1:12">
       <c r="A163" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B163" t="s">
         <v>202</v>
@@ -14081,7 +14081,7 @@
     </row>
     <row r="168" spans="1:12">
       <c r="A168" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B168" t="s">
         <v>207</v>
@@ -14224,7 +14224,7 @@
     </row>
     <row r="172" spans="1:12">
       <c r="A172" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B172" t="s">
         <v>211</v>
@@ -14245,7 +14245,7 @@
         <v>1607</v>
       </c>
       <c r="I172" t="s">
-        <v>1673</v>
+        <v>1672</v>
       </c>
       <c r="J172" t="s">
         <v>1919</v>
@@ -14294,7 +14294,7 @@
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B174" t="s">
         <v>213</v>
@@ -14315,7 +14315,7 @@
         <v>1607</v>
       </c>
       <c r="I174" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
       <c r="J174" t="s">
         <v>1921</v>
@@ -14469,7 +14469,7 @@
     </row>
     <row r="179" spans="1:12">
       <c r="A179" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B179" t="s">
         <v>218</v>
@@ -14490,7 +14490,7 @@
         <v>1607</v>
       </c>
       <c r="I179" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J179" t="s">
         <v>1926</v>
@@ -14574,7 +14574,7 @@
     </row>
     <row r="182" spans="1:12">
       <c r="A182" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B182" t="s">
         <v>221</v>
@@ -14959,7 +14959,7 @@
     </row>
     <row r="193" spans="1:12">
       <c r="A193" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B193" t="s">
         <v>232</v>
@@ -15085,7 +15085,7 @@
         <v>1607</v>
       </c>
       <c r="I196" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J196" t="s">
         <v>1943</v>
@@ -15204,7 +15204,7 @@
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B200" t="s">
         <v>239</v>
@@ -15449,7 +15449,7 @@
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B207" t="s">
         <v>246</v>
@@ -15554,7 +15554,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B210" t="s">
         <v>249</v>
@@ -15575,7 +15575,7 @@
         <v>1607</v>
       </c>
       <c r="I210" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J210" t="s">
         <v>1956</v>
@@ -15624,7 +15624,7 @@
     </row>
     <row r="212" spans="1:12">
       <c r="A212" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B212" t="s">
         <v>251</v>
@@ -15694,7 +15694,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B214" t="s">
         <v>253</v>
@@ -16030,7 +16030,7 @@
         <v>1607</v>
       </c>
       <c r="I223" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
       <c r="J223" t="s">
         <v>1968</v>
@@ -16044,7 +16044,7 @@
     </row>
     <row r="224" spans="1:12">
       <c r="A224" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B224" t="s">
         <v>263</v>
@@ -16079,7 +16079,7 @@
     </row>
     <row r="225" spans="1:12">
       <c r="A225" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B225" t="s">
         <v>264</v>
@@ -16184,7 +16184,7 @@
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B228" t="s">
         <v>267</v>
@@ -16219,7 +16219,7 @@
     </row>
     <row r="229" spans="1:12">
       <c r="A229" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B229" t="s">
         <v>268</v>
@@ -16254,7 +16254,7 @@
     </row>
     <row r="230" spans="1:12">
       <c r="A230" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B230" t="s">
         <v>269</v>
@@ -16429,7 +16429,7 @@
     </row>
     <row r="235" spans="1:12">
       <c r="A235" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B235" t="s">
         <v>274</v>
@@ -16450,7 +16450,7 @@
         <v>1607</v>
       </c>
       <c r="I235" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J235" t="s">
         <v>1980</v>
@@ -16569,7 +16569,7 @@
     </row>
     <row r="239" spans="1:12">
       <c r="A239" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B239" t="s">
         <v>278</v>
@@ -16849,7 +16849,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B247" t="s">
         <v>286</v>
@@ -16870,7 +16870,7 @@
         <v>1607</v>
       </c>
       <c r="I247" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J247" t="s">
         <v>1992</v>
@@ -17094,7 +17094,7 @@
     </row>
     <row r="254" spans="1:12">
       <c r="A254" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B254" t="s">
         <v>293</v>
@@ -17199,7 +17199,7 @@
     </row>
     <row r="257" spans="1:12">
       <c r="A257" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B257" t="s">
         <v>296</v>
@@ -17374,7 +17374,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B262" t="s">
         <v>301</v>
@@ -17724,7 +17724,7 @@
     </row>
     <row r="272" spans="1:12">
       <c r="A272" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B272" t="s">
         <v>311</v>
@@ -17794,7 +17794,7 @@
     </row>
     <row r="274" spans="1:12">
       <c r="A274" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B274" t="s">
         <v>313</v>
@@ -17815,7 +17815,7 @@
         <v>1607</v>
       </c>
       <c r="I274" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J274" t="s">
         <v>2019</v>
@@ -17990,7 +17990,7 @@
         <v>1607</v>
       </c>
       <c r="I279" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="J279" t="s">
         <v>2024</v>
@@ -18004,7 +18004,7 @@
     </row>
     <row r="280" spans="1:12">
       <c r="A280" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B280" t="s">
         <v>319</v>
@@ -18109,7 +18109,7 @@
     </row>
     <row r="283" spans="1:12">
       <c r="A283" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B283" t="s">
         <v>322</v>
@@ -18214,7 +18214,7 @@
     </row>
     <row r="286" spans="1:12">
       <c r="A286" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B286" t="s">
         <v>325</v>
@@ -18354,7 +18354,7 @@
     </row>
     <row r="290" spans="1:12">
       <c r="A290" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B290" t="s">
         <v>329</v>
@@ -18427,7 +18427,7 @@
     </row>
     <row r="292" spans="1:12">
       <c r="A292" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B292" t="s">
         <v>331</v>
@@ -18462,7 +18462,7 @@
     </row>
     <row r="293" spans="1:12">
       <c r="A293" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B293" t="s">
         <v>332</v>
@@ -18567,7 +18567,7 @@
     </row>
     <row r="296" spans="1:12">
       <c r="A296" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B296" t="s">
         <v>335</v>
@@ -18672,7 +18672,7 @@
     </row>
     <row r="299" spans="1:12">
       <c r="A299" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B299" t="s">
         <v>338</v>
@@ -18707,7 +18707,7 @@
     </row>
     <row r="300" spans="1:12">
       <c r="A300" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B300" t="s">
         <v>339</v>
@@ -18728,7 +18728,7 @@
         <v>1607</v>
       </c>
       <c r="I300" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J300" t="s">
         <v>2045</v>
@@ -18777,7 +18777,7 @@
     </row>
     <row r="302" spans="1:12">
       <c r="A302" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B302" t="s">
         <v>341</v>
@@ -18812,7 +18812,7 @@
     </row>
     <row r="303" spans="1:12">
       <c r="A303" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B303" t="s">
         <v>342</v>
@@ -18917,7 +18917,7 @@
     </row>
     <row r="306" spans="1:12">
       <c r="A306" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B306" t="s">
         <v>345</v>
@@ -18938,7 +18938,7 @@
         <v>1607</v>
       </c>
       <c r="I306" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J306" t="s">
         <v>2051</v>
@@ -18952,7 +18952,7 @@
     </row>
     <row r="307" spans="1:12">
       <c r="A307" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B307" t="s">
         <v>346</v>
@@ -19022,7 +19022,7 @@
     </row>
     <row r="309" spans="1:12">
       <c r="A309" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B309" t="s">
         <v>348</v>
@@ -19232,7 +19232,7 @@
     </row>
     <row r="315" spans="1:12">
       <c r="A315" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B315" t="s">
         <v>354</v>
@@ -19267,7 +19267,7 @@
     </row>
     <row r="316" spans="1:12">
       <c r="A316" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B316" t="s">
         <v>355</v>
@@ -19512,7 +19512,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B323" t="s">
         <v>362</v>
@@ -19547,7 +19547,7 @@
     </row>
     <row r="324" spans="1:12">
       <c r="A324" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B324" t="s">
         <v>363</v>
@@ -19757,7 +19757,7 @@
     </row>
     <row r="330" spans="1:12">
       <c r="A330" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B330" t="s">
         <v>369</v>
@@ -19813,7 +19813,7 @@
         <v>1607</v>
       </c>
       <c r="I331" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="J331" t="s">
         <v>2076</v>
@@ -19900,7 +19900,7 @@
     </row>
     <row r="334" spans="1:12">
       <c r="A334" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B334" t="s">
         <v>373</v>
@@ -19970,7 +19970,7 @@
     </row>
     <row r="336" spans="1:12">
       <c r="A336" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B336" t="s">
         <v>375</v>
@@ -20005,7 +20005,7 @@
     </row>
     <row r="337" spans="1:12">
       <c r="A337" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B337" t="s">
         <v>376</v>
@@ -20183,7 +20183,7 @@
     </row>
     <row r="342" spans="1:12">
       <c r="A342" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B342" t="s">
         <v>381</v>
@@ -20204,7 +20204,7 @@
         <v>1607</v>
       </c>
       <c r="I342" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J342" t="s">
         <v>2087</v>
@@ -20218,7 +20218,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B343" t="s">
         <v>382</v>
@@ -20358,7 +20358,7 @@
     </row>
     <row r="347" spans="1:12">
       <c r="A347" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B347" t="s">
         <v>386</v>
@@ -20498,7 +20498,7 @@
     </row>
     <row r="351" spans="1:12">
       <c r="A351" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B351" t="s">
         <v>390</v>
@@ -20953,7 +20953,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B364" t="s">
         <v>403</v>
@@ -21023,7 +21023,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B366" t="s">
         <v>405</v>
@@ -21093,7 +21093,7 @@
     </row>
     <row r="368" spans="1:12">
       <c r="A368" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B368" t="s">
         <v>407</v>
@@ -21163,7 +21163,7 @@
     </row>
     <row r="370" spans="1:12">
       <c r="A370" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B370" t="s">
         <v>409</v>
@@ -21198,7 +21198,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B371" t="s">
         <v>410</v>
@@ -21268,7 +21268,7 @@
     </row>
     <row r="373" spans="1:12">
       <c r="A373" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B373" t="s">
         <v>412</v>
@@ -21653,7 +21653,7 @@
     </row>
     <row r="384" spans="1:12">
       <c r="A384" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B384" t="s">
         <v>423</v>
@@ -21758,7 +21758,7 @@
     </row>
     <row r="387" spans="1:12">
       <c r="A387" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B387" t="s">
         <v>426</v>
@@ -21779,7 +21779,7 @@
         <v>1607</v>
       </c>
       <c r="I387" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J387" t="s">
         <v>2132</v>
@@ -21793,7 +21793,7 @@
     </row>
     <row r="388" spans="1:12">
       <c r="A388" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B388" t="s">
         <v>427</v>
@@ -21933,7 +21933,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B392" t="s">
         <v>431</v>
@@ -22213,7 +22213,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B400" t="s">
         <v>439</v>
@@ -22248,7 +22248,7 @@
     </row>
     <row r="401" spans="1:12">
       <c r="A401" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B401" t="s">
         <v>440</v>
@@ -22283,7 +22283,7 @@
     </row>
     <row r="402" spans="1:12">
       <c r="A402" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B402" t="s">
         <v>441</v>
@@ -22318,7 +22318,7 @@
     </row>
     <row r="403" spans="1:12">
       <c r="A403" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B403" t="s">
         <v>442</v>
@@ -22493,7 +22493,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B408" t="s">
         <v>447</v>
@@ -22563,7 +22563,7 @@
     </row>
     <row r="410" spans="1:12">
       <c r="A410" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B410" t="s">
         <v>449</v>
@@ -22773,7 +22773,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B416" t="s">
         <v>455</v>
@@ -22808,7 +22808,7 @@
     </row>
     <row r="417" spans="1:12">
       <c r="A417" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B417" t="s">
         <v>456</v>
@@ -22843,7 +22843,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B418" t="s">
         <v>457</v>
@@ -22864,7 +22864,7 @@
         <v>1607</v>
       </c>
       <c r="I418" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J418" t="s">
         <v>2163</v>
@@ -23021,7 +23021,7 @@
     </row>
     <row r="423" spans="1:12">
       <c r="A423" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B423" t="s">
         <v>462</v>
@@ -23056,7 +23056,7 @@
     </row>
     <row r="424" spans="1:12">
       <c r="A424" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B424" t="s">
         <v>463</v>
@@ -23112,7 +23112,7 @@
         <v>1607</v>
       </c>
       <c r="I425" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="J425" t="s">
         <v>2170</v>
@@ -23444,7 +23444,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B435" t="s">
         <v>474</v>
@@ -23479,7 +23479,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B436" t="s">
         <v>475</v>
@@ -23619,7 +23619,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B440" t="s">
         <v>479</v>
@@ -23654,7 +23654,7 @@
     </row>
     <row r="441" spans="1:12">
       <c r="A441" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B441" t="s">
         <v>480</v>
@@ -23689,7 +23689,7 @@
     </row>
     <row r="442" spans="1:12">
       <c r="A442" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B442" t="s">
         <v>481</v>
@@ -23759,7 +23759,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B444" t="s">
         <v>483</v>
@@ -23794,7 +23794,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B445" t="s">
         <v>484</v>
@@ -23815,7 +23815,7 @@
         <v>1607</v>
       </c>
       <c r="I445" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J445" t="s">
         <v>2190</v>
@@ -23829,7 +23829,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B446" t="s">
         <v>485</v>
@@ -23864,7 +23864,7 @@
     </row>
     <row r="447" spans="1:12">
       <c r="A447" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B447" t="s">
         <v>486</v>
@@ -23934,7 +23934,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B449" t="s">
         <v>488</v>
@@ -23969,7 +23969,7 @@
     </row>
     <row r="450" spans="1:12">
       <c r="A450" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B450" t="s">
         <v>489</v>
@@ -24004,7 +24004,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B451" t="s">
         <v>490</v>
@@ -24039,7 +24039,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B452" t="s">
         <v>491</v>
@@ -24063,7 +24063,7 @@
         <v>1614</v>
       </c>
       <c r="I452" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J452" t="s">
         <v>2197</v>
@@ -24098,7 +24098,7 @@
         <v>1607</v>
       </c>
       <c r="I453" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
       <c r="J453" t="s">
         <v>2198</v>
@@ -24112,7 +24112,7 @@
     </row>
     <row r="454" spans="1:12">
       <c r="A454" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B454" t="s">
         <v>493</v>
@@ -24147,7 +24147,7 @@
     </row>
     <row r="455" spans="1:12">
       <c r="A455" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B455" t="s">
         <v>494</v>
@@ -24182,7 +24182,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B456" t="s">
         <v>495</v>
@@ -24252,7 +24252,7 @@
     </row>
     <row r="458" spans="1:12">
       <c r="A458" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B458" t="s">
         <v>497</v>
@@ -24287,7 +24287,7 @@
     </row>
     <row r="459" spans="1:12">
       <c r="A459" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B459" t="s">
         <v>498</v>
@@ -24322,7 +24322,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B460" t="s">
         <v>499</v>
@@ -24357,7 +24357,7 @@
     </row>
     <row r="461" spans="1:12">
       <c r="A461" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B461" t="s">
         <v>500</v>
@@ -24378,7 +24378,7 @@
         <v>1607</v>
       </c>
       <c r="I461" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J461" t="s">
         <v>2206</v>
@@ -24392,7 +24392,7 @@
     </row>
     <row r="462" spans="1:12">
       <c r="A462" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B462" t="s">
         <v>501</v>
@@ -24427,7 +24427,7 @@
     </row>
     <row r="463" spans="1:12">
       <c r="A463" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B463" t="s">
         <v>502</v>
@@ -24462,7 +24462,7 @@
     </row>
     <row r="464" spans="1:12">
       <c r="A464" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B464" t="s">
         <v>503</v>
@@ -24532,7 +24532,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B466" t="s">
         <v>505</v>
@@ -24637,7 +24637,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B469" t="s">
         <v>508</v>
@@ -24672,7 +24672,7 @@
     </row>
     <row r="470" spans="1:12">
       <c r="A470" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B470" t="s">
         <v>509</v>
@@ -24707,7 +24707,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B471" t="s">
         <v>510</v>
@@ -24812,7 +24812,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B474" t="s">
         <v>513</v>
@@ -24917,7 +24917,7 @@
     </row>
     <row r="477" spans="1:12">
       <c r="A477" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B477" t="s">
         <v>516</v>
@@ -25022,7 +25022,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B480" t="s">
         <v>519</v>
@@ -25232,7 +25232,7 @@
     </row>
     <row r="486" spans="1:12">
       <c r="A486" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B486" t="s">
         <v>525</v>
@@ -25267,7 +25267,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B487" t="s">
         <v>526</v>
@@ -25442,7 +25442,7 @@
     </row>
     <row r="492" spans="1:12">
       <c r="A492" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B492" t="s">
         <v>531</v>
@@ -25463,7 +25463,7 @@
         <v>1607</v>
       </c>
       <c r="I492" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J492" t="s">
         <v>2236</v>
@@ -25477,7 +25477,7 @@
     </row>
     <row r="493" spans="1:12">
       <c r="A493" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B493" t="s">
         <v>532</v>
@@ -25536,7 +25536,7 @@
         <v>1615</v>
       </c>
       <c r="I494" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J494" t="s">
         <v>2238</v>
@@ -25571,7 +25571,7 @@
         <v>1607</v>
       </c>
       <c r="I495" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J495" t="s">
         <v>2239</v>
@@ -25606,7 +25606,7 @@
         <v>1607</v>
       </c>
       <c r="I496" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J496" t="s">
         <v>2239</v>
@@ -25620,7 +25620,7 @@
     </row>
     <row r="497" spans="1:12">
       <c r="A497" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B497" t="s">
         <v>535</v>
@@ -25655,7 +25655,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B498" t="s">
         <v>536</v>
@@ -25690,7 +25690,7 @@
     </row>
     <row r="499" spans="1:12">
       <c r="A499" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B499" t="s">
         <v>537</v>
@@ -25900,7 +25900,7 @@
     </row>
     <row r="505" spans="1:12">
       <c r="A505" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B505" t="s">
         <v>543</v>
@@ -26075,7 +26075,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B510" t="s">
         <v>548</v>
@@ -26096,7 +26096,7 @@
         <v>1607</v>
       </c>
       <c r="I510" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J510" t="s">
         <v>2253</v>
@@ -26145,7 +26145,7 @@
     </row>
     <row r="512" spans="1:12">
       <c r="A512" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B512" t="s">
         <v>550</v>
@@ -26320,7 +26320,7 @@
     </row>
     <row r="517" spans="1:12">
       <c r="A517" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B517" t="s">
         <v>555</v>
@@ -26358,7 +26358,7 @@
     </row>
     <row r="518" spans="1:12">
       <c r="A518" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B518" t="s">
         <v>556</v>
@@ -26393,7 +26393,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B519" t="s">
         <v>557</v>
@@ -26428,7 +26428,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B520" t="s">
         <v>558</v>
@@ -26498,7 +26498,7 @@
     </row>
     <row r="522" spans="1:12">
       <c r="A522" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B522" t="s">
         <v>560</v>
@@ -26603,7 +26603,7 @@
     </row>
     <row r="525" spans="1:12">
       <c r="A525" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B525" t="s">
         <v>563</v>
@@ -26638,7 +26638,7 @@
     </row>
     <row r="526" spans="1:12">
       <c r="A526" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B526" t="s">
         <v>564</v>
@@ -26659,7 +26659,7 @@
         <v>1607</v>
       </c>
       <c r="I526" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J526" t="s">
         <v>2269</v>
@@ -26673,7 +26673,7 @@
     </row>
     <row r="527" spans="1:12">
       <c r="A527" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B527" t="s">
         <v>565</v>
@@ -26743,7 +26743,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B529" t="s">
         <v>567</v>
@@ -26778,7 +26778,7 @@
     </row>
     <row r="530" spans="1:12">
       <c r="A530" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B530" t="s">
         <v>568</v>
@@ -26813,7 +26813,7 @@
     </row>
     <row r="531" spans="1:12">
       <c r="A531" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B531" t="s">
         <v>569</v>
@@ -26921,7 +26921,7 @@
     </row>
     <row r="534" spans="1:12">
       <c r="A534" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B534" t="s">
         <v>572</v>
@@ -27026,7 +27026,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B537" t="s">
         <v>575</v>
@@ -27096,7 +27096,7 @@
     </row>
     <row r="539" spans="1:12">
       <c r="A539" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B539" t="s">
         <v>577</v>
@@ -27131,7 +27131,7 @@
     </row>
     <row r="540" spans="1:12">
       <c r="A540" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B540" t="s">
         <v>578</v>
@@ -27201,7 +27201,7 @@
     </row>
     <row r="542" spans="1:12">
       <c r="A542" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B542" t="s">
         <v>580</v>
@@ -27271,7 +27271,7 @@
     </row>
     <row r="544" spans="1:12">
       <c r="A544" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B544" t="s">
         <v>582</v>
@@ -27306,7 +27306,7 @@
     </row>
     <row r="545" spans="1:12">
       <c r="A545" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B545" t="s">
         <v>583</v>
@@ -27376,7 +27376,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B547" t="s">
         <v>585</v>
@@ -27411,7 +27411,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B548" t="s">
         <v>586</v>
@@ -27446,7 +27446,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B549" t="s">
         <v>587</v>
@@ -27467,7 +27467,7 @@
         <v>1607</v>
       </c>
       <c r="I549" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J549" t="s">
         <v>2292</v>
@@ -27481,7 +27481,7 @@
     </row>
     <row r="550" spans="1:12">
       <c r="A550" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B550" t="s">
         <v>588</v>
@@ -27516,7 +27516,7 @@
     </row>
     <row r="551" spans="1:12">
       <c r="A551" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B551" t="s">
         <v>589</v>
@@ -27537,7 +27537,7 @@
         <v>1607</v>
       </c>
       <c r="I551" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J551" t="s">
         <v>2253</v>
@@ -27551,7 +27551,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B552" t="s">
         <v>590</v>
@@ -27586,7 +27586,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B553" t="s">
         <v>591</v>
@@ -27610,7 +27610,7 @@
         <v>1617</v>
       </c>
       <c r="I553" t="s">
-        <v>1650</v>
+        <v>1683</v>
       </c>
       <c r="J553" t="s">
         <v>2295</v>
@@ -27624,7 +27624,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B554" t="s">
         <v>592</v>
@@ -27799,7 +27799,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B559" t="s">
         <v>597</v>
@@ -27834,7 +27834,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B560" t="s">
         <v>598</v>
@@ -27869,7 +27869,7 @@
     </row>
     <row r="561" spans="1:12">
       <c r="A561" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B561" t="s">
         <v>599</v>
@@ -28009,7 +28009,7 @@
     </row>
     <row r="565" spans="1:12">
       <c r="A565" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B565" t="s">
         <v>603</v>
@@ -28044,7 +28044,7 @@
     </row>
     <row r="566" spans="1:12">
       <c r="A566" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B566" t="s">
         <v>604</v>
@@ -28079,7 +28079,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B567" t="s">
         <v>605</v>
@@ -28170,7 +28170,7 @@
         <v>1607</v>
       </c>
       <c r="I569" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J569" t="s">
         <v>2311</v>
@@ -28184,7 +28184,7 @@
     </row>
     <row r="570" spans="1:12">
       <c r="A570" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B570" t="s">
         <v>608</v>
@@ -28219,7 +28219,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B571" t="s">
         <v>609</v>
@@ -28240,7 +28240,7 @@
         <v>1607</v>
       </c>
       <c r="I571" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J571" t="s">
         <v>2313</v>
@@ -28254,7 +28254,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B572" t="s">
         <v>610</v>
@@ -28289,7 +28289,7 @@
     </row>
     <row r="573" spans="1:12">
       <c r="A573" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B573" t="s">
         <v>611</v>
@@ -28310,7 +28310,7 @@
         <v>1607</v>
       </c>
       <c r="I573" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J573" t="s">
         <v>2315</v>
@@ -28324,7 +28324,7 @@
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B574" t="s">
         <v>612</v>
@@ -28359,7 +28359,7 @@
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B575" t="s">
         <v>613</v>
@@ -28394,7 +28394,7 @@
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B576" t="s">
         <v>614</v>
@@ -28429,7 +28429,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B577" t="s">
         <v>615</v>
@@ -28502,7 +28502,7 @@
     </row>
     <row r="579" spans="1:12">
       <c r="A579" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B579" t="s">
         <v>617</v>
@@ -28537,7 +28537,7 @@
     </row>
     <row r="580" spans="1:12">
       <c r="A580" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B580" t="s">
         <v>618</v>
@@ -28607,7 +28607,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B582" t="s">
         <v>620</v>
@@ -28642,7 +28642,7 @@
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B583" t="s">
         <v>621</v>
@@ -28782,7 +28782,7 @@
     </row>
     <row r="587" spans="1:12">
       <c r="A587" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B587" t="s">
         <v>625</v>
@@ -28817,7 +28817,7 @@
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B588" t="s">
         <v>626</v>
@@ -28852,7 +28852,7 @@
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B589" t="s">
         <v>627</v>
@@ -28887,7 +28887,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B590" t="s">
         <v>628</v>
@@ -28922,7 +28922,7 @@
     </row>
     <row r="591" spans="1:12">
       <c r="A591" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B591" t="s">
         <v>629</v>
@@ -28957,7 +28957,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B592" t="s">
         <v>630</v>
@@ -28992,7 +28992,7 @@
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B593" t="s">
         <v>631</v>
@@ -29027,7 +29027,7 @@
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B594" t="s">
         <v>632</v>
@@ -29062,7 +29062,7 @@
     </row>
     <row r="595" spans="1:12">
       <c r="A595" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B595" t="s">
         <v>633</v>
@@ -29097,7 +29097,7 @@
     </row>
     <row r="596" spans="1:12">
       <c r="A596" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B596" t="s">
         <v>634</v>
@@ -29132,7 +29132,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B597" t="s">
         <v>635</v>
@@ -29167,7 +29167,7 @@
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B598" t="s">
         <v>636</v>
@@ -29202,7 +29202,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B599" t="s">
         <v>637</v>
@@ -29237,7 +29237,7 @@
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B600" t="s">
         <v>638</v>
@@ -29272,7 +29272,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -29307,7 +29307,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B602" t="s">
         <v>640</v>
@@ -29342,7 +29342,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B603" t="s">
         <v>641</v>
@@ -29377,7 +29377,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B604" t="s">
         <v>642</v>
@@ -29412,7 +29412,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B605" t="s">
         <v>643</v>
@@ -29447,7 +29447,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B606" t="s">
         <v>644</v>
@@ -29520,7 +29520,7 @@
     </row>
     <row r="608" spans="1:12">
       <c r="A608" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B608" t="s">
         <v>646</v>
@@ -29555,7 +29555,7 @@
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B609" t="s">
         <v>647</v>
@@ -29625,7 +29625,7 @@
     </row>
     <row r="611" spans="1:12">
       <c r="A611" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B611" t="s">
         <v>649</v>
@@ -29660,7 +29660,7 @@
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B612" t="s">
         <v>650</v>
@@ -29695,7 +29695,7 @@
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B613" t="s">
         <v>651</v>
@@ -29730,7 +29730,7 @@
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B614" t="s">
         <v>652</v>
@@ -29765,7 +29765,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B615" t="s">
         <v>653</v>
@@ -29786,7 +29786,7 @@
         <v>1607</v>
       </c>
       <c r="I615" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J615" t="s">
         <v>2355</v>
@@ -29800,7 +29800,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B616" t="s">
         <v>654</v>
@@ -29835,7 +29835,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B617" t="s">
         <v>655</v>
@@ -29870,7 +29870,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B618" t="s">
         <v>656</v>
@@ -29905,7 +29905,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B619" t="s">
         <v>657</v>
@@ -29981,7 +29981,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B621" t="s">
         <v>659</v>
@@ -30054,7 +30054,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B623" t="s">
         <v>661</v>
@@ -30089,7 +30089,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B624" t="s">
         <v>662</v>
@@ -30127,7 +30127,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B625" t="s">
         <v>663</v>
@@ -30273,7 +30273,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B629" t="s">
         <v>667</v>
@@ -30381,7 +30381,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B632" t="s">
         <v>670</v>
@@ -30416,7 +30416,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B633" t="s">
         <v>671</v>
@@ -30451,7 +30451,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B634" t="s">
         <v>672</v>
@@ -30486,7 +30486,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B635" t="s">
         <v>673</v>
@@ -30559,7 +30559,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B637" t="s">
         <v>675</v>
@@ -30594,7 +30594,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B638" t="s">
         <v>676</v>
@@ -30653,7 +30653,7 @@
         <v>1625</v>
       </c>
       <c r="I639" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="J639" t="s">
         <v>2378</v>
@@ -30667,7 +30667,7 @@
     </row>
     <row r="640" spans="1:12">
       <c r="A640" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B640" t="s">
         <v>678</v>
@@ -30702,7 +30702,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B641" t="s">
         <v>679</v>
@@ -30737,7 +30737,7 @@
     </row>
     <row r="642" spans="1:12">
       <c r="A642" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B642" t="s">
         <v>680</v>
@@ -30772,7 +30772,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B643" t="s">
         <v>681</v>
@@ -30807,7 +30807,7 @@
     </row>
     <row r="644" spans="1:12">
       <c r="A644" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B644" t="s">
         <v>682</v>
@@ -30842,7 +30842,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B645" t="s">
         <v>683</v>
@@ -30877,7 +30877,7 @@
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B646" t="s">
         <v>684</v>
@@ -30915,7 +30915,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B647" t="s">
         <v>685</v>
@@ -30950,7 +30950,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B648" t="s">
         <v>686</v>
@@ -30985,7 +30985,7 @@
     </row>
     <row r="649" spans="1:12">
       <c r="A649" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B649" t="s">
         <v>687</v>
@@ -31023,7 +31023,7 @@
     </row>
     <row r="650" spans="1:12">
       <c r="A650" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B650" t="s">
         <v>688</v>
@@ -31058,7 +31058,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B651" t="s">
         <v>689</v>
@@ -31093,7 +31093,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B652" t="s">
         <v>690</v>
@@ -31128,7 +31128,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B653" t="s">
         <v>691</v>
@@ -31163,7 +31163,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B654" t="s">
         <v>692</v>
@@ -31198,7 +31198,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B655" t="s">
         <v>693</v>
@@ -31233,7 +31233,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B656" t="s">
         <v>694</v>
@@ -31268,7 +31268,7 @@
     </row>
     <row r="657" spans="1:12">
       <c r="A657" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B657" t="s">
         <v>695</v>
@@ -31303,7 +31303,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B658" t="s">
         <v>696</v>
@@ -31338,7 +31338,7 @@
     </row>
     <row r="659" spans="1:12">
       <c r="A659" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B659" t="s">
         <v>697</v>
@@ -31373,7 +31373,7 @@
     </row>
     <row r="660" spans="1:12">
       <c r="A660" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B660" t="s">
         <v>698</v>
@@ -31408,7 +31408,7 @@
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B661" t="s">
         <v>699</v>
@@ -31443,7 +31443,7 @@
     </row>
     <row r="662" spans="1:12">
       <c r="A662" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B662" t="s">
         <v>700</v>
@@ -31478,7 +31478,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B663" t="s">
         <v>701</v>
@@ -31516,7 +31516,7 @@
     </row>
     <row r="664" spans="1:12">
       <c r="A664" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B664" t="s">
         <v>702</v>
@@ -31551,7 +31551,7 @@
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B665" t="s">
         <v>703</v>
@@ -31586,7 +31586,7 @@
     </row>
     <row r="666" spans="1:12">
       <c r="A666" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B666" t="s">
         <v>704</v>
@@ -31621,7 +31621,7 @@
     </row>
     <row r="667" spans="1:12">
       <c r="A667" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B667" t="s">
         <v>705</v>
@@ -31656,7 +31656,7 @@
     </row>
     <row r="668" spans="1:12">
       <c r="A668" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B668" t="s">
         <v>706</v>
@@ -31691,7 +31691,7 @@
     </row>
     <row r="669" spans="1:12">
       <c r="A669" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B669" t="s">
         <v>707</v>
@@ -31726,7 +31726,7 @@
     </row>
     <row r="670" spans="1:12">
       <c r="A670" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B670" t="s">
         <v>708</v>
@@ -31761,7 +31761,7 @@
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B671" t="s">
         <v>709</v>
@@ -31793,7 +31793,7 @@
     </row>
     <row r="672" spans="1:12">
       <c r="A672" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B672" t="s">
         <v>710</v>

</xml_diff>